<commit_message>
auto update queens news 2026-03-08T13:10:15Z
</commit_message>
<xml_diff>
--- a/data/output/queens_dev_news.xlsx
+++ b/data/output/queens_dev_news.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H1"/>
+  <dimension ref="A1:H2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -469,6 +469,44 @@
           <t>content_preview</t>
         </is>
       </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Permits Filed for 28-23 31st Street in Astoria, Queens</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>https://newyorkyimby.com/2026/03/permits-filed-for-28-23-31st-street-in-astoria-queens.html</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Permits have been filed for an 11-story mixed-use building at 28-23 31st Street in &lt;a href="https://newyorkyimby.com/neighborhoods/astoria"&gt;Astoria&lt;/a&gt;, Queens. Located between Newtown Avenue and 28th Road, the interior lot is near the 30th Avenue subway station, served by the N and W trains. Marios Mouzouris of Marvan Properties Inc. is listed as the owner behind the applications.</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>2026-03-08T10:30:16+00:00</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>Sun, 08 Mar 2026 10:30:16 +0000</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>YIMBY</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>YIMBY - Astoria</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
auto update queens news 2026-03-09T13:39:00Z
</commit_message>
<xml_diff>
--- a/data/output/queens_dev_news.xlsx
+++ b/data/output/queens_dev_news.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H2"/>
+  <dimension ref="A1:H1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -469,44 +469,6 @@
           <t>content_preview</t>
         </is>
       </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>Permits Filed for 28-23 31st Street in Astoria, Queens</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>https://newyorkyimby.com/2026/03/permits-filed-for-28-23-31st-street-in-astoria-queens.html</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>Permits have been filed for an 11-story mixed-use building at 28-23 31st Street in &lt;a href="https://newyorkyimby.com/neighborhoods/astoria"&gt;Astoria&lt;/a&gt;, Queens. Located between Newtown Avenue and 28th Road, the interior lot is near the 30th Avenue subway station, served by the N and W trains. Marios Mouzouris of Marvan Properties Inc. is listed as the owner behind the applications.</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>2026-03-08T10:30:16+00:00</t>
-        </is>
-      </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>Sun, 08 Mar 2026 10:30:16 +0000</t>
-        </is>
-      </c>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t>YIMBY</t>
-        </is>
-      </c>
-      <c r="G2" t="inlineStr">
-        <is>
-          <t>YIMBY - Astoria</t>
-        </is>
-      </c>
-      <c r="H2" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
auto update queens news 2026-04-19T13:33:08Z
</commit_message>
<xml_diff>
--- a/data/output/queens_dev_news.xlsx
+++ b/data/output/queens_dev_news.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H1"/>
+  <dimension ref="A1:H2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -469,6 +469,44 @@
           <t>content_preview</t>
         </is>
       </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>New Rendering Reveled for 51-02 Roosevelt Avenue in Sunnyside, Queens</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>https://newyorkyimby.com/2026/04/new-rendering-reveled-for-51-02-roosevelt-avenue-in-sunnyside-queens.html</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>A new rendering has been revealed for 51-02 Roosevelt Avenue, a 19-story mixed-use building in &lt;a href="https://newyorkyimby.com/neighborhoods/sunnyside"&gt;Sunnyside&lt;/a&gt;, Queens. Designed by Studio C Architects and developed by Zobuilden LLC, the structure will yield 84 condominium units, an ambulatory health facility, and ground-floor retail space, according to permits filed last month. The property is alternately addressed as 43-23 51st Street and bounded by Roosevelt Avenue to the north and 51st Street to the west.</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>2026-04-19T12:00:18+00:00</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>Sun, 19 Apr 2026 12:00:18 +0000</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>YIMBY</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>YIMBY - Sunnyside</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
auto update queens news 2026-04-20T14:08:37Z
</commit_message>
<xml_diff>
--- a/data/output/queens_dev_news.xlsx
+++ b/data/output/queens_dev_news.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H2"/>
+  <dimension ref="A1:H1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -469,44 +469,6 @@
           <t>content_preview</t>
         </is>
       </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>New Rendering Reveled for 51-02 Roosevelt Avenue in Sunnyside, Queens</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>https://newyorkyimby.com/2026/04/new-rendering-reveled-for-51-02-roosevelt-avenue-in-sunnyside-queens.html</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>A new rendering has been revealed for 51-02 Roosevelt Avenue, a 19-story mixed-use building in &lt;a href="https://newyorkyimby.com/neighborhoods/sunnyside"&gt;Sunnyside&lt;/a&gt;, Queens. Designed by Studio C Architects and developed by Zobuilden LLC, the structure will yield 84 condominium units, an ambulatory health facility, and ground-floor retail space, according to permits filed last month. The property is alternately addressed as 43-23 51st Street and bounded by Roosevelt Avenue to the north and 51st Street to the west.</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>2026-04-19T12:00:18+00:00</t>
-        </is>
-      </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>Sun, 19 Apr 2026 12:00:18 +0000</t>
-        </is>
-      </c>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t>YIMBY</t>
-        </is>
-      </c>
-      <c r="G2" t="inlineStr">
-        <is>
-          <t>YIMBY - Sunnyside</t>
-        </is>
-      </c>
-      <c r="H2" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
auto update queens news 2026-04-29T14:29:25Z
</commit_message>
<xml_diff>
--- a/data/output/queens_dev_news.xlsx
+++ b/data/output/queens_dev_news.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H1"/>
+  <dimension ref="A1:H8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -467,6 +467,280 @@
       <c r="H1" s="1" t="inlineStr">
         <is>
           <t>content_preview</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>136-15 38th Avenue’s Exterior Progresses In Flushing, Queens</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>https://newyorkyimby.com/2026/02/136-15-38th-avenues-exterior-progresses-in-flushing-queens.html</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Exterior work is progressing on 136-15 38th Avenue, a nine-story mixed-use building in &lt;a href="https://newyorkyimby.com/neighborhoods/flushing"&gt;Flushing&lt;/a&gt;, Queens. Designed by Angelo Ng &amp;#38; Anthony Ng Architects Studio for W H Plaza LLC, the 105-foot-tall structure will span nearly 24,000 square feet and yield ten condominium units with an average scope of 1,730 square feet. The project will also include 8,220 square feet of commercial space, 4,884 square feet of community facility space, and a 29-foot-long rear yard. The property is located between Main Street and 138th Street.</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>2026-02-27T13:00:43+00:00</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>Fri, 27 Feb 2026 13:00:43 +0000</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>YIMBY</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>YIMBY - Flushing</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>By: Michael Young and Matt Pruznick 8:00 am on February 27, 2026 Exterior work is progressing on 136-15 38th Avenue, a nine-story mixed-use building in Flushing, Queens. Designed by Angelo Ng &amp; Anthony Ng Architects Studio for W H Plaza LLC, the 105-foot-tall structure will span nearly 24,000 square feet and yield ten condominium units with an average scope of 1,730 square feet. The project will also include 8,220 square feet of commercial space, 4,884 square feet of community facility space, and a 29-foot-long rear yard. The property is located between Main Street and 138th Street. Most of the building has been enclosed since our last update in January 2025, when work had stalled with the reinforced concrete superstructure topped out and bare. The floor-to-ceiling windows are now fully in place on the main southern elevation, along with the glass railings on the tower’s signature wavy balconies. The lot line walls are finished in gray brick with horizontal bands lining the floor plates. Work is still finishing up on the multi-story podium, which remains obscured behind scaffolding and construction netting. 136-15 38th Avenue. Photo by Michael Young. 136-15 38th Avenue. Photo by Mi</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Queens Public Library At Rego Park Breaks Ground at 91–41 63rd Drive in Rego Park, Queens</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>https://newyorkyimby.com/2025/12/queens-public-library-at-rego-park-breaks-ground-at-91-41-63rd-drive-in-rego-park-queens.html</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Construction has broken ground on the Queens Public Library at Rego Park, located at 91–41 63rd Drive in &lt;a href="https://newyorkyimby.com/neighborhoods/rego-park"&gt;Rego Park&lt;/a&gt;, Queens. Designed by Weiss/Manfredi and managed by the Department of Design and Construction (DDC) on behalf of Queens Public Library, the three-story, 18,000-square-foot facility will replace the existing one-story, 7,500-square-foot branch. The site is located at the corner of 63rd Drive and Austin Street.</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>2025-12-15T12:30:50+00:00</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>Mon, 15 Dec 2025 12:30:50 +0000</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>YIMBY</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>YIMBY - Rego Park</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>By: Michael Young and Matt Pruznick 7:30 am on December 15, 2025 Construction has broken ground on the Queens Public Library at Rego Park, located at 91–41 63rd Drive in Rego Park, Queens. Designed by Weiss/Manfredi and managed by the Department of Design and Construction (DDC) on behalf of Queens Public Library, the three-story, 18,000-square-foot facility will replace the existing one-story, 7,500-square-foot branch. The site is located at the corner of 63rd Drive and Austin Street. A groundbreaking ceremony was held on December 9 in front of the current library. The Queens Public Library at Rego Park groundbreaking ceremony on December 9. Photo credit: DDC/Matthew Lapiska The rendering in the main photo looks southwest at the new structure from the intersection. The building will feature a distinctive massing with inward-sloping walls on both frontages. The façade will be composed of blue-green brick with interlocking L-shaped cutouts of floor-to-ceiling glass. Below is a street-level perspective looking southeast along Austin Street. The new Queens Public Library at Rego Park. Designed by Wiess/ Manfredi.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>ABS Partners seeks zoning change for 378K sf, approximately 394-unit mixed-use tower in Hell’s Kitchen</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>https://www.pincusco.com/abs-partners-seeks-zoning-change-for-378k-sf-approximately-394-unit-mixed-use-tower-in-hells-kitchen/</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>An entity affiliated with ABS Partners Real Estate and Modell Investment Team, 515 West 57th</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>NaT</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr"/>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>PincusCo</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>PincusCo - Home</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>Development 515 West 57th Street (red) (Credit - Cyclomedia) An entity affiliated with ABS Partners Real Estate and Modell Investment Team, 515 West 57th Street Leasehold LLC, submitted a proposal yesterday seeking a zoning change to develop a 377,970-square-foot, mixed residential and commercial development with approximately 394 dwelling units at 515 West 57th Street in Hell’s Kitchen, Manhattan. An estimated 119 of the residential units would be affordable, the filing says. This is an application that will be heard through the city’s Uniform Land Use Review Process (ULURP). The application seeks to rezone the target property, 515 West 57th Street (outlined in red), but the application if approved would also rezone three additional properties: a 368,195-square-foot office condominium building at 521 West 57th Street (outlined in blue); a 11,380-square-foot auto body shop at 505 West 57th Street (outlined in yellow); and a 67,511-square foot hotel at 534 West 58th Street, built in approximately 2014 (outlined in green). File 2025M0360 LINK ABS Partners Real Estate and Randy Modell’s Modell Investment Team through the entity 515 West 57th Street Leasehold LLC signed a 75-year groun</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Chang Biao Zheng pays $4.5M for 32-unit dev site in Flushing</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>https://www.pincusco.com/chang-biao-zheng-pays-4-5m-for-two-industrial-properties-in-flushing/</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Chang Biao Zheng through the entity Danny Family LLC paid $4.5 million to Shalom Zirkiev</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>NaT</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr"/>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>PincusCo</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>PincusCo - Home</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>Transfers 141-10 32nd Avenue schematic diagram (Credit - Michael Muroff architect via DOB) Chang Biao Zheng through the entity Danny Family LLC paid $4.5 million to Shalom Zirkiev through the entity Lm Re 1 LLC for the industrial building (G1) at 141-10 32nd Avenue in Flushing, Queens and industrial building (G1) at 141-12 32nd Avenue in Flushing, Queens. The expected use is ground up development. On these lots, there is one active new building construction project, Q00769923, for a 32-unit, 36,252 square-foot R-2 building. The project was submitted by Shalom Zirkiev with plans filed July 12, 2022 and it has not been permitted yet. In updated DOB plans, the individual Yanjuan Chen is identified as the owner, taking over these development plans. The sale closed on April 13, 2026 and was recorded on April 24, 2026. The two properties have 4,800 square feet of built space and 23,308 square feet of additional air rights for a total buildable of 28,080 square feet according to a PincusCo analysis of city data. The sale price per built square foot is $937 and the price per buildable square foot is $160 per the PincusCo analysis. (The price per square foot analysis is the transaction pric</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Ioannis Likidis pays $3.8M for 8-unit walkup in LIC</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>https://www.pincusco.com/ioannis-likidis-pays-3-8m-for-8-unit-walkup-in-lic/</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Ioannis Likidis through the entity 47 Vernon LLC paid $3.8 million to Andrew Anzalone through</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>NaT</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr"/>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>PincusCo</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>PincusCo - Home</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>Transfers 47-27 Vernon Blvd (Credit - Cyclomedia) Ioannis Likidis through the entity 47 Vernon LLC paid $3.8 million to Andrew Anzalone through the entity 47-27 Vernon Blvd LLC for the eight-unit residential walkup building (C7) at 47-27 Vernon Blvd in Long Island City, Queens. The expected use is cash flowing. The deal closed on April 17, 2026 and was recorded on April 24, 2026. The property has 8,050 square feet of built space according to a PincusCo analysis of city data. The sale price per built square foot is $465 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) The signatory for Andrew Anzalone was Andrew Anzalone. The signatory for Ioannis Likidis was Ioannis Likidis. The contract date was December 4, 2025. Prior sales, articles and revenue Prior to this transaction, PincusCo has records that the buyer Ioannis Likidis purchased five properties in four transactions for a total of $25.2 million and has no record it sold any properties over the past 24 months. The seller Andrew Anzalone had not purchased any other properties and had not sold any</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Leon Hedvat pays $3.5M for retail condos in Grand Central through bankruptcy</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>https://www.pincusco.com/behrooz-hedvat-pays-3-5m-for-retail-condos-in-grand-central-through-bankruptcy/</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>UPDATED 2:21 p.m., April 28, 2026: Leon Hedvat through the entity 32 Partners LLC paid</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>NaT</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr"/>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>PincusCo</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>PincusCo - Home</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>Transfers 32 West 39th Street (Credit - Cyclomedia) UPDATED 2:21 p.m., April 28, 2026: Leon Hedvat through the entity 32 Partners LLC paid $3.5 million through a bankruptcy for three retail condominium units and a storage unit at the office and retail condo building 32 West 39th Street in Grand Central, Manhattan. The expected use is cash flowing. The prior owner was Aron Rosenberg’s R&amp;B Realty Group through the entity 32 W. 39th Street Sole Member LLC, which placed the asset into bankruptcy. The deal closed on April 17, 2026 and was recorded on April 24, 2026. The four properties have 13,983 square feet of built space according to a PincusCo analysis of city data. The sale price per built square foot is $246 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) The signatory for R&amp;B Realty Group was David Wallen. The signatory for Leon Hedvat was Behrooz Hedvat . The contract date was February 11, 2026. Maltz Auctions was marketing the properties. Prior sales, articles and revenue Prior to this transaction, PincusCo has records that the buyer Behrooz He</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Investor pays $4.4M for industrial in Bedford Stuyvesant</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>https://www.pincusco.com/investor-pays-4-4m-for-industrial-in-bedford-stuyvesant/</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>An investor through the entity 111 Spencer LLC paid $4.4 million to Tobias Strulovitch through</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>NaT</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr"/>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>PincusCo</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>PincusCo - Home</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>Transfers 111 Spencer Street (Credit - Cyclomedia) An investor through the entity 111 Spencer LLC paid $4.4 million to Tobias Strulovitch through the entity Tal Hashmayim LLC for the industrial building (E1) at 111 Spencer Street in Bedford Stuyvesant, Brooklyn. The expected use is cash flowing. The deal closed on April 16, 2026 and was recorded on April 24, 2026. The property has 5,000 square feet of built space for a total buildable of 5,000 square feet according to a PincusCo analysis of city data. The sale price per built square foot is $880 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) The seller bought the property on July 19, 2023, for $7.5 million. The signatory for Tobias Strulovitch was Tobias Strulovitch. The contract date was August 28, 2025. Prior sales, articles and revenue Prior to this transaction, PincusCo has no record that the buyer had purchased any other properties and has no record it sold any properties over the past 24 months. The seller Tobias Strulovitch had not purchased any other properties and had not sold any propert</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto update queens news 2026-04-30T14:22:47Z
</commit_message>
<xml_diff>
--- a/data/output/queens_dev_news.xlsx
+++ b/data/output/queens_dev_news.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H8"/>
+  <dimension ref="A1:H10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -473,108 +473,88 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>136-15 38th Avenue’s Exterior Progresses In Flushing, Queens</t>
+          <t>Z Capital Group pays $2.5M for two properties in Rockaway Beach</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>https://newyorkyimby.com/2026/02/136-15-38th-avenues-exterior-progresses-in-flushing-queens.html</t>
+          <t>https://www.pincusco.com/z-capital-group-pays-2-5m-for-two-properties-in-rockaway-beach/</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Exterior work is progressing on 136-15 38th Avenue, a nine-story mixed-use building in &lt;a href="https://newyorkyimby.com/neighborhoods/flushing"&gt;Flushing&lt;/a&gt;, Queens. Designed by Angelo Ng &amp;#38; Anthony Ng Architects Studio for W H Plaza LLC, the 105-foot-tall structure will span nearly 24,000 square feet and yield ten condominium units with an average scope of 1,730 square feet. The project will also include 8,220 square feet of commercial space, 4,884 square feet of community facility space, and a 29-foot-long rear yard. The property is located between Main Street and 138th Street.</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>2026-02-27T13:00:43+00:00</t>
-        </is>
-      </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>Fri, 27 Feb 2026 13:00:43 +0000</t>
-        </is>
-      </c>
+          <t>Z Capital Group through the entity Melo Z Phantom Cap LLC paid $2.5 million to</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr"/>
+      <c r="E2" t="inlineStr"/>
       <c r="F2" t="inlineStr">
         <is>
-          <t>YIMBY</t>
+          <t>PincusCo</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>YIMBY - Flushing</t>
+          <t>PincusCo - Home</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>By: Michael Young and Matt Pruznick 8:00 am on February 27, 2026 Exterior work is progressing on 136-15 38th Avenue, a nine-story mixed-use building in Flushing, Queens. Designed by Angelo Ng &amp; Anthony Ng Architects Studio for W H Plaza LLC, the 105-foot-tall structure will span nearly 24,000 square feet and yield ten condominium units with an average scope of 1,730 square feet. The project will also include 8,220 square feet of commercial space, 4,884 square feet of community facility space, and a 29-foot-long rear yard. The property is located between Main Street and 138th Street. Most of the building has been enclosed since our last update in January 2025, when work had stalled with the reinforced concrete superstructure topped out and bare. The floor-to-ceiling windows are now fully in place on the main southern elevation, along with the glass railings on the tower’s signature wavy balconies. The lot line walls are finished in gray brick with horizontal bands lining the floor plates. Work is still finishing up on the multi-story podium, which remains obscured behind scaffolding and construction netting. 136-15 38th Avenue. Photo by Michael Young. 136-15 38th Avenue. Photo by Mi</t>
+          <t>Transfers 2-22 Beach 97th Street (Credit - Cyclomedia) Z Capital Group through the entity Melo Z Phantom Cap LLC paid $2.5 million to Robert Falco through the entity Robert Victoria Incorporated for the eight-unit property (C7) at 2-22 Beach 97th Street in Rockaway Beach, Queens and an adjacent parcel (V0) on Beach 97th Street in Rockaway Beach, Queens. The deal closed on March 20, 2026 and was recorded on April 28, 2026. The two properties have 6,240 square feet of built space and 12,552 square feet of additional air rights for a total buildable of 18,765 square feet according to a PincusCo analysis of city data. The sale price per built square foot is $400 and the price per buildable square foot is $133 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) The signatory for Robert Falco was Richard Edward Gresio. The signatory for Israel Babayev’s Z Capital Group was Ariel Rabanipour. The contract date was November 24, 2025. Prior sales, articles and revenue Prior to this transaction, PincusCo has records that the buyer Z Capital Group purchased five p</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Queens Public Library At Rego Park Breaks Ground at 91–41 63rd Drive in Rego Park, Queens</t>
+          <t>Owemanco pays $3.8M to Firebird for 21-unit rental in Crown Heights, was $4.3M in 2020</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>https://newyorkyimby.com/2025/12/queens-public-library-at-rego-park-breaks-ground-at-91-41-63rd-drive-in-rego-park-queens.html</t>
+          <t>https://www.pincusco.com/owemanco-pays-3-8m-to-firebird-for-21-unit-rental-in-crown-heights-was-4-3m-in-2020/</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Construction has broken ground on the Queens Public Library at Rego Park, located at 91–41 63rd Drive in &lt;a href="https://newyorkyimby.com/neighborhoods/rego-park"&gt;Rego Park&lt;/a&gt;, Queens. Designed by Weiss/Manfredi and managed by the Department of Design and Construction (DDC) on behalf of Queens Public Library, the three-story, 18,000-square-foot facility will replace the existing one-story, 7,500-square-foot branch. The site is located at the corner of 63rd Drive and Austin Street.</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>2025-12-15T12:30:50+00:00</t>
-        </is>
-      </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>Mon, 15 Dec 2025 12:30:50 +0000</t>
-        </is>
-      </c>
+          <t>Owemanco through the entity Owemanco’s Crown Heights Run L.P. paid $3.8 million to Firebird Grove</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr"/>
+      <c r="E3" t="inlineStr"/>
       <c r="F3" t="inlineStr">
         <is>
-          <t>YIMBY</t>
+          <t>PincusCo</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>YIMBY - Rego Park</t>
+          <t>PincusCo - Home</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>By: Michael Young and Matt Pruznick 7:30 am on December 15, 2025 Construction has broken ground on the Queens Public Library at Rego Park, located at 91–41 63rd Drive in Rego Park, Queens. Designed by Weiss/Manfredi and managed by the Department of Design and Construction (DDC) on behalf of Queens Public Library, the three-story, 18,000-square-foot facility will replace the existing one-story, 7,500-square-foot branch. The site is located at the corner of 63rd Drive and Austin Street. A groundbreaking ceremony was held on December 9 in front of the current library. The Queens Public Library at Rego Park groundbreaking ceremony on December 9. Photo credit: DDC/Matthew Lapiska The rendering in the main photo looks southwest at the new structure from the intersection. The building will feature a distinctive massing with inward-sloping walls on both frontages. The façade will be composed of blue-green brick with interlocking L-shaped cutouts of floor-to-ceiling glass. Below is a street-level perspective looking southeast along Austin Street. The new Queens Public Library at Rego Park. Designed by Wiess/ Manfredi.</t>
+          <t>Transfers 665 St Marks Avenue (Credit - Cyclomedia) Owemanco through the entity Owemanco’s Crown Heights Run L.P. paid $3.8 million to Firebird Grove through the entity OR 665 St. Marks LLC for the 21-unit residential elevator building (D9) at 665 St Marks Avenue in Crown Heights, Brooklyn. The expected use is cash flowing. The deal closed on March 30, 2026 and was recorded on April 28, 2026. The property has 17,790 square feet of built space according to a PincusCo analysis of city data. The sale price per built square foot is $213 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) The seller bought the property on October 6, 2020, for $4.3 million. The signatory for Firebird Grove was Adam Semler . The signatory for Owemanco was Sohail Zayona . The contract date was November 12, 2025. Prior sales, articles and revenue Prior to this transaction, PincusCo has records that the buyer Owemanco purchased three properties in three transactions for a total of $19 million and has no record it sold any properties over the past 24 months. The seller Firebird G</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>ABS Partners seeks zoning change for 378K sf, approximately 394-unit mixed-use tower in Hell’s Kitchen</t>
+          <t>JSAF Capital pays $4.2M for 19-unit rental in Flatbush</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>https://www.pincusco.com/abs-partners-seeks-zoning-change-for-378k-sf-approximately-394-unit-mixed-use-tower-in-hells-kitchen/</t>
+          <t>https://www.pincusco.com/jsaf-capital-pays-4-2m-for-19-unit-rental-in-flatbush/</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>An entity affiliated with ABS Partners Real Estate and Modell Investment Team, 515 West 57th</t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>NaT</t>
-        </is>
-      </c>
+          <t>JSAF Capital through the entity Bedat Holding LLC paid $4.2 million to Loeffler family through</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr"/>
       <c r="E4" t="inlineStr"/>
       <c r="F4" t="inlineStr">
         <is>
@@ -588,31 +568,27 @@
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>Development 515 West 57th Street (red) (Credit - Cyclomedia) An entity affiliated with ABS Partners Real Estate and Modell Investment Team, 515 West 57th Street Leasehold LLC, submitted a proposal yesterday seeking a zoning change to develop a 377,970-square-foot, mixed residential and commercial development with approximately 394 dwelling units at 515 West 57th Street in Hell’s Kitchen, Manhattan. An estimated 119 of the residential units would be affordable, the filing says. This is an application that will be heard through the city’s Uniform Land Use Review Process (ULURP). The application seeks to rezone the target property, 515 West 57th Street (outlined in red), but the application if approved would also rezone three additional properties: a 368,195-square-foot office condominium building at 521 West 57th Street (outlined in blue); a 11,380-square-foot auto body shop at 505 West 57th Street (outlined in yellow); and a 67,511-square foot hotel at 534 West 58th Street, built in approximately 2014 (outlined in green). File 2025M0360 LINK ABS Partners Real Estate and Randy Modell’s Modell Investment Team through the entity 515 West 57th Street Leasehold LLC signed a 75-year groun</t>
+          <t>Transfers 1710 Newkirk Avenue (Credit - Cyclomedia) JSAF Capital through the entity Bedat Holding LLC paid $4.2 million to Loeffler family through the entity 1710 L.L.C. for the 19-unit residential elevator building (D1) at 1710 Newkirk Avenue in Flatbush, Brooklyn. The expected use is cash flowing. The deal closed on April 17, 2026 and was recorded on April 28, 2026. The property has 17,213 square feet of built space according to a PincusCo analysis of city data. The sale price per built square foot is $244 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) The signatory for Erica Loeffler and Antoinette Loeffler was Erica Loeffler. The signatory for JSAF Capital was Joseph Safdie . The contract date was March 2, 2026. Prior sales, articles and revenue Prior to this transaction, PincusCo has records that the buyer JSAF Capital purchased three properties in three transactions for a total of $6.8 million and has no record it sold any properties over the past 24 months. The seller Erica Loeffler had not purchased any other properties and had not sold an</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Chang Biao Zheng pays $4.5M for 32-unit dev site in Flushing</t>
+          <t>Kings Capital pays $7.2M for 20-unit walkup in Alphabet City</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>https://www.pincusco.com/chang-biao-zheng-pays-4-5m-for-two-industrial-properties-in-flushing/</t>
+          <t>https://www.pincusco.com/kings-capital-pays-7-2m-for-20-unit-walkup-in-alphabet-city/</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Chang Biao Zheng through the entity Danny Family LLC paid $4.5 million to Shalom Zirkiev</t>
-        </is>
-      </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>NaT</t>
-        </is>
-      </c>
+          <t>Kings Capital through the entity 109 East 29th LLC paid $7.2 million to the entity</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr"/>
       <c r="E5" t="inlineStr"/>
       <c r="F5" t="inlineStr">
         <is>
@@ -626,31 +602,27 @@
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>Transfers 141-10 32nd Avenue schematic diagram (Credit - Michael Muroff architect via DOB) Chang Biao Zheng through the entity Danny Family LLC paid $4.5 million to Shalom Zirkiev through the entity Lm Re 1 LLC for the industrial building (G1) at 141-10 32nd Avenue in Flushing, Queens and industrial building (G1) at 141-12 32nd Avenue in Flushing, Queens. The expected use is ground up development. On these lots, there is one active new building construction project, Q00769923, for a 32-unit, 36,252 square-foot R-2 building. The project was submitted by Shalom Zirkiev with plans filed July 12, 2022 and it has not been permitted yet. In updated DOB plans, the individual Yanjuan Chen is identified as the owner, taking over these development plans. The sale closed on April 13, 2026 and was recorded on April 24, 2026. The two properties have 4,800 square feet of built space and 23,308 square feet of additional air rights for a total buildable of 28,080 square feet according to a PincusCo analysis of city data. The sale price per built square foot is $937 and the price per buildable square foot is $160 per the PincusCo analysis. (The price per square foot analysis is the transaction pric</t>
+          <t xml:space="preserve">Transfers 515 East 12th Street (Credit - Cyclomedia) Kings Capital through the entity 109 East 29th LLC paid $7.2 million to the entity 491 Bayonne LLC for the 20-unit residential walkup building (C7) at 515 East 12th Street in Alphabet City, Manhattan. The expected use is cash flowing. The deal closed on April 27, 2026 and was recorded on April 29, 2026. The property has 9,309 square feet of built space and 1,006 square feet of additional air rights for a total buildable of 10,324 square feet according to a PincusCo analysis of city data. The sale price per built square foot is $778 and the price per buildable square foot is $702 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) The signatories for the sellers Marshall Aronow, David Aronow, and Anna Bauder were David Aronow and Andrew Lee. The signatory for Kings Capital was Jeffrey Znaty . The contract date was December 29, 2025. Prior sales, articles and revenue Prior to this transaction, PincusCo has records that the buyer Kings Capital purchased four properties in three transactions for a total </t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Ioannis Likidis pays $3.8M for 8-unit walkup in LIC</t>
+          <t>Avery Hall, Brodsky Org. pay $49M for dev site in Crown Heights</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>https://www.pincusco.com/ioannis-likidis-pays-3-8m-for-8-unit-walkup-in-lic/</t>
+          <t>https://www.pincusco.com/avery-hall-brodsky-org-pay-49m-for-dev-site-in-crown-heights/</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Ioannis Likidis through the entity 47 Vernon LLC paid $3.8 million to Andrew Anzalone through</t>
-        </is>
-      </c>
-      <c r="D6" t="inlineStr">
-        <is>
-          <t>NaT</t>
-        </is>
-      </c>
+          <t>Avery Hall Investments and Brodsky Organization paid $49 million to two sellers in two transactions</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr"/>
       <c r="E6" t="inlineStr"/>
       <c r="F6" t="inlineStr">
         <is>
@@ -664,31 +636,27 @@
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>Transfers 47-27 Vernon Blvd (Credit - Cyclomedia) Ioannis Likidis through the entity 47 Vernon LLC paid $3.8 million to Andrew Anzalone through the entity 47-27 Vernon Blvd LLC for the eight-unit residential walkup building (C7) at 47-27 Vernon Blvd in Long Island City, Queens. The expected use is cash flowing. The deal closed on April 17, 2026 and was recorded on April 24, 2026. The property has 8,050 square feet of built space according to a PincusCo analysis of city data. The sale price per built square foot is $465 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) The signatory for Andrew Anzalone was Andrew Anzalone. The signatory for Ioannis Likidis was Ioannis Likidis. The contract date was December 4, 2025. Prior sales, articles and revenue Prior to this transaction, PincusCo has records that the buyer Ioannis Likidis purchased five properties in four transactions for a total of $25.2 million and has no record it sold any properties over the past 24 months. The seller Andrew Anzalone had not purchased any other properties and had not sold any</t>
+          <t>Top Story Transfers 962 Pacific Street (Credit - Cyclomedia) Avery Hall Investments and Brodsky Organization paid $49 million to two sellers in two transactions for a development site in Crown Heights, Brooklyn. In the larger transaction, Avery Hall Investments and Brodsky Organization through the entity Pacific Dean Owner LLC paid $33 million to Nadine Oelsner through the entity 962 Pacific St LLC for the development parcel (V1) at 962 Pacific Street in Crown Heights, Brooklyn. The expected use is ground up development. The deal closed on April 14, 2026 and was recorded on April 29, 2026. The property has zero square feet of built space and 33,415 square feet of additional air rights for a total buildable of 33,415 square feet according to a PincusCo analysis of city data. The sale price per buildable square foot is $987 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) The signatory for Nadine Oelsner was Nadine Oelsner. The signatory for Avery Hall Investments , Brodsky Organization , and Monadnock Construction was Avishy Fisher . The contract dat</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Leon Hedvat pays $3.5M for retail condos in Grand Central through bankruptcy</t>
+          <t>Palwinder Singh pays $12.8M for likely dev site in LIC</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>https://www.pincusco.com/behrooz-hedvat-pays-3-5m-for-retail-condos-in-grand-central-through-bankruptcy/</t>
+          <t>https://www.pincusco.com/palwinder-singh-pays-12-8m-for-likely-dev-site-in-lic/</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>UPDATED 2:21 p.m., April 28, 2026: Leon Hedvat through the entity 32 Partners LLC paid</t>
-        </is>
-      </c>
-      <c r="D7" t="inlineStr">
-        <is>
-          <t>NaT</t>
-        </is>
-      </c>
+          <t>Palwinder Singh (who often partners with Aditya Shah) paid $12.8 million to Antonio Restivo for</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr"/>
       <c r="E7" t="inlineStr"/>
       <c r="F7" t="inlineStr">
         <is>
@@ -702,31 +670,27 @@
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>Transfers 32 West 39th Street (Credit - Cyclomedia) UPDATED 2:21 p.m., April 28, 2026: Leon Hedvat through the entity 32 Partners LLC paid $3.5 million through a bankruptcy for three retail condominium units and a storage unit at the office and retail condo building 32 West 39th Street in Grand Central, Manhattan. The expected use is cash flowing. The prior owner was Aron Rosenberg’s R&amp;B Realty Group through the entity 32 W. 39th Street Sole Member LLC, which placed the asset into bankruptcy. The deal closed on April 17, 2026 and was recorded on April 24, 2026. The four properties have 13,983 square feet of built space according to a PincusCo analysis of city data. The sale price per built square foot is $246 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) The signatory for R&amp;B Realty Group was David Wallen. The signatory for Leon Hedvat was Behrooz Hedvat . The contract date was February 11, 2026. Maltz Auctions was marketing the properties. Prior sales, articles and revenue Prior to this transaction, PincusCo has records that the buyer Behrooz He</t>
+          <t xml:space="preserve">Transfers 531 47th Avenue (Credit - Cyclomedia) Palwinder Singh (who often partners with Aditya Shah) paid $12.8 million to Antonio Restivo for a likely development site in Long Island City in two transactions. In the first, Palwinder Singh through the entity 47th Ave LIC LLC paid $6.4 million to Antonio Restivo through the entity Island Point Properties 11, Inc. for the vacant lot (G7) at 5-31 47th Avenue in Long Island City, Queens. The expected use is ground up development. The deal closed on April 21, 2026 and was recorded on April 29, 2026. The property has zero square feet of built space and 8,150 square feet of additional air rights for a total buildable of 8,150 square feet according to a PincusCo analysis of city data. The sale price per buildable square foot is $785 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) In the second, Palwinder Singh through the entity 47th Ave LIC LLC paid $6.4 million to Antonio Restivo through the entity 5-33 Realty LLC for the vacant lot (G7) at 5-33 47th Avenue in Long Island City, Queens. The expected use </t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Investor pays $4.4M for industrial in Bedford Stuyvesant</t>
+          <t>Rialto Capital takes title to APF’s Midtown West office in foreclosure valued at $46.9M</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>https://www.pincusco.com/investor-pays-4-4m-for-industrial-in-bedford-stuyvesant/</t>
+          <t>https://www.pincusco.com/rialto-capital-takes-title-to-apfs-midtown-west-office-in-foreclosure-valued-at-46-9m/</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>An investor through the entity 111 Spencer LLC paid $4.4 million to Tobias Strulovitch through</t>
-        </is>
-      </c>
-      <c r="D8" t="inlineStr">
-        <is>
-          <t>NaT</t>
-        </is>
-      </c>
+          <t>Rialto Capital Management through the entity RSS Comm2014-Ccre15- Ny W4f, LLC through a judicial foreclosure</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr"/>
       <c r="E8" t="inlineStr"/>
       <c r="F8" t="inlineStr">
         <is>
@@ -740,7 +704,75 @@
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>Transfers 111 Spencer Street (Credit - Cyclomedia) An investor through the entity 111 Spencer LLC paid $4.4 million to Tobias Strulovitch through the entity Tal Hashmayim LLC for the industrial building (E1) at 111 Spencer Street in Bedford Stuyvesant, Brooklyn. The expected use is cash flowing. The deal closed on April 16, 2026 and was recorded on April 24, 2026. The property has 5,000 square feet of built space for a total buildable of 5,000 square feet according to a PincusCo analysis of city data. The sale price per built square foot is $880 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) The seller bought the property on July 19, 2023, for $7.5 million. The signatory for Tobias Strulovitch was Tobias Strulovitch. The contract date was August 28, 2025. Prior sales, articles and revenue Prior to this transaction, PincusCo has no record that the buyer had purchased any other properties and has no record it sold any properties over the past 24 months. The seller Tobias Strulovitch had not purchased any other properties and had not sold any propert</t>
+          <t>Transfers 25 West 45th Street (Credit - Cyclomedia) Rialto Capital Management through the entity RSS Comm2014-Ccre15- Ny W4f, LLC through a judicial foreclosure for the office building (O6) at 25 West 45th Street in Midtown West, Manhattan. The expected use is hold for sale. The prior owner, APF Properties, lost the asset through this foreclosure auction. The city valued the transfer at $46.9 million. The deal closed on April 17, 2026 and was recorded on April 29, 2026. The property has 187,567 square feet of built space according to a PincusCo analysis of city data. The sale price per built square foot is $250 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) The seller bought the property on January 31, 2022, for $64.2 million. The signatory for APF Properties was Christy DeMelfi . The signatory for Rialto Capital Management was Adam Singer . The contract date was April 17, 2026. The former owner was APF Properties, led by Kenneth S. Aschendorf, who lost it in the action 850160/2024 filed in New York County Supreme Court. PincusCo does not consider</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Benny Wercberger signs $19.5M construction loan for 99-unit project in Mt Hope</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>https://www.pincusco.com/benny-wercberger-signs-19-5m-construction-loan-for-99-unit-project-in-mt-hope/</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Benny Wercberger through the entity Mt Hope 27 LLC as borrower signed a new construction</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr"/>
+      <c r="E9" t="inlineStr"/>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>PincusCo</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>PincusCo - Home</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>Transfers 29 Mt Hope Place (Credit - Cyclomedia) Benny Wercberger through the entity Mt Hope 27 LLC as borrower signed a new construction loan with lender NorthEast Community Bank for a 99-unit project planned for 27-29 Mt Hope Place in Mt Hope, Bronx. The deal closed on April 23, 2026 and was recorded on April 29, 2026. The property has 4,096 square feet of built space and 14,718 square feet of additional air rights for a total buildable of 18,812 square feet according to a PincusCo analysis of city data. The loan price per built square foot is $4,757 and the price per buildable square foot is $1,035 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) The owner bought the property on November 10, 2025, for $3.5 million. The signatory for Benny Wercberger was Benny Wercberger. This is for a 99-unit building on lots 32, 33. Joel Brach of Buildhouser borrowed $21.1 million for an affiliated 99-unit project next door at 23 Mt Hope Place. Prior sales, articles and revenue The owners according to the Department of Housing Preservation and Development includ</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Joel Brach signs $21.1M construction loan for 99-unit project in Mt Hope</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>https://www.pincusco.com/joel-brach-signs-21-1m-construction-loan-for-99-unit-project-in-mt-hope/</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Buildhouser through the entity Mt Hope 23 LLC as borrower signed a new construction loan</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr"/>
+      <c r="E10" t="inlineStr"/>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>PincusCo</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>PincusCo - Home</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>Transfers 23 Mt Hope Place axonometric diagram (Credit - Nikolai Katz architect via DOB) Buildhouser through the entity Mt Hope 23 LLC as borrower signed a new construction loan with lender NorthEast Community Bank through the entity Northeast Community Bank valued at $21.1 million for the 99-unit project planned for 23 Mt Hope Place in Mt Hope, Bronx. On the lot, there is one active new building construction project, X01222893, for a 99-unit, 71,622 square-foot residential (R-2) building. The project was submitted by Buildhouser and filed by Joel Brach with plans filed May 16, 2025 and permitted March 19, 2026. The deal closed on April 23, 2026 and was recorded on April 29, 2026. The property has 3,420 square feet of built space and 15,406 square feet of additional air rights for a total buildable of 18,812 square feet according to a PincusCo analysis of city data. The loan price per planned development square foot is $295 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) The owner bought the property on October 3, 2025, for $1.9 million. The signat</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto update queens news 2026-05-01T13:52:20Z
</commit_message>
<xml_diff>
--- a/data/output/queens_dev_news.xlsx
+++ b/data/output/queens_dev_news.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H10"/>
+  <dimension ref="A1:H4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -473,17 +473,17 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Z Capital Group pays $2.5M for two properties in Rockaway Beach</t>
+          <t>JEMB files 28-unit, single-floor conversion plan for 75 Broad in FiDi</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>https://www.pincusco.com/z-capital-group-pays-2-5m-for-two-properties-in-rockaway-beach/</t>
+          <t>https://www.pincusco.com/jemb-files-28-unit-single-floor-conversion-plan-for-75-broad-in-fidi/</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Z Capital Group through the entity Melo Z Phantom Cap LLC paid $2.5 million to</t>
+          <t>JEMB Realty submitted a major alteration application to convert the second floor of the office</t>
         </is>
       </c>
       <c r="D2" t="inlineStr"/>
@@ -500,24 +500,24 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>Transfers 2-22 Beach 97th Street (Credit - Cyclomedia) Z Capital Group through the entity Melo Z Phantom Cap LLC paid $2.5 million to Robert Falco through the entity Robert Victoria Incorporated for the eight-unit property (C7) at 2-22 Beach 97th Street in Rockaway Beach, Queens and an adjacent parcel (V0) on Beach 97th Street in Rockaway Beach, Queens. The deal closed on March 20, 2026 and was recorded on April 28, 2026. The two properties have 6,240 square feet of built space and 12,552 square feet of additional air rights for a total buildable of 18,765 square feet according to a PincusCo analysis of city data. The sale price per built square foot is $400 and the price per buildable square foot is $133 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) The signatory for Robert Falco was Richard Edward Gresio. The signatory for Israel Babayev’s Z Capital Group was Ariel Rabanipour. The contract date was November 24, 2025. Prior sales, articles and revenue Prior to this transaction, PincusCo has records that the buyer Z Capital Group purchased five p</t>
+          <t>Development 61 Broad Street also known as 75 Broad Street (Credit - Cyclomedia) JEMB Realty submitted a major alteration application to convert the second floor of the office building at 75 Broad Street, in the filing referred to as 61 Broad Street, in the Financial District, Manhattan, from office space to 28 residential units. The plan was filed on April 29, 2026, with the New York City Department of Buildings under job number M01355263. The project is described in the filing as: application filed for the conversion of the 2nd floor to residential use as shown on the filed plans. The applicant is the Registered Architect John Cetra of Cetraruddy Architecture. The building’s certificate of occupancy says the 34-story, 661,283-square-foot structure is an office building with school use on the first floor. The neighborhood In Financial District, The majority, or 74 percent of the 79.9 million square feet of commercial built space are office buildings, with elevator buildings next occupying 15 percent of the space. In sales, Financial District has the 4th highest sale turnover among other neighborhoods in the city with $2.3 billion in sales volume in the last two years. For developme</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Owemanco pays $3.8M to Firebird for 21-unit rental in Crown Heights, was $4.3M in 2020</t>
+          <t>Bawabeh Holdings seeks rezone to build up to 972 units in East Flatbush</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>https://www.pincusco.com/owemanco-pays-3-8m-to-firebird-for-21-unit-rental-in-crown-heights-was-4-3m-in-2020/</t>
+          <t>https://www.pincusco.com/bawabeh-holdings-seeks-rezone-to-build-up-to-972-units-in-east-flatbush/</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Owemanco through the entity Owemanco’s Crown Heights Run L.P. paid $3.8 million to Firebird Grove</t>
+          <t>Bawabeh Holdings through the entity Midyan Gate Realty No. 2 LLC submitted an application with</t>
         </is>
       </c>
       <c r="D3" t="inlineStr"/>
@@ -534,24 +534,24 @@
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>Transfers 665 St Marks Avenue (Credit - Cyclomedia) Owemanco through the entity Owemanco’s Crown Heights Run L.P. paid $3.8 million to Firebird Grove through the entity OR 665 St. Marks LLC for the 21-unit residential elevator building (D9) at 665 St Marks Avenue in Crown Heights, Brooklyn. The expected use is cash flowing. The deal closed on March 30, 2026 and was recorded on April 28, 2026. The property has 17,790 square feet of built space according to a PincusCo analysis of city data. The sale price per built square foot is $213 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) The seller bought the property on October 6, 2020, for $4.3 million. The signatory for Firebird Grove was Adam Semler . The signatory for Owemanco was Sohail Zayona . The contract date was November 12, 2025. Prior sales, articles and revenue Prior to this transaction, PincusCo has records that the buyer Owemanco purchased three properties in three transactions for a total of $19 million and has no record it sold any properties over the past 24 months. The seller Firebird G</t>
+          <t>Chart_Frontpage Development Top Story East 98th Street project portion (Credit - IMC Architecture) Bawabeh Holdings through the entity Midyan Gate Realty No. 2 LLC submitted an application with the city seeking zoning changes to develop approximately 972 residential units in a nine-building development with a total of 1.2 million square feet along East 98th Street in the East Flatbush neighborhood of Brooklyn. The application for Uniform Land Use Review Procedure (ULURP) has two separate documents, and one describes a slightly smaller version of the project, with 786 dwelling units and 778,374 square feet. The document with the larger figures is the Environmental Assessment Statement.</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>JSAF Capital pays $4.2M for 19-unit rental in Flatbush</t>
+          <t>Yitzchok Schwartz pays $6M through bankruptcy for likely dev site in Bedford Stuyvesant</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>https://www.pincusco.com/jsaf-capital-pays-4-2m-for-19-unit-rental-in-flatbush/</t>
+          <t>https://www.pincusco.com/yitzchok-schwartz-pays-6m-through-bankruptcy-for-likely-dev-site-in-bedford-stuyvesant/</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>JSAF Capital through the entity Bedat Holding LLC paid $4.2 million to Loeffler family through</t>
+          <t>Yitzchok Schwartz through the entity Van Buren II LLC paid $6 million through a bankruptcy</t>
         </is>
       </c>
       <c r="D4" t="inlineStr"/>
@@ -568,211 +568,7 @@
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>Transfers 1710 Newkirk Avenue (Credit - Cyclomedia) JSAF Capital through the entity Bedat Holding LLC paid $4.2 million to Loeffler family through the entity 1710 L.L.C. for the 19-unit residential elevator building (D1) at 1710 Newkirk Avenue in Flatbush, Brooklyn. The expected use is cash flowing. The deal closed on April 17, 2026 and was recorded on April 28, 2026. The property has 17,213 square feet of built space according to a PincusCo analysis of city data. The sale price per built square foot is $244 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) The signatory for Erica Loeffler and Antoinette Loeffler was Erica Loeffler. The signatory for JSAF Capital was Joseph Safdie . The contract date was March 2, 2026. Prior sales, articles and revenue Prior to this transaction, PincusCo has records that the buyer JSAF Capital purchased three properties in three transactions for a total of $6.8 million and has no record it sold any properties over the past 24 months. The seller Erica Loeffler had not purchased any other properties and had not sold an</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>Kings Capital pays $7.2M for 20-unit walkup in Alphabet City</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>https://www.pincusco.com/kings-capital-pays-7-2m-for-20-unit-walkup-in-alphabet-city/</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>Kings Capital through the entity 109 East 29th LLC paid $7.2 million to the entity</t>
-        </is>
-      </c>
-      <c r="D5" t="inlineStr"/>
-      <c r="E5" t="inlineStr"/>
-      <c r="F5" t="inlineStr">
-        <is>
-          <t>PincusCo</t>
-        </is>
-      </c>
-      <c r="G5" t="inlineStr">
-        <is>
-          <t>PincusCo - Home</t>
-        </is>
-      </c>
-      <c r="H5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Transfers 515 East 12th Street (Credit - Cyclomedia) Kings Capital through the entity 109 East 29th LLC paid $7.2 million to the entity 491 Bayonne LLC for the 20-unit residential walkup building (C7) at 515 East 12th Street in Alphabet City, Manhattan. The expected use is cash flowing. The deal closed on April 27, 2026 and was recorded on April 29, 2026. The property has 9,309 square feet of built space and 1,006 square feet of additional air rights for a total buildable of 10,324 square feet according to a PincusCo analysis of city data. The sale price per built square foot is $778 and the price per buildable square foot is $702 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) The signatories for the sellers Marshall Aronow, David Aronow, and Anna Bauder were David Aronow and Andrew Lee. The signatory for Kings Capital was Jeffrey Znaty . The contract date was December 29, 2025. Prior sales, articles and revenue Prior to this transaction, PincusCo has records that the buyer Kings Capital purchased four properties in three transactions for a total </t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>Avery Hall, Brodsky Org. pay $49M for dev site in Crown Heights</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>https://www.pincusco.com/avery-hall-brodsky-org-pay-49m-for-dev-site-in-crown-heights/</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>Avery Hall Investments and Brodsky Organization paid $49 million to two sellers in two transactions</t>
-        </is>
-      </c>
-      <c r="D6" t="inlineStr"/>
-      <c r="E6" t="inlineStr"/>
-      <c r="F6" t="inlineStr">
-        <is>
-          <t>PincusCo</t>
-        </is>
-      </c>
-      <c r="G6" t="inlineStr">
-        <is>
-          <t>PincusCo - Home</t>
-        </is>
-      </c>
-      <c r="H6" t="inlineStr">
-        <is>
-          <t>Top Story Transfers 962 Pacific Street (Credit - Cyclomedia) Avery Hall Investments and Brodsky Organization paid $49 million to two sellers in two transactions for a development site in Crown Heights, Brooklyn. In the larger transaction, Avery Hall Investments and Brodsky Organization through the entity Pacific Dean Owner LLC paid $33 million to Nadine Oelsner through the entity 962 Pacific St LLC for the development parcel (V1) at 962 Pacific Street in Crown Heights, Brooklyn. The expected use is ground up development. The deal closed on April 14, 2026 and was recorded on April 29, 2026. The property has zero square feet of built space and 33,415 square feet of additional air rights for a total buildable of 33,415 square feet according to a PincusCo analysis of city data. The sale price per buildable square foot is $987 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) The signatory for Nadine Oelsner was Nadine Oelsner. The signatory for Avery Hall Investments , Brodsky Organization , and Monadnock Construction was Avishy Fisher . The contract dat</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>Palwinder Singh pays $12.8M for likely dev site in LIC</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>https://www.pincusco.com/palwinder-singh-pays-12-8m-for-likely-dev-site-in-lic/</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>Palwinder Singh (who often partners with Aditya Shah) paid $12.8 million to Antonio Restivo for</t>
-        </is>
-      </c>
-      <c r="D7" t="inlineStr"/>
-      <c r="E7" t="inlineStr"/>
-      <c r="F7" t="inlineStr">
-        <is>
-          <t>PincusCo</t>
-        </is>
-      </c>
-      <c r="G7" t="inlineStr">
-        <is>
-          <t>PincusCo - Home</t>
-        </is>
-      </c>
-      <c r="H7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Transfers 531 47th Avenue (Credit - Cyclomedia) Palwinder Singh (who often partners with Aditya Shah) paid $12.8 million to Antonio Restivo for a likely development site in Long Island City in two transactions. In the first, Palwinder Singh through the entity 47th Ave LIC LLC paid $6.4 million to Antonio Restivo through the entity Island Point Properties 11, Inc. for the vacant lot (G7) at 5-31 47th Avenue in Long Island City, Queens. The expected use is ground up development. The deal closed on April 21, 2026 and was recorded on April 29, 2026. The property has zero square feet of built space and 8,150 square feet of additional air rights for a total buildable of 8,150 square feet according to a PincusCo analysis of city data. The sale price per buildable square foot is $785 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) In the second, Palwinder Singh through the entity 47th Ave LIC LLC paid $6.4 million to Antonio Restivo through the entity 5-33 Realty LLC for the vacant lot (G7) at 5-33 47th Avenue in Long Island City, Queens. The expected use </t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>Rialto Capital takes title to APF’s Midtown West office in foreclosure valued at $46.9M</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>https://www.pincusco.com/rialto-capital-takes-title-to-apfs-midtown-west-office-in-foreclosure-valued-at-46-9m/</t>
-        </is>
-      </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>Rialto Capital Management through the entity RSS Comm2014-Ccre15- Ny W4f, LLC through a judicial foreclosure</t>
-        </is>
-      </c>
-      <c r="D8" t="inlineStr"/>
-      <c r="E8" t="inlineStr"/>
-      <c r="F8" t="inlineStr">
-        <is>
-          <t>PincusCo</t>
-        </is>
-      </c>
-      <c r="G8" t="inlineStr">
-        <is>
-          <t>PincusCo - Home</t>
-        </is>
-      </c>
-      <c r="H8" t="inlineStr">
-        <is>
-          <t>Transfers 25 West 45th Street (Credit - Cyclomedia) Rialto Capital Management through the entity RSS Comm2014-Ccre15- Ny W4f, LLC through a judicial foreclosure for the office building (O6) at 25 West 45th Street in Midtown West, Manhattan. The expected use is hold for sale. The prior owner, APF Properties, lost the asset through this foreclosure auction. The city valued the transfer at $46.9 million. The deal closed on April 17, 2026 and was recorded on April 29, 2026. The property has 187,567 square feet of built space according to a PincusCo analysis of city data. The sale price per built square foot is $250 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) The seller bought the property on January 31, 2022, for $64.2 million. The signatory for APF Properties was Christy DeMelfi . The signatory for Rialto Capital Management was Adam Singer . The contract date was April 17, 2026. The former owner was APF Properties, led by Kenneth S. Aschendorf, who lost it in the action 850160/2024 filed in New York County Supreme Court. PincusCo does not consider</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>Benny Wercberger signs $19.5M construction loan for 99-unit project in Mt Hope</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>https://www.pincusco.com/benny-wercberger-signs-19-5m-construction-loan-for-99-unit-project-in-mt-hope/</t>
-        </is>
-      </c>
-      <c r="C9" t="inlineStr">
-        <is>
-          <t>Benny Wercberger through the entity Mt Hope 27 LLC as borrower signed a new construction</t>
-        </is>
-      </c>
-      <c r="D9" t="inlineStr"/>
-      <c r="E9" t="inlineStr"/>
-      <c r="F9" t="inlineStr">
-        <is>
-          <t>PincusCo</t>
-        </is>
-      </c>
-      <c r="G9" t="inlineStr">
-        <is>
-          <t>PincusCo - Home</t>
-        </is>
-      </c>
-      <c r="H9" t="inlineStr">
-        <is>
-          <t>Transfers 29 Mt Hope Place (Credit - Cyclomedia) Benny Wercberger through the entity Mt Hope 27 LLC as borrower signed a new construction loan with lender NorthEast Community Bank for a 99-unit project planned for 27-29 Mt Hope Place in Mt Hope, Bronx. The deal closed on April 23, 2026 and was recorded on April 29, 2026. The property has 4,096 square feet of built space and 14,718 square feet of additional air rights for a total buildable of 18,812 square feet according to a PincusCo analysis of city data. The loan price per built square foot is $4,757 and the price per buildable square foot is $1,035 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) The owner bought the property on November 10, 2025, for $3.5 million. The signatory for Benny Wercberger was Benny Wercberger. This is for a 99-unit building on lots 32, 33. Joel Brach of Buildhouser borrowed $21.1 million for an affiliated 99-unit project next door at 23 Mt Hope Place. Prior sales, articles and revenue The owners according to the Department of Housing Preservation and Development includ</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>Joel Brach signs $21.1M construction loan for 99-unit project in Mt Hope</t>
-        </is>
-      </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>https://www.pincusco.com/joel-brach-signs-21-1m-construction-loan-for-99-unit-project-in-mt-hope/</t>
-        </is>
-      </c>
-      <c r="C10" t="inlineStr">
-        <is>
-          <t>Buildhouser through the entity Mt Hope 23 LLC as borrower signed a new construction loan</t>
-        </is>
-      </c>
-      <c r="D10" t="inlineStr"/>
-      <c r="E10" t="inlineStr"/>
-      <c r="F10" t="inlineStr">
-        <is>
-          <t>PincusCo</t>
-        </is>
-      </c>
-      <c r="G10" t="inlineStr">
-        <is>
-          <t>PincusCo - Home</t>
-        </is>
-      </c>
-      <c r="H10" t="inlineStr">
-        <is>
-          <t>Transfers 23 Mt Hope Place axonometric diagram (Credit - Nikolai Katz architect via DOB) Buildhouser through the entity Mt Hope 23 LLC as borrower signed a new construction loan with lender NorthEast Community Bank through the entity Northeast Community Bank valued at $21.1 million for the 99-unit project planned for 23 Mt Hope Place in Mt Hope, Bronx. On the lot, there is one active new building construction project, X01222893, for a 99-unit, 71,622 square-foot residential (R-2) building. The project was submitted by Buildhouser and filed by Joel Brach with plans filed May 16, 2025 and permitted March 19, 2026. The deal closed on April 23, 2026 and was recorded on April 29, 2026. The property has 3,420 square feet of built space and 15,406 square feet of additional air rights for a total buildable of 18,812 square feet according to a PincusCo analysis of city data. The loan price per planned development square foot is $295 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) The owner bought the property on October 3, 2025, for $1.9 million. The signat</t>
+          <t xml:space="preserve">Transfers Yitzchok Schwartz through the entity Van Buren II LLC paid $6 million through a bankruptcy to Upper Room Baptist Church through the entity Richard J Corbi, Esq, Chapter 11 Operating Trustee for the specialty building (M1) at 180 Van Buren in Bedford Stuyvesant, Brooklyn. The expected use is ground up development. The deal closed on April 21, 2026 and was recorded on April 28, 2026. The property has 12,610 square feet of built space and 17,400 square feet of additional air rights for a total buildable of 30,000 square feet according to a PincusCo analysis of city data. The sale price per built square foot is $475 and the price per buildable square foot is $200 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) The signatory for Upper Room Baptist Church was Richard J. Corbi. The signatory for Yitzchok Schwartz was Yitzchok Schwartz. The contract date was December 22, 2025. The bankruptcy was filed in 2025 in the Eastern District of New York under index number 25-40070-nhl. Prior sales, articles and revenue Prior to this transaction, PincusCo </t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto update queens news 2026-05-02T13:45:53Z
</commit_message>
<xml_diff>
--- a/data/output/queens_dev_news.xlsx
+++ b/data/output/queens_dev_news.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H4"/>
+  <dimension ref="A1:H7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -473,17 +473,17 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>JEMB files 28-unit, single-floor conversion plan for 75 Broad in FiDi</t>
+          <t>Young-Hee Lowe pays $8.5M to Mews Property for 12-unit rental in Grand Central</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>https://www.pincusco.com/jemb-files-28-unit-single-floor-conversion-plan-for-75-broad-in-fidi/</t>
+          <t>https://www.pincusco.com/young-hee-lowe-pays-8-5m-to-mews-property-for-12-unit-rental-in-grand-central/</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>JEMB Realty submitted a major alteration application to convert the second floor of the office</t>
+          <t>Young-Hee Lowe through the entity 130 East 37 Street LLC paid $8.5 million to Mews</t>
         </is>
       </c>
       <c r="D2" t="inlineStr"/>
@@ -500,24 +500,24 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>Development 61 Broad Street also known as 75 Broad Street (Credit - Cyclomedia) JEMB Realty submitted a major alteration application to convert the second floor of the office building at 75 Broad Street, in the filing referred to as 61 Broad Street, in the Financial District, Manhattan, from office space to 28 residential units. The plan was filed on April 29, 2026, with the New York City Department of Buildings under job number M01355263. The project is described in the filing as: application filed for the conversion of the 2nd floor to residential use as shown on the filed plans. The applicant is the Registered Architect John Cetra of Cetraruddy Architecture. The building’s certificate of occupancy says the 34-story, 661,283-square-foot structure is an office building with school use on the first floor. The neighborhood In Financial District, The majority, or 74 percent of the 79.9 million square feet of commercial built space are office buildings, with elevator buildings next occupying 15 percent of the space. In sales, Financial District has the 4th highest sale turnover among other neighborhoods in the city with $2.3 billion in sales volume in the last two years. For developme</t>
+          <t>Transfers 130 East 37th Street (Credit - Cyclomedia) Young-Hee Lowe through the entity 130 East 37 Street LLC paid $8.5 million to Mews Property through the entity Whitehall Ennismore 37 LLC for the 12-unit residential elevator building (D3) at 130 East 37th Street in Grand Central, Manhattan. The expected use is cash flowing. The deal closed on April 17, 2026 and was recorded on April 30, 2026. The property has 5,570 square feet of built space and 3,821 square feet of additional air rights for a total buildable of 9,390 square feet according to a PincusCo analysis of city data. The sale price per built square foot is $1,526 and the price per buildable square foot is $905 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) The seller bought the property on February 11, 2021, for $3.4 million. The signatory for Mews Property was W. Alexander Budney . The signatory for Young-Hee Lowe was Young-Hee Lowe. The contract date was March 25, 2026. Prior sales, articles and revenue Prior to this transaction, PincusCo has no record that the buyer Young-Hee Lowe h</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Bawabeh Holdings seeks rezone to build up to 972 units in East Flatbush</t>
+          <t>Zelig Weiss signs contract as buyer with Francmen Realty for likely dev site in Jamaica</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>https://www.pincusco.com/bawabeh-holdings-seeks-rezone-to-build-up-to-972-units-in-east-flatbush/</t>
+          <t>https://www.pincusco.com/zelig-weiss-signs-contract-as-buyer-with-francmen-realty-for-likely-dev-site-in-jamaica/</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Bawabeh Holdings through the entity Midyan Gate Realty No. 2 LLC submitted an application with</t>
+          <t>Zelig Weiss through the entity 165 Residence LLC signed a contract as buyer with Francmen</t>
         </is>
       </c>
       <c r="D3" t="inlineStr"/>
@@ -534,24 +534,24 @@
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>Chart_Frontpage Development Top Story East 98th Street project portion (Credit - IMC Architecture) Bawabeh Holdings through the entity Midyan Gate Realty No. 2 LLC submitted an application with the city seeking zoning changes to develop approximately 972 residential units in a nine-building development with a total of 1.2 million square feet along East 98th Street in the East Flatbush neighborhood of Brooklyn. The application for Uniform Land Use Review Procedure (ULURP) has two separate documents, and one describes a slightly smaller version of the project, with 786 dwelling units and 778,374 square feet. The document with the larger figures is the Environmental Assessment Statement.</t>
+          <t>Transfers 89-49 164th Street (Credit - Cyclomedia) Zelig Weiss through the entity 165 Residence LLC signed a contract as buyer with Francmen Realty as seller for the retail building (K1) at 89-49 164th Street in Jamaica, Queens. The expected use is ground up development. The price was not disclosed on the memorandum of contract. The memorandum of contract was signed on on March 10, 2026 and was recorded on April 30, 2026. The property has 23,250 square feet of built space and 93,000 square feet of additional air rights for a total buildable of 116,250 square feet according to a PincusCo analysis of city data. The signatory for Francmen Realty was Zelig Weiss. Prior sales, articles and revenue Prior to this transaction, PincusCo has no record that the buyer Zelig Weiss had purchased any other properties and has no record it sold any properties over the past 24 months. The seller Francmen Realty had not purchased any other properties and sold three properties in three transactions for a total of $13.5 million over the same time period. The 23,250-square-foot property generated revenue of $1.2 million or $53 per square foot, according to the most recent income and expense figures. The</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Yitzchok Schwartz pays $6M through bankruptcy for likely dev site in Bedford Stuyvesant</t>
+          <t>Sabet Group pays $4.3M for 10-unit walkup in Alphabet City</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>https://www.pincusco.com/yitzchok-schwartz-pays-6m-through-bankruptcy-for-likely-dev-site-in-bedford-stuyvesant/</t>
+          <t>https://www.pincusco.com/sabet-group-pays-4-3m-for-10-unit-walkup-in-alphabet-city/</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Yitzchok Schwartz through the entity Van Buren II LLC paid $6 million through a bankruptcy</t>
+          <t>Sabet Group through the entity 502 E 12 St Holdings LLC paid $4.3 million to</t>
         </is>
       </c>
       <c r="D4" t="inlineStr"/>
@@ -568,7 +568,109 @@
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Transfers Yitzchok Schwartz through the entity Van Buren II LLC paid $6 million through a bankruptcy to Upper Room Baptist Church through the entity Richard J Corbi, Esq, Chapter 11 Operating Trustee for the specialty building (M1) at 180 Van Buren in Bedford Stuyvesant, Brooklyn. The expected use is ground up development. The deal closed on April 21, 2026 and was recorded on April 28, 2026. The property has 12,610 square feet of built space and 17,400 square feet of additional air rights for a total buildable of 30,000 square feet according to a PincusCo analysis of city data. The sale price per built square foot is $475 and the price per buildable square foot is $200 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) The signatory for Upper Room Baptist Church was Richard J. Corbi. The signatory for Yitzchok Schwartz was Yitzchok Schwartz. The contract date was December 22, 2025. The bankruptcy was filed in 2025 in the Eastern District of New York under index number 25-40070-nhl. Prior sales, articles and revenue Prior to this transaction, PincusCo </t>
+          <t>Transfers 502 East 12th Street (Credit - Cyclomedia) Sabet Group through the entity 502 E 12 St Holdings LLC paid $4.3 million to Norma Herrick through the entity Herrick 502 LLC for the 10-unit residential walkup building (C4) at 502 East 12th Street in Alphabet City, Manhattan. The expected use is cash flowing. The deal closed on April 29, 2026 and was recorded on April 30, 2026. The property has 6,300 square feet of built space according to a PincusCo analysis of city data. The sale price per built square foot is $678 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) The signatory for Norma Herrick was Norma Herrick. The signatory for Sabet Group was Alfred Sabetfard . The contract date was January 26, 2026. Prior sales, articles and revenue Prior to this transaction, PincusCo has records that the buyer Sabet Group purchased 18 properties in 17 transactions for a total of $116.3 million and has no record it sold any properties over the past 24 months. The seller Norma Herrick had not purchased any other properties and had not sold any properties o</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>James Rogers-Gahan pays $9.2M to RYCO Capital for mixed-use in Greenwich Village</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>https://www.pincusco.com/james-rogers-gahan-pays-9-2m-to-ryco-capital-for-mixed-use-in-greenwich-village/</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>James Rogers-Gahan through the entity 280 Bleecker Street Owner LLC paid $9.2 million to RYCO</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr"/>
+      <c r="E5" t="inlineStr"/>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>PincusCo</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>PincusCo - Home</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>Transfers 280 Bleecker Street (Credit - Cyclomedia) James Rogers-Gahan through the entity 280 Bleecker Street Owner LLC paid $9.2 million to RYCO Capital through the entity Keystone 280 Bleecker LLC for the three-unit mixed-use building (S3) at 280 Bleecker Street in Greenwich Village, Manhattan. The expected use is cash flowing. The deal closed on April 23, 2026 and was recorded on April 30, 2026. The property has 4,208 square feet of built space and 1,511 square feet of additional air rights for a total buildable of 5,713 square feet according to a PincusCo analysis of city data. The sale price per built square foot is $2,198 and the price per buildable square foot is $1,618 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) The seller bought the property on April 16, 2021, for $4.8 million. The signatory for RYCO Capital was James D. Ryan III. The signatory for James Rogers-Gahan was James Rogers-Gahan. The contract date was December 12, 2025. Prior sales, articles and revenue Prior to this transaction, PincusCo has no record that the buyer James R</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Hikari Power Z Co. pays $15.2M to Kriss, Lockhill Properties for 20-unit walkup in Midtown East</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>https://www.pincusco.com/hikari-power-z-co-pays-15-2m-to-kriss-lockhill-properties-for-residential-walkup-in-midtown-east/</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Hikari Power Z Co. through the entity Hikari Power Z Co., Ltd. paid $15.2 million</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr"/>
+      <c r="E6" t="inlineStr"/>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>PincusCo</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>PincusCo - Home</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>Transfers 246 East 53rd Street (Credit - Cyclomedia) Hikari Power Z Co. through the entity Hikari Power Z Co., Ltd. paid $15.2 million to Jody Kriss and Lockhill Properties through the entity 246 E 53rd Owner LLC for the 20-unit residential walkup building (C7) at 246 East 53rd Street in Midtown East, Manhattan. The expected use is cash flowing. The deal closed on April 20, 2026 and was recorded on April 30, 2026. The property has 12,915 square feet of built space and 468 square feet of additional air rights for a total buildable of 13,388 square feet according to a PincusCo analysis of city data. The sale price per built square foot is $1,176 and the price per buildable square foot is $1,135 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) The sellers bought the property on February 14, 2025, for $8.1 million. The signatory for Jody Kriss and Lockhill Properties was Parke Leatherman and Jody Kriss. The signatory for Hikari Power Z Co. was Michael A. Mulia . The contract date was January 5, 2026. Prior sales, articles and revenue Prior to this trans</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Gulf Coast Commercial pays $4M to Related Companies for mixed-use in Chelsea</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>https://www.pincusco.com/gulf-coast-commercial-pays-4m-to-related-companies-for-mixed-use-in-chelsea/</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Florida-based Gulf Coast Commercial through the entity 559 West 22nd Development, LLC paid $4 million</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr"/>
+      <c r="E7" t="inlineStr"/>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>PincusCo</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>PincusCo - Home</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>Transfers 162 11th Avenue (Credit - Cyclomedia) Florida-based Gulf Coast Commercial through the entity 559 West 22nd Development, LLC paid $4 million to Related Companies through the entity 22nd And 11th Associates, L.L.C. for the mixed-use building (K9) at 162 11th Avenue in Chelsea, Manhattan. The expected use is cash flowing. The deal closed on April 27, 2026 and was recorded on April 30, 2026. The property has 7,408 square feet of built space and 6,515 square feet of additional air rights for a total buildable of 13,919 square feet according to a PincusCo analysis of city data. The sale price per built square foot is $539 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) The seller bought the property on October 10, 2017, for $16.6 million. The signatory for Related Companies was Andrew Orchulli . The signatory for Gulf Coast Commercial was Philip J. McCabe . The contract date was February 27, 2026. Related utilized 6,538 square feet of the excess development rights for its apartment project at 555 West 22nd Street, in 2019. Prior sales, articles</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto update queens news 2026-05-03T13:46:43Z
</commit_message>
<xml_diff>
--- a/data/output/queens_dev_news.xlsx
+++ b/data/output/queens_dev_news.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H7"/>
+  <dimension ref="A1:H1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -467,210 +467,6 @@
       <c r="H1" s="1" t="inlineStr">
         <is>
           <t>content_preview</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>Young-Hee Lowe pays $8.5M to Mews Property for 12-unit rental in Grand Central</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>https://www.pincusco.com/young-hee-lowe-pays-8-5m-to-mews-property-for-12-unit-rental-in-grand-central/</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>Young-Hee Lowe through the entity 130 East 37 Street LLC paid $8.5 million to Mews</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr"/>
-      <c r="E2" t="inlineStr"/>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t>PincusCo</t>
-        </is>
-      </c>
-      <c r="G2" t="inlineStr">
-        <is>
-          <t>PincusCo - Home</t>
-        </is>
-      </c>
-      <c r="H2" t="inlineStr">
-        <is>
-          <t>Transfers 130 East 37th Street (Credit - Cyclomedia) Young-Hee Lowe through the entity 130 East 37 Street LLC paid $8.5 million to Mews Property through the entity Whitehall Ennismore 37 LLC for the 12-unit residential elevator building (D3) at 130 East 37th Street in Grand Central, Manhattan. The expected use is cash flowing. The deal closed on April 17, 2026 and was recorded on April 30, 2026. The property has 5,570 square feet of built space and 3,821 square feet of additional air rights for a total buildable of 9,390 square feet according to a PincusCo analysis of city data. The sale price per built square foot is $1,526 and the price per buildable square foot is $905 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) The seller bought the property on February 11, 2021, for $3.4 million. The signatory for Mews Property was W. Alexander Budney . The signatory for Young-Hee Lowe was Young-Hee Lowe. The contract date was March 25, 2026. Prior sales, articles and revenue Prior to this transaction, PincusCo has no record that the buyer Young-Hee Lowe h</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>Zelig Weiss signs contract as buyer with Francmen Realty for likely dev site in Jamaica</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>https://www.pincusco.com/zelig-weiss-signs-contract-as-buyer-with-francmen-realty-for-likely-dev-site-in-jamaica/</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>Zelig Weiss through the entity 165 Residence LLC signed a contract as buyer with Francmen</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr"/>
-      <c r="E3" t="inlineStr"/>
-      <c r="F3" t="inlineStr">
-        <is>
-          <t>PincusCo</t>
-        </is>
-      </c>
-      <c r="G3" t="inlineStr">
-        <is>
-          <t>PincusCo - Home</t>
-        </is>
-      </c>
-      <c r="H3" t="inlineStr">
-        <is>
-          <t>Transfers 89-49 164th Street (Credit - Cyclomedia) Zelig Weiss through the entity 165 Residence LLC signed a contract as buyer with Francmen Realty as seller for the retail building (K1) at 89-49 164th Street in Jamaica, Queens. The expected use is ground up development. The price was not disclosed on the memorandum of contract. The memorandum of contract was signed on on March 10, 2026 and was recorded on April 30, 2026. The property has 23,250 square feet of built space and 93,000 square feet of additional air rights for a total buildable of 116,250 square feet according to a PincusCo analysis of city data. The signatory for Francmen Realty was Zelig Weiss. Prior sales, articles and revenue Prior to this transaction, PincusCo has no record that the buyer Zelig Weiss had purchased any other properties and has no record it sold any properties over the past 24 months. The seller Francmen Realty had not purchased any other properties and sold three properties in three transactions for a total of $13.5 million over the same time period. The 23,250-square-foot property generated revenue of $1.2 million or $53 per square foot, according to the most recent income and expense figures. The</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>Sabet Group pays $4.3M for 10-unit walkup in Alphabet City</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>https://www.pincusco.com/sabet-group-pays-4-3m-for-10-unit-walkup-in-alphabet-city/</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>Sabet Group through the entity 502 E 12 St Holdings LLC paid $4.3 million to</t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr"/>
-      <c r="E4" t="inlineStr"/>
-      <c r="F4" t="inlineStr">
-        <is>
-          <t>PincusCo</t>
-        </is>
-      </c>
-      <c r="G4" t="inlineStr">
-        <is>
-          <t>PincusCo - Home</t>
-        </is>
-      </c>
-      <c r="H4" t="inlineStr">
-        <is>
-          <t>Transfers 502 East 12th Street (Credit - Cyclomedia) Sabet Group through the entity 502 E 12 St Holdings LLC paid $4.3 million to Norma Herrick through the entity Herrick 502 LLC for the 10-unit residential walkup building (C4) at 502 East 12th Street in Alphabet City, Manhattan. The expected use is cash flowing. The deal closed on April 29, 2026 and was recorded on April 30, 2026. The property has 6,300 square feet of built space according to a PincusCo analysis of city data. The sale price per built square foot is $678 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) The signatory for Norma Herrick was Norma Herrick. The signatory for Sabet Group was Alfred Sabetfard . The contract date was January 26, 2026. Prior sales, articles and revenue Prior to this transaction, PincusCo has records that the buyer Sabet Group purchased 18 properties in 17 transactions for a total of $116.3 million and has no record it sold any properties over the past 24 months. The seller Norma Herrick had not purchased any other properties and had not sold any properties o</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>James Rogers-Gahan pays $9.2M to RYCO Capital for mixed-use in Greenwich Village</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>https://www.pincusco.com/james-rogers-gahan-pays-9-2m-to-ryco-capital-for-mixed-use-in-greenwich-village/</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>James Rogers-Gahan through the entity 280 Bleecker Street Owner LLC paid $9.2 million to RYCO</t>
-        </is>
-      </c>
-      <c r="D5" t="inlineStr"/>
-      <c r="E5" t="inlineStr"/>
-      <c r="F5" t="inlineStr">
-        <is>
-          <t>PincusCo</t>
-        </is>
-      </c>
-      <c r="G5" t="inlineStr">
-        <is>
-          <t>PincusCo - Home</t>
-        </is>
-      </c>
-      <c r="H5" t="inlineStr">
-        <is>
-          <t>Transfers 280 Bleecker Street (Credit - Cyclomedia) James Rogers-Gahan through the entity 280 Bleecker Street Owner LLC paid $9.2 million to RYCO Capital through the entity Keystone 280 Bleecker LLC for the three-unit mixed-use building (S3) at 280 Bleecker Street in Greenwich Village, Manhattan. The expected use is cash flowing. The deal closed on April 23, 2026 and was recorded on April 30, 2026. The property has 4,208 square feet of built space and 1,511 square feet of additional air rights for a total buildable of 5,713 square feet according to a PincusCo analysis of city data. The sale price per built square foot is $2,198 and the price per buildable square foot is $1,618 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) The seller bought the property on April 16, 2021, for $4.8 million. The signatory for RYCO Capital was James D. Ryan III. The signatory for James Rogers-Gahan was James Rogers-Gahan. The contract date was December 12, 2025. Prior sales, articles and revenue Prior to this transaction, PincusCo has no record that the buyer James R</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>Hikari Power Z Co. pays $15.2M to Kriss, Lockhill Properties for 20-unit walkup in Midtown East</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>https://www.pincusco.com/hikari-power-z-co-pays-15-2m-to-kriss-lockhill-properties-for-residential-walkup-in-midtown-east/</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>Hikari Power Z Co. through the entity Hikari Power Z Co., Ltd. paid $15.2 million</t>
-        </is>
-      </c>
-      <c r="D6" t="inlineStr"/>
-      <c r="E6" t="inlineStr"/>
-      <c r="F6" t="inlineStr">
-        <is>
-          <t>PincusCo</t>
-        </is>
-      </c>
-      <c r="G6" t="inlineStr">
-        <is>
-          <t>PincusCo - Home</t>
-        </is>
-      </c>
-      <c r="H6" t="inlineStr">
-        <is>
-          <t>Transfers 246 East 53rd Street (Credit - Cyclomedia) Hikari Power Z Co. through the entity Hikari Power Z Co., Ltd. paid $15.2 million to Jody Kriss and Lockhill Properties through the entity 246 E 53rd Owner LLC for the 20-unit residential walkup building (C7) at 246 East 53rd Street in Midtown East, Manhattan. The expected use is cash flowing. The deal closed on April 20, 2026 and was recorded on April 30, 2026. The property has 12,915 square feet of built space and 468 square feet of additional air rights for a total buildable of 13,388 square feet according to a PincusCo analysis of city data. The sale price per built square foot is $1,176 and the price per buildable square foot is $1,135 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) The sellers bought the property on February 14, 2025, for $8.1 million. The signatory for Jody Kriss and Lockhill Properties was Parke Leatherman and Jody Kriss. The signatory for Hikari Power Z Co. was Michael A. Mulia . The contract date was January 5, 2026. Prior sales, articles and revenue Prior to this trans</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>Gulf Coast Commercial pays $4M to Related Companies for mixed-use in Chelsea</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>https://www.pincusco.com/gulf-coast-commercial-pays-4m-to-related-companies-for-mixed-use-in-chelsea/</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>Florida-based Gulf Coast Commercial through the entity 559 West 22nd Development, LLC paid $4 million</t>
-        </is>
-      </c>
-      <c r="D7" t="inlineStr"/>
-      <c r="E7" t="inlineStr"/>
-      <c r="F7" t="inlineStr">
-        <is>
-          <t>PincusCo</t>
-        </is>
-      </c>
-      <c r="G7" t="inlineStr">
-        <is>
-          <t>PincusCo - Home</t>
-        </is>
-      </c>
-      <c r="H7" t="inlineStr">
-        <is>
-          <t>Transfers 162 11th Avenue (Credit - Cyclomedia) Florida-based Gulf Coast Commercial through the entity 559 West 22nd Development, LLC paid $4 million to Related Companies through the entity 22nd And 11th Associates, L.L.C. for the mixed-use building (K9) at 162 11th Avenue in Chelsea, Manhattan. The expected use is cash flowing. The deal closed on April 27, 2026 and was recorded on April 30, 2026. The property has 7,408 square feet of built space and 6,515 square feet of additional air rights for a total buildable of 13,919 square feet according to a PincusCo analysis of city data. The sale price per built square foot is $539 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) The seller bought the property on October 10, 2017, for $16.6 million. The signatory for Related Companies was Andrew Orchulli . The signatory for Gulf Coast Commercial was Philip J. McCabe . The contract date was February 27, 2026. Related utilized 6,538 square feet of the excess development rights for its apartment project at 555 West 22nd Street, in 2019. Prior sales, articles</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto update queens news 2026-05-04T14:28:24Z
</commit_message>
<xml_diff>
--- a/data/output/queens_dev_news.xlsx
+++ b/data/output/queens_dev_news.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H1"/>
+  <dimension ref="A1:H6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -467,6 +467,176 @@
       <c r="H1" s="1" t="inlineStr">
         <is>
           <t>content_preview</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Veeru Dhillon signs $10M refi with Spring Bank for hotel in Williamsburg</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>https://www.pincusco.com/veeru-dhillon-signs-10m-refi-with-spring-bank-for-hotel-in-williamsburg/</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Veeru Dhillon through the entity Union Hotel Park, LLC as borrower signed a refi loan</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr"/>
+      <c r="E2" t="inlineStr"/>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>PincusCo</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>PincusCo - Home</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>Transfers 437 Union Avenue (Credit - Cyclomedia) Veeru Dhillon through the entity Union Hotel Park, LLC as borrower signed a refi loan with lender Spring Bank through the entity Spring Bank valued at $10 million for the hotel building (H9) at 437 Union Avenue in Williamsburg, Brooklyn. The deal closed on February 12, 2026 and was recorded on May 1, 2026. The prior lender was Customers Bank which held debt that had an original loan amount of $10.7 million.The property has 18,046 square feet of built space according to a PincusCo analysis of city data. The loan price per built square foot is $554 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) The owner bought the property on September 15, 2010, for $253,000. The signatory for Veeru Dhillon was Veeru Dhillon. The signatory for Spring Bank was Akbar Rizvi . Prior sales, articles and revenue The 18,046-square-foot property generated revenue of $1.3 million or $75 per square foot, according to the most recent income and expense figures. The property</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>RSLT Capital Management pays $5.1M for mixed-use in Greenpoint</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>https://www.pincusco.com/rslt-capital-management-pays-5-1m-for-mixed-use-in-greenpoint/</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>RSLT Capital Management paid $5.1 million to Ezra Mashaal and Ron Obadiah for two mixed-use</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr"/>
+      <c r="E3" t="inlineStr"/>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>PincusCo</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>PincusCo - Home</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>Transfers 644 Manhattan Avenue (Credit - Cyclomedia) RSLT Capital Management paid $5.1 million to Ezra Mashaal and Ron Obadiah for two mixed-use buildings in Greenpoint, Brooklyn, in two transactions. In the first, RSLT Capital Management through the entity 644 Manhattan Owner LLC paid $2.7 million to Ezra Mashaal and Ron Obadiah through the entity 644 And 730 Manhattan Ave. E LLC for the mixed-use building (K2) at 644 Manhattan Avenue in Greenpoint, Brooklyn. The deal closed on April 15, 2026 and was recorded on May 1, 2026. The property has 3,608 square feet of built space and 3,900 square feet of additional air rights for a total buildable of 7,500 square feet according to a PincusCo analysis of city data. The sale price per built square foot is $748 and the price per buildable square foot is $360 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) The seller bought the property on July 20, 2016, for $3.4 million. In the second, RSLT Capital Management through the entity 730 Manhattan Owner LLC paid $2.4 million to Ezra Mashaal and Ron Obadiah throu</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Sovereign Partners, HudsonPoint sign $268M acquisition loan with Ladder for office, retail in Midtown East</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>https://www.pincusco.com/sovereign-partners-hudsonpoint-sign-268m-acquisition-loan-with-ladder-for-office-retail-in-midtown-east/</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Sovereign Partners and HudsonPoint Capital signed a $268 million acquisition loan package with Ladder Capital</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr"/>
+      <c r="E4" t="inlineStr"/>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>PincusCo</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>PincusCo - Home</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>Transfers 575 FIfth Avenue (Credit - Cyclomedia) Sovereign Partners and HudsonPoint Capital signed a $268 million acquisition loan package with Ladder Capital for office and retail at 575 Fifth Avenue in Midtown East, Manhattan in two transaction covering four commercial condominium tax lots. In the larger loan covering the office portion, Sovereign Partners and HudsonPoint Capital through the entity 575 5th Owners, LLC as borrower signed an acquisition loan with lender Ladder Capital through the entity Ladder Capital Finance LLC valued at $220 million for the office condo at 575 Fifth Avenue in Midtown East, Manhattan. The deal closed on April 16, 2026 and was recorded on May 1, 2026. The prior lender was TPG Real Estate Partners which held debt that had an original loan amount of $300.8 million. The property has 371,374 square feet of built space according to a PincusCo analysis of city data. The loan price per built square foot is $592 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) In the smaller loan covering the retail portion, Sovereign Part</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Joel Weiss, Isaac Silberstein pay $8.5M for 29-unit rental in Highbridge</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>https://www.pincusco.com/joel-weiss-isaac-silberstein-pay-8-5m-for-29-unit-rental-in-highbridge/</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Joel Weiss and Isaac Silberstein through the entity Edward Sunshine LLC paid $8.5 million to</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr"/>
+      <c r="E5" t="inlineStr"/>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>PincusCo</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>PincusCo - Home</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Transfers 1285 Edward L. Grant Highway (Credit - Cyclomedia) Joel Weiss and Isaac Silberstein through the entity Edward Sunshine LLC paid $8.5 million to Robert Kahen through the entity ELG Holdings LLC for the 29-unit residential elevator building (D1) at 1285 Edward L. Grant Highway in Highbridge, Bronx. The expected use is cash flowing. The deal closed on March 31, 2026 and was recorded on May 1, 2026. The property has 27,066 square feet of built space according to a PincusCo analysis of city data. The sale price per built square foot is $314 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) The signatory for Robert Kahen was Robert Kahen. The contract date was July 11, 2025. Prior sales, articles and revenue Prior to this transaction, PincusCo has records that the buyer Joel Weiss purchased seven properties in five transactions for a total of $17.4 million and sold two properties in two transactions for a total of $3.8 million over the past 24 months. The seller Robert Kahen purchased two properties in one transaction for a total of $2.7 million </t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Valon Pilku files plans for 3 buildings, 208 units in Crown Heights</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>https://www.pincusco.com/valon-pilku-files-plans-for-3-buildings-208-units-in-crown-heights/</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Valon Pilku filed plans for three buildings with a total of 208 units on a</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr"/>
+      <c r="E6" t="inlineStr"/>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>PincusCo</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>PincusCo - Home</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Development 971 Dean Street (Credit - Cyclomedia) Valon Pilku filed plans for three buildings with a total of 208 units on a single tax lot in Crown Heights, Brooklyn. In the largest project, Valon Pilku submitted a new building construction project for an 82-unit, 84,378 square-foot residential (R-2) building at 971 Dean Street in Crown Heights, Brooklyn. The plan was filed with the New York City Department of Buildings on April 29, 2026 under job number B01390326. It calls for the construction of a 11-story building. The project is described in the filing as: (please assign to dev hub, it should be assigned to same examiner as job b01390460-i1 and b01390458-i1 as its same zoning lot with same scope of work, applicant and owner) proposed new 11 story and cellar 82 unit mixed use building. The applicant is the Registered Architect Kao Hwa Lee of Kao Hwa Lee Architects Pc. In the second-largest project, Valon Pilku submitted a new building construction project for a 82-unit, 73,051-square-foot residential (R-2) building at 985 Dean Street in Crown Heights, Brooklyn. The plan was filed on April 29, 2026. It calls for the construction of a 119-foot-tall, eleven-story building and was </t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto update queens news 2026-05-05T14:23:13Z
</commit_message>
<xml_diff>
--- a/data/output/queens_dev_news.xlsx
+++ b/data/output/queens_dev_news.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H6"/>
+  <dimension ref="A1:H3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -473,17 +473,17 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Veeru Dhillon signs $10M refi with Spring Bank for hotel in Williamsburg</t>
+          <t>Peter Riguardi Jr. sells mixed-use in Williamsburg for $3.7M</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>https://www.pincusco.com/veeru-dhillon-signs-10m-refi-with-spring-bank-for-hotel-in-williamsburg/</t>
+          <t>https://www.pincusco.com/peter-riguardi-jr-sells-mixed-use-in-williamsburg-for-3-7m/</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Veeru Dhillon through the entity Union Hotel Park, LLC as borrower signed a refi loan</t>
+          <t>The anonymous entity 32 Richardson, LLC paid $3.7 million to Peter Riguardi Jr. for the</t>
         </is>
       </c>
       <c r="D2" t="inlineStr"/>
@@ -500,24 +500,24 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>Transfers 437 Union Avenue (Credit - Cyclomedia) Veeru Dhillon through the entity Union Hotel Park, LLC as borrower signed a refi loan with lender Spring Bank through the entity Spring Bank valued at $10 million for the hotel building (H9) at 437 Union Avenue in Williamsburg, Brooklyn. The deal closed on February 12, 2026 and was recorded on May 1, 2026. The prior lender was Customers Bank which held debt that had an original loan amount of $10.7 million.The property has 18,046 square feet of built space according to a PincusCo analysis of city data. The loan price per built square foot is $554 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) The owner bought the property on September 15, 2010, for $253,000. The signatory for Veeru Dhillon was Veeru Dhillon. The signatory for Spring Bank was Akbar Rizvi . Prior sales, articles and revenue The 18,046-square-foot property generated revenue of $1.3 million or $75 per square foot, according to the most recent income and expense figures. The property</t>
+          <t>Transfers 32 Richardson Street (Credit - Cyclomedia) The anonymous entity 32 Richardson, LLC paid $3.7 million to Peter Riguardi Jr. for the mixed-use building (K4) at 32 Richardson Street in Williamsburg, Brooklyn. The seller is the son of JLL Chairman Peter Riguardi. The deal closed on April 28, 2026 and was recorded on May 4, 2026. The property has 3,885 square feet of built space and 1,125 square feet of additional air rights for a total buildable of 5,000 square feet according to a PincusCo analysis of city data. The sale price per built square foot is $952 and the price per buildable square foot is $740 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) The seller bought the property on November 22, 2013, for $2.9 million. The signatory for Peter Riguardi Jr. was Peter Riguardi Jr.. The signatory for the buyer was M. Nader Ahari . The contract date was March 20, 2026. Prior sales, articles and revenue Prior to this transaction, PincusCo has no record that the buyer M. Nader Ahari registered had purchased any other properties and has no record it</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>RSLT Capital Management pays $5.1M for mixed-use in Greenpoint</t>
+          <t>Westbridge Realty Group files plans for 99 units in Washington Heights</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>https://www.pincusco.com/rslt-capital-management-pays-5-1m-for-mixed-use-in-greenpoint/</t>
+          <t>https://www.pincusco.com/westbridge-realty-group-files-plans-for-99-units-in-washington-heights/</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>RSLT Capital Management paid $5.1 million to Ezra Mashaal and Ron Obadiah for two mixed-use</t>
+          <t>Westbridge Realty Group submitted a new building construction project for a 99-unit, 67,048-square-foot residential (R-2)</t>
         </is>
       </c>
       <c r="D3" t="inlineStr"/>
@@ -534,109 +534,7 @@
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>Transfers 644 Manhattan Avenue (Credit - Cyclomedia) RSLT Capital Management paid $5.1 million to Ezra Mashaal and Ron Obadiah for two mixed-use buildings in Greenpoint, Brooklyn, in two transactions. In the first, RSLT Capital Management through the entity 644 Manhattan Owner LLC paid $2.7 million to Ezra Mashaal and Ron Obadiah through the entity 644 And 730 Manhattan Ave. E LLC for the mixed-use building (K2) at 644 Manhattan Avenue in Greenpoint, Brooklyn. The deal closed on April 15, 2026 and was recorded on May 1, 2026. The property has 3,608 square feet of built space and 3,900 square feet of additional air rights for a total buildable of 7,500 square feet according to a PincusCo analysis of city data. The sale price per built square foot is $748 and the price per buildable square foot is $360 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) The seller bought the property on July 20, 2016, for $3.4 million. In the second, RSLT Capital Management through the entity 730 Manhattan Owner LLC paid $2.4 million to Ezra Mashaal and Ron Obadiah throu</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>Sovereign Partners, HudsonPoint sign $268M acquisition loan with Ladder for office, retail in Midtown East</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>https://www.pincusco.com/sovereign-partners-hudsonpoint-sign-268m-acquisition-loan-with-ladder-for-office-retail-in-midtown-east/</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>Sovereign Partners and HudsonPoint Capital signed a $268 million acquisition loan package with Ladder Capital</t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr"/>
-      <c r="E4" t="inlineStr"/>
-      <c r="F4" t="inlineStr">
-        <is>
-          <t>PincusCo</t>
-        </is>
-      </c>
-      <c r="G4" t="inlineStr">
-        <is>
-          <t>PincusCo - Home</t>
-        </is>
-      </c>
-      <c r="H4" t="inlineStr">
-        <is>
-          <t>Transfers 575 FIfth Avenue (Credit - Cyclomedia) Sovereign Partners and HudsonPoint Capital signed a $268 million acquisition loan package with Ladder Capital for office and retail at 575 Fifth Avenue in Midtown East, Manhattan in two transaction covering four commercial condominium tax lots. In the larger loan covering the office portion, Sovereign Partners and HudsonPoint Capital through the entity 575 5th Owners, LLC as borrower signed an acquisition loan with lender Ladder Capital through the entity Ladder Capital Finance LLC valued at $220 million for the office condo at 575 Fifth Avenue in Midtown East, Manhattan. The deal closed on April 16, 2026 and was recorded on May 1, 2026. The prior lender was TPG Real Estate Partners which held debt that had an original loan amount of $300.8 million. The property has 371,374 square feet of built space according to a PincusCo analysis of city data. The loan price per built square foot is $592 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) In the smaller loan covering the retail portion, Sovereign Part</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>Joel Weiss, Isaac Silberstein pay $8.5M for 29-unit rental in Highbridge</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>https://www.pincusco.com/joel-weiss-isaac-silberstein-pay-8-5m-for-29-unit-rental-in-highbridge/</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>Joel Weiss and Isaac Silberstein through the entity Edward Sunshine LLC paid $8.5 million to</t>
-        </is>
-      </c>
-      <c r="D5" t="inlineStr"/>
-      <c r="E5" t="inlineStr"/>
-      <c r="F5" t="inlineStr">
-        <is>
-          <t>PincusCo</t>
-        </is>
-      </c>
-      <c r="G5" t="inlineStr">
-        <is>
-          <t>PincusCo - Home</t>
-        </is>
-      </c>
-      <c r="H5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Transfers 1285 Edward L. Grant Highway (Credit - Cyclomedia) Joel Weiss and Isaac Silberstein through the entity Edward Sunshine LLC paid $8.5 million to Robert Kahen through the entity ELG Holdings LLC for the 29-unit residential elevator building (D1) at 1285 Edward L. Grant Highway in Highbridge, Bronx. The expected use is cash flowing. The deal closed on March 31, 2026 and was recorded on May 1, 2026. The property has 27,066 square feet of built space according to a PincusCo analysis of city data. The sale price per built square foot is $314 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) The signatory for Robert Kahen was Robert Kahen. The contract date was July 11, 2025. Prior sales, articles and revenue Prior to this transaction, PincusCo has records that the buyer Joel Weiss purchased seven properties in five transactions for a total of $17.4 million and sold two properties in two transactions for a total of $3.8 million over the past 24 months. The seller Robert Kahen purchased two properties in one transaction for a total of $2.7 million </t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>Valon Pilku files plans for 3 buildings, 208 units in Crown Heights</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>https://www.pincusco.com/valon-pilku-files-plans-for-3-buildings-208-units-in-crown-heights/</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>Valon Pilku filed plans for three buildings with a total of 208 units on a</t>
-        </is>
-      </c>
-      <c r="D6" t="inlineStr"/>
-      <c r="E6" t="inlineStr"/>
-      <c r="F6" t="inlineStr">
-        <is>
-          <t>PincusCo</t>
-        </is>
-      </c>
-      <c r="G6" t="inlineStr">
-        <is>
-          <t>PincusCo - Home</t>
-        </is>
-      </c>
-      <c r="H6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Development 971 Dean Street (Credit - Cyclomedia) Valon Pilku filed plans for three buildings with a total of 208 units on a single tax lot in Crown Heights, Brooklyn. In the largest project, Valon Pilku submitted a new building construction project for an 82-unit, 84,378 square-foot residential (R-2) building at 971 Dean Street in Crown Heights, Brooklyn. The plan was filed with the New York City Department of Buildings on April 29, 2026 under job number B01390326. It calls for the construction of a 11-story building. The project is described in the filing as: (please assign to dev hub, it should be assigned to same examiner as job b01390460-i1 and b01390458-i1 as its same zoning lot with same scope of work, applicant and owner) proposed new 11 story and cellar 82 unit mixed use building. The applicant is the Registered Architect Kao Hwa Lee of Kao Hwa Lee Architects Pc. In the second-largest project, Valon Pilku submitted a new building construction project for a 82-unit, 73,051-square-foot residential (R-2) building at 985 Dean Street in Crown Heights, Brooklyn. The plan was filed on April 29, 2026. It calls for the construction of a 119-foot-tall, eleven-story building and was </t>
+          <t>Development 4388 Broadway rendering (Credit - Leandro Nils Dickson architect via DOB) Westbridge Realty Group submitted a new building construction project for a 99-unit, 67,048-square-foot residential (R-2) building at 4388 Broadway in Washington Heights, Manhattan. The plan was filed on April 28, 2026. It calls for the construction of a 150-foot-tall, sixteen-story building and was filed with the New York City Department of Buildings under job number M01393124. The project is described in the filing as: subject building is a sixteen-story building. The applicant is the Registered Architect Leandro Dickson of Leandro Nils Dickson Architect, LLC. Storage Post sold the development site on December 30, 2025, for $4.3 million to Steven Westreich‘s Westbridge Realty Group. 4388 Broadway The neighborhood</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto update queens news 2026-05-06T14:44:28Z
</commit_message>
<xml_diff>
--- a/data/output/queens_dev_news.xlsx
+++ b/data/output/queens_dev_news.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H3"/>
+  <dimension ref="A1:H4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -473,17 +473,17 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Peter Riguardi Jr. sells mixed-use in Williamsburg for $3.7M</t>
+          <t>Aron Stark closes on $13.58M purchase of dev site on Union Square East</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>https://www.pincusco.com/peter-riguardi-jr-sells-mixed-use-in-williamsburg-for-3-7m/</t>
+          <t>https://www.pincusco.com/aron-stark-closes-on-13-58m-purchase-of-dev-site-on-union-square-east/</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>The anonymous entity 32 Richardson, LLC paid $3.7 million to Peter Riguardi Jr. for the</t>
+          <t>Aron Stark paid $13.58 million to T30 Capital for the development site at 34 Union</t>
         </is>
       </c>
       <c r="D2" t="inlineStr"/>
@@ -500,24 +500,24 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>Transfers 32 Richardson Street (Credit - Cyclomedia) The anonymous entity 32 Richardson, LLC paid $3.7 million to Peter Riguardi Jr. for the mixed-use building (K4) at 32 Richardson Street in Williamsburg, Brooklyn. The seller is the son of JLL Chairman Peter Riguardi. The deal closed on April 28, 2026 and was recorded on May 4, 2026. The property has 3,885 square feet of built space and 1,125 square feet of additional air rights for a total buildable of 5,000 square feet according to a PincusCo analysis of city data. The sale price per built square foot is $952 and the price per buildable square foot is $740 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) The seller bought the property on November 22, 2013, for $2.9 million. The signatory for Peter Riguardi Jr. was Peter Riguardi Jr.. The signatory for the buyer was M. Nader Ahari . The contract date was March 20, 2026. Prior sales, articles and revenue Prior to this transaction, PincusCo has no record that the buyer M. Nader Ahari registered had purchased any other properties and has no record it</t>
+          <t>Transfers 34 Union Square East (Credit - Cyclomedia) Aron Stark paid $13.58 million to T30 Capital for the development site at 34 Union Square East in Manhattan, in a sale that closed on May 1, 2026, after going into contract in October 2025, according to person familiar with the transaction. As of publication, the sale had not yet been recorded in city records. The Real Deal reported on the transaction when it went into contract. After going into contract but before closing, Aron Stark submitted a new building construction project for a 29-unit, 30,946 square-foot residential (R-2) building at 34 Union Square East, filed under the alternate name 100 East 16th Street. The plan was filed on March 9, 2026. It calls for the construction of a 124-foot tall, 12-story building and was filed with the New York City Department of Buildings under job number M01364168. The architect is Kao Hwa Lee Architects PC. The project is described in the filing as: proposed new 12-story and cellar 29-unit mixed-use building. Aron Stark is the younger cousin of another real estate investor with the same name. Shay Zach of GAIA Property Group and Alexandra Marolda of Avison Young brokered the sale.</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Westbridge Realty Group files plans for 99 units in Washington Heights</t>
+          <t>ZD Jasper seeks zoning change to build 143 units in Sunnyside</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>https://www.pincusco.com/westbridge-realty-group-files-plans-for-99-units-in-washington-heights/</t>
+          <t>https://www.pincusco.com/zd-jasper-seeks-zoning-change-to-build-143-units-in-sunnyside/</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Westbridge Realty Group submitted a new building construction project for a 99-unit, 67,048-square-foot residential (R-2)</t>
+          <t>ZD Jasper Realty through the entity ZDJ Greenpoint LLC submitted a proposal to the city</t>
         </is>
       </c>
       <c r="D3" t="inlineStr"/>
@@ -534,7 +534,41 @@
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>Development 4388 Broadway rendering (Credit - Leandro Nils Dickson architect via DOB) Westbridge Realty Group submitted a new building construction project for a 99-unit, 67,048-square-foot residential (R-2) building at 4388 Broadway in Washington Heights, Manhattan. The plan was filed on April 28, 2026. It calls for the construction of a 150-foot-tall, sixteen-story building and was filed with the New York City Department of Buildings under job number M01393124. The project is described in the filing as: subject building is a sixteen-story building. The applicant is the Registered Architect Leandro Dickson of Leandro Nils Dickson Architect, LLC. Storage Post sold the development site on December 30, 2025, for $4.3 million to Steven Westreich‘s Westbridge Realty Group. 4388 Broadway The neighborhood</t>
+          <t>Chart_Frontpage Development Top Story 44-17 Greenpoint Avenue (Credit - Cyclomedia) ZD Jasper Realty through the entity ZDJ Greenpoint LLC submitted a proposal to the city for the construction of a 143-unit, 142,593-square-foot, 11-story, mixed-use development at 44-17 Greenpoint Avenue in Sunnyside, Queens. The parcel is the former Queens Assembly Hall for the Jehovah’s Witnesses, who sold the parcel to ZD Jasper Realty in 2024 for $16.3 million. Jasper Wu of ZD Jasper Realty, which was founded by Zhidong Wu, filed the plans with the city’s Department of City Planning yesterday seeking the zoning and Mandatory Inclusionary Housing changes through a Uniform Land Use Review Procedure (ULURP) application.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Yoel Teitelbaum signs contract to buy gas station in Crown Heights for undisclosed amount</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>https://www.pincusco.com/yoel-teitelbaum-signs-contract-to-buy-gas-station-in-crown-heights-for-undisclosed-amount/</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Yoel Teitelbaum through the entity 1062 Atlantic Avenue LLC signed a contract as buyer with</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr"/>
+      <c r="E4" t="inlineStr"/>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>PincusCo</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>PincusCo - Home</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>Transfers 1062 Atlantic Avenue (Credit - Cyclomedia) Yoel Teitelbaum through the entity 1062 Atlantic Avenue LLC signed a contract as buyer with Esther Zernitsky through the entity Manny Enterprises LLC as seller for the industrial building (G4) at 1062 Atlantic Avenue in Crown Heights, Brooklyn. The sale price was not disclosed but Teitelbaum has made a $400,000 deposit. The memorandum of contract says the closing it set for no later than September 19, 2026. The memorandum of contract was signed on September 19, 2024 and was recorded on May 4, 2026. The property has 2,184 square feet of built space and 4,850 square feet of additional air rights for a total buildable of 7,029 square feet according to a PincusCo analysis of city data. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) The signatory for Esther Zernitsky was Esther Zernitsky. The signatory for Yoel Teitelbaum was Yoel Teitelbaum. Prior sales, articles and revenue Prior to this transaction, PincusCo has no record that the buyer Yoel Teitelbaum had purchased any other properties and has no record it sold any propert</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto update queens news 2026-05-07T14:47:21Z
</commit_message>
<xml_diff>
--- a/data/output/queens_dev_news.xlsx
+++ b/data/output/queens_dev_news.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H4"/>
+  <dimension ref="A1:H11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -473,54 +473,66 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Aron Stark closes on $13.58M purchase of dev site on Union Square East</t>
+          <t>Permits Filed for 16-77 George Street in Ridgewood, Queens</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>https://www.pincusco.com/aron-stark-closes-on-13-58m-purchase-of-dev-site-on-union-square-east/</t>
+          <t>https://newyorkyimby.com/2026/05/permits-filed-for-16-77-george-street-in-ridgewood-queens.html</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Aron Stark paid $13.58 million to T30 Capital for the development site at 34 Union</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr"/>
-      <c r="E2" t="inlineStr"/>
+          <t>Permits have been filed for a single-story house of worship building at 16-77 George Street in &lt;a href="https://newyorkyimby.com/neighborhoods/Ridgewood"&gt;Ridgewood&lt;/a&gt;, Queens. Located between Wyckoff Avenue and Cypress Avenue, the lot is near the Halsey Street subway station, served by the L train. Jason Rivera under the CONSTRUCTIONLAB LLC is listed as the owner behind the applications.</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>2026-05-07T10:30:19+00:00</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>Thu, 07 May 2026 10:30:19 +0000</t>
+        </is>
+      </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>PincusCo</t>
+          <t>YIMBY</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>PincusCo - Home</t>
+          <t>YIMBY - Ridgewood</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>Transfers 34 Union Square East (Credit - Cyclomedia) Aron Stark paid $13.58 million to T30 Capital for the development site at 34 Union Square East in Manhattan, in a sale that closed on May 1, 2026, after going into contract in October 2025, according to person familiar with the transaction. As of publication, the sale had not yet been recorded in city records. The Real Deal reported on the transaction when it went into contract. After going into contract but before closing, Aron Stark submitted a new building construction project for a 29-unit, 30,946 square-foot residential (R-2) building at 34 Union Square East, filed under the alternate name 100 East 16th Street. The plan was filed on March 9, 2026. It calls for the construction of a 124-foot tall, 12-story building and was filed with the New York City Department of Buildings under job number M01364168. The architect is Kao Hwa Lee Architects PC. The project is described in the filing as: proposed new 12-story and cellar 29-unit mixed-use building. Aron Stark is the younger cousin of another real estate investor with the same name. Shay Zach of GAIA Property Group and Alexandra Marolda of Avison Young brokered the sale.</t>
+          <t>By: Vanessa Londono 6:30 am on May 7, 2026 Permits have been filed for a single-story house of worship at 16-77 George Street in Ridgewood, Queens. Located between Wyckoff Avenue and Cypress Avenue, the lot is near the Halsey Street subway station, served by the L train. Jason Rivera under the CONSTRUCTIONLAB LLC is listed as the owner behind the applications. The proposed 45-foot-tall development will yield 13,597 square feet, with 9,479 square feet designated for community facility space. The steel-based structure will also have four enclosed parking spaces. Sherif Abdel-Meseh of Urban Design Engineering is listed as the architect of record. Demolition permits were filed last month for the gas station that was previously on the site. An estimated completion date has not been announced. Subscribe to YIMBY’s daily e-mail Follow YIMBYgram for real-time photo updates Like YIMBY on Facebook Follow YIMBY’s Twitter for the latest in YIMBYnews</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>ZD Jasper seeks zoning change to build 143 units in Sunnyside</t>
+          <t>SL Property Group pays $7.8M to MNM Properties for 20-unit UWS walkup</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>https://www.pincusco.com/zd-jasper-seeks-zoning-change-to-build-143-units-in-sunnyside/</t>
+          <t>https://www.pincusco.com/sl-property-group-pays-7-8m-to-mnm-properties-for-20-unit-uws-walkup/</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>ZD Jasper Realty through the entity ZDJ Greenpoint LLC submitted a proposal to the city</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr"/>
+          <t>SL Property Group through the entity 430 Ams Owner LLC paid $7.8 million to MNM</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>NaT</t>
+        </is>
+      </c>
       <c r="E3" t="inlineStr"/>
       <c r="F3" t="inlineStr">
         <is>
@@ -534,27 +546,31 @@
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>Chart_Frontpage Development Top Story 44-17 Greenpoint Avenue (Credit - Cyclomedia) ZD Jasper Realty through the entity ZDJ Greenpoint LLC submitted a proposal to the city for the construction of a 143-unit, 142,593-square-foot, 11-story, mixed-use development at 44-17 Greenpoint Avenue in Sunnyside, Queens. The parcel is the former Queens Assembly Hall for the Jehovah’s Witnesses, who sold the parcel to ZD Jasper Realty in 2024 for $16.3 million. Jasper Wu of ZD Jasper Realty, which was founded by Zhidong Wu, filed the plans with the city’s Department of City Planning yesterday seeking the zoning and Mandatory Inclusionary Housing changes through a Uniform Land Use Review Procedure (ULURP) application.</t>
+          <t>Transfers 430 Amsterdam Avenue (Credit - Cyclomedia) SL Property Group through the entity 430 Ams Owner LLC paid $7.8 million to MNM Properties through the entity 430 Amsterdam Partners LLC for the 20-unit residential walkup building (C7) at 430 Amsterdam Avenue in Upper West Side, Manhattan. The expected use is cash flowing. The deal closed on April 30, 2026 and was recorded on May 5, 2026. The property has 13,945 square feet of built space and 7,859 square feet of additional air rights for a total buildable of 21,808 square feet according to a PincusCo analysis of city data. The sale price per built square foot is $561 and the price per buildable square foot is $358 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) The seller bought the property on July 30, 2004, for $4 million. The signatory for MNM Properties was Mitchell Banchik and Theodore Lanzi. The signatory for SL Property Group was Sean Lefkovits . The contract date was January 14, 2026. Prior sales, articles and revenue Prior to this transaction, PincusCo has records that the buyer SL Pro</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Yoel Teitelbaum signs contract to buy gas station in Crown Heights for undisclosed amount</t>
+          <t>Alf Naman Real Estate pays $10M to Regal Ventures for retail in NoMad</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>https://www.pincusco.com/yoel-teitelbaum-signs-contract-to-buy-gas-station-in-crown-heights-for-undisclosed-amount/</t>
+          <t>https://www.pincusco.com/alf-naman-real-estate-pays-10m-to-regal-ventures-for-retail-in-nomad/</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Yoel Teitelbaum through the entity 1062 Atlantic Avenue LLC signed a contract as buyer with</t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr"/>
+          <t>Alf Naman Real Estate through the entity 36 Owners LLC paid $10 million to Regal</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>NaT</t>
+        </is>
+      </c>
       <c r="E4" t="inlineStr"/>
       <c r="F4" t="inlineStr">
         <is>
@@ -568,7 +584,273 @@
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>Transfers 1062 Atlantic Avenue (Credit - Cyclomedia) Yoel Teitelbaum through the entity 1062 Atlantic Avenue LLC signed a contract as buyer with Esther Zernitsky through the entity Manny Enterprises LLC as seller for the industrial building (G4) at 1062 Atlantic Avenue in Crown Heights, Brooklyn. The sale price was not disclosed but Teitelbaum has made a $400,000 deposit. The memorandum of contract says the closing it set for no later than September 19, 2026. The memorandum of contract was signed on September 19, 2024 and was recorded on May 4, 2026. The property has 2,184 square feet of built space and 4,850 square feet of additional air rights for a total buildable of 7,029 square feet according to a PincusCo analysis of city data. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) The signatory for Esther Zernitsky was Esther Zernitsky. The signatory for Yoel Teitelbaum was Yoel Teitelbaum. Prior sales, articles and revenue Prior to this transaction, PincusCo has no record that the buyer Yoel Teitelbaum had purchased any other properties and has no record it sold any propert</t>
+          <t>Transfers 36 West 28th Street (Credit - Cyclomedia) Alf Naman Real Estate through the entity 36 Owners LLC paid $10 million to Regal Ventures through the entity 36 West Associates LLC for the retail building (K1) at 36 West 28th Street in NoMad, Manhattan. PincusCo expects the use is ground up development, however Alf Naman declined to comment. The deal closed on April 30, 2026 and was recorded on May 5, 2026. The property has 3,216 square feet of built space and 21,506 square feet of additional air rights for a total buildable of 24,720 square feet according to a PincusCo analysis of city data. The sale price per built square foot is $3,109 and the price per buildable square foot is $404 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) The seller bought the property on August 16, 2012, for $5 million. The signatory for Regal Ventures was Elyahu Cohen . The signatory for Alf Naman Real Estate was Jesse H. Young . The contract date was March 31, 2025. Prior sales, articles and revenue Prior to this transaction, PincusCo has records that the buyer Alf</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Jeff Sutton’s Wharton Properties pays $5.2M for mixed-use retail in Brighton Beach</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>https://www.pincusco.com/jeff-suttons-wharton-properties-pays-5-2m-for-two-mixed-use-properties-in-brighton-beach/</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Jeff Sutton’s Wharton Properties through the entity 614-616 Bright Beach LLC paid $5.2 million to</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>NaT</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr"/>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>PincusCo</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>PincusCo - Home</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>Transfers 614-616 Brighton Beach Avenue (Credit - Cyclomedia) Jeff Sutton’s Wharton Properties through the entity 614-616 Bright Beach LLC paid $5.2 million to Seth Rubinstein and Ira Rubinstein through the entity SIR Realty Corp. for the two-unit mixed-use building (S2) at 614 Brighton Beach Avenue in Brighton Beach, Brooklyn and the adjacent two-unit mixed-use building (S2) at 616 Brighton Beach Avenue. The expected use is cash flowing. Wharton Properties controls two buildings on the other side of the street a block to the west at 517-519 Brighton Beach Avenue through a 30-year net lease expiring in 2038. The deal closed on April 28, 2026 and was recorded on May 5, 2026. The two properties have 8,398 square feet of built space and 198 square feet of additional air rights for a total buildable of 8,434 square feet according to a PincusCo analysis of city data. The sale price per built square foot is $619 and the price per buildable square foot is $616 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) The signatory for Seth Rubinstein and Ira Rubins</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Lightstone Group signs $17.6M refi with JLL for 46-unit UWS rental</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>https://www.pincusco.com/lightstone-group-signs-17-6m-refi-with-jll-for-46-unit-uws-rental/</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Lightstone Group through the entity 309 West 99th Street Associates LLC as borrower signed a</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>NaT</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr"/>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>PincusCo</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>PincusCo - Home</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>Transfers 305 West 99th Street (Credit - Cyclomedia) Lightstone Group through the entity 309 West 99th Street Associates LLC as borrower signed a refi loan with lender JLL through the entity JLL Real Estate Capital, LLC valued at $17.6 million for the 46-unit residential elevator building (D3) at 305 West 99th Street in Upper West Side, Manhattan. The deal closed on April 20, 2026 and was recorded on May 5, 2026. The prior lenders were members of the Einy family which held debt that had an original loan amount of $10 million. The property has 48,099 square feet of built space according to a PincusCo analysis of city data. The loan price per built square foot is $365 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) The owner bought the property on May 19, 2020, for $18.5 million. The signatory for Lightstone Group was Joseph E. Teichman . The signatory for JLL was Omar Lopez . Prior sales, articles and revenue The owners according to the Department of Housing Preservation and Development includes Meir Milgraum, head officer and Jacob Eisenstein, agen</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Joel Schwartz signs $23M refi with Ponce for new 48-unit rental in Cypress Hills</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>https://www.pincusco.com/joel-schwartz-signs-23m-refi-with-ponce-bank-for-newly-built-48-unit-rental-in-cypress-hills/</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Joel Schwartz through the entity 3051 Atlantic Bx LLC as borrower signed a refi loan</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>NaT</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr"/>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>PincusCo</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>PincusCo - Home</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>Transfers 3051 Atlantic Avenue (Credit - Cyclomedia) Joel Schwartz through the entity 3051 Atlantic Bx LLC as borrower signed a refi loan with lender Ponce Bank valued at $23 million for the 48-unit residential elevator building (D7) at 3051 Atlantic Avenue in Cypress Hills, Brooklyn. The deal closed on April 27, 2026 and was recorded on May 5, 2026. The prior lender was Yakar Partners which held debt that had an original loan amount of $17.5 million. The property has 38,688 square feet of built space according to a PincusCo analysis of city data. The loan price per built square foot is $594 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) The owner bought the property on March 31, 2023, for $2.1 million. The signatory for Joel Schwartz was Joel Schwartz. The signatory for Ponce Bank was Steven A. Tsavaris . Prior sales, articles and revenue The owner according to the Department of Housing Preservation and Development is Charles Schwartz, head officer. The business entity is 3051 Atlantic Bx Llc. The property</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Maheshchand Ratanji signs $23M construction loan for hotel project in Flatbush</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>https://www.pincusco.com/maheshchand-ratanji-signs-23m-construction-loan-for-hotel-project-in-flatbush/</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Maheshchand M. Ratanji through the entity 1045 Flatbush Avenue LLC as borrower signed a construction</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>NaT</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr"/>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>PincusCo</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>PincusCo - Home</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Transfers 1041 Flatbush Avenue (Credit - Cyclomedia) Maheshchand M. Ratanji through the entity 1045 Flatbush Avenue LLC as borrower signed a construction loan with lender State Bank of Texas valued at $23 million for the hotel development site (V1) at 1041 Flatbush Avenue in Flatbush, Brooklyn. On the lot, there is one active new building construction project, 340795483, for a 150-unit, 59,290 square-foot hotel (R-1) building. The project was submitted by Maheshchand Ratanji and filed by Nehalkumar Gandhi with plans filed December 10, 2020 and permitted October 7, 2024. The deal closed on April 22, 2026 and was recorded on May 5, 2026. The prior lender was State Bank of Texas which held debt that had an original loan amount of $4.3 million. The price per planned development square foot is $388 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) The owner bought the property on July 29, 2019, for $8.8 million. The signatory for Maheshchand M. Ratanji was Maheshchand M. Ratanji. The signatory for State Bank of Texas was Melody Collins . The property The </t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>EDRE Development pays $8.2M for 8-unit walkup in Williamsburg</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>https://www.pincusco.com/edre-development-pays-8-2m-for-8-unit-walkup-in-williamsburg/</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>EDRE Development through the entity 35 South 3rd Owner, LLC paid $8.2 million to John</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>NaT</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr"/>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>PincusCo</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>PincusCo - Home</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>Transfers 37 South 3rd Street (Credit - Cyclomedia) EDRE Development through the entity 35 South 3rd Owner, LLC paid $8.2 million to John McNulty through the entity Southside Restoration Corp. for the eight-unit residential walkup building (C7) at 37 South 3rd Street in Williamsburg, Brooklyn. The deal closed on April 27, 2026 and was recorded on May 6, 2026. The property has 12,172 square feet of built space and 7,373 square feet of additional air rights for a total buildable of 19,575 square feet according to a PincusCo analysis of city data. The sale price per built square foot is $677 and the price per buildable square foot is $421 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) The signatory for John McNulty was John McNulty. The signatory for EDRE Development was Harel Edery . The contract date was August 13, 2025. To finance the purchase, EDRE Development borrowed $6.2 million from S3 Capital. Prior sales, articles and revenue Prior to this transaction, PincusCo has records that the buyer EDRE Development purchased one property in one transa</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Psychotherapy and counseling nonprofit pays $3.5M for parking lot in Melrose</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>https://www.pincusco.com/new-york-psychotherapy-pays-3-5m-for-parking-lot-in-melrose/</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>The nonprofit New York Psychotherapy and Counseling Center paid $3.5 million to the entity 622</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>NaT</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr"/>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>PincusCo</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>PincusCo - Home</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>Transfers 622 Courtlandt Avenue (Credit - Cyclomedia) The nonprofit New York Psychotherapy and Counseling Center paid $3.5 million to the entity 622 Courtlandt LLC for a three-parcel parking lot (G6) at 616, 620 and 622 Courtlandt Avenue in Melrose, Bronx. The expected use is owner-occupied. The New York Psychotherapy and Counseling Center has a large office building a block away at 579 Courtlandt Avenue. The deal closed on April 23, 2026 and was recorded on May 6, 2026. The three properties have zero square feet of built space and 31,138 square feet of additional air rights for a total buildable of 31,138 square feet according to a PincusCo analysis of city data. The sale price per buildable square foot is $110 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) The signatories for the sellers Amarendra Deshmukh and Jyotsna Deshmukh were Amarendra Deshmukh and Jyotsna Deshmukh. The signatory for New York Psychotherapy and Counseling Center was Elliot Klein . The contract date was April 23, 2026. David Simone of Concourse Realty Partners brokered the s</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Lotte pays $491.1M to Archdiocese of NY for three properties in Midtown East</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>https://www.pincusco.com/lotte-pays-491-1m-to-archdiocese-of-ny-for-three-properties-in-midtown-east/</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Lotte Corporation through the entity Lotte Hotel New York Palace, LLC paid $491.1 million through</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>NaT</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr"/>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>PincusCo</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>PincusCo - Home</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>Transfers 455 Madison Avenue (Credit - Cyclomedia) Lotte Corporation through the entity Lotte Hotel New York Palace, LLC paid $491.1 million through a ground leased fee to Archdiocese of New York and Roman Catholic Church through the entity The Archdiocese Of New York for the hotel building (H1) at 455 Madison Avenue in Midtown East, Manhattan, retail building (O5) at 457 Madison Avenue in Midtown East, Manhattan, and retail building (K2) at 35 East 50th Street in Midtown East, Manhattan. The expected use is cash flowing. The deal closed on April 30, 2026 and was recorded on May 6, 2026. The three properties have 866,090 square feet of built space and 56,256 square feet of additional air rights according to a PincusCo analysis of city data. The sale price per built square foot is $567 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) The signatory for Archdiocese of New York and Roman Catholic Church was John Cahill . The signatory for Lotte Corporation was Jihong Lee . The contract date was November 12, 2025. PincusCo reported on this transaction in</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto update queens news 2026-05-08T14:14:27Z
</commit_message>
<xml_diff>
--- a/data/output/queens_dev_news.xlsx
+++ b/data/output/queens_dev_news.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H11"/>
+  <dimension ref="A1:H6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -473,66 +473,54 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Permits Filed for 16-77 George Street in Ridgewood, Queens</t>
+          <t>World Wide Group signs $34.5M refi with MetLife for 124-unit LIC rental</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>https://newyorkyimby.com/2026/05/permits-filed-for-16-77-george-street-in-ridgewood-queens.html</t>
+          <t>https://www.pincusco.com/world-wide-group-signs-34-5m-refi-with-metlife-for-124-unit-lic-rental/</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Permits have been filed for a single-story house of worship building at 16-77 George Street in &lt;a href="https://newyorkyimby.com/neighborhoods/Ridgewood"&gt;Ridgewood&lt;/a&gt;, Queens. Located between Wyckoff Avenue and Cypress Avenue, the lot is near the Halsey Street subway station, served by the L train. Jason Rivera under the CONSTRUCTIONLAB LLC is listed as the owner behind the applications.</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>2026-05-07T10:30:19+00:00</t>
-        </is>
-      </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>Thu, 07 May 2026 10:30:19 +0000</t>
-        </is>
-      </c>
+          <t>World Wide Group through the entity WWG Crescent 2 LLC as borrower signed a refi</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr"/>
+      <c r="E2" t="inlineStr"/>
       <c r="F2" t="inlineStr">
         <is>
-          <t>YIMBY</t>
+          <t>PincusCo</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>YIMBY - Ridgewood</t>
+          <t>PincusCo - Home</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>By: Vanessa Londono 6:30 am on May 7, 2026 Permits have been filed for a single-story house of worship at 16-77 George Street in Ridgewood, Queens. Located between Wyckoff Avenue and Cypress Avenue, the lot is near the Halsey Street subway station, served by the L train. Jason Rivera under the CONSTRUCTIONLAB LLC is listed as the owner behind the applications. The proposed 45-foot-tall development will yield 13,597 square feet, with 9,479 square feet designated for community facility space. The steel-based structure will also have four enclosed parking spaces. Sherif Abdel-Meseh of Urban Design Engineering is listed as the architect of record. Demolition permits were filed last month for the gas station that was previously on the site. An estimated completion date has not been announced. Subscribe to YIMBY’s daily e-mail Follow YIMBYgram for real-time photo updates Like YIMBY on Facebook Follow YIMBY’s Twitter for the latest in YIMBYnews</t>
+          <t>Transfers 42-15 Crescent Street (Credit - Cyclomedia) World Wide Group through the entity WWG Crescent 2 LLC as borrower signed a refi loan with lender MetLife through the entity Metlife Real Estate Lending LLC valued at $34.5 million for the 124-unit residential elevator building (D7) at 42-15 Crescent Street in Long Island City, Queens. The deal closed on April 24, 2026 and was recorded on May 6, 2026. The prior lender was Helaba which held debt that had an original loan amount of $32 million. The property has 110,743 square feet of built space according to a PincusCo analysis of city data. The loan price per built square foot is $311 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) The owner bought the property on March 17, 2016, for $70 million. The signatory for World Wide Group was Jodi Gerstman . The signatory for MetLife was Brett Ulrich . Prior sales, articles and revenue The owners according to the Department of Housing Preservation and Development includes Jodi Gerstman, head officer and Neal Cohen, officer. The business entities are Rose</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>SL Property Group pays $7.8M to MNM Properties for 20-unit UWS walkup</t>
+          <t>Ekstein Development signs $58M refi with MetLife for new 107-unit rental in Bushwick</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>https://www.pincusco.com/sl-property-group-pays-7-8m-to-mnm-properties-for-20-unit-uws-walkup/</t>
+          <t>https://www.pincusco.com/ekstein-development-signs-58m-refi-with-metlife-for-new-107-unit-rental-in-bushwick/</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>SL Property Group through the entity 430 Ams Owner LLC paid $7.8 million to MNM</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>NaT</t>
-        </is>
-      </c>
+          <t>Ekstein Development Group through the entity 1333 Broadway LLC as borrower signed a refi loan</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr"/>
       <c r="E3" t="inlineStr"/>
       <c r="F3" t="inlineStr">
         <is>
@@ -546,31 +534,27 @@
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>Transfers 430 Amsterdam Avenue (Credit - Cyclomedia) SL Property Group through the entity 430 Ams Owner LLC paid $7.8 million to MNM Properties through the entity 430 Amsterdam Partners LLC for the 20-unit residential walkup building (C7) at 430 Amsterdam Avenue in Upper West Side, Manhattan. The expected use is cash flowing. The deal closed on April 30, 2026 and was recorded on May 5, 2026. The property has 13,945 square feet of built space and 7,859 square feet of additional air rights for a total buildable of 21,808 square feet according to a PincusCo analysis of city data. The sale price per built square foot is $561 and the price per buildable square foot is $358 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) The seller bought the property on July 30, 2004, for $4 million. The signatory for MNM Properties was Mitchell Banchik and Theodore Lanzi. The signatory for SL Property Group was Sean Lefkovits . The contract date was January 14, 2026. Prior sales, articles and revenue Prior to this transaction, PincusCo has records that the buyer SL Pro</t>
+          <t>Transfers 1333 Broadway (Credit - Cyclomedia) Ekstein Development Group through the entity 1333 Broadway LLC as borrower signed a refi loan with lender MetLife through the entity Metropolitan Tower Life Insurance Company valued at $58 million for the 107-unit residential elevator building (D7) at 1333 Broadway in Bushwick, Brooklyn. The deal closed on April 24, 2026 and was recorded on May 6, 2026. The prior lender was Santander Bank which held debt that had an original loan amount of $48.8 million. The property has 120,403 square feet of built space according to a PincusCo analysis of city data. The loan price per built square foot is $481 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) The owner bought the property on December 6, 2019, for $16.7 million. The signatory for Ekstein Development Group was Erik Ekstein . The signatory for MetLife was Anthony Soldi . Prior sales, articles and revenue The 120,403-square-foot property generated revenue of $3.8 million or $31 per square foot, according to the most recent income and expense figures.</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Alf Naman Real Estate pays $10M to Regal Ventures for retail in NoMad</t>
+          <t>United Construction, New Land Capital sign $18.5M construction loan for 48-unit project in Flushing</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>https://www.pincusco.com/alf-naman-real-estate-pays-10m-to-regal-ventures-for-retail-in-nomad/</t>
+          <t>https://www.pincusco.com/united-construction-new-land-capital-sign-18-5m-construction-loan-with-preferred-bank-for-in-flushing/</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Alf Naman Real Estate through the entity 36 Owners LLC paid $10 million to Regal</t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>NaT</t>
-        </is>
-      </c>
+          <t>United Construction &amp; Development Group and New Land Capital through the entity 32nd Ave Holding</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr"/>
       <c r="E4" t="inlineStr"/>
       <c r="F4" t="inlineStr">
         <is>
@@ -584,31 +568,27 @@
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>Transfers 36 West 28th Street (Credit - Cyclomedia) Alf Naman Real Estate through the entity 36 Owners LLC paid $10 million to Regal Ventures through the entity 36 West Associates LLC for the retail building (K1) at 36 West 28th Street in NoMad, Manhattan. PincusCo expects the use is ground up development, however Alf Naman declined to comment. The deal closed on April 30, 2026 and was recorded on May 5, 2026. The property has 3,216 square feet of built space and 21,506 square feet of additional air rights for a total buildable of 24,720 square feet according to a PincusCo analysis of city data. The sale price per built square foot is $3,109 and the price per buildable square foot is $404 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) The seller bought the property on August 16, 2012, for $5 million. The signatory for Regal Ventures was Elyahu Cohen . The signatory for Alf Naman Real Estate was Jesse H. Young . The contract date was March 31, 2025. Prior sales, articles and revenue Prior to this transaction, PincusCo has records that the buyer Alf</t>
+          <t>Transfers 141-05 32nd Avenue axonometric diagram (Credit - Ning Lu architect via DOB) United Construction &amp; Development Group and New Land Capital through the entity 32nd Ave Holding LLC as borrower signed a new construction loan with lender Preferred Bank valued at $18.5 million for the property at 141-05 32nd Avenue in Flushing, Queens. On the lot, there is one active new building construction project, Q00983687, for a 48-unit, 36,927 square-foot residential (R-2) building. The project was submitted by United Construction &amp; Development Group and filed by Jiashu Xu with plans filed February 13, 2024 and permitted February 18, 2025. The deal closed on April 21, 2026 and was recorded on May 6, 2026. The loan price per planned development square foot is $501 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) The signatory for United Construction &amp; Development Group and New Land Capital was Hangyuan Zhang . Violations and lawsuits</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Jeff Sutton’s Wharton Properties pays $5.2M for mixed-use retail in Brighton Beach</t>
+          <t>United Construction &amp; Development signs $17.9M construction loan for 47-unit project in Flushing</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>https://www.pincusco.com/jeff-suttons-wharton-properties-pays-5-2m-for-two-mixed-use-properties-in-brighton-beach/</t>
+          <t>https://www.pincusco.com/united-construction-development-signs-17-9m-construction-loan-for-47-unit-project-in-flushing/</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Jeff Sutton’s Wharton Properties through the entity 614-616 Bright Beach LLC paid $5.2 million to</t>
-        </is>
-      </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>NaT</t>
-        </is>
-      </c>
+          <t>United Construction &amp; Development Group through the entity 32nd Ave Management LLC as borrower signed</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr"/>
       <c r="E5" t="inlineStr"/>
       <c r="F5" t="inlineStr">
         <is>
@@ -622,31 +602,27 @@
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>Transfers 614-616 Brighton Beach Avenue (Credit - Cyclomedia) Jeff Sutton’s Wharton Properties through the entity 614-616 Bright Beach LLC paid $5.2 million to Seth Rubinstein and Ira Rubinstein through the entity SIR Realty Corp. for the two-unit mixed-use building (S2) at 614 Brighton Beach Avenue in Brighton Beach, Brooklyn and the adjacent two-unit mixed-use building (S2) at 616 Brighton Beach Avenue. The expected use is cash flowing. Wharton Properties controls two buildings on the other side of the street a block to the west at 517-519 Brighton Beach Avenue through a 30-year net lease expiring in 2038. The deal closed on April 28, 2026 and was recorded on May 5, 2026. The two properties have 8,398 square feet of built space and 198 square feet of additional air rights for a total buildable of 8,434 square feet according to a PincusCo analysis of city data. The sale price per built square foot is $619 and the price per buildable square foot is $616 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) The signatory for Seth Rubinstein and Ira Rubins</t>
+          <t>Transfers 140-28 31st Drive axonometric diagram (Credit - Ning Lu architect via DOB) United Construction &amp; Development Group through the entity 32nd Ave Management LLC as borrower signed a new construction loan with lender Preferred Bank valued at $17.9 million for the specialty building (Q3) at 140-28 31st Drive in Flushing, Queens. On the lot, there is one active new building construction project, Q01000858, for a 47-unit, 35,611 square-foot residential (R-2) building. The project was submitted by United Construction &amp; Development Group and filed by Jiashu Xu with plans filed February 13, 2024 and permitted July 8, 2025. The deal closed on April 21, 2026 and was recorded on May 6, 2026. The prior lender was Maspeth Federal Savings which held debt that had an original loan amount of $8 million. The property has 20,400 square feet of built space and 33,913 square feet of additional air rights for a total buildable of 54,262 square feet according to a PincusCo analysis of city data. The loan price per built square foot is $877 and the price per buildable square foot is $329 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Lightstone Group signs $17.6M refi with JLL for 46-unit UWS rental</t>
+          <t>Ronnie Ebrani files plans for 9 units in Flatbush</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>https://www.pincusco.com/lightstone-group-signs-17-6m-refi-with-jll-for-46-unit-uws-rental/</t>
+          <t>https://www.pincusco.com/ronnie-ebrani-files-plans-for-9-units-in-flatbush/</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Lightstone Group through the entity 309 West 99th Street Associates LLC as borrower signed a</t>
-        </is>
-      </c>
-      <c r="D6" t="inlineStr">
-        <is>
-          <t>NaT</t>
-        </is>
-      </c>
+          <t>Ronnie Ebrani submitted a major alteration application to convert a three-unit, 4,740-square-foot residential (J-2) building</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr"/>
       <c r="E6" t="inlineStr"/>
       <c r="F6" t="inlineStr">
         <is>
@@ -660,197 +636,7 @@
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>Transfers 305 West 99th Street (Credit - Cyclomedia) Lightstone Group through the entity 309 West 99th Street Associates LLC as borrower signed a refi loan with lender JLL through the entity JLL Real Estate Capital, LLC valued at $17.6 million for the 46-unit residential elevator building (D3) at 305 West 99th Street in Upper West Side, Manhattan. The deal closed on April 20, 2026 and was recorded on May 5, 2026. The prior lenders were members of the Einy family which held debt that had an original loan amount of $10 million. The property has 48,099 square feet of built space according to a PincusCo analysis of city data. The loan price per built square foot is $365 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) The owner bought the property on May 19, 2020, for $18.5 million. The signatory for Lightstone Group was Joseph E. Teichman . The signatory for JLL was Omar Lopez . Prior sales, articles and revenue The owners according to the Department of Housing Preservation and Development includes Meir Milgraum, head officer and Jacob Eisenstein, agen</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>Joel Schwartz signs $23M refi with Ponce for new 48-unit rental in Cypress Hills</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>https://www.pincusco.com/joel-schwartz-signs-23m-refi-with-ponce-bank-for-newly-built-48-unit-rental-in-cypress-hills/</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>Joel Schwartz through the entity 3051 Atlantic Bx LLC as borrower signed a refi loan</t>
-        </is>
-      </c>
-      <c r="D7" t="inlineStr">
-        <is>
-          <t>NaT</t>
-        </is>
-      </c>
-      <c r="E7" t="inlineStr"/>
-      <c r="F7" t="inlineStr">
-        <is>
-          <t>PincusCo</t>
-        </is>
-      </c>
-      <c r="G7" t="inlineStr">
-        <is>
-          <t>PincusCo - Home</t>
-        </is>
-      </c>
-      <c r="H7" t="inlineStr">
-        <is>
-          <t>Transfers 3051 Atlantic Avenue (Credit - Cyclomedia) Joel Schwartz through the entity 3051 Atlantic Bx LLC as borrower signed a refi loan with lender Ponce Bank valued at $23 million for the 48-unit residential elevator building (D7) at 3051 Atlantic Avenue in Cypress Hills, Brooklyn. The deal closed on April 27, 2026 and was recorded on May 5, 2026. The prior lender was Yakar Partners which held debt that had an original loan amount of $17.5 million. The property has 38,688 square feet of built space according to a PincusCo analysis of city data. The loan price per built square foot is $594 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) The owner bought the property on March 31, 2023, for $2.1 million. The signatory for Joel Schwartz was Joel Schwartz. The signatory for Ponce Bank was Steven A. Tsavaris . Prior sales, articles and revenue The owner according to the Department of Housing Preservation and Development is Charles Schwartz, head officer. The business entity is 3051 Atlantic Bx Llc. The property</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>Maheshchand Ratanji signs $23M construction loan for hotel project in Flatbush</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>https://www.pincusco.com/maheshchand-ratanji-signs-23m-construction-loan-for-hotel-project-in-flatbush/</t>
-        </is>
-      </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>Maheshchand M. Ratanji through the entity 1045 Flatbush Avenue LLC as borrower signed a construction</t>
-        </is>
-      </c>
-      <c r="D8" t="inlineStr">
-        <is>
-          <t>NaT</t>
-        </is>
-      </c>
-      <c r="E8" t="inlineStr"/>
-      <c r="F8" t="inlineStr">
-        <is>
-          <t>PincusCo</t>
-        </is>
-      </c>
-      <c r="G8" t="inlineStr">
-        <is>
-          <t>PincusCo - Home</t>
-        </is>
-      </c>
-      <c r="H8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Transfers 1041 Flatbush Avenue (Credit - Cyclomedia) Maheshchand M. Ratanji through the entity 1045 Flatbush Avenue LLC as borrower signed a construction loan with lender State Bank of Texas valued at $23 million for the hotel development site (V1) at 1041 Flatbush Avenue in Flatbush, Brooklyn. On the lot, there is one active new building construction project, 340795483, for a 150-unit, 59,290 square-foot hotel (R-1) building. The project was submitted by Maheshchand Ratanji and filed by Nehalkumar Gandhi with plans filed December 10, 2020 and permitted October 7, 2024. The deal closed on April 22, 2026 and was recorded on May 5, 2026. The prior lender was State Bank of Texas which held debt that had an original loan amount of $4.3 million. The price per planned development square foot is $388 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) The owner bought the property on July 29, 2019, for $8.8 million. The signatory for Maheshchand M. Ratanji was Maheshchand M. Ratanji. The signatory for State Bank of Texas was Melody Collins . The property The </t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>EDRE Development pays $8.2M for 8-unit walkup in Williamsburg</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>https://www.pincusco.com/edre-development-pays-8-2m-for-8-unit-walkup-in-williamsburg/</t>
-        </is>
-      </c>
-      <c r="C9" t="inlineStr">
-        <is>
-          <t>EDRE Development through the entity 35 South 3rd Owner, LLC paid $8.2 million to John</t>
-        </is>
-      </c>
-      <c r="D9" t="inlineStr">
-        <is>
-          <t>NaT</t>
-        </is>
-      </c>
-      <c r="E9" t="inlineStr"/>
-      <c r="F9" t="inlineStr">
-        <is>
-          <t>PincusCo</t>
-        </is>
-      </c>
-      <c r="G9" t="inlineStr">
-        <is>
-          <t>PincusCo - Home</t>
-        </is>
-      </c>
-      <c r="H9" t="inlineStr">
-        <is>
-          <t>Transfers 37 South 3rd Street (Credit - Cyclomedia) EDRE Development through the entity 35 South 3rd Owner, LLC paid $8.2 million to John McNulty through the entity Southside Restoration Corp. for the eight-unit residential walkup building (C7) at 37 South 3rd Street in Williamsburg, Brooklyn. The deal closed on April 27, 2026 and was recorded on May 6, 2026. The property has 12,172 square feet of built space and 7,373 square feet of additional air rights for a total buildable of 19,575 square feet according to a PincusCo analysis of city data. The sale price per built square foot is $677 and the price per buildable square foot is $421 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) The signatory for John McNulty was John McNulty. The signatory for EDRE Development was Harel Edery . The contract date was August 13, 2025. To finance the purchase, EDRE Development borrowed $6.2 million from S3 Capital. Prior sales, articles and revenue Prior to this transaction, PincusCo has records that the buyer EDRE Development purchased one property in one transa</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>Psychotherapy and counseling nonprofit pays $3.5M for parking lot in Melrose</t>
-        </is>
-      </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>https://www.pincusco.com/new-york-psychotherapy-pays-3-5m-for-parking-lot-in-melrose/</t>
-        </is>
-      </c>
-      <c r="C10" t="inlineStr">
-        <is>
-          <t>The nonprofit New York Psychotherapy and Counseling Center paid $3.5 million to the entity 622</t>
-        </is>
-      </c>
-      <c r="D10" t="inlineStr">
-        <is>
-          <t>NaT</t>
-        </is>
-      </c>
-      <c r="E10" t="inlineStr"/>
-      <c r="F10" t="inlineStr">
-        <is>
-          <t>PincusCo</t>
-        </is>
-      </c>
-      <c r="G10" t="inlineStr">
-        <is>
-          <t>PincusCo - Home</t>
-        </is>
-      </c>
-      <c r="H10" t="inlineStr">
-        <is>
-          <t>Transfers 622 Courtlandt Avenue (Credit - Cyclomedia) The nonprofit New York Psychotherapy and Counseling Center paid $3.5 million to the entity 622 Courtlandt LLC for a three-parcel parking lot (G6) at 616, 620 and 622 Courtlandt Avenue in Melrose, Bronx. The expected use is owner-occupied. The New York Psychotherapy and Counseling Center has a large office building a block away at 579 Courtlandt Avenue. The deal closed on April 23, 2026 and was recorded on May 6, 2026. The three properties have zero square feet of built space and 31,138 square feet of additional air rights for a total buildable of 31,138 square feet according to a PincusCo analysis of city data. The sale price per buildable square foot is $110 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) The signatories for the sellers Amarendra Deshmukh and Jyotsna Deshmukh were Amarendra Deshmukh and Jyotsna Deshmukh. The signatory for New York Psychotherapy and Counseling Center was Elliot Klein . The contract date was April 23, 2026. David Simone of Concourse Realty Partners brokered the s</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>Lotte pays $491.1M to Archdiocese of NY for three properties in Midtown East</t>
-        </is>
-      </c>
-      <c r="B11" t="inlineStr">
-        <is>
-          <t>https://www.pincusco.com/lotte-pays-491-1m-to-archdiocese-of-ny-for-three-properties-in-midtown-east/</t>
-        </is>
-      </c>
-      <c r="C11" t="inlineStr">
-        <is>
-          <t>Lotte Corporation through the entity Lotte Hotel New York Palace, LLC paid $491.1 million through</t>
-        </is>
-      </c>
-      <c r="D11" t="inlineStr">
-        <is>
-          <t>NaT</t>
-        </is>
-      </c>
-      <c r="E11" t="inlineStr"/>
-      <c r="F11" t="inlineStr">
-        <is>
-          <t>PincusCo</t>
-        </is>
-      </c>
-      <c r="G11" t="inlineStr">
-        <is>
-          <t>PincusCo - Home</t>
-        </is>
-      </c>
-      <c r="H11" t="inlineStr">
-        <is>
-          <t>Transfers 455 Madison Avenue (Credit - Cyclomedia) Lotte Corporation through the entity Lotte Hotel New York Palace, LLC paid $491.1 million through a ground leased fee to Archdiocese of New York and Roman Catholic Church through the entity The Archdiocese Of New York for the hotel building (H1) at 455 Madison Avenue in Midtown East, Manhattan, retail building (O5) at 457 Madison Avenue in Midtown East, Manhattan, and retail building (K2) at 35 East 50th Street in Midtown East, Manhattan. The expected use is cash flowing. The deal closed on April 30, 2026 and was recorded on May 6, 2026. The three properties have 866,090 square feet of built space and 56,256 square feet of additional air rights according to a PincusCo analysis of city data. The sale price per built square foot is $567 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) The signatory for Archdiocese of New York and Roman Catholic Church was John Cahill . The signatory for Lotte Corporation was Jihong Lee . The contract date was November 12, 2025. PincusCo reported on this transaction in</t>
+          <t>Development 2587 Bedford Avenue axonometric diagram and section (Credit - Payam Rahmanan architect via DOB) Ronnie Ebrani submitted a major alteration application to convert a three-unit, 4,740-square-foot residential (J-2) building at 2587 Bedford Avenue in Flatbush, Brooklyn, into a nine-unit building. The plan was filed on April 16, 2026. It calls for an increase in size from a 32-foot-tall, three-story building to a 43-foot-tall, four-story building with nine dwelling units building and was filed with the New York City Department of Buildings under job number B01382316. The project is described in the filing as: conversion of existing 3 family dwelling to 9 family and vertical enlargement (1 additional story and penthouse). refiling of previously reviewed job under B01155660 in order to select alt-CO to meet new building requirements as required by the examiner. The applicant is the Registered Architect Payam Rahmanan of Rahmanan Architecture + Planning PC. Ronnie Ebrani bought the building in May 2024 for $960,000. The neighborhood In Flatbush, The majority, or 54 percent of the 37.4 million square feet of commercial built space are elevator buildings, with walkup buildings ne</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto update queens news 2026-05-09T13:50:06Z
</commit_message>
<xml_diff>
--- a/data/output/queens_dev_news.xlsx
+++ b/data/output/queens_dev_news.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H6"/>
+  <dimension ref="A1:H7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -473,17 +473,17 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>World Wide Group signs $34.5M refi with MetLife for 124-unit LIC rental</t>
+          <t>Rubin Equities signs $14.3M refi loan with CDK Capital XVII for industrial in Mt Eden</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>https://www.pincusco.com/world-wide-group-signs-34-5m-refi-with-metlife-for-124-unit-lic-rental/</t>
+          <t>https://www.pincusco.com/rubin-equities-signs-14-3m-refi-loan-with-cdk-capital-xvii-for-industrial-in-mt-eden/</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>World Wide Group through the entity WWG Crescent 2 LLC as borrower signed a refi</t>
+          <t>Rubin Equities through the entity 1342 Inwood LLC as borrower signed a refi loan with</t>
         </is>
       </c>
       <c r="D2" t="inlineStr"/>
@@ -500,24 +500,24 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>Transfers 42-15 Crescent Street (Credit - Cyclomedia) World Wide Group through the entity WWG Crescent 2 LLC as borrower signed a refi loan with lender MetLife through the entity Metlife Real Estate Lending LLC valued at $34.5 million for the 124-unit residential elevator building (D7) at 42-15 Crescent Street in Long Island City, Queens. The deal closed on April 24, 2026 and was recorded on May 6, 2026. The prior lender was Helaba which held debt that had an original loan amount of $32 million. The property has 110,743 square feet of built space according to a PincusCo analysis of city data. The loan price per built square foot is $311 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) The owner bought the property on March 17, 2016, for $70 million. The signatory for World Wide Group was Jodi Gerstman . The signatory for MetLife was Brett Ulrich . Prior sales, articles and revenue The owners according to the Department of Housing Preservation and Development includes Jodi Gerstman, head officer and Neal Cohen, officer. The business entities are Rose</t>
+          <t xml:space="preserve">Transfers 1342 Inwood Avenue (Credit - Cyclomedia) Rubin Equities through the entity 1342 Inwood LLC as borrower signed a refi loan with lender CDK Capital XVII valued at $14.3 million for the industrial building (F5) at 1342 Inwood Avenue in Mt Eden, Bronx. PincusCo could not determine the principals behind the lender. The deal closed on April 23, 2026 and was recorded on May 6, 2026. The prior lender was Fairview Partners Investment Management which held debt that had an original loan amount of $12.8 million. The property has 56,250 square feet of built space and 81,470 square feet of additional air rights for a total buildable of 137,767 square feet according to a PincusCo analysis of city data. The loan price per built square foot is $253 and the price per buildable square foot is $103 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) The owner bought the property on March 1, 2023, for $20.5 million. The signatory for Rubin Equities was Sam Rubin . The signatory for CDK Capital XVII was Hillel Lazarus . The property The industrial building in Mt </t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Ekstein Development signs $58M refi with MetLife for new 107-unit rental in Bushwick</t>
+          <t>Montperia Group pays $13M to Vision Enterprises Management for office in Bayside</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>https://www.pincusco.com/ekstein-development-signs-58m-refi-with-metlife-for-new-107-unit-rental-in-bushwick/</t>
+          <t>https://www.pincusco.com/montperia-group-pays-13m-to-vision-enterprises-management-for-office-in-bayside/</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Ekstein Development Group through the entity 1333 Broadway LLC as borrower signed a refi loan</t>
+          <t>Montperia Group through the entity Bayside 88 Corp. paid $13 million to Vision Enterprises Management</t>
         </is>
       </c>
       <c r="D3" t="inlineStr"/>
@@ -534,24 +534,24 @@
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>Transfers 1333 Broadway (Credit - Cyclomedia) Ekstein Development Group through the entity 1333 Broadway LLC as borrower signed a refi loan with lender MetLife through the entity Metropolitan Tower Life Insurance Company valued at $58 million for the 107-unit residential elevator building (D7) at 1333 Broadway in Bushwick, Brooklyn. The deal closed on April 24, 2026 and was recorded on May 6, 2026. The prior lender was Santander Bank which held debt that had an original loan amount of $48.8 million. The property has 120,403 square feet of built space according to a PincusCo analysis of city data. The loan price per built square foot is $481 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) The owner bought the property on December 6, 2019, for $16.7 million. The signatory for Ekstein Development Group was Erik Ekstein . The signatory for MetLife was Anthony Soldi . Prior sales, articles and revenue The 120,403-square-foot property generated revenue of $3.8 million or $31 per square foot, according to the most recent income and expense figures.</t>
+          <t>Transfers 42-40 Bell Boulevard (Credit - Cyclomedia) Montperia Group through the entity Bayside 88 Corp. paid $13 million to Vision Enterprises Management through the entity P &amp; L Associates, LLC for the office building (O2) at 42-40 Bell Boulevard in Bayside, Queens. The expected use is cash flowing. The deal closed on April 28, 2026 and was recorded on May 5, 2026. The property has 61,620 square feet of built space according to a PincusCo analysis of city data. The sale price per built square foot is $210 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) The signatory for Vision Enterprises Management was Leonard Zangas . The signatory for Montperia Group was Alex Lau . The contract date was February 12, 2026. Prior sales, articles and revenue Prior to this transaction, PincusCo has no record that the buyer Montperia Group had purchased any other properties and sold two properties in two transactions for a total of $9.1 million over the past 24 months. The seller Vision Enterprises Management had not purchased any other properties and sold seven pr</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>United Construction, New Land Capital sign $18.5M construction loan for 48-unit project in Flushing</t>
+          <t>Empire Management signs $21.5M refi loan with Derby Copeland for 31-unit rental in Chelsea</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>https://www.pincusco.com/united-construction-new-land-capital-sign-18-5m-construction-loan-with-preferred-bank-for-in-flushing/</t>
+          <t>https://www.pincusco.com/empire-management-signs-21-5m-refi-loan-with-derby-copeland-for-31-unit-rental-in-chelsea/</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>United Construction &amp; Development Group and New Land Capital through the entity 32nd Ave Holding</t>
+          <t>Empire Management through the entity Chelsea 261 W21-Rt LLC as borrower signed a refi loan</t>
         </is>
       </c>
       <c r="D4" t="inlineStr"/>
@@ -568,24 +568,24 @@
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>Transfers 141-05 32nd Avenue axonometric diagram (Credit - Ning Lu architect via DOB) United Construction &amp; Development Group and New Land Capital through the entity 32nd Ave Holding LLC as borrower signed a new construction loan with lender Preferred Bank valued at $18.5 million for the property at 141-05 32nd Avenue in Flushing, Queens. On the lot, there is one active new building construction project, Q00983687, for a 48-unit, 36,927 square-foot residential (R-2) building. The project was submitted by United Construction &amp; Development Group and filed by Jiashu Xu with plans filed February 13, 2024 and permitted February 18, 2025. The deal closed on April 21, 2026 and was recorded on May 6, 2026. The loan price per planned development square foot is $501 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) The signatory for United Construction &amp; Development Group and New Land Capital was Hangyuan Zhang . Violations and lawsuits</t>
+          <t>Transfers 216 8th Avenue (Credit - Cyclomedia) Empire Management through the entity Chelsea 261 W21-Rt LLC as borrower signed a refi loan with lender Derby Copeland Capital through the entity Fcr Dc Jv Holdings LLC valued at $21.5 million for the 31-unit residential elevator building (D7) at 216 8th Avenue in Chelsea, Manhattan. The deal closed on April 30, 2026 and was recorded on May 6, 2026. The prior lender was Flagstar Bank which held debt that had an original loan amount of $12.2 million. The property has 32,325 square feet of built space according to a PincusCo analysis of city data. The loan price per built square foot is $665 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) The owner bought the property on November 30, 2004, for $15.2 million. The signatory for Empire Management was Fred Ohebshalom . The signatory for Derby Copeland Capital was Jesse Hutcher . Prior sales, articles and revenue The owners according to the Department of Housing Preservation and Development includes Ramin Shalom, head officer and E Polanco, site manager. The b</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>United Construction &amp; Development signs $17.9M construction loan for 47-unit project in Flushing</t>
+          <t>DIB Management signs $9M refi with OceanFirst for commercial in Sunset Park</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>https://www.pincusco.com/united-construction-development-signs-17-9m-construction-loan-for-47-unit-project-in-flushing/</t>
+          <t>https://www.pincusco.com/dib-management-signs-9m-refi-with-oceanfirst-for-industrial-in-sunset-park/</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>United Construction &amp; Development Group through the entity 32nd Ave Management LLC as borrower signed</t>
+          <t>DIB Management through the entity Sunset Commercial Property, LLC as borrower signed a refi loan</t>
         </is>
       </c>
       <c r="D5" t="inlineStr"/>
@@ -602,24 +602,24 @@
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>Transfers 140-28 31st Drive axonometric diagram (Credit - Ning Lu architect via DOB) United Construction &amp; Development Group through the entity 32nd Ave Management LLC as borrower signed a new construction loan with lender Preferred Bank valued at $17.9 million for the specialty building (Q3) at 140-28 31st Drive in Flushing, Queens. On the lot, there is one active new building construction project, Q01000858, for a 47-unit, 35,611 square-foot residential (R-2) building. The project was submitted by United Construction &amp; Development Group and filed by Jiashu Xu with plans filed February 13, 2024 and permitted July 8, 2025. The deal closed on April 21, 2026 and was recorded on May 6, 2026. The prior lender was Maspeth Federal Savings which held debt that had an original loan amount of $8 million. The property has 20,400 square feet of built space and 33,913 square feet of additional air rights for a total buildable of 54,262 square feet according to a PincusCo analysis of city data. The loan price per built square foot is $877 and the price per buildable square foot is $329 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet</t>
+          <t>Transfers 201 42nd Street (Credit - Cyclomedia) DIB Management through the entity Sunset Commercial Property, LLC as borrower signed a refi loan with lender OceanFirst Bank valued at $9 million for the industrial building (F5) at 201 42nd Street in Sunset Park, Brooklyn. The deal closed on April 21, 2026 and was recorded on May 6, 2026. The prior lender was Northeast Bank which held debt that had an original loan amount of $7.6 million.The property has 104,182 square feet of built space according to a PincusCo analysis of city data. The loan price per built square foot is $86 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) The owner bought the property on July 11, 2007, for $8.8 million. The signatory for DIB Management was Ramona Luckert . The signatory for OceanFirst Bank was Annmarie Sorena . Prior sales, articles and revenue The 104,182-square-foot property generated revenue of $1.7 million or $16 per square foot, according to the most recent income and expense figures. The property</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Ronnie Ebrani files plans for 9 units in Flatbush</t>
+          <t>Chaim Porges pays $3M for industrial in Sunset Park</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>https://www.pincusco.com/ronnie-ebrani-files-plans-for-9-units-in-flatbush/</t>
+          <t>https://www.pincusco.com/chaim-porges-pays-3m-for-industrial-in-sunset-park/</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Ronnie Ebrani submitted a major alteration application to convert a three-unit, 4,740-square-foot residential (J-2) building</t>
+          <t>Chaim Porges through the entity 251 43st Lll paid $3 million to Blend Bekteshi through</t>
         </is>
       </c>
       <c r="D6" t="inlineStr"/>
@@ -636,7 +636,41 @@
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>Development 2587 Bedford Avenue axonometric diagram and section (Credit - Payam Rahmanan architect via DOB) Ronnie Ebrani submitted a major alteration application to convert a three-unit, 4,740-square-foot residential (J-2) building at 2587 Bedford Avenue in Flatbush, Brooklyn, into a nine-unit building. The plan was filed on April 16, 2026. It calls for an increase in size from a 32-foot-tall, three-story building to a 43-foot-tall, four-story building with nine dwelling units building and was filed with the New York City Department of Buildings under job number B01382316. The project is described in the filing as: conversion of existing 3 family dwelling to 9 family and vertical enlargement (1 additional story and penthouse). refiling of previously reviewed job under B01155660 in order to select alt-CO to meet new building requirements as required by the examiner. The applicant is the Registered Architect Payam Rahmanan of Rahmanan Architecture + Planning PC. Ronnie Ebrani bought the building in May 2024 for $960,000. The neighborhood In Flatbush, The majority, or 54 percent of the 37.4 million square feet of commercial built space are elevator buildings, with walkup buildings ne</t>
+          <t>Transfers 251 43rd Street (Credit - Cyclomedia) Chaim Porges through the entity 251 43st Lll paid $3 million to Blend Bekteshi through the entity Blend 251 LLC for the industrial building (E1) at 251 43rd Street in Sunset Park, Brooklyn. The deal closed on April 13, 2026 and was recorded on May 6, 2026. The property has 7,000 square feet of built space and 7,012 square feet of additional air rights for a total buildable of 14,024 square feet according to a PincusCo analysis of city data. The sale price per built square foot is $425 and the price per buildable square foot is $212 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) The seller bought the property on January 19, 2024, for $2.3 million. The signatory for Blend Bekteshi was Blend Bekteshi. The signatory for Chaim Porges was Chaim Porges. The contract date was April 13, 2026. Prior sales, articles and revenue Prior to this transaction, PincusCo has no record that the buyer Chaim Porges had purchased any other properties and has no record it sold any properties over the past 24 months. The sel</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Omid Mashieh pays $2.5M for 3-family in Williamsburg</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>https://www.pincusco.com/omid-mashieh-pays-2-5m-for-3-family-in-williamsburg/</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Omid Mashieh through the entity MTEK Henry LLC paid $2.5 million for the three-unit building</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr"/>
+      <c r="E7" t="inlineStr"/>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>PincusCo</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>PincusCo - Home</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>Transfers 9A North Henry Street (Credit - Cyclomedia) Omid Mashieh through the entity MTEK Henry LLC paid $2.5 million for the three-unit building (C0) at 9A North Henry Street in Williamsburg, Brooklyn. The expected use is renovation. The deal closed on April 16, 2026 and was recorded on May 6, 2026. The property has 4,200 square feet of built space and 800 square feet of additional air rights for a total buildable of 5,000 square feet according to a PincusCo analysis of city data. The sale price per built square foot is $595 and the price per buildable square foot is $500 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) The signatory for Alfonso A. Pettenato was Lucille Pettenato. The signatory for Omid Mashieh was Omid Mashieh. The contract date was January 8, 2026. Prior sales, articles and revenue Prior to this transaction, PincusCo has records that the buyer Omid Mashieh purchased four properties in four transactions for a total of $9.7 million and sold six properties in six transactions for a total of $14.9 million over the past 24 months. Th</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto update queens news 2026-05-10T13:53:02Z
</commit_message>
<xml_diff>
--- a/data/output/queens_dev_news.xlsx
+++ b/data/output/queens_dev_news.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H7"/>
+  <dimension ref="A1:H1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -467,210 +467,6 @@
       <c r="H1" s="1" t="inlineStr">
         <is>
           <t>content_preview</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>Rubin Equities signs $14.3M refi loan with CDK Capital XVII for industrial in Mt Eden</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>https://www.pincusco.com/rubin-equities-signs-14-3m-refi-loan-with-cdk-capital-xvii-for-industrial-in-mt-eden/</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>Rubin Equities through the entity 1342 Inwood LLC as borrower signed a refi loan with</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr"/>
-      <c r="E2" t="inlineStr"/>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t>PincusCo</t>
-        </is>
-      </c>
-      <c r="G2" t="inlineStr">
-        <is>
-          <t>PincusCo - Home</t>
-        </is>
-      </c>
-      <c r="H2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Transfers 1342 Inwood Avenue (Credit - Cyclomedia) Rubin Equities through the entity 1342 Inwood LLC as borrower signed a refi loan with lender CDK Capital XVII valued at $14.3 million for the industrial building (F5) at 1342 Inwood Avenue in Mt Eden, Bronx. PincusCo could not determine the principals behind the lender. The deal closed on April 23, 2026 and was recorded on May 6, 2026. The prior lender was Fairview Partners Investment Management which held debt that had an original loan amount of $12.8 million. The property has 56,250 square feet of built space and 81,470 square feet of additional air rights for a total buildable of 137,767 square feet according to a PincusCo analysis of city data. The loan price per built square foot is $253 and the price per buildable square foot is $103 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) The owner bought the property on March 1, 2023, for $20.5 million. The signatory for Rubin Equities was Sam Rubin . The signatory for CDK Capital XVII was Hillel Lazarus . The property The industrial building in Mt </t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>Montperia Group pays $13M to Vision Enterprises Management for office in Bayside</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>https://www.pincusco.com/montperia-group-pays-13m-to-vision-enterprises-management-for-office-in-bayside/</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>Montperia Group through the entity Bayside 88 Corp. paid $13 million to Vision Enterprises Management</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr"/>
-      <c r="E3" t="inlineStr"/>
-      <c r="F3" t="inlineStr">
-        <is>
-          <t>PincusCo</t>
-        </is>
-      </c>
-      <c r="G3" t="inlineStr">
-        <is>
-          <t>PincusCo - Home</t>
-        </is>
-      </c>
-      <c r="H3" t="inlineStr">
-        <is>
-          <t>Transfers 42-40 Bell Boulevard (Credit - Cyclomedia) Montperia Group through the entity Bayside 88 Corp. paid $13 million to Vision Enterprises Management through the entity P &amp; L Associates, LLC for the office building (O2) at 42-40 Bell Boulevard in Bayside, Queens. The expected use is cash flowing. The deal closed on April 28, 2026 and was recorded on May 5, 2026. The property has 61,620 square feet of built space according to a PincusCo analysis of city data. The sale price per built square foot is $210 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) The signatory for Vision Enterprises Management was Leonard Zangas . The signatory for Montperia Group was Alex Lau . The contract date was February 12, 2026. Prior sales, articles and revenue Prior to this transaction, PincusCo has no record that the buyer Montperia Group had purchased any other properties and sold two properties in two transactions for a total of $9.1 million over the past 24 months. The seller Vision Enterprises Management had not purchased any other properties and sold seven pr</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>Empire Management signs $21.5M refi loan with Derby Copeland for 31-unit rental in Chelsea</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>https://www.pincusco.com/empire-management-signs-21-5m-refi-loan-with-derby-copeland-for-31-unit-rental-in-chelsea/</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>Empire Management through the entity Chelsea 261 W21-Rt LLC as borrower signed a refi loan</t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr"/>
-      <c r="E4" t="inlineStr"/>
-      <c r="F4" t="inlineStr">
-        <is>
-          <t>PincusCo</t>
-        </is>
-      </c>
-      <c r="G4" t="inlineStr">
-        <is>
-          <t>PincusCo - Home</t>
-        </is>
-      </c>
-      <c r="H4" t="inlineStr">
-        <is>
-          <t>Transfers 216 8th Avenue (Credit - Cyclomedia) Empire Management through the entity Chelsea 261 W21-Rt LLC as borrower signed a refi loan with lender Derby Copeland Capital through the entity Fcr Dc Jv Holdings LLC valued at $21.5 million for the 31-unit residential elevator building (D7) at 216 8th Avenue in Chelsea, Manhattan. The deal closed on April 30, 2026 and was recorded on May 6, 2026. The prior lender was Flagstar Bank which held debt that had an original loan amount of $12.2 million. The property has 32,325 square feet of built space according to a PincusCo analysis of city data. The loan price per built square foot is $665 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) The owner bought the property on November 30, 2004, for $15.2 million. The signatory for Empire Management was Fred Ohebshalom . The signatory for Derby Copeland Capital was Jesse Hutcher . Prior sales, articles and revenue The owners according to the Department of Housing Preservation and Development includes Ramin Shalom, head officer and E Polanco, site manager. The b</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>DIB Management signs $9M refi with OceanFirst for commercial in Sunset Park</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>https://www.pincusco.com/dib-management-signs-9m-refi-with-oceanfirst-for-industrial-in-sunset-park/</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>DIB Management through the entity Sunset Commercial Property, LLC as borrower signed a refi loan</t>
-        </is>
-      </c>
-      <c r="D5" t="inlineStr"/>
-      <c r="E5" t="inlineStr"/>
-      <c r="F5" t="inlineStr">
-        <is>
-          <t>PincusCo</t>
-        </is>
-      </c>
-      <c r="G5" t="inlineStr">
-        <is>
-          <t>PincusCo - Home</t>
-        </is>
-      </c>
-      <c r="H5" t="inlineStr">
-        <is>
-          <t>Transfers 201 42nd Street (Credit - Cyclomedia) DIB Management through the entity Sunset Commercial Property, LLC as borrower signed a refi loan with lender OceanFirst Bank valued at $9 million for the industrial building (F5) at 201 42nd Street in Sunset Park, Brooklyn. The deal closed on April 21, 2026 and was recorded on May 6, 2026. The prior lender was Northeast Bank which held debt that had an original loan amount of $7.6 million.The property has 104,182 square feet of built space according to a PincusCo analysis of city data. The loan price per built square foot is $86 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) The owner bought the property on July 11, 2007, for $8.8 million. The signatory for DIB Management was Ramona Luckert . The signatory for OceanFirst Bank was Annmarie Sorena . Prior sales, articles and revenue The 104,182-square-foot property generated revenue of $1.7 million or $16 per square foot, according to the most recent income and expense figures. The property</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>Chaim Porges pays $3M for industrial in Sunset Park</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>https://www.pincusco.com/chaim-porges-pays-3m-for-industrial-in-sunset-park/</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>Chaim Porges through the entity 251 43st Lll paid $3 million to Blend Bekteshi through</t>
-        </is>
-      </c>
-      <c r="D6" t="inlineStr"/>
-      <c r="E6" t="inlineStr"/>
-      <c r="F6" t="inlineStr">
-        <is>
-          <t>PincusCo</t>
-        </is>
-      </c>
-      <c r="G6" t="inlineStr">
-        <is>
-          <t>PincusCo - Home</t>
-        </is>
-      </c>
-      <c r="H6" t="inlineStr">
-        <is>
-          <t>Transfers 251 43rd Street (Credit - Cyclomedia) Chaim Porges through the entity 251 43st Lll paid $3 million to Blend Bekteshi through the entity Blend 251 LLC for the industrial building (E1) at 251 43rd Street in Sunset Park, Brooklyn. The deal closed on April 13, 2026 and was recorded on May 6, 2026. The property has 7,000 square feet of built space and 7,012 square feet of additional air rights for a total buildable of 14,024 square feet according to a PincusCo analysis of city data. The sale price per built square foot is $425 and the price per buildable square foot is $212 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) The seller bought the property on January 19, 2024, for $2.3 million. The signatory for Blend Bekteshi was Blend Bekteshi. The signatory for Chaim Porges was Chaim Porges. The contract date was April 13, 2026. Prior sales, articles and revenue Prior to this transaction, PincusCo has no record that the buyer Chaim Porges had purchased any other properties and has no record it sold any properties over the past 24 months. The sel</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>Omid Mashieh pays $2.5M for 3-family in Williamsburg</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>https://www.pincusco.com/omid-mashieh-pays-2-5m-for-3-family-in-williamsburg/</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>Omid Mashieh through the entity MTEK Henry LLC paid $2.5 million for the three-unit building</t>
-        </is>
-      </c>
-      <c r="D7" t="inlineStr"/>
-      <c r="E7" t="inlineStr"/>
-      <c r="F7" t="inlineStr">
-        <is>
-          <t>PincusCo</t>
-        </is>
-      </c>
-      <c r="G7" t="inlineStr">
-        <is>
-          <t>PincusCo - Home</t>
-        </is>
-      </c>
-      <c r="H7" t="inlineStr">
-        <is>
-          <t>Transfers 9A North Henry Street (Credit - Cyclomedia) Omid Mashieh through the entity MTEK Henry LLC paid $2.5 million for the three-unit building (C0) at 9A North Henry Street in Williamsburg, Brooklyn. The expected use is renovation. The deal closed on April 16, 2026 and was recorded on May 6, 2026. The property has 4,200 square feet of built space and 800 square feet of additional air rights for a total buildable of 5,000 square feet according to a PincusCo analysis of city data. The sale price per built square foot is $595 and the price per buildable square foot is $500 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) The signatory for Alfonso A. Pettenato was Lucille Pettenato. The signatory for Omid Mashieh was Omid Mashieh. The contract date was January 8, 2026. Prior sales, articles and revenue Prior to this transaction, PincusCo has records that the buyer Omid Mashieh purchased four properties in four transactions for a total of $9.7 million and sold six properties in six transactions for a total of $14.9 million over the past 24 months. Th</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto update queens news 2026-05-11T15:34:27Z
</commit_message>
<xml_diff>
--- a/data/output/queens_dev_news.xlsx
+++ b/data/output/queens_dev_news.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H1"/>
+  <dimension ref="A1:H8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -467,6 +467,244 @@
       <c r="H1" s="1" t="inlineStr">
         <is>
           <t>content_preview</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Omnia Properties signs $45M refi loan with Valley for 57-unit building in Lower East Side</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>https://www.pincusco.com/omnia-properties-signs-45m-refi-loan-with-valley-for-57-unit-building-in-lower-east-side/</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Omnia Properties through the entity 185 Chrystie Street LLC as borrower signed a refi loan</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr"/>
+      <c r="E2" t="inlineStr"/>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>PincusCo</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>PincusCo - Home</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Transfers 183 Chrystie Street (Credit - Cyclomedia) Omnia Properties through the entity 185 Chrystie Street LLC as borrower signed a refi loan with lender Valley National Bank through the entity Valley National Bank valued at $45 million for the four condominium units that make up the property at 183 Chrystie Street in Lower East Side, Manhattan, property at 183 Chrystie Street in Lower East Side, Manhattan, and property at 183 Chrystie Street in Lower East Side, Manhattan. The building has an alternate address of 4 Freeman Alley. The deal closed on April 28, 2026 and was recorded on May 8, 2026. The prior lender was Valley National Bank which held debt that had an original loan amount of $35 million. The four properties have 73,949 square feet of built space according to a PincusCo analysis of city data. The loan price per built square foot is $608.50 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) The signatory for Omnia Properties was David Paz .  The block On the tax block of 183 Chrystie Street, PincusCo has identified the owners of 11 of the </t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Lightstone Group signs $19.2M refi with JLL for 34-unit UWS rental</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>https://www.pincusco.com/lightstone-group-signs-19-2m-refi-with-jll-for-34-unit-uws-rental/</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Lightstone Group through the entity 317 West 99th Street Associates LLC as borrower signed a</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr"/>
+      <c r="E3" t="inlineStr"/>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>PincusCo</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>PincusCo - Home</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Transfers 317 West 99th Street (Credit - Cyclomedia) Lightstone Group through the entity 317 West 99th Street Associates LLC as borrower signed a refi loan with lender JLL through the entity JLL Real Estate Capital, LLC valued at $19.2 million for the 34-unit residential elevator building (D3) at 317 West 99th Street in Upper West Side, Manhattan. The deal closed on April 20, 2026 and was recorded on May 7, 2026. The prior lender was Sofia Einy which held debt that had an original loan amount of $10 million. The property has 47,851 square feet of built space according to a PincusCo analysis of city data. The loan price per built square foot is $400 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) The owner bought the property on May 19, 2020, for $18.5 million. The signatory for Lightstone Group was Joseph E. Teichman . The signatory for JLL was Omar Lopez . On the same day, Lightstone Group through the entity 309 West 99th Street Associates LLC as borrower signed a refi loan with lender JLL through the entity JLL Real Estate Capital, LLC valued at </t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>$5M refi signed with Liberty Mutual Insurance Company for LIC industrial</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>https://www.pincusco.com/5m-refi-signed-with-liberty-mutual-insurance-company-for-lic-industrial/</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Salvatore DiLorenzo through the entity Jas 12th Street Holding LLC as borrower signed a refi</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr"/>
+      <c r="E4" t="inlineStr"/>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>PincusCo</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>PincusCo - Home</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>Transfers 42-20 12th Street (Credit - Cyclomedia) Salvatore DiLorenzo through the entity Jas 12th Street Holding LLC as borrower signed a refi loan with lender Liberty Mutual Insurance Company valued at $5 million for the industrial building (F9) at 42-20 12th Street in Long Island City, Queens. The deal closed on April 20, 2026 and was recorded on May 7, 2026. The property has 9,764 square feet of built space and 7,077 square feet of additional air rights for a total buildable of 16,850 square feet according to a PincusCo analysis of city data. The loan price per built square foot is $512 and the price per buildable square foot is $296 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) The owner bought the property on December 20, 2021, for $3.3 million. The signatory for the borrower as member, was Salvatore J. DiLorenzo. The signatory for Liberty Mutual Insurance Company was Rachel Walsh . Prior sales, articles and revenue The 9,764-square-foot property generated revenue of $187,078 or $19 per square foot, according to the most recent income and ex</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Timber Equities signs $27.5M refi loan with JLL for 60-unit rental in Inwood</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>https://www.pincusco.com/timber-equities-signs-27-5m-refi-loan-with-jll-for-residential-elevator-in-inwood/</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Timber Equities through the entity 5055 Broadway L.P. as borrower signed a refi loan with</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr"/>
+      <c r="E5" t="inlineStr"/>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>PincusCo</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>PincusCo - Home</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>Transfers 5055 Broadway (Credit - Cyclomedia) Timber Equities through the entity 5055 Broadway L.P. as borrower signed a refi loan with lender JLL through the entity Lrecs Holdings Iia, L.L.C. valued at $27.5 million for the 60-unit residential elevator building (D6) at 5055 Broadway in Inwood, Manhattan. On the lot, there is one active new building construction project, M00578593, for a 60-unit, 43,203 square-foot R-2 building. The project was submitted by Timber Equities and filed by Michel Perle with plans filed September 8, 2021 and permitted August 28, 2024. The deal closed on May 4, 2026 and was recorded on May 7, 2026. The prior lender was Bank Hapoalim which held debt that had an original loan amount of $21 million.The property has 44,651 square feet of built space according to a PincusCo analysis of city data. The loan price per built square foot is $615 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) The owner bought the property on October 29, 2020, for $3.4 million. The signatory for Timber Equities was Joseph Seidenfeld . The signatory</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Timber Equities signs $35.6M refi loan with JLL for new 94-unit rental in Harlem</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>https://www.pincusco.com/timber-equities-signs-35-6m-refi-loan-with-jll-for-residential-elevator-in-harlem/</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Timber Equities through the entity 2460 Fdb Lp as borrower signed a refi loan with</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr"/>
+      <c r="E6" t="inlineStr"/>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>PincusCo</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>PincusCo - Home</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>Transfers 2460 Frederick Douglass Boulevard (Credit - Cyclomedia) Timber Equities through the entity 2460 Fdb Lp as borrower signed a refi loan with lender JLL through the entity Lrecs Holdings Iia, L.L.C. valued at $35.6 million for the 94-unit residential elevator building (D6) at 2460 Frederick Douglass Boulevard in Harlem, Manhattan. On the lot, there was a new building construction project, M00686955, for a 94-unit, 89,166 square-foot residential (R-2) building. The project was submitted by Timber Equities and filed by Michel Perle with plans filed February 28, 2022 and permitted February 21, 2024. The loas closed on May 4, 2026 and was recorded on May 7, 2026. The prior lender was Webster Bank which held debt that had an original loan amount of $26.5 million.The property has 58,196 square feet of built space according to a PincusCo analysis of city data. The loan price per built square foot is $611 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) The owner bought the property on November 18, 2022, for $2.4 million. The signatory for Timber Equ</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Xiang Wei Zhou pays $4.2M to Santander Bank for office in Astoria</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>https://www.pincusco.com/xiang-wei-zhou-pays-4-2m-to-santander-bank-for-office-in-astoria/</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Xiang Wei Zhou through the entity Hung Yuen Holdings Inc. paid $4.2 million to Santander</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr"/>
+      <c r="E7" t="inlineStr"/>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>PincusCo</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>PincusCo - Home</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>Transfers 37-10 Broadway (Credit - Cyclomedia) Xiang Wei Zhou through the entity Hung Yuen Holdings Inc. paid $4.2 million to Santander Bank through the entity Santander Bank, N.A. for the office building (O5) at 37-10 Broadway in Astoria, Queens. The expected use is cash flowing. The deal closed on April 15, 2026 and was recorded on May 7, 2026. The property has 10,275 square feet of built space and 5,853 square feet of additional air rights for a total buildable of 16,110 square feet according to a PincusCo analysis of city data. The sale price per built square foot is $405 and the price per buildable square foot is $258 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) The seller bought the property on January 30, 2009, for $50.9 million. The signatory for Santander Bank was Michael Kuronen . The contract date was March 12, 2026. Prior sales, articles and revenue Prior to this transaction, PincusCo has no record that the buyer Xiang Wei Zhou had purchased any other properties and has no record it sold any properties over the past 24 months. The se</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Nilin Zhang, Qiao Chen pay $9.9M for industrial in Maspeth</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>https://www.pincusco.com/nilin-zhang-qiao-chen-pay-9-9m-for-industrial-in-maspeth/</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Nilin Zhang and Qiao Chen through the entity 72-02 51st Ave Inc. paid $9.9 million</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr"/>
+      <c r="E8" t="inlineStr"/>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>PincusCo</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>PincusCo - Home</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>Transfers 72-02 51st Avenue (Credit -Cyclomedia) Nilin Zhang and Qiao Chen through the entity 72-02 51st Ave Inc. paid $9.9 million for the industrial building (E1) at 72-02 51st Avenue in Maspeth, Queens. The expected use is cash flowing. The deal closed on April 23, 2026 and was recorded on May 7, 2026. The property has 20,726 square feet of built space and 3,392 square feet of additional air rights for a total buildable of 24,230 square feet according to a PincusCo analysis of city data. The sale price per built square foot is $476 and the price per buildable square foot is $407 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) The signatory for Ciro Salvia and Paolo Salvia was Ciro Salvia and Paolo Salvia. The signatory for Nilin Zhang and Qiao Chen was Nilin Zhang. The contract date was December 22, 2025. Prior sales, articles and revenue Prior to this transaction, PincusCo has no record that the buyer Nilin Zhang had purchased any other properties and has no record it sold any properties over the past 24 months. The seller Ciro Salvia had not p</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto update queens news 2026-05-12T14:52:04Z
</commit_message>
<xml_diff>
--- a/data/output/queens_dev_news.xlsx
+++ b/data/output/queens_dev_news.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H8"/>
+  <dimension ref="A1:H10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -473,17 +473,17 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Omnia Properties signs $45M refi loan with Valley for 57-unit building in Lower East Side</t>
+          <t>Top 2025 construction lenders for NYC ground up, rehab, conversion: PincusCo analysis</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>https://www.pincusco.com/omnia-properties-signs-45m-refi-loan-with-valley-for-57-unit-building-in-lower-east-side/</t>
+          <t>https://www.pincusco.com/top-2025-construction-lenders-for-nyc-ground-up-rehab-conversion-pincusco-analysis/</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Omnia Properties through the entity 185 Chrystie Street LLC as borrower signed a refi loan</t>
+          <t>New York City’s construction lending landscape in 2025 was defined by a significant investment of</t>
         </is>
       </c>
       <c r="D2" t="inlineStr"/>
@@ -500,24 +500,24 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Transfers 183 Chrystie Street (Credit - Cyclomedia) Omnia Properties through the entity 185 Chrystie Street LLC as borrower signed a refi loan with lender Valley National Bank through the entity Valley National Bank valued at $45 million for the four condominium units that make up the property at 183 Chrystie Street in Lower East Side, Manhattan, property at 183 Chrystie Street in Lower East Side, Manhattan, and property at 183 Chrystie Street in Lower East Side, Manhattan. The building has an alternate address of 4 Freeman Alley. The deal closed on April 28, 2026 and was recorded on May 8, 2026. The prior lender was Valley National Bank which held debt that had an original loan amount of $35 million. The four properties have 73,949 square feet of built space according to a PincusCo analysis of city data. The loan price per built square foot is $608.50 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) The signatory for Omnia Properties was David Paz .  The block On the tax block of 183 Chrystie Street, PincusCo has identified the owners of 11 of the </t>
+          <t>Chart_Frontpage Top Story Transfers New York City’s construction lending landscape in 2025 was defined by a significant investment of private capital, as specialized debt funds and regional banks aggressively filled the demand. While public agencies like the city’s Housing Development Corporation continued to provide significant volume, targeting affordable housing, the bulk of the overall activity is private and bank financing for new construction and substantial rehabilitation projects. Total volume for the top 105 lenders showed a marked concentration of power among a handful of private firms that managed to scale their operations even as interest rates remained elevated. Lenders provided borrowers $23.3 billion in 344 deals in 2025, compared to $17.1 billion in 275 deals in 2024, the PincusCo analysis showed. Methodology: PincusCo Media counted loans of $5 million and up, by their document date. If a lender provided a land loan along with the building loan and project loan, the land loan was included. Rehabilitation loans included two very different types of loans — one for property conversion for example an office building to residential, while the type of loan was to renovate</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Lightstone Group signs $19.2M refi with JLL for 34-unit UWS rental</t>
+          <t>Zhi Wen Li pays $7M to Viewgrow Capital Asset Management for 24-unit walkup in Chelsea</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>https://www.pincusco.com/lightstone-group-signs-19-2m-refi-with-jll-for-34-unit-uws-rental/</t>
+          <t>https://www.pincusco.com/zhi-wen-li-pays-7m-to-viewgrow-capital-asset-management-for-24-unit-walkup-in-chelsea/</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Lightstone Group through the entity 317 West 99th Street Associates LLC as borrower signed a</t>
+          <t>Zhi Wen Li through the entity Z&amp;L Enterprise LLC paid $7 million to Viewgrow Capital</t>
         </is>
       </c>
       <c r="D3" t="inlineStr"/>
@@ -534,24 +534,24 @@
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Transfers 317 West 99th Street (Credit - Cyclomedia) Lightstone Group through the entity 317 West 99th Street Associates LLC as borrower signed a refi loan with lender JLL through the entity JLL Real Estate Capital, LLC valued at $19.2 million for the 34-unit residential elevator building (D3) at 317 West 99th Street in Upper West Side, Manhattan. The deal closed on April 20, 2026 and was recorded on May 7, 2026. The prior lender was Sofia Einy which held debt that had an original loan amount of $10 million. The property has 47,851 square feet of built space according to a PincusCo analysis of city data. The loan price per built square foot is $400 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) The owner bought the property on May 19, 2020, for $18.5 million. The signatory for Lightstone Group was Joseph E. Teichman . The signatory for JLL was Omar Lopez . On the same day, Lightstone Group through the entity 309 West 99th Street Associates LLC as borrower signed a refi loan with lender JLL through the entity JLL Real Estate Capital, LLC valued at </t>
+          <t xml:space="preserve">Transfers 239 West 20th Street (Credit - Cyclomedia) Zhi Wen Li through the entity Z&amp;L Enterprise LLC paid $7 million to Viewgrow Capital Asset Management through the entity 239 West 20th Street, LLC for the 24-unit residential walkup building (C4) at 239 West 20th Street in Chelsea, Manhattan. The expected use is cash flowing. The deal closed on April 23, 2026 and was recorded on May 7, 2026. The property has 8,898 square feet of built space according to a PincusCo analysis of city data. The sale price per built square foot is $781 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) The seller bought the property on May 4, 2011, for $5.6 million. The signatory for Viewgrow Capital Asset Management was Neil Madsen . The signatory for Zhi Wen Li was Zhi Wen Li. The contract date was February 11, 2026. Prior sales, articles and revenue Prior to this transaction, PincusCo has no record that the buyer Zhi Wen Li had purchased any other properties and has no record it sold any properties over the past 24 months. The seller Viewgrow Capital Asset Management </t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>$5M refi signed with Liberty Mutual Insurance Company for LIC industrial</t>
+          <t>Albert Dayan sells mixed-use in Park Slope for $3.5M</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>https://www.pincusco.com/5m-refi-signed-with-liberty-mutual-insurance-company-for-lic-industrial/</t>
+          <t>https://www.pincusco.com/albert-dayan-sells-mixed-use-in-park-slope-for-3-5m/</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Salvatore DiLorenzo through the entity Jas 12th Street Holding LLC as borrower signed a refi</t>
+          <t>The entity Lake View Run LLC paid $3.5 million to Albert Dayan through the entity</t>
         </is>
       </c>
       <c r="D4" t="inlineStr"/>
@@ -568,24 +568,24 @@
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>Transfers 42-20 12th Street (Credit - Cyclomedia) Salvatore DiLorenzo through the entity Jas 12th Street Holding LLC as borrower signed a refi loan with lender Liberty Mutual Insurance Company valued at $5 million for the industrial building (F9) at 42-20 12th Street in Long Island City, Queens. The deal closed on April 20, 2026 and was recorded on May 7, 2026. The property has 9,764 square feet of built space and 7,077 square feet of additional air rights for a total buildable of 16,850 square feet according to a PincusCo analysis of city data. The loan price per built square foot is $512 and the price per buildable square foot is $296 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) The owner bought the property on December 20, 2021, for $3.3 million. The signatory for the borrower as member, was Salvatore J. DiLorenzo. The signatory for Liberty Mutual Insurance Company was Rachel Walsh . Prior sales, articles and revenue The 9,764-square-foot property generated revenue of $187,078 or $19 per square foot, according to the most recent income and ex</t>
+          <t xml:space="preserve">Transfers 323 5th Avenue (Credit - Cyclomedia) The entity Lake View Run LLC paid $3.5 million to Albert Dayan through the entity 323 5th Aretz LLC for the two-unit mixed-use building (S2) at 323 5th Avenue in Park Slope, Brooklyn. The deal closed on April 30, 2026 and was recorded on May 7, 2026. The property has 2,851 square feet of built space and 934 square feet of additional air rights for a total buildable of 3,789 square feet according to a PincusCo analysis of city data. The sale price per built square foot is $1,227 and the price per buildable square foot is $923 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) The seller bought the property on July 11, 2024, for $2.6 million. The signatory for Albert Dayan was Albert Dayan. The contract date was March 5, 2026. Prior sales, articles and revenue Prior to this transaction, PincusCo has no record that the buyer had purchased any other properties and has no record it sold any properties over the past 24 months. The seller Albert Dayan purchased eight properties in eight transactions for a total </t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Timber Equities signs $27.5M refi loan with JLL for 60-unit rental in Inwood</t>
+          <t>Ascenterra Development pays $4.7M for 4-family in Carroll Gardens</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>https://www.pincusco.com/timber-equities-signs-27-5m-refi-loan-with-jll-for-residential-elevator-in-inwood/</t>
+          <t>https://www.pincusco.com/ascenterra-development-pays-4-7m-for-4-family-in-carroll-gardens/</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Timber Equities through the entity 5055 Broadway L.P. as borrower signed a refi loan with</t>
+          <t>Ascenterra Development through the entity 32 Douglass, LLC paid $4.7 million for the four-unit building</t>
         </is>
       </c>
       <c r="D5" t="inlineStr"/>
@@ -602,24 +602,24 @@
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>Transfers 5055 Broadway (Credit - Cyclomedia) Timber Equities through the entity 5055 Broadway L.P. as borrower signed a refi loan with lender JLL through the entity Lrecs Holdings Iia, L.L.C. valued at $27.5 million for the 60-unit residential elevator building (D6) at 5055 Broadway in Inwood, Manhattan. On the lot, there is one active new building construction project, M00578593, for a 60-unit, 43,203 square-foot R-2 building. The project was submitted by Timber Equities and filed by Michel Perle with plans filed September 8, 2021 and permitted August 28, 2024. The deal closed on May 4, 2026 and was recorded on May 7, 2026. The prior lender was Bank Hapoalim which held debt that had an original loan amount of $21 million.The property has 44,651 square feet of built space according to a PincusCo analysis of city data. The loan price per built square foot is $615 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) The owner bought the property on October 29, 2020, for $3.4 million. The signatory for Timber Equities was Joseph Seidenfeld . The signatory</t>
+          <t>Transfers 32 Douglass Street (Credit - Cyclomedia) Ascenterra Development through the entity 32 Douglass, LLC paid $4.7 million for the four-unit building (C3) at 32 Douglass Street in Carroll Gardens, Brooklyn. The deal closed on April 29, 2026 and was recorded on May 7, 2026. The property has 3,060 square feet of built space and 1,950 square feet of additional air rights for a total buildable of 5,000 square feet according to a PincusCo analysis of city data. The sale price per built square foot is $1,519 and the price per buildable square foot is $930 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) The signatories for the sellers were Michael Mele, Thomas Mele, and Rita Mele. The signatory for Ascenterra Development was Aran Scott . The contract date was December 1, 2025. Prior sales, articles and revenue Prior to this transaction, PincusCo has records that the buyer Ascenterra Development purchased three properties in three transactions for a total of $11.9 million and has no record it sold any properties over the past 24 months. The seller Mic</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Timber Equities signs $35.6M refi loan with JLL for new 94-unit rental in Harlem</t>
+          <t>One Investment Management, RXR record transfer valued at $141.5M for 61 Broadway in FiDi</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>https://www.pincusco.com/timber-equities-signs-35-6m-refi-loan-with-jll-for-residential-elevator-in-harlem/</t>
+          <t>https://www.pincusco.com/one-investment-management-rxr-record-transfer-valued-at-141-5m-for-61-broadway-in-fidi/</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Timber Equities through the entity 2460 Fdb Lp as borrower signed a refi loan with</t>
+          <t>One Investment Management and RXR Realty through the entity RXR 61 Broadway LLC Investor Blocker</t>
         </is>
       </c>
       <c r="D6" t="inlineStr"/>
@@ -636,24 +636,24 @@
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>Transfers 2460 Frederick Douglass Boulevard (Credit - Cyclomedia) Timber Equities through the entity 2460 Fdb Lp as borrower signed a refi loan with lender JLL through the entity Lrecs Holdings Iia, L.L.C. valued at $35.6 million for the 94-unit residential elevator building (D6) at 2460 Frederick Douglass Boulevard in Harlem, Manhattan. On the lot, there was a new building construction project, M00686955, for a 94-unit, 89,166 square-foot residential (R-2) building. The project was submitted by Timber Equities and filed by Michel Perle with plans filed February 28, 2022 and permitted February 21, 2024. The loas closed on May 4, 2026 and was recorded on May 7, 2026. The prior lender was Webster Bank which held debt that had an original loan amount of $26.5 million.The property has 58,196 square feet of built space according to a PincusCo analysis of city data. The loan price per built square foot is $611 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) The owner bought the property on November 18, 2022, for $2.4 million. The signatory for Timber Equ</t>
+          <t>Top Story Transfers 61 Broadway (Credit - Cyclomedia) One Investment Management and RXR Realty through the entity RXR 61 Broadway LLC Investor Blocker JV LLC acquired control of the office building (O4) at 61 Broadway in the Financial District, Manhattan, from another RXR Realty entity, RXR 61 Broadway Owner LLC, in a transfer valued for tax purposes at $141.5 million. It’s unclear if that is the value of the equity on top the $475 million in construction and tax equity financing. RXR did not immediately respond to a request for comment. The parties paid about $4.6 million in transfer taxes. The deal closed on May 1, 2026 and was recorded on May 8, 2026. The property has 650,740 square feet of built space according to a PincusCo analysis of city data. The sale price per built square foot is $217 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) RXR bought the property on May 23, 2014, for $330 million. In 2023, RXR and prior lender Aareal considered a deed-in-lieu of foreclosure, but that was never consummated. That default apparently effectively wip</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Xiang Wei Zhou pays $4.2M to Santander Bank for office in Astoria</t>
+          <t>Saffayeh Group, Fouerti Realty close on previously reported $19M Chelsea conversion project</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>https://www.pincusco.com/xiang-wei-zhou-pays-4-2m-to-santander-bank-for-office-in-astoria/</t>
+          <t>https://www.pincusco.com/saffayeh-group-fouerti-realty-close-on-previously-reported-19m-chelsea-conversion-purchase/</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Xiang Wei Zhou through the entity Hung Yuen Holdings Inc. paid $4.2 million to Santander</t>
+          <t>Saffayeh Group and Fouerti Realty through the entity 324 West 15th Street LLC recorded their</t>
         </is>
       </c>
       <c r="D7" t="inlineStr"/>
@@ -670,24 +670,24 @@
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>Transfers 37-10 Broadway (Credit - Cyclomedia) Xiang Wei Zhou through the entity Hung Yuen Holdings Inc. paid $4.2 million to Santander Bank through the entity Santander Bank, N.A. for the office building (O5) at 37-10 Broadway in Astoria, Queens. The expected use is cash flowing. The deal closed on April 15, 2026 and was recorded on May 7, 2026. The property has 10,275 square feet of built space and 5,853 square feet of additional air rights for a total buildable of 16,110 square feet according to a PincusCo analysis of city data. The sale price per built square foot is $405 and the price per buildable square foot is $258 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) The seller bought the property on January 30, 2009, for $50.9 million. The signatory for Santander Bank was Michael Kuronen . The contract date was March 12, 2026. Prior sales, articles and revenue Prior to this transaction, PincusCo has no record that the buyer Xiang Wei Zhou had purchased any other properties and has no record it sold any properties over the past 24 months. The se</t>
+          <t>Transfers 324 West 15th Street (Credit - Cyclomedia) Saffayeh Group and Fouerti Realty through the entity 324 West 15th Street LLC recorded their $19 million purchase from the Corlears School for the school building (W8) at 324 West 15th Street in Chelsea, Manhattan. The expected use is conversion to residential. The deal closed on May 4, 2026 and was recorded on May 8, 2026. The property has 19,777 square feet of built space and 9,409 square feet of additional air rights for a total buildable of 29,176 square feet according to a PincusCo analysis of city data. The sale price per built square foot is $960 and the price per buildable square foot is $651 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) The signatory for Corlears School was David Egolf. The signatory for Saffayeh Group and Fouerti Realty was Elie Fouerti . The contract date was September 25, 2025. PincusCo exclusively reported this on April 14, 2026. Prior sales, articles and revenue Prior to this transaction, PincusCo has no record that the buyer Saffayeh Group had purchased any other</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Nilin Zhang, Qiao Chen pay $9.9M for industrial in Maspeth</t>
+          <t>Rester Management, Carthage up debt to $113.9M with Dwight Capital for 168-unit rental in Harlem</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>https://www.pincusco.com/nilin-zhang-qiao-chen-pay-9-9m-for-industrial-in-maspeth/</t>
+          <t>https://www.pincusco.com/rester-management-carthage-up-debt-to-113-9m-with-dwight-capital-for-168-unit-rental-in-harlem/</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Nilin Zhang and Qiao Chen through the entity 72-02 51st Ave Inc. paid $9.9 million</t>
+          <t>Rester Management and Carthage Advisors through the entity Carthage 124th L.P. as borrower signed financed</t>
         </is>
       </c>
       <c r="D8" t="inlineStr"/>
@@ -704,7 +704,75 @@
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>Transfers 72-02 51st Avenue (Credit -Cyclomedia) Nilin Zhang and Qiao Chen through the entity 72-02 51st Ave Inc. paid $9.9 million for the industrial building (E1) at 72-02 51st Avenue in Maspeth, Queens. The expected use is cash flowing. The deal closed on April 23, 2026 and was recorded on May 7, 2026. The property has 20,726 square feet of built space and 3,392 square feet of additional air rights for a total buildable of 24,230 square feet according to a PincusCo analysis of city data. The sale price per built square foot is $476 and the price per buildable square foot is $407 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) The signatory for Ciro Salvia and Paolo Salvia was Ciro Salvia and Paolo Salvia. The signatory for Nilin Zhang and Qiao Chen was Nilin Zhang. The contract date was December 22, 2025. Prior sales, articles and revenue Prior to this transaction, PincusCo has no record that the buyer Nilin Zhang had purchased any other properties and has no record it sold any properties over the past 24 months. The seller Ciro Salvia had not p</t>
+          <t>Transfers 2070 Adam C Powell Blvd (Credit - Cyclomedia) Rester Management and Carthage Advisors through the entity Carthage 124th L.P. as borrower signed financed for just under $9 million in additional debt loan with lender Dwight Capital through the entity Dwight Capital LLC for a total loan of $113.9 million for the 168-unit residential elevator building (D3) at 2070 Adam C. Powell Boulevard in Harlem, Manhattan. The deal closed on April 27, 2026 and was recorded on May 8, 2026. The prior lender was Dwight Capital which held debt that had an original loan amount of $105 million.The property has 165,607 square feet of built space according to a PincusCo analysis of city data. The loan price per built square foot is $687 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) The owner bought the property on December 19, 2017, for $27.8 million. The signatory for Rester Management and Carthage Advisors was Sari Drazin . Prior sales, articles and revenue The owner according to the Department of Housing Preservation and Development is Ari Drazin, head offic</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>G Holdings signs $63M refi with Brookfield for hotel in Garment District</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>https://www.pincusco.com/g-holdings-signs-63m-refi-with-brookfield-for-hotel-in-garment-district/</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>G Holdings through the entity Granite Park LLC as borrower signed a refi loan with</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr"/>
+      <c r="E9" t="inlineStr"/>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>PincusCo</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>PincusCo - Home</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>Transfers 117 West 39th Street (Credit - Cyclomedia) G Holdings through the entity Granite Park LLC as borrower signed a refi loan with lender Brookfield Properties through the entity B Ul LLC valued at $63 million for the Courtyard by Marriott New York Manhattan/Times Square hotel building (H3) at 114 West 40th Street with an alternate address of 117 West 39th Street in the Garment District, Manhattan. The deal closed on April 27, 2026 and was recorded on May 8, 2026. The prior lender was Bank Hapoalim which held debt that had an original loan amount of $71 million. The property has 126,398 square feet of built space according to a PincusCo analysis of city data. The loan price per built square foot is $498 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) The signatory for G Holdings was Ronnie Gross . The signatory for Brookfield Properties was Laura Stepp . Prior sales, articles and revenue The 126,398-square-foot property generated revenue of $25 million or $198 per square foot, according to the most recent income and expense figures. The proper</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Firebird Grove sells mixed-use in Boerum Hill for $3M</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>https://www.pincusco.com/firebird-grove-sells-mixed-use-in-boerum-hill-for-3m/</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Joseph Daskal through the entity 32 4th Avenue LLC paid $3 million to Firebird Grove</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr"/>
+      <c r="E10" t="inlineStr"/>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>PincusCo</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>PincusCo - Home</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>Transfers 40 4th Avenue (Credit - Cyclomedia) Joseph Daskal through the entity 32 4th Avenue LLC paid $3 million to Firebird Grove through the entity OR 40 Fourth, LLC for the four-unit mixed-use building (S9) at 40 4th Avenue in Boerum Hill, Brooklyn. The deal closed on April 22, 2026 and was recorded on May 8, 2026. The property has 4,000 square feet of built space and 4,424 square feet of additional air rights for a total buildable of 8,428 square feet according to a PincusCo analysis of city data. The sale price per built square foot is $762 and the price per buildable square foot is $361 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) The seller bought the property on September 22, 2020, for $2.4 million. The signatory for Firebird Grove was Adam Semler . The signatory for Joseph Daskal was Joseph Daskal. The contract date was March 10, 2026. Prior sales, articles and revenue Prior to this transaction, PincusCo has records that the buyer Joseph Daskal purchased one property in one transaction for a total of $4.4 million and has no record it so</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto update queens news 2026-05-13T15:12:50Z
</commit_message>
<xml_diff>
--- a/data/output/queens_dev_news.xlsx
+++ b/data/output/queens_dev_news.xlsx
@@ -473,17 +473,17 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Top 2025 construction lenders for NYC ground up, rehab, conversion: PincusCo analysis</t>
+          <t>FBL Development pays $11.2M to Kenneth Kerim for likely dev site in Sunnyside</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>https://www.pincusco.com/top-2025-construction-lenders-for-nyc-ground-up-rehab-conversion-pincusco-analysis/</t>
+          <t>https://www.pincusco.com/fbl-development-pays-11-2m-to-kenneth-kerim-for-likely-dev-site-in-sunnyside/</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>New York City’s construction lending landscape in 2025 was defined by a significant investment of</t>
+          <t>FBL Development through the entity Amara 3939 LLC paid $11.2 million to Kenneth Kerim through</t>
         </is>
       </c>
       <c r="D2" t="inlineStr"/>
@@ -500,24 +500,24 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>Chart_Frontpage Top Story Transfers New York City’s construction lending landscape in 2025 was defined by a significant investment of private capital, as specialized debt funds and regional banks aggressively filled the demand. While public agencies like the city’s Housing Development Corporation continued to provide significant volume, targeting affordable housing, the bulk of the overall activity is private and bank financing for new construction and substantial rehabilitation projects. Total volume for the top 105 lenders showed a marked concentration of power among a handful of private firms that managed to scale their operations even as interest rates remained elevated. Lenders provided borrowers $23.3 billion in 344 deals in 2025, compared to $17.1 billion in 275 deals in 2024, the PincusCo analysis showed. Methodology: PincusCo Media counted loans of $5 million and up, by their document date. If a lender provided a land loan along with the building loan and project loan, the land loan was included. Rehabilitation loans included two very different types of loans — one for property conversion for example an office building to residential, while the type of loan was to renovate</t>
+          <t>Transfers 39-39 Queens Blvd (Credit - Cyclomedia) FBL Development through the entity Amara 3939 LLC paid $11.2 million to Kenneth Kerim through the entity Kd Kerim LLC for the retail property at 39-39 Queens Boulevard in Sunnyside, Queens. The expected use is ground up development. The deal closed on April 17, 2026 and was recorded on May 12, 2026. The property has 9,500 square feet of built space according to a PincusCo analysis of city data. The sale price per built square foot is $1,174 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) The signatory for Kenneth Kerim was Kenneth D. Kerim . The signatory for FBL Development was Yong Chen . The contract date was February 26, 2026. Prior sales, articles and revenue Prior to this transaction, PincusCo has records that the buyer FBL Development purchased two properties in one transaction for a total of $5.6 million and has no record it sold any properties over the past 24 months. The seller Kenneth Kerim had not purchased any other properties and had not sold any properties over the same time period. T</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Zhi Wen Li pays $7M to Viewgrow Capital Asset Management for 24-unit walkup in Chelsea</t>
+          <t>Joel Basch pays $17.2M to Lichtschein family for treatment facility building in Coney Island</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>https://www.pincusco.com/zhi-wen-li-pays-7m-to-viewgrow-capital-asset-management-for-24-unit-walkup-in-chelsea/</t>
+          <t>https://www.pincusco.com/joel-basch-pays-17-2m-to-lichtschein-family-for-treatment-facility-building-in-coney-island/</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Zhi Wen Li through the entity Z&amp;L Enterprise LLC paid $7 million to Viewgrow Capital</t>
+          <t>Joel Basch through the entity Surf Propco LLC paid $17.2 million to the Lichtschein family</t>
         </is>
       </c>
       <c r="D3" t="inlineStr"/>
@@ -534,24 +534,24 @@
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Transfers 239 West 20th Street (Credit - Cyclomedia) Zhi Wen Li through the entity Z&amp;L Enterprise LLC paid $7 million to Viewgrow Capital Asset Management through the entity 239 West 20th Street, LLC for the 24-unit residential walkup building (C4) at 239 West 20th Street in Chelsea, Manhattan. The expected use is cash flowing. The deal closed on April 23, 2026 and was recorded on May 7, 2026. The property has 8,898 square feet of built space according to a PincusCo analysis of city data. The sale price per built square foot is $781 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) The seller bought the property on May 4, 2011, for $5.6 million. The signatory for Viewgrow Capital Asset Management was Neil Madsen . The signatory for Zhi Wen Li was Zhi Wen Li. The contract date was February 11, 2026. Prior sales, articles and revenue Prior to this transaction, PincusCo has no record that the buyer Zhi Wen Li had purchased any other properties and has no record it sold any properties over the past 24 months. The seller Viewgrow Capital Asset Management </t>
+          <t xml:space="preserve">Top Story Transfers 2316 Surf Avenue (Credit - Cyclomedia Joel Basch through the entity Surf Propco LLC paid $17.2 million to the Lichtschein family including Robert, David, and Raphael, through the entity King David Of Brooklyn for the former nursing home at 2316 Surf Avenue in Coney Island, Brooklyn. The expected use is to rent the property to an affiliated operating company, Surfpoint Recovery LLC, which provides drug treatment services. The deal closed on May 5, 2026 and was recorded on May 12, 2026. The property has 40,344 square feet of built space according to a PincusCo analysis of city data. The sale price per built square foot is $426 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) The signatory for the Lichtschein family was Raphael Lichtschein. The signatory for Joel Basch was Joel Basch. The contract date was March 26, 2026. Joel Basch and Liberty One Group member Yosef Rabinowitz are 40% owner of Surfpoint Recovery LLC which is the operator of the rehab treatment facility. Surfpoint Recovery has an address at the office building 5518 </t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Albert Dayan sells mixed-use in Park Slope for $3.5M</t>
+          <t>Sholom Adelman pays $3.2M for 3-story office in Midwood</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>https://www.pincusco.com/albert-dayan-sells-mixed-use-in-park-slope-for-3-5m/</t>
+          <t>https://www.pincusco.com/sholom-adelman-pays-3-2m-for-3-story-office-in-midwood/</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>The entity Lake View Run LLC paid $3.5 million to Albert Dayan through the entity</t>
+          <t>Sholom Adelman through the entity 1915-1917 Ocean Avenue LLC paid $3.2 million to Gennady Kiselman</t>
         </is>
       </c>
       <c r="D4" t="inlineStr"/>
@@ -568,24 +568,24 @@
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Transfers 323 5th Avenue (Credit - Cyclomedia) The entity Lake View Run LLC paid $3.5 million to Albert Dayan through the entity 323 5th Aretz LLC for the two-unit mixed-use building (S2) at 323 5th Avenue in Park Slope, Brooklyn. The deal closed on April 30, 2026 and was recorded on May 7, 2026. The property has 2,851 square feet of built space and 934 square feet of additional air rights for a total buildable of 3,789 square feet according to a PincusCo analysis of city data. The sale price per built square foot is $1,227 and the price per buildable square foot is $923 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) The seller bought the property on July 11, 2024, for $2.6 million. The signatory for Albert Dayan was Albert Dayan. The contract date was March 5, 2026. Prior sales, articles and revenue Prior to this transaction, PincusCo has no record that the buyer had purchased any other properties and has no record it sold any properties over the past 24 months. The seller Albert Dayan purchased eight properties in eight transactions for a total </t>
+          <t>Transfers 1915-1917 Ocean Avenue (Credit - Cyclomedia) Sholom Adelman through the entity 1915-1917 Ocean Avenue LLC paid $3.2 million to Gennady Kiselman through the entity 1915 Ocean Avenue, LLC for the property three-story office building at 1915-1917 Ocean Avenue in Midwood, Brooklyn. The expected use is cash flowing. The deal closed on May 6, 2026 and was recorded on May 12, 2026. The property has 16,500 square feet of built space according to a PincusCo analysis of city data. The sale price per built square foot is $193 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) The signatory for Gennady Kiselman was Mikhail Litt . The signatory for Sholom Adelman was Sholom Adelman. The contract date was December 25, 2025. Prior sales, articles and revenue Prior to this transaction, PincusCo has no record that the buyer Sholom Adelman had purchased any other properties and has no record it sold any properties over the past 24 months. The seller Gennady Kiselman had not purchased any other properties and had not sold any properties over the same time peri</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Ascenterra Development pays $4.7M for 4-family in Carroll Gardens</t>
+          <t>Lin Qiong Fan pays $4.4M for dev site in Whitestone</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>https://www.pincusco.com/ascenterra-development-pays-4-7m-for-4-family-in-carroll-gardens/</t>
+          <t>https://www.pincusco.com/lin-qiong-fan-pays-4-4m-to-temple-gates-of-prayer-congregation-shaarai-tefilla-for-in-whitestone/</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Ascenterra Development through the entity 32 Douglass, LLC paid $4.7 million for the four-unit building</t>
+          <t>Lin Qiong Fan through the entity 145-17 Willets Point Development LLC paid $4.4 million to</t>
         </is>
       </c>
       <c r="D5" t="inlineStr"/>
@@ -602,24 +602,24 @@
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>Transfers 32 Douglass Street (Credit - Cyclomedia) Ascenterra Development through the entity 32 Douglass, LLC paid $4.7 million for the four-unit building (C3) at 32 Douglass Street in Carroll Gardens, Brooklyn. The deal closed on April 29, 2026 and was recorded on May 7, 2026. The property has 3,060 square feet of built space and 1,950 square feet of additional air rights for a total buildable of 5,000 square feet according to a PincusCo analysis of city data. The sale price per built square foot is $1,519 and the price per buildable square foot is $930 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) The signatories for the sellers were Michael Mele, Thomas Mele, and Rita Mele. The signatory for Ascenterra Development was Aran Scott . The contract date was December 1, 2025. Prior sales, articles and revenue Prior to this transaction, PincusCo has records that the buyer Ascenterra Development purchased three properties in three transactions for a total of $11.9 million and has no record it sold any properties over the past 24 months. The seller Mic</t>
+          <t>Transfers 145-17 Willets Point Blvd (Credit - Cyclomedia) Lin Qiong Fan through the entity 145-17 Willets Point Development LLC paid $4.4 million to Temple Gates of Prayer Congregation Shaarai Tefilla for the development site at 145-17 Willets Point Boulevard in Whitestone, Queens. The expected use is ground up development. The deal closed on April 21, 2026 and was recorded on May 12, 2026. The property has zero square feet of built space on a 18,910 square foot parcel, according to a PincusCo analysis of city data. The seller bought the property on December 16, 2019, for $5.3 million. The signatory for Temple Gates of Prayer Congregation Shaarai Tefilla was Barry Grodenchik. The signatory for Lin Qiong Fan was Lin Qiong Fan. The contract date was December 9, 2024. Prior sales, articles and revenue Prior to this transaction, PincusCo has no record that the buyer Lin Qiong Fan had purchased any other properties and has no record it sold any properties over the past 24 months. The seller Temple Gates of Prayer Congregation Shaarai Tefilla had not purchased any other properties and had not sold any properties over the same time period. The property</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>One Investment Management, RXR record transfer valued at $141.5M for 61 Broadway in FiDi</t>
+          <t>Congregation Machne Chaim signs $20M loan with Webster Bank for school in Bensonhurst</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>https://www.pincusco.com/one-investment-management-rxr-record-transfer-valued-at-141-5m-for-61-broadway-in-fidi/</t>
+          <t>https://www.pincusco.com/congregation-machne-chaim-signs-20m-refi-with-webster-bank-for-school-in-bensonhurst/</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>One Investment Management and RXR Realty through the entity RXR 61 Broadway LLC Investor Blocker</t>
+          <t>Congregation Machne Chaim through the entity Bais Sarah Educational Center For Girls as borrower signed</t>
         </is>
       </c>
       <c r="D6" t="inlineStr"/>
@@ -636,24 +636,24 @@
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>Top Story Transfers 61 Broadway (Credit - Cyclomedia) One Investment Management and RXR Realty through the entity RXR 61 Broadway LLC Investor Blocker JV LLC acquired control of the office building (O4) at 61 Broadway in the Financial District, Manhattan, from another RXR Realty entity, RXR 61 Broadway Owner LLC, in a transfer valued for tax purposes at $141.5 million. It’s unclear if that is the value of the equity on top the $475 million in construction and tax equity financing. RXR did not immediately respond to a request for comment. The parties paid about $4.6 million in transfer taxes. The deal closed on May 1, 2026 and was recorded on May 8, 2026. The property has 650,740 square feet of built space according to a PincusCo analysis of city data. The sale price per built square foot is $217 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) RXR bought the property on May 23, 2014, for $330 million. In 2023, RXR and prior lender Aareal considered a deed-in-lieu of foreclosure, but that was never consummated. That default apparently effectively wip</t>
+          <t xml:space="preserve">Transfers 6101 16th Avenue (Credit - Cyclomedia) Congregation Machne Chaim through the entity Bais Sarah Educational Center For Girls as borrower signed a loan with lender Webster Bank through the entity Webster Bank, National Association valued at $20 million for the specialty building (W2) at 6101 16th Avenue in Bensonhurst, Brooklyn. The deal closed on April 30, 2026 and was recorded on May 11, 2026. The prior lender was Bank of Princeton which held debt that had an original loan amount of $5 million. The property has 61,148 square feet of built space according to a PincusCo analysis of city data. The loan price per built square foot is $327 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) The owner bought the property on November 5, 2003, for $7 million. The signatory for Congregation Machne Chaim was Nuchem Klein . The signatory for Webster Bank was Lisa Congemi . The property The specialty building in Bensonhurst has 61,148 square feet of built space according to a PincusCo analysis of city data. The parcel has frontage of 200 feet and is 190 </t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Saffayeh Group, Fouerti Realty close on previously reported $19M Chelsea conversion project</t>
+          <t>David Chan files plans for 3-story retail, school, medical building in Maspeth</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>https://www.pincusco.com/saffayeh-group-fouerti-realty-close-on-previously-reported-19m-chelsea-conversion-purchase/</t>
+          <t>https://www.pincusco.com/david-chan-files-plans-for-3-story-retail-school-medical-building-in-maspeth/</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Saffayeh Group and Fouerti Realty through the entity 324 West 15th Street LLC recorded their</t>
+          <t>David Chan submitted a new building construction project for a 11,831-square-foot retail and commercial building</t>
         </is>
       </c>
       <c r="D7" t="inlineStr"/>
@@ -670,24 +670,24 @@
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>Transfers 324 West 15th Street (Credit - Cyclomedia) Saffayeh Group and Fouerti Realty through the entity 324 West 15th Street LLC recorded their $19 million purchase from the Corlears School for the school building (W8) at 324 West 15th Street in Chelsea, Manhattan. The expected use is conversion to residential. The deal closed on May 4, 2026 and was recorded on May 8, 2026. The property has 19,777 square feet of built space and 9,409 square feet of additional air rights for a total buildable of 29,176 square feet according to a PincusCo analysis of city data. The sale price per built square foot is $960 and the price per buildable square foot is $651 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) The signatory for Corlears School was David Egolf. The signatory for Saffayeh Group and Fouerti Realty was Elie Fouerti . The contract date was September 25, 2025. PincusCo exclusively reported this on April 14, 2026. Prior sales, articles and revenue Prior to this transaction, PincusCo has no record that the buyer Saffayeh Group had purchased any other</t>
+          <t>Development 50-53 69th Street axonometric diagram (Credit - Chang Hwa Tan architect via DOB) David Chan submitted a new building construction project for a 11,831-square-foot retail and commercial building at 50-53 69th Street in Maspeth, Queens. The plan was filed on May 11, 2026. It calls for the construction of a 39-foot-tall, three-story building and was filed with the New York City Department of Buildings under job number Q01381850. The project is described in the filing as: proposed a 3-story commercial building. The applicant is the Registered Architect Chang Tan of Tan Architect P.C. The plans call for 2,188 square feet of retail on the ground floor and 2,379 square feet in the cellar; a school or daycare on the 4,665 square-foot second floor; and an ambulatory health facility on the 2,207-square-foot third floor. Sai Ho Chan and David Chan bought the property for $1.55 million in 2025. The neighborhood</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Rester Management, Carthage up debt to $113.9M with Dwight Capital for 168-unit rental in Harlem</t>
+          <t>Stagg Group files plans for 68 units in Astoria</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>https://www.pincusco.com/rester-management-carthage-up-debt-to-113-9m-with-dwight-capital-for-168-unit-rental-in-harlem/</t>
+          <t>https://www.pincusco.com/stagg-group-files-plans-for-68-units-in-astoria/</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Rester Management and Carthage Advisors through the entity Carthage 124th L.P. as borrower signed financed</t>
+          <t>Stagg Group submitted a new building construction project for a 68-unit, 82,960-square-foot residential (R-2) building</t>
         </is>
       </c>
       <c r="D8" t="inlineStr"/>
@@ -704,24 +704,24 @@
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>Transfers 2070 Adam C Powell Blvd (Credit - Cyclomedia) Rester Management and Carthage Advisors through the entity Carthage 124th L.P. as borrower signed financed for just under $9 million in additional debt loan with lender Dwight Capital through the entity Dwight Capital LLC for a total loan of $113.9 million for the 168-unit residential elevator building (D3) at 2070 Adam C. Powell Boulevard in Harlem, Manhattan. The deal closed on April 27, 2026 and was recorded on May 8, 2026. The prior lender was Dwight Capital which held debt that had an original loan amount of $105 million.The property has 165,607 square feet of built space according to a PincusCo analysis of city data. The loan price per built square foot is $687 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) The owner bought the property on December 19, 2017, for $27.8 million. The signatory for Rester Management and Carthage Advisors was Sari Drazin . Prior sales, articles and revenue The owner according to the Department of Housing Preservation and Development is Ari Drazin, head offic</t>
+          <t>Development 29-12 Hoyt Avenue axonometric diagram (Credit Minkuk Kim architect via DOB) Stagg Group submitted a new building construction project for a 68-unit, 82,960-square-foot residential (R-2) building at 29-12 Hoyt Avenue South in Astoria, Queens. The plan was filed on May 11, 2026. It calls for the construction of a 94-foot-tall, nine-story building and was filed with the New York City Department of Buildings under job number Q01395583. The project is described in the filing as: construction of a new 9-story building consisting of 68 apartment units.. The applicant is the Registered Architect Minkuk Kim of MK Architect Studio. Mark Stagg of Stagg Group submitted the plans. Property records show the building is owned by an entity that appears unrelated to Stagg Group. The most recent sale was in 2012 for $830,000. The neighborhood In Astoria, The bulk, or 36 percent of the 40.2 million square feet of commercial built space are walkup buildings, with elevator buildings next occupying 31 percent of the space. In sales, Astoria has near average sales volume among other neighborhoods with $851.5 million in sales volume in the last two years and is the 2nd highest in Queens. For d</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>G Holdings signs $63M refi with Brookfield for hotel in Garment District</t>
+          <t>Prospect Development files plans for 9 apartments on single floor in Garment District commercial</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>https://www.pincusco.com/g-holdings-signs-63m-refi-with-brookfield-for-hotel-in-garment-district/</t>
+          <t>https://www.pincusco.com/prospect-development-files-plans-for-9-apartments-on-single-floor-in-garment-district-commercial/</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>G Holdings through the entity Granite Park LLC as borrower signed a refi loan with</t>
+          <t>Prospect Development Group submitted a major alteration application for a rehab of 109,416-square-foot commercial building</t>
         </is>
       </c>
       <c r="D9" t="inlineStr"/>
@@ -738,24 +738,24 @@
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>Transfers 117 West 39th Street (Credit - Cyclomedia) G Holdings through the entity Granite Park LLC as borrower signed a refi loan with lender Brookfield Properties through the entity B Ul LLC valued at $63 million for the Courtyard by Marriott New York Manhattan/Times Square hotel building (H3) at 114 West 40th Street with an alternate address of 117 West 39th Street in the Garment District, Manhattan. The deal closed on April 27, 2026 and was recorded on May 8, 2026. The prior lender was Bank Hapoalim which held debt that had an original loan amount of $71 million. The property has 126,398 square feet of built space according to a PincusCo analysis of city data. The loan price per built square foot is $498 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) The signatory for G Holdings was Ronnie Gross . The signatory for Brookfield Properties was Laura Stepp . Prior sales, articles and revenue The 126,398-square-foot property generated revenue of $25 million or $198 per square foot, according to the most recent income and expense figures. The proper</t>
+          <t>Development 229 West 36th Street (Credit - Google Earth) Prospect Development Group submitted a major alteration application for a rehab of 109,416-square-foot commercial building (COM) at 229 West 36th Street in the Garment District, Manhattan. The plan was filed on May 6, 2026. It calls for a conversion of the 12th floor of the 121-foot-tall, twelve-story building and was filed with the New York City Department of Buildings under job number M01395574. The project is described in the filing as: application filed to convert the twelfth (12th) floor of the existing twelve (12)-story commercial building to residential use as per plans. The applicant is the Registered Architect Kao Hwa Lee of Kao Hwa Lee Architects Pc. Konstantin Gubareff of Prospect Development Group submitted the plans. Cayre Equities and A&amp;H Acquisitions bought the building for $19.2 million in May 2025. The neighborhood In Garment District, The majority, or 69 percent of the 52.3 million square feet of commercial built space are office buildings, with hotel buildings next occupying 13 percent of the space. In sales, Garment District has the 10th highest sale turnover among other neighborhoods in the city with $1.4</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Firebird Grove sells mixed-use in Boerum Hill for $3M</t>
+          <t>Stellar Management signs $77.5M refi loan with Nuveen for hotel in Upper West Side</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>https://www.pincusco.com/firebird-grove-sells-mixed-use-in-boerum-hill-for-3m/</t>
+          <t>https://www.pincusco.com/stellar-management-signs-77-5m-refi-loan-with-nuveen-for-hotel-in-upper-west-side/</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Joseph Daskal through the entity 32 4th Avenue LLC paid $3 million to Firebird Grove</t>
+          <t>Stellar Management through the entity Windermere Owners LLC as borrower signed a refi loan with</t>
         </is>
       </c>
       <c r="D10" t="inlineStr"/>
@@ -772,7 +772,7 @@
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>Transfers 40 4th Avenue (Credit - Cyclomedia) Joseph Daskal through the entity 32 4th Avenue LLC paid $3 million to Firebird Grove through the entity OR 40 Fourth, LLC for the four-unit mixed-use building (S9) at 40 4th Avenue in Boerum Hill, Brooklyn. The deal closed on April 22, 2026 and was recorded on May 8, 2026. The property has 4,000 square feet of built space and 4,424 square feet of additional air rights for a total buildable of 8,428 square feet according to a PincusCo analysis of city data. The sale price per built square foot is $762 and the price per buildable square foot is $361 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) The seller bought the property on September 22, 2020, for $2.4 million. The signatory for Firebird Grove was Adam Semler . The signatory for Joseph Daskal was Joseph Daskal. The contract date was March 10, 2026. Prior sales, articles and revenue Prior to this transaction, PincusCo has records that the buyer Joseph Daskal purchased one property in one transaction for a total of $4.4 million and has no record it so</t>
+          <t>Transfers 666 West End Avenue (Credit - Cyclomedia) Stellar Management through the entity Windermere Owners LLC as borrower signed a refi loan with lender Nuveen through the entity Teachers Insurance And Annuity Association Of valued at $77.5 million for the hotel building (H6) at 666 West End Avenue in Upper West Side, Manhattan. The deal closed on May 1, 2026 and was recorded on May 7, 2026. The prior lender was Adler &amp; Stachenfeld registered which held debt that had an original loan amount of $95 million.The property has 279,316 square feet of built space according to a PincusCo analysis of city data. The loan price per built square foot is $277 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) The owner bought the property on November 18, 2010, for $68.5 million. The signatory for Stellar Management was Adam Roman . The signatory for Nuveen was Grace A. Cole . Prior sales, articles and revenue The owners according to the Department of Housing Preservation and Development includes Smajlje Srdanovic, head officer and Arianit Jakupaj, officer. The b</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto update queens news 2026-05-14T14:38:02Z
</commit_message>
<xml_diff>
--- a/data/output/queens_dev_news.xlsx
+++ b/data/output/queens_dev_news.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H10"/>
+  <dimension ref="A1:H7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -473,17 +473,17 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>FBL Development pays $11.2M to Kenneth Kerim for likely dev site in Sunnyside</t>
+          <t>Joseph Fazzia pays $4.5M for mixed-use in Rossville</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>https://www.pincusco.com/fbl-development-pays-11-2m-to-kenneth-kerim-for-likely-dev-site-in-sunnyside/</t>
+          <t>https://www.pincusco.com/joseph-fazzia-pays-4-5m-for-mixed-use-in-rossville/</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>FBL Development through the entity Amara 3939 LLC paid $11.2 million to Kenneth Kerim through</t>
+          <t>Joseph Fazzia paid $4.5 million to Michael Freundlich through the entity 2200 A.K.R. Associates LLC</t>
         </is>
       </c>
       <c r="D2" t="inlineStr"/>
@@ -500,24 +500,24 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>Transfers 39-39 Queens Blvd (Credit - Cyclomedia) FBL Development through the entity Amara 3939 LLC paid $11.2 million to Kenneth Kerim through the entity Kd Kerim LLC for the retail property at 39-39 Queens Boulevard in Sunnyside, Queens. The expected use is ground up development. The deal closed on April 17, 2026 and was recorded on May 12, 2026. The property has 9,500 square feet of built space according to a PincusCo analysis of city data. The sale price per built square foot is $1,174 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) The signatory for Kenneth Kerim was Kenneth D. Kerim . The signatory for FBL Development was Yong Chen . The contract date was February 26, 2026. Prior sales, articles and revenue Prior to this transaction, PincusCo has records that the buyer FBL Development purchased two properties in one transaction for a total of $5.6 million and has no record it sold any properties over the past 24 months. The seller Kenneth Kerim had not purchased any other properties and had not sold any properties over the same time period. T</t>
+          <t>Transfers 2200 Arthur Kill Road (Credit - Cyclomedia) Joseph Fazzia paid $4.5 million to Michael Freundlich through the entity 2200 A.K.R. Associates LLC for the mixed-use building (K2) at 2200 Arthur Kill Road in Rossville, Staten Island. The deal closed on March 20, 2026 and was recorded on May 13, 2026. The property has 12,480 square feet of built space and 88,830 square feet of additional air rights for a total buildable of 101,520 square feet according to a PincusCo analysis of city data. The sale price per built square foot is $360 and the price per buildable square foot is $44 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) The signatory for Michael Freundlich was Michael Freundlich. The signatory for Joseph Fazzia was Joseph Fazzia Sr. Prior sales, articles and revenue Prior to this transaction, PincusCo has records that the buyer Joseph Fazzia purchased three properties in one transaction for a total of $7.2 million and has no record it sold any properties over the past 24 months. The seller Michael Freundlich had not purchased any other p</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Joel Basch pays $17.2M to Lichtschein family for treatment facility building in Coney Island</t>
+          <t>Safehold Inc. files plans for 32 apartments on single floor of office building in Midtown West</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>https://www.pincusco.com/joel-basch-pays-17-2m-to-lichtschein-family-for-treatment-facility-building-in-coney-island/</t>
+          <t>https://www.pincusco.com/safehold-inc-files-conversion-plans-for-32-units-on-single-floor-in-midtown-west/</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Joel Basch through the entity Surf Propco LLC paid $17.2 million to the Lichtschein family</t>
+          <t>Elisha Blechner of Safehold Inc. submitted a major alteration application for the conversion of a</t>
         </is>
       </c>
       <c r="D3" t="inlineStr"/>
@@ -534,24 +534,24 @@
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Top Story Transfers 2316 Surf Avenue (Credit - Cyclomedia Joel Basch through the entity Surf Propco LLC paid $17.2 million to the Lichtschein family including Robert, David, and Raphael, through the entity King David Of Brooklyn for the former nursing home at 2316 Surf Avenue in Coney Island, Brooklyn. The expected use is to rent the property to an affiliated operating company, Surfpoint Recovery LLC, which provides drug treatment services. The deal closed on May 5, 2026 and was recorded on May 12, 2026. The property has 40,344 square feet of built space according to a PincusCo analysis of city data. The sale price per built square foot is $426 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) The signatory for the Lichtschein family was Raphael Lichtschein. The signatory for Joel Basch was Joel Basch. The contract date was March 26, 2026. Joel Basch and Liberty One Group member Yosef Rabinowitz are 40% owner of Surfpoint Recovery LLC which is the operator of the rehab treatment facility. Surfpoint Recovery has an address at the office building 5518 </t>
+          <t>Development 135 West 50th Street (Credit - Google Earth) Elisha Blechner of Safehold Inc. submitted a major alteration application for the conversion of a single floor of the commercial office (COM) building at 135 West 50th Street in Midtown West, Manhattan from commercial to 32 apartments. The plan was filed on May 12, 2026. It calls for work in the 248-foot-tall, 23-story building and was filed with the New York City Department of Buildings under job number M01400622. The project is described in the filing as: MPP project-000000631. Filing for conversion of the 12th floor from commercial to residential use as shown, no change to the rest of the building. The applicant is the Registered Architect Ambrose Aliaga Kelly of Gensler. This is the first such application to convert a portion of the building to residential, a PincusCo review shows. In October 2024, PincusCo reported that Texas-based Thakkar Developers through the entity TD 135 West 50 LLC paid $8.5 million to UBS Realty Investors through the entity 135 West 50th Street Lessee LLC for the ground lease that controls the office building (O4) at 135 West 50th Street in Midtown West, Manhattan. The fee is owned by Safehold Inc</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Sholom Adelman pays $3.2M for 3-story office in Midwood</t>
+          <t>Shanshan Peng files plans for 26 units in Long Island City</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>https://www.pincusco.com/sholom-adelman-pays-3-2m-for-3-story-office-in-midwood/</t>
+          <t>https://www.pincusco.com/shanshan-peng-files-plans-for-26-units-in-long-island-city/</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Sholom Adelman through the entity 1915-1917 Ocean Avenue LLC paid $3.2 million to Gennady Kiselman</t>
+          <t>Shanshan Peng submitted a new building construction project for a 26-unit, 27,496-square-foot residential (R-2) building</t>
         </is>
       </c>
       <c r="D4" t="inlineStr"/>
@@ -568,24 +568,24 @@
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>Transfers 1915-1917 Ocean Avenue (Credit - Cyclomedia) Sholom Adelman through the entity 1915-1917 Ocean Avenue LLC paid $3.2 million to Gennady Kiselman through the entity 1915 Ocean Avenue, LLC for the property three-story office building at 1915-1917 Ocean Avenue in Midwood, Brooklyn. The expected use is cash flowing. The deal closed on May 6, 2026 and was recorded on May 12, 2026. The property has 16,500 square feet of built space according to a PincusCo analysis of city data. The sale price per built square foot is $193 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) The signatory for Gennady Kiselman was Mikhail Litt . The signatory for Sholom Adelman was Sholom Adelman. The contract date was December 25, 2025. Prior sales, articles and revenue Prior to this transaction, PincusCo has no record that the buyer Sholom Adelman had purchased any other properties and has no record it sold any properties over the past 24 months. The seller Gennady Kiselman had not purchased any other properties and had not sold any properties over the same time peri</t>
+          <t>Development 37-31 29th Street schematic plan and elevations (Credit - Murat Mutlu architect via DOB) Shanshan Peng submitted a new building construction project for a 26-unit, 27,496-square-foot residential (R-2) building at 37-31 29 Street in Long Island City, Queens. The plan was filed on May 12, 2026. It calls for the construction of a 79-foot-tall, seven-story building and was filed with the New York City Department of Buildings under job number Q01381898. The project is described in the filing as: propose a 7-story mixed-use building comprising commercial spaces and 26 class a apartments with 20% of qualifying affordable housing units (uap development). obtain a new certificate of occupancy.. The applicant is the Registered Architect Murat Mutlu of Inoa Architecture Inc. 37-31 29th Street The neighborhood In Long Island City, The bulk, or 32 percent of the 60.1 million square feet of commercial built space are industrial buildings, with elevator buildings next occupying 31 percent of the space. In sales, Long Island City has near average sales volume among other neighborhoods with $1.1 billion in sales volume in the last two years and is the highest in Queens. For development,</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Lin Qiong Fan pays $4.4M for dev site in Whitestone</t>
+          <t>Satinder Singh pays $2.1M for parking lot in South Ozone Park, SLG owns next door</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>https://www.pincusco.com/lin-qiong-fan-pays-4-4m-to-temple-gates-of-prayer-congregation-shaarai-tefilla-for-in-whitestone/</t>
+          <t>https://www.pincusco.com/satinder-singh-pays-2-1m-for-parking-lot-in-south-ozone-park-slg-owns-next-door/</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Lin Qiong Fan through the entity 145-17 Willets Point Development LLC paid $4.4 million to</t>
+          <t>Satinder Singh through the entity Vas Ny LLC paid $2.1 million to Lawrence Greenfield through</t>
         </is>
       </c>
       <c r="D5" t="inlineStr"/>
@@ -602,24 +602,24 @@
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>Transfers 145-17 Willets Point Blvd (Credit - Cyclomedia) Lin Qiong Fan through the entity 145-17 Willets Point Development LLC paid $4.4 million to Temple Gates of Prayer Congregation Shaarai Tefilla for the development site at 145-17 Willets Point Boulevard in Whitestone, Queens. The expected use is ground up development. The deal closed on April 21, 2026 and was recorded on May 12, 2026. The property has zero square feet of built space on a 18,910 square foot parcel, according to a PincusCo analysis of city data. The seller bought the property on December 16, 2019, for $5.3 million. The signatory for Temple Gates of Prayer Congregation Shaarai Tefilla was Barry Grodenchik. The signatory for Lin Qiong Fan was Lin Qiong Fan. The contract date was December 9, 2024. Prior sales, articles and revenue Prior to this transaction, PincusCo has no record that the buyer Lin Qiong Fan had purchased any other properties and has no record it sold any properties over the past 24 months. The seller Temple Gates of Prayer Congregation Shaarai Tefilla had not purchased any other properties and had not sold any properties over the same time period. The property</t>
+          <t>Transfers 107-26 Rockaway Blvd and 107-30 Rockaway Blvd (Credit - Google Earth) Satinder Singh through the entity Vas Ny LLC paid $2.1 million to Lawrence Greenfield through the entity Elwin Corp for the parking facility (G1) at 107-26 Rockaway Boulevard in South Ozone Park, Queens. The giant REIT SL Green Realty owns the vacant lot next door, at 107-30 Rockaway Boulevard, which it bought in 2008 for $1.35 million. The deal closed on April 17, 2026 and was recorded on May 11, 2026. The property has 2,800 square feet of built space and 4,700 square feet of additional air rights for a total buildable of 7,500 square feet according to a PincusCo analysis of city data. The sale price per built square foot is $750 and the price per buildable square foot is $280 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) The signatory for Lawrence Greenfield was Lawrence Greenfield. The signatory for Satinder Singh was Satinder Singh. The contract date was May 2, 2025. Prior sales, articles and revenue Prior to this transaction, PincusCo has no record that the buyer</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Congregation Machne Chaim signs $20M loan with Webster Bank for school in Bensonhurst</t>
+          <t>Kenneth Chan signs $60M refi with Centennial Bank for tv studio in Greenpoint</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>https://www.pincusco.com/congregation-machne-chaim-signs-20m-refi-with-webster-bank-for-school-in-bensonhurst/</t>
+          <t>https://www.pincusco.com/kenneth-chan-signs-60m-refi-with-centennial-bank-for-tv-studio-in-greenpoint/</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Congregation Machne Chaim through the entity Bais Sarah Educational Center For Girls as borrower signed</t>
+          <t>Kenneth Chan through the entity Java Landing, LLC as borrower signed a refi loan with</t>
         </is>
       </c>
       <c r="D6" t="inlineStr"/>
@@ -636,24 +636,24 @@
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t xml:space="preserve">Transfers 6101 16th Avenue (Credit - Cyclomedia) Congregation Machne Chaim through the entity Bais Sarah Educational Center For Girls as borrower signed a loan with lender Webster Bank through the entity Webster Bank, National Association valued at $20 million for the specialty building (W2) at 6101 16th Avenue in Bensonhurst, Brooklyn. The deal closed on April 30, 2026 and was recorded on May 11, 2026. The prior lender was Bank of Princeton which held debt that had an original loan amount of $5 million. The property has 61,148 square feet of built space according to a PincusCo analysis of city data. The loan price per built square foot is $327 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) The owner bought the property on November 5, 2003, for $7 million. The signatory for Congregation Machne Chaim was Nuchem Klein . The signatory for Webster Bank was Lisa Congemi . The property The specialty building in Bensonhurst has 61,148 square feet of built space according to a PincusCo analysis of city data. The parcel has frontage of 200 feet and is 190 </t>
+          <t>Transfers 8 Java Street (Credit - Cyclomedia) Kenneth Chan through the entity Java Landing, LLC as borrower signed a refi loan with lender Centennial Bank through the entity Centennial Bank valued at $60 million for the television studio building (J6) at 8 Java Street in Greenpoint, Brooklyn. The deal closed on April 30, 2026 and was recorded on May 11, 2026. The prior lender was Series 2022-BNK44 and serviced by Trimont which held debt that had an original loan amount of $50 million. The property has 98,910 square feet of built space and 139,160 square feet of additional air rights for a total buildable of 238,140 square feet according to a PincusCo analysis of city data. The loan price per built square foot is $606 and the price per buildable square foot is $251 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) The signatory for Kenneth Chan was Kenneth Chan. The signatory for Centennial Bank was Francillia Le Blanc . The property The specialty building in Greenpoint has 98,910 square feet of built space and 139,160 square feet of additional air ri</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>David Chan files plans for 3-story retail, school, medical building in Maspeth</t>
+          <t>ID Real Estate Partners sells office in Garment District for $9M</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>https://www.pincusco.com/david-chan-files-plans-for-3-story-retail-school-medical-building-in-maspeth/</t>
+          <t>https://www.pincusco.com/id-real-estate-partners-sells-office-in-garment-district-for-9m/</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>David Chan submitted a new building construction project for a 11,831-square-foot retail and commercial building</t>
+          <t>The entity 242 West 38th Partners LLC with unknown ownership, paid $9 million to ID</t>
         </is>
       </c>
       <c r="D7" t="inlineStr"/>
@@ -670,109 +670,7 @@
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>Development 50-53 69th Street axonometric diagram (Credit - Chang Hwa Tan architect via DOB) David Chan submitted a new building construction project for a 11,831-square-foot retail and commercial building at 50-53 69th Street in Maspeth, Queens. The plan was filed on May 11, 2026. It calls for the construction of a 39-foot-tall, three-story building and was filed with the New York City Department of Buildings under job number Q01381850. The project is described in the filing as: proposed a 3-story commercial building. The applicant is the Registered Architect Chang Tan of Tan Architect P.C. The plans call for 2,188 square feet of retail on the ground floor and 2,379 square feet in the cellar; a school or daycare on the 4,665 square-foot second floor; and an ambulatory health facility on the 2,207-square-foot third floor. Sai Ho Chan and David Chan bought the property for $1.55 million in 2025. The neighborhood</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>Stagg Group files plans for 68 units in Astoria</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>https://www.pincusco.com/stagg-group-files-plans-for-68-units-in-astoria/</t>
-        </is>
-      </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>Stagg Group submitted a new building construction project for a 68-unit, 82,960-square-foot residential (R-2) building</t>
-        </is>
-      </c>
-      <c r="D8" t="inlineStr"/>
-      <c r="E8" t="inlineStr"/>
-      <c r="F8" t="inlineStr">
-        <is>
-          <t>PincusCo</t>
-        </is>
-      </c>
-      <c r="G8" t="inlineStr">
-        <is>
-          <t>PincusCo - Home</t>
-        </is>
-      </c>
-      <c r="H8" t="inlineStr">
-        <is>
-          <t>Development 29-12 Hoyt Avenue axonometric diagram (Credit Minkuk Kim architect via DOB) Stagg Group submitted a new building construction project for a 68-unit, 82,960-square-foot residential (R-2) building at 29-12 Hoyt Avenue South in Astoria, Queens. The plan was filed on May 11, 2026. It calls for the construction of a 94-foot-tall, nine-story building and was filed with the New York City Department of Buildings under job number Q01395583. The project is described in the filing as: construction of a new 9-story building consisting of 68 apartment units.. The applicant is the Registered Architect Minkuk Kim of MK Architect Studio. Mark Stagg of Stagg Group submitted the plans. Property records show the building is owned by an entity that appears unrelated to Stagg Group. The most recent sale was in 2012 for $830,000. The neighborhood In Astoria, The bulk, or 36 percent of the 40.2 million square feet of commercial built space are walkup buildings, with elevator buildings next occupying 31 percent of the space. In sales, Astoria has near average sales volume among other neighborhoods with $851.5 million in sales volume in the last two years and is the 2nd highest in Queens. For d</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>Prospect Development files plans for 9 apartments on single floor in Garment District commercial</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>https://www.pincusco.com/prospect-development-files-plans-for-9-apartments-on-single-floor-in-garment-district-commercial/</t>
-        </is>
-      </c>
-      <c r="C9" t="inlineStr">
-        <is>
-          <t>Prospect Development Group submitted a major alteration application for a rehab of 109,416-square-foot commercial building</t>
-        </is>
-      </c>
-      <c r="D9" t="inlineStr"/>
-      <c r="E9" t="inlineStr"/>
-      <c r="F9" t="inlineStr">
-        <is>
-          <t>PincusCo</t>
-        </is>
-      </c>
-      <c r="G9" t="inlineStr">
-        <is>
-          <t>PincusCo - Home</t>
-        </is>
-      </c>
-      <c r="H9" t="inlineStr">
-        <is>
-          <t>Development 229 West 36th Street (Credit - Google Earth) Prospect Development Group submitted a major alteration application for a rehab of 109,416-square-foot commercial building (COM) at 229 West 36th Street in the Garment District, Manhattan. The plan was filed on May 6, 2026. It calls for a conversion of the 12th floor of the 121-foot-tall, twelve-story building and was filed with the New York City Department of Buildings under job number M01395574. The project is described in the filing as: application filed to convert the twelfth (12th) floor of the existing twelve (12)-story commercial building to residential use as per plans. The applicant is the Registered Architect Kao Hwa Lee of Kao Hwa Lee Architects Pc. Konstantin Gubareff of Prospect Development Group submitted the plans. Cayre Equities and A&amp;H Acquisitions bought the building for $19.2 million in May 2025. The neighborhood In Garment District, The majority, or 69 percent of the 52.3 million square feet of commercial built space are office buildings, with hotel buildings next occupying 13 percent of the space. In sales, Garment District has the 10th highest sale turnover among other neighborhoods in the city with $1.4</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>Stellar Management signs $77.5M refi loan with Nuveen for hotel in Upper West Side</t>
-        </is>
-      </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>https://www.pincusco.com/stellar-management-signs-77-5m-refi-loan-with-nuveen-for-hotel-in-upper-west-side/</t>
-        </is>
-      </c>
-      <c r="C10" t="inlineStr">
-        <is>
-          <t>Stellar Management through the entity Windermere Owners LLC as borrower signed a refi loan with</t>
-        </is>
-      </c>
-      <c r="D10" t="inlineStr"/>
-      <c r="E10" t="inlineStr"/>
-      <c r="F10" t="inlineStr">
-        <is>
-          <t>PincusCo</t>
-        </is>
-      </c>
-      <c r="G10" t="inlineStr">
-        <is>
-          <t>PincusCo - Home</t>
-        </is>
-      </c>
-      <c r="H10" t="inlineStr">
-        <is>
-          <t>Transfers 666 West End Avenue (Credit - Cyclomedia) Stellar Management through the entity Windermere Owners LLC as borrower signed a refi loan with lender Nuveen through the entity Teachers Insurance And Annuity Association Of valued at $77.5 million for the hotel building (H6) at 666 West End Avenue in Upper West Side, Manhattan. The deal closed on May 1, 2026 and was recorded on May 7, 2026. The prior lender was Adler &amp; Stachenfeld registered which held debt that had an original loan amount of $95 million.The property has 279,316 square feet of built space according to a PincusCo analysis of city data. The loan price per built square foot is $277 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) The owner bought the property on November 18, 2010, for $68.5 million. The signatory for Stellar Management was Adam Roman . The signatory for Nuveen was Grace A. Cole . Prior sales, articles and revenue The owners according to the Department of Housing Preservation and Development includes Smajlje Srdanovic, head officer and Arianit Jakupaj, officer. The b</t>
+          <t>Transfers 242 West 38th Street (Credit - Cyclomedia) The entity 242 West 38th Partners LLC with unknown ownership, paid $9 million to ID Real Estate Partners through the entity 242 West 38th Street, LLC for the office building (O6) at 242 West 38th Street in Garment District, Manhattan. The deal closed on May 7, 2026 and was recorded on May 11, 2026. The property has 47,661 square feet of built space according to a PincusCo analysis of city data. The sale price per built square foot is $188 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) The signatory for ID Real Estate Partners was Ira Z. Fishman . The signatory for the buyer was attorney Joseph Cohen . The contract date was December 31, 2025. Prior sales, articles and revenue The seller ID Real Estate Partners had not purchased any other properties and had not sold any properties over the past 24 months. The 47,661-square-foot property generated revenue of $1.2 million or $26 per square foot, according to the most recent income and expense figures. The property</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto update queens news 2026-05-15T14:32:23Z
</commit_message>
<xml_diff>
--- a/data/output/queens_dev_news.xlsx
+++ b/data/output/queens_dev_news.xlsx
@@ -473,17 +473,17 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Joseph Fazzia pays $4.5M for mixed-use in Rossville</t>
+          <t>Habitat Living NYC pays $2.5M for 8-unit townhouse in Crown Heights</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>https://www.pincusco.com/joseph-fazzia-pays-4-5m-for-mixed-use-in-rossville/</t>
+          <t>https://www.pincusco.com/habitat-living-nyc-pays-2-5m-for-8-unit-townhouse-in-crown-heights/</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Joseph Fazzia paid $4.5 million to Michael Freundlich through the entity 2200 A.K.R. Associates LLC</t>
+          <t>Habitat Living NYC through the entity Habitat On Prospect LLC paid $2.5 million to Myrtho</t>
         </is>
       </c>
       <c r="D2" t="inlineStr"/>
@@ -500,24 +500,24 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>Transfers 2200 Arthur Kill Road (Credit - Cyclomedia) Joseph Fazzia paid $4.5 million to Michael Freundlich through the entity 2200 A.K.R. Associates LLC for the mixed-use building (K2) at 2200 Arthur Kill Road in Rossville, Staten Island. The deal closed on March 20, 2026 and was recorded on May 13, 2026. The property has 12,480 square feet of built space and 88,830 square feet of additional air rights for a total buildable of 101,520 square feet according to a PincusCo analysis of city data. The sale price per built square foot is $360 and the price per buildable square foot is $44 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) The signatory for Michael Freundlich was Michael Freundlich. The signatory for Joseph Fazzia was Joseph Fazzia Sr. Prior sales, articles and revenue Prior to this transaction, PincusCo has records that the buyer Joseph Fazzia purchased three properties in one transaction for a total of $7.2 million and has no record it sold any properties over the past 24 months. The seller Michael Freundlich had not purchased any other p</t>
+          <t>Transfers 447 Prospect Place (Credit - Cyclomedia) Habitat Living NYC through the entity Habitat On Prospect LLC paid $2.5 million to Myrtho Ferdinand through the entity 447 Prospect Street LLC for the eight-unit property at 447 Prospect Place in Crown Heights, Brooklyn. The expected use is cash flowing. The deal closed on April 30, 2026 and was recorded on May 12, 2026. The property has 8,884 square feet of built space according to a PincusCo analysis of city data. The sale price per built square foot is $281 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) The signatory for Myrtho Ferdinand was Myrtho Ferdinand. The signatory for Habitat Living NYC was Elliot Steinmetz . The contract date was March 26, 2026. Prior sales, articles and revenue Prior to this transaction, PincusCo has records that the buyer Habitat Living NYC purchased two properties in two transactions for a total of $8.4 million and has no record it sold any properties over the past 24 months. The seller Myrtho Ferdinand had not purchased any other properties and had not sold any pr</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Safehold Inc. files plans for 32 apartments on single floor of office building in Midtown West</t>
+          <t>Vista Group of Companies signs $36.5M refi for hotel in South Ozone Park</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>https://www.pincusco.com/safehold-inc-files-conversion-plans-for-32-units-on-single-floor-in-midtown-west/</t>
+          <t>https://www.pincusco.com/vista-group-of-companies-signs-36-5m-refi-for-hotel-in-south-ozone-park/</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Elisha Blechner of Safehold Inc. submitted a major alteration application for the conversion of a</t>
+          <t>Vista Group of Companies through the entity JFK Hotel Owner, LLC as borrower signed a</t>
         </is>
       </c>
       <c r="D3" t="inlineStr"/>
@@ -534,24 +534,24 @@
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>Development 135 West 50th Street (Credit - Google Earth) Elisha Blechner of Safehold Inc. submitted a major alteration application for the conversion of a single floor of the commercial office (COM) building at 135 West 50th Street in Midtown West, Manhattan from commercial to 32 apartments. The plan was filed on May 12, 2026. It calls for work in the 248-foot-tall, 23-story building and was filed with the New York City Department of Buildings under job number M01400622. The project is described in the filing as: MPP project-000000631. Filing for conversion of the 12th floor from commercial to residential use as shown, no change to the rest of the building. The applicant is the Registered Architect Ambrose Aliaga Kelly of Gensler. This is the first such application to convert a portion of the building to residential, a PincusCo review shows. In October 2024, PincusCo reported that Texas-based Thakkar Developers through the entity TD 135 West 50 LLC paid $8.5 million to UBS Realty Investors through the entity 135 West 50th Street Lessee LLC for the ground lease that controls the office building (O4) at 135 West 50th Street in Midtown West, Manhattan. The fee is owned by Safehold Inc</t>
+          <t>Transfers 135-30 140th Street (Credit - Cyclomedia) Vista Group of Companies through the entity JFK Hotel Owner, LLC as borrower signed a refi loan with lender Webster Bank valued at $36.5 million for the DoubleTree by Hilton New York JFK Airport hotel building (H2) at 135-30 140th Street in South Ozone Park, Queens. The deal closed on April 30, 2026 and was recorded on May 13, 2026. The prior lender was Webster Bank which held debt that had an original loan amount of $39 million. The property has 199,873 square feet of built space according to a PincusCo analysis of city data. The loan price per built square foot is $182 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) The owner bought the property on December 22, 2021, for $36.5 million. The signatory for Vista Group of Companies was Ally Visram. The signatory for Webster Bank was Michael Savarese . Prior sales, articles and revenue The owners according to the Department of Housing Preservation and Development includes Ally Visram, head officer and Luis Paz, site manager. The business entity is JF</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Shanshan Peng files plans for 26 units in Long Island City</t>
+          <t>Vornado, Aurora sign $161M refi with UBS for two office properties in Chelsea</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>https://www.pincusco.com/shanshan-peng-files-plans-for-26-units-in-long-island-city/</t>
+          <t>https://www.pincusco.com/vornado-aurora-signs-161m-refi-with-ubs-for-two-office-properties-in-chelsea/</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Shanshan Peng submitted a new building construction project for a 26-unit, 27,496-square-foot residential (R-2) building</t>
+          <t>Vornado Realty Trust and Aurora Capital Associates through the entity 61 Ninth Avenue Development LLC</t>
         </is>
       </c>
       <c r="D4" t="inlineStr"/>
@@ -568,24 +568,24 @@
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>Development 37-31 29th Street schematic plan and elevations (Credit - Murat Mutlu architect via DOB) Shanshan Peng submitted a new building construction project for a 26-unit, 27,496-square-foot residential (R-2) building at 37-31 29 Street in Long Island City, Queens. The plan was filed on May 12, 2026. It calls for the construction of a 79-foot-tall, seven-story building and was filed with the New York City Department of Buildings under job number Q01381898. The project is described in the filing as: propose a 7-story mixed-use building comprising commercial spaces and 26 class a apartments with 20% of qualifying affordable housing units (uap development). obtain a new certificate of occupancy.. The applicant is the Registered Architect Murat Mutlu of Inoa Architecture Inc. 37-31 29th Street The neighborhood In Long Island City, The bulk, or 32 percent of the 60.1 million square feet of commercial built space are industrial buildings, with elevator buildings next occupying 31 percent of the space. In sales, Long Island City has near average sales volume among other neighborhoods with $1.1 billion in sales volume in the last two years and is the highest in Queens. For development,</t>
+          <t>Transfers 61 9th Avenue (Credit - Cyclomedia) Vornado Realty Trust and Aurora Capital Associates through the entity 61 Ninth Avenue Development LLC as borrower signed a refi loan with lender UBS through the entity UBS AG, Stamford Branch valued at $161 million for two office properties including the office building (O6) at 61 9th Avenue in Chelsea, Manhattan and the adjacent office building (O6) at 404 West 15th Street. The deal closed on May 8, 2026 and was recorded on May 13, 2026. The prior lender was Landesbank Baden-Wurttemberg which held debt that had an original loan amount of $167.5 million. The two properties have 277,626 square feet of built space according to a PincusCo analysis of city data. The loan price per built square foot is $579 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) The signatory for Vornado Realty Trust and Aurora Capital Associates was Steven Borenstein . A Vornado press release said the prior loan was $155 million. Because multiple properties have been transacted, some of the following sections will follow the proper</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Satinder Singh pays $2.1M for parking lot in South Ozone Park, SLG owns next door</t>
+          <t>Walter Wilfinger pays $4M to Annal Management for 68-unit rental elevator in Concourse Village</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>https://www.pincusco.com/satinder-singh-pays-2-1m-for-parking-lot-in-south-ozone-park-slg-owns-next-door/</t>
+          <t>https://www.pincusco.com/walter-wilfinger-pays-4m-to-annal-management-for-68-unit-rental-elevator-in-concourse-village/</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Satinder Singh through the entity Vas Ny LLC paid $2.1 million to Lawrence Greenfield through</t>
+          <t>Walter Wilfinger through the entity Hwy Realty LLC paid $4 million to Annal Management through</t>
         </is>
       </c>
       <c r="D5" t="inlineStr"/>
@@ -602,24 +602,24 @@
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>Transfers 107-26 Rockaway Blvd and 107-30 Rockaway Blvd (Credit - Google Earth) Satinder Singh through the entity Vas Ny LLC paid $2.1 million to Lawrence Greenfield through the entity Elwin Corp for the parking facility (G1) at 107-26 Rockaway Boulevard in South Ozone Park, Queens. The giant REIT SL Green Realty owns the vacant lot next door, at 107-30 Rockaway Boulevard, which it bought in 2008 for $1.35 million. The deal closed on April 17, 2026 and was recorded on May 11, 2026. The property has 2,800 square feet of built space and 4,700 square feet of additional air rights for a total buildable of 7,500 square feet according to a PincusCo analysis of city data. The sale price per built square foot is $750 and the price per buildable square foot is $280 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) The signatory for Lawrence Greenfield was Lawrence Greenfield. The signatory for Satinder Singh was Satinder Singh. The contract date was May 2, 2025. Prior sales, articles and revenue Prior to this transaction, PincusCo has no record that the buyer</t>
+          <t>Transfers 1181 Sheridan Avenue (Credit - Cyclomedia) Walter Wilfinger through the entity Hwy Realty LLC paid $4 million to Annal Management through the entity H &amp; H Equities II, Inc. for the 68-unit residential elevator building (D1) at 1181 Sheridan Avenue in Concourse Village, Bronx. The expected use is cash flowing. The deal closed on April 30, 2026 and was recorded on May 13, 2026. The property has 72,276 square feet of built space and 28,913 square feet of additional air rights for a total buildable of 101,196 square feet according to a PincusCo analysis of city data. The sale price per built square foot is $54 and the price per buildable square foot is $39 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) The signatory for Annal Management was Aida Spitzer . The signatory for Walter Wilfinger was Walter Wilfinger. The contract date was February 25, 2026. Prior sales, articles and revenue Prior to this transaction, PincusCo has records that the buyer Walter Wilfinger purchased two properties in two transactions for a total of $9 million and sold</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Kenneth Chan signs $60M refi with Centennial Bank for tv studio in Greenpoint</t>
+          <t>Habitat Living NYC pays $4M for 2-family in Carroll Gardens</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>https://www.pincusco.com/kenneth-chan-signs-60m-refi-with-centennial-bank-for-tv-studio-in-greenpoint/</t>
+          <t>https://www.pincusco.com/habitat-living-nyc-pays-4m-for-2-family-in-carroll-gardens/</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Kenneth Chan through the entity Java Landing, LLC as borrower signed a refi loan with</t>
+          <t>Habitat Living NYC through the entity Habitat On Degraw 2 LLC paid $4 million for</t>
         </is>
       </c>
       <c r="D6" t="inlineStr"/>
@@ -636,24 +636,24 @@
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>Transfers 8 Java Street (Credit - Cyclomedia) Kenneth Chan through the entity Java Landing, LLC as borrower signed a refi loan with lender Centennial Bank through the entity Centennial Bank valued at $60 million for the television studio building (J6) at 8 Java Street in Greenpoint, Brooklyn. The deal closed on April 30, 2026 and was recorded on May 11, 2026. The prior lender was Series 2022-BNK44 and serviced by Trimont which held debt that had an original loan amount of $50 million. The property has 98,910 square feet of built space and 139,160 square feet of additional air rights for a total buildable of 238,140 square feet according to a PincusCo analysis of city data. The loan price per built square foot is $606 and the price per buildable square foot is $251 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) The signatory for Kenneth Chan was Kenneth Chan. The signatory for Centennial Bank was Francillia Le Blanc . The property The specialty building in Greenpoint has 98,910 square feet of built space and 139,160 square feet of additional air ri</t>
+          <t>Transfers 303 Degraw Street (Credit - Cyclomedia) Habitat Living NYC through the entity Habitat On Degraw 2 LLC paid $4 million for the two-unit building (B9) at 303 Degraw Street in Carroll Gardens, Brooklyn. The deal closed on April 30, 2026 and was recorded on May 13, 2026. The property has 3,000 square feet of built space and 1,961 square feet of additional air rights for a total buildable of 4,966 square feet according to a PincusCo analysis of city data. The sale price per built square foot is $1,333 and the price per buildable square foot is $805 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) The signatory for the seller was Joan Folwell. The signatory for Habitat Living NYC was Elliot Steinmetz . The contract date was December 31, 2025. Prior sales, articles and revenue Prior to this transaction, PincusCo has records that the buyer Habitat Living NYC purchased three properties in three transactions for a total of $10.9 million and has no record it sold any properties over the past 24 months. The seller Joan Folwell had not purchased any ot</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>ID Real Estate Partners sells office in Garment District for $9M</t>
+          <t>UWS mixed-use sells for $4M</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>https://www.pincusco.com/id-real-estate-partners-sells-office-in-garment-district-for-9m/</t>
+          <t>https://www.pincusco.com/uws-mixed-use-sells-for-4m/</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>The entity 242 West 38th Partners LLC with unknown ownership, paid $9 million to ID</t>
+          <t>The entity 307 Amsterdam Ave NY LLC paid $4 million to the entity 307 Amsterdam</t>
         </is>
       </c>
       <c r="D7" t="inlineStr"/>
@@ -670,7 +670,7 @@
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>Transfers 242 West 38th Street (Credit - Cyclomedia) The entity 242 West 38th Partners LLC with unknown ownership, paid $9 million to ID Real Estate Partners through the entity 242 West 38th Street, LLC for the office building (O6) at 242 West 38th Street in Garment District, Manhattan. The deal closed on May 7, 2026 and was recorded on May 11, 2026. The property has 47,661 square feet of built space according to a PincusCo analysis of city data. The sale price per built square foot is $188 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) The signatory for ID Real Estate Partners was Ira Z. Fishman . The signatory for the buyer was attorney Joseph Cohen . The contract date was December 31, 2025. Prior sales, articles and revenue The seller ID Real Estate Partners had not purchased any other properties and had not sold any properties over the past 24 months. The 47,661-square-foot property generated revenue of $1.2 million or $26 per square foot, according to the most recent income and expense figures. The property</t>
+          <t>Transfers 307 Amsterdam Avenue (Credit - Cyclomedia) The entity 307 Amsterdam Ave NY LLC paid $4 million to the entity 307 Amsterdam Avenue LLC for the four-unit mixed-use building (S4) at 307 Amsterdam Avenue in Upper West Side, Manhattan. The deal closed on April 28, 2026 and was recorded on May 13, 2026. The property has 4,080 square feet of built space and 6,279 square feet of additional air rights for a total buildable of 10,355 square feet according to a PincusCo analysis of city data. The sale price per built square foot is $992 and the price per buildable square foot is $391 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) The signatories for the sellers were Antoinette Yanni and Roseanne Yanni. The signatory for the buyer was Susan Chury. The contract date was January 21, 2026. Prior sales, articles and revenue Prior to this transaction, PincusCo has no record that the buyer Susan Chury had purchased any other properties and has no record it sold any properties over the past 24 months. The seller Antoinette Yanni had not purchased any other</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto update queens news 2026-05-16T13:57:24Z
</commit_message>
<xml_diff>
--- a/data/output/queens_dev_news.xlsx
+++ b/data/output/queens_dev_news.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H7"/>
+  <dimension ref="A1:H10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -473,17 +473,17 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Habitat Living NYC pays $2.5M for 8-unit townhouse in Crown Heights</t>
+          <t>Carolwood, Empire Capital, partners, acquire SoHo office in $36M deed-in-lieu</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>https://www.pincusco.com/habitat-living-nyc-pays-2-5m-for-8-unit-townhouse-in-crown-heights/</t>
+          <t>https://www.pincusco.com/carolwood-empire-capital-partners-acquire-office-in-soho-in-36m-deed-in-lieu/</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Habitat Living NYC through the entity Habitat On Prospect LLC paid $2.5 million to Myrtho</t>
+          <t>Empire Capital Holdings, Carolwood, Jeremy Aiden, and an affiliate of Husein Jafferjee through the entity</t>
         </is>
       </c>
       <c r="D2" t="inlineStr"/>
@@ -500,24 +500,24 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>Transfers 447 Prospect Place (Credit - Cyclomedia) Habitat Living NYC through the entity Habitat On Prospect LLC paid $2.5 million to Myrtho Ferdinand through the entity 447 Prospect Street LLC for the eight-unit property at 447 Prospect Place in Crown Heights, Brooklyn. The expected use is cash flowing. The deal closed on April 30, 2026 and was recorded on May 12, 2026. The property has 8,884 square feet of built space according to a PincusCo analysis of city data. The sale price per built square foot is $281 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) The signatory for Myrtho Ferdinand was Myrtho Ferdinand. The signatory for Habitat Living NYC was Elliot Steinmetz . The contract date was March 26, 2026. Prior sales, articles and revenue Prior to this transaction, PincusCo has records that the buyer Habitat Living NYC purchased two properties in two transactions for a total of $8.4 million and has no record it sold any properties over the past 24 months. The seller Myrtho Ferdinand had not purchased any other properties and had not sold any pr</t>
+          <t>Transfers 261-267 Canal Street (Credit - Cyclomedia) Empire Capital Holdings, Carolwood, Jeremy Aiden, and an affiliate of Husein Jafferjee through the entity 1-21 Howard Aidan TIC LLC (and others) acquired through a deed-in-lieu of foreclosure valued at $36 million, to HCRE Hung &amp; Chong Real Estate through the entity 267 Canal Street Corp. for the office building (O5) at 261-267 Canal Street in Little Italy, Manhattan. The deal closed on May 4, 2026 and was recorded on May 14, 2026. The property has 103,047 square feet of built space and 58,552 square feet of additional air rights for a total buildable of 161,649 square feet according to a PincusCo analysis of city data. The sale price per built square foot is $349 and the price per buildable square foot is $222 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) The signatory for HCRE Hung &amp; Chong Real Estate was Philip Chong . The signatory for Empire Capital Holdings , Carolwood , Jeremy Aiden, and Husein Jafferjee was Abraham Khalili , Jeremy Aidan, Adam Rubin, and Husein Jafferjee. The contract d</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Vista Group of Companies signs $36.5M refi for hotel in South Ozone Park</t>
+          <t>Yue Hu Xu pays $13.5M to Tri-Boro Shelving &amp; Partition for industrial in Ridgewood</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>https://www.pincusco.com/vista-group-of-companies-signs-36-5m-refi-for-hotel-in-south-ozone-park/</t>
+          <t>https://www.pincusco.com/yue-hu-xu-pays-13-5m-to-tri-boro-shelving-partition-for-industrial-in-ridgewood/</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Vista Group of Companies through the entity JFK Hotel Owner, LLC as borrower signed a</t>
+          <t>Yue Hu Xu through the entity Fresh Fort LLC paid $13.5 million to Tri-Boro Shelving</t>
         </is>
       </c>
       <c r="D3" t="inlineStr"/>
@@ -534,24 +534,24 @@
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>Transfers 135-30 140th Street (Credit - Cyclomedia) Vista Group of Companies through the entity JFK Hotel Owner, LLC as borrower signed a refi loan with lender Webster Bank valued at $36.5 million for the DoubleTree by Hilton New York JFK Airport hotel building (H2) at 135-30 140th Street in South Ozone Park, Queens. The deal closed on April 30, 2026 and was recorded on May 13, 2026. The prior lender was Webster Bank which held debt that had an original loan amount of $39 million. The property has 199,873 square feet of built space according to a PincusCo analysis of city data. The loan price per built square foot is $182 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) The owner bought the property on December 22, 2021, for $36.5 million. The signatory for Vista Group of Companies was Ally Visram. The signatory for Webster Bank was Michael Savarese . Prior sales, articles and revenue The owners according to the Department of Housing Preservation and Development includes Ally Visram, head officer and Luis Paz, site manager. The business entity is JF</t>
+          <t>Transfers 19-40 Flushing Avenue (Credit - Cyclomedia) Yue Hu Xu through the entity Fresh Fort LLC paid $13.5 million to Tri-Boro Shelving &amp; Partition for the industrial building (E1) at 19-40 Flushing Avenue in Ridgewood, Queens. The deal closed on April 28, 2026 and was recorded on May 14, 2026. The property has 25,234 square feet of built space and 8,867 square feet of additional air rights for a total buildable of 34,107 square feet according to a PincusCo analysis of city data. The sale price per built square foot is $534 and the price per buildable square foot is $395 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) The seller bought the property on January 7, 2016, for $10.5 million. The signatory for Tri-Boro Shelving &amp; Partition was John S. DeMaio . The signatory for Yue Hu Xu was Yue Hu Xu. The contract date was April 28, 2026. Prior sales, articles and revenue Prior to this transaction, PincusCo has no record that the buyer Yue Hu Xu had purchased any other properties and has no record it sold any properties over the past 24 months. The se</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Vornado, Aurora sign $161M refi with UBS for two office properties in Chelsea</t>
+          <t>Manaf Saker affiliate pays $6.3M for 3-family in Chelsea</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>https://www.pincusco.com/vornado-aurora-signs-161m-refi-with-ubs-for-two-office-properties-in-chelsea/</t>
+          <t>https://www.pincusco.com/manaf-saker-affiliate-pays-6-3m-for-3-family-in-chelsea/</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Vornado Realty Trust and Aurora Capital Associates through the entity 61 Ninth Avenue Development LLC</t>
+          <t>Manaf Saker through the entity Condor 426 W 22st Nyc LLC paid $6.3 million to</t>
         </is>
       </c>
       <c r="D4" t="inlineStr"/>
@@ -568,24 +568,24 @@
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>Transfers 61 9th Avenue (Credit - Cyclomedia) Vornado Realty Trust and Aurora Capital Associates through the entity 61 Ninth Avenue Development LLC as borrower signed a refi loan with lender UBS through the entity UBS AG, Stamford Branch valued at $161 million for two office properties including the office building (O6) at 61 9th Avenue in Chelsea, Manhattan and the adjacent office building (O6) at 404 West 15th Street. The deal closed on May 8, 2026 and was recorded on May 13, 2026. The prior lender was Landesbank Baden-Wurttemberg which held debt that had an original loan amount of $167.5 million. The two properties have 277,626 square feet of built space according to a PincusCo analysis of city data. The loan price per built square foot is $579 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) The signatory for Vornado Realty Trust and Aurora Capital Associates was Steven Borenstein . A Vornado press release said the prior loan was $155 million. Because multiple properties have been transacted, some of the following sections will follow the proper</t>
+          <t>Transfers 426 West 22nd Street (Credit - Cyclomedia) Manaf Saker through the entity Condor 426 W 22st Nyc LLC paid $6.3 million to Maurice Haroche through the entity 426 West 22nd Associates, LLC for the three-unit building (C0) at 426 West 22nd Street in Chelsea, Manhattan. The deal closed on April 30, 2026 and was recorded on May 14, 2026. The property has 3,440 square feet of built space and 1,994 square feet of additional air rights for a total buildable of 5,439 square feet according to a PincusCo analysis of city data. The sale price per built square foot is $1,831 and the price per buildable square foot is $1,158 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) The seller bought the property on August 8, 2016, for $7.3 million. The signatory for Maurice Haroche was Peter Graubard . The signatory for Manaf Saker was Manaf Saker, who is a dental surgeon. The contract date was February 9, 2026. Prior sales, articles and revenue Prior to this transaction, PincusCo has no record that the buyer Manaf Saker had purchased any other properties and has</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Walter Wilfinger pays $4M to Annal Management for 68-unit rental elevator in Concourse Village</t>
+          <t>Chestnut Holdings pays $2.5M to Milbrook Properties for 29-unit walkup in Fordham Heights</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>https://www.pincusco.com/walter-wilfinger-pays-4m-to-annal-management-for-68-unit-rental-elevator-in-concourse-village/</t>
+          <t>https://www.pincusco.com/chestnut-holdings-pays-2-5m-to-milbrook-properties-for-29-unit-walkup-in-fordham-heights/</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Walter Wilfinger through the entity Hwy Realty LLC paid $4 million to Annal Management through</t>
+          <t>Chestnut Holdings of New York through the entity 2387 Morris LLC paid $2.5 million to</t>
         </is>
       </c>
       <c r="D5" t="inlineStr"/>
@@ -602,24 +602,24 @@
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>Transfers 1181 Sheridan Avenue (Credit - Cyclomedia) Walter Wilfinger through the entity Hwy Realty LLC paid $4 million to Annal Management through the entity H &amp; H Equities II, Inc. for the 68-unit residential elevator building (D1) at 1181 Sheridan Avenue in Concourse Village, Bronx. The expected use is cash flowing. The deal closed on April 30, 2026 and was recorded on May 13, 2026. The property has 72,276 square feet of built space and 28,913 square feet of additional air rights for a total buildable of 101,196 square feet according to a PincusCo analysis of city data. The sale price per built square foot is $54 and the price per buildable square foot is $39 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) The signatory for Annal Management was Aida Spitzer . The signatory for Walter Wilfinger was Walter Wilfinger. The contract date was February 25, 2026. Prior sales, articles and revenue Prior to this transaction, PincusCo has records that the buyer Walter Wilfinger purchased two properties in two transactions for a total of $9 million and sold</t>
+          <t xml:space="preserve">Transfers 2387 Morris Avenue (Credit - Cyclomedia) Chestnut Holdings of New York through the entity 2387 Morris LLC paid $2.5 million to Milbrook Properties through the entity R.V. Properties LLC for the 29-unit residential walkup building (C7) at 2387 Morris Avenue in Fordham Heights, Bronx. The expected use is cash flowing. The deal closed on May 1, 2026 and was recorded on May 14, 2026. The property has 35,429 square feet of built space and 4,887 square feet of additional air rights for a total buildable of 40,303 square feet according to a PincusCo analysis of city data. The sale price per built square foot is $71 and the price per buildable square foot is $63 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) The signatory for Milbrook Properties was Charles Hirsch . The signatory for Chestnut Holdings of New York was Anthony Simari . The contract date was March 6, 2026. Prior sales, articles and revenue Prior to this transaction, PincusCo has records that the buyer Chestnut Holdings of New York purchased five properties in four transactions for </t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Habitat Living NYC pays $4M for 2-family in Carroll Gardens</t>
+          <t>Lightstone Group acquires office condos in Midtown for $14.6M through bankruptcy</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>https://www.pincusco.com/habitat-living-nyc-pays-4m-for-2-family-in-carroll-gardens/</t>
+          <t>https://www.pincusco.com/lightstone-group-acquires-office-condos-in-midtown-for-14-6m-through-bankruptcy/</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Habitat Living NYC through the entity Habitat On Degraw 2 LLC paid $4 million for</t>
+          <t>Lightstone Group through the entity 32 W 39th St Owner LLC through a bankruptcy acquired</t>
         </is>
       </c>
       <c r="D6" t="inlineStr"/>
@@ -636,24 +636,24 @@
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>Transfers 303 Degraw Street (Credit - Cyclomedia) Habitat Living NYC through the entity Habitat On Degraw 2 LLC paid $4 million for the two-unit building (B9) at 303 Degraw Street in Carroll Gardens, Brooklyn. The deal closed on April 30, 2026 and was recorded on May 13, 2026. The property has 3,000 square feet of built space and 1,961 square feet of additional air rights for a total buildable of 4,966 square feet according to a PincusCo analysis of city data. The sale price per built square foot is $1,333 and the price per buildable square foot is $805 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) The signatory for the seller was Joan Folwell. The signatory for Habitat Living NYC was Elliot Steinmetz . The contract date was December 31, 2025. Prior sales, articles and revenue Prior to this transaction, PincusCo has records that the buyer Habitat Living NYC purchased three properties in three transactions for a total of $10.9 million and has no record it sold any properties over the past 24 months. The seller Joan Folwell had not purchased any ot</t>
+          <t>Transfers 32 West 39th Street (Credit - Cyclomedia) Lightstone Group through the entity 32 W 39th St Owner LLC through a bankruptcy acquired seven office condominium units at 32 West 39th Street in Grand Central, Manhattan, in a transaction valued at $14.6 million. The former owner, R&amp;B Realty Group through the entity 32 W. 39th Street Sole Member LLC, led by Aron Rosenberg, filed for bankruptcy in 2024. The deal closed on April 23, 2026 and was recorded on May 14, 2026. The seven properties have 33,553 square feet of built space according to a PincusCo analysis of city data. The sale price per built square foot is $435 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) The signatory for the bankrupt affiliate of R&amp;B Realty Group was David Wallace . The signatory for Lightstone Group was Joseph E. Teichman . The contract date was February 11, 2026. This is the lender taking back the property through bankruptcy. Lightstone Group in 2022 provided loans totaling $52 million covering this and other property, then the borrower filed bankruptcy in 2024. The</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>UWS mixed-use sells for $4M</t>
+          <t>Durgaj Properties signs $10.9M construction loan for 41-unit project in Belmont</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>https://www.pincusco.com/uws-mixed-use-sells-for-4m/</t>
+          <t>https://www.pincusco.com/durgaj-properties-signs-10-9m-construction-loan-with-northeast-community-for-development-in-belmont-little-italy/</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>The entity 307 Amsterdam Ave NY LLC paid $4 million to the entity 307 Amsterdam</t>
+          <t>Durgaj Properties through the entity 2278 Arthur Avenue LLC as borrower signed a new construction</t>
         </is>
       </c>
       <c r="D7" t="inlineStr"/>
@@ -670,7 +670,109 @@
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>Transfers 307 Amsterdam Avenue (Credit - Cyclomedia) The entity 307 Amsterdam Ave NY LLC paid $4 million to the entity 307 Amsterdam Avenue LLC for the four-unit mixed-use building (S4) at 307 Amsterdam Avenue in Upper West Side, Manhattan. The deal closed on April 28, 2026 and was recorded on May 13, 2026. The property has 4,080 square feet of built space and 6,279 square feet of additional air rights for a total buildable of 10,355 square feet according to a PincusCo analysis of city data. The sale price per built square foot is $992 and the price per buildable square foot is $391 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) The signatories for the sellers were Antoinette Yanni and Roseanne Yanni. The signatory for the buyer was Susan Chury. The contract date was January 21, 2026. Prior sales, articles and revenue Prior to this transaction, PincusCo has no record that the buyer Susan Chury had purchased any other properties and has no record it sold any properties over the past 24 months. The seller Antoinette Yanni had not purchased any other</t>
+          <t>Transfers 2276 Arthur Avenue axonometric diagram (Credit - Jakov Saric architect via DOB) Durgaj Properties through the entity 2278 Arthur Avenue LLC as borrower signed a new construction loan with lender NorthEast Community Bank valued at $10.9 million for the 41-unit project at 2276 Arthur Avenue in Belmont, Bronx. On the lot, there is one active new building construction project, X01245967, for a 41-unit, 27,736 square-foot residential (R-2) building. The project was submitted by Durgaj Properties and filed by Paul Durgaj with plans filed July 3, 2025 and permitted March 30, 2026. The deal closed on May 1, 2026 and was recorded on May 14, 2026. The prior lender was NorthEast Community Bank which held debt that had an original loan amount of $925,000. The loan price per planned development square foot is $393 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) The owner bought the property on July 27, 2023, for $1.9 million. The property The development building with 2 residential units in Belmont/Little Italy has 4,560 square feet of built space and</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>AG Holding Group signs $17M construction loan with Kearny for 67-unit project in Bedford Park</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>https://www.pincusco.com/ag-holding-group-signs-17m-construction-loan-with-kearny-for-67-unit-project-in-bedford-park/</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>AG Holding Group through the entity 21 E 198 Realty LLC as borrower signed a</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr"/>
+      <c r="E8" t="inlineStr"/>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>PincusCo</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>PincusCo - Home</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Transfers 21 East 198th Street axonometric diagram (Credit - John Nicholas Backos architect via DOB) AG Holding Group through the entity 21 E 198 Realty LLC as borrower signed a new construction loan with lender Kearny Bank valued at $17 million for the 67-unit project at 21 East 198th Street in Bedford Park, Bronx. On the lot, there is one active new building construction project, X01089171, for a 67-unit, 43,613-square-foot residential (R-2) building. The project is led by Andrea Gjini with plans filed April 23, 2025 and permitted February 9, 2026. The deal closed on April 17, 2026 and was recorded on May 14, 2026. The prior lender was Houlihan &amp; O’Malley Commercial Services which held debt that had an original loan amount of $1.6 million. The loan price per planned development square foot is $390 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) The owner bought the property on October 22, 2024, for $1.8 million. The signatory for AG Holding Group was Andrea Gjini . The signatory for Kearny Bank was Jonathan Atkinson . The property The parcel has </t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Arker Companies signs $6.3M refi with Customers Bank for retail, parking in Edgemere</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>https://www.pincusco.com/arker-companies-signs-6-3m-refi-with-customers-bank-for-retail-parking-in-edgemere/</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Arker Companies through the entity Ec A1 Commercial LLC as borrower signed a refi loan</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr"/>
+      <c r="E9" t="inlineStr"/>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>PincusCo</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>PincusCo - Home</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Transfers 5125 Beach Channel Drive and 302 Beach 53rd Street; and the parking condo with the address 5123 Beach Channel Drive (Credit - Cyclomedia) Arker Companies through the entity Ec A1 Commercial LLC as borrower signed a refi loan with lender Customers Bank valued at $6.3 million for three commercial condominium units at the base of a mixed-use building in Edgemere, Queens. The units are two retail condos with the addresses at 5125 Beach Channel Drive and 302 Beach 53rd Street; and the parking condo with the address 5123 Beach Channel Drive. These units are at the base of a residential condominium unit which includes 194 apartments and is not part of this refinance. The deal closed on April 30, 2026 and was recorded on May 11, 2026. The prior lender was Wells Fargo which held debt that had an original loan amount of $6.4 million. The three properties have 49,014 square feet of built space according to a PincusCo analysis of city data. The loan price per built square foot is $128 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) The signatory for </t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Forest Hill Jewish Center signs $18M initial loan with Valley National Bank in Forest Hills</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>https://www.pincusco.com/forest-hill-jewish-center-signs-18m-initial-loan-with-valley-national-bank-in-forest-hills/</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Forest Hill Jewish Center through the entity The Forest Hills Jewish Center as borrower signed</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr"/>
+      <c r="E10" t="inlineStr"/>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>PincusCo</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>PincusCo - Home</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>Transfers 106-06 Queens Boulevard (Credit - Cyclomedia) Forest Hill Jewish Center through the entity The Forest Hills Jewish Center as borrower signed a initial loan with lender Valley National Bank valued at $18 million for the property at 106-06 Queens Boulevard in Forest Hills, Queens. The deal closed on April 20, 2026 and was recorded on May 12, 2026. The property has 67,780 square feet of built space according to a PincusCo analysis of city data. The loan price per built square foot is $265 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) The signatory for Forest Hill Jewish Center was Gary Kerzner . The property The property in Forest Hills has 67,780 square feet of built space according to a PincusCo analysis of city data. The parcel has a total lot size of 67,780 square feet. The city-designated market value for the property in 2022 is $22.2 million. Transaction Participants</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto update queens news 2026-05-17T13:55:13Z
</commit_message>
<xml_diff>
--- a/data/output/queens_dev_news.xlsx
+++ b/data/output/queens_dev_news.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H10"/>
+  <dimension ref="A1:H1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -467,312 +467,6 @@
       <c r="H1" s="1" t="inlineStr">
         <is>
           <t>content_preview</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>Carolwood, Empire Capital, partners, acquire SoHo office in $36M deed-in-lieu</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>https://www.pincusco.com/carolwood-empire-capital-partners-acquire-office-in-soho-in-36m-deed-in-lieu/</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>Empire Capital Holdings, Carolwood, Jeremy Aiden, and an affiliate of Husein Jafferjee through the entity</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr"/>
-      <c r="E2" t="inlineStr"/>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t>PincusCo</t>
-        </is>
-      </c>
-      <c r="G2" t="inlineStr">
-        <is>
-          <t>PincusCo - Home</t>
-        </is>
-      </c>
-      <c r="H2" t="inlineStr">
-        <is>
-          <t>Transfers 261-267 Canal Street (Credit - Cyclomedia) Empire Capital Holdings, Carolwood, Jeremy Aiden, and an affiliate of Husein Jafferjee through the entity 1-21 Howard Aidan TIC LLC (and others) acquired through a deed-in-lieu of foreclosure valued at $36 million, to HCRE Hung &amp; Chong Real Estate through the entity 267 Canal Street Corp. for the office building (O5) at 261-267 Canal Street in Little Italy, Manhattan. The deal closed on May 4, 2026 and was recorded on May 14, 2026. The property has 103,047 square feet of built space and 58,552 square feet of additional air rights for a total buildable of 161,649 square feet according to a PincusCo analysis of city data. The sale price per built square foot is $349 and the price per buildable square foot is $222 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) The signatory for HCRE Hung &amp; Chong Real Estate was Philip Chong . The signatory for Empire Capital Holdings , Carolwood , Jeremy Aiden, and Husein Jafferjee was Abraham Khalili , Jeremy Aidan, Adam Rubin, and Husein Jafferjee. The contract d</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>Yue Hu Xu pays $13.5M to Tri-Boro Shelving &amp; Partition for industrial in Ridgewood</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>https://www.pincusco.com/yue-hu-xu-pays-13-5m-to-tri-boro-shelving-partition-for-industrial-in-ridgewood/</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>Yue Hu Xu through the entity Fresh Fort LLC paid $13.5 million to Tri-Boro Shelving</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr"/>
-      <c r="E3" t="inlineStr"/>
-      <c r="F3" t="inlineStr">
-        <is>
-          <t>PincusCo</t>
-        </is>
-      </c>
-      <c r="G3" t="inlineStr">
-        <is>
-          <t>PincusCo - Home</t>
-        </is>
-      </c>
-      <c r="H3" t="inlineStr">
-        <is>
-          <t>Transfers 19-40 Flushing Avenue (Credit - Cyclomedia) Yue Hu Xu through the entity Fresh Fort LLC paid $13.5 million to Tri-Boro Shelving &amp; Partition for the industrial building (E1) at 19-40 Flushing Avenue in Ridgewood, Queens. The deal closed on April 28, 2026 and was recorded on May 14, 2026. The property has 25,234 square feet of built space and 8,867 square feet of additional air rights for a total buildable of 34,107 square feet according to a PincusCo analysis of city data. The sale price per built square foot is $534 and the price per buildable square foot is $395 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) The seller bought the property on January 7, 2016, for $10.5 million. The signatory for Tri-Boro Shelving &amp; Partition was John S. DeMaio . The signatory for Yue Hu Xu was Yue Hu Xu. The contract date was April 28, 2026. Prior sales, articles and revenue Prior to this transaction, PincusCo has no record that the buyer Yue Hu Xu had purchased any other properties and has no record it sold any properties over the past 24 months. The se</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>Manaf Saker affiliate pays $6.3M for 3-family in Chelsea</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>https://www.pincusco.com/manaf-saker-affiliate-pays-6-3m-for-3-family-in-chelsea/</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>Manaf Saker through the entity Condor 426 W 22st Nyc LLC paid $6.3 million to</t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr"/>
-      <c r="E4" t="inlineStr"/>
-      <c r="F4" t="inlineStr">
-        <is>
-          <t>PincusCo</t>
-        </is>
-      </c>
-      <c r="G4" t="inlineStr">
-        <is>
-          <t>PincusCo - Home</t>
-        </is>
-      </c>
-      <c r="H4" t="inlineStr">
-        <is>
-          <t>Transfers 426 West 22nd Street (Credit - Cyclomedia) Manaf Saker through the entity Condor 426 W 22st Nyc LLC paid $6.3 million to Maurice Haroche through the entity 426 West 22nd Associates, LLC for the three-unit building (C0) at 426 West 22nd Street in Chelsea, Manhattan. The deal closed on April 30, 2026 and was recorded on May 14, 2026. The property has 3,440 square feet of built space and 1,994 square feet of additional air rights for a total buildable of 5,439 square feet according to a PincusCo analysis of city data. The sale price per built square foot is $1,831 and the price per buildable square foot is $1,158 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) The seller bought the property on August 8, 2016, for $7.3 million. The signatory for Maurice Haroche was Peter Graubard . The signatory for Manaf Saker was Manaf Saker, who is a dental surgeon. The contract date was February 9, 2026. Prior sales, articles and revenue Prior to this transaction, PincusCo has no record that the buyer Manaf Saker had purchased any other properties and has</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>Chestnut Holdings pays $2.5M to Milbrook Properties for 29-unit walkup in Fordham Heights</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>https://www.pincusco.com/chestnut-holdings-pays-2-5m-to-milbrook-properties-for-29-unit-walkup-in-fordham-heights/</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>Chestnut Holdings of New York through the entity 2387 Morris LLC paid $2.5 million to</t>
-        </is>
-      </c>
-      <c r="D5" t="inlineStr"/>
-      <c r="E5" t="inlineStr"/>
-      <c r="F5" t="inlineStr">
-        <is>
-          <t>PincusCo</t>
-        </is>
-      </c>
-      <c r="G5" t="inlineStr">
-        <is>
-          <t>PincusCo - Home</t>
-        </is>
-      </c>
-      <c r="H5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Transfers 2387 Morris Avenue (Credit - Cyclomedia) Chestnut Holdings of New York through the entity 2387 Morris LLC paid $2.5 million to Milbrook Properties through the entity R.V. Properties LLC for the 29-unit residential walkup building (C7) at 2387 Morris Avenue in Fordham Heights, Bronx. The expected use is cash flowing. The deal closed on May 1, 2026 and was recorded on May 14, 2026. The property has 35,429 square feet of built space and 4,887 square feet of additional air rights for a total buildable of 40,303 square feet according to a PincusCo analysis of city data. The sale price per built square foot is $71 and the price per buildable square foot is $63 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) The signatory for Milbrook Properties was Charles Hirsch . The signatory for Chestnut Holdings of New York was Anthony Simari . The contract date was March 6, 2026. Prior sales, articles and revenue Prior to this transaction, PincusCo has records that the buyer Chestnut Holdings of New York purchased five properties in four transactions for </t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>Lightstone Group acquires office condos in Midtown for $14.6M through bankruptcy</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>https://www.pincusco.com/lightstone-group-acquires-office-condos-in-midtown-for-14-6m-through-bankruptcy/</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>Lightstone Group through the entity 32 W 39th St Owner LLC through a bankruptcy acquired</t>
-        </is>
-      </c>
-      <c r="D6" t="inlineStr"/>
-      <c r="E6" t="inlineStr"/>
-      <c r="F6" t="inlineStr">
-        <is>
-          <t>PincusCo</t>
-        </is>
-      </c>
-      <c r="G6" t="inlineStr">
-        <is>
-          <t>PincusCo - Home</t>
-        </is>
-      </c>
-      <c r="H6" t="inlineStr">
-        <is>
-          <t>Transfers 32 West 39th Street (Credit - Cyclomedia) Lightstone Group through the entity 32 W 39th St Owner LLC through a bankruptcy acquired seven office condominium units at 32 West 39th Street in Grand Central, Manhattan, in a transaction valued at $14.6 million. The former owner, R&amp;B Realty Group through the entity 32 W. 39th Street Sole Member LLC, led by Aron Rosenberg, filed for bankruptcy in 2024. The deal closed on April 23, 2026 and was recorded on May 14, 2026. The seven properties have 33,553 square feet of built space according to a PincusCo analysis of city data. The sale price per built square foot is $435 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) The signatory for the bankrupt affiliate of R&amp;B Realty Group was David Wallace . The signatory for Lightstone Group was Joseph E. Teichman . The contract date was February 11, 2026. This is the lender taking back the property through bankruptcy. Lightstone Group in 2022 provided loans totaling $52 million covering this and other property, then the borrower filed bankruptcy in 2024. The</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>Durgaj Properties signs $10.9M construction loan for 41-unit project in Belmont</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>https://www.pincusco.com/durgaj-properties-signs-10-9m-construction-loan-with-northeast-community-for-development-in-belmont-little-italy/</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>Durgaj Properties through the entity 2278 Arthur Avenue LLC as borrower signed a new construction</t>
-        </is>
-      </c>
-      <c r="D7" t="inlineStr"/>
-      <c r="E7" t="inlineStr"/>
-      <c r="F7" t="inlineStr">
-        <is>
-          <t>PincusCo</t>
-        </is>
-      </c>
-      <c r="G7" t="inlineStr">
-        <is>
-          <t>PincusCo - Home</t>
-        </is>
-      </c>
-      <c r="H7" t="inlineStr">
-        <is>
-          <t>Transfers 2276 Arthur Avenue axonometric diagram (Credit - Jakov Saric architect via DOB) Durgaj Properties through the entity 2278 Arthur Avenue LLC as borrower signed a new construction loan with lender NorthEast Community Bank valued at $10.9 million for the 41-unit project at 2276 Arthur Avenue in Belmont, Bronx. On the lot, there is one active new building construction project, X01245967, for a 41-unit, 27,736 square-foot residential (R-2) building. The project was submitted by Durgaj Properties and filed by Paul Durgaj with plans filed July 3, 2025 and permitted March 30, 2026. The deal closed on May 1, 2026 and was recorded on May 14, 2026. The prior lender was NorthEast Community Bank which held debt that had an original loan amount of $925,000. The loan price per planned development square foot is $393 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) The owner bought the property on July 27, 2023, for $1.9 million. The property The development building with 2 residential units in Belmont/Little Italy has 4,560 square feet of built space and</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>AG Holding Group signs $17M construction loan with Kearny for 67-unit project in Bedford Park</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>https://www.pincusco.com/ag-holding-group-signs-17m-construction-loan-with-kearny-for-67-unit-project-in-bedford-park/</t>
-        </is>
-      </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>AG Holding Group through the entity 21 E 198 Realty LLC as borrower signed a</t>
-        </is>
-      </c>
-      <c r="D8" t="inlineStr"/>
-      <c r="E8" t="inlineStr"/>
-      <c r="F8" t="inlineStr">
-        <is>
-          <t>PincusCo</t>
-        </is>
-      </c>
-      <c r="G8" t="inlineStr">
-        <is>
-          <t>PincusCo - Home</t>
-        </is>
-      </c>
-      <c r="H8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Transfers 21 East 198th Street axonometric diagram (Credit - John Nicholas Backos architect via DOB) AG Holding Group through the entity 21 E 198 Realty LLC as borrower signed a new construction loan with lender Kearny Bank valued at $17 million for the 67-unit project at 21 East 198th Street in Bedford Park, Bronx. On the lot, there is one active new building construction project, X01089171, for a 67-unit, 43,613-square-foot residential (R-2) building. The project is led by Andrea Gjini with plans filed April 23, 2025 and permitted February 9, 2026. The deal closed on April 17, 2026 and was recorded on May 14, 2026. The prior lender was Houlihan &amp; O’Malley Commercial Services which held debt that had an original loan amount of $1.6 million. The loan price per planned development square foot is $390 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) The owner bought the property on October 22, 2024, for $1.8 million. The signatory for AG Holding Group was Andrea Gjini . The signatory for Kearny Bank was Jonathan Atkinson . The property The parcel has </t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>Arker Companies signs $6.3M refi with Customers Bank for retail, parking in Edgemere</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>https://www.pincusco.com/arker-companies-signs-6-3m-refi-with-customers-bank-for-retail-parking-in-edgemere/</t>
-        </is>
-      </c>
-      <c r="C9" t="inlineStr">
-        <is>
-          <t>Arker Companies through the entity Ec A1 Commercial LLC as borrower signed a refi loan</t>
-        </is>
-      </c>
-      <c r="D9" t="inlineStr"/>
-      <c r="E9" t="inlineStr"/>
-      <c r="F9" t="inlineStr">
-        <is>
-          <t>PincusCo</t>
-        </is>
-      </c>
-      <c r="G9" t="inlineStr">
-        <is>
-          <t>PincusCo - Home</t>
-        </is>
-      </c>
-      <c r="H9" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Transfers 5125 Beach Channel Drive and 302 Beach 53rd Street; and the parking condo with the address 5123 Beach Channel Drive (Credit - Cyclomedia) Arker Companies through the entity Ec A1 Commercial LLC as borrower signed a refi loan with lender Customers Bank valued at $6.3 million for three commercial condominium units at the base of a mixed-use building in Edgemere, Queens. The units are two retail condos with the addresses at 5125 Beach Channel Drive and 302 Beach 53rd Street; and the parking condo with the address 5123 Beach Channel Drive. These units are at the base of a residential condominium unit which includes 194 apartments and is not part of this refinance. The deal closed on April 30, 2026 and was recorded on May 11, 2026. The prior lender was Wells Fargo which held debt that had an original loan amount of $6.4 million. The three properties have 49,014 square feet of built space according to a PincusCo analysis of city data. The loan price per built square foot is $128 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) The signatory for </t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>Forest Hill Jewish Center signs $18M initial loan with Valley National Bank in Forest Hills</t>
-        </is>
-      </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>https://www.pincusco.com/forest-hill-jewish-center-signs-18m-initial-loan-with-valley-national-bank-in-forest-hills/</t>
-        </is>
-      </c>
-      <c r="C10" t="inlineStr">
-        <is>
-          <t>Forest Hill Jewish Center through the entity The Forest Hills Jewish Center as borrower signed</t>
-        </is>
-      </c>
-      <c r="D10" t="inlineStr"/>
-      <c r="E10" t="inlineStr"/>
-      <c r="F10" t="inlineStr">
-        <is>
-          <t>PincusCo</t>
-        </is>
-      </c>
-      <c r="G10" t="inlineStr">
-        <is>
-          <t>PincusCo - Home</t>
-        </is>
-      </c>
-      <c r="H10" t="inlineStr">
-        <is>
-          <t>Transfers 106-06 Queens Boulevard (Credit - Cyclomedia) Forest Hill Jewish Center through the entity The Forest Hills Jewish Center as borrower signed a initial loan with lender Valley National Bank valued at $18 million for the property at 106-06 Queens Boulevard in Forest Hills, Queens. The deal closed on April 20, 2026 and was recorded on May 12, 2026. The property has 67,780 square feet of built space according to a PincusCo analysis of city data. The loan price per built square foot is $265 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) The signatory for Forest Hill Jewish Center was Gary Kerzner . The property The property in Forest Hills has 67,780 square feet of built space according to a PincusCo analysis of city data. The parcel has a total lot size of 67,780 square feet. The city-designated market value for the property in 2022 is $22.2 million. Transaction Participants</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto update queens news 2026-05-18T15:55:18Z
</commit_message>
<xml_diff>
--- a/data/output/queens_dev_news.xlsx
+++ b/data/output/queens_dev_news.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H1"/>
+  <dimension ref="A1:H10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -470,6 +470,312 @@
         </is>
       </c>
     </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>EMP Capital Group files plans for 198 units in Astoria</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>https://www.pincusco.com/emp-capital-group-files-plans-for-198-units-in-astoria/</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>EMP Capital Group filed two new building plans, each with 99 units, for a total</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr"/>
+      <c r="E2" t="inlineStr"/>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>PincusCo</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>PincusCo - Home</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>Development 35-43 37th Street (Credit - Cyclomedia) EMP Capital Group filed two new building plans, each with 99 units, for a total of 198 units in Astoria, Queens. The filings show the zoning lot includes five tax lots, including lot 1, which EMP Capital Group purchased for $15.4 million in February 2026. In the first filing, EMP Capital Group submitted a new building construction project for a 99-unit, 111,492-square-foot residential (R-2) building at 37-09 36th Avenue in Astoria, Queens. The plan was filed on May 12, 2026. It calls for the construction of a 285-foot-tall, 26-story building and was filed with the New York City Department of Buildings under job number Q01388823. The project is described in the filing as: proposed twenty-six (26) story + cellar mixed-use building.. The applicant is the Registered Architect Ralph Kowalcyzk of Issac &amp; Stern Architects, P.C. Elie Pariente of EMP Capital Group submitted the plans. In the second, EMP Capital Group submitted a new building construction project for a 99-unit, 90,058-square-foot residential (R-2) building at 35-43 37th Street in Astoria, Queens. The plan was filed on May 13, 2026. It calls for the construction of a 285-foo</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Indigo Developers files plans for 69 units in Bedford Park</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>https://www.pincusco.com/indigo-developers-files-plans-for-69-units-in-bedford-park/</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Indigo Developers submitted a new building construction project for a 69-unit, 6,088-square-foot residential (R-2) building</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr"/>
+      <c r="E3" t="inlineStr"/>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>PincusCo</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>PincusCo - Home</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>Development 201 East 198th Street axonometric diagram (Credit- Nikolai Katz architect via DOB) Indigo Developers submitted a new building construction project for a 69-unit, 6,088-square-foot residential (R-2) building at 201 East 198th Street in Bedford Park, Bronx. The plan was filed on May 14, 2026. It calls for the construction of a 123-foot-tall, thirteen-story building and was filed with the New York City Department of Buildings under job number X01401011. The project is described in the filing as: (please assign to dev hub) proposing new 13 story building with a total of 69 dwelling units. The applicant is the Registered Architect Nikolai Katz of Nikolai Katz Architect. Yanky Indig of Indigo Developers submitted the plans. The neighborhood In Bedford Park, The bulk, or 49 percent of the 20.3 million square feet of commercial built space are elevator buildings, with walkup buildings next occupying 27 percent of the space. In sales, Bedford Park has near average sales volume among other neighborhoods with $164 million in sales volume in the last two years and is the 6th highest in Bronx. For development, Bedford Park has near average amount of major developments among other ne</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Joseph Rukaj signs $11.6M construction loan with Bayport for development in Kingsbridge Heights</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>https://www.pincusco.com/joseph-rukaj-signs-11-6m-construction-loan-with-bayport-for-development-in-kingsbridge-heights/</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Joseph Rukaj through the entity 3852 Bailey Ave Property LLC as borrower signed a new</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr"/>
+      <c r="E4" t="inlineStr"/>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>PincusCo</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>PincusCo - Home</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>Transfers 3848 Bailey Avenue axonometric diagram (Credit - Jakov Saric architect via DOB) Joseph Rukaj through the entity 3852 Bailey Ave Property LLC as borrower signed a new construction loan with lender Bayport Funding through the entity Bayport Funding LLC valued at $11.6 million for the three-unit development building (V0) at 3848 Bailey Avenue in Kingsbridge Heights, Bronx. On the lot, there is one active new building construction project, X01244736, for a 41-unit, 27,890 square-foot residential (R-2) building. The project was submitted by Joseph Rukaj and filed by Joseph Rukaj with plans filed October 9, 2025 and it has not been permitted yet. The deal closed on April 28, 2026 and was recorded on May 15, 2026. The property has 1,440 square feet of built space and 10,780 square feet of additional air rights for a total buildable of 10,780 square feet according to a PincusCo analysis of city data. The loan price per built square foot is $8,046 and the price per buildable square foot is $1,074 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) The</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Highpoint Property signs $14.8M refi with Natixis for 12 units in East Village</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>https://www.pincusco.com/highpoint-property-signs-14-8m-refi-with-natixis-for-12-units-in-east-village/</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Highpoint Property Group through the entity 436 And 442 East 13th Street Owner LLC as</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr"/>
+      <c r="E5" t="inlineStr"/>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>PincusCo</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>PincusCo - Home</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Transfers 436 East 13th Street (Credit - Cyclomedia) Highpoint Property Group through the entity 436 And 442 East 13th Street Owner LLC as borrower signed a refi loan with lender Natixis through the entity Natixis Real Estate Capital LLC valued at $14.8 million for two residential elevator properties with 12 residential units including the six-unit residential elevator building (D3) at 436 East 13th Street and six-unit residential elevator building (D3) at 442 East 13th Street in East Village, Manhattan. The deal closed on May 7, 2026 and was recorded on May 15, 2026. The prior lender was Prime Finance which held debt that had an original loan amount of $16 million.The two properties have 25,444 square feet of built space according to a PincusCo analysis of city data. The loan price per built square foot is $581 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) The signatory for Highpoint Property Group was Drew Popkin . The signatory for Natixis was Jonathan Rechner and Melissa Naturman . Prior sales, articles and revenue The owner according to the </t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Seema Vaid signs $37M refi for hotel, retail in Lower East Side</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>https://www.pincusco.com/seema-vaid-signs-37m-refi-for-four-properties-in-lower-east-side/</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Seema Vaid through the entity The Downtown LLC as borrower signed a refi loan with</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr"/>
+      <c r="E6" t="inlineStr"/>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>PincusCo</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>PincusCo - Home</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>Transfers 107 Rivington Street (Credit - Cyclomedia) Seema Vaid through the entity The Downtown LLC as borrower signed a refi loan with lender Bank of America at $37 million for four properties in the Lower East Side, Manhattan, with 11 residential units including the Hotel on Rivington building (H2) at 107 Rivington Street, the retail building (K4) at 105 Rivington Street, and the three-unit mixed-use building (S9) at 121 Essex Street. The deal closed on May 6, 2026 and was recorded on May 15, 2026. The prior lender was was the trust Series 2016-GC37 serviced by Trimont which held debt that had an original loan amount of $36.5 million. The four properties have 76,514 square feet of built space and 3,492 square feet of additional air rights according to a PincusCo analysis of city data. The loan price per built square foot is $483 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) The signatory for Seema Vaid was Seema Vaid. The signatory for Bank of America was Kathleen Flock . Because multiple properties have been transacted, some of the following s</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Haussmann signs $40.8M construction loan with AmFirst for 84-unit project in Harlem</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>https://www.pincusco.com/haussmann-signs-40-8m-construction-loan-with-amfirst-for-84-unit-project-in-harlem/</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Haussmann Development through the entity 16 Convent LLC as borrower signed a new construction loan</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr"/>
+      <c r="E7" t="inlineStr"/>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>PincusCo</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>PincusCo - Home</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>Transfers 16 Convent Avenue axonometric diagram (Credit - Nickolas D. Kazalas architect via DOB) Haussmann Development through the entity 16 Convent LLC as borrower signed a new construction loan with lender AmFirst Life Insurance Company through the entity Amfirst Life Insurance Company I.I., For The valued at $40.8 million for the industrial building (G7) at 16 Convent Avenue in Harlem, Manhattan. On the lot, there is one active new building construction project, M01274493, for a 84-unit, 65,170 square-foot residential (R-2) building. The project was submitted by Haussmann Development and filed by Josef Goodman with plans filed September 12, 2025 and permitted May 1, 2026. The deal closed on May 7, 2026 and was recorded on May 15, 2026. The property has zero square feet of built space and 30,528 square feet of additional air rights for a total buildable of 30,528 square feet according to a PincusCo analysis of city data. The loan price per built square foot is $N/A and the price per buildable square foot is $1,334 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights h</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Midwood Investment signs $200M construction loan with Affinius for residential elevator in Gowanus</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>https://www.pincusco.com/midwood-investment-signs-200m-construction-loan-with-affinius-for-residential-elevator-in-gowanus/</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Midwood Investment &amp; Development through the entity Dobode Holdings LLC as borrower signed a new</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr"/>
+      <c r="E8" t="inlineStr"/>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>PincusCo</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>PincusCo - Home</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>Transfers 192 Douglass Street axonometric diagram (Credit - Manish Chadha architect via DOB) Midwood Investment &amp; Development through the entity Dobode Holdings LLC as borrower signed a new construction loan with lender Affinius Capital through the entity Sm Tactical Finance Iii-J LLC valued at $200 million for the 274-unit residential elevator building (D7) at 192 Douglass Street in Gowanus, Brooklyn. On the lot, there is one active new building construction project, B00621504, for a 274-unit, 241,789 square-foot residential (R-2) building. The project was submitted by Midwood Investment &amp; Development and filed by John Usdan with plans filed December 1, 2021 and permitted December 17, 2025. The deal closed on December 10, 2025 and was recorded on May 15, 2026. The prior lender was Affinius Capital which held debt that had an original loan amount of $14.2 million.The property has 301,105 square feet of built space according to a PincusCo analysis of city data. The loan price per built square foot is $664 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sol</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>JEMB Realty signs $186.5M refi for 375-unit rental in Windsor Terrace</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>https://www.pincusco.com/jemb-realty-signs-186-5m-refi-for-375-unit-rental-in-windsor-terrace/</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>JEMB Realty through the entity 312 Coney Island Avenue LLC as borrower signed a refi</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr"/>
+      <c r="E9" t="inlineStr"/>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>PincusCo</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>PincusCo - Home</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>Transfers 11 Ocean Parkway (Credit - Cyclomedia) JEMB Realty through the entity 312 Coney Island Avenue LLC as borrower signed a refi loan with lender Deutsche Bank valued at $186.5 million for the 375-unit residential elevator building (D7) at 11 Ocean Parkway in Windsor Terrace, Brooklyn. The deal closed on May 7, 2026 and was recorded on May 15, 2026. The prior lender was Wells Fargo which held debt that had an original loan amount of $149 million. The property has 393,092 square feet of built space according to a PincusCo analysis of city data. The loan price per built square foot is $474 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) The signatory for JEMB Realty was Morris Jerome . The signatory for Deutsche Bank was Peter Castro and David Goodman . Prior sales, articles and revenue The owners according to the Department of Housing Preservation and Development includes Dennis Rauchet, head officer and Sebastian Fileccia, site manager. The business entities are Rose Property Mgmt Grp Llc and 312 Coney Island Avenue Llc. The 393,092-square-foo</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Soloviev signs $1.8B refi with Bank of America, Wells Fargo, Citibank for 9 West 57th in Midtown West</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>https://www.pincusco.com/soloviev-signs-1-8b-refi-with-bank-of-america-wells-fargo-citibank-for-9-west-57th-in-midtown-west/</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Soloviev Group through the entity Solow Building Company II, L.L.C. as borrower signed a refi</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr"/>
+      <c r="E10" t="inlineStr"/>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>PincusCo</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>PincusCo - Home</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>Transfers 9 West 57th Street (Credit - Cyclomedia) Soloviev Group through the entity Solow Building Company II, L.L.C. as borrower signed a refi loan with lender Bank of America, Wells Fargo, and Citibank valued at $1800 million for the office building (O4) at 9 West 57th Street in Midtown West, Manhattan. The deal closed on May 8, 2026 and was recorded on May 15, 2026. The prior lender was the trust Series 2016-Nine serviced by Trimont which held debt that had an original loan amount of $1.2 billion. The property has 1,698,259 square feet of built space according to a PincusCo analysis of city data. The loan price per built square foot is $1,059 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) The signatory for Soloviev Group was Stefan Q. Soloviev . The signatory for Bank of America , Wells Fargo , and Citibank was Steven Wasser , John G. Nicol , and Jonathan Misher . Simultaneously with the refinancing, Stefan Soloviev terminated a 99-year ground lease executed in 1968 that his late father Sheldon Solow signed with himself as both landlord and te</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
auto update queens news 2026-05-19T15:47:28Z
</commit_message>
<xml_diff>
--- a/data/output/queens_dev_news.xlsx
+++ b/data/output/queens_dev_news.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H10"/>
+  <dimension ref="A1:H7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -473,17 +473,17 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>EMP Capital Group files plans for 198 units in Astoria</t>
+          <t>Shabse Fuchs files plans for 50 units in Tribeca</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>https://www.pincusco.com/emp-capital-group-files-plans-for-198-units-in-astoria/</t>
+          <t>https://www.pincusco.com/shabse-fuchs-files-plans-for-50-units-in-tribeca/</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>EMP Capital Group filed two new building plans, each with 99 units, for a total</t>
+          <t>Shabse Fuchs submitted a new building construction project for a 50-unit, 51,008-square-foot residential (R-2) building</t>
         </is>
       </c>
       <c r="D2" t="inlineStr"/>
@@ -500,24 +500,24 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>Development 35-43 37th Street (Credit - Cyclomedia) EMP Capital Group filed two new building plans, each with 99 units, for a total of 198 units in Astoria, Queens. The filings show the zoning lot includes five tax lots, including lot 1, which EMP Capital Group purchased for $15.4 million in February 2026. In the first filing, EMP Capital Group submitted a new building construction project for a 99-unit, 111,492-square-foot residential (R-2) building at 37-09 36th Avenue in Astoria, Queens. The plan was filed on May 12, 2026. It calls for the construction of a 285-foot-tall, 26-story building and was filed with the New York City Department of Buildings under job number Q01388823. The project is described in the filing as: proposed twenty-six (26) story + cellar mixed-use building.. The applicant is the Registered Architect Ralph Kowalcyzk of Issac &amp; Stern Architects, P.C. Elie Pariente of EMP Capital Group submitted the plans. In the second, EMP Capital Group submitted a new building construction project for a 99-unit, 90,058-square-foot residential (R-2) building at 35-43 37th Street in Astoria, Queens. The plan was filed on May 13, 2026. It calls for the construction of a 285-foo</t>
+          <t>Development 317 Broadway (Credit - Cyclomedia) Shabse Fuchs submitted a new building construction project for a 50-unit, 51,008-square-foot residential (R-2) building at 317 Broadway in Tribeca, Manhattan. The plan was filed on May 15, 2026. It calls for the construction of a 215-foot-tall, 21-story building and was filed with the New York City Department of Buildings under job number M01400243. The project is described in the filing as: proposed twenty-one story mixed-use building with cellar. The applicant is the Registered Architect Hamish Whitefield of Hamish Whitefield Architects P.C. Shabse Fuchs of Steel Boyz submitted the plans. The city property website Acris shows the Laboz family’s United American Land as the owner of the parcels at 315 Broadway and 317 Broadway. 315 Broadway is a landmarked building. The city’s Landmarks Preservation Commission approved a plan United American Land submitted in 2020 for a larger building at 315 and 317 Broadway. This new proposed building uses 13,000 square feet of development rights from 315 Broadway, but only rises above 317 Broadway’s lot, a PincusCo analysis of DOB records shows. 317 Broadway The neighborhood In Tribeca, The bulk, or</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Indigo Developers files plans for 69 units in Bedford Park</t>
+          <t>Olymbec, Lockhill pay $11.1M for 15-unit walkup in East Village</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>https://www.pincusco.com/indigo-developers-files-plans-for-69-units-in-bedford-park/</t>
+          <t>https://www.pincusco.com/olymbec-lockhill-pay-11-1m-for-15-unit-walkup-in-east-village/</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Indigo Developers submitted a new building construction project for a 69-unit, 6,088-square-foot residential (R-2) building</t>
+          <t>Montreal-based Olymbec and Lockhill Properties through the entity 21-23 East 7th LLC paid $11.1 million</t>
         </is>
       </c>
       <c r="D3" t="inlineStr"/>
@@ -534,24 +534,24 @@
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>Development 201 East 198th Street axonometric diagram (Credit- Nikolai Katz architect via DOB) Indigo Developers submitted a new building construction project for a 69-unit, 6,088-square-foot residential (R-2) building at 201 East 198th Street in Bedford Park, Bronx. The plan was filed on May 14, 2026. It calls for the construction of a 123-foot-tall, thirteen-story building and was filed with the New York City Department of Buildings under job number X01401011. The project is described in the filing as: (please assign to dev hub) proposing new 13 story building with a total of 69 dwelling units. The applicant is the Registered Architect Nikolai Katz of Nikolai Katz Architect. Yanky Indig of Indigo Developers submitted the plans. The neighborhood In Bedford Park, The bulk, or 49 percent of the 20.3 million square feet of commercial built space are elevator buildings, with walkup buildings next occupying 27 percent of the space. In sales, Bedford Park has near average sales volume among other neighborhoods with $164 million in sales volume in the last two years and is the 6th highest in Bronx. For development, Bedford Park has near average amount of major developments among other ne</t>
+          <t>Transfers 21 East 7th Street (Credit - Cyclomedia) Montreal-based Olymbec and Lockhill Properties through the entity 21-23 East 7th LLC paid $11.1 million to Christina Isaly through the entity Cooper Partners for the 15-unit residential walkup building (C7) at 21-23 East 7th Street in East Village, Manhattan. The expected use is cash flowing. The deal closed on April 28, 2026 and was recorded on May 18, 2026. The property has 14,400 square feet of built space and 1,209 square feet of additional air rights for a total buildable of 15,600 square feet according to a PincusCo analysis of city data. The sale price per built square foot is $770 and the price per buildable square foot is $711 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) The signatory for Christina Isaly was Christina P. Isaly. The signatory for Olymbec and Lockhill Properties was Jason Berger. The contract date was January 28, 2026. Lockhill Properties acquired a 25% stake, while Olymbec acquired 75%. Prior sales, articles and revenue Prior to this transaction, PincusCo has no record t</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Joseph Rukaj signs $11.6M construction loan with Bayport for development in Kingsbridge Heights</t>
+          <t>Extell pays $19M to Kairos for Friars Club building in Midtown East</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>https://www.pincusco.com/joseph-rukaj-signs-11-6m-construction-loan-with-bayport-for-development-in-kingsbridge-heights/</t>
+          <t>https://www.pincusco.com/extell-pays-19m-to-kairos-for-friars-club-building-in-midtown-east/</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Joseph Rukaj through the entity 3852 Bailey Ave Property LLC as borrower signed a new</t>
+          <t>Extell Development through the entity 57 East 55th Street LLC paid $19 million to Kairos</t>
         </is>
       </c>
       <c r="D4" t="inlineStr"/>
@@ -568,24 +568,24 @@
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>Transfers 3848 Bailey Avenue axonometric diagram (Credit - Jakov Saric architect via DOB) Joseph Rukaj through the entity 3852 Bailey Ave Property LLC as borrower signed a new construction loan with lender Bayport Funding through the entity Bayport Funding LLC valued at $11.6 million for the three-unit development building (V0) at 3848 Bailey Avenue in Kingsbridge Heights, Bronx. On the lot, there is one active new building construction project, X01244736, for a 41-unit, 27,890 square-foot residential (R-2) building. The project was submitted by Joseph Rukaj and filed by Joseph Rukaj with plans filed October 9, 2025 and it has not been permitted yet. The deal closed on April 28, 2026 and was recorded on May 15, 2026. The property has 1,440 square feet of built space and 10,780 square feet of additional air rights for a total buildable of 10,780 square feet according to a PincusCo analysis of city data. The loan price per built square foot is $8,046 and the price per buildable square foot is $1,074 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) The</t>
+          <t>Transfers 57 East 55th Street (Credit - Cyclomedia) Extell Development through the entity 57 East 55th Street LLC paid $19 million to Kairos Investment Management Company through the entity Kairos Friars Club Re, LLC for the landmarked Friars Club building (P9) at 57 East 55th Street in Midtown East, Manhattan. The expected use is cash flowing. The deal closed on April 23, 2026 and was recorded on May 18, 2026. The property has 14,541 square feet of built space according to a PincusCo analysis of city data. The sale price per built square foot is $1,306 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) The seller, the former lender, acquired the property on February 21, 2025, in a transaction valued at $15.5 million. The signatory for Kairos Investment Management Company was Jonathan A. Needell . The signatory for Extell Development was Marc Kwestel . The contract date was December 18, 2025. Prior sales, articles and revenue Prior to this transaction, PincusCo has records that the buyer Extell Development purchased 32 properties in 16 transactions fo</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Highpoint Property signs $14.8M refi with Natixis for 12 units in East Village</t>
+          <t>David Brecher pays $23.5M to Warren Cohen for 119-unit rental in Midwood</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>https://www.pincusco.com/highpoint-property-signs-14-8m-refi-with-natixis-for-12-units-in-east-village/</t>
+          <t>https://www.pincusco.com/david-brecher-pays-23-5m-to-warren-cohen-for-residential-elevator-in-midwood/</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Highpoint Property Group through the entity 436 And 442 East 13th Street Owner LLC as</t>
+          <t>David Brecher through the entity Brelan 1000 Ocean Parkway LLC paid $23.5 million to Warren</t>
         </is>
       </c>
       <c r="D5" t="inlineStr"/>
@@ -602,24 +602,24 @@
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Transfers 436 East 13th Street (Credit - Cyclomedia) Highpoint Property Group through the entity 436 And 442 East 13th Street Owner LLC as borrower signed a refi loan with lender Natixis through the entity Natixis Real Estate Capital LLC valued at $14.8 million for two residential elevator properties with 12 residential units including the six-unit residential elevator building (D3) at 436 East 13th Street and six-unit residential elevator building (D3) at 442 East 13th Street in East Village, Manhattan. The deal closed on May 7, 2026 and was recorded on May 15, 2026. The prior lender was Prime Finance which held debt that had an original loan amount of $16 million.The two properties have 25,444 square feet of built space according to a PincusCo analysis of city data. The loan price per built square foot is $581 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) The signatory for Highpoint Property Group was Drew Popkin . The signatory for Natixis was Jonathan Rechner and Melissa Naturman . Prior sales, articles and revenue The owner according to the </t>
+          <t>Transfers 996 Ocean Parkway (Credit - Cyclomedia) David Brecher through the entity Brelan 1000 Ocean Parkway LLC paid $23.5 million to Warren Cohen through the entity Parcjay Apartments, LLC for the 119-unit residential elevator building (D7) at 996 Ocean Parkway in Midwood, Brooklyn. The expected use is cash flowing. The deal closed on May 12, 2026 and was recorded on May 18, 2026. The property has 154,378 square feet of built space according to a PincusCo analysis of city data. The sale price per built square foot is $152 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) The seller bought the property on August 1, 2024, for $1.2 million. The signatory for Warren Cohen was Warren Cohen. The signatory for David Brecher was David Brecher . The contract date was December 30, 2025. Prior sales, articles and revenue Prior to this transaction, PincusCo has no record that the buyer had purchased any other properties and has no record it sold any properties over the past 24 months. The seller Warren Cohen had not purchased any other properties and had not s</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Seema Vaid signs $37M refi for hotel, retail in Lower East Side</t>
+          <t>Adam Woodward affiliate pays $45M for mixed-use in Nolita, adds to assemblage</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>https://www.pincusco.com/seema-vaid-signs-37m-refi-for-four-properties-in-lower-east-side/</t>
+          <t>https://www.pincusco.com/adam-woodward-affiliate-pays-45m-for-mixed-use-in-nolita-adds-to-assemblage/</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Seema Vaid through the entity The Downtown LLC as borrower signed a refi loan with</t>
+          <t>Adam Woodward through the entity TTC Investments XV LLC in care of Building Equity Management,</t>
         </is>
       </c>
       <c r="D6" t="inlineStr"/>
@@ -636,24 +636,24 @@
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>Transfers 107 Rivington Street (Credit - Cyclomedia) Seema Vaid through the entity The Downtown LLC as borrower signed a refi loan with lender Bank of America at $37 million for four properties in the Lower East Side, Manhattan, with 11 residential units including the Hotel on Rivington building (H2) at 107 Rivington Street, the retail building (K4) at 105 Rivington Street, and the three-unit mixed-use building (S9) at 121 Essex Street. The deal closed on May 6, 2026 and was recorded on May 15, 2026. The prior lender was was the trust Series 2016-GC37 serviced by Trimont which held debt that had an original loan amount of $36.5 million. The four properties have 76,514 square feet of built space and 3,492 square feet of additional air rights according to a PincusCo analysis of city data. The loan price per built square foot is $483 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) The signatory for Seema Vaid was Seema Vaid. The signatory for Bank of America was Kathleen Flock . Because multiple properties have been transacted, some of the following s</t>
+          <t>Chart_Frontpage Top Story Transfers 236 Bowery (Credit - Cyclomedia) Adam Woodward through the entity TTC Investments XV LLC in care of Building Equity Management, paid $45 million to Anton Mayer as heir to the late Frank D. Carone through the entity 236 Bowery LLC for the mixed-use building (K4) at 236 Bowery in Nolita, Manhattan. The expected use is ground up development. The deal closed on May 12, 2026 and was recorded on May 18, 2026. The property has 10,054 square feet of built space and 6,737 square feet of additional air rights for a total buildable of 16,794 square feet according to a PincusCo analysis of city data. The sale price per built square foot is $4,473 and the price per buildable square foot is $2,678 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) The signatory for Anton Mayer and Frank D. Carone was Anton F. Mayer . The signatory for Adam Woodward was David Dailey. The contract date was March 26, 2026. Frank D. Carone owned a 70% stake in a portfolio of companies that owned a restaurant supply company and real estate on the Bowe</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Haussmann signs $40.8M construction loan with AmFirst for 84-unit project in Harlem</t>
+          <t>Hennick &amp; Company pays $66.2M to BD Hotels for hotel in Midtown West</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>https://www.pincusco.com/haussmann-signs-40-8m-construction-loan-with-amfirst-for-84-unit-project-in-harlem/</t>
+          <t>https://www.pincusco.com/hennick-company-pays-66-2m-to-bd-hotels-for-hotel-in-midtown-west/</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Haussmann Development through the entity 16 Convent LLC as borrower signed a new construction loan</t>
+          <t>Toronto-based Hennick &amp; Company through the entity 15 West 56th St Inc paid $66.2 million</t>
         </is>
       </c>
       <c r="D7" t="inlineStr"/>
@@ -670,109 +670,7 @@
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>Transfers 16 Convent Avenue axonometric diagram (Credit - Nickolas D. Kazalas architect via DOB) Haussmann Development through the entity 16 Convent LLC as borrower signed a new construction loan with lender AmFirst Life Insurance Company through the entity Amfirst Life Insurance Company I.I., For The valued at $40.8 million for the industrial building (G7) at 16 Convent Avenue in Harlem, Manhattan. On the lot, there is one active new building construction project, M01274493, for a 84-unit, 65,170 square-foot residential (R-2) building. The project was submitted by Haussmann Development and filed by Josef Goodman with plans filed September 12, 2025 and permitted May 1, 2026. The deal closed on May 7, 2026 and was recorded on May 15, 2026. The property has zero square feet of built space and 30,528 square feet of additional air rights for a total buildable of 30,528 square feet according to a PincusCo analysis of city data. The loan price per built square foot is $N/A and the price per buildable square foot is $1,334 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights h</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>Midwood Investment signs $200M construction loan with Affinius for residential elevator in Gowanus</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>https://www.pincusco.com/midwood-investment-signs-200m-construction-loan-with-affinius-for-residential-elevator-in-gowanus/</t>
-        </is>
-      </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>Midwood Investment &amp; Development through the entity Dobode Holdings LLC as borrower signed a new</t>
-        </is>
-      </c>
-      <c r="D8" t="inlineStr"/>
-      <c r="E8" t="inlineStr"/>
-      <c r="F8" t="inlineStr">
-        <is>
-          <t>PincusCo</t>
-        </is>
-      </c>
-      <c r="G8" t="inlineStr">
-        <is>
-          <t>PincusCo - Home</t>
-        </is>
-      </c>
-      <c r="H8" t="inlineStr">
-        <is>
-          <t>Transfers 192 Douglass Street axonometric diagram (Credit - Manish Chadha architect via DOB) Midwood Investment &amp; Development through the entity Dobode Holdings LLC as borrower signed a new construction loan with lender Affinius Capital through the entity Sm Tactical Finance Iii-J LLC valued at $200 million for the 274-unit residential elevator building (D7) at 192 Douglass Street in Gowanus, Brooklyn. On the lot, there is one active new building construction project, B00621504, for a 274-unit, 241,789 square-foot residential (R-2) building. The project was submitted by Midwood Investment &amp; Development and filed by John Usdan with plans filed December 1, 2021 and permitted December 17, 2025. The deal closed on December 10, 2025 and was recorded on May 15, 2026. The prior lender was Affinius Capital which held debt that had an original loan amount of $14.2 million.The property has 301,105 square feet of built space according to a PincusCo analysis of city data. The loan price per built square foot is $664 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sol</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>JEMB Realty signs $186.5M refi for 375-unit rental in Windsor Terrace</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>https://www.pincusco.com/jemb-realty-signs-186-5m-refi-for-375-unit-rental-in-windsor-terrace/</t>
-        </is>
-      </c>
-      <c r="C9" t="inlineStr">
-        <is>
-          <t>JEMB Realty through the entity 312 Coney Island Avenue LLC as borrower signed a refi</t>
-        </is>
-      </c>
-      <c r="D9" t="inlineStr"/>
-      <c r="E9" t="inlineStr"/>
-      <c r="F9" t="inlineStr">
-        <is>
-          <t>PincusCo</t>
-        </is>
-      </c>
-      <c r="G9" t="inlineStr">
-        <is>
-          <t>PincusCo - Home</t>
-        </is>
-      </c>
-      <c r="H9" t="inlineStr">
-        <is>
-          <t>Transfers 11 Ocean Parkway (Credit - Cyclomedia) JEMB Realty through the entity 312 Coney Island Avenue LLC as borrower signed a refi loan with lender Deutsche Bank valued at $186.5 million for the 375-unit residential elevator building (D7) at 11 Ocean Parkway in Windsor Terrace, Brooklyn. The deal closed on May 7, 2026 and was recorded on May 15, 2026. The prior lender was Wells Fargo which held debt that had an original loan amount of $149 million. The property has 393,092 square feet of built space according to a PincusCo analysis of city data. The loan price per built square foot is $474 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) The signatory for JEMB Realty was Morris Jerome . The signatory for Deutsche Bank was Peter Castro and David Goodman . Prior sales, articles and revenue The owners according to the Department of Housing Preservation and Development includes Dennis Rauchet, head officer and Sebastian Fileccia, site manager. The business entities are Rose Property Mgmt Grp Llc and 312 Coney Island Avenue Llc. The 393,092-square-foo</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>Soloviev signs $1.8B refi with Bank of America, Wells Fargo, Citibank for 9 West 57th in Midtown West</t>
-        </is>
-      </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>https://www.pincusco.com/soloviev-signs-1-8b-refi-with-bank-of-america-wells-fargo-citibank-for-9-west-57th-in-midtown-west/</t>
-        </is>
-      </c>
-      <c r="C10" t="inlineStr">
-        <is>
-          <t>Soloviev Group through the entity Solow Building Company II, L.L.C. as borrower signed a refi</t>
-        </is>
-      </c>
-      <c r="D10" t="inlineStr"/>
-      <c r="E10" t="inlineStr"/>
-      <c r="F10" t="inlineStr">
-        <is>
-          <t>PincusCo</t>
-        </is>
-      </c>
-      <c r="G10" t="inlineStr">
-        <is>
-          <t>PincusCo - Home</t>
-        </is>
-      </c>
-      <c r="H10" t="inlineStr">
-        <is>
-          <t>Transfers 9 West 57th Street (Credit - Cyclomedia) Soloviev Group through the entity Solow Building Company II, L.L.C. as borrower signed a refi loan with lender Bank of America, Wells Fargo, and Citibank valued at $1800 million for the office building (O4) at 9 West 57th Street in Midtown West, Manhattan. The deal closed on May 8, 2026 and was recorded on May 15, 2026. The prior lender was the trust Series 2016-Nine serviced by Trimont which held debt that had an original loan amount of $1.2 billion. The property has 1,698,259 square feet of built space according to a PincusCo analysis of city data. The loan price per built square foot is $1,059 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) The signatory for Soloviev Group was Stefan Q. Soloviev . The signatory for Bank of America , Wells Fargo , and Citibank was Steven Wasser , John G. Nicol , and Jonathan Misher . Simultaneously with the refinancing, Stefan Soloviev terminated a 99-year ground lease executed in 1968 that his late father Sheldon Solow signed with himself as both landlord and te</t>
+          <t xml:space="preserve">Top Story Transfers 15 West 56th Street (Credit - Cyclomedia) Toronto-based Hennick &amp; Company through the entity 15 West 56th St Inc paid $66.2 million to BD Hotels through the entity BDC 56 LLC for the closed Chambers Hotel building (H1) at 13-15 West 56th Street in Midtown West, Manhattan. The deal closed on May 5, 2026 and was recorded on May 18, 2026. The property has 54,959 square feet of built space according to a PincusCo analysis of city data. The sale price per built square foot is $1,204 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) The signatory for BD Hotels was Richard Born . The signatory for Hennick &amp; Company was Jory Hennick . The contract date was March 21, 2026. In November 1998, BD Hotels purchased the property from the Gottesman family for $5.2 million, according to a PincusCo analysis of the transfer records, borrowing in 1999 $4.25 million. The Commercial Observer reported on the sale yesterday. Prior sales, articles and revenue Prior to this transaction, PincusCo has no record that the buyer Hennick &amp; Company had purchased </t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto update queens news 2026-05-20T15:53:36Z
</commit_message>
<xml_diff>
--- a/data/output/queens_dev_news.xlsx
+++ b/data/output/queens_dev_news.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H7"/>
+  <dimension ref="A1:H10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -473,17 +473,17 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Shabse Fuchs files plans for 50 units in Tribeca</t>
+          <t>Heartfelt Townhouse Builders files plans for 74 units in Jamaica</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>https://www.pincusco.com/shabse-fuchs-files-plans-for-50-units-in-tribeca/</t>
+          <t>https://www.pincusco.com/heartfelt-townhouse-builders-files-plans-for-74-units-in-jamaica/</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Shabse Fuchs submitted a new building construction project for a 50-unit, 51,008-square-foot residential (R-2) building</t>
+          <t>Heartfelt Townhouse Builders submitted a new building construction project for a 74-unit, 58,408-square-foot residential (R-2)</t>
         </is>
       </c>
       <c r="D2" t="inlineStr"/>
@@ -500,24 +500,24 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>Development 317 Broadway (Credit - Cyclomedia) Shabse Fuchs submitted a new building construction project for a 50-unit, 51,008-square-foot residential (R-2) building at 317 Broadway in Tribeca, Manhattan. The plan was filed on May 15, 2026. It calls for the construction of a 215-foot-tall, 21-story building and was filed with the New York City Department of Buildings under job number M01400243. The project is described in the filing as: proposed twenty-one story mixed-use building with cellar. The applicant is the Registered Architect Hamish Whitefield of Hamish Whitefield Architects P.C. Shabse Fuchs of Steel Boyz submitted the plans. The city property website Acris shows the Laboz family’s United American Land as the owner of the parcels at 315 Broadway and 317 Broadway. 315 Broadway is a landmarked building. The city’s Landmarks Preservation Commission approved a plan United American Land submitted in 2020 for a larger building at 315 and 317 Broadway. This new proposed building uses 13,000 square feet of development rights from 315 Broadway, but only rises above 317 Broadway’s lot, a PincusCo analysis of DOB records shows. 317 Broadway The neighborhood In Tribeca, The bulk, or</t>
+          <t>Development 143-24 94th Avenue axonometric diagram (Credit - Joseph Frankl architect via DOB) Heartfelt Townhouse Builders submitted a new building construction project for a 74-unit, 58,408-square-foot residential (R-2) building at 143-24 94 Avenue in Jamaica, Queens. The plan was filed on May 18, 2026. It calls for the construction of a 145-foot-tall, fourteen-story building and was filed with the New York City Department of Buildings under job number Q01377260. The project is described in the filing as: proposed fourteen (14) story residential use building. The applicant is the Registered Architect Joseph Frankl of JFA Architects &amp; Engineers. Joel Weiss of Heartfelt Townhouse Builders submitted the plans. The plans call for a fitness center and recreation room on the first floor, and apartments on floors two to 14. 143-24 94th Avenue The neighborhood</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Olymbec, Lockhill pay $11.1M for 15-unit walkup in East Village</t>
+          <t>Maddd Equities pays $6.8M for likely dev site in Mott Haven</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>https://www.pincusco.com/olymbec-lockhill-pay-11-1m-for-15-unit-walkup-in-east-village/</t>
+          <t>https://www.pincusco.com/maddd-equities-pays-6-8m-to-for-likely-dev-site-in-mott-haven/</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Montreal-based Olymbec and Lockhill Properties through the entity 21-23 East 7th LLC paid $11.1 million</t>
+          <t>Maddd Equities through the entity 825 E 140 Street LLC paid $6.8 million to Raz</t>
         </is>
       </c>
       <c r="D3" t="inlineStr"/>
@@ -534,24 +534,24 @@
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>Transfers 21 East 7th Street (Credit - Cyclomedia) Montreal-based Olymbec and Lockhill Properties through the entity 21-23 East 7th LLC paid $11.1 million to Christina Isaly through the entity Cooper Partners for the 15-unit residential walkup building (C7) at 21-23 East 7th Street in East Village, Manhattan. The expected use is cash flowing. The deal closed on April 28, 2026 and was recorded on May 18, 2026. The property has 14,400 square feet of built space and 1,209 square feet of additional air rights for a total buildable of 15,600 square feet according to a PincusCo analysis of city data. The sale price per built square foot is $770 and the price per buildable square foot is $711 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) The signatory for Christina Isaly was Christina P. Isaly. The signatory for Olymbec and Lockhill Properties was Jason Berger. The contract date was January 28, 2026. Lockhill Properties acquired a 25% stake, while Olymbec acquired 75%. Prior sales, articles and revenue Prior to this transaction, PincusCo has no record t</t>
+          <t>Transfers 820 East 141st Street (Credit - Cyclomedia) Maddd Equities through the entity 825 E 140 Street LLC paid $6.8 million to Raz Itzhaki, Eyal Golan, Jason Friedland, Benjamin Friedland, and Michael Friedland for the likely development site, currently an industrial building (F1) at 820 East 141st Street in Mott Haven, Bronx. The expected use is ground up development. The deal closed on May 4, 2026 and was recorded on May 18, 2026. The property has 33,000 square feet of built space and 31,850 square feet of additional air rights for a total buildable of 65,000 square feet according to a PincusCo analysis of city data. The sale price per built square foot is $204 and the price per buildable square foot is $103 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) The seller bought the property on October 29, 2020, for $8.3 million. The signatories for the sellers were Raz Itzhaki, Eyal Golan, Jason Friedland, Benjamin Friedland, and Michael Friedland. The signatory for Maddd Equities was Jorge Madruga . The contract date was February 6, 2025. Prior sa</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Extell pays $19M to Kairos for Friars Club building in Midtown East</t>
+          <t>Arthur Gabriel pays $2.8M to Ramer &amp; Saperstein for 8-unit walkup in Park Slope</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>https://www.pincusco.com/extell-pays-19m-to-kairos-for-friars-club-building-in-midtown-east/</t>
+          <t>https://www.pincusco.com/arthur-gabriel-pays-2-8m-to-ramer-saperstein-for-8-unit-walkup-in-park-slope/</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Extell Development through the entity 57 East 55th Street LLC paid $19 million to Kairos</t>
+          <t>Arthur Gabriel through the entity 528 5th St Realty LLC paid $2.8 million to Ramer</t>
         </is>
       </c>
       <c r="D4" t="inlineStr"/>
@@ -568,24 +568,24 @@
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>Transfers 57 East 55th Street (Credit - Cyclomedia) Extell Development through the entity 57 East 55th Street LLC paid $19 million to Kairos Investment Management Company through the entity Kairos Friars Club Re, LLC for the landmarked Friars Club building (P9) at 57 East 55th Street in Midtown East, Manhattan. The expected use is cash flowing. The deal closed on April 23, 2026 and was recorded on May 18, 2026. The property has 14,541 square feet of built space according to a PincusCo analysis of city data. The sale price per built square foot is $1,306 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) The seller, the former lender, acquired the property on February 21, 2025, in a transaction valued at $15.5 million. The signatory for Kairos Investment Management Company was Jonathan A. Needell . The signatory for Extell Development was Marc Kwestel . The contract date was December 18, 2025. Prior sales, articles and revenue Prior to this transaction, PincusCo has records that the buyer Extell Development purchased 32 properties in 16 transactions fo</t>
+          <t>Transfers 528 5th Street (Credit - Cyclomedia) Arthur Gabriel through the entity 528 5th St Realty LLC paid $2.8 million to Ramer &amp; Saperstein through the entity 528 Fifth Street LLC for the eight-unit residential walkup building (C1) at 528 5th Street in Park Slope, Brooklyn. The expected use is cash flowing. The deal closed on May 5, 2026 and was recorded on May 18, 2026. The property has 7,104 square feet of built space according to a PincusCo analysis of city data. The sale price per built square foot is $394 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) The seller bought the property on July 31, 2018, for $4.2 million. The signatory for Ramer &amp; Saperstein was Adam Ramer . The signatory for Arthur Gabriel was Arthur Gabriel. The contract date was March 20, 2026. Prior sales, articles and revenue Prior to this transaction, PincusCo has records that the buyer Arthur Gabriel purchased 16 properties in 16 transactions for a total of $65 million and has no record it sold any properties over the past 24 months. The seller Ramer &amp; Saperstein had not</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>David Brecher pays $23.5M to Warren Cohen for 119-unit rental in Midwood</t>
+          <t>Walter Wilfinger pays $7.7M to Annal Management for 111-unit rental in Concourse Village</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>https://www.pincusco.com/david-brecher-pays-23-5m-to-warren-cohen-for-residential-elevator-in-midwood/</t>
+          <t>https://www.pincusco.com/walter-wilfinger-pays-7-7m-to-annal-management-for-111-unit-rental-in-concourse-village/</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>David Brecher through the entity Brelan 1000 Ocean Parkway LLC paid $23.5 million to Warren</t>
+          <t>Walter Wilfinger through the entity Ote Realty LLC paid $7.7 million to Annal Management through</t>
         </is>
       </c>
       <c r="D5" t="inlineStr"/>
@@ -602,24 +602,24 @@
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>Transfers 996 Ocean Parkway (Credit - Cyclomedia) David Brecher through the entity Brelan 1000 Ocean Parkway LLC paid $23.5 million to Warren Cohen through the entity Parcjay Apartments, LLC for the 119-unit residential elevator building (D7) at 996 Ocean Parkway in Midwood, Brooklyn. The expected use is cash flowing. The deal closed on May 12, 2026 and was recorded on May 18, 2026. The property has 154,378 square feet of built space according to a PincusCo analysis of city data. The sale price per built square foot is $152 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) The seller bought the property on August 1, 2024, for $1.2 million. The signatory for Warren Cohen was Warren Cohen. The signatory for David Brecher was David Brecher . The contract date was December 30, 2025. Prior sales, articles and revenue Prior to this transaction, PincusCo has no record that the buyer had purchased any other properties and has no record it sold any properties over the past 24 months. The seller Warren Cohen had not purchased any other properties and had not s</t>
+          <t>Transfers 185 Mcclellan Street (Credit - Cyclomedia) Walter Wilfinger through the entity Ote Realty LLC paid $7.7 million to Annal Management through the entity H &amp; H Equities, Inc. for the 111-unit residential elevator building (D7) at 185 Mcclellan Street in Concourse Village, Bronx. The expected use is cash flowing. The deal closed on April 30, 2026 and was recorded on May 18, 2026. The property has 123,000 square feet of built space and 56,267 square feet of additional air rights for a total buildable of 179,221 square feet according to a PincusCo analysis of city data. The sale price per built square foot is $62 and the price per buildable square foot is $43 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) The signatory for Annal Management was Aida Spitzer . The signatory for Walter Wilfinger was Walter Wilfinger. The contract date was February 25, 2026. Prior sales, articles and revenue Prior to this transaction, PincusCo has records that the buyer Walter Wilfinger purchased three properties in three transactions for a total of $13 million an</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Adam Woodward affiliate pays $45M for mixed-use in Nolita, adds to assemblage</t>
+          <t>Jason, David Bijur pay $6.8M to Neue Urban for 12-unit walkup in Crown Heights</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>https://www.pincusco.com/adam-woodward-affiliate-pays-45m-for-mixed-use-in-nolita-adds-to-assemblage/</t>
+          <t>https://www.pincusco.com/jason-david-bijur-pay-6-8m-to-neue-urban-for-12-unit-walkup-in-crown-heights/</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Adam Woodward through the entity TTC Investments XV LLC in care of Building Equity Management,</t>
+          <t>Jason Bijur and David Bijur through the entity 821 Caroll LLC paid $6.8 million to</t>
         </is>
       </c>
       <c r="D6" t="inlineStr"/>
@@ -636,24 +636,24 @@
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>Chart_Frontpage Top Story Transfers 236 Bowery (Credit - Cyclomedia) Adam Woodward through the entity TTC Investments XV LLC in care of Building Equity Management, paid $45 million to Anton Mayer as heir to the late Frank D. Carone through the entity 236 Bowery LLC for the mixed-use building (K4) at 236 Bowery in Nolita, Manhattan. The expected use is ground up development. The deal closed on May 12, 2026 and was recorded on May 18, 2026. The property has 10,054 square feet of built space and 6,737 square feet of additional air rights for a total buildable of 16,794 square feet according to a PincusCo analysis of city data. The sale price per built square foot is $4,473 and the price per buildable square foot is $2,678 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) The signatory for Anton Mayer and Frank D. Carone was Anton F. Mayer . The signatory for Adam Woodward was David Dailey. The contract date was March 26, 2026. Frank D. Carone owned a 70% stake in a portfolio of companies that owned a restaurant supply company and real estate on the Bowe</t>
+          <t>Transfers 1467 Bedford Avenue (Credit - Cyclomedia) Jason Bijur and David Bijur through the entity 821 Caroll LLC paid $6.8 million to Neue Urban through the entity 1467 Bedford Street LLC for the 12-unit residential walkup building (C7) at 1467 Bedford Avenue in Crown Heights, Brooklyn. The expected use is cash flowing. The deal closed on May 12, 2026 and was recorded on May 19, 2026. The property has 9,078 square feet of built space and 544 square feet of additional air rights for a total buildable of 9,615 square feet according to a PincusCo analysis of city data. The sale price per built square foot is $743 and the price per buildable square foot is $702 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) The seller bought the property on June 21, 2022, for $5.4 million. The signatory for Neue Urban was Zachary Ehrlich . The signatory for Jason Bijur and David Bijur was David Bijur. The contract date was January 26, 2026. To finance the purchase, the Bijurs borrowed $4.39 million from Emerald Creek Capital. Prior sales, articles and revenue Prior t</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Hennick &amp; Company pays $66.2M to BD Hotels for hotel in Midtown West</t>
+          <t>Robert Guo files plans for 91 units in Maspeth</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>https://www.pincusco.com/hennick-company-pays-66-2m-to-bd-hotels-for-hotel-in-midtown-west/</t>
+          <t>https://www.pincusco.com/robert-guo-files-plans-for-91-units-in-maspeth/</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Toronto-based Hennick &amp; Company through the entity 15 West 56th St Inc paid $66.2 million</t>
+          <t>Robert Guo submitted a new building construction project for a 91-unit, 91,404-square-foot residential (R-2) building</t>
         </is>
       </c>
       <c r="D7" t="inlineStr"/>
@@ -670,7 +670,109 @@
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t xml:space="preserve">Top Story Transfers 15 West 56th Street (Credit - Cyclomedia) Toronto-based Hennick &amp; Company through the entity 15 West 56th St Inc paid $66.2 million to BD Hotels through the entity BDC 56 LLC for the closed Chambers Hotel building (H1) at 13-15 West 56th Street in Midtown West, Manhattan. The deal closed on May 5, 2026 and was recorded on May 18, 2026. The property has 54,959 square feet of built space according to a PincusCo analysis of city data. The sale price per built square foot is $1,204 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) The signatory for BD Hotels was Richard Born . The signatory for Hennick &amp; Company was Jory Hennick . The contract date was March 21, 2026. In November 1998, BD Hotels purchased the property from the Gottesman family for $5.2 million, according to a PincusCo analysis of the transfer records, borrowing in 1999 $4.25 million. The Commercial Observer reported on the sale yesterday. Prior sales, articles and revenue Prior to this transaction, PincusCo has no record that the buyer Hennick &amp; Company had purchased </t>
+          <t>Development 70-20 Queens Boulevard axonometric diagram (Credit - Angelo S. Ng architect via DOB) Robert Guo submitted a new building construction project for a 91-unit, 91,404-square-foot residential (R-2) building at 70-20 Queens Boulevard in Maspeth, Queens. The plan was filed on May 18, 2026. It calls for the construction of a 145-foot-tall, fifteen-story building and was filed with the New York City Department of Buildings under job number Q01389162. The project is described in the filing as: filing 15-story mixed-use building with commercial and community facilities. The applicant is the Registered Architect Angelo Ng of Angelo Ng + Anthony Ng Architects S. The plans call for a car dealership on the first floor, a daycare and outdoor recreational space on the second floor, and apartments on floors two to 15. Fei Guo purchased this parcel in 2022 for $5.9 million. 70-20 Queens Boulevard</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Benchmark pays $42M to Heller Realty for 90-unit UWS rental</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>https://www.pincusco.com/benchmark-real-estate-group-pays-42m-to-heller-realty-for-residential-elevator-in-upper-west-side/</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Benchmark Real Estate Group through the entity Benchmark 698 LLC paid $42 million to Heller</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr"/>
+      <c r="E8" t="inlineStr"/>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>PincusCo</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>PincusCo - Home</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Transfers 698 West End Avenue (Credit - Cyclomedia) Benchmark Real Estate Group through the entity Benchmark 698 LLC paid $42 million to Heller Realty through the entity 698 D Realty LLC for the 90-unit residential elevator building (D3) at 698 West End Avenue in Upper West Side, Manhattan. The expected use is cash flowing. The deal closed on May 11, 2026 and was recorded on May 19, 2026. The property has 91,494 square feet of built space according to a PincusCo analysis of city data. The sale price per built square foot is $459 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) The signatory for Heller Realty was Steven Stein. The signatory for Benchmark Real Estate Group was Jordan Vogel . The contract date was April 1, 2026. Benchmark financed the purchase with a $21.87 million loan from Flagstar Bank. The signatory for Flagstar Bank was Abraham Kaidanian . Prior sales, articles and revenue Prior to this transaction, PincusCo has records that the buyer Benchmark Real Estate Group purchased one property in one transaction for a total of $66 million </t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>RXR, OneIM sign $420M construction loan with Apollo for resi conversion in FiDi</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>https://www.pincusco.com/rxr-oneim-signs-420m-construction-loan-with-apollo-for-resi-conversion-in-fidi/</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>RXR Realty and OneIM through the entity RXR 61 Broadway Owner LLC as borrower signed</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr"/>
+      <c r="E9" t="inlineStr"/>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>PincusCo</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>PincusCo - Home</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>Transfers 61 Broadway (Credit - Cyclomedia) RXR Realty and OneIM through the entity RXR 61 Broadway Owner LLC as borrower signed a senior construction loan with lender Apollo Global Management through the entity Athene Annuity And Life Company valued at $315.5 million for the office building (O4) at 61 Broadway in Financial District, Manhattan. In addition, Apollo provided a $104.5 million mezzanine loan to RXR and OneIM The deal closed on February 26, 2026 and was recorded on May 19, 2026. The prior lender was Aareal Capital which held debt that had an original loan amount of $240 million.The property has 650,740 square feet of built space according to a PincusCo analysis of city data. The loan price per built square foot is $484 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) The owner bought the property on May 23, 2014, for $330 million. The signatory for RXR Realty was Jason Barnett . RXR filed the first New York City Department of Buildings plan to convert commercial to residential with the job number M01315725, seeking to create 21 apartment</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Dune, Turnbridge sign $379.1M refi with Strategic Value Partners for logistics in Mott Haven</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>https://www.pincusco.com/dune-turnbridge-sign-379-1m-refi-with-strategic-value-partners-for-logistics-in-mott-haven/</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Dune Real Estate Partners and Turnbridge Equities through the entity 980 BLC Owner LLC as</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr"/>
+      <c r="E10" t="inlineStr"/>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>PincusCo</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>PincusCo - Home</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>Transfers 980 East 149th Street (Credit - Cyclomedia) Dune Real Estate Partners and Turnbridge Equities through the entity 980 BLC Owner LLC as borrower signed a refi loan with lender Strategic Value Partners through the entity Re Globe Lender I L.P. valued at $379.1 million for the Bronx Logistics Center industrial building (E9) at 980 East 149th Street in Mott Haven, Bronx, and two adjacent tax lots. The deal closed on May 8, 2026 and was recorded on May 19, 2026. The prior lender was KKR which held debt that had an original loan amount of $381.2 million. The three properties have 986,360 square feet of built space and 250,096 square feet of additional air rights for a total buildable of 1,236,006 square feet according to a PincusCo analysis of city data. The loan price per built square foot is $384 and the price per buildable square foot is $306 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) The signatory for Dune Real Estate Partners and Turnbridge Equities was Ryan Nelson . The signatory for Strategic Value Partners was Lewis Schwartz . Prior</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto update queens news 2026-05-21T15:49:42Z
</commit_message>
<xml_diff>
--- a/data/output/queens_dev_news.xlsx
+++ b/data/output/queens_dev_news.xlsx
@@ -473,17 +473,17 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Heartfelt Townhouse Builders files plans for 74 units in Jamaica</t>
+          <t>Bowery assemblage grows to six tax parcels in Nolita</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>https://www.pincusco.com/heartfelt-townhouse-builders-files-plans-for-74-units-in-jamaica/</t>
+          <t>https://www.pincusco.com/bowery-assemblage-grows-to-six-tax-parcels-in-nolita/</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Heartfelt Townhouse Builders submitted a new building construction project for a 74-unit, 58,408-square-foot residential (R-2)</t>
+          <t>The entity TTC Investments XV LLC, which PincusCo connects with Adam Woodward, paid $3 million</t>
         </is>
       </c>
       <c r="D2" t="inlineStr"/>
@@ -500,24 +500,24 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>Development 143-24 94th Avenue axonometric diagram (Credit - Joseph Frankl architect via DOB) Heartfelt Townhouse Builders submitted a new building construction project for a 74-unit, 58,408-square-foot residential (R-2) building at 143-24 94 Avenue in Jamaica, Queens. The plan was filed on May 18, 2026. It calls for the construction of a 145-foot-tall, fourteen-story building and was filed with the New York City Department of Buildings under job number Q01377260. The project is described in the filing as: proposed fourteen (14) story residential use building. The applicant is the Registered Architect Joseph Frankl of JFA Architects &amp; Engineers. Joel Weiss of Heartfelt Townhouse Builders submitted the plans. The plans call for a fitness center and recreation room on the first floor, and apartments on floors two to 14. 143-24 94th Avenue The neighborhood</t>
+          <t>Transfers The entity TTC Investments XV LLC, which PincusCo connects with Adam Woodward, paid $3 million to Anton Mayer and others through the entity 232 Bowery LLC for the mixed-use building (K4) at 244 Bowery in Nolita, Manhattan. The expected use is ground up development. Affiliates of Adam Woodward own five other tax parcels near the corner of Bowery and Prince Street. The deal closed on May 12, 2026 and was recorded on May 19, 2026. The property has 3,595 square feet of built space and 3,095 square feet of additional air rights for a total buildable of 6,697 square feet according to a PincusCo analysis of city data. The sale price per built square foot is $841 and the price per buildable square foot is $451 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) The signatory for Anton Mayer and Frank D. Carone was Anton F. Mayer . The signatory for Adam Woodward was David Dailey. The contract date was March 26, 2026. Also on May 12, but recorded a day earlier, the Woodward affiliate purchased the adjacent parcel 236 Bowery for $45 million from the sa</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Maddd Equities pays $6.8M for likely dev site in Mott Haven</t>
+          <t>Abraham Biller signs $22.6M construction loan with NorthEast Community for 85-unit project in East Harlem</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>https://www.pincusco.com/maddd-equities-pays-6-8m-to-for-likely-dev-site-in-mott-haven/</t>
+          <t>https://www.pincusco.com/abraham-biller-signs-22-6m-construction-loan-with-northeast-community-for-85-unit-project-in-east-harlem/</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Maddd Equities through the entity 825 E 140 Street LLC paid $6.8 million to Raz</t>
+          <t>Abraham Biller through the entity Second Avenue Tyh LLC as borrower signed a new construction</t>
         </is>
       </c>
       <c r="D3" t="inlineStr"/>
@@ -534,24 +534,24 @@
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>Transfers 820 East 141st Street (Credit - Cyclomedia) Maddd Equities through the entity 825 E 140 Street LLC paid $6.8 million to Raz Itzhaki, Eyal Golan, Jason Friedland, Benjamin Friedland, and Michael Friedland for the likely development site, currently an industrial building (F1) at 820 East 141st Street in Mott Haven, Bronx. The expected use is ground up development. The deal closed on May 4, 2026 and was recorded on May 18, 2026. The property has 33,000 square feet of built space and 31,850 square feet of additional air rights for a total buildable of 65,000 square feet according to a PincusCo analysis of city data. The sale price per built square foot is $204 and the price per buildable square foot is $103 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) The seller bought the property on October 29, 2020, for $8.3 million. The signatories for the sellers were Raz Itzhaki, Eyal Golan, Jason Friedland, Benjamin Friedland, and Michael Friedland. The signatory for Maddd Equities was Jorge Madruga . The contract date was February 6, 2025. Prior sa</t>
+          <t xml:space="preserve">Transfers 2367 Second Avenue (Credit - Cyclomedia) Abraham Biller through the entity Second Avenue Tyh LLC as borrower signed a new construction loan with lender NorthEast Community Bank through the entity Northeast Community Bank valued at $22.6 million for four properties including the specialty building (I5) at 2367 2nd Avenue in East Harlem, Manhattan. On these lots, there is one active new building construction project, M01270610, for a 85-unit, 57,840 square-foot residential (R-2) building. The project was submitted by Abraham Biller and filed by Abraham Biller with plans filed August 21, 2025 and it has not been permitted yet. The deal closed on May 12, 2026 and was recorded on May 19, 2026. The loan price per planned development zoning square foot is $390 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) The signatory for Abraham Biller was Abraham Biller. Violations and lawsuits There were no lawsuits or bankruptcies filed against the properties for the past 24 months. In addition, according to city public data, the properties have received </t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Arthur Gabriel pays $2.8M to Ramer &amp; Saperstein for 8-unit walkup in Park Slope</t>
+          <t>Shkreli, Lumaj sign $22.5M construction loan with NorthEast Community for 99-unit project in Bedford Park</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>https://www.pincusco.com/arthur-gabriel-pays-2-8m-to-ramer-saperstein-for-8-unit-walkup-in-park-slope/</t>
+          <t>https://www.pincusco.com/shkreli-lumaj-sign-22-5m-construction-loan-with-northeast-community-for-development-in-bedford-park/</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Arthur Gabriel through the entity 528 5th St Realty LLC paid $2.8 million to Ramer</t>
+          <t>Deda M. Shkreli and Nicky Lumaj through the entity 2877 Valentine LLC as borrower signed</t>
         </is>
       </c>
       <c r="D4" t="inlineStr"/>
@@ -568,24 +568,24 @@
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>Transfers 528 5th Street (Credit - Cyclomedia) Arthur Gabriel through the entity 528 5th St Realty LLC paid $2.8 million to Ramer &amp; Saperstein through the entity 528 Fifth Street LLC for the eight-unit residential walkup building (C1) at 528 5th Street in Park Slope, Brooklyn. The expected use is cash flowing. The deal closed on May 5, 2026 and was recorded on May 18, 2026. The property has 7,104 square feet of built space according to a PincusCo analysis of city data. The sale price per built square foot is $394 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) The seller bought the property on July 31, 2018, for $4.2 million. The signatory for Ramer &amp; Saperstein was Adam Ramer . The signatory for Arthur Gabriel was Arthur Gabriel. The contract date was March 20, 2026. Prior sales, articles and revenue Prior to this transaction, PincusCo has records that the buyer Arthur Gabriel purchased 16 properties in 16 transactions for a total of $65 million and has no record it sold any properties over the past 24 months. The seller Ramer &amp; Saperstein had not</t>
+          <t>Transfers 2879 Valentine Avenue (Credit - Cyclomedia) Deda M. Shkreli and Nicky Lumaj through the entity 2877 Valentine LLC as borrower signed a new construction loan with lender NorthEast Community Bank through the entity Northeast Community Bank valued at $22.5 million for the 99-unit development project at 2879 Valentine Avenue in Bedford Park, Bronx. On the lot, there is one active new building construction project, X01129500, for a 99-unit residential (R-2) building. The project was submitted by Paulin Lumaj and filed by Paulin Lumaj with plans filed November 14, 2024 and permitted January 21, 2026. The deal closed on May 7, 2026 and was recorded on May 19, 2026. The prior lender was NorthEast Community Bank which held debt that had an original loan amount of $3.6 million.The property has 2,618 square feet of built space and 61,705 square feet of additional air rights for a total buildable of 61,705 square feet according to a PincusCo analysis of city data. The loan price per buildable square foot is $364 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have be</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Walter Wilfinger pays $7.7M to Annal Management for 111-unit rental in Concourse Village</t>
+          <t>Arthur Gabriel pays $4.5M to Ramer &amp; Saperstein for 8-unit walkup in Clinton Hill</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>https://www.pincusco.com/walter-wilfinger-pays-7-7m-to-annal-management-for-111-unit-rental-in-concourse-village/</t>
+          <t>https://www.pincusco.com/arthur-gabriel-pays-4-5m-to-ramer-saperstein-for-8-unit-walkup-in-clinton-hill/</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Walter Wilfinger through the entity Ote Realty LLC paid $7.7 million to Annal Management through</t>
+          <t>Arthur Gabriel through the entity 293 Grand Ave Realty LLC paid $4.5 million to Ramer</t>
         </is>
       </c>
       <c r="D5" t="inlineStr"/>
@@ -602,24 +602,24 @@
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>Transfers 185 Mcclellan Street (Credit - Cyclomedia) Walter Wilfinger through the entity Ote Realty LLC paid $7.7 million to Annal Management through the entity H &amp; H Equities, Inc. for the 111-unit residential elevator building (D7) at 185 Mcclellan Street in Concourse Village, Bronx. The expected use is cash flowing. The deal closed on April 30, 2026 and was recorded on May 18, 2026. The property has 123,000 square feet of built space and 56,267 square feet of additional air rights for a total buildable of 179,221 square feet according to a PincusCo analysis of city data. The sale price per built square foot is $62 and the price per buildable square foot is $43 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) The signatory for Annal Management was Aida Spitzer . The signatory for Walter Wilfinger was Walter Wilfinger. The contract date was February 25, 2026. Prior sales, articles and revenue Prior to this transaction, PincusCo has records that the buyer Walter Wilfinger purchased three properties in three transactions for a total of $13 million an</t>
+          <t>Transfers 293 Grand Avenue (Credit - Cyclomedia) Arthur Gabriel through the entity 293 Grand Ave Realty LLC paid $4.5 million to Ramer &amp; Saperstein through the entity Pn Grand Holdings, LLC for the eight-unit residential walkup building (C1) at 293 Grand Avenue in Clinton Hill, Brooklyn. The expected use is cash flowing. The deal closed on May 5, 2026 and was recorded on May 20, 2026. The property has 10,500 square feet of built space according to a PincusCo analysis of city data. The sale price per built square foot is $428 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) The seller bought the property on January 13, 2005, for $1 million. The signatory for Ramer &amp; Saperstein was Michael Saperstein and Adam Ramer . The signatory for Arthur Gabriel was Arthur Gabriel. The contract date was March 20, 2026. Prior sales, articles and revenue Prior to this transaction, PincusCo has records that the buyer Arthur Gabriel purchased 17 properties in 17 transactions for a total of $67.8 million and has no record it sold any properties over the past 24 months.</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Jason, David Bijur pay $6.8M to Neue Urban for 12-unit walkup in Crown Heights</t>
+          <t>Yaakov Gluck pays $10.4M to Schwimmers for 12-unit, mixed-use in Borough Park</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>https://www.pincusco.com/jason-david-bijur-pay-6-8m-to-neue-urban-for-12-unit-walkup-in-crown-heights/</t>
+          <t>https://www.pincusco.com/yaakov-gluck-pays-10-4m-to-schwimmers-for-mixed-use-in-borough-park/</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Jason Bijur and David Bijur through the entity 821 Caroll LLC paid $6.8 million to</t>
+          <t>Yaakov Gluck through the entity 1267 57th St Holdings LLC paid $10.4 million to Jacob</t>
         </is>
       </c>
       <c r="D6" t="inlineStr"/>
@@ -636,24 +636,24 @@
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>Transfers 1467 Bedford Avenue (Credit - Cyclomedia) Jason Bijur and David Bijur through the entity 821 Caroll LLC paid $6.8 million to Neue Urban through the entity 1467 Bedford Street LLC for the 12-unit residential walkup building (C7) at 1467 Bedford Avenue in Crown Heights, Brooklyn. The expected use is cash flowing. The deal closed on May 12, 2026 and was recorded on May 19, 2026. The property has 9,078 square feet of built space and 544 square feet of additional air rights for a total buildable of 9,615 square feet according to a PincusCo analysis of city data. The sale price per built square foot is $743 and the price per buildable square foot is $702 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) The seller bought the property on June 21, 2022, for $5.4 million. The signatory for Neue Urban was Zachary Ehrlich . The signatory for Jason Bijur and David Bijur was David Bijur. The contract date was January 26, 2026. To finance the purchase, the Bijurs borrowed $4.39 million from Emerald Creek Capital. Prior sales, articles and revenue Prior t</t>
+          <t>Transfers 1267 57th Street (Credit - Cyclomedia) Yaakov Gluck through the entity 1267 57th St Holdings LLC paid $10.4 million to Jacob Schwimmer and Solomon Schwimmer through the entity Heights 57 Development LLC for the 12-unit plus office, mixed-use building at 1267 57th Street in Borough Park, Brooklyn. The expected use is cash flowing. The deal closed on May 1, 2026 and was recorded on May 20, 2026. The two commercial condominium units that make up the building, one with 12 residential apartments and one that is an office condo unit, have 30,607 square feet of built space according to a PincusCo analysis of city data. The sale price per built square foot is $341 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) The signatory for Jacob Schwimmer and Solomon Schwimmer was Jacob Schwimmer. The signatory for Yaakov Gluck was Yaakov Gluck. The contract date was August 21, 2024. Prior sales, articles and revenue Prior to this transaction, PincusCo has no record that the buyer Yaakov Gluck had purchased any other properties and has no record it sold any</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Robert Guo files plans for 91 units in Maspeth</t>
+          <t>School bus firm Pioneer Transportation pays $7M for parking in Charleston</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>https://www.pincusco.com/robert-guo-files-plans-for-91-units-in-maspeth/</t>
+          <t>https://www.pincusco.com/school-bus-firm-pioneer-transportation-pays-7m-for-parking-in-charleston/</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Robert Guo submitted a new building construction project for a 91-unit, 91,404-square-foot residential (R-2) building</t>
+          <t>Pioneer Transportation through the entity Sharrotts Partners LLC paid $7 million to Nancy English through</t>
         </is>
       </c>
       <c r="D7" t="inlineStr"/>
@@ -670,24 +670,24 @@
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>Development 70-20 Queens Boulevard axonometric diagram (Credit - Angelo S. Ng architect via DOB) Robert Guo submitted a new building construction project for a 91-unit, 91,404-square-foot residential (R-2) building at 70-20 Queens Boulevard in Maspeth, Queens. The plan was filed on May 18, 2026. It calls for the construction of a 145-foot-tall, fifteen-story building and was filed with the New York City Department of Buildings under job number Q01389162. The project is described in the filing as: filing 15-story mixed-use building with commercial and community facilities. The applicant is the Registered Architect Angelo Ng of Angelo Ng + Anthony Ng Architects S. The plans call for a car dealership on the first floor, a daycare and outdoor recreational space on the second floor, and apartments on floors two to 15. Fei Guo purchased this parcel in 2022 for $5.9 million. 70-20 Queens Boulevard</t>
+          <t>Transfers 448 Sharrotts Road (Credit - Cyclomedia) Pioneer Transportation through the entity Sharrotts Partners LLC paid $7 million to Nancy English through the entity Gateway Associates, LLC for the industrial building (G9) at 448 Sharrotts Road in Charleston, Staten Island. The expected use is owner-occupied. The deal closed on March 13, 2026 and was recorded on May 20, 2026. The property has 5,135 square feet of built space and 106,306 square feet of additional air rights for a total buildable of 111,902 square feet according to a PincusCo analysis of city data. The sale price per built square foot is $1,363 and the price per buildable square foot is $62 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) The signatory for Nancy English was Nancy English. The signatory for Pioneer Transportation was Neil Strahl . The contract date was February 27, 2026. Sharrotts Partners LLC is misspelled as Sharrots Partners LLC in portions of the transfer records. Prior sales, articles and revenue Prior to this transaction, PincusCo has no record that the buyer P</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Benchmark pays $42M to Heller Realty for 90-unit UWS rental</t>
+          <t>Dalan Real Estate pays $7.3M to Nazarian Property Group for mixed-use in Greenwich Village</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>https://www.pincusco.com/benchmark-real-estate-group-pays-42m-to-heller-realty-for-residential-elevator-in-upper-west-side/</t>
+          <t>https://www.pincusco.com/dalan-real-estate-pays-7-3m-to-nazarian-property-group-for-mixed-use-in-greenwich-village/</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Benchmark Real Estate Group through the entity Benchmark 698 LLC paid $42 million to Heller</t>
+          <t>The Wrublin family’s Dalan Real Estate paid $7.3 million to Nazarian Property Group for two</t>
         </is>
       </c>
       <c r="D8" t="inlineStr"/>
@@ -704,24 +704,24 @@
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t xml:space="preserve">Transfers 698 West End Avenue (Credit - Cyclomedia) Benchmark Real Estate Group through the entity Benchmark 698 LLC paid $42 million to Heller Realty through the entity 698 D Realty LLC for the 90-unit residential elevator building (D3) at 698 West End Avenue in Upper West Side, Manhattan. The expected use is cash flowing. The deal closed on May 11, 2026 and was recorded on May 19, 2026. The property has 91,494 square feet of built space according to a PincusCo analysis of city data. The sale price per built square foot is $459 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) The signatory for Heller Realty was Steven Stein. The signatory for Benchmark Real Estate Group was Jordan Vogel . The contract date was April 1, 2026. Benchmark financed the purchase with a $21.87 million loan from Flagstar Bank. The signatory for Flagstar Bank was Abraham Kaidanian . Prior sales, articles and revenue Prior to this transaction, PincusCo has records that the buyer Benchmark Real Estate Group purchased one property in one transaction for a total of $66 million </t>
+          <t>Transfers 18-20 Christopher Street (Credit - Cyclomedia) The Wrublin family’s Dalan Real Estate paid $7.3 million to Nazarian Property Group for two adjacent mixed-use buildings, 18 and 20 Christopher Street, in Greenwich Village, Manhattan, in two transactions. In the first, Dalan Real Estate through the entity Aw Christopher Tic LLC paid $3.65 million to Nazarian Property Group through the entity 20 Christopher Street, LLC for the four-unit mixed-use building (S4) at 20 Christopher Street in Greenwich Village, Manhattan. The expected use is cash flowing. The deal closed on May 6, 2026 and was recorded on May 20, 2026. The property has 1,554 square feet of built space and 1,463 square feet of additional air rights for a total buildable of 3,013 square feet according to a PincusCo analysis of city data. The sale price per built square foot is $2,352 and the price per buildable square foot is $1,213 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) The seller bought the property on April 27, 2022, for $2.4 million. In the second, Dalan Real Estate thr</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>RXR, OneIM sign $420M construction loan with Apollo for resi conversion in FiDi</t>
+          <t>City pays $10M for school dev site in Great Kills</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>https://www.pincusco.com/rxr-oneim-signs-420m-construction-loan-with-apollo-for-resi-conversion-in-fidi/</t>
+          <t>https://www.pincusco.com/city-pays-10m-for-school-dev-site-in-great-kills/</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>RXR Realty and OneIM through the entity RXR 61 Broadway Owner LLC as borrower signed</t>
+          <t>The City of New York’s NYC School Construction Authority paid $10 million to Anthony Fontana</t>
         </is>
       </c>
       <c r="D9" t="inlineStr"/>
@@ -738,24 +738,24 @@
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>Transfers 61 Broadway (Credit - Cyclomedia) RXR Realty and OneIM through the entity RXR 61 Broadway Owner LLC as borrower signed a senior construction loan with lender Apollo Global Management through the entity Athene Annuity And Life Company valued at $315.5 million for the office building (O4) at 61 Broadway in Financial District, Manhattan. In addition, Apollo provided a $104.5 million mezzanine loan to RXR and OneIM The deal closed on February 26, 2026 and was recorded on May 19, 2026. The prior lender was Aareal Capital which held debt that had an original loan amount of $240 million.The property has 650,740 square feet of built space according to a PincusCo analysis of city data. The loan price per built square foot is $484 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) The owner bought the property on May 23, 2014, for $330 million. The signatory for RXR Realty was Jason Barnett . RXR filed the first New York City Department of Buildings plan to convert commercial to residential with the job number M01315725, seeking to create 21 apartment</t>
+          <t>Transfers 5 - 51 East Reading Avenue (Credit - NYC Department of City Planning) The City of New York’s NYC School Construction Authority paid $10 million to Anthony Fontana through the entity East Reading Holdings LLC for an 18-parcel development site (V0) including 17 East Reading Avenue in Great Kills, Staten Island. The expected use is ground up development. The deal closed on April 21, 2026 and was recorded on May 20, 2026. The 18 properties have zero square feet of built space and 7,788 square feet of additional air rights for a total buildable of 7,788 square feet according to a PincusCo analysis of city data. The sale price per built square foot is $N/A and the price per buildable square foot is $1,283 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) The signatory for Anthony Fontana was Anthony Fontana. The signatory for NYC School Construction Authority was Tina Isselbacher . The contract date was March 20, 2025. Anthony Fontana had filed plans to build single-family homes on the parcel.  Prior sales, articles and revenue</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Dune, Turnbridge sign $379.1M refi with Strategic Value Partners for logistics in Mott Haven</t>
+          <t>Hospitality company Crew pays $4.5M for mixed-use in Brooklyn Heights</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>https://www.pincusco.com/dune-turnbridge-sign-379-1m-refi-with-strategic-value-partners-for-logistics-in-mott-haven/</t>
+          <t>https://www.pincusco.com/hospitality-company-crew-pays-4-5m-for-mixed-use-in-brooklyn-heights/</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Dune Real Estate Partners and Turnbridge Equities through the entity 980 BLC Owner LLC as</t>
+          <t>The hospitality company Crew through the entity 73 Atlantic Avenue Developer LLC paid $4.5 million</t>
         </is>
       </c>
       <c r="D10" t="inlineStr"/>
@@ -772,7 +772,7 @@
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>Transfers 980 East 149th Street (Credit - Cyclomedia) Dune Real Estate Partners and Turnbridge Equities through the entity 980 BLC Owner LLC as borrower signed a refi loan with lender Strategic Value Partners through the entity Re Globe Lender I L.P. valued at $379.1 million for the Bronx Logistics Center industrial building (E9) at 980 East 149th Street in Mott Haven, Bronx, and two adjacent tax lots. The deal closed on May 8, 2026 and was recorded on May 19, 2026. The prior lender was KKR which held debt that had an original loan amount of $381.2 million. The three properties have 986,360 square feet of built space and 250,096 square feet of additional air rights for a total buildable of 1,236,006 square feet according to a PincusCo analysis of city data. The loan price per built square foot is $384 and the price per buildable square foot is $306 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) The signatory for Dune Real Estate Partners and Turnbridge Equities was Ryan Nelson . The signatory for Strategic Value Partners was Lewis Schwartz . Prior</t>
+          <t>Transfers 73 Atlantic Avenue (Credit - Cyclomedia) The hospitality company Crew through the entity 73 Atlantic Avenue Developer LLC paid $4.5 million to Joseph F. Montero through the entity 73 Atlantic Ave., LLC for the three-unit mixed-use building (S3) at 73 Atlantic Avenue in Brooklyn Heights, Brooklyn. The expected use is owner-occupied and cash flowing. This is the location for the 90-year-old Montero Bar &amp; Grill, which Crew acquired, according to the New York Post, which reported on the restaurant sale in January 2026. Crew plans to maintain the bar as it is, the report said. The deal closed on April 24, 2026 and was recorded on May 20, 2026. The property has 3,780 square feet of built space according to a PincusCo analysis of city data. The sale price per built square foot is $1,190 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) The signatory for Joseph F. Montero was Joseph F. Montero. The signatories for Crew were company founders – and brothers – Miles Pincus and Alexander Pincus . The contract date was November 7, 2025. Miles and Alexan</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto update queens news 2026-05-22T15:19:22Z
</commit_message>
<xml_diff>
--- a/data/output/queens_dev_news.xlsx
+++ b/data/output/queens_dev_news.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H10"/>
+  <dimension ref="A1:H8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -473,17 +473,17 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Bowery assemblage grows to six tax parcels in Nolita</t>
+          <t>Premier Equities signs $9.2M refi loan with Peapack for retail in SoHo</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>https://www.pincusco.com/bowery-assemblage-grows-to-six-tax-parcels-in-nolita/</t>
+          <t>https://www.pincusco.com/premier-equities-signs-9-2m-refi-loan-with-peapack-for-retail-in-soho/</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>The entity TTC Investments XV LLC, which PincusCo connects with Adam Woodward, paid $3 million</t>
+          <t>Premier Equities through the entity Premier 158 Mercer LLC as borrower signed a refi loan</t>
         </is>
       </c>
       <c r="D2" t="inlineStr"/>
@@ -500,24 +500,24 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>Transfers The entity TTC Investments XV LLC, which PincusCo connects with Adam Woodward, paid $3 million to Anton Mayer and others through the entity 232 Bowery LLC for the mixed-use building (K4) at 244 Bowery in Nolita, Manhattan. The expected use is ground up development. Affiliates of Adam Woodward own five other tax parcels near the corner of Bowery and Prince Street. The deal closed on May 12, 2026 and was recorded on May 19, 2026. The property has 3,595 square feet of built space and 3,095 square feet of additional air rights for a total buildable of 6,697 square feet according to a PincusCo analysis of city data. The sale price per built square foot is $841 and the price per buildable square foot is $451 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) The signatory for Anton Mayer and Frank D. Carone was Anton F. Mayer . The signatory for Adam Woodward was David Dailey. The contract date was March 26, 2026. Also on May 12, but recorded a day earlier, the Woodward affiliate purchased the adjacent parcel 236 Bowery for $45 million from the sa</t>
+          <t xml:space="preserve">Transfers Premier Equities through the entity Premier 158 Mercer LLC as borrower signed a refi loan with lender Peapack Private Bank &amp; Trust valued at $9.2 million for the retail condo at 158 Mercer Street in SoHo, Manhattan. The deal closed on April 28, 2026 and was recorded on May 21, 2026. The prior lender was Webster Bank which held debt that had an original loan amount of $15 million. The property has 4,251 square feet of built space according to a PincusCo analysis of city data. The loan price per built square foot is $2,152 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) The owner bought the property on February 6, 2015, for $16 million. The signatory for Premier Equities was Mark D. Mermel . The signatory for Peapack Private Bank &amp; Trust was Nicholas LaMorte. The property The retail condo in SoHo has 4,251 square feet of built space according to a PincusCo analysis of city data. The parcel has a total lot size of 4,251 square feet. The city-designated market value for the property in 2022 is $6.6 million. Violations and lawsuits There were </t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Abraham Biller signs $22.6M construction loan with NorthEast Community for 85-unit project in East Harlem</t>
+          <t>Corem Property Group signs $78.5M refi loan with affiliate for office in Penn Plaza</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>https://www.pincusco.com/abraham-biller-signs-22-6m-construction-loan-with-northeast-community-for-85-unit-project-in-east-harlem/</t>
+          <t>https://www.pincusco.com/corem-property-group-signs-78-5m-refi-loan-with-affiliate-for-office-in-penn-plaza/</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Abraham Biller through the entity Second Avenue Tyh LLC as borrower signed a new construction</t>
+          <t>Corem Property Group through the entity 1241 Broadway LLC as borrower signed a refi loan</t>
         </is>
       </c>
       <c r="D3" t="inlineStr"/>
@@ -534,24 +534,24 @@
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Transfers 2367 Second Avenue (Credit - Cyclomedia) Abraham Biller through the entity Second Avenue Tyh LLC as borrower signed a new construction loan with lender NorthEast Community Bank through the entity Northeast Community Bank valued at $22.6 million for four properties including the specialty building (I5) at 2367 2nd Avenue in East Harlem, Manhattan. On these lots, there is one active new building construction project, M01270610, for a 85-unit, 57,840 square-foot residential (R-2) building. The project was submitted by Abraham Biller and filed by Abraham Biller with plans filed August 21, 2025 and it has not been permitted yet. The deal closed on May 12, 2026 and was recorded on May 19, 2026. The loan price per planned development zoning square foot is $390 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) The signatory for Abraham Biller was Abraham Biller. Violations and lawsuits There were no lawsuits or bankruptcies filed against the properties for the past 24 months. In addition, according to city public data, the properties have received </t>
+          <t>Transfers 1241 Broadway (Credit - Cyclomedia) Corem Property Group through the entity 1241 Broadway LLC as borrower signed a refi loan with an affiliate, the entity Corem Charlotta AB, valued at $78.5 million for the office building (O4) at 1241 Broadway in Penn Plaza, Manhattan. The deal closed on May 11, 2026 and was recorded on May 21, 2026. The prior lender was Deutsche Pfandbriefbank which held debt that had an original loan amount of $90 million. The property has 178,884 square feet of built space and 28,826 square feet of additional air rights for a total buildable of 191,325 square feet according to a PincusCo analysis of city data. The loan price per built square foot is $438 and the price per buildable square foot is $410 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) The signatory for Corem Property Group was David Roll . The signatory for Corem Property Group was Emelie Morndal . Prior sales, articles and revenue The 178,884-square-foot property generated revenue of $11.5 million or $64 per square foot, according to the most recent inc</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Shkreli, Lumaj sign $22.5M construction loan with NorthEast Community for 99-unit project in Bedford Park</t>
+          <t>Sheya Ungar pays $2.6M for 4-family in Williamsburg</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>https://www.pincusco.com/shkreli-lumaj-sign-22-5m-construction-loan-with-northeast-community-for-development-in-bedford-park/</t>
+          <t>https://www.pincusco.com/sheya-ungar-pays-2-6m-for-4-family-in-williamsburg/</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Deda M. Shkreli and Nicky Lumaj through the entity 2877 Valentine LLC as borrower signed</t>
+          <t>Sheya Ungar through the entity Cggo Bunim LLC paid $2.6 million for the four-unit building</t>
         </is>
       </c>
       <c r="D4" t="inlineStr"/>
@@ -568,24 +568,24 @@
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>Transfers 2879 Valentine Avenue (Credit - Cyclomedia) Deda M. Shkreli and Nicky Lumaj through the entity 2877 Valentine LLC as borrower signed a new construction loan with lender NorthEast Community Bank through the entity Northeast Community Bank valued at $22.5 million for the 99-unit development project at 2879 Valentine Avenue in Bedford Park, Bronx. On the lot, there is one active new building construction project, X01129500, for a 99-unit residential (R-2) building. The project was submitted by Paulin Lumaj and filed by Paulin Lumaj with plans filed November 14, 2024 and permitted January 21, 2026. The deal closed on May 7, 2026 and was recorded on May 19, 2026. The prior lender was NorthEast Community Bank which held debt that had an original loan amount of $3.6 million.The property has 2,618 square feet of built space and 61,705 square feet of additional air rights for a total buildable of 61,705 square feet according to a PincusCo analysis of city data. The loan price per buildable square foot is $364 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have be</t>
+          <t xml:space="preserve">Transfers 127 Penn Street (Credit - Cyclomedia) Sheya Ungar through the entity Cggo Bunim LLC paid $2.6 million for the four-unit building (C3) at 127 Penn Street in Williamsburg, Brooklyn. The deal closed on April 21, 2026 and was recorded on May 21, 2026. The property has 2,640 square feet of built space and 2,749 square feet of additional air rights for a total buildable of 5,387 square feet according to a PincusCo analysis of city data. The sale price per built square foot is $977 and the price per buildable square foot is $479 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) The signatory for the sellers were Lewis Gluck and Rachel Hopstein. The signatory for Sheya Ungar was Sheya Ungar. The contract date was April 21, 2026. Prior sales, articles and revenue Prior to this transaction, PincusCo has no record that the buyer Sheya Ungar had purchased any other properties and has no record it sold any properties over the past 24 months. The seller Lewis Gluck had not purchased any other properties and had not sold any properties over the same time </t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Arthur Gabriel pays $4.5M to Ramer &amp; Saperstein for 8-unit walkup in Clinton Hill</t>
+          <t>Shabse Fuchs files plans for 31 units in Bushwick</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>https://www.pincusco.com/arthur-gabriel-pays-4-5m-to-ramer-saperstein-for-8-unit-walkup-in-clinton-hill/</t>
+          <t>https://www.pincusco.com/shabse-fuchs-files-plans-for-31-units-in-bushwick/</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Arthur Gabriel through the entity 293 Grand Ave Realty LLC paid $4.5 million to Ramer</t>
+          <t>Shabse Fuchs submitted a new building construction project for a 46-unit, 23,207-square-foot residential (R-2) building</t>
         </is>
       </c>
       <c r="D5" t="inlineStr"/>
@@ -602,24 +602,24 @@
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>Transfers 293 Grand Avenue (Credit - Cyclomedia) Arthur Gabriel through the entity 293 Grand Ave Realty LLC paid $4.5 million to Ramer &amp; Saperstein through the entity Pn Grand Holdings, LLC for the eight-unit residential walkup building (C1) at 293 Grand Avenue in Clinton Hill, Brooklyn. The expected use is cash flowing. The deal closed on May 5, 2026 and was recorded on May 20, 2026. The property has 10,500 square feet of built space according to a PincusCo analysis of city data. The sale price per built square foot is $428 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) The seller bought the property on January 13, 2005, for $1 million. The signatory for Ramer &amp; Saperstein was Michael Saperstein and Adam Ramer . The signatory for Arthur Gabriel was Arthur Gabriel. The contract date was March 20, 2026. Prior sales, articles and revenue Prior to this transaction, PincusCo has records that the buyer Arthur Gabriel purchased 17 properties in 17 transactions for a total of $67.8 million and has no record it sold any properties over the past 24 months.</t>
+          <t>Development 102 Wyckoff Avenue axonometric diagram (Credit - Naresh Manangu professional engineer via DOB) Shabse Fuchs submitted a new building construction project for a 46-unit, 23,207-square-foot residential (R-2) building at 102 Wyckoff Avenue in Bushwick, Brooklyn. The plan was filed on May 20, 2026. It calls for the construction of a 82-foot-tall, eight-story building and was filed with the New York City Department of Buildings under job number B01401889. The project is described in the filing as: proposed 8-story and cellar residential and community facility building. The applicant is the Professional Engineer Naresh Mahangu of NKM Engineering PLLC. There are already 15 residential units on the tax block, the filing shows, for a total of 46 units on the tax block. The site is currently occupied by a six-story parking deck. The plans call for an ambulatory medical care facility on the ground floor and apartments on floors two to eight. 102 Wyckoff Avenue  The neighborhood</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Yaakov Gluck pays $10.4M to Schwimmers for 12-unit, mixed-use in Borough Park</t>
+          <t>Wagner College pays $30M for former St. John’s University campus on Staten Island</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>https://www.pincusco.com/yaakov-gluck-pays-10-4m-to-schwimmers-for-mixed-use-in-borough-park/</t>
+          <t>https://www.pincusco.com/wagner-college-pays-30m-for-former-st-johns-university-campus-on-staten-island/</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Yaakov Gluck through the entity 1267 57th St Holdings LLC paid $10.4 million to Jacob</t>
+          <t>The private higher educational school Wagner College through the entity Seahawks Realty LLC paid the</t>
         </is>
       </c>
       <c r="D6" t="inlineStr"/>
@@ -636,24 +636,24 @@
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>Transfers 1267 57th Street (Credit - Cyclomedia) Yaakov Gluck through the entity 1267 57th St Holdings LLC paid $10.4 million to Jacob Schwimmer and Solomon Schwimmer through the entity Heights 57 Development LLC for the 12-unit plus office, mixed-use building at 1267 57th Street in Borough Park, Brooklyn. The expected use is cash flowing. The deal closed on May 1, 2026 and was recorded on May 20, 2026. The two commercial condominium units that make up the building, one with 12 residential apartments and one that is an office condo unit, have 30,607 square feet of built space according to a PincusCo analysis of city data. The sale price per built square foot is $341 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) The signatory for Jacob Schwimmer and Solomon Schwimmer was Jacob Schwimmer. The signatory for Yaakov Gluck was Yaakov Gluck. The contract date was August 21, 2024. Prior sales, articles and revenue Prior to this transaction, PincusCo has no record that the buyer Yaakov Gluck had purchased any other properties and has no record it sold any</t>
+          <t>Transfers 300 Howard Avenue (Credit - Cyclomedia) The private higher educational school Wagner College through the entity Seahawks Realty LLC paid the Queens-based St. John’s University $30 million for the 10-building educational campus (W6) including the address 300 Howard Avenue in Silver Lake, Staten Island. The deal closed on May 11, 2026 and was recorded on May 21, 2026. The property has 146,855 square feet of built space and 395,307 square feet of additional air rights for a total buildable of 539,055 square feet according to a PincusCo analysis of city data. The sale price per built square foot is $204 and the price per buildable square foot is $55 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) The Staten Island Advance reported on the sale previously but did not include the price, but the report noted that Metropolitan Commercial Bank provided an undisclosed amount of financing. Prior sales, articles and revenue Prior to this transaction, PincusCo has no record that the buyer Wagner College had purchased any other properties and has no rec</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>School bus firm Pioneer Transportation pays $7M for parking in Charleston</t>
+          <t>Meadow Partners signs $19M rehab construction loan for 2 walkups in Williamsburg</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>https://www.pincusco.com/school-bus-firm-pioneer-transportation-pays-7m-for-parking-in-charleston/</t>
+          <t>https://www.pincusco.com/meadow-partners-signs-19m-rehab-construction-loan-for-2-walkup-in-williamsburg/</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Pioneer Transportation through the entity Sharrotts Partners LLC paid $7 million to Nancy English through</t>
+          <t>Meadow Partners through the entity 65-75 Roebling Owner, LLC as borrower signed a rehab construction</t>
         </is>
       </c>
       <c r="D7" t="inlineStr"/>
@@ -670,24 +670,24 @@
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>Transfers 448 Sharrotts Road (Credit - Cyclomedia) Pioneer Transportation through the entity Sharrotts Partners LLC paid $7 million to Nancy English through the entity Gateway Associates, LLC for the industrial building (G9) at 448 Sharrotts Road in Charleston, Staten Island. The expected use is owner-occupied. The deal closed on March 13, 2026 and was recorded on May 20, 2026. The property has 5,135 square feet of built space and 106,306 square feet of additional air rights for a total buildable of 111,902 square feet according to a PincusCo analysis of city data. The sale price per built square foot is $1,363 and the price per buildable square foot is $62 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) The signatory for Nancy English was Nancy English. The signatory for Pioneer Transportation was Neil Strahl . The contract date was February 27, 2026. Sharrotts Partners LLC is misspelled as Sharrots Partners LLC in portions of the transfer records. Prior sales, articles and revenue Prior to this transaction, PincusCo has no record that the buyer P</t>
+          <t>Transfers 83 Roebling Street (Credit - Cyclomedia) Meadow Partners through the entity 65-75 Roebling Owner, LLC as borrower signed a rehab construction loan with lender Customers Bank valued at $19 million for two residential walkups with 55 residential units including the 31-unit residential walkup building (C1) at 83 Roebling Street in Williamsburg, Brooklyn and 24-unit residential walkup building (C7) at 65 Roebling Street in Williamsburg, Brooklyn. The deal closed on March 30, 2026 and was recorded on May 21, 2026. The prior lender was Customers Bank which held debt that had an original loan amount of $11.37 million. The two properties have 65,750 square feet of built space and 9,250 square feet of additional air rights for a total buildable of 75,000 square feet according to a PincusCo analysis of city data. The loan price per built square foot is $288 and the price per buildable square foot is $253 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) The signatory for Meadow Partners was Timothy P. Yantz . This is a rehab construction loan of $7.6</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Dalan Real Estate pays $7.3M to Nazarian Property Group for mixed-use in Greenwich Village</t>
+          <t>Far Rockaway Orthodox girls school approved for $21.4M construction loan</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>https://www.pincusco.com/dalan-real-estate-pays-7-3m-to-nazarian-property-group-for-mixed-use-in-greenwich-village/</t>
+          <t>https://www.pincusco.com/far-rockaway-orthodox-girls-school-approved-for-21-4m-construction-loan/</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>The Wrublin family’s Dalan Real Estate paid $7.3 million to Nazarian Property Group for two</t>
+          <t>The Orthodox girls school Bnos Bais Yaakov of Far Rockaway secured an approval from the</t>
         </is>
       </c>
       <c r="D8" t="inlineStr"/>
@@ -704,75 +704,7 @@
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>Transfers 18-20 Christopher Street (Credit - Cyclomedia) The Wrublin family’s Dalan Real Estate paid $7.3 million to Nazarian Property Group for two adjacent mixed-use buildings, 18 and 20 Christopher Street, in Greenwich Village, Manhattan, in two transactions. In the first, Dalan Real Estate through the entity Aw Christopher Tic LLC paid $3.65 million to Nazarian Property Group through the entity 20 Christopher Street, LLC for the four-unit mixed-use building (S4) at 20 Christopher Street in Greenwich Village, Manhattan. The expected use is cash flowing. The deal closed on May 6, 2026 and was recorded on May 20, 2026. The property has 1,554 square feet of built space and 1,463 square feet of additional air rights for a total buildable of 3,013 square feet according to a PincusCo analysis of city data. The sale price per built square foot is $2,352 and the price per buildable square foot is $1,213 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) The seller bought the property on April 27, 2022, for $2.4 million. In the second, Dalan Real Estate thr</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>City pays $10M for school dev site in Great Kills</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>https://www.pincusco.com/city-pays-10m-for-school-dev-site-in-great-kills/</t>
-        </is>
-      </c>
-      <c r="C9" t="inlineStr">
-        <is>
-          <t>The City of New York’s NYC School Construction Authority paid $10 million to Anthony Fontana</t>
-        </is>
-      </c>
-      <c r="D9" t="inlineStr"/>
-      <c r="E9" t="inlineStr"/>
-      <c r="F9" t="inlineStr">
-        <is>
-          <t>PincusCo</t>
-        </is>
-      </c>
-      <c r="G9" t="inlineStr">
-        <is>
-          <t>PincusCo - Home</t>
-        </is>
-      </c>
-      <c r="H9" t="inlineStr">
-        <is>
-          <t>Transfers 5 - 51 East Reading Avenue (Credit - NYC Department of City Planning) The City of New York’s NYC School Construction Authority paid $10 million to Anthony Fontana through the entity East Reading Holdings LLC for an 18-parcel development site (V0) including 17 East Reading Avenue in Great Kills, Staten Island. The expected use is ground up development. The deal closed on April 21, 2026 and was recorded on May 20, 2026. The 18 properties have zero square feet of built space and 7,788 square feet of additional air rights for a total buildable of 7,788 square feet according to a PincusCo analysis of city data. The sale price per built square foot is $N/A and the price per buildable square foot is $1,283 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) The signatory for Anthony Fontana was Anthony Fontana. The signatory for NYC School Construction Authority was Tina Isselbacher . The contract date was March 20, 2025. Anthony Fontana had filed plans to build single-family homes on the parcel.  Prior sales, articles and revenue</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>Hospitality company Crew pays $4.5M for mixed-use in Brooklyn Heights</t>
-        </is>
-      </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>https://www.pincusco.com/hospitality-company-crew-pays-4-5m-for-mixed-use-in-brooklyn-heights/</t>
-        </is>
-      </c>
-      <c r="C10" t="inlineStr">
-        <is>
-          <t>The hospitality company Crew through the entity 73 Atlantic Avenue Developer LLC paid $4.5 million</t>
-        </is>
-      </c>
-      <c r="D10" t="inlineStr"/>
-      <c r="E10" t="inlineStr"/>
-      <c r="F10" t="inlineStr">
-        <is>
-          <t>PincusCo</t>
-        </is>
-      </c>
-      <c r="G10" t="inlineStr">
-        <is>
-          <t>PincusCo - Home</t>
-        </is>
-      </c>
-      <c r="H10" t="inlineStr">
-        <is>
-          <t>Transfers 73 Atlantic Avenue (Credit - Cyclomedia) The hospitality company Crew through the entity 73 Atlantic Avenue Developer LLC paid $4.5 million to Joseph F. Montero through the entity 73 Atlantic Ave., LLC for the three-unit mixed-use building (S3) at 73 Atlantic Avenue in Brooklyn Heights, Brooklyn. The expected use is owner-occupied and cash flowing. This is the location for the 90-year-old Montero Bar &amp; Grill, which Crew acquired, according to the New York Post, which reported on the restaurant sale in January 2026. Crew plans to maintain the bar as it is, the report said. The deal closed on April 24, 2026 and was recorded on May 20, 2026. The property has 3,780 square feet of built space according to a PincusCo analysis of city data. The sale price per built square foot is $1,190 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) The signatory for Joseph F. Montero was Joseph F. Montero. The signatories for Crew were company founders – and brothers – Miles Pincus and Alexander Pincus . The contract date was November 7, 2025. Miles and Alexan</t>
+          <t>Transfers 1207 Caffrey Avenue axonometrict diagram (Credit - Fariba Makooi architect via DOB) The Orthodox girls school Bnos Bais Yaakov of Far Rockaway secured an approval from the New York State Attorney General to obtain a new mortgage loan of up to $21.4 million from Bank United to fund the development of a new 68,000-square-foot high school building, and pay off an existing loan, at its campus in Far Rockaway, Queens. The commercial financing package will fund the construction of a new building at 1207 Caffrey Avenue through job number Q01129479 (with an alternate address of 613 Beach 9th Street) in the Far Rockaway neighborhood. It will pay off an older loan from Dime Community Bank secured by the existing school building at 609 Beach 9th Street. The regulatory petition, filed by the non-profit corporation under the state’s Not-for-Profit Corporation Law and Religious Corporations Law, was verified on May 1, 2026, and officially cleared by Assistant Attorney General Jeffrey Chester on May 19, 2026. The real estate footprint underlying the transaction encompasses block 15584, lot 16 for 609 Beach 9th Street and block 15585, proposed lot 16, for 1207 Caffrey Avenue. However, th</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto update queens news 2026-05-23T14:00:40Z
</commit_message>
<xml_diff>
--- a/data/output/queens_dev_news.xlsx
+++ b/data/output/queens_dev_news.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H8"/>
+  <dimension ref="A1:H5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -473,17 +473,17 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Premier Equities signs $9.2M refi loan with Peapack for retail in SoHo</t>
+          <t>Gorjian Real Estate pays $2.6M for 20-unit LES walkup</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>https://www.pincusco.com/premier-equities-signs-9-2m-refi-loan-with-peapack-for-retail-in-soho/</t>
+          <t>https://www.pincusco.com/gorjian-real-estate-pays-2-6m-for-20-unit-les-walkup/</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Premier Equities through the entity Premier 158 Mercer LLC as borrower signed a refi loan</t>
+          <t>Gorjian Real Estate Group through the entity GG 85 Ludlow LLC paid $2.6 million to</t>
         </is>
       </c>
       <c r="D2" t="inlineStr"/>
@@ -500,24 +500,24 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Transfers Premier Equities through the entity Premier 158 Mercer LLC as borrower signed a refi loan with lender Peapack Private Bank &amp; Trust valued at $9.2 million for the retail condo at 158 Mercer Street in SoHo, Manhattan. The deal closed on April 28, 2026 and was recorded on May 21, 2026. The prior lender was Webster Bank which held debt that had an original loan amount of $15 million. The property has 4,251 square feet of built space according to a PincusCo analysis of city data. The loan price per built square foot is $2,152 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) The owner bought the property on February 6, 2015, for $16 million. The signatory for Premier Equities was Mark D. Mermel . The signatory for Peapack Private Bank &amp; Trust was Nicholas LaMorte. The property The retail condo in SoHo has 4,251 square feet of built space according to a PincusCo analysis of city data. The parcel has a total lot size of 4,251 square feet. The city-designated market value for the property in 2022 is $6.6 million. Violations and lawsuits There were </t>
+          <t>Transfers 85 Ludlow Street (Credit - Cyclomedia) Gorjian Real Estate Group through the entity GG 85 Ludlow LLC paid $2.6 million to the entity Jema Holdings LLC for the 20-unit residential walkup building (C7) at 85 Ludlow Street in Lower East Side, Manhattan. The expected use is cash flowing. The deal closed on May 12, 2026 and was recorded on May 20, 2026. The property has 8,680 square feet of built space and 109 square feet of additional air rights for a total buildable of 8,784 square feet according to a PincusCo analysis of city data. The sale price per built square foot is $299 and the price per buildable square foot is $295 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) The signatories for the seller were Carol May, Jenny May Maiello, and Sherman Mei. The signatory for Gorjian Real Estate Group was Justin J. Gorjian . The contract date was March 13, 2026. Prior sales, articles and revenue Prior to this transaction, PincusCo has records that the buyer Gorjian Real Estate Group purchased seven properties in six transactions for a total of $28</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Corem Property Group signs $78.5M refi loan with affiliate for office in Penn Plaza</t>
+          <t>Revamp NYC files plans for 49 units in Riverdale</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>https://www.pincusco.com/corem-property-group-signs-78-5m-refi-loan-with-affiliate-for-office-in-penn-plaza/</t>
+          <t>https://www.pincusco.com/revamp-nyc-files-plans-for-49-units-in-riverdale/</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Corem Property Group through the entity 1241 Broadway LLC as borrower signed a refi loan</t>
+          <t>Revamp NYC submitted a new building construction project for a 49-unit, 30,646-square-foot residential (R-2) building</t>
         </is>
       </c>
       <c r="D3" t="inlineStr"/>
@@ -534,24 +534,24 @@
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>Transfers 1241 Broadway (Credit - Cyclomedia) Corem Property Group through the entity 1241 Broadway LLC as borrower signed a refi loan with an affiliate, the entity Corem Charlotta AB, valued at $78.5 million for the office building (O4) at 1241 Broadway in Penn Plaza, Manhattan. The deal closed on May 11, 2026 and was recorded on May 21, 2026. The prior lender was Deutsche Pfandbriefbank which held debt that had an original loan amount of $90 million. The property has 178,884 square feet of built space and 28,826 square feet of additional air rights for a total buildable of 191,325 square feet according to a PincusCo analysis of city data. The loan price per built square foot is $438 and the price per buildable square foot is $410 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) The signatory for Corem Property Group was David Roll . The signatory for Corem Property Group was Emelie Morndal . Prior sales, articles and revenue The 178,884-square-foot property generated revenue of $11.5 million or $64 per square foot, according to the most recent inc</t>
+          <t>Development 3230 Fairfield Avenue axonometric diagram (l.) and elevation (Credit - Mohammad Ahead professional engineer via DOB) (1) Revamp NYC submitted a new building construction project for a 49-unit, 30,646-square-foot residential (R-2) building at 3230 Fairfield Avenue in Riverdale, Bronx. The plan was filed on May 20, 2026. It calls for the construction of a 63-foot-tall, seven-story building and was filed with the New York City Department of Buildings under job number X01404499. The project is described in the filing as: subject building is a seven-story building. The applicant is the Professional Engineer Mohammad Ahead of Mohammad Ahead, Pe. Israel Tishler of Revamp NYC submitted the plans. The plans have no commercial space such as retail or office. The plans call for apartments on the first through the sixth floors. The seventh floor is “elevator and stairs bulkhead, with green roof zone area.” 3230 Fairfield Avenue The neighborhood</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Sheya Ungar pays $2.6M for 4-family in Williamsburg</t>
+          <t>Tomohiko Shimura pays $3.2M to Stellar for 25-unit rental in Harlem owned 37 years</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>https://www.pincusco.com/sheya-ungar-pays-2-6m-for-4-family-in-williamsburg/</t>
+          <t>https://www.pincusco.com/tomohiko-shimura-pays-3-2m-to-stellar-for-25-unit-rental-in-harlem-owned-37-years/</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Sheya Ungar through the entity Cggo Bunim LLC paid $2.6 million for the four-unit building</t>
+          <t>Tomohiko Shimura through the entity 123rd Holdings LLC paid $3.2 million to Stellar Management through</t>
         </is>
       </c>
       <c r="D4" t="inlineStr"/>
@@ -568,24 +568,24 @@
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Transfers 127 Penn Street (Credit - Cyclomedia) Sheya Ungar through the entity Cggo Bunim LLC paid $2.6 million for the four-unit building (C3) at 127 Penn Street in Williamsburg, Brooklyn. The deal closed on April 21, 2026 and was recorded on May 21, 2026. The property has 2,640 square feet of built space and 2,749 square feet of additional air rights for a total buildable of 5,387 square feet according to a PincusCo analysis of city data. The sale price per built square foot is $977 and the price per buildable square foot is $479 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) The signatory for the sellers were Lewis Gluck and Rachel Hopstein. The signatory for Sheya Ungar was Sheya Ungar. The contract date was April 21, 2026. Prior sales, articles and revenue Prior to this transaction, PincusCo has no record that the buyer Sheya Ungar had purchased any other properties and has no record it sold any properties over the past 24 months. The seller Lewis Gluck had not purchased any other properties and had not sold any properties over the same time </t>
+          <t>Transfers 15 West 123rd Street (Credit - Cyclomedia) Tomohiko Shimura through the entity 123rd Holdings LLC paid $3.2 million to Stellar Management through the entity One One Morris Park Associates, L.L.C. for the 25-unit residential elevator building (D1) at 11-15 West 123rd Street in Harlem, Manhattan. The expected use is cash flowing. The deal closed on May 14, 2026 and was recorded on May 21, 2026. The property has 23,946 square feet of built space according to a PincusCo analysis of city data. The sale price per built square foot is $135 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) The signatory for Stellar Management was Adam Roman . The signatory for Tomohiko Shimura was Tomohiko Shimura. The contract date was March 31, 2026. Stellar Management, which was formed in 1985, purchased the building on April 14, 1989, 37 years ago, for $303,000 (the sale price is calculated to a PincusCo analysis of transfer records) with a $170,000 mortgage. The 1989 buyer entity was in care of the firm Gluck, Witkoff &amp; Katz, a partnership led by Laurence Gluc</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Shabse Fuchs files plans for 31 units in Bushwick</t>
+          <t>NFS Development files plans for 63 units in Bedford Park</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>https://www.pincusco.com/shabse-fuchs-files-plans-for-31-units-in-bushwick/</t>
+          <t>https://www.pincusco.com/nfs-development-files-plans-for-63-units-in-bedford-park/</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Shabse Fuchs submitted a new building construction project for a 46-unit, 23,207-square-foot residential (R-2) building</t>
+          <t>Nush and Franco Sukaj’s NFS Development submitted a new building construction project for a 63-unit,</t>
         </is>
       </c>
       <c r="D5" t="inlineStr"/>
@@ -602,109 +602,7 @@
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>Development 102 Wyckoff Avenue axonometric diagram (Credit - Naresh Manangu professional engineer via DOB) Shabse Fuchs submitted a new building construction project for a 46-unit, 23,207-square-foot residential (R-2) building at 102 Wyckoff Avenue in Bushwick, Brooklyn. The plan was filed on May 20, 2026. It calls for the construction of a 82-foot-tall, eight-story building and was filed with the New York City Department of Buildings under job number B01401889. The project is described in the filing as: proposed 8-story and cellar residential and community facility building. The applicant is the Professional Engineer Naresh Mahangu of NKM Engineering PLLC. There are already 15 residential units on the tax block, the filing shows, for a total of 46 units on the tax block. The site is currently occupied by a six-story parking deck. The plans call for an ambulatory medical care facility on the ground floor and apartments on floors two to eight. 102 Wyckoff Avenue  The neighborhood</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>Wagner College pays $30M for former St. John’s University campus on Staten Island</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>https://www.pincusco.com/wagner-college-pays-30m-for-former-st-johns-university-campus-on-staten-island/</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>The private higher educational school Wagner College through the entity Seahawks Realty LLC paid the</t>
-        </is>
-      </c>
-      <c r="D6" t="inlineStr"/>
-      <c r="E6" t="inlineStr"/>
-      <c r="F6" t="inlineStr">
-        <is>
-          <t>PincusCo</t>
-        </is>
-      </c>
-      <c r="G6" t="inlineStr">
-        <is>
-          <t>PincusCo - Home</t>
-        </is>
-      </c>
-      <c r="H6" t="inlineStr">
-        <is>
-          <t>Transfers 300 Howard Avenue (Credit - Cyclomedia) The private higher educational school Wagner College through the entity Seahawks Realty LLC paid the Queens-based St. John’s University $30 million for the 10-building educational campus (W6) including the address 300 Howard Avenue in Silver Lake, Staten Island. The deal closed on May 11, 2026 and was recorded on May 21, 2026. The property has 146,855 square feet of built space and 395,307 square feet of additional air rights for a total buildable of 539,055 square feet according to a PincusCo analysis of city data. The sale price per built square foot is $204 and the price per buildable square foot is $55 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) The Staten Island Advance reported on the sale previously but did not include the price, but the report noted that Metropolitan Commercial Bank provided an undisclosed amount of financing. Prior sales, articles and revenue Prior to this transaction, PincusCo has no record that the buyer Wagner College had purchased any other properties and has no rec</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>Meadow Partners signs $19M rehab construction loan for 2 walkups in Williamsburg</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>https://www.pincusco.com/meadow-partners-signs-19m-rehab-construction-loan-for-2-walkup-in-williamsburg/</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>Meadow Partners through the entity 65-75 Roebling Owner, LLC as borrower signed a rehab construction</t>
-        </is>
-      </c>
-      <c r="D7" t="inlineStr"/>
-      <c r="E7" t="inlineStr"/>
-      <c r="F7" t="inlineStr">
-        <is>
-          <t>PincusCo</t>
-        </is>
-      </c>
-      <c r="G7" t="inlineStr">
-        <is>
-          <t>PincusCo - Home</t>
-        </is>
-      </c>
-      <c r="H7" t="inlineStr">
-        <is>
-          <t>Transfers 83 Roebling Street (Credit - Cyclomedia) Meadow Partners through the entity 65-75 Roebling Owner, LLC as borrower signed a rehab construction loan with lender Customers Bank valued at $19 million for two residential walkups with 55 residential units including the 31-unit residential walkup building (C1) at 83 Roebling Street in Williamsburg, Brooklyn and 24-unit residential walkup building (C7) at 65 Roebling Street in Williamsburg, Brooklyn. The deal closed on March 30, 2026 and was recorded on May 21, 2026. The prior lender was Customers Bank which held debt that had an original loan amount of $11.37 million. The two properties have 65,750 square feet of built space and 9,250 square feet of additional air rights for a total buildable of 75,000 square feet according to a PincusCo analysis of city data. The loan price per built square foot is $288 and the price per buildable square foot is $253 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) The signatory for Meadow Partners was Timothy P. Yantz . This is a rehab construction loan of $7.6</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>Far Rockaway Orthodox girls school approved for $21.4M construction loan</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>https://www.pincusco.com/far-rockaway-orthodox-girls-school-approved-for-21-4m-construction-loan/</t>
-        </is>
-      </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>The Orthodox girls school Bnos Bais Yaakov of Far Rockaway secured an approval from the</t>
-        </is>
-      </c>
-      <c r="D8" t="inlineStr"/>
-      <c r="E8" t="inlineStr"/>
-      <c r="F8" t="inlineStr">
-        <is>
-          <t>PincusCo</t>
-        </is>
-      </c>
-      <c r="G8" t="inlineStr">
-        <is>
-          <t>PincusCo - Home</t>
-        </is>
-      </c>
-      <c r="H8" t="inlineStr">
-        <is>
-          <t>Transfers 1207 Caffrey Avenue axonometrict diagram (Credit - Fariba Makooi architect via DOB) The Orthodox girls school Bnos Bais Yaakov of Far Rockaway secured an approval from the New York State Attorney General to obtain a new mortgage loan of up to $21.4 million from Bank United to fund the development of a new 68,000-square-foot high school building, and pay off an existing loan, at its campus in Far Rockaway, Queens. The commercial financing package will fund the construction of a new building at 1207 Caffrey Avenue through job number Q01129479 (with an alternate address of 613 Beach 9th Street) in the Far Rockaway neighborhood. It will pay off an older loan from Dime Community Bank secured by the existing school building at 609 Beach 9th Street. The regulatory petition, filed by the non-profit corporation under the state’s Not-for-Profit Corporation Law and Religious Corporations Law, was verified on May 1, 2026, and officially cleared by Assistant Attorney General Jeffrey Chester on May 19, 2026. The real estate footprint underlying the transaction encompasses block 15584, lot 16 for 609 Beach 9th Street and block 15585, proposed lot 16, for 1207 Caffrey Avenue. However, th</t>
+          <t>Development 2868 Jerome Avenue axonometric diagram and section (Credit - Mohammad Badaly architect via DOB) Nush and Franco Sukaj’s NFS Development submitted a new building construction project for a 63-unit, 47,785-square-foot residential (R-2) building at 2868 Jerome Avenue in Bedford Park, Bronx. The plan was filed on May 20, 2026. It calls for the construction of a 121-foot-tall, thirteen-story building and was filed with the New York City Department of Buildings under job number X01393299. The project is described in the filing as: proposed new 63-unit use group II apartment building, 13-story with cellar. The applicant is the Registered Architect Mohammad Badaly of Badaly Architects. Nush Sukaj of NFS Development submitted the plans. Nush Sukaj and Franco Sukaj bought the property for $4.1 million from a religious organization. 2868 Jerome Avenue The neighborhood</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto update queens news 2026-05-24T13:57:22Z
</commit_message>
<xml_diff>
--- a/data/output/queens_dev_news.xlsx
+++ b/data/output/queens_dev_news.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H5"/>
+  <dimension ref="A1:H1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -467,142 +467,6 @@
       <c r="H1" s="1" t="inlineStr">
         <is>
           <t>content_preview</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>Gorjian Real Estate pays $2.6M for 20-unit LES walkup</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>https://www.pincusco.com/gorjian-real-estate-pays-2-6m-for-20-unit-les-walkup/</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>Gorjian Real Estate Group through the entity GG 85 Ludlow LLC paid $2.6 million to</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr"/>
-      <c r="E2" t="inlineStr"/>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t>PincusCo</t>
-        </is>
-      </c>
-      <c r="G2" t="inlineStr">
-        <is>
-          <t>PincusCo - Home</t>
-        </is>
-      </c>
-      <c r="H2" t="inlineStr">
-        <is>
-          <t>Transfers 85 Ludlow Street (Credit - Cyclomedia) Gorjian Real Estate Group through the entity GG 85 Ludlow LLC paid $2.6 million to the entity Jema Holdings LLC for the 20-unit residential walkup building (C7) at 85 Ludlow Street in Lower East Side, Manhattan. The expected use is cash flowing. The deal closed on May 12, 2026 and was recorded on May 20, 2026. The property has 8,680 square feet of built space and 109 square feet of additional air rights for a total buildable of 8,784 square feet according to a PincusCo analysis of city data. The sale price per built square foot is $299 and the price per buildable square foot is $295 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) The signatories for the seller were Carol May, Jenny May Maiello, and Sherman Mei. The signatory for Gorjian Real Estate Group was Justin J. Gorjian . The contract date was March 13, 2026. Prior sales, articles and revenue Prior to this transaction, PincusCo has records that the buyer Gorjian Real Estate Group purchased seven properties in six transactions for a total of $28</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>Revamp NYC files plans for 49 units in Riverdale</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>https://www.pincusco.com/revamp-nyc-files-plans-for-49-units-in-riverdale/</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>Revamp NYC submitted a new building construction project for a 49-unit, 30,646-square-foot residential (R-2) building</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr"/>
-      <c r="E3" t="inlineStr"/>
-      <c r="F3" t="inlineStr">
-        <is>
-          <t>PincusCo</t>
-        </is>
-      </c>
-      <c r="G3" t="inlineStr">
-        <is>
-          <t>PincusCo - Home</t>
-        </is>
-      </c>
-      <c r="H3" t="inlineStr">
-        <is>
-          <t>Development 3230 Fairfield Avenue axonometric diagram (l.) and elevation (Credit - Mohammad Ahead professional engineer via DOB) (1) Revamp NYC submitted a new building construction project for a 49-unit, 30,646-square-foot residential (R-2) building at 3230 Fairfield Avenue in Riverdale, Bronx. The plan was filed on May 20, 2026. It calls for the construction of a 63-foot-tall, seven-story building and was filed with the New York City Department of Buildings under job number X01404499. The project is described in the filing as: subject building is a seven-story building. The applicant is the Professional Engineer Mohammad Ahead of Mohammad Ahead, Pe. Israel Tishler of Revamp NYC submitted the plans. The plans have no commercial space such as retail or office. The plans call for apartments on the first through the sixth floors. The seventh floor is “elevator and stairs bulkhead, with green roof zone area.” 3230 Fairfield Avenue The neighborhood</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>Tomohiko Shimura pays $3.2M to Stellar for 25-unit rental in Harlem owned 37 years</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>https://www.pincusco.com/tomohiko-shimura-pays-3-2m-to-stellar-for-25-unit-rental-in-harlem-owned-37-years/</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>Tomohiko Shimura through the entity 123rd Holdings LLC paid $3.2 million to Stellar Management through</t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr"/>
-      <c r="E4" t="inlineStr"/>
-      <c r="F4" t="inlineStr">
-        <is>
-          <t>PincusCo</t>
-        </is>
-      </c>
-      <c r="G4" t="inlineStr">
-        <is>
-          <t>PincusCo - Home</t>
-        </is>
-      </c>
-      <c r="H4" t="inlineStr">
-        <is>
-          <t>Transfers 15 West 123rd Street (Credit - Cyclomedia) Tomohiko Shimura through the entity 123rd Holdings LLC paid $3.2 million to Stellar Management through the entity One One Morris Park Associates, L.L.C. for the 25-unit residential elevator building (D1) at 11-15 West 123rd Street in Harlem, Manhattan. The expected use is cash flowing. The deal closed on May 14, 2026 and was recorded on May 21, 2026. The property has 23,946 square feet of built space according to a PincusCo analysis of city data. The sale price per built square foot is $135 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) The signatory for Stellar Management was Adam Roman . The signatory for Tomohiko Shimura was Tomohiko Shimura. The contract date was March 31, 2026. Stellar Management, which was formed in 1985, purchased the building on April 14, 1989, 37 years ago, for $303,000 (the sale price is calculated to a PincusCo analysis of transfer records) with a $170,000 mortgage. The 1989 buyer entity was in care of the firm Gluck, Witkoff &amp; Katz, a partnership led by Laurence Gluc</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>NFS Development files plans for 63 units in Bedford Park</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>https://www.pincusco.com/nfs-development-files-plans-for-63-units-in-bedford-park/</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>Nush and Franco Sukaj’s NFS Development submitted a new building construction project for a 63-unit,</t>
-        </is>
-      </c>
-      <c r="D5" t="inlineStr"/>
-      <c r="E5" t="inlineStr"/>
-      <c r="F5" t="inlineStr">
-        <is>
-          <t>PincusCo</t>
-        </is>
-      </c>
-      <c r="G5" t="inlineStr">
-        <is>
-          <t>PincusCo - Home</t>
-        </is>
-      </c>
-      <c r="H5" t="inlineStr">
-        <is>
-          <t>Development 2868 Jerome Avenue axonometric diagram and section (Credit - Mohammad Badaly architect via DOB) Nush and Franco Sukaj’s NFS Development submitted a new building construction project for a 63-unit, 47,785-square-foot residential (R-2) building at 2868 Jerome Avenue in Bedford Park, Bronx. The plan was filed on May 20, 2026. It calls for the construction of a 121-foot-tall, thirteen-story building and was filed with the New York City Department of Buildings under job number X01393299. The project is described in the filing as: proposed new 63-unit use group II apartment building, 13-story with cellar. The applicant is the Registered Architect Mohammad Badaly of Badaly Architects. Nush Sukaj of NFS Development submitted the plans. Nush Sukaj and Franco Sukaj bought the property for $4.1 million from a religious organization. 2868 Jerome Avenue The neighborhood</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto update queens news 2026-05-25T15:27:44Z
</commit_message>
<xml_diff>
--- a/data/output/queens_dev_news.xlsx
+++ b/data/output/queens_dev_news.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H1"/>
+  <dimension ref="A1:H3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -467,6 +467,74 @@
       <c r="H1" s="1" t="inlineStr">
         <is>
           <t>content_preview</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Related seeks 99K sf transit bonus for 625 Madison office project in Midtown East</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>https://www.pincusco.com/related-seeks-99k-sf-transit-bonus-for-625-madison-office-project-in-midtown-east/</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Real estate developer Related Companies submitted an application last week to the City Planning Commission</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr"/>
+      <c r="E2" t="inlineStr"/>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>PincusCo</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>PincusCo - Home</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>Development 625 Madison Avenue elevations from ULURP application (Credit - Gensler via DCP) Real estate developer Related Companies submitted an application last week to the City Planning Commission asking for 99,413 square feet of additional zoning floor area in its high end office project at 625 Madison Avenue in Midtown East, Manhattan. The additional development potential would be in exchange for Related making major transit improvements at the Fifth Avenue/59th Street subway station. The application, part of the city’s Uniform Land Use Review Procedure (ULURP), was submitted May 21, 2026. Project 2024M0267 LINK The regulatory filings were advanced to facilitate the construction of a 34-story, 800-foot-tall office and retail development on the east side of Madison Avenue between 58th and 59th streets. The site is vacant following the demolition last year of a building originally constructed in 1956. To increase the density of the project, the developer is utilizing a dual-track strategy that combines the 99,413-square-foot floor area bonus from mass transit infrastructure improvements, with a separate 29,780-square-foot transfer of development rights from a nearby, unidentified</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>TF Cornerstone advances 1,060-unit Greenpoint project with new ULURP filing</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>https://www.pincusco.com/tf-cornerstone-advances-1060-unit-greenpoint-project-with-new-ulurp-filing/</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>TF Cornerstone through the entity 2 Noble North LLC, submitted a design framework to the</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr"/>
+      <c r="E3" t="inlineStr"/>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>PincusCo</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>PincusCo - Home</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>Development 45 West Street on an undisclosed portion of 57 West Street, which is outlined (Credit - Google Earth) TF Cornerstone through the entity 2 Noble North LLC, submitted a design framework to the Department of City Planning under project number 2026K0129 last week, a required procedural step for its 1,060-unit project in Greenpoint, Brooklyn, that is located on the waterfront facing the East River. The application was filed May 21, 2026. Project 2026K0129 LINK The filing seeks mandatory chairperson certifications under Zoning Resolution Section 62-811, an essential regulatory clearance needed to proceed with the construction of an 880,295-square-foot mixed-use, two-tower complex on a vacant 173,834-square-foot waterfront lot at 2 Noble Street. While the towers are technically “as-of-right” regarding density and height , TF Cornerstone could not build them without this filing.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto update queens news 2026-05-26T16:06:02Z
</commit_message>
<xml_diff>
--- a/data/output/queens_dev_news.xlsx
+++ b/data/output/queens_dev_news.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H3"/>
+  <dimension ref="A1:H5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -473,17 +473,17 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Related seeks 99K sf transit bonus for 625 Madison office project in Midtown East</t>
+          <t>WellLife Network files plans for 165 units in Brownsville</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>https://www.pincusco.com/related-seeks-99k-sf-transit-bonus-for-625-madison-office-project-in-midtown-east/</t>
+          <t>https://www.pincusco.com/welllife-network-files-plans-for-165-units-in-brownsville/</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Real estate developer Related Companies submitted an application last week to the City Planning Commission</t>
+          <t>WellLife Network submitted a new building construction project for a 165-unit, 105,697-square-foot residential (R-2) building</t>
         </is>
       </c>
       <c r="D2" t="inlineStr"/>
@@ -500,24 +500,24 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>Development 625 Madison Avenue elevations from ULURP application (Credit - Gensler via DCP) Real estate developer Related Companies submitted an application last week to the City Planning Commission asking for 99,413 square feet of additional zoning floor area in its high end office project at 625 Madison Avenue in Midtown East, Manhattan. The additional development potential would be in exchange for Related making major transit improvements at the Fifth Avenue/59th Street subway station. The application, part of the city’s Uniform Land Use Review Procedure (ULURP), was submitted May 21, 2026. Project 2024M0267 LINK The regulatory filings were advanced to facilitate the construction of a 34-story, 800-foot-tall office and retail development on the east side of Madison Avenue between 58th and 59th streets. The site is vacant following the demolition last year of a building originally constructed in 1956. To increase the density of the project, the developer is utilizing a dual-track strategy that combines the 99,413-square-foot floor area bonus from mass transit infrastructure improvements, with a separate 29,780-square-foot transfer of development rights from a nearby, unidentified</t>
+          <t>Development 129 Osborn Street axonometric diagram (Credit - Alen Moghaddam architect via DOB) WellLife Network submitted a new building construction project for a 165-unit, 105,697-square-foot residential (R-2) building at 129 Osborn Street in Brownsville, Brooklyn. The plan was filed on May 20, 2026. It calls for the construction of a 110-foot-tall, eleven-story building and was filed with the New York City Department of Buildings under job number B01352178. The project is described in the filing as: propose a new 11-story mixed-use building (use group II for affordable housing and IIIb for community facility) as per the plan. obtain the new certificate of occupancy. The applicant is the Registered Architect Alen Moghaddam of Urban Architectural Initiatives. Alyse LaRue of WellLife Network submitted the plans. WellLife Network, a nonprofit, paid $8.7 million on April 22, 2025, for the development site to Russell and Brian Fedele, in two transactions. 129 Osborn Street The neighborhood</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>TF Cornerstone advances 1,060-unit Greenpoint project with new ULURP filing</t>
+          <t>Lian Wu Shao pays $4.2M for five-parcel dev site in Astoria</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>https://www.pincusco.com/tf-cornerstone-advances-1060-unit-greenpoint-project-with-new-ulurp-filing/</t>
+          <t>https://www.pincusco.com/lian-wu-shao-pays-4-2m-for-five-parcel-dev-site-in-astoria/</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>TF Cornerstone through the entity 2 Noble North LLC, submitted a design framework to the</t>
+          <t>Lian Wu Shao through the entity 26 Astoria LLC paid $4.2 million to Filingeri family</t>
         </is>
       </c>
       <c r="D3" t="inlineStr"/>
@@ -534,7 +534,75 @@
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>Development 45 West Street on an undisclosed portion of 57 West Street, which is outlined (Credit - Google Earth) TF Cornerstone through the entity 2 Noble North LLC, submitted a design framework to the Department of City Planning under project number 2026K0129 last week, a required procedural step for its 1,060-unit project in Greenpoint, Brooklyn, that is located on the waterfront facing the East River. The application was filed May 21, 2026. Project 2026K0129 LINK The filing seeks mandatory chairperson certifications under Zoning Resolution Section 62-811, an essential regulatory clearance needed to proceed with the construction of an 880,295-square-foot mixed-use, two-tower complex on a vacant 173,834-square-foot waterfront lot at 2 Noble Street. While the towers are technically “as-of-right” regarding density and height , TF Cornerstone could not build them without this filing.</t>
+          <t>Transfers 302 26th Avenue, 3-04 26th Avenue, 26-11 3rd Street, and 26-09 3rd Street (Credit - Google Earth) Lian Wu Shao through the entity 26 Astoria LLC paid $4.2 million to Filingeri family through the entity SBM, LLC for the five-parcel development site in Astoria, Queens, including the industrial building (F9) at 302 26th Avenue, the single-family building (A1) at 26-11 3rd Street, and the two-unit building (B2) at 3-04 26th Avenue. The expected use is ground up development. The deal closed on May 1, 2026 and was recorded on May 22, 2026. The five properties have 5,268 square feet of built space and 17,699 square feet of additional air rights for a total buildable of 22,980 square feet according to a PincusCo analysis of city data. The sale price per built square foot is $787 and the price per buildable square foot is $180 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) The signatory for Filingeri Family was Benedetto G. Filingeri. The signatory for Lian Wu Shao was Lian Wu Shao. The contract date was May 1, 2026. Because multiple properties h</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Simon Liu pays $3.1M for two retail condos in Chelsea</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>https://www.pincusco.com/simon-liu-pays-3-1m-for-two-retail-condos-in-chelsea/</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Simon Liu through the entity 362 Eighth Avenue LLC paid $3.1 million to the entity</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr"/>
+      <c r="E4" t="inlineStr"/>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>PincusCo</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>PincusCo - Home</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>Transfers 261 West 28th Street (Credit - Cyclomedia) Simon Liu through the entity 362 Eighth Avenue LLC paid $3.1 million to the entity 261 W 28th Lender LLC in care of Wachtel Missry, for two retail condominium units at 261 West 28th Street in Chelsea, Manhattan. The deal closed on May 14, 2026 and was recorded on May 22, 2026. The two properties have 4,107 square feet of built space according to a PincusCo analysis of city data. The sale price per built square foot is $754 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) The signatory for the buyer was Wachtel Missry attorney Ralph A. Dweck. The signatory for Simon Liu was Simon Liu. The contract date was March 31, 2026. BronfmanHaymes Real Estate Partners developed the condominium building, and lost these retail units to a lender, with anonymous ownership in care of the law firm Wachtel Missry, in December 2025. Prior sales, articles and revenue Prior to this transaction, PincusCo has no record that the buyer Simon Liu had purchased any other properties and has no record it sold any properties ov</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Rogers Equities pays $6M for portion of 85-unit dev site in Gowanus</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>https://www.pincusco.com/rogers-equities-pays-6m-for-portion-of-85-unit-dev-site-in-gowanus/</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Rogers Equities paid $6 million for two adjacent 2-family buildings in Gowanus, Brooklyn, in two</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr"/>
+      <c r="E5" t="inlineStr"/>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>PincusCo</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>PincusCo - Home</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>Transfers 244A 7th Street (Credit - Cyclomedia) Rogers Equities paid $6 million for two adjacent 2-family buildings in Gowanus, Brooklyn, in two transactions with separate sellers. The expected use is ground up development. The 85-unit development project has a 5-parcel zoning lot. As of publication only two of the five units, these two, show Rogers Equities as the owner in city records. The other three parcels are 244 7th Street, 416 4th Avenue and 418 4th Avenue. On these lots, there is one active new building construction project, B01315432, for a 85-unit, 60,085 square-foot residential (R-2) building. The project was submitted by Rogers Equities and filed by Abe Waldman with plans filed January 22, 2026 and it has not been permitted yet. In the first, Rogers Equities through the entity 416 4th Ave Realty LLC paid $3 million for the two-unit building (B3) at 244A 7th Street in Gowanus, Brooklyn. The deal closed on May 12, 2026 and was recorded on May 22, 2026. The property has 1,575 square feet of built space and 7,805 square feet of additional air rights for a total buildable of 9,379 square feet according to a PincusCo analysis of city data. The sale price per built square foo</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto update queens news 2026-05-27T16:10:32Z
</commit_message>
<xml_diff>
--- a/data/output/queens_dev_news.xlsx
+++ b/data/output/queens_dev_news.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H5"/>
+  <dimension ref="A1:H9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -473,17 +473,17 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>WellLife Network files plans for 165 units in Brownsville</t>
+          <t>Happy Living Management files plans for 8 units in Soundview</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>https://www.pincusco.com/welllife-network-files-plans-for-165-units-in-brownsville/</t>
+          <t>https://www.pincusco.com/happy-living-management-files-plans-for-8-units-in-soundview/</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>WellLife Network submitted a new building construction project for a 165-unit, 105,697-square-foot residential (R-2) building</t>
+          <t>Happy Living Management submitted a major alteration application for the conversion of a two-unit, two-story</t>
         </is>
       </c>
       <c r="D2" t="inlineStr"/>
@@ -500,24 +500,24 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>Development 129 Osborn Street axonometric diagram (Credit - Alen Moghaddam architect via DOB) WellLife Network submitted a new building construction project for a 165-unit, 105,697-square-foot residential (R-2) building at 129 Osborn Street in Brownsville, Brooklyn. The plan was filed on May 20, 2026. It calls for the construction of a 110-foot-tall, eleven-story building and was filed with the New York City Department of Buildings under job number B01352178. The project is described in the filing as: propose a new 11-story mixed-use building (use group II for affordable housing and IIIb for community facility) as per the plan. obtain the new certificate of occupancy. The applicant is the Registered Architect Alen Moghaddam of Urban Architectural Initiatives. Alyse LaRue of WellLife Network submitted the plans. WellLife Network, a nonprofit, paid $8.7 million on April 22, 2025, for the development site to Russell and Brian Fedele, in two transactions. 129 Osborn Street The neighborhood</t>
+          <t>Development 714 Taylor Avenue isometric diagram (Credit - Sharon Broyn architect via DOB) Happy Living Management submitted a major alteration application for the conversion of a two-unit, two-story residential (RES) building at 714 Taylor Avenue in Soundview, Bronx, to an eight-unit, three-story building. The plan was filed on May 25, 2026. It calls for an increase in size from a 22-foot-tall, two-story with 2 dwelling units to a 42-foot-tall, three-story with 8 dwelling units building and was filed with the New York City Department of Buildings under job number X01398999. The project is described in the filing as: application filed herewith to vertically enlarge an existing 2 story + cellar 2 family building to a 3 story + cellar 8 family building. The applicant is the Registered Architect Sharon Broyn of Basch A+D Corp. Jacob Zicherman of Happy Living Management submitted the plans. The neighborhood In Soundview, The majority, or 60 percent of the 21.7 million square feet of commercial built space are elevator buildings, with walkup buildings next occupying 20 percent of the space. In sales, Soundview has near average sales volume among other neighborhoods with $184.5 million in</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Lian Wu Shao pays $4.2M for five-parcel dev site in Astoria</t>
+          <t>10-unit UWS building sells for $4.2M</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>https://www.pincusco.com/lian-wu-shao-pays-4-2m-for-five-parcel-dev-site-in-astoria/</t>
+          <t>https://www.pincusco.com/10-unit-uws-building-sells-for-4-2m/</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Lian Wu Shao through the entity 26 Astoria LLC paid $4.2 million to Filingeri family</t>
+          <t>The entity 318 West 77th Street LLC in care of Building Equity Management, paid $4.2</t>
         </is>
       </c>
       <c r="D3" t="inlineStr"/>
@@ -534,24 +534,24 @@
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>Transfers 302 26th Avenue, 3-04 26th Avenue, 26-11 3rd Street, and 26-09 3rd Street (Credit - Google Earth) Lian Wu Shao through the entity 26 Astoria LLC paid $4.2 million to Filingeri family through the entity SBM, LLC for the five-parcel development site in Astoria, Queens, including the industrial building (F9) at 302 26th Avenue, the single-family building (A1) at 26-11 3rd Street, and the two-unit building (B2) at 3-04 26th Avenue. The expected use is ground up development. The deal closed on May 1, 2026 and was recorded on May 22, 2026. The five properties have 5,268 square feet of built space and 17,699 square feet of additional air rights for a total buildable of 22,980 square feet according to a PincusCo analysis of city data. The sale price per built square foot is $787 and the price per buildable square foot is $180 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) The signatory for Filingeri Family was Benedetto G. Filingeri. The signatory for Lian Wu Shao was Lian Wu Shao. The contract date was May 1, 2026. Because multiple properties h</t>
+          <t>Transfers 318 West 77th Street (Credit - Cyclomedia) The entity 318 West 77th Street LLC in care of Building Equity Management, paid $4.2 million to Nicholas Osso through the entity Nicholas S. Osso, L.L.C. for the 10-unit residential walkup building (C1) at 318 West 77th Street in Upper West Side, Manhattan. The expected use is cash flowing. The deal closed on May 11, 2026 and was recorded on May 26, 2026. The property has 6,380 square feet of built space and 2,607 square feet of additional air rights for a total buildable of 8,992 square feet according to a PincusCo analysis of city data. The sale price per built square foot is $666 and the price per buildable square foot is $472 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) The signatory for Nicholas Osso was Nicholas S. Osso . The signatory for the buyer was Kathryn Lecusay. The contract date was January 29, 2026. Prior sales, articles and revenue Prior to this transaction, PincusCo has no record that the buyer Building Equity Management registered had purchased any other properties and has n</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Simon Liu pays $3.1M for two retail condos in Chelsea</t>
+          <t>Peter Florey of D&amp;F Development acquires 16-unit Friedman Management rental in Lenox Hill for $9.4M</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>https://www.pincusco.com/simon-liu-pays-3-1m-for-two-retail-condos-in-chelsea/</t>
+          <t>https://www.pincusco.com/peter-florey-of-df-development-acquires-16-unit-friedman-management-rental-in-lenox-hill-for-9-4m/</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Simon Liu through the entity 362 Eighth Avenue LLC paid $3.1 million to the entity</t>
+          <t>Peter Florey of D&amp;F Development Group through the entity NYC Prop 1 LLC paid $9.4</t>
         </is>
       </c>
       <c r="D4" t="inlineStr"/>
@@ -568,24 +568,24 @@
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>Transfers 261 West 28th Street (Credit - Cyclomedia) Simon Liu through the entity 362 Eighth Avenue LLC paid $3.1 million to the entity 261 W 28th Lender LLC in care of Wachtel Missry, for two retail condominium units at 261 West 28th Street in Chelsea, Manhattan. The deal closed on May 14, 2026 and was recorded on May 22, 2026. The two properties have 4,107 square feet of built space according to a PincusCo analysis of city data. The sale price per built square foot is $754 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) The signatory for the buyer was Wachtel Missry attorney Ralph A. Dweck. The signatory for Simon Liu was Simon Liu. The contract date was March 31, 2026. BronfmanHaymes Real Estate Partners developed the condominium building, and lost these retail units to a lender, with anonymous ownership in care of the law firm Wachtel Missry, in December 2025. Prior sales, articles and revenue Prior to this transaction, PincusCo has no record that the buyer Simon Liu had purchased any other properties and has no record it sold any properties ov</t>
+          <t>Transfers 11 East 78th Street (Credit - Cyclomedia) Peter Florey of D&amp;F Development Group through the entity NYC Prop 1 LLC paid $9.4 million to Friedman Management through the entity 11e78 Realty LLC for the 16-unit residential elevator building (D3) at 11 East 78th Street in Lenox Hill, Manhattan. The expected use is cash flowing. The deal closed on May 13, 2026 and was recorded on May 26, 2026. The property has 8,234 square feet of built space and 1,992 square feet of additional air rights for a total buildable of 10,216 square feet according to a PincusCo analysis of city data. The sale price per built square foot is $1,147 and the price per buildable square foot is $925 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) The signatory for Friedman Management was Robert Friedman . The signatory for D&amp;F Development Group was Peter Florey . The contract date was May 13, 2026. Prior sales, articles and revenue Prior to this transaction, PincusCo has records that the buyer D&amp;F Development Group purchased one property in one transaction for a total of $</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Rogers Equities pays $6M for portion of 85-unit dev site in Gowanus</t>
+          <t>Debt-holder Capstone acquires Madison Capital, Vornado office building in SoHo in $51.4M transfer</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>https://www.pincusco.com/rogers-equities-pays-6m-for-portion-of-85-unit-dev-site-in-gowanus/</t>
+          <t>https://www.pincusco.com/debt-holder-capstone-acquires-madison-capital-vornado-office-building-in-soho-in-51-4m-transfer/</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Rogers Equities paid $6 million for two adjacent 2-family buildings in Gowanus, Brooklyn, in two</t>
+          <t>Note-owner Capstone Equities through the entity CE 140 Crosby Owner LLC acquired the office building</t>
         </is>
       </c>
       <c r="D5" t="inlineStr"/>
@@ -602,7 +602,143 @@
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>Transfers 244A 7th Street (Credit - Cyclomedia) Rogers Equities paid $6 million for two adjacent 2-family buildings in Gowanus, Brooklyn, in two transactions with separate sellers. The expected use is ground up development. The 85-unit development project has a 5-parcel zoning lot. As of publication only two of the five units, these two, show Rogers Equities as the owner in city records. The other three parcels are 244 7th Street, 416 4th Avenue and 418 4th Avenue. On these lots, there is one active new building construction project, B01315432, for a 85-unit, 60,085 square-foot residential (R-2) building. The project was submitted by Rogers Equities and filed by Abe Waldman with plans filed January 22, 2026 and it has not been permitted yet. In the first, Rogers Equities through the entity 416 4th Ave Realty LLC paid $3 million for the two-unit building (B3) at 244A 7th Street in Gowanus, Brooklyn. The deal closed on May 12, 2026 and was recorded on May 22, 2026. The property has 1,575 square feet of built space and 7,805 square feet of additional air rights for a total buildable of 9,379 square feet according to a PincusCo analysis of city data. The sale price per built square foo</t>
+          <t xml:space="preserve">Transfers 140 Crosby Street (Credit - Cyclomedia) Note-owner Capstone Equities through the entity CE 140 Crosby Owner LLC acquired the office building (O5) at 140 Crosby Street in SoHo, Manhattan from Madison Capital and Vornado Realty Trust through the entity MC 19 East Houston LLC, in a transfer valued for tax purposes at $51.4 million. The expected use is cash flowing. The deal closed on May 14, 2026 and was recorded on May 26, 2026. The property has 32,282 square feet of built space and 23,398 square feet of additional air rights for a total buildable of 55,710 square feet according to a PincusCo analysis of city data. The sale price per built square foot is $1,593 and the price per buildable square foot is $923 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) The seller bought the property on May 20, 2016, for $38.8 million, then constructed the new, existing building. The signatory for Madison Capital was J. Joseph Jacobson . The signatory for Capstone Equities was Avi Kollenscher . The contract date was May 14, 2026. Capstone bought the debt </t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Chestnut Holdings pays $9.4M to Gould Investors for residential elevator in Carnegie Hill</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>https://www.pincusco.com/chestnut-holdings-pays-9-4m-to-gould-investors-for-residential-elevator-in-carnegie-hill/</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Chestnut Holdings Of New York through the entity 96th Street Realty LLC paid $9.4 million</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr"/>
+      <c r="E6" t="inlineStr"/>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>PincusCo</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>PincusCo - Home</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>Transfers 155 East 96th Street (Credit - Cyclomedia) Chestnut Holdings Of New York through the entity 96th Street Realty LLC paid $9.4 million to Gould Investors through the entity Gould East 96th Street LLC for the 40-unit residential elevator building (D3) at 155 East 96th Street in Carnegie Hill, Manhattan. The expected use is cash flowing. The deal closed on May 19, 2026 and was recorded on May 26, 2026. The property has 37,065 square feet of built space and 57,769 square feet of additional air rights for a total buildable of 94,860 square feet according to a PincusCo analysis of city data. The sale price per built square foot is $252 and the price per buildable square foot is $98 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) The seller bought the property on May 31, 2018, for $25.4 million. The signatory for Gould Investors was Mark H. Lundy . The signatory for Chestnut Holdings Of New York was Anthony Simari . The contract date was March 10, 2026. Prior sales, articles and revenue Prior to this transaction, PincusCo has records that the buy</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>AG Holding Group pays $3.1M for 99-unit dev site in Mt Hope</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>https://www.pincusco.com/ag-holding-group-pays-3-1m-for-99-unit-dev-site-in-mt-hope/</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>AG Holding Group through the entity 1917 Morris LLC paid $3.1 million to Annal Management</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr"/>
+      <c r="E7" t="inlineStr"/>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>PincusCo</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>PincusCo - Home</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Transfers 1917 Morris Avenue axonometric diagram (Credit - John Backos architect via DOB) AG Holding Group through the entity 1917 Morris LLC paid $3.1 million to Annal Management through the entity 1915 Morris Avenue Corp. for the 99-unit development site that is currently a parking lot (G7) at 1917 Morris Avenue in Mt Hope, Bronx. The expected use is ground up development. AG Holding Group filed plans under job number X01399986, for a 99-unit, 59,704 square-foot residential (R-2) building submitted by Andrea Gjini on May 12, 2026 and it has not been permitted yet. The sale closed on May 12, 2026 and was recorded on May 26, 2026. The property has zero square feet of built space and 40,635 square feet of additional air rights for a total buildable of 40,635 square feet according to a PincusCo analysis of city data. The sale price per buildable square foot is $77 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) The signatory for Annal Management was Amy Chasin . The signatory for AG Holding Group was Andrea Gjini . The contract date was November 25, </t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Candor Capital signs ground lease valued at $3.2M for 65-unit dev site in Park Slope</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>https://www.pincusco.com/candor-capital-signs-3-2m-for-65-unit-dev-site-in-park-slope/</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Candor Capital through the entity St Johns Pl Holdings LLC as tenant signed a 49-year</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr"/>
+      <c r="E8" t="inlineStr"/>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>PincusCo</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>PincusCo - Home</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>Transfers 354 Flatbush Avenue (Credit - Cyclomedia) Candor Capital through the entity St Johns Pl Holdings LLC as tenant signed a 49-year ground lease valued at $3.2 million with landlords Michael Pintchik and Matthew Pintchik through the entity MBP 354 Flatbush TIC LLC for the development site that is currently a retail building (K7) at 358 Flatbush Avenue in Park Slope, Brooklyn. The expected use is ground up development. On the lot, there is one active new building construction project, B01367848, for a 65-unit, 62,548 square-foot residential (R-2) building. The project was submitted by Ami Weinstock and filed by Ami Weinstock with plans filed May 20, 2026 and it has not been permitted yet. The deal closed on May 15, 2026 and was recorded on May 26, 2026. The property has 5,965 square feet of built space and 17,895 square feet of additional air rights for a total buildable of 23,860 square feet according to a PincusCo analysis of city data. The sale price per built square foot is $543 and the price per buildable square foot is $135 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assu</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Arben Mitaj files plans for 22 units in Wakefield</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>https://www.pincusco.com/arben-mitaj-files-plans-for-22-units-in-wakefield/</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Arben Mitaj submitted a new building construction project for a 22-unit, 16,032-square-foot residential (R-2) building</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr"/>
+      <c r="E9" t="inlineStr"/>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>PincusCo</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>PincusCo - Home</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>Development 625 East 222nd Street axonometric diagram (Credit - Mohammad Badaly architect via DOB) Arben Mitaj submitted a new building construction project for a 22-unit, 16,032-square-foot residential (R-2) building at 625 East 222nd Street in Wakefield, the Bronx. The plan was filed on May 21, 2026. It calls for the construction of a 50-foot-tall, five-story building and was filed with the New York City Department of Buildings under job number X01391499. The project is described in the filing as: proposed new 22-unit group II &amp; III(b) apartment building, two tax lots on one zoning lot, 5-story without cellar, construction class i-b.. The applicant is the Registered Architect Mohammad Badaly of Badaly Architects. The plans call for medical offices on the ground floor and apartments on the first through the fifth floor. 625 East 222nd Street The neighborhood</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto update queens news 2026-05-28T16:30:47Z
</commit_message>
<xml_diff>
--- a/data/output/queens_dev_news.xlsx
+++ b/data/output/queens_dev_news.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H9"/>
+  <dimension ref="A1:H5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -473,17 +473,17 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Happy Living Management files plans for 8 units in Soundview</t>
+          <t>Elishaevs, Soolaev, sign $12.8M loan with ConnectOne for retail center in Forest Hills</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>https://www.pincusco.com/happy-living-management-files-plans-for-8-units-in-soundview/</t>
+          <t>https://www.pincusco.com/elishaevs-soolaev-sign-12-8m-loan-with-connectone-for-retail-center-in-forest-hills/</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Happy Living Management submitted a major alteration application for the conversion of a two-unit, two-story</t>
+          <t>Natanielle S. Elishaev, Gavriel Soolaev, and Ronit Elishaev through the entity Queens Blvd 104 LLC</t>
         </is>
       </c>
       <c r="D2" t="inlineStr"/>
@@ -500,24 +500,24 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>Development 714 Taylor Avenue isometric diagram (Credit - Sharon Broyn architect via DOB) Happy Living Management submitted a major alteration application for the conversion of a two-unit, two-story residential (RES) building at 714 Taylor Avenue in Soundview, Bronx, to an eight-unit, three-story building. The plan was filed on May 25, 2026. It calls for an increase in size from a 22-foot-tall, two-story with 2 dwelling units to a 42-foot-tall, three-story with 8 dwelling units building and was filed with the New York City Department of Buildings under job number X01398999. The project is described in the filing as: application filed herewith to vertically enlarge an existing 2 story + cellar 2 family building to a 3 story + cellar 8 family building. The applicant is the Registered Architect Sharon Broyn of Basch A+D Corp. Jacob Zicherman of Happy Living Management submitted the plans. The neighborhood In Soundview, The majority, or 60 percent of the 21.7 million square feet of commercial built space are elevator buildings, with walkup buildings next occupying 20 percent of the space. In sales, Soundview has near average sales volume among other neighborhoods with $184.5 million in</t>
+          <t>Transfers 104-15 Queens Boulevard (Credit - Google) Natanielle S. Elishaev, Gavriel Soolaev, and Ronit Elishaev through the entity Queens Blvd 104 LLC as borrower signed a initial loan with lender ConnectOne Bank through the entity Connectone Bank valued at $12.8 million for the retail strip center complex (K1) at 104-15 Queens Boulevard in Forest Hills, Queens. The deal closed on May 19, 2026 and was recorded on May 27, 2026. The property has 23,780 square feet of built space and 115,804 square feet of additional air rights for a total buildable of 139,777 square feet according to a PincusCo analysis of city data. The loan price per built square foot is $536 and the price per buildable square foot is $91 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) The owners bought the property on August 28, 2025, for $25.9 million. The signatory for Natanielle S. Elishaev , Gavriel Soolaev , and Ronit Elishaev was Natanielle S. Elishaev, Gavriel Soolaev, and Ronit Elishaev. Prior sales, articles and revenue The 23,780-square-foot property generated revenue of</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>10-unit UWS building sells for $4.2M</t>
+          <t>Eun Rae Jo pays $16.3M to Revere Capital for mixed-use in Flatiron District</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>https://www.pincusco.com/10-unit-uws-building-sells-for-4-2m/</t>
+          <t>https://www.pincusco.com/eun-rae-jo-pays-16-3m-to-revere-capital-for-in-flatiron-district/</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>The entity 318 West 77th Street LLC in care of Building Equity Management, paid $4.2</t>
+          <t>Eun Rae Jo through the entity 16 Joe 18 LLC paid $16.3 million to Revere</t>
         </is>
       </c>
       <c r="D3" t="inlineStr"/>
@@ -534,24 +534,24 @@
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>Transfers 318 West 77th Street (Credit - Cyclomedia) The entity 318 West 77th Street LLC in care of Building Equity Management, paid $4.2 million to Nicholas Osso through the entity Nicholas S. Osso, L.L.C. for the 10-unit residential walkup building (C1) at 318 West 77th Street in Upper West Side, Manhattan. The expected use is cash flowing. The deal closed on May 11, 2026 and was recorded on May 26, 2026. The property has 6,380 square feet of built space and 2,607 square feet of additional air rights for a total buildable of 8,992 square feet according to a PincusCo analysis of city data. The sale price per built square foot is $666 and the price per buildable square foot is $472 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) The signatory for Nicholas Osso was Nicholas S. Osso . The signatory for the buyer was Kathryn Lecusay. The contract date was January 29, 2026. Prior sales, articles and revenue Prior to this transaction, PincusCo has no record that the buyer Building Equity Management registered had purchased any other properties and has n</t>
+          <t>Transfers 16 East 18th Street (Credit - Cyclomedia) Eun Rae Jo through the entity 16 Joe 18 LLC paid $16.3 million to Revere Capital through the entity Nyc 18th Street LLC for the eight-unit property (DB) at 16 East 18th Street in Flatiron District, Manhattan. The expected use is cash flowing. The deal closed on April 17, 2026 and was recorded on May 27, 2026. The property has 20,258 square feet of built space according to a PincusCo analysis of city data. The sale price per built square foot is $804 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) The seller bought the property on July 1, 2022, for $3.7 million. The signatory for Revere Capital was Clark Briner . The signatory for Eun Rae Jo was Hyun Jun An . The contract date was February 6, 2026. Prior sales, articles and revenue Prior to this transaction, PincusCo has records that the buyer Eun Rae Jo purchased one property in one transaction for a total of $6.6 million and has no record it sold any properties over the past 24 months. The seller Revere Capital had not purchased any other propert</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Peter Florey of D&amp;F Development acquires 16-unit Friedman Management rental in Lenox Hill for $9.4M</t>
+          <t>Rogers Equities pays $8.625M for portion of 85-unit dev site in Gowanus</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>https://www.pincusco.com/peter-florey-of-df-development-acquires-16-unit-friedman-management-rental-in-lenox-hill-for-9-4m/</t>
+          <t>https://www.pincusco.com/rogers-equities-pays-8-625m-for-portion-of-85-unit-dev-site-in-gowanus/</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Peter Florey of D&amp;F Development Group through the entity NYC Prop 1 LLC paid $9.4</t>
+          <t>Abraham Waldman’s Rogers Equities paid $8.625 million for two buildings that form a portion of</t>
         </is>
       </c>
       <c r="D4" t="inlineStr"/>
@@ -568,24 +568,24 @@
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>Transfers 11 East 78th Street (Credit - Cyclomedia) Peter Florey of D&amp;F Development Group through the entity NYC Prop 1 LLC paid $9.4 million to Friedman Management through the entity 11e78 Realty LLC for the 16-unit residential elevator building (D3) at 11 East 78th Street in Lenox Hill, Manhattan. The expected use is cash flowing. The deal closed on May 13, 2026 and was recorded on May 26, 2026. The property has 8,234 square feet of built space and 1,992 square feet of additional air rights for a total buildable of 10,216 square feet according to a PincusCo analysis of city data. The sale price per built square foot is $1,147 and the price per buildable square foot is $925 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) The signatory for Friedman Management was Robert Friedman . The signatory for D&amp;F Development Group was Peter Florey . The contract date was May 13, 2026. Prior sales, articles and revenue Prior to this transaction, PincusCo has records that the buyer D&amp;F Development Group purchased one property in one transaction for a total of $</t>
+          <t>Transfers 416-418 4th Avenue (Credit - Cyclomedia) Abraham Waldman’s Rogers Equities paid $8.625 million for two buildings that form a portion of the five property footprint for an 85-unit project in Gowanus, Brooklyn. Rogers Equities already recorded the closed sales for 244A and 246 7th Street, for $6 million. In the first of the new closings, Rogers Equities through the entity 416 4th Ave Realty LLC paid $4.7 million to Nida Nagi Esa through the entity 248 Park Slope LLC for the six-unit mixed-use building (S5) at 416 4th Avenue in Gowanus, Brooklyn. The expected use is ground up development. The deal closed on May 12, 2026 and was recorded on May 27, 2026. The property has 7,280 square feet of built space and 3,676 square feet of additional air rights for a total buildable of 10,956 square feet according to a PincusCo analysis of city data. The sale price per built square foot is $641 and the price per buildable square foot is $426 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) The signatory for Nida Nagi Esa was Nida Nagi Esa. The signatory f</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Debt-holder Capstone acquires Madison Capital, Vornado office building in SoHo in $51.4M transfer</t>
+          <t>Rabsky pays $30M to Braha, ISJ, Jenel, Buhm Roe, Nakash for office in FiDi, Blackstone was foreclosing</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>https://www.pincusco.com/debt-holder-capstone-acquires-madison-capital-vornado-office-building-in-soho-in-51-4m-transfer/</t>
+          <t>https://www.pincusco.com/rabsky-pays-30m-to-braha-isj-jenel-buhm-roe-nakash-for-office-in-fidi-blackstone-was-foreclosing/</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Note-owner Capstone Equities through the entity CE 140 Crosby Owner LLC acquired the office building</t>
+          <t>Rabsky Group through the entity 267 Broadway LLC paid $30 million to Ralph Braha, ISJ</t>
         </is>
       </c>
       <c r="D5" t="inlineStr"/>
@@ -602,143 +602,7 @@
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Transfers 140 Crosby Street (Credit - Cyclomedia) Note-owner Capstone Equities through the entity CE 140 Crosby Owner LLC acquired the office building (O5) at 140 Crosby Street in SoHo, Manhattan from Madison Capital and Vornado Realty Trust through the entity MC 19 East Houston LLC, in a transfer valued for tax purposes at $51.4 million. The expected use is cash flowing. The deal closed on May 14, 2026 and was recorded on May 26, 2026. The property has 32,282 square feet of built space and 23,398 square feet of additional air rights for a total buildable of 55,710 square feet according to a PincusCo analysis of city data. The sale price per built square foot is $1,593 and the price per buildable square foot is $923 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) The seller bought the property on May 20, 2016, for $38.8 million, then constructed the new, existing building. The signatory for Madison Capital was J. Joseph Jacobson . The signatory for Capstone Equities was Avi Kollenscher . The contract date was May 14, 2026. Capstone bought the debt </t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>Chestnut Holdings pays $9.4M to Gould Investors for residential elevator in Carnegie Hill</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>https://www.pincusco.com/chestnut-holdings-pays-9-4m-to-gould-investors-for-residential-elevator-in-carnegie-hill/</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>Chestnut Holdings Of New York through the entity 96th Street Realty LLC paid $9.4 million</t>
-        </is>
-      </c>
-      <c r="D6" t="inlineStr"/>
-      <c r="E6" t="inlineStr"/>
-      <c r="F6" t="inlineStr">
-        <is>
-          <t>PincusCo</t>
-        </is>
-      </c>
-      <c r="G6" t="inlineStr">
-        <is>
-          <t>PincusCo - Home</t>
-        </is>
-      </c>
-      <c r="H6" t="inlineStr">
-        <is>
-          <t>Transfers 155 East 96th Street (Credit - Cyclomedia) Chestnut Holdings Of New York through the entity 96th Street Realty LLC paid $9.4 million to Gould Investors through the entity Gould East 96th Street LLC for the 40-unit residential elevator building (D3) at 155 East 96th Street in Carnegie Hill, Manhattan. The expected use is cash flowing. The deal closed on May 19, 2026 and was recorded on May 26, 2026. The property has 37,065 square feet of built space and 57,769 square feet of additional air rights for a total buildable of 94,860 square feet according to a PincusCo analysis of city data. The sale price per built square foot is $252 and the price per buildable square foot is $98 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) The seller bought the property on May 31, 2018, for $25.4 million. The signatory for Gould Investors was Mark H. Lundy . The signatory for Chestnut Holdings Of New York was Anthony Simari . The contract date was March 10, 2026. Prior sales, articles and revenue Prior to this transaction, PincusCo has records that the buy</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>AG Holding Group pays $3.1M for 99-unit dev site in Mt Hope</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>https://www.pincusco.com/ag-holding-group-pays-3-1m-for-99-unit-dev-site-in-mt-hope/</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>AG Holding Group through the entity 1917 Morris LLC paid $3.1 million to Annal Management</t>
-        </is>
-      </c>
-      <c r="D7" t="inlineStr"/>
-      <c r="E7" t="inlineStr"/>
-      <c r="F7" t="inlineStr">
-        <is>
-          <t>PincusCo</t>
-        </is>
-      </c>
-      <c r="G7" t="inlineStr">
-        <is>
-          <t>PincusCo - Home</t>
-        </is>
-      </c>
-      <c r="H7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Transfers 1917 Morris Avenue axonometric diagram (Credit - John Backos architect via DOB) AG Holding Group through the entity 1917 Morris LLC paid $3.1 million to Annal Management through the entity 1915 Morris Avenue Corp. for the 99-unit development site that is currently a parking lot (G7) at 1917 Morris Avenue in Mt Hope, Bronx. The expected use is ground up development. AG Holding Group filed plans under job number X01399986, for a 99-unit, 59,704 square-foot residential (R-2) building submitted by Andrea Gjini on May 12, 2026 and it has not been permitted yet. The sale closed on May 12, 2026 and was recorded on May 26, 2026. The property has zero square feet of built space and 40,635 square feet of additional air rights for a total buildable of 40,635 square feet according to a PincusCo analysis of city data. The sale price per buildable square foot is $77 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) The signatory for Annal Management was Amy Chasin . The signatory for AG Holding Group was Andrea Gjini . The contract date was November 25, </t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>Candor Capital signs ground lease valued at $3.2M for 65-unit dev site in Park Slope</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>https://www.pincusco.com/candor-capital-signs-3-2m-for-65-unit-dev-site-in-park-slope/</t>
-        </is>
-      </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>Candor Capital through the entity St Johns Pl Holdings LLC as tenant signed a 49-year</t>
-        </is>
-      </c>
-      <c r="D8" t="inlineStr"/>
-      <c r="E8" t="inlineStr"/>
-      <c r="F8" t="inlineStr">
-        <is>
-          <t>PincusCo</t>
-        </is>
-      </c>
-      <c r="G8" t="inlineStr">
-        <is>
-          <t>PincusCo - Home</t>
-        </is>
-      </c>
-      <c r="H8" t="inlineStr">
-        <is>
-          <t>Transfers 354 Flatbush Avenue (Credit - Cyclomedia) Candor Capital through the entity St Johns Pl Holdings LLC as tenant signed a 49-year ground lease valued at $3.2 million with landlords Michael Pintchik and Matthew Pintchik through the entity MBP 354 Flatbush TIC LLC for the development site that is currently a retail building (K7) at 358 Flatbush Avenue in Park Slope, Brooklyn. The expected use is ground up development. On the lot, there is one active new building construction project, B01367848, for a 65-unit, 62,548 square-foot residential (R-2) building. The project was submitted by Ami Weinstock and filed by Ami Weinstock with plans filed May 20, 2026 and it has not been permitted yet. The deal closed on May 15, 2026 and was recorded on May 26, 2026. The property has 5,965 square feet of built space and 17,895 square feet of additional air rights for a total buildable of 23,860 square feet according to a PincusCo analysis of city data. The sale price per built square foot is $543 and the price per buildable square foot is $135 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assu</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>Arben Mitaj files plans for 22 units in Wakefield</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>https://www.pincusco.com/arben-mitaj-files-plans-for-22-units-in-wakefield/</t>
-        </is>
-      </c>
-      <c r="C9" t="inlineStr">
-        <is>
-          <t>Arben Mitaj submitted a new building construction project for a 22-unit, 16,032-square-foot residential (R-2) building</t>
-        </is>
-      </c>
-      <c r="D9" t="inlineStr"/>
-      <c r="E9" t="inlineStr"/>
-      <c r="F9" t="inlineStr">
-        <is>
-          <t>PincusCo</t>
-        </is>
-      </c>
-      <c r="G9" t="inlineStr">
-        <is>
-          <t>PincusCo - Home</t>
-        </is>
-      </c>
-      <c r="H9" t="inlineStr">
-        <is>
-          <t>Development 625 East 222nd Street axonometric diagram (Credit - Mohammad Badaly architect via DOB) Arben Mitaj submitted a new building construction project for a 22-unit, 16,032-square-foot residential (R-2) building at 625 East 222nd Street in Wakefield, the Bronx. The plan was filed on May 21, 2026. It calls for the construction of a 50-foot-tall, five-story building and was filed with the New York City Department of Buildings under job number X01391499. The project is described in the filing as: proposed new 22-unit group II &amp; III(b) apartment building, two tax lots on one zoning lot, 5-story without cellar, construction class i-b.. The applicant is the Registered Architect Mohammad Badaly of Badaly Architects. The plans call for medical offices on the ground floor and apartments on the first through the fifth floor. 625 East 222nd Street The neighborhood</t>
+          <t>Transfers 267 Broadway (Credit - Cyclomedia) Rabsky Group through the entity 267 Broadway LLC paid $30 million to Ralph Braha, ISJ Management, Jenel Management, Buhm Roe, and Nakash Holdings through the entity 267 Property Corp. for the office building (O5) at 267 Broadway in Financial District, Manhattan. Blackstone Group had filed a pre-foreclosure action over a $25 million loan, in 2024. The expected use is redevelopment. The deal closed on May 14, 2026 and was recorded on May 27, 2026. The property has 29,000 square feet of built space and 22,709 square feet of additional air rights for a total buildable of 51,730 square feet according to a PincusCo analysis of city data. The sale price per built square foot is $1,034 and the price per buildable square foot is $579 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) The signatory for Ralph Braha , ISJ Management , Jenel Management , Buhm Roe , and Nakash Holdings was Ralph Braha. The signatory for Rabsky Group was Abraham Kohn . The contract date was February 19, 2026. To finance the purchase, Rabs</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto update queens news 2026-05-29T16:07:36Z
</commit_message>
<xml_diff>
--- a/data/output/queens_dev_news.xlsx
+++ b/data/output/queens_dev_news.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H5"/>
+  <dimension ref="A1:H7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -473,17 +473,17 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Elishaevs, Soolaev, sign $12.8M loan with ConnectOne for retail center in Forest Hills</t>
+          <t>Hiwin Group signs $40M construction loan with Cathay for 55-unit condo in Flatiron District</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>https://www.pincusco.com/elishaevs-soolaev-sign-12-8m-loan-with-connectone-for-retail-center-in-forest-hills/</t>
+          <t>https://www.pincusco.com/hiwin-group-signs-40m-construction-loan-with-cathay-for-development-in-flatiron-district/</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Natanielle S. Elishaev, Gavriel Soolaev, and Ronit Elishaev through the entity Queens Blvd 104 LLC</t>
+          <t>Hiwin Group USA through the entity Hw W 14th St LLC as borrower signed a</t>
         </is>
       </c>
       <c r="D2" t="inlineStr"/>
@@ -500,24 +500,24 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>Transfers 104-15 Queens Boulevard (Credit - Google) Natanielle S. Elishaev, Gavriel Soolaev, and Ronit Elishaev through the entity Queens Blvd 104 LLC as borrower signed a initial loan with lender ConnectOne Bank through the entity Connectone Bank valued at $12.8 million for the retail strip center complex (K1) at 104-15 Queens Boulevard in Forest Hills, Queens. The deal closed on May 19, 2026 and was recorded on May 27, 2026. The property has 23,780 square feet of built space and 115,804 square feet of additional air rights for a total buildable of 139,777 square feet according to a PincusCo analysis of city data. The loan price per built square foot is $536 and the price per buildable square foot is $91 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) The owners bought the property on August 28, 2025, for $25.9 million. The signatory for Natanielle S. Elishaev , Gavriel Soolaev , and Ronit Elishaev was Natanielle S. Elishaev, Gavriel Soolaev, and Ronit Elishaev. Prior sales, articles and revenue The 23,780-square-foot property generated revenue of</t>
+          <t xml:space="preserve">Transfers 35 West 14th Street (Credit - Cyclomedia) Hiwin Group USA through the entity Hw W 14th St LLC as borrower signed a new construction loan with lender Cathay Bank through the entity Cathay Bank valued at $40 million for the development building (V1) at 31 West 14th Street, also known as 35 West 14th Street, in Flatiron District, Manhattan. Hiwin Group USA by Harry Song filed plans, M01096333, for a 55-unit, 54,707 square-foot residential (R-2) building on August 22, 2024 that were permitted November 21, 2025. The loan closed on April 27, 2026 and was recorded on May 28, 2026. The prior lender was Cathay Bank which held debt that had an original loan amount of $8 million. The loan price per planned zoning square foot is $731 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) The owner bought the property on October 12, 2020, for $5.4 million. The signatory for Hiwin Group USA was Heli Song . The signatory for Cathay Bank was Steven Chen . The property The development building in Flatiron District has 7,368 square feet of built space and 45,908 </t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Eun Rae Jo pays $16.3M to Revere Capital for mixed-use in Flatiron District</t>
+          <t>Yossel Lichtman pays $25.6M to Pearl Realty Management for likely dev site in Greenpoint</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>https://www.pincusco.com/eun-rae-jo-pays-16-3m-to-revere-capital-for-in-flatiron-district/</t>
+          <t>https://www.pincusco.com/yossel-lichtman-pays-25-6m-to-pearl-realty-management-for-dev-site-in-greenpoint/</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Eun Rae Jo through the entity 16 Joe 18 LLC paid $16.3 million to Revere</t>
+          <t>Yossel Lichtman through the entity Seventy West Realty LLC paid $25.6 million to Pearl Realty</t>
         </is>
       </c>
       <c r="D3" t="inlineStr"/>
@@ -534,24 +534,24 @@
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>Transfers 16 East 18th Street (Credit - Cyclomedia) Eun Rae Jo through the entity 16 Joe 18 LLC paid $16.3 million to Revere Capital through the entity Nyc 18th Street LLC for the eight-unit property (DB) at 16 East 18th Street in Flatiron District, Manhattan. The expected use is cash flowing. The deal closed on April 17, 2026 and was recorded on May 27, 2026. The property has 20,258 square feet of built space according to a PincusCo analysis of city data. The sale price per built square foot is $804 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) The seller bought the property on July 1, 2022, for $3.7 million. The signatory for Revere Capital was Clark Briner . The signatory for Eun Rae Jo was Hyun Jun An . The contract date was February 6, 2026. Prior sales, articles and revenue Prior to this transaction, PincusCo has records that the buyer Eun Rae Jo purchased one property in one transaction for a total of $6.6 million and has no record it sold any properties over the past 24 months. The seller Revere Capital had not purchased any other propert</t>
+          <t xml:space="preserve">Transfers 54 Milton Street aka N_A West Street (Credit - Cyclomedia) Yossel Lichtman through the entity Seventy West Realty LLC paid $25.6 million to Pearl Realty Management through the entity 72 West LLC for the vacant lot at 54 Milton Street with an alternate address on West Street, in Brooklyn. The expected use is ground up development. The deal closed on May 20, 2026 and was recorded on May 28, 2026. The property has zero square feet of built space according to a PincusCo analysis of city data. The signatory for Pearl Realty Management was Jack Guttman. The signatory for Yossel Lichtman was Yossel Lichtman. The contract date was January 26, 2026. This property was previously part of the tax lot 1, 72 West Street, which is occupied by a Pearl Realty warehouse. Prior sales, articles and revenue Prior to this transaction, PincusCo has records that the buyer Yossel Lichtman purchased one property in one transaction for a total of $2.7 million and has no record it sold any properties over the past 24 months. The seller Pearl Realty Management purchased six properties in six transactions for a total of $140.9 million and sold 14 properties in eight transactions for a total of $392.1 </t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Rogers Equities pays $8.625M for portion of 85-unit dev site in Gowanus</t>
+          <t>United Overseas Bank takes over Vanke’s Bush Tower ground lease in $51.8M filing</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>https://www.pincusco.com/rogers-equities-pays-8-625m-for-portion-of-85-unit-dev-site-in-gowanus/</t>
+          <t>https://www.pincusco.com/united-overseas-bank-takes-over-vankes-garment-district-ground-lease-in-51-8m-filing/</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Abraham Waldman’s Rogers Equities paid $8.625 million for two buildings that form a portion of</t>
+          <t>United Overseas Bank through the entity United Overseas Bank Limited New York Agency took control</t>
         </is>
       </c>
       <c r="D4" t="inlineStr"/>
@@ -568,24 +568,24 @@
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>Transfers 416-418 4th Avenue (Credit - Cyclomedia) Abraham Waldman’s Rogers Equities paid $8.625 million for two buildings that form a portion of the five property footprint for an 85-unit project in Gowanus, Brooklyn. Rogers Equities already recorded the closed sales for 244A and 246 7th Street, for $6 million. In the first of the new closings, Rogers Equities through the entity 416 4th Ave Realty LLC paid $4.7 million to Nida Nagi Esa through the entity 248 Park Slope LLC for the six-unit mixed-use building (S5) at 416 4th Avenue in Gowanus, Brooklyn. The expected use is ground up development. The deal closed on May 12, 2026 and was recorded on May 27, 2026. The property has 7,280 square feet of built space and 3,676 square feet of additional air rights for a total buildable of 10,956 square feet according to a PincusCo analysis of city data. The sale price per built square foot is $641 and the price per buildable square foot is $426 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) The signatory for Nida Nagi Esa was Nida Nagi Esa. The signatory f</t>
+          <t xml:space="preserve">Chart_Frontpage Top Story Transfers 130 West 42nd Street (Credit - Cyclomedia) United Overseas Bank through the entity United Overseas Bank Limited New York Agency took control of the ground lease controlling the Bush Tower office building (O4) at 130 West 42nd Street in the Garment District, Manhattan, from the former lessee Vanke, through the entity 130w42 Trs LLC, in a transaction valued at $51.8 million. The expected use is hold for sale. The deal closed on May 11, 2026 and was recorded on May 28, 2026. The property has 217,855 square feet of built space according to a PincusCo analysis of city data. The sale price per built square foot is $237 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) The signatory for Vanke was Elliot J. Rishty . The signatory for United Overseas Bank was Eriberto de Guzman . This is not described as a deed-in-lieu of foreclosure but PincusCo is tracking it as one since it’s the borrower giving the property (the ground leasehold) back to the lender. United Overseas Bank provided a $120 million loan in 2018 to Vanke and </t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Rabsky pays $30M to Braha, ISJ, Jenel, Buhm Roe, Nakash for office in FiDi, Blackstone was foreclosing</t>
+          <t>Solomon Schwimmer signs $5.36M contract for Longwood building set for 88-unit conversion</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>https://www.pincusco.com/rabsky-pays-30m-to-braha-isj-jenel-buhm-roe-nakash-for-office-in-fidi-blackstone-was-foreclosing/</t>
+          <t>https://www.pincusco.com/solomon-schwimmer-signs-5-36m-contract-for-88-unit-dev-site-in-longwood/</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Rabsky Group through the entity 267 Broadway LLC paid $30 million to Ralph Braha, ISJ</t>
+          <t>The New York State Attorney General’s office approved a contract in which the nonprofit Boom!Community</t>
         </is>
       </c>
       <c r="D5" t="inlineStr"/>
@@ -602,7 +602,75 @@
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>Transfers 267 Broadway (Credit - Cyclomedia) Rabsky Group through the entity 267 Broadway LLC paid $30 million to Ralph Braha, ISJ Management, Jenel Management, Buhm Roe, and Nakash Holdings through the entity 267 Property Corp. for the office building (O5) at 267 Broadway in Financial District, Manhattan. Blackstone Group had filed a pre-foreclosure action over a $25 million loan, in 2024. The expected use is redevelopment. The deal closed on May 14, 2026 and was recorded on May 27, 2026. The property has 29,000 square feet of built space and 22,709 square feet of additional air rights for a total buildable of 51,730 square feet according to a PincusCo analysis of city data. The sale price per built square foot is $1,034 and the price per buildable square foot is $579 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) The signatory for Ralph Braha , ISJ Management , Jenel Management , Buhm Roe , and Nakash Holdings was Ralph Braha. The signatory for Rabsky Group was Abraham Kohn . The contract date was February 19, 2026. To finance the purchase, Rabs</t>
+          <t>Transfers 846 Brook Avenue aka 3144 Third Avenue (Credit - Cyclomedia) The New York State Attorney General’s office approved a contract in which the nonprofit Boom!Community Services will sell its 33,208-square-foot, five-story building at 846 Brook Avenue, with an alternate address of 3144 Third Avenue, in Longwood, the Bronx, to Solomon Schwimmer’s 3144 3rd Avenue LLC for $5.36 million. Schwimmer filed plans this week to convert the commercial building into 88 residential units. This Solomon Schwimmer is not the same Solomon Schwimmer who leads Twin Group Associates. The price per foot based on the current building size is $161 per foot. Solomon “Sol” Schwimmer of 3991 Saxon Ave LLC submitted a major alteration application for the conversion of the 33,208 square-foot commercial (COM) building at 846 Brook Avenue in Longwood, Bronx, to a residential building with 88 apartments. The filing states the building has 27,833 square feet of zoning square feet. The plan was filed with the New York City Department of Buildings on May 25, 2026 under job number X01406972. The project is described in the filing as: application filed herewith to convert an existing five-story community facilit</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>FBE Limited signs $27.5M refi with Argentic for 60-unit rental in Crown Heights</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>https://www.pincusco.com/fbe-limited-signs-27-5m-refi-with-argentic-for-60-unit-rental-in-crown-heights/</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>FBE Limited through the entity Ebf Washington Owner LLC as borrower signed a refi loan</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr"/>
+      <c r="E6" t="inlineStr"/>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>PincusCo</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>PincusCo - Home</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Transfers 781 Washington Avenue (Credit - Cyclomedia) FBE Limited through the entity Ebf Washington Owner LLC as borrower signed a refi loan with lender Argentic Investment Management through the entity Argentic Real Estate Finance 2 LLC valued at $27.5 million for the 60-unit residential elevator building (D5) at 781 Washington Avenue in Crown Heights, Brooklyn. The deal closed on May 5, 2026 and was recorded on May 27, 2026. The prior lender was Webster Bank which held debt that had an original loan amount of $23.7 million.The property has 47,764 square feet of built space and 18,321 square feet of additional air rights for a total buildable of 66,024 square feet according to a PincusCo analysis of city data. The loan price per built square foot is $575 and the price per buildable square foot is $416 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) The owner bought the property on November 30, 2022, for $30.5 million. The signatory for FBE Limited was Yehoshua Leib Fruchthandler . The signatory for Argentic Investment Management was Ryan Supple . </t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Alchemy Properties pays $58.5M for conversion site in Tribeca</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>https://www.pincusco.com/alchemy-properties-pays-58-5m-for-conversion-site-in-tribeca/</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Alchemy Properties through the entity North Moore Property Owner LLC paid $58.5 million to Calicchio</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr"/>
+      <c r="E7" t="inlineStr"/>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>PincusCo</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>PincusCo - Home</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>Transfers 56 North Moore Street axonometric diagram (Credit - Eran Chen architect via DOB) Alchemy Properties through the entity North Moore Property Owner LLC paid $58.5 million to Calicchio family through the entity A John LLC for the industrial building (G1) at 56 North Moore Street in Tribeca, Manhattan. The expected use is redevelopment to residential condominiums, according to the Commercial Observer. There is a major alteration project, M01367190, for a nine-unit, 53,196 square-foot residential (R-2) building submitted by Andrew Kellner with plans filed March 27, 2026 and it has not been permitted yet. The sale closed on May 5, 2026 and was recorded on May 27, 2026. The property has 41,067 square feet of built space and 11,753 square feet of additional air rights for a total buildable of 52,801 square feet according to a PincusCo analysis of city data. The sale price per built square foot is $1,424 and the price per buildable square foot is $1,107 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) The signatory for the Calicchio family was John</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto update queens news 2026-05-30T14:01:56Z
</commit_message>
<xml_diff>
--- a/data/output/queens_dev_news.xlsx
+++ b/data/output/queens_dev_news.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H7"/>
+  <dimension ref="A1:H1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -467,210 +467,6 @@
       <c r="H1" s="1" t="inlineStr">
         <is>
           <t>content_preview</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>Hiwin Group signs $40M construction loan with Cathay for 55-unit condo in Flatiron District</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>https://www.pincusco.com/hiwin-group-signs-40m-construction-loan-with-cathay-for-development-in-flatiron-district/</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>Hiwin Group USA through the entity Hw W 14th St LLC as borrower signed a</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr"/>
-      <c r="E2" t="inlineStr"/>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t>PincusCo</t>
-        </is>
-      </c>
-      <c r="G2" t="inlineStr">
-        <is>
-          <t>PincusCo - Home</t>
-        </is>
-      </c>
-      <c r="H2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Transfers 35 West 14th Street (Credit - Cyclomedia) Hiwin Group USA through the entity Hw W 14th St LLC as borrower signed a new construction loan with lender Cathay Bank through the entity Cathay Bank valued at $40 million for the development building (V1) at 31 West 14th Street, also known as 35 West 14th Street, in Flatiron District, Manhattan. Hiwin Group USA by Harry Song filed plans, M01096333, for a 55-unit, 54,707 square-foot residential (R-2) building on August 22, 2024 that were permitted November 21, 2025. The loan closed on April 27, 2026 and was recorded on May 28, 2026. The prior lender was Cathay Bank which held debt that had an original loan amount of $8 million. The loan price per planned zoning square foot is $731 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) The owner bought the property on October 12, 2020, for $5.4 million. The signatory for Hiwin Group USA was Heli Song . The signatory for Cathay Bank was Steven Chen . The property The development building in Flatiron District has 7,368 square feet of built space and 45,908 </t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>Yossel Lichtman pays $25.6M to Pearl Realty Management for likely dev site in Greenpoint</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>https://www.pincusco.com/yossel-lichtman-pays-25-6m-to-pearl-realty-management-for-dev-site-in-greenpoint/</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>Yossel Lichtman through the entity Seventy West Realty LLC paid $25.6 million to Pearl Realty</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr"/>
-      <c r="E3" t="inlineStr"/>
-      <c r="F3" t="inlineStr">
-        <is>
-          <t>PincusCo</t>
-        </is>
-      </c>
-      <c r="G3" t="inlineStr">
-        <is>
-          <t>PincusCo - Home</t>
-        </is>
-      </c>
-      <c r="H3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Transfers 54 Milton Street aka N_A West Street (Credit - Cyclomedia) Yossel Lichtman through the entity Seventy West Realty LLC paid $25.6 million to Pearl Realty Management through the entity 72 West LLC for the vacant lot at 54 Milton Street with an alternate address on West Street, in Brooklyn. The expected use is ground up development. The deal closed on May 20, 2026 and was recorded on May 28, 2026. The property has zero square feet of built space according to a PincusCo analysis of city data. The signatory for Pearl Realty Management was Jack Guttman. The signatory for Yossel Lichtman was Yossel Lichtman. The contract date was January 26, 2026. This property was previously part of the tax lot 1, 72 West Street, which is occupied by a Pearl Realty warehouse. Prior sales, articles and revenue Prior to this transaction, PincusCo has records that the buyer Yossel Lichtman purchased one property in one transaction for a total of $2.7 million and has no record it sold any properties over the past 24 months. The seller Pearl Realty Management purchased six properties in six transactions for a total of $140.9 million and sold 14 properties in eight transactions for a total of $392.1 </t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>United Overseas Bank takes over Vanke’s Bush Tower ground lease in $51.8M filing</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>https://www.pincusco.com/united-overseas-bank-takes-over-vankes-garment-district-ground-lease-in-51-8m-filing/</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>United Overseas Bank through the entity United Overseas Bank Limited New York Agency took control</t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr"/>
-      <c r="E4" t="inlineStr"/>
-      <c r="F4" t="inlineStr">
-        <is>
-          <t>PincusCo</t>
-        </is>
-      </c>
-      <c r="G4" t="inlineStr">
-        <is>
-          <t>PincusCo - Home</t>
-        </is>
-      </c>
-      <c r="H4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Chart_Frontpage Top Story Transfers 130 West 42nd Street (Credit - Cyclomedia) United Overseas Bank through the entity United Overseas Bank Limited New York Agency took control of the ground lease controlling the Bush Tower office building (O4) at 130 West 42nd Street in the Garment District, Manhattan, from the former lessee Vanke, through the entity 130w42 Trs LLC, in a transaction valued at $51.8 million. The expected use is hold for sale. The deal closed on May 11, 2026 and was recorded on May 28, 2026. The property has 217,855 square feet of built space according to a PincusCo analysis of city data. The sale price per built square foot is $237 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) The signatory for Vanke was Elliot J. Rishty . The signatory for United Overseas Bank was Eriberto de Guzman . This is not described as a deed-in-lieu of foreclosure but PincusCo is tracking it as one since it’s the borrower giving the property (the ground leasehold) back to the lender. United Overseas Bank provided a $120 million loan in 2018 to Vanke and </t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>Solomon Schwimmer signs $5.36M contract for Longwood building set for 88-unit conversion</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>https://www.pincusco.com/solomon-schwimmer-signs-5-36m-contract-for-88-unit-dev-site-in-longwood/</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>The New York State Attorney General’s office approved a contract in which the nonprofit Boom!Community</t>
-        </is>
-      </c>
-      <c r="D5" t="inlineStr"/>
-      <c r="E5" t="inlineStr"/>
-      <c r="F5" t="inlineStr">
-        <is>
-          <t>PincusCo</t>
-        </is>
-      </c>
-      <c r="G5" t="inlineStr">
-        <is>
-          <t>PincusCo - Home</t>
-        </is>
-      </c>
-      <c r="H5" t="inlineStr">
-        <is>
-          <t>Transfers 846 Brook Avenue aka 3144 Third Avenue (Credit - Cyclomedia) The New York State Attorney General’s office approved a contract in which the nonprofit Boom!Community Services will sell its 33,208-square-foot, five-story building at 846 Brook Avenue, with an alternate address of 3144 Third Avenue, in Longwood, the Bronx, to Solomon Schwimmer’s 3144 3rd Avenue LLC for $5.36 million. Schwimmer filed plans this week to convert the commercial building into 88 residential units. This Solomon Schwimmer is not the same Solomon Schwimmer who leads Twin Group Associates. The price per foot based on the current building size is $161 per foot. Solomon “Sol” Schwimmer of 3991 Saxon Ave LLC submitted a major alteration application for the conversion of the 33,208 square-foot commercial (COM) building at 846 Brook Avenue in Longwood, Bronx, to a residential building with 88 apartments. The filing states the building has 27,833 square feet of zoning square feet. The plan was filed with the New York City Department of Buildings on May 25, 2026 under job number X01406972. The project is described in the filing as: application filed herewith to convert an existing five-story community facilit</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>FBE Limited signs $27.5M refi with Argentic for 60-unit rental in Crown Heights</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>https://www.pincusco.com/fbe-limited-signs-27-5m-refi-with-argentic-for-60-unit-rental-in-crown-heights/</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>FBE Limited through the entity Ebf Washington Owner LLC as borrower signed a refi loan</t>
-        </is>
-      </c>
-      <c r="D6" t="inlineStr"/>
-      <c r="E6" t="inlineStr"/>
-      <c r="F6" t="inlineStr">
-        <is>
-          <t>PincusCo</t>
-        </is>
-      </c>
-      <c r="G6" t="inlineStr">
-        <is>
-          <t>PincusCo - Home</t>
-        </is>
-      </c>
-      <c r="H6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Transfers 781 Washington Avenue (Credit - Cyclomedia) FBE Limited through the entity Ebf Washington Owner LLC as borrower signed a refi loan with lender Argentic Investment Management through the entity Argentic Real Estate Finance 2 LLC valued at $27.5 million for the 60-unit residential elevator building (D5) at 781 Washington Avenue in Crown Heights, Brooklyn. The deal closed on May 5, 2026 and was recorded on May 27, 2026. The prior lender was Webster Bank which held debt that had an original loan amount of $23.7 million.The property has 47,764 square feet of built space and 18,321 square feet of additional air rights for a total buildable of 66,024 square feet according to a PincusCo analysis of city data. The loan price per built square foot is $575 and the price per buildable square foot is $416 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) The owner bought the property on November 30, 2022, for $30.5 million. The signatory for FBE Limited was Yehoshua Leib Fruchthandler . The signatory for Argentic Investment Management was Ryan Supple . </t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>Alchemy Properties pays $58.5M for conversion site in Tribeca</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>https://www.pincusco.com/alchemy-properties-pays-58-5m-for-conversion-site-in-tribeca/</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>Alchemy Properties through the entity North Moore Property Owner LLC paid $58.5 million to Calicchio</t>
-        </is>
-      </c>
-      <c r="D7" t="inlineStr"/>
-      <c r="E7" t="inlineStr"/>
-      <c r="F7" t="inlineStr">
-        <is>
-          <t>PincusCo</t>
-        </is>
-      </c>
-      <c r="G7" t="inlineStr">
-        <is>
-          <t>PincusCo - Home</t>
-        </is>
-      </c>
-      <c r="H7" t="inlineStr">
-        <is>
-          <t>Transfers 56 North Moore Street axonometric diagram (Credit - Eran Chen architect via DOB) Alchemy Properties through the entity North Moore Property Owner LLC paid $58.5 million to Calicchio family through the entity A John LLC for the industrial building (G1) at 56 North Moore Street in Tribeca, Manhattan. The expected use is redevelopment to residential condominiums, according to the Commercial Observer. There is a major alteration project, M01367190, for a nine-unit, 53,196 square-foot residential (R-2) building submitted by Andrew Kellner with plans filed March 27, 2026 and it has not been permitted yet. The sale closed on May 5, 2026 and was recorded on May 27, 2026. The property has 41,067 square feet of built space and 11,753 square feet of additional air rights for a total buildable of 52,801 square feet according to a PincusCo analysis of city data. The sale price per built square foot is $1,424 and the price per buildable square foot is $1,107 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) The signatory for the Calicchio family was John</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto update queens news 2026-06-01T18:15:38Z
</commit_message>
<xml_diff>
--- a/data/output/queens_dev_news.xlsx
+++ b/data/output/queens_dev_news.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H1"/>
+  <dimension ref="A1:H10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -470,6 +470,312 @@
         </is>
       </c>
     </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Heng Ken Hom pays $4M to Langsam Property for 68-unit walkup in Concourse</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>https://www.pincusco.com/heng-ken-hom-pays-4m-to-langsam-property-for-68-unit-walkup-in-concourse/</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Heng Ken Hom through the entity 1265 Housing LLC paid $4 million to Langsam Property</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr"/>
+      <c r="E2" t="inlineStr"/>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>PincusCo</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>PincusCo - Home</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>Transfers 1265 Walton Avenue (Credit - Cyclomedia) Heng Ken Hom through the entity 1265 Housing LLC paid $4 million to Langsam Property Services through the entity 1265 Realty Associates LLC for the 68-unit residential walkup building (C1) at 1265 Walton Avenue in Concourse, Bronx. The expected use is cash flowing. The deal closed on May 12, 2026 and was recorded on May 28, 2026. The property has 71,850 square feet of built space and 35,184 square feet of additional air rights for a total buildable of 106,975 square feet according to a PincusCo analysis of city data. The sale price per built square foot is $54 and the price per buildable square foot is $36 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) The signatory for Langsam Property Services was Mark Engel . The signatory for Heng Ken Hom was Heng Ken Hom. The contract date was January 23, 2026. Prior sales, articles and revenue Prior to this transaction, PincusCo has no record that the buyer Heng Ken Hom had purchased any other properties and has no record it sold any properties over the past</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Platinum Realty Associates pays $3.6M to Getty Realty for retail in Cypress Hills</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>https://www.pincusco.com/platinum-realty-associates-pays-3-6m-to-getty-realty-for-retail-in-cypress-hills/</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Platinum Realty Associates through the entity 115-20 Jam LLC paid $3.6 million to Getty Realty</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr"/>
+      <c r="E3" t="inlineStr"/>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>PincusCo</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>PincusCo - Home</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>Transfers 3513 Atlantic Avenue (Credit - Cyclomedia) Platinum Realty Associates through the entity 115-20 Jam LLC paid $3.6 million to Getty Realty Corp. through the entity Leemilt’S Petroleum, Inc. for the retail building (K1) at 3513 Atlantic Avenue in Cypress Hills, Brooklyn. The expected use is cash flowing. The deal closed on May 11, 2026 and was recorded on May 28, 2026. The property has 6,816 square feet of built space and 21,386 square feet of additional air rights for a total buildable of 28,140 square feet according to a PincusCo analysis of city data. The sale price per built square foot is $528 and the price per buildable square foot is $127 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) The signatory for Getty Realty Corp. was Phoebe Slater. The signatory for Platinum Realty Associates was David Koptiev . The contract date was March 13, 2026. Prior sales, articles and revenue Prior to this transaction, PincusCo has records that the buyer Platinum Realty Associates purchased 18 properties in 11 transactions for a total of $69.5 million</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Berry, Blimi Perlstein pay $4.5M for dev site in Borough Park</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>https://www.pincusco.com/berry-blimi-perlstein-pays-4-5m-for-dev-site-in-borough-park/</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Berry Perlstein and Blimi Perlstein through the entity 1257 Holdings LLC paid $4.5 million to</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr"/>
+      <c r="E4" t="inlineStr"/>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>PincusCo</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>PincusCo - Home</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>Transfers 1243 57th Street (Credit - Cyclomedia) Berry Perlstein and Blimi Perlstein through the entity 1257 Holdings LLC paid $4.5 million to the entity 1233-57 St. LLC for the development parcels (V0) at 1243 57th Street, 1239 57th Street and 1235 57th Street in Borough Park, Brooklyn. The expected use is ground up development. The deal closed on May 13, 2026 and was recorded on May 28, 2026. The three properties have zero square feet of built space and 12,019 square feet of additional air rights for a total buildable of 12,019 square feet according to a PincusCo analysis of city data. The sale price per buildable square foot is $374 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) The signatories for the sellers were Ellis Mirsky, Lawrence Raxenberg, Philip Rosen, and Nunziata Mazzei. The signatory for Berry Perlstein and Blimi Perlstein was Berry Perlstein. The contract date was February 5, 2025. To finance the purchase and development, Berry Perlstein and Blimi Perlstein through the entity 1257 Holdings LLC as borrower signed a new construction</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Rockrose signs $69.6M refi with JLL for 148-unit rental in West Village</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>https://www.pincusco.com/rockrose-signs-69-6m-refi-with-jll-for-148-unit-rental-in-west-village/</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Rockrose Development through the entity 100 Jane Street L.P. as borrower signed a refi loan</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr"/>
+      <c r="E5" t="inlineStr"/>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>PincusCo</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>PincusCo - Home</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>Transfers 100 Jane Street (Credit - Cyclomedia) Rockrose Development through the entity 100 Jane Street L.P. as borrower signed a refi loan with lender JLL through the entity Jll Real Estate Capital, LLC valued at $69.6 million for the 148-unit residential elevator building (D3) at 100 Jane Street in West Village, Manhattan. The deal closed on May 20, 2026 and was recorded on May 28, 2026. The prior lender was Wells Fargo which held debt that had an original loan amount of $65 million. The property has 123,646 square feet of built space according to a PincusCo analysis of city data. The loan price per built square foot is $562 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) The signatory for Rockrose Development was Richard A. Brancato . The signatory for JLL was Raymond M. Owono . Prior sales, articles and revenue The owners according to the Department of Housing Preservation and Development includes Joseph Flanagan, head officer and Alyssa Brennan, officer. The business entities are Rockrose Development LLC and 100 Jane Street L.P. The 123,646-sq</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Yili Teng pays $4.7M to owner-occupier for industrial in Greenwood Heights</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>https://www.pincusco.com/yili-teng-pays-4-7m-to-scutum-north-america-for-industrial-in-greenwood-heights/</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Yili Teng through the entity 703 3rd Ave Bk LLC paid $4.7 million to security</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr"/>
+      <c r="E6" t="inlineStr"/>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>PincusCo</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>PincusCo - Home</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>Transfers 703 3rd Avenue (Credit - Cyclomedia) Yili Teng through the entity 703 3rd Ave Bk LLC paid $4.7 million to security systems installer Scutum North America through the entity 703 3rd Ave LLC for the industrial building (G2) at 703 3rd Avenue in Greenwood Heights, Brooklyn. Scutum North America is a long-time owner-occupier of the building. The deal closed on April 30, 2026 and was recorded on May 28, 2026. The property has 9,680 square feet of built space according to a PincusCo analysis of city data. The sale price per built square foot is $485 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) The seller bought the property on January 21, 2016, for $3.4 million. The signatory for Scutum North America was Michael Vitarelli . The signatory for Yili Teng was Yili Teng. The contract date was February 13, 2016. Prior sales, articles and revenue Prior to this transaction, PincusCo has no record that the buyer Yili Teng had purchased any other properties and has no record it sold any properties over the past 24 months. The seller Scutum North Ameri</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Luis Camargo pays $4.8M for 10-unit rental in Melrose</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>https://www.pincusco.com/luis-camargo-pays-4-8m-for-10-unit-rental-in-melrose/</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Luis Camargo through the entity Hs 706 Corporate Avenue, Inc. paid $4.8 million to Mario</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr"/>
+      <c r="E7" t="inlineStr"/>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>PincusCo</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>PincusCo - Home</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Transfers 706 Courtlandt Avenue (Credit - Cyclomedia) Luis Camargo through the entity Hs 706 Corporate Avenue, Inc. paid $4.8 million to Mario Jacovino through the entity 706 Courtlandt Avenue LLC for the 10-unit residential elevator building (D7) at 706 Courtlandt Avenue in Melrose, Bronx. The expected use is cash flowing. The deal closed on May 14, 2026 and was recorded on May 28, 2026. The property has 17,860 square feet of built space according to a PincusCo analysis of city data. The sale price per built square foot is $268 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) The seller bought the property on August 15, 2014, for $425,000. The signatory for Mario Jacovino was Mario Jacovino. The signatory for Luis Camargo was Luis Fernando Camargo . The contract date was July 17, 2024. Prior sales, articles and revenue Prior to this transaction, PincusCo has no record that the buyer Luis Camargo had purchased any other properties and has no record it sold any properties over the past 24 months. The seller Mario Jacovino had not purchased any other </t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Jade Century Properties pays $31M for mixed-use in Astoria</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>https://www.pincusco.com/jade-century-properties-pays-31m-for-mixed-use-in-astoria/</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Jade Century Properties through the entity 47 Northern Blvd LLC paid $31 million to Mi</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr"/>
+      <c r="E8" t="inlineStr"/>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>PincusCo</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>PincusCo - Home</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>Top Story Transfers 47-15 34th Avenue (Credit - Cyclomedia) Jade Century Properties through the entity 47 Northern Blvd LLC paid $31 million to Mi Song Park and Ashley Cho through the entity Ashley Young LLC for the mixed-use building (K4) at 47-15 34th Avenue in Astoria, Queens. The expected use is ground up development. The deal closed on May 13, 2026 and was recorded on May 29, 2026. The property has 23,164 square feet of built space and 101,412 square feet of additional air rights for a total buildable of 124,692 square feet according to a PincusCo analysis of city data. The sale price per built square foot is $1,338 and the price per buildable square foot is $248 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) The seller bought the property on February 14, 2008, for $6.6 million. The signatory for Mi Song Park and Ashley Cho was Ashley Cho. The signatory for Jade Century Properties was Xiaorong Zhai . The contract date was December 17, 2025. Prior sales, articles and revenue Prior to this transaction, PincusCo has records that the buyer Jade C</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Kassin Sabbagh Realty affiliate pays $7M for 9-unit rental in Upper West Side</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>https://www.pincusco.com/kassin-sabbagh-realty-affiliate-pays-7m-for-9-unit-rental-in-upper-west-side/</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Kassin Sabbagh Realty through the entity 323 West 80th Street LLC paid $7 million to</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr"/>
+      <c r="E9" t="inlineStr"/>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>PincusCo</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>PincusCo - Home</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>Transfers 323 West 80th Street (Credit - Cyclomedia) Kassin Sabbagh Realty through the entity 323 West 80th Street LLC paid $7 million to William F. DeSeta through the entity 80th Street Realty LLC for the nine-unit residential elevator building (D3) at 323 West 80th Street in Upper West Side, Manhattan. The expected use is cash flowing. The deal closed on May 14, 2026 and was recorded on May 29, 2026. The property has 9,768 square feet of built space and 9,730 square feet of additional air rights for a total buildable of 19,500 square feet according to a PincusCo analysis of city data. The sale price per built square foot is $716 and the price per buildable square foot is $358 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) The signatory for William F. DeSeta was Jonathan Helfer . The signatory for Kassin Sabbagh Realty was Abraham J. Kassin . The contract date was May 2, 2026. Prior sales, articles and revenue Prior to this transaction, PincusCo has records that the buyer Kassin Sabbagh Realty purchased properties in four transactions for a total</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Joseph Ienco pays $14.7M to long-time restaurateur for 8-unit mixed-use in West Village</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>https://www.pincusco.com/joseph-ienco-pays-14-7m-to-long-time-restaurateur-for-8-unit-mixed-use-in-west-village/</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Joseph Ienco through the entity Abington Village LLC paid $14.7 million to Alain Laurent through</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr"/>
+      <c r="E10" t="inlineStr"/>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>PincusCo</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>PincusCo - Home</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>Transfers 605 Hudson Street (Credit - Cyclomedia) Joseph Ienco through the entity Abington Village LLC paid $14.7 million to Alain Laurent through the entity 605 Hudson Ltd. for the eight-unit residential walkup building (C7) at 605 Hudson Street, home to the French bistro La Ripaille for 46 years, in the West Village, Manhattan. The expected use is cash flowing. The deal closed on May 8, 2026 and was recorded on May 29, 2026. The property has 9,915 square feet of built space according to a PincusCo analysis of city data. The sale price per built square foot is $1,483 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) The signatory for Alain Laurent was Alain Laurent. The signatory for Joseph Ienco was Joseph Ienco. The contract date was October 6, 2025. Alain Laurent and Patrick Laurent opened La Ripaille in 1980, which announced it would close in 2024, but did not close until this year. The New York Times reviewed it in 1983, saying it was, “opened three years ago by Patrick and Alain Laurent, and their wives, Theresa and Nelly, who are in charge of</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
auto update queens news 2026-06-02T16:53:45Z
</commit_message>
<xml_diff>
--- a/data/output/queens_dev_news.xlsx
+++ b/data/output/queens_dev_news.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H10"/>
+  <dimension ref="A1:H1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -467,312 +467,6 @@
       <c r="H1" s="1" t="inlineStr">
         <is>
           <t>content_preview</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>Heng Ken Hom pays $4M to Langsam Property for 68-unit walkup in Concourse</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>https://www.pincusco.com/heng-ken-hom-pays-4m-to-langsam-property-for-68-unit-walkup-in-concourse/</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>Heng Ken Hom through the entity 1265 Housing LLC paid $4 million to Langsam Property</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr"/>
-      <c r="E2" t="inlineStr"/>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t>PincusCo</t>
-        </is>
-      </c>
-      <c r="G2" t="inlineStr">
-        <is>
-          <t>PincusCo - Home</t>
-        </is>
-      </c>
-      <c r="H2" t="inlineStr">
-        <is>
-          <t>Transfers 1265 Walton Avenue (Credit - Cyclomedia) Heng Ken Hom through the entity 1265 Housing LLC paid $4 million to Langsam Property Services through the entity 1265 Realty Associates LLC for the 68-unit residential walkup building (C1) at 1265 Walton Avenue in Concourse, Bronx. The expected use is cash flowing. The deal closed on May 12, 2026 and was recorded on May 28, 2026. The property has 71,850 square feet of built space and 35,184 square feet of additional air rights for a total buildable of 106,975 square feet according to a PincusCo analysis of city data. The sale price per built square foot is $54 and the price per buildable square foot is $36 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) The signatory for Langsam Property Services was Mark Engel . The signatory for Heng Ken Hom was Heng Ken Hom. The contract date was January 23, 2026. Prior sales, articles and revenue Prior to this transaction, PincusCo has no record that the buyer Heng Ken Hom had purchased any other properties and has no record it sold any properties over the past</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>Platinum Realty Associates pays $3.6M to Getty Realty for retail in Cypress Hills</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>https://www.pincusco.com/platinum-realty-associates-pays-3-6m-to-getty-realty-for-retail-in-cypress-hills/</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>Platinum Realty Associates through the entity 115-20 Jam LLC paid $3.6 million to Getty Realty</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr"/>
-      <c r="E3" t="inlineStr"/>
-      <c r="F3" t="inlineStr">
-        <is>
-          <t>PincusCo</t>
-        </is>
-      </c>
-      <c r="G3" t="inlineStr">
-        <is>
-          <t>PincusCo - Home</t>
-        </is>
-      </c>
-      <c r="H3" t="inlineStr">
-        <is>
-          <t>Transfers 3513 Atlantic Avenue (Credit - Cyclomedia) Platinum Realty Associates through the entity 115-20 Jam LLC paid $3.6 million to Getty Realty Corp. through the entity Leemilt’S Petroleum, Inc. for the retail building (K1) at 3513 Atlantic Avenue in Cypress Hills, Brooklyn. The expected use is cash flowing. The deal closed on May 11, 2026 and was recorded on May 28, 2026. The property has 6,816 square feet of built space and 21,386 square feet of additional air rights for a total buildable of 28,140 square feet according to a PincusCo analysis of city data. The sale price per built square foot is $528 and the price per buildable square foot is $127 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) The signatory for Getty Realty Corp. was Phoebe Slater. The signatory for Platinum Realty Associates was David Koptiev . The contract date was March 13, 2026. Prior sales, articles and revenue Prior to this transaction, PincusCo has records that the buyer Platinum Realty Associates purchased 18 properties in 11 transactions for a total of $69.5 million</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>Berry, Blimi Perlstein pay $4.5M for dev site in Borough Park</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>https://www.pincusco.com/berry-blimi-perlstein-pays-4-5m-for-dev-site-in-borough-park/</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>Berry Perlstein and Blimi Perlstein through the entity 1257 Holdings LLC paid $4.5 million to</t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr"/>
-      <c r="E4" t="inlineStr"/>
-      <c r="F4" t="inlineStr">
-        <is>
-          <t>PincusCo</t>
-        </is>
-      </c>
-      <c r="G4" t="inlineStr">
-        <is>
-          <t>PincusCo - Home</t>
-        </is>
-      </c>
-      <c r="H4" t="inlineStr">
-        <is>
-          <t>Transfers 1243 57th Street (Credit - Cyclomedia) Berry Perlstein and Blimi Perlstein through the entity 1257 Holdings LLC paid $4.5 million to the entity 1233-57 St. LLC for the development parcels (V0) at 1243 57th Street, 1239 57th Street and 1235 57th Street in Borough Park, Brooklyn. The expected use is ground up development. The deal closed on May 13, 2026 and was recorded on May 28, 2026. The three properties have zero square feet of built space and 12,019 square feet of additional air rights for a total buildable of 12,019 square feet according to a PincusCo analysis of city data. The sale price per buildable square foot is $374 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) The signatories for the sellers were Ellis Mirsky, Lawrence Raxenberg, Philip Rosen, and Nunziata Mazzei. The signatory for Berry Perlstein and Blimi Perlstein was Berry Perlstein. The contract date was February 5, 2025. To finance the purchase and development, Berry Perlstein and Blimi Perlstein through the entity 1257 Holdings LLC as borrower signed a new construction</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>Rockrose signs $69.6M refi with JLL for 148-unit rental in West Village</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>https://www.pincusco.com/rockrose-signs-69-6m-refi-with-jll-for-148-unit-rental-in-west-village/</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>Rockrose Development through the entity 100 Jane Street L.P. as borrower signed a refi loan</t>
-        </is>
-      </c>
-      <c r="D5" t="inlineStr"/>
-      <c r="E5" t="inlineStr"/>
-      <c r="F5" t="inlineStr">
-        <is>
-          <t>PincusCo</t>
-        </is>
-      </c>
-      <c r="G5" t="inlineStr">
-        <is>
-          <t>PincusCo - Home</t>
-        </is>
-      </c>
-      <c r="H5" t="inlineStr">
-        <is>
-          <t>Transfers 100 Jane Street (Credit - Cyclomedia) Rockrose Development through the entity 100 Jane Street L.P. as borrower signed a refi loan with lender JLL through the entity Jll Real Estate Capital, LLC valued at $69.6 million for the 148-unit residential elevator building (D3) at 100 Jane Street in West Village, Manhattan. The deal closed on May 20, 2026 and was recorded on May 28, 2026. The prior lender was Wells Fargo which held debt that had an original loan amount of $65 million. The property has 123,646 square feet of built space according to a PincusCo analysis of city data. The loan price per built square foot is $562 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) The signatory for Rockrose Development was Richard A. Brancato . The signatory for JLL was Raymond M. Owono . Prior sales, articles and revenue The owners according to the Department of Housing Preservation and Development includes Joseph Flanagan, head officer and Alyssa Brennan, officer. The business entities are Rockrose Development LLC and 100 Jane Street L.P. The 123,646-sq</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>Yili Teng pays $4.7M to owner-occupier for industrial in Greenwood Heights</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>https://www.pincusco.com/yili-teng-pays-4-7m-to-scutum-north-america-for-industrial-in-greenwood-heights/</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>Yili Teng through the entity 703 3rd Ave Bk LLC paid $4.7 million to security</t>
-        </is>
-      </c>
-      <c r="D6" t="inlineStr"/>
-      <c r="E6" t="inlineStr"/>
-      <c r="F6" t="inlineStr">
-        <is>
-          <t>PincusCo</t>
-        </is>
-      </c>
-      <c r="G6" t="inlineStr">
-        <is>
-          <t>PincusCo - Home</t>
-        </is>
-      </c>
-      <c r="H6" t="inlineStr">
-        <is>
-          <t>Transfers 703 3rd Avenue (Credit - Cyclomedia) Yili Teng through the entity 703 3rd Ave Bk LLC paid $4.7 million to security systems installer Scutum North America through the entity 703 3rd Ave LLC for the industrial building (G2) at 703 3rd Avenue in Greenwood Heights, Brooklyn. Scutum North America is a long-time owner-occupier of the building. The deal closed on April 30, 2026 and was recorded on May 28, 2026. The property has 9,680 square feet of built space according to a PincusCo analysis of city data. The sale price per built square foot is $485 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) The seller bought the property on January 21, 2016, for $3.4 million. The signatory for Scutum North America was Michael Vitarelli . The signatory for Yili Teng was Yili Teng. The contract date was February 13, 2016. Prior sales, articles and revenue Prior to this transaction, PincusCo has no record that the buyer Yili Teng had purchased any other properties and has no record it sold any properties over the past 24 months. The seller Scutum North Ameri</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>Luis Camargo pays $4.8M for 10-unit rental in Melrose</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>https://www.pincusco.com/luis-camargo-pays-4-8m-for-10-unit-rental-in-melrose/</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>Luis Camargo through the entity Hs 706 Corporate Avenue, Inc. paid $4.8 million to Mario</t>
-        </is>
-      </c>
-      <c r="D7" t="inlineStr"/>
-      <c r="E7" t="inlineStr"/>
-      <c r="F7" t="inlineStr">
-        <is>
-          <t>PincusCo</t>
-        </is>
-      </c>
-      <c r="G7" t="inlineStr">
-        <is>
-          <t>PincusCo - Home</t>
-        </is>
-      </c>
-      <c r="H7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Transfers 706 Courtlandt Avenue (Credit - Cyclomedia) Luis Camargo through the entity Hs 706 Corporate Avenue, Inc. paid $4.8 million to Mario Jacovino through the entity 706 Courtlandt Avenue LLC for the 10-unit residential elevator building (D7) at 706 Courtlandt Avenue in Melrose, Bronx. The expected use is cash flowing. The deal closed on May 14, 2026 and was recorded on May 28, 2026. The property has 17,860 square feet of built space according to a PincusCo analysis of city data. The sale price per built square foot is $268 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) The seller bought the property on August 15, 2014, for $425,000. The signatory for Mario Jacovino was Mario Jacovino. The signatory for Luis Camargo was Luis Fernando Camargo . The contract date was July 17, 2024. Prior sales, articles and revenue Prior to this transaction, PincusCo has no record that the buyer Luis Camargo had purchased any other properties and has no record it sold any properties over the past 24 months. The seller Mario Jacovino had not purchased any other </t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>Jade Century Properties pays $31M for mixed-use in Astoria</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>https://www.pincusco.com/jade-century-properties-pays-31m-for-mixed-use-in-astoria/</t>
-        </is>
-      </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>Jade Century Properties through the entity 47 Northern Blvd LLC paid $31 million to Mi</t>
-        </is>
-      </c>
-      <c r="D8" t="inlineStr"/>
-      <c r="E8" t="inlineStr"/>
-      <c r="F8" t="inlineStr">
-        <is>
-          <t>PincusCo</t>
-        </is>
-      </c>
-      <c r="G8" t="inlineStr">
-        <is>
-          <t>PincusCo - Home</t>
-        </is>
-      </c>
-      <c r="H8" t="inlineStr">
-        <is>
-          <t>Top Story Transfers 47-15 34th Avenue (Credit - Cyclomedia) Jade Century Properties through the entity 47 Northern Blvd LLC paid $31 million to Mi Song Park and Ashley Cho through the entity Ashley Young LLC for the mixed-use building (K4) at 47-15 34th Avenue in Astoria, Queens. The expected use is ground up development. The deal closed on May 13, 2026 and was recorded on May 29, 2026. The property has 23,164 square feet of built space and 101,412 square feet of additional air rights for a total buildable of 124,692 square feet according to a PincusCo analysis of city data. The sale price per built square foot is $1,338 and the price per buildable square foot is $248 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) The seller bought the property on February 14, 2008, for $6.6 million. The signatory for Mi Song Park and Ashley Cho was Ashley Cho. The signatory for Jade Century Properties was Xiaorong Zhai . The contract date was December 17, 2025. Prior sales, articles and revenue Prior to this transaction, PincusCo has records that the buyer Jade C</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>Kassin Sabbagh Realty affiliate pays $7M for 9-unit rental in Upper West Side</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>https://www.pincusco.com/kassin-sabbagh-realty-affiliate-pays-7m-for-9-unit-rental-in-upper-west-side/</t>
-        </is>
-      </c>
-      <c r="C9" t="inlineStr">
-        <is>
-          <t>Kassin Sabbagh Realty through the entity 323 West 80th Street LLC paid $7 million to</t>
-        </is>
-      </c>
-      <c r="D9" t="inlineStr"/>
-      <c r="E9" t="inlineStr"/>
-      <c r="F9" t="inlineStr">
-        <is>
-          <t>PincusCo</t>
-        </is>
-      </c>
-      <c r="G9" t="inlineStr">
-        <is>
-          <t>PincusCo - Home</t>
-        </is>
-      </c>
-      <c r="H9" t="inlineStr">
-        <is>
-          <t>Transfers 323 West 80th Street (Credit - Cyclomedia) Kassin Sabbagh Realty through the entity 323 West 80th Street LLC paid $7 million to William F. DeSeta through the entity 80th Street Realty LLC for the nine-unit residential elevator building (D3) at 323 West 80th Street in Upper West Side, Manhattan. The expected use is cash flowing. The deal closed on May 14, 2026 and was recorded on May 29, 2026. The property has 9,768 square feet of built space and 9,730 square feet of additional air rights for a total buildable of 19,500 square feet according to a PincusCo analysis of city data. The sale price per built square foot is $716 and the price per buildable square foot is $358 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) The signatory for William F. DeSeta was Jonathan Helfer . The signatory for Kassin Sabbagh Realty was Abraham J. Kassin . The contract date was May 2, 2026. Prior sales, articles and revenue Prior to this transaction, PincusCo has records that the buyer Kassin Sabbagh Realty purchased properties in four transactions for a total</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>Joseph Ienco pays $14.7M to long-time restaurateur for 8-unit mixed-use in West Village</t>
-        </is>
-      </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>https://www.pincusco.com/joseph-ienco-pays-14-7m-to-long-time-restaurateur-for-8-unit-mixed-use-in-west-village/</t>
-        </is>
-      </c>
-      <c r="C10" t="inlineStr">
-        <is>
-          <t>Joseph Ienco through the entity Abington Village LLC paid $14.7 million to Alain Laurent through</t>
-        </is>
-      </c>
-      <c r="D10" t="inlineStr"/>
-      <c r="E10" t="inlineStr"/>
-      <c r="F10" t="inlineStr">
-        <is>
-          <t>PincusCo</t>
-        </is>
-      </c>
-      <c r="G10" t="inlineStr">
-        <is>
-          <t>PincusCo - Home</t>
-        </is>
-      </c>
-      <c r="H10" t="inlineStr">
-        <is>
-          <t>Transfers 605 Hudson Street (Credit - Cyclomedia) Joseph Ienco through the entity Abington Village LLC paid $14.7 million to Alain Laurent through the entity 605 Hudson Ltd. for the eight-unit residential walkup building (C7) at 605 Hudson Street, home to the French bistro La Ripaille for 46 years, in the West Village, Manhattan. The expected use is cash flowing. The deal closed on May 8, 2026 and was recorded on May 29, 2026. The property has 9,915 square feet of built space according to a PincusCo analysis of city data. The sale price per built square foot is $1,483 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) The signatory for Alain Laurent was Alain Laurent. The signatory for Joseph Ienco was Joseph Ienco. The contract date was October 6, 2025. Alain Laurent and Patrick Laurent opened La Ripaille in 1980, which announced it would close in 2024, but did not close until this year. The New York Times reviewed it in 1983, saying it was, “opened three years ago by Patrick and Alain Laurent, and their wives, Theresa and Nelly, who are in charge of</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto update queens news 2026-06-03T17:13:41Z
</commit_message>
<xml_diff>
--- a/data/output/queens_dev_news.xlsx
+++ b/data/output/queens_dev_news.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H1"/>
+  <dimension ref="A1:H8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -467,6 +467,244 @@
       <c r="H1" s="1" t="inlineStr">
         <is>
           <t>content_preview</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Samara NY pays $3.1M for mixed-use in Williamsburg</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>https://www.pincusco.com/samara-ny-pays-3-1m-for-mixed-use-in-williamsburg/</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Samara NY through the entity 857 Park Place LLC paid $3.1 million to Mieczyslaw Cielepak</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr"/>
+      <c r="E2" t="inlineStr"/>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>PincusCo</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>PincusCo - Home</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>Transfers 175 Richardson Street (Credit - Cyclomedia) Samara NY through the entity 857 Park Place LLC paid $3.1 million to Mieczyslaw Cielepak through the entity 175 Richardson Street LLC for the mixed-use building (S0) at 175 Richardson Street in Williamsburg, Brooklyn. The expected use is cash flowing. The deal closed on May 21, 2026 and was recorded on June 2, 2026. The property has 4,695 square feet of built space according to a PincusCo analysis of city data. The sale price per built square foot is $670 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) The seller bought the property on April 20, 2023, for $1.1 million. The signatory for Mieczyslaw Cielepak was Mieczyslaw Cielepak. The contract date was January 30, 2026. Prior sales, articles and revenue Prior to this transaction, PincusCo has no record that the buyer Samara NY had purchased any other properties and sold one property in one transaction for a total of $2.5 million over the past 24 months. The seller Mieczyslaw Cielepak had not purchased any other properties and had not sold any pr</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Brookfield, QIA sign $1.9B refi at 2 Manhattan West</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>https://www.pincusco.com/brookfield-qia-sign-1-9b-refi-at-2-manhattan-west/</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Brookfield Properties and the Qatar Investment Authority through the entity Bop Mw Retail Subsidiary LLC</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr"/>
+      <c r="E3" t="inlineStr"/>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>PincusCo</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>PincusCo - Home</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>Transfers 375 Ninth Avenue (Credit - Cyclomedia) Brookfield Properties and the Qatar Investment Authority through the entity Bop Mw Retail Subsidiary LLC as borrower signed a refi loan with lender Wells Fargo, Bank of America, Bank of Montreal, Citibank, Deutsche Bank, and Santander Bank valued at $1.9 billion for 2 Manhattan West in Penn Station, Manhattan. The deal closed on May 15, 2026 and was recorded on June 2, 2026. The five properties have 1,899,740 square feet of built space according to a PincusCo analysis of city data. The loan price per built square foot is $1,000 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) The signatory for Brookfield Properties and the Qatar Investment Authority was Justin Kollender . The signatory for Wells Fargo , Bank of America , Bank of Montreal , Citibank , Deutsche Bank , and Santander Bank was Jeffrey L. Cirillo , Steven Wasser , Michael S. Birajiclian , Ana Rosu Marmann , David Goodman , Brandon Atkins , Stefanos Arethas, and Anthony Marino. Crain’s New York reported on the refinancing May 12, 2026. Devel</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Jacob Elul files plans for 71 units in Cypress Hills</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>https://www.pincusco.com/jacob-elul-files-plans-for-71-units-in-cypress-hills/</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Jacob Elul submitted a new building construction project for a 71-unit, 57,415-square-foot residential (R-2) building</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr"/>
+      <c r="E4" t="inlineStr"/>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>PincusCo</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>PincusCo - Home</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>Development 138 New Jersey Avenue axonometric diagram (Credit - Stephen Conte architect via DOB) Jacob Elul submitted a new building construction project for a 71-unit, 57,415-square-foot residential (R-2) building at 138 New Jersey Avenue in Cypress Hills, Brooklyn. The plan was filed on June 1, 2026. It calls for the construction of a 100-foot-tall, ten-story building and was filed with the New York City Department of Buildings under job number B01373493. The project is described in the filing as: propose 10-story residential building as per plan. The applicant is the Registered Architect Stephen Conte of StudiosC Architecture. This 10-story residential building features 71 Class A apartments with eight units on floors 2 through 9 and six on the 10th floor. The ground level includes a 7-space parking garage, mail and package rooms, laundry facilities, and bike storage for 36 bicycles. Amenities include a 10th-floor fitness room and a rooftop terrace for residents. Supporting infrastructure such as mechanical, electrical, and elevator equipment rooms is located on the ground floor and roof levels. 138 New Jersey Avenue wdt_ID wdt_created_by wdt_created_at wdt_last_edited_by wdt_la</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Barone Management signs contract to buy Laurelton dev site, price not disclosed</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>https://www.pincusco.com/barone-management-signs-contract-to-buy-laurelton-dev-site-price-not-disclosed/</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Barone Management through the entity BMAD Springfield LLC signed a contract as buyer with Evan</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr"/>
+      <c r="E5" t="inlineStr"/>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>PincusCo</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>PincusCo - Home</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>Transfers 223-01 Merrick Boulevard (Credit - Cyclomedia) Barone Management through the entity BMAD Springfield LLC signed a contract as buyer with Evan Tannor through the entity Merrick Boulevard Acquisitions, LLC, as seller, for the industrial properties in Laurelton, Queens, including 223-15 Merrick Boulevard, 223-01 Merrick Boulevard. The expected use is ground up development. The price was not disclosed. The deal closed on April 1, 2026 and was recorded on June 2, 2026. The three properties have 1,155 square feet of built space and 51,416 square feet of additional air rights for a total buildable of 52,582 square feet according to a PincusCo analysis of city data. The signatory for Evan Tannor was Evan Tannor. The signatory for Barone Management was Scott Barone . The memorandum of contract says the closing date is July 27, 2027. Prior sales, articles and revenue Prior to this transaction, PincusCo has records that the buyer Barone Management purchased three properties in two transactions for a total of $19.8 million and sold two properties in one transaction for a total of $85 million over the past 24 months. The seller Evan Tannor had not purchased any other properties and ha</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Alon Ashourzadeh pays $3.4M for mixed-use in Carroll Gardens</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>https://www.pincusco.com/alon-ashourzadeh-pays-3-4m-for-mixed-use-in-carroll-gardens/</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Alon Ashourzadeh through the entity 445 Court LLC paid $3.4 million for the three-unit mixed-use</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr"/>
+      <c r="E6" t="inlineStr"/>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>PincusCo</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>PincusCo - Home</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>Transfers 445 Court Street (Credit - Cyclomedia) Alon Ashourzadeh through the entity 445 Court LLC paid $3.4 million for the three-unit mixed-use building (S3) at 445 Court Street in Carroll Gardens, Brooklyn. The expected use is renovation and cash flowing. The deal closed on May 4, 2026 and was recorded on June 2, 2026. The property has 3,936 square feet of built space and 1,152 square feet of additional air rights for a total buildable of 5,085 square feet according to a PincusCo analysis of city data. The sale price per built square foot is $851 and the price per buildable square foot is $659 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) The signatory for the estate of the late Ralph DiBenedetto was Ralph DiBenedetto Jr. . The signatory for Alon Ashourzadeh was Stephen Siminou . The contract date was August 27, 2025. Ralph DiBenedetto died. Alon Ashourzadeh signed a memorandum of contract of sale recorded in December 2025. DiBenedetto Jr. sold 423 Court Street to Alon Ashourzadeh in 2022. To finance the purchase and construction, Alon Ashourz</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Metro Loft, Quantum sign $169.5M construction loan for 337-unit resi conversion in Midtown East</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>https://www.pincusco.com/metro-loft-quantum-sign-169-5m-construction-loan-for-337-unit-resi-conversion-in-midtown-east/</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Metro Loft Management and Quantum Pacific Group through the entity 767 Third Property Owner LLC</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr"/>
+      <c r="E7" t="inlineStr"/>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>PincusCo</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>PincusCo - Home</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>Transfers 767 3rd Avenue (Credit - Cyclomedia) Metro Loft Management and Quantum Pacific Group through the entity 767 Third Property Owner LLC as borrower signed a rehab construction loan with lender Bank Hapoalim valued at $169.5 million for the conversion of the office building (O4) at 767 Third Avenue in Midtown East, Manhattan, to a mixed-used building with 337 units. On the lot, there is one active major alteration construction project, M01237433, for a 337-unit, 217,243 square-foot residential (R-2) building. The project was submitted by Metro Loft Management and filed by Robert Travis with plans filed July 30, 2025 and permitted April 6, 2026. The deal closed on May 19, 2026 and was recorded on June 2, 2026. The prior lender was Bank Hapoalim which held debt that had an original loan amount of $55 million.The property has 286,212 square feet of built space according to a PincusCo analysis of city data. The loan price per built square foot is $592 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) The owner bought the property on December 31, 20</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Anish Berry pays $7M to dentist Nitin Doshi for offices in Flushing, UWS</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>https://www.pincusco.com/anish-berry-pays-7m-to-nitin-doshi-for-office-in-flushing-uws/</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Anish Berry paid $7 million to dentist Nitin Doshi for an office building in Flushing,</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr"/>
+      <c r="E8" t="inlineStr"/>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>PincusCo</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>PincusCo - Home</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>Transfers 43-55 147th Street (Credit - Cyclomedia) Anish Berry paid $7 million to dentist Nitin Doshi for an office building in Flushing, Queens, and an office condominium unit in the Upper West Side of Manhattan in two transactions. In the first, Anish Berry through the entity 4355 Realty NY LLC paid $4 million to Nitin Doshi through the entity Flushing Medical Arts Building Inc. for the office building (O2) at 43-55 147th Street in Flushing, Queens. The deal closed on May 19, 2026 and was recorded on June 2, 2026. The property has 10,856 square feet of built space according to a PincusCo analysis of city data. The sale price per built square foot is $368 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) In the second, Anish Berry through the entity 130 Realty Ny LLC paid $3 million to Nitin Doshi through the entity West 79th Street Realty Associates LLC for the office condo at 130 West 79th Street in Upper West Side, Manhattan. The deal closed on May 19, 2026 and was recorded on June 2, 2026. The property has 5,326 square feet of built space accord</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto update queens news 2026-06-04T15:38:38Z
</commit_message>
<xml_diff>
--- a/data/output/queens_dev_news.xlsx
+++ b/data/output/queens_dev_news.xlsx
@@ -473,17 +473,17 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Samara NY pays $3.1M for mixed-use in Williamsburg</t>
+          <t>Spectra Construction signs $28M construction loan for 43-unit project in NoMad</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>https://www.pincusco.com/samara-ny-pays-3-1m-for-mixed-use-in-williamsburg/</t>
+          <t>https://www.pincusco.com/spectra-construction-signs-28m-construction-loan-for-43-unit-project-in-nomad/</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Samara NY through the entity 857 Park Place LLC paid $3.1 million to Mieczyslaw Cielepak</t>
+          <t>Spectra Construction and Development through the entity Ww Lexington, LLC as borrower signed a new</t>
         </is>
       </c>
       <c r="D2" t="inlineStr"/>
@@ -500,24 +500,24 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>Transfers 175 Richardson Street (Credit - Cyclomedia) Samara NY through the entity 857 Park Place LLC paid $3.1 million to Mieczyslaw Cielepak through the entity 175 Richardson Street LLC for the mixed-use building (S0) at 175 Richardson Street in Williamsburg, Brooklyn. The expected use is cash flowing. The deal closed on May 21, 2026 and was recorded on June 2, 2026. The property has 4,695 square feet of built space according to a PincusCo analysis of city data. The sale price per built square foot is $670 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) The seller bought the property on April 20, 2023, for $1.1 million. The signatory for Mieczyslaw Cielepak was Mieczyslaw Cielepak. The contract date was January 30, 2026. Prior sales, articles and revenue Prior to this transaction, PincusCo has no record that the buyer Samara NY had purchased any other properties and sold one property in one transaction for a total of $2.5 million over the past 24 months. The seller Mieczyslaw Cielepak had not purchased any other properties and had not sold any pr</t>
+          <t xml:space="preserve">Transfers 129 East 28th Street isometric diagram (Credit - Alexander Zhitnik architect via DOB) Spectra Construction and Development through the entity Ww Lexington, LLC as borrower signed a new construction loan with lender Castellan Capital through the entity 120 Lexington LLC valued at $28 million for three tax lots making up the 43-unit project at 129 East 28th Street in NoMad, Manhattan. On these lots, there is a new building project, M01230688, for a 43-unit, 38,405 square-foot residential (R-2) building submitted by Spectra Construction and Development and filed by Daniel Klaynberg with plans filed July 21, 2025 and it has not been permitted yet. The loan closed on April 30, 2026 and was recorded on June 2, 2026. The loan price per planned development square foot is $729 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) The signatory for Spectra Construction and Development was Daniel Klaynberg . ZD1 DOB Zoning Diagram </t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Brookfield, QIA sign $1.9B refi at 2 Manhattan West</t>
+          <t>Sackman Enterprises signs $10.69M refi with Chase for four walkups in Manhattan</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>https://www.pincusco.com/brookfield-qia-sign-1-9b-refi-at-2-manhattan-west/</t>
+          <t>https://www.pincusco.com/sackman-enterprises-signs-10-69m-refi-with-chase-for-four-walkup-in-manhattan/</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Brookfield Properties and the Qatar Investment Authority through the entity Bop Mw Retail Subsidiary LLC</t>
+          <t>Sackman Enterprises through the entity Marsac Realty, LLC as borrower signed a refi loan with</t>
         </is>
       </c>
       <c r="D3" t="inlineStr"/>
@@ -534,24 +534,24 @@
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>Transfers 375 Ninth Avenue (Credit - Cyclomedia) Brookfield Properties and the Qatar Investment Authority through the entity Bop Mw Retail Subsidiary LLC as borrower signed a refi loan with lender Wells Fargo, Bank of America, Bank of Montreal, Citibank, Deutsche Bank, and Santander Bank valued at $1.9 billion for 2 Manhattan West in Penn Station, Manhattan. The deal closed on May 15, 2026 and was recorded on June 2, 2026. The five properties have 1,899,740 square feet of built space according to a PincusCo analysis of city data. The loan price per built square foot is $1,000 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) The signatory for Brookfield Properties and the Qatar Investment Authority was Justin Kollender . The signatory for Wells Fargo , Bank of America , Bank of Montreal , Citibank , Deutsche Bank , and Santander Bank was Jeffrey L. Cirillo , Steven Wasser , Michael S. Birajiclian , Ana Rosu Marmann , David Goodman , Brandon Atkins , Stefanos Arethas, and Anthony Marino. Crain’s New York reported on the refinancing May 12, 2026. Devel</t>
+          <t>Transfers 203 West 84th Street (Credit - Cyclomedia) Sackman Enterprises through the entity Marsac Realty, LLC as borrower signed a refi loan with lender JPMorgan Chase valued at $10.69 million for four residential walkup properties with 35 residential units including the 10-unit residential walkup building (C7) at 203 West 84th Street in Upper West Side, Manhattan, eight-unit residential walkup building (C7) at 730 10th Avenue in Hell’s Kitchen, Manhattan, and nine-unit residential walkup building (C7) at 732 10th Avenue in Hell’s Kitchen, Manhattan. The deal closed on April 30, 2026 and was recorded on June 2, 2026. The prior lender was JPMorgan Chase which in 2015 provided debt that had an original loan amount of $10.69 million.The four properties have 25,091 square feet of built space and 11,657 square feet of additional air rights for a total buildable of 36,439 square feet according to a PincusCo analysis of city data. The loan price per built square foot is $426 and the price per buildable square foot is $293 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights h</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Jacob Elul files plans for 71 units in Cypress Hills</t>
+          <t>Aleksander Haxhari signs $11.1M construction loan for 53-unit project in Allerton</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>https://www.pincusco.com/jacob-elul-files-plans-for-71-units-in-cypress-hills/</t>
+          <t>https://www.pincusco.com/aleksander-haxhari-signs-11-1m-construction-loan-for-53-unit-project-in-allerton/</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Jacob Elul submitted a new building construction project for a 71-unit, 57,415-square-foot residential (R-2) building</t>
+          <t>Aleksander Haxhari through the entity BPE Realty LLC as borrower signed a construction loan with</t>
         </is>
       </c>
       <c r="D4" t="inlineStr"/>
@@ -568,24 +568,24 @@
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>Development 138 New Jersey Avenue axonometric diagram (Credit - Stephen Conte architect via DOB) Jacob Elul submitted a new building construction project for a 71-unit, 57,415-square-foot residential (R-2) building at 138 New Jersey Avenue in Cypress Hills, Brooklyn. The plan was filed on June 1, 2026. It calls for the construction of a 100-foot-tall, ten-story building and was filed with the New York City Department of Buildings under job number B01373493. The project is described in the filing as: propose 10-story residential building as per plan. The applicant is the Registered Architect Stephen Conte of StudiosC Architecture. This 10-story residential building features 71 Class A apartments with eight units on floors 2 through 9 and six on the 10th floor. The ground level includes a 7-space parking garage, mail and package rooms, laundry facilities, and bike storage for 36 bicycles. Amenities include a 10th-floor fitness room and a rooftop terrace for residents. Supporting infrastructure such as mechanical, electrical, and elevator equipment rooms is located on the ground floor and roof levels. 138 New Jersey Avenue wdt_ID wdt_created_by wdt_created_at wdt_last_edited_by wdt_la</t>
+          <t>Transfers 2282 Bronx Park East axonometric diagram (Credit - Fernando Geremia architect via DOB) Aleksander Haxhari through the entity BPE Realty LLC as borrower signed a construction loan with lender NorthEast Community Bank valued at $11.1 million for the 53-unit project at 2282 Bronx Park East in Allerton, Bronx. On the lot, there is one active new building construction project, X01056756, for a 53-unit, 32,181 square-foot residential (R-2) building. The project was submitted by Aleksander Haxhari on June 7, 2024 and it was permitted December 17, 2025. The loan closed on May 27, 2026 and was recorded on June 2, 2026. The prior lender was Suma Federal Credit Union which held debt that had an original loan amount of $765,000. The property has 6,028 square feet of built space and 31,004 square feet of additional air rights for a total buildable of 31,004 square feet according to a PincusCo analysis of city data. The loan price per built square foot is $1,841 and the price per buildable square foot is $358 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been so</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Barone Management signs contract to buy Laurelton dev site, price not disclosed</t>
+          <t>Claremont Companies ups debt to $56.5M with City National for hotel in Hudson Square</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>https://www.pincusco.com/barone-management-signs-contract-to-buy-laurelton-dev-site-price-not-disclosed/</t>
+          <t>https://www.pincusco.com/claremont-companies-ups-debt-to-56-5m-with-city-national-for-hotel-in-hudson-square/</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Barone Management through the entity BMAD Springfield LLC signed a contract as buyer with Evan</t>
+          <t>Claremont Companies through the entity Soho Hotel LLC as borrower signed a refi loan with</t>
         </is>
       </c>
       <c r="D5" t="inlineStr"/>
@@ -602,24 +602,24 @@
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>Transfers 223-01 Merrick Boulevard (Credit - Cyclomedia) Barone Management through the entity BMAD Springfield LLC signed a contract as buyer with Evan Tannor through the entity Merrick Boulevard Acquisitions, LLC, as seller, for the industrial properties in Laurelton, Queens, including 223-15 Merrick Boulevard, 223-01 Merrick Boulevard. The expected use is ground up development. The price was not disclosed. The deal closed on April 1, 2026 and was recorded on June 2, 2026. The three properties have 1,155 square feet of built space and 51,416 square feet of additional air rights for a total buildable of 52,582 square feet according to a PincusCo analysis of city data. The signatory for Evan Tannor was Evan Tannor. The signatory for Barone Management was Scott Barone . The memorandum of contract says the closing date is July 27, 2027. Prior sales, articles and revenue Prior to this transaction, PincusCo has records that the buyer Barone Management purchased three properties in two transactions for a total of $19.8 million and sold two properties in one transaction for a total of $85 million over the past 24 months. The seller Evan Tannor had not purchased any other properties and ha</t>
+          <t>Transfers 181 Varick Street (Credit - Cyclomedia) Claremont Companies through the entity Soho Hotel LLC as borrower signed a refi loan with lender City National Bank through the entity City National Bank valued at $56.5 million for the Courtyard by Marriott New York Manhattan/SoHo hotel building (H2) at 181 Varick Street in Hudson Square, Manhattan. The deal closed on May 22, 2026 and was recorded on June 2, 2026. The prior lender was Thrivent which held debt that had an original loan amount of $35 million. The property has 52,155 square feet of built space according to a PincusCo analysis of city data. The loan price per built square foot is $1,083 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) The owner bought the property on October 30, 2019, for $59.4 million. The signatory for Claremont Companies was company president, Ned Carney . The signatory for City National Bank was Luke Millikin . Prior sales, articles and revenue The owners according to the Department of Housing Preservation and Development includes Patrick Carney, head officer. The b</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Alon Ashourzadeh pays $3.4M for mixed-use in Carroll Gardens</t>
+          <t>Abdiel Capital pays $13.1M to Starwood for landmarked Norwood House in Chelsea</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>https://www.pincusco.com/alon-ashourzadeh-pays-3-4m-for-mixed-use-in-carroll-gardens/</t>
+          <t>https://www.pincusco.com/abdiel-capital-pays-13-1m-to-starwood-for-landmarked-3-family-in-chelsea/</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Alon Ashourzadeh through the entity 445 Court LLC paid $3.4 million for the three-unit mixed-use</t>
+          <t>Abdiel Capital Advisors through the entity Norwood House LLC paid $13.1 million through a real</t>
         </is>
       </c>
       <c r="D6" t="inlineStr"/>
@@ -636,24 +636,24 @@
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>Transfers 445 Court Street (Credit - Cyclomedia) Alon Ashourzadeh through the entity 445 Court LLC paid $3.4 million for the three-unit mixed-use building (S3) at 445 Court Street in Carroll Gardens, Brooklyn. The expected use is renovation and cash flowing. The deal closed on May 4, 2026 and was recorded on June 2, 2026. The property has 3,936 square feet of built space and 1,152 square feet of additional air rights for a total buildable of 5,085 square feet according to a PincusCo analysis of city data. The sale price per built square foot is $851 and the price per buildable square foot is $659 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) The signatory for the estate of the late Ralph DiBenedetto was Ralph DiBenedetto Jr. . The signatory for Alon Ashourzadeh was Stephen Siminou . The contract date was August 27, 2025. Ralph DiBenedetto died. Alon Ashourzadeh signed a memorandum of contract of sale recorded in December 2025. DiBenedetto Jr. sold 423 Court Street to Alon Ashourzadeh in 2022. To finance the purchase and construction, Alon Ashourz</t>
+          <t>Transfers 241 West 14th Street (Credit - Cyclomedia) Abdiel Capital Advisors through the entity Norwood House LLC paid $13.1 million through a real estate owned transaction to Starwood Mortgage Capital through the entity 241 Norwood, LLC for the three-unit building (C0), a city landmark known as the Andrew S. Norwood House, at 241 West 14th Street in Chelsea, Manhattan. The deal closed on May 15, 2026 and was recorded on June 3, 2026. The property has 7,830 square feet of built space and 10,297 square feet of additional air rights for a total buildable of 18,126 square feet according to a PincusCo analysis of city data. The sale price per built square foot is $1,666 and the price per buildable square foot is $719 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) The seller bought the property on July 12, 2024, for $3 million. The signatory for Starwood Mortgage Capital was Adam Behlman . The signatory for Abdiel Capital Advisors was Colin Moran . The contract date was April 15, 2026. Starwood Capital Group through the entity 241 Norwood, LLC as the f</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Metro Loft, Quantum sign $169.5M construction loan for 337-unit resi conversion in Midtown East</t>
+          <t>SilverLining Development NY pays $16M for dev site in West Village</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>https://www.pincusco.com/metro-loft-quantum-sign-169-5m-construction-loan-for-337-unit-resi-conversion-in-midtown-east/</t>
+          <t>https://www.pincusco.com/silverlining-development-ny-pays-16m-for-dev-site-in-west-village/</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Metro Loft Management and Quantum Pacific Group through the entity 767 Third Property Owner LLC</t>
+          <t>SilverLining Development NY through the entity Leroy Street Owner LLC paid $16 million to Santa</t>
         </is>
       </c>
       <c r="D7" t="inlineStr"/>
@@ -670,24 +670,24 @@
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>Transfers 767 3rd Avenue (Credit - Cyclomedia) Metro Loft Management and Quantum Pacific Group through the entity 767 Third Property Owner LLC as borrower signed a rehab construction loan with lender Bank Hapoalim valued at $169.5 million for the conversion of the office building (O4) at 767 Third Avenue in Midtown East, Manhattan, to a mixed-used building with 337 units. On the lot, there is one active major alteration construction project, M01237433, for a 337-unit, 217,243 square-foot residential (R-2) building. The project was submitted by Metro Loft Management and filed by Robert Travis with plans filed July 30, 2025 and permitted April 6, 2026. The deal closed on May 19, 2026 and was recorded on June 2, 2026. The prior lender was Bank Hapoalim which held debt that had an original loan amount of $55 million.The property has 286,212 square feet of built space according to a PincusCo analysis of city data. The loan price per built square foot is $592 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) The owner bought the property on December 31, 20</t>
+          <t>Transfers 152-154 Leroy Street (Credit - Cyclomedia) SilverLining Development NY through the entity Leroy Street Owner LLC paid $16 million to Santa Fe-based Zydeco 66 through the entity Heretofore, LLC for the parking lot (G7) at 152-154 Leroy Street in West Village, Manhattan. The expected use is ground up development. The deal closed on May 20, 2026 and was recorded on June 3, 2026. The property has zero square feet of built space and 27,980 square feet of additional air rights for a total buildable of 27,980 square feet according to a PincusCo analysis of city data. The sale price per built square foot is $N/A and the price per buildable square foot is $571 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) The seller bought the property on December 27, 2012, for $10.25 million. The signatory for Zydeco 66 was Richard Yates . The signatory for SilverLining Development NY was Aden Wiener . The contract date was May 20, 2026. PincusCo reported on the transaction when it went into contract, but did not have the price. Prior sales, articles and revenu</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Anish Berry pays $7M to dentist Nitin Doshi for offices in Flushing, UWS</t>
+          <t>Northwell Health pays $229.6M to Vornado for mixed-use in Rego Park</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>https://www.pincusco.com/anish-berry-pays-7m-to-nitin-doshi-for-office-in-flushing-uws/</t>
+          <t>https://www.pincusco.com/northwell-health-pays-229-6m-to-vornado-for-mixed-use-in-rego-park/</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Anish Berry paid $7 million to dentist Nitin Doshi for an office building in Flushing,</t>
+          <t>Northwell Health paid $229.6 million to Vornado Realty Trust through the entity Alexander’s Rego Shopping</t>
         </is>
       </c>
       <c r="D8" t="inlineStr"/>
@@ -704,7 +704,7 @@
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>Transfers 43-55 147th Street (Credit - Cyclomedia) Anish Berry paid $7 million to dentist Nitin Doshi for an office building in Flushing, Queens, and an office condominium unit in the Upper West Side of Manhattan in two transactions. In the first, Anish Berry through the entity 4355 Realty NY LLC paid $4 million to Nitin Doshi through the entity Flushing Medical Arts Building Inc. for the office building (O2) at 43-55 147th Street in Flushing, Queens. The deal closed on May 19, 2026 and was recorded on June 2, 2026. The property has 10,856 square feet of built space according to a PincusCo analysis of city data. The sale price per built square foot is $368 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) In the second, Anish Berry through the entity 130 Realty Ny LLC paid $3 million to Nitin Doshi through the entity West 79th Street Realty Associates LLC for the office condo at 130 West 79th Street in Upper West Side, Manhattan. The deal closed on May 19, 2026 and was recorded on June 2, 2026. The property has 5,326 square feet of built space accord</t>
+          <t>Transfers 96-05 Queens Boulevard (Credit - Cyclomedia) Northwell Health paid $229.6 million to Vornado Realty Trust through the entity Alexander’s Rego Shopping Center, Inc. for the mixed-use building (K3) at 96-05 Queens Boulevard in Rego Park, Queens. The expected use is owner-occupied. The deal closed on May 27, 2026 and was recorded on June 3, 2026. The property has 860,000 square feet of built space according to a PincusCo analysis of city data. The sale price per built square foot is $267 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) The seller bought the property on March 24, 2005, for $58 million. The signatory for Vornado Realty Trust was Steven J. Borenstein . The signatory for Northwell Health was Kevin Beiner . The contract date was May 27, 2026. Prior sales, articles and revenue Prior to this transaction, PincusCo has records that the buyer Northwell Health purchased two properties in two transactions for a total of $18.7 million and has no record it sold any properties over the past 24 months. The seller Vornado Realty Trust purchas</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto update queens news 2026-06-05T15:26:54Z
</commit_message>
<xml_diff>
--- a/data/output/queens_dev_news.xlsx
+++ b/data/output/queens_dev_news.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H8"/>
+  <dimension ref="A1:H6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -473,17 +473,17 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Spectra Construction signs $28M construction loan for 43-unit project in NoMad</t>
+          <t>Gabriel Weiser pays $4.8M for office in Tribeca</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>https://www.pincusco.com/spectra-construction-signs-28m-construction-loan-for-43-unit-project-in-nomad/</t>
+          <t>https://www.pincusco.com/gabriel-weiser-pays-4-8m-for-office-in-tribeca/</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Spectra Construction and Development through the entity Ww Lexington, LLC as borrower signed a new</t>
+          <t>Gabriel Weiser through the entity 132 W Broadway LLC paid $4.8 million to the entity</t>
         </is>
       </c>
       <c r="D2" t="inlineStr"/>
@@ -500,24 +500,24 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Transfers 129 East 28th Street isometric diagram (Credit - Alexander Zhitnik architect via DOB) Spectra Construction and Development through the entity Ww Lexington, LLC as borrower signed a new construction loan with lender Castellan Capital through the entity 120 Lexington LLC valued at $28 million for three tax lots making up the 43-unit project at 129 East 28th Street in NoMad, Manhattan. On these lots, there is a new building project, M01230688, for a 43-unit, 38,405 square-foot residential (R-2) building submitted by Spectra Construction and Development and filed by Daniel Klaynberg with plans filed July 21, 2025 and it has not been permitted yet. The loan closed on April 30, 2026 and was recorded on June 2, 2026. The loan price per planned development square foot is $729 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) The signatory for Spectra Construction and Development was Daniel Klaynberg . ZD1 DOB Zoning Diagram </t>
+          <t xml:space="preserve">Transfers 132 West Broadway (Credit - Cyclomedia) Gabriel Weiser through the entity 132 W Broadway LLC paid $4.8 million to the entity Joy B, LLC for the office building (O2) at 132 West Broadway in Tribeca, Manhattan. The deal closed on May 21, 2026 and was recorded on June 4, 2026. The property has 2,500 square feet of built space and 5,102 square feet of additional air rights for a total buildable of 7,603 square feet according to a PincusCo analysis of city data. The sale price per built square foot is $1,940 and the price per buildable square foot is $637 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) The signatory for the seller was Neil Bradley. The signatory for Gabriel Weiser was Gabriel Weiser. The contract date was March 19, 2026. Prior sales, articles and revenue Prior to this transaction, PincusCo has records that the buyer Gabriel Weiser purchased one property in one transaction for a total of $2.7 million and has no record it sold any properties over the past 24 months. The seller Neil Bradley had not purchased any other properties </t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Sackman Enterprises signs $10.69M refi with Chase for four walkups in Manhattan</t>
+          <t>Anbau Inc. pays $7M for 7-unit walkup in Greenwich Village</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>https://www.pincusco.com/sackman-enterprises-signs-10-69m-refi-with-chase-for-four-walkup-in-manhattan/</t>
+          <t>https://www.pincusco.com/anbau-inc-pays-7m-for-7-unit-walkup-in-greenwich-village/</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Sackman Enterprises through the entity Marsac Realty, LLC as borrower signed a refi loan with</t>
+          <t>Anbau Inc. through the entity 127 W 12th Owner LLC paid $7 million for the</t>
         </is>
       </c>
       <c r="D3" t="inlineStr"/>
@@ -534,24 +534,24 @@
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>Transfers 203 West 84th Street (Credit - Cyclomedia) Sackman Enterprises through the entity Marsac Realty, LLC as borrower signed a refi loan with lender JPMorgan Chase valued at $10.69 million for four residential walkup properties with 35 residential units including the 10-unit residential walkup building (C7) at 203 West 84th Street in Upper West Side, Manhattan, eight-unit residential walkup building (C7) at 730 10th Avenue in Hell’s Kitchen, Manhattan, and nine-unit residential walkup building (C7) at 732 10th Avenue in Hell’s Kitchen, Manhattan. The deal closed on April 30, 2026 and was recorded on June 2, 2026. The prior lender was JPMorgan Chase which in 2015 provided debt that had an original loan amount of $10.69 million.The four properties have 25,091 square feet of built space and 11,657 square feet of additional air rights for a total buildable of 36,439 square feet according to a PincusCo analysis of city data. The loan price per built square foot is $426 and the price per buildable square foot is $293 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights h</t>
+          <t>Transfers 127 West 12th Street (Credit - Cyclomedia) Anbau Inc. through the entity 127 W 12th Owner LLC paid $7 million for the seven-unit residential walkup building (C5) at 127 West 12th Street in Greenwich Village, Manhattan. The expected use is cash flowing. The deal closed on May 18, 2026 and was recorded on June 4, 2026. The property has 4,299 square feet of built space and 1,347 square feet of additional air rights for a total buildable of 5,644 square feet according to a PincusCo analysis of city data. The sale price per built square foot is $1,628 and the price per buildable square foot is $1,240 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) The signatory for the seller, a trust for Alan Johnson, was Monika Staiger Johnson . The signatory for Anbau Inc. was Steven Gorey . The contract date was February 15, 2026. Prior sales, articles and revenue Prior to this transaction, PincusCo has records that the buyer Anbau, Inc. purchased one property in one transaction for a total of $4.3 million and sold one property in one transaction for a tot</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Aleksander Haxhari signs $11.1M construction loan for 53-unit project in Allerton</t>
+          <t>Savo Brothers pays $8.3M for dev site in Staten Island’s Sunnyside</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>https://www.pincusco.com/aleksander-haxhari-signs-11-1m-construction-loan-for-53-unit-project-in-allerton/</t>
+          <t>https://www.pincusco.com/savo-brothers-pays-8-3m-for-dev-site-in-staten-islands-sunnyside/</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Aleksander Haxhari through the entity BPE Realty LLC as borrower signed a construction loan with</t>
+          <t>Savo Brothers through the entity 2025 Richmond Avenue LLC paid the entity Clove Gardens I,</t>
         </is>
       </c>
       <c r="D4" t="inlineStr"/>
@@ -568,24 +568,24 @@
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>Transfers 2282 Bronx Park East axonometric diagram (Credit - Fernando Geremia architect via DOB) Aleksander Haxhari through the entity BPE Realty LLC as borrower signed a construction loan with lender NorthEast Community Bank valued at $11.1 million for the 53-unit project at 2282 Bronx Park East in Allerton, Bronx. On the lot, there is one active new building construction project, X01056756, for a 53-unit, 32,181 square-foot residential (R-2) building. The project was submitted by Aleksander Haxhari on June 7, 2024 and it was permitted December 17, 2025. The loan closed on May 27, 2026 and was recorded on June 2, 2026. The prior lender was Suma Federal Credit Union which held debt that had an original loan amount of $765,000. The property has 6,028 square feet of built space and 31,004 square feet of additional air rights for a total buildable of 31,004 square feet according to a PincusCo analysis of city data. The loan price per built square foot is $1,841 and the price per buildable square foot is $358 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been so</t>
+          <t xml:space="preserve">Transfers 18-20 Bristol Avenue (Credit - Cyclomedia) Savo Brothers through the entity 2025 Richmond Avenue LLC paid the entity Clove Gardens I, LLC, $8.3 million for nursing home buildings (N2) at 18 and 20 Bristol Avenue in Sunnyside, Staten Island. 20 Bristol Avenue was the former home of the Swedish Home for the Aged. The expected use is ground up development and/or redevelopment. The deal closed on May 19, 2026 and was recorded on June 4, 2026. The two properties have a total buildable of 64,631 square feet according to a PincusCo analysis of city data. The sale price per buildable square foot is $129 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) Clove Gardens I had a plan to build a 100-unit assisted living project on the parcel, according to a listing from Crexi. Prior sales, articles and revenue Prior to this transaction, PincusCo has records that the buyer Savo Brothers purchased eight properties in one transaction for a total of $4 million and sold one property in one transaction for a total of $10.2 million over the past 24 months. The </t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Claremont Companies ups debt to $56.5M with City National for hotel in Hudson Square</t>
+          <t>Delshah, AM Property, REALM $130M purchase of Tishman, GIC’s CitySpire gets recorded</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>https://www.pincusco.com/claremont-companies-ups-debt-to-56-5m-with-city-national-for-hotel-in-hudson-square/</t>
+          <t>https://www.pincusco.com/delshah-am-property-realm-130m-purchase-of-tishman-gics-cityspire-gets-recorded/</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Claremont Companies through the entity Soho Hotel LLC as borrower signed a refi loan with</t>
+          <t>Delshah Capital , AM Property Holding , and REALM through the entity CitySpire JV LLC</t>
         </is>
       </c>
       <c r="D5" t="inlineStr"/>
@@ -602,24 +602,24 @@
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>Transfers 181 Varick Street (Credit - Cyclomedia) Claremont Companies through the entity Soho Hotel LLC as borrower signed a refi loan with lender City National Bank through the entity City National Bank valued at $56.5 million for the Courtyard by Marriott New York Manhattan/SoHo hotel building (H2) at 181 Varick Street in Hudson Square, Manhattan. The deal closed on May 22, 2026 and was recorded on June 2, 2026. The prior lender was Thrivent which held debt that had an original loan amount of $35 million. The property has 52,155 square feet of built space according to a PincusCo analysis of city data. The loan price per built square foot is $1,083 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) The owner bought the property on October 30, 2019, for $59.4 million. The signatory for Claremont Companies was company president, Ned Carney . The signatory for City National Bank was Luke Millikin . Prior sales, articles and revenue The owners according to the Department of Housing Preservation and Development includes Patrick Carney, head officer. The b</t>
+          <t xml:space="preserve">Top Story Transfers 150 West 56th Street (Credit - Cyclomedia) Delshah Capital , AM Property Holding , and REALM through the entity CitySpire JV LLC paid Tishman Speyer and the Singapore sovereign fund GIC through the entity CitySpire REIT, Inc., $130 million for the office and retail condominium unit of the CitySpire tower spanning 24 floors at 150 West 56th Street in Midtown West, Manhattan. The Commercial Observer reported on the sale in February 2026. Prior news articles used a slightly higher price, but a representative from Delshah Capital said the $130 million figure was correct. The deal closed on May 26, 2026 and was recorded on June 4, 2026. The property has 309,391 square feet of built space according to a PincusCo analysis of city data. The sale price per built square foot is $420 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) Michael Shah‘s Delshah Capital, AM Property Holding, and their investors form a group that owns a 50 percent stake in the venture, and is the managing member, while partner REALM owns the remaining 50 percent. A </t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Abdiel Capital pays $13.1M to Starwood for landmarked Norwood House in Chelsea</t>
+          <t>Javeri Capital pays $11.4M for 7-unit rental in Nolita</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>https://www.pincusco.com/abdiel-capital-pays-13-1m-to-starwood-for-landmarked-3-family-in-chelsea/</t>
+          <t>https://www.pincusco.com/javeri-capital-pays-11-4m-for-7-unit-rental-in-nolita/</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Abdiel Capital Advisors through the entity Norwood House LLC paid $13.1 million through a real</t>
+          <t>Javeri Capital through the entity 196 Bowery Owner LLC paid $11.4 million to the entity</t>
         </is>
       </c>
       <c r="D6" t="inlineStr"/>
@@ -636,75 +636,7 @@
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>Transfers 241 West 14th Street (Credit - Cyclomedia) Abdiel Capital Advisors through the entity Norwood House LLC paid $13.1 million through a real estate owned transaction to Starwood Mortgage Capital through the entity 241 Norwood, LLC for the three-unit building (C0), a city landmark known as the Andrew S. Norwood House, at 241 West 14th Street in Chelsea, Manhattan. The deal closed on May 15, 2026 and was recorded on June 3, 2026. The property has 7,830 square feet of built space and 10,297 square feet of additional air rights for a total buildable of 18,126 square feet according to a PincusCo analysis of city data. The sale price per built square foot is $1,666 and the price per buildable square foot is $719 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) The seller bought the property on July 12, 2024, for $3 million. The signatory for Starwood Mortgage Capital was Adam Behlman . The signatory for Abdiel Capital Advisors was Colin Moran . The contract date was April 15, 2026. Starwood Capital Group through the entity 241 Norwood, LLC as the f</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>SilverLining Development NY pays $16M for dev site in West Village</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>https://www.pincusco.com/silverlining-development-ny-pays-16m-for-dev-site-in-west-village/</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>SilverLining Development NY through the entity Leroy Street Owner LLC paid $16 million to Santa</t>
-        </is>
-      </c>
-      <c r="D7" t="inlineStr"/>
-      <c r="E7" t="inlineStr"/>
-      <c r="F7" t="inlineStr">
-        <is>
-          <t>PincusCo</t>
-        </is>
-      </c>
-      <c r="G7" t="inlineStr">
-        <is>
-          <t>PincusCo - Home</t>
-        </is>
-      </c>
-      <c r="H7" t="inlineStr">
-        <is>
-          <t>Transfers 152-154 Leroy Street (Credit - Cyclomedia) SilverLining Development NY through the entity Leroy Street Owner LLC paid $16 million to Santa Fe-based Zydeco 66 through the entity Heretofore, LLC for the parking lot (G7) at 152-154 Leroy Street in West Village, Manhattan. The expected use is ground up development. The deal closed on May 20, 2026 and was recorded on June 3, 2026. The property has zero square feet of built space and 27,980 square feet of additional air rights for a total buildable of 27,980 square feet according to a PincusCo analysis of city data. The sale price per built square foot is $N/A and the price per buildable square foot is $571 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) The seller bought the property on December 27, 2012, for $10.25 million. The signatory for Zydeco 66 was Richard Yates . The signatory for SilverLining Development NY was Aden Wiener . The contract date was May 20, 2026. PincusCo reported on the transaction when it went into contract, but did not have the price. Prior sales, articles and revenu</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>Northwell Health pays $229.6M to Vornado for mixed-use in Rego Park</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>https://www.pincusco.com/northwell-health-pays-229-6m-to-vornado-for-mixed-use-in-rego-park/</t>
-        </is>
-      </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>Northwell Health paid $229.6 million to Vornado Realty Trust through the entity Alexander’s Rego Shopping</t>
-        </is>
-      </c>
-      <c r="D8" t="inlineStr"/>
-      <c r="E8" t="inlineStr"/>
-      <c r="F8" t="inlineStr">
-        <is>
-          <t>PincusCo</t>
-        </is>
-      </c>
-      <c r="G8" t="inlineStr">
-        <is>
-          <t>PincusCo - Home</t>
-        </is>
-      </c>
-      <c r="H8" t="inlineStr">
-        <is>
-          <t>Transfers 96-05 Queens Boulevard (Credit - Cyclomedia) Northwell Health paid $229.6 million to Vornado Realty Trust through the entity Alexander’s Rego Shopping Center, Inc. for the mixed-use building (K3) at 96-05 Queens Boulevard in Rego Park, Queens. The expected use is owner-occupied. The deal closed on May 27, 2026 and was recorded on June 3, 2026. The property has 860,000 square feet of built space according to a PincusCo analysis of city data. The sale price per built square foot is $267 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) The seller bought the property on March 24, 2005, for $58 million. The signatory for Vornado Realty Trust was Steven J. Borenstein . The signatory for Northwell Health was Kevin Beiner . The contract date was May 27, 2026. Prior sales, articles and revenue Prior to this transaction, PincusCo has records that the buyer Northwell Health purchased two properties in two transactions for a total of $18.7 million and has no record it sold any properties over the past 24 months. The seller Vornado Realty Trust purchas</t>
+          <t>Transfers 196 Bowery (Credit - Cyclomedia) Javeri Capital through the entity 196 Bowery Owner LLC paid $11.4 million to the entity Bowery Square Corp. for the seven-unit residential elevator building (D6) at 196 Bowery in Nolita, Manhattan. The expected use is cash flowing. The deal closed on May 26, 2026 and was recorded on June 4, 2026. The property has 15,128 square feet of built space according to a PincusCo analysis of city data. The sale price per built square foot is $753 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) The signatories for the sellers were for Kai Hi Fung, Kin Yee Wong, and Kin Chi Au. The signatory for Javeri Capital was Atit Javeri . The contract date was January 27, 2026. Prior sales, articles and revenue Prior to this transaction, PincusCo has no record that the buyer Javeri Capital had purchased any other properties and has no record it sold any properties over the past 24 months. The seller Kai Hi Fung had not purchased any other properties and had not sold any properties over the same time period. The former owners acc</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto update queens news 2026-06-06T14:06:12Z
</commit_message>
<xml_diff>
--- a/data/output/queens_dev_news.xlsx
+++ b/data/output/queens_dev_news.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H6"/>
+  <dimension ref="A1:H9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -473,17 +473,17 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Gabriel Weiser pays $4.8M for office in Tribeca</t>
+          <t>Two80 Real Estate pays $5M for 36-unit walkup in Washington Heights</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>https://www.pincusco.com/gabriel-weiser-pays-4-8m-for-office-in-tribeca/</t>
+          <t>https://www.pincusco.com/two80-real-estate-pays-5m-for-36-unit-walkup-in-washington-heights/</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Gabriel Weiser through the entity 132 W Broadway LLC paid $4.8 million to the entity</t>
+          <t>Two80 Real Estate Ventures through the entity 120 Haven Realty LLC paid $5 million to</t>
         </is>
       </c>
       <c r="D2" t="inlineStr"/>
@@ -500,24 +500,24 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Transfers 132 West Broadway (Credit - Cyclomedia) Gabriel Weiser through the entity 132 W Broadway LLC paid $4.8 million to the entity Joy B, LLC for the office building (O2) at 132 West Broadway in Tribeca, Manhattan. The deal closed on May 21, 2026 and was recorded on June 4, 2026. The property has 2,500 square feet of built space and 5,102 square feet of additional air rights for a total buildable of 7,603 square feet according to a PincusCo analysis of city data. The sale price per built square foot is $1,940 and the price per buildable square foot is $637 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) The signatory for the seller was Neil Bradley. The signatory for Gabriel Weiser was Gabriel Weiser. The contract date was March 19, 2026. Prior sales, articles and revenue Prior to this transaction, PincusCo has records that the buyer Gabriel Weiser purchased one property in one transaction for a total of $2.7 million and has no record it sold any properties over the past 24 months. The seller Neil Bradley had not purchased any other properties </t>
+          <t>Transfers Two80 Real Estate Ventures through the entity 120 Haven Realty LLC paid $5 million to Marina Kafarski through the entity Hudson Cliff Realty, L.L.C. for the 36-unit residential walkup building (C1) at 120 Haven Avenue in Washington Heights, Manhattan. The expected use is cash flowing. The deal closed on May 28, 2026 and was recorded on June 3, 2026. The property has 25,755 square feet of built space and 54,523 square feet of additional air rights for a total buildable of 80,252 square feet according to a PincusCo analysis of city data. The sale price per built square foot is $195 and the price per buildable square foot is $62 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) The signatory for Marina Kafarski was Marina Kafarski. The signatory for Two80 Real Estate Ventures was Jesse Deutch . The contract date was March 6, 2026. Prior sales, articles and revenue Prior to this transaction, PincusCo has records that the buyer Two80 Real Estate Ventures purchased 10 properties in 10 transactions for a total of $65.7 million and has no record it</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Anbau Inc. pays $7M for 7-unit walkup in Greenwich Village</t>
+          <t>Adam Croman, Jake Croman pay $2.3M for 19-unit walkup in Little Italy</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>https://www.pincusco.com/anbau-inc-pays-7m-for-7-unit-walkup-in-greenwich-village/</t>
+          <t>https://www.pincusco.com/adam-croman-jake-croman-pay-2-3m-for-19-unit-walkup-in-little-italy/</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Anbau Inc. through the entity 127 W 12th Owner LLC paid $7 million for the</t>
+          <t>Adam Croman and Jake Croman through the entity 118 Mulberry LLC paid $2.3 million to</t>
         </is>
       </c>
       <c r="D3" t="inlineStr"/>
@@ -534,24 +534,24 @@
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>Transfers 127 West 12th Street (Credit - Cyclomedia) Anbau Inc. through the entity 127 W 12th Owner LLC paid $7 million for the seven-unit residential walkup building (C5) at 127 West 12th Street in Greenwich Village, Manhattan. The expected use is cash flowing. The deal closed on May 18, 2026 and was recorded on June 4, 2026. The property has 4,299 square feet of built space and 1,347 square feet of additional air rights for a total buildable of 5,644 square feet according to a PincusCo analysis of city data. The sale price per built square foot is $1,628 and the price per buildable square foot is $1,240 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) The signatory for the seller, a trust for Alan Johnson, was Monika Staiger Johnson . The signatory for Anbau Inc. was Steven Gorey . The contract date was February 15, 2026. Prior sales, articles and revenue Prior to this transaction, PincusCo has records that the buyer Anbau, Inc. purchased one property in one transaction for a total of $4.3 million and sold one property in one transaction for a tot</t>
+          <t>Transfers Adam Croman and Jake Croman through the entity 118 Mulberry LLC paid $2.3 million to Martin Jajan through the entity 118 Mulberry Realty LLC for the 19-unit residential walkup building (C7) at 118 Mulberry Street in Little Italy, Manhattan. The expected use is cash flowing. The deal closed on May 13, 2026 and was recorded on June 3, 2026. The property has 11,154 square feet of built space and 18,839 square feet of additional air rights for a total buildable of 30,003 square feet according to a PincusCo analysis of city data. The sale price per built square foot is $204 and the price per buildable square foot is $75 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) The signatory for Martin Jajan was Martin Jajan. The signatory for Adam Croman and Jake Croman was Harriet Croman . The contract date was February 5, 2026. Traded reported the sale, but not the buyer. Adam and Jake are sons of real estate investors Steven Croman and Harriet Croman. Prior sales, articles and revenue Prior to this transaction, PincusCo has no record that the buyer A</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Savo Brothers pays $8.3M for dev site in Staten Island’s Sunnyside</t>
+          <t>Borough Developers, David Tabak sign $40M refi with QuadReal for rental in Gramercy</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>https://www.pincusco.com/savo-brothers-pays-8-3m-for-dev-site-in-staten-islands-sunnyside/</t>
+          <t>https://www.pincusco.com/borough-developers-david-tabak-sign-40m-refi-with-quadreal-for-rental-in-gramercy/</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Savo Brothers through the entity 2025 Richmond Avenue LLC paid the entity Clove Gardens I,</t>
+          <t>Borough Developers and David Tabak through the entity Three One Three LLC as borrower signed</t>
         </is>
       </c>
       <c r="D4" t="inlineStr"/>
@@ -568,24 +568,24 @@
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Transfers 18-20 Bristol Avenue (Credit - Cyclomedia) Savo Brothers through the entity 2025 Richmond Avenue LLC paid the entity Clove Gardens I, LLC, $8.3 million for nursing home buildings (N2) at 18 and 20 Bristol Avenue in Sunnyside, Staten Island. 20 Bristol Avenue was the former home of the Swedish Home for the Aged. The expected use is ground up development and/or redevelopment. The deal closed on May 19, 2026 and was recorded on June 4, 2026. The two properties have a total buildable of 64,631 square feet according to a PincusCo analysis of city data. The sale price per buildable square foot is $129 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) Clove Gardens I had a plan to build a 100-unit assisted living project on the parcel, according to a listing from Crexi. Prior sales, articles and revenue Prior to this transaction, PincusCo has records that the buyer Savo Brothers purchased eight properties in one transaction for a total of $4 million and sold one property in one transaction for a total of $10.2 million over the past 24 months. The </t>
+          <t>Transfers 313 East 17th Street (Credit - Cyclomedia) Borough Developers and David Tabak through the entity Three One Three LLC as borrower signed a refi loan with lender QuadReal Property Group through the entity Qr Us Finance Reit LLC valued at $40 million for the 87-unit residential rental building at 313 East 17th Street in Gramercy, Manhattan and the adjacent nine-unit rental building at 321 East 17th Street. The deal closed on May 20, 2026 and was recorded on June 3, 2026. The prior lender was Valley National Bank which held debt that had an original loan amount of $24.8 million.The two properties have 77,499 square feet of built space and 5,478 square feet of additional air rights for a total buildable of 78,488 square feet according to a PincusCo analysis of city data. The loan price per built square foot is $516 and the price per buildable square foot is $509 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) David Tabak signed for the borrowers with an alternate version of his name, Meir D. Tabak. The signatory for QuadReal Property Group was</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Delshah, AM Property, REALM $130M purchase of Tishman, GIC’s CitySpire gets recorded</t>
+          <t>Firebird Grove signs $20M refi with Morgan Stanley for 10 properties in Greenwich Village</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>https://www.pincusco.com/delshah-am-property-realm-130m-purchase-of-tishman-gics-cityspire-gets-recorded/</t>
+          <t>https://www.pincusco.com/firebird-grove-signs-20m-refi-with-morgan-stanley-for-10-properties-in-greenwich-village/</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Delshah Capital , AM Property Holding , and REALM through the entity CitySpire JV LLC</t>
+          <t>Firebird Grove through the entity OR Patchin Place LLC as borrower signed a refi loan</t>
         </is>
       </c>
       <c r="D5" t="inlineStr"/>
@@ -602,24 +602,24 @@
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Top Story Transfers 150 West 56th Street (Credit - Cyclomedia) Delshah Capital , AM Property Holding , and REALM through the entity CitySpire JV LLC paid Tishman Speyer and the Singapore sovereign fund GIC through the entity CitySpire REIT, Inc., $130 million for the office and retail condominium unit of the CitySpire tower spanning 24 floors at 150 West 56th Street in Midtown West, Manhattan. The Commercial Observer reported on the sale in February 2026. Prior news articles used a slightly higher price, but a representative from Delshah Capital said the $130 million figure was correct. The deal closed on May 26, 2026 and was recorded on June 4, 2026. The property has 309,391 square feet of built space according to a PincusCo analysis of city data. The sale price per built square foot is $420 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) Michael Shah‘s Delshah Capital, AM Property Holding, and their investors form a group that owns a 50 percent stake in the venture, and is the managing member, while partner REALM owns the remaining 50 percent. A </t>
+          <t>Transfers 9 Patchin Place (Credit: Google) Firebird Grove through the entity OR Patchin Place LLC as borrower signed a refi loan with lender Morgan Stanley through the entity Morgan Stanley Private Bank valued at $20 million for 10 properties with 33 residential units including the four-unit mixed-use building (S4) at 9 Patchin Place in Greenwich Village, Manhattan, five-unit residential walkup building (C2) at 7 Patchin Place in Greenwich Village, Manhattan, and 1-4 family building (A4) at 1 Patchin Place in Greenwich Village, Manhattan. The deal closed on May 20, 2026 and was recorded on June 3, 2026. The prior lender was Derby Copeland Capital which held debt that had an original loan amount of $17 million. The 10 properties have 25,647 square feet of built space and 8,464 square feet of additional air rights for a total buildable of 32,255 square feet according to a PincusCo analysis of city data. The loan price per built square foot is $779 and the price per buildable square foot is $620 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) The sign</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Javeri Capital pays $11.4M for 7-unit rental in Nolita</t>
+          <t>Justin Management signs $63.2M refi with Chase for two properties in Penn Plaza</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>https://www.pincusco.com/javeri-capital-pays-11-4m-for-7-unit-rental-in-nolita/</t>
+          <t>https://www.pincusco.com/justin-management-signs-63-2m-refi-with-chase-for-two-properties-in-penn-plaza/</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Javeri Capital through the entity 196 Bowery Owner LLC paid $11.4 million to the entity</t>
+          <t>Justin Management through the entity 1239 Operating LLC as borrower signed a refi loan with</t>
         </is>
       </c>
       <c r="D6" t="inlineStr"/>
@@ -636,7 +636,109 @@
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>Transfers 196 Bowery (Credit - Cyclomedia) Javeri Capital through the entity 196 Bowery Owner LLC paid $11.4 million to the entity Bowery Square Corp. for the seven-unit residential elevator building (D6) at 196 Bowery in Nolita, Manhattan. The expected use is cash flowing. The deal closed on May 26, 2026 and was recorded on June 4, 2026. The property has 15,128 square feet of built space according to a PincusCo analysis of city data. The sale price per built square foot is $753 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) The signatories for the sellers were for Kai Hi Fung, Kin Yee Wong, and Kin Chi Au. The signatory for Javeri Capital was Atit Javeri . The contract date was January 27, 2026. Prior sales, articles and revenue Prior to this transaction, PincusCo has no record that the buyer Javeri Capital had purchased any other properties and has no record it sold any properties over the past 24 months. The seller Kai Hi Fung had not purchased any other properties and had not sold any properties over the same time period. The former owners acc</t>
+          <t>Transfers 856 Sixth Avenue (Credit - Cyclomedia) Justin Management through the entity 1239 Operating LLC as borrower signed a refi loan with lender JPMorgan Chase valued at $63.2 million for two properties including the office building (O6) at 856 Sixth Avenue and the retail (K4) building at 864 Sixth Avenue in Penn Plaza, Manhattan. The deal closed on May 21, 2026 and was recorded on June 3, 2026. The prior lender was First Republic Bank which held debt that had an original loan amount of $65 million provided in 2013 and 2019. The two properties have 193,000 square feet of built space and 151,540 square feet of additional air rights for a total buildable of 344,525 square feet according to a PincusCo analysis of city data. The loan price per built square foot is $327 and the price per buildable square foot is $183 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) The signatories for Justin Management were Jeffrey Justin and David Justin . The signatory for JPMorgan Chase was Ursula Flores . Prior sales, articles and revenue Out of the two properties</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Yin Chou Hu pays $9M for potential dev site in Flushing</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>https://www.pincusco.com/yin-chou-hu-pays-9m-for-potential-dev-site-in-flushing/</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Yin Chou Hu through the entity Northern Plaza LLC paid $9 million to the entity</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr"/>
+      <c r="E7" t="inlineStr"/>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>PincusCo</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>PincusCo - Home</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Transfers 146-13 Northern Boulevard (Credit - Cyclomedia) Yin Chou Hu through the entity Northern Plaza LLC paid $9 million to the entity Ric Rac North L.L.C for the retail building (K1) at 146-13 Northern Boulevard in Flushing, Queens. The expected use is ground up development, as it was marketed as a potential development site. The deal closed on May 19, 2026 and was recorded on June 4, 2026. The property has 1,710 square feet of built space and 21,541 square feet of additional air rights for a total buildable of 23,264 square feet according to a PincusCo analysis of city data. The sale price per built square foot is $5,263 and the price per buildable square foot is $386 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) The signatory for Richard Berkley and Carol Berkley was Benjamin Brash . The signatory for Yin Chou Hu was Yin Chou Hu. The contract date was February 20, 2026. Traded reported the sale as a development site. Cushman &amp; Wakefield was marketing it on Crexi as well. Prior sales, articles and revenue Prior to this transaction, PincusCo </t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Lender Emerald Creek Capital takes title to LES office, following $32M bankruptcy</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>https://www.pincusco.com/lender-emerald-creek-capital-takes-title-to-les-office-following-32m-bankruptcy/</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Lender Emerald Creek Capital through the entity ECC Bowery LLC, took title to the 18-unit</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr"/>
+      <c r="E8" t="inlineStr"/>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>PincusCo</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>PincusCo - Home</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>Transfers 139 Bowery (Credit - Cyclomedia) Lender Emerald Creek Capital through the entity ECC Bowery LLC, took title to the 18-unit mixed-use building (O6) at 139 Bowery in the Lower East Side, Manhattan, with a transfer value of $49.5 million. The expected use is hold for sale. The former owner Hung Kwong Leung through the entity Global Joint Venture, Inc., filed bankruptcy a year ago following a default on a $32 million loan Emerald Creek Capital provided in 2019. The title transfer closed on May 21, 2026, and was recorded on June 4, 2026. The property has 58,390 square feet of built space according to a PincusCo analysis of city data. The sale price per built square foot is $847 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) The signatory for Hung Kwong Leung was Kevin J. Nash. The signatory for Emerald Creek Capital was Mark Penna. The contract date was May 21, 2026. Just over one year ago, Hung Kwong Leung as president of Global Joint Venture Inc., the sponsor of a mixed-use condominium project at 139 Bowery with 18 residential units, commer</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>ESRT pays $113.6M to Cohen Brothers for 2 ground leased fee properties in Manhattan</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>https://www.pincusco.com/esrt-pays-113-6m-to-cohen-brothers-for-2-ground-leased-fee-properties-in-manhattan/</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Empire State Realty Trust, also known as ESRT, paid $113.6 million to Charles Cohen’s Cohen</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr"/>
+      <c r="E9" t="inlineStr"/>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>PincusCo</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>PincusCo - Home</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>Chart_Frontpage Transfers 1400 Broadway (Credit - Cyclomedia) Empire State Realty Trust, also known as ESRT, paid $113.6 million to Charles Cohen’s Cohen Brothers Realty for two ground leased fee properties in Manhattan, in two transactions. In both cases, ESRT is the ground tenant, so with these transactions is taking full control of both properties. In the larger, Empire State Realty Trust through the entity ESRT 1400 Broadway Fee, L.L.C. paid $61.3 million to Cohen Brothers Realty through the entity 112-1400 Trade Properties LLC for the ground leased fee office building (O4) at 1400 Broadway in Garment District, Manhattan. The expected use is cash flowing. The deal closed on May 20, 2026 and was recorded on June 4, 2026. The property has 768,321 square feet of built space according to a PincusCo analysis of city data. The sale price per built square foot is $79 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) In the second, Empire State Realty Trust through the entity Esrt 112 West 34th Street Fee, L.L.C. paid $52.3 million to Cohen Brothers Real</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto update queens news 2026-06-07T14:18:30Z
</commit_message>
<xml_diff>
--- a/data/output/queens_dev_news.xlsx
+++ b/data/output/queens_dev_news.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H9"/>
+  <dimension ref="A1:H1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -467,278 +467,6 @@
       <c r="H1" s="1" t="inlineStr">
         <is>
           <t>content_preview</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>Two80 Real Estate pays $5M for 36-unit walkup in Washington Heights</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>https://www.pincusco.com/two80-real-estate-pays-5m-for-36-unit-walkup-in-washington-heights/</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>Two80 Real Estate Ventures through the entity 120 Haven Realty LLC paid $5 million to</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr"/>
-      <c r="E2" t="inlineStr"/>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t>PincusCo</t>
-        </is>
-      </c>
-      <c r="G2" t="inlineStr">
-        <is>
-          <t>PincusCo - Home</t>
-        </is>
-      </c>
-      <c r="H2" t="inlineStr">
-        <is>
-          <t>Transfers Two80 Real Estate Ventures through the entity 120 Haven Realty LLC paid $5 million to Marina Kafarski through the entity Hudson Cliff Realty, L.L.C. for the 36-unit residential walkup building (C1) at 120 Haven Avenue in Washington Heights, Manhattan. The expected use is cash flowing. The deal closed on May 28, 2026 and was recorded on June 3, 2026. The property has 25,755 square feet of built space and 54,523 square feet of additional air rights for a total buildable of 80,252 square feet according to a PincusCo analysis of city data. The sale price per built square foot is $195 and the price per buildable square foot is $62 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) The signatory for Marina Kafarski was Marina Kafarski. The signatory for Two80 Real Estate Ventures was Jesse Deutch . The contract date was March 6, 2026. Prior sales, articles and revenue Prior to this transaction, PincusCo has records that the buyer Two80 Real Estate Ventures purchased 10 properties in 10 transactions for a total of $65.7 million and has no record it</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>Adam Croman, Jake Croman pay $2.3M for 19-unit walkup in Little Italy</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>https://www.pincusco.com/adam-croman-jake-croman-pay-2-3m-for-19-unit-walkup-in-little-italy/</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>Adam Croman and Jake Croman through the entity 118 Mulberry LLC paid $2.3 million to</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr"/>
-      <c r="E3" t="inlineStr"/>
-      <c r="F3" t="inlineStr">
-        <is>
-          <t>PincusCo</t>
-        </is>
-      </c>
-      <c r="G3" t="inlineStr">
-        <is>
-          <t>PincusCo - Home</t>
-        </is>
-      </c>
-      <c r="H3" t="inlineStr">
-        <is>
-          <t>Transfers Adam Croman and Jake Croman through the entity 118 Mulberry LLC paid $2.3 million to Martin Jajan through the entity 118 Mulberry Realty LLC for the 19-unit residential walkup building (C7) at 118 Mulberry Street in Little Italy, Manhattan. The expected use is cash flowing. The deal closed on May 13, 2026 and was recorded on June 3, 2026. The property has 11,154 square feet of built space and 18,839 square feet of additional air rights for a total buildable of 30,003 square feet according to a PincusCo analysis of city data. The sale price per built square foot is $204 and the price per buildable square foot is $75 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) The signatory for Martin Jajan was Martin Jajan. The signatory for Adam Croman and Jake Croman was Harriet Croman . The contract date was February 5, 2026. Traded reported the sale, but not the buyer. Adam and Jake are sons of real estate investors Steven Croman and Harriet Croman. Prior sales, articles and revenue Prior to this transaction, PincusCo has no record that the buyer A</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>Borough Developers, David Tabak sign $40M refi with QuadReal for rental in Gramercy</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>https://www.pincusco.com/borough-developers-david-tabak-sign-40m-refi-with-quadreal-for-rental-in-gramercy/</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>Borough Developers and David Tabak through the entity Three One Three LLC as borrower signed</t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr"/>
-      <c r="E4" t="inlineStr"/>
-      <c r="F4" t="inlineStr">
-        <is>
-          <t>PincusCo</t>
-        </is>
-      </c>
-      <c r="G4" t="inlineStr">
-        <is>
-          <t>PincusCo - Home</t>
-        </is>
-      </c>
-      <c r="H4" t="inlineStr">
-        <is>
-          <t>Transfers 313 East 17th Street (Credit - Cyclomedia) Borough Developers and David Tabak through the entity Three One Three LLC as borrower signed a refi loan with lender QuadReal Property Group through the entity Qr Us Finance Reit LLC valued at $40 million for the 87-unit residential rental building at 313 East 17th Street in Gramercy, Manhattan and the adjacent nine-unit rental building at 321 East 17th Street. The deal closed on May 20, 2026 and was recorded on June 3, 2026. The prior lender was Valley National Bank which held debt that had an original loan amount of $24.8 million.The two properties have 77,499 square feet of built space and 5,478 square feet of additional air rights for a total buildable of 78,488 square feet according to a PincusCo analysis of city data. The loan price per built square foot is $516 and the price per buildable square foot is $509 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) David Tabak signed for the borrowers with an alternate version of his name, Meir D. Tabak. The signatory for QuadReal Property Group was</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>Firebird Grove signs $20M refi with Morgan Stanley for 10 properties in Greenwich Village</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>https://www.pincusco.com/firebird-grove-signs-20m-refi-with-morgan-stanley-for-10-properties-in-greenwich-village/</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>Firebird Grove through the entity OR Patchin Place LLC as borrower signed a refi loan</t>
-        </is>
-      </c>
-      <c r="D5" t="inlineStr"/>
-      <c r="E5" t="inlineStr"/>
-      <c r="F5" t="inlineStr">
-        <is>
-          <t>PincusCo</t>
-        </is>
-      </c>
-      <c r="G5" t="inlineStr">
-        <is>
-          <t>PincusCo - Home</t>
-        </is>
-      </c>
-      <c r="H5" t="inlineStr">
-        <is>
-          <t>Transfers 9 Patchin Place (Credit: Google) Firebird Grove through the entity OR Patchin Place LLC as borrower signed a refi loan with lender Morgan Stanley through the entity Morgan Stanley Private Bank valued at $20 million for 10 properties with 33 residential units including the four-unit mixed-use building (S4) at 9 Patchin Place in Greenwich Village, Manhattan, five-unit residential walkup building (C2) at 7 Patchin Place in Greenwich Village, Manhattan, and 1-4 family building (A4) at 1 Patchin Place in Greenwich Village, Manhattan. The deal closed on May 20, 2026 and was recorded on June 3, 2026. The prior lender was Derby Copeland Capital which held debt that had an original loan amount of $17 million. The 10 properties have 25,647 square feet of built space and 8,464 square feet of additional air rights for a total buildable of 32,255 square feet according to a PincusCo analysis of city data. The loan price per built square foot is $779 and the price per buildable square foot is $620 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) The sign</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>Justin Management signs $63.2M refi with Chase for two properties in Penn Plaza</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>https://www.pincusco.com/justin-management-signs-63-2m-refi-with-chase-for-two-properties-in-penn-plaza/</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>Justin Management through the entity 1239 Operating LLC as borrower signed a refi loan with</t>
-        </is>
-      </c>
-      <c r="D6" t="inlineStr"/>
-      <c r="E6" t="inlineStr"/>
-      <c r="F6" t="inlineStr">
-        <is>
-          <t>PincusCo</t>
-        </is>
-      </c>
-      <c r="G6" t="inlineStr">
-        <is>
-          <t>PincusCo - Home</t>
-        </is>
-      </c>
-      <c r="H6" t="inlineStr">
-        <is>
-          <t>Transfers 856 Sixth Avenue (Credit - Cyclomedia) Justin Management through the entity 1239 Operating LLC as borrower signed a refi loan with lender JPMorgan Chase valued at $63.2 million for two properties including the office building (O6) at 856 Sixth Avenue and the retail (K4) building at 864 Sixth Avenue in Penn Plaza, Manhattan. The deal closed on May 21, 2026 and was recorded on June 3, 2026. The prior lender was First Republic Bank which held debt that had an original loan amount of $65 million provided in 2013 and 2019. The two properties have 193,000 square feet of built space and 151,540 square feet of additional air rights for a total buildable of 344,525 square feet according to a PincusCo analysis of city data. The loan price per built square foot is $327 and the price per buildable square foot is $183 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) The signatories for Justin Management were Jeffrey Justin and David Justin . The signatory for JPMorgan Chase was Ursula Flores . Prior sales, articles and revenue Out of the two properties</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>Yin Chou Hu pays $9M for potential dev site in Flushing</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>https://www.pincusco.com/yin-chou-hu-pays-9m-for-potential-dev-site-in-flushing/</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>Yin Chou Hu through the entity Northern Plaza LLC paid $9 million to the entity</t>
-        </is>
-      </c>
-      <c r="D7" t="inlineStr"/>
-      <c r="E7" t="inlineStr"/>
-      <c r="F7" t="inlineStr">
-        <is>
-          <t>PincusCo</t>
-        </is>
-      </c>
-      <c r="G7" t="inlineStr">
-        <is>
-          <t>PincusCo - Home</t>
-        </is>
-      </c>
-      <c r="H7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Transfers 146-13 Northern Boulevard (Credit - Cyclomedia) Yin Chou Hu through the entity Northern Plaza LLC paid $9 million to the entity Ric Rac North L.L.C for the retail building (K1) at 146-13 Northern Boulevard in Flushing, Queens. The expected use is ground up development, as it was marketed as a potential development site. The deal closed on May 19, 2026 and was recorded on June 4, 2026. The property has 1,710 square feet of built space and 21,541 square feet of additional air rights for a total buildable of 23,264 square feet according to a PincusCo analysis of city data. The sale price per built square foot is $5,263 and the price per buildable square foot is $386 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) The signatory for Richard Berkley and Carol Berkley was Benjamin Brash . The signatory for Yin Chou Hu was Yin Chou Hu. The contract date was February 20, 2026. Traded reported the sale as a development site. Cushman &amp; Wakefield was marketing it on Crexi as well. Prior sales, articles and revenue Prior to this transaction, PincusCo </t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>Lender Emerald Creek Capital takes title to LES office, following $32M bankruptcy</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>https://www.pincusco.com/lender-emerald-creek-capital-takes-title-to-les-office-following-32m-bankruptcy/</t>
-        </is>
-      </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>Lender Emerald Creek Capital through the entity ECC Bowery LLC, took title to the 18-unit</t>
-        </is>
-      </c>
-      <c r="D8" t="inlineStr"/>
-      <c r="E8" t="inlineStr"/>
-      <c r="F8" t="inlineStr">
-        <is>
-          <t>PincusCo</t>
-        </is>
-      </c>
-      <c r="G8" t="inlineStr">
-        <is>
-          <t>PincusCo - Home</t>
-        </is>
-      </c>
-      <c r="H8" t="inlineStr">
-        <is>
-          <t>Transfers 139 Bowery (Credit - Cyclomedia) Lender Emerald Creek Capital through the entity ECC Bowery LLC, took title to the 18-unit mixed-use building (O6) at 139 Bowery in the Lower East Side, Manhattan, with a transfer value of $49.5 million. The expected use is hold for sale. The former owner Hung Kwong Leung through the entity Global Joint Venture, Inc., filed bankruptcy a year ago following a default on a $32 million loan Emerald Creek Capital provided in 2019. The title transfer closed on May 21, 2026, and was recorded on June 4, 2026. The property has 58,390 square feet of built space according to a PincusCo analysis of city data. The sale price per built square foot is $847 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) The signatory for Hung Kwong Leung was Kevin J. Nash. The signatory for Emerald Creek Capital was Mark Penna. The contract date was May 21, 2026. Just over one year ago, Hung Kwong Leung as president of Global Joint Venture Inc., the sponsor of a mixed-use condominium project at 139 Bowery with 18 residential units, commer</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>ESRT pays $113.6M to Cohen Brothers for 2 ground leased fee properties in Manhattan</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>https://www.pincusco.com/esrt-pays-113-6m-to-cohen-brothers-for-2-ground-leased-fee-properties-in-manhattan/</t>
-        </is>
-      </c>
-      <c r="C9" t="inlineStr">
-        <is>
-          <t>Empire State Realty Trust, also known as ESRT, paid $113.6 million to Charles Cohen’s Cohen</t>
-        </is>
-      </c>
-      <c r="D9" t="inlineStr"/>
-      <c r="E9" t="inlineStr"/>
-      <c r="F9" t="inlineStr">
-        <is>
-          <t>PincusCo</t>
-        </is>
-      </c>
-      <c r="G9" t="inlineStr">
-        <is>
-          <t>PincusCo - Home</t>
-        </is>
-      </c>
-      <c r="H9" t="inlineStr">
-        <is>
-          <t>Chart_Frontpage Transfers 1400 Broadway (Credit - Cyclomedia) Empire State Realty Trust, also known as ESRT, paid $113.6 million to Charles Cohen’s Cohen Brothers Realty for two ground leased fee properties in Manhattan, in two transactions. In both cases, ESRT is the ground tenant, so with these transactions is taking full control of both properties. In the larger, Empire State Realty Trust through the entity ESRT 1400 Broadway Fee, L.L.C. paid $61.3 million to Cohen Brothers Realty through the entity 112-1400 Trade Properties LLC for the ground leased fee office building (O4) at 1400 Broadway in Garment District, Manhattan. The expected use is cash flowing. The deal closed on May 20, 2026 and was recorded on June 4, 2026. The property has 768,321 square feet of built space according to a PincusCo analysis of city data. The sale price per built square foot is $79 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) In the second, Empire State Realty Trust through the entity Esrt 112 West 34th Street Fee, L.L.C. paid $52.3 million to Cohen Brothers Real</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto update queens news 2026-06-08T16:16:08Z
</commit_message>
<xml_diff>
--- a/data/output/queens_dev_news.xlsx
+++ b/data/output/queens_dev_news.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H1"/>
+  <dimension ref="A1:H4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -467,6 +467,108 @@
       <c r="H1" s="1" t="inlineStr">
         <is>
           <t>content_preview</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>ACAN Development files plans for 36 units in Belmont</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>https://www.pincusco.com/adam-nieweg-files-plans-for-36-units-in-belmont-little-italy/</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>ACAN Development submitted a new building construction project for a 36-unit, 27,244-square-foot residential (R-2) building</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr"/>
+      <c r="E2" t="inlineStr"/>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>PincusCo</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>PincusCo - Home</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>Development 2302 Hughes Avenue axonometric diagram (Credit - Jakov Saric architect via DOB) ACAN Development submitted a new building construction project for a 36-unit, 27,244-square-foot residential (R-2) building at 2302 Hughes Avenue in Belmont, Bronx. The plan was filed on June 3, 2026. It calls for the construction of a 70-foot-tall, six-story building and was filed with the New York City Department of Buildings under job number X01337563. The project is described in the filing as: erection of a new 6 story + cellar and penthouse residential building. The applicant is the Registered Architect Jakov Saric of Node Architecture, Engineering, Consulting PC. Adam Nieweg of ACAN Development submitted the plans. The 34 apartments are distributed across floors one through six and a penthouse level. There is no retail or commercial space in the building. There are three units on the first floor, six units each on floors two to six, and a penthouse unit on the penthouse floor. ZD1 DOB Zoning Diagram 2302 Hughes Avenue</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Danil Shimonov files plans for 18 units in Briarwood</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>https://www.pincusco.com/danil-shimonov-files-plans-for-18-units-in-briarwood/</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Danil Shimonov submitted a new building construction project for a 18-unit, 14,908-square-foot residential (R-2) building</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr"/>
+      <c r="E3" t="inlineStr"/>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>PincusCo</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>PincusCo - Home</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>Development 143-08 84th Road axonometric diagram (Credit - Gerald J. Caliendo architect via DOB) Danil Shimonov submitted a new building construction project for a 18-unit, 14,908-square-foot residential (R-2) building at 143-08 84th Road in Briarwood, Queens. The plan was filed on June 2, 2026. It calls for the construction of a 58-foot-tall, six-story building and was filed with the New York City Department of Buildings under job number Q01409428. The project is described in the filing as: proposed new 6-story residential building and to obtain new certificate of occupancy. The applicant is the Registered Architect Gerald Caliendo of Gerald Caliendo Architects. The 18 apartments are on floors one through six, with no retail or commercial space. There are two units on the first floor, four units on the second floor and three units each on floors three through six. ZD1 DOB Zoning Diagram 143-08 84th Road</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Apex Investments files plans for 224 units in East Flatbush</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>https://www.pincusco.com/apex-investments-files-plans-for-224-units-in-east-flatbush/</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Apex Investments submitted a new building construction project for a 224-unit, 198,437-square-foot residential (R-2) building</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr"/>
+      <c r="E4" t="inlineStr"/>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>PincusCo</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>PincusCo - Home</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>Development 530 Utica Avenue axonometric diagram, two views (Credit - Shay Alster architect via DOB) Apex Investments submitted a new building construction project for a 224-unit, 198,437-square-foot residential (R-2) building at 530 Utica Avenue in East Flatbush, Brooklyn. The plan was filed on June 4, 2026. It calls for the construction of a 177-foot-tall, fifteen-story building and was filed with the New York City Department of Buildings under job number B01400199. The project is described in the filing as: filing herewith to erect a 15 story mix use building as per plans. The applicant is the Registered Architect Shay Alster of Gf55 Architects Llp. Mimi Ho submitted the plans. ZD1 DOB Zoning Diagram 530 Utica Avenue The 16-story mixed-use building comprises 224 apartments spread across floors 2 through 15, with ground-floor retail and business offices. The cellar houses residential amenities including a laundry, playroom, lounge, and computer room, alongside mercantile storage and bike facilities.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto update queens news 2026-06-09T15:25:50Z
</commit_message>
<xml_diff>
--- a/data/output/queens_dev_news.xlsx
+++ b/data/output/queens_dev_news.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H4"/>
+  <dimension ref="A1:H9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -473,17 +473,17 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>ACAN Development files plans for 36 units in Belmont</t>
+          <t>Liberty One Group signs $9.7M refi with M&amp;T in Cypress Hills</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>https://www.pincusco.com/adam-nieweg-files-plans-for-36-units-in-belmont-little-italy/</t>
+          <t>https://www.pincusco.com/liberty-one-group-signs-9-7m-refi-with-mt-for-two-properties-in-cypress-hills/</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>ACAN Development submitted a new building construction project for a 36-unit, 27,244-square-foot residential (R-2) building</t>
+          <t>Liberty One Group through the entity 74 Eldert Realty LLC as borrower signed a refi</t>
         </is>
       </c>
       <c r="D2" t="inlineStr"/>
@@ -500,24 +500,24 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>Development 2302 Hughes Avenue axonometric diagram (Credit - Jakov Saric architect via DOB) ACAN Development submitted a new building construction project for a 36-unit, 27,244-square-foot residential (R-2) building at 2302 Hughes Avenue in Belmont, Bronx. The plan was filed on June 3, 2026. It calls for the construction of a 70-foot-tall, six-story building and was filed with the New York City Department of Buildings under job number X01337563. The project is described in the filing as: erection of a new 6 story + cellar and penthouse residential building. The applicant is the Registered Architect Jakov Saric of Node Architecture, Engineering, Consulting PC. Adam Nieweg of ACAN Development submitted the plans. The 34 apartments are distributed across floors one through six and a penthouse level. There is no retail or commercial space in the building. There are three units on the first floor, six units each on floors two to six, and a penthouse unit on the penthouse floor. ZD1 DOB Zoning Diagram 2302 Hughes Avenue</t>
+          <t>Transfers 74 Eldert Lane (Credit - Cyclomedia) Liberty One Group through the entity 74 Eldert Realty LLC as borrower signed a refi loan with lender M&amp;T Bank through the entity Manufacturers And Traders Trust Company valued at $9.7 million for two properties including the specialty building (M9) at 74 Eldert Lane in Cypress Hills, Brooklyn and industrial building (G7) at 82 Eldert Lane in Cypress Hills, Brooklyn. The deal closed on May 19, 2026 and was recorded on June 5, 2026. The prior lender was M&amp;T Bank which held debt that had an original loan amount of $7.8 million.The two properties have 15,624 square feet of built space and 3,123 square feet of additional air rights according to a PincusCo analysis of city data. The loan price per built square foot is $620 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) The signatory for Liberty One Group was Joel Shafran . The signatory for M&amp;T Bank was Adam Bavifard . Because multiple properties have been transacted, some of the following sections will follow the property with the largest assessed value, w</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Danil Shimonov files plans for 18 units in Briarwood</t>
+          <t>Vijayalayan Krishnan pays $2.5M to HAP Investments in East Harlem</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>https://www.pincusco.com/danil-shimonov-files-plans-for-18-units-in-briarwood/</t>
+          <t>https://www.pincusco.com/vijayalayan-krishnan-pays-2-5m-to-hap-investments-in-east-harlem/</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Danil Shimonov submitted a new building construction project for a 18-unit, 14,908-square-foot residential (R-2) building</t>
+          <t>Vijayalayan Krishnan through the entity 419 Tavo LLC paid $2.5 million to HAP Investments through</t>
         </is>
       </c>
       <c r="D3" t="inlineStr"/>
@@ -534,24 +534,24 @@
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>Development 143-08 84th Road axonometric diagram (Credit - Gerald J. Caliendo architect via DOB) Danil Shimonov submitted a new building construction project for a 18-unit, 14,908-square-foot residential (R-2) building at 143-08 84th Road in Briarwood, Queens. The plan was filed on June 2, 2026. It calls for the construction of a 58-foot-tall, six-story building and was filed with the New York City Department of Buildings under job number Q01409428. The project is described in the filing as: proposed new 6-story residential building and to obtain new certificate of occupancy. The applicant is the Registered Architect Gerald Caliendo of Gerald Caliendo Architects. The 18 apartments are on floors one through six, with no retail or commercial space. There are two units on the first floor, four units on the second floor and three units each on floors three through six. ZD1 DOB Zoning Diagram 143-08 84th Road</t>
+          <t>Transfers 419 East 117th Street (Credit - Cyclomedia) Vijayalayan Krishnan through the entity 419 Tavo LLC paid $2.5 million to HAP Investments through the entity E117 Mazal Holdings LLC for the eight-unit residential walkup building (C1) at 419 East 117th Street in East Harlem, Manhattan. The expected use is cash flowing. The deal closed on May 29, 2026 and was recorded on June 5, 2026. The property has 5,655 square feet of built space and 18 square feet of additional air rights for a total buildable of 5,676 square feet according to a PincusCo analysis of city data. The sale price per built square foot is $437 and the price per buildable square foot is $436 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) The seller bought the property on December 20, 2010, for $610,000. The signatory for HAP Investments was Eran Polack . The signatory for Vijayalayan Krishnan was Vijayalayan Krishnan. The contract date was February 18, 2026. Prior sales, articles and revenue Prior to this transaction, PincusCo has no record that the buyer Vijayalayan Krishnan had</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Apex Investments files plans for 224 units in East Flatbush</t>
+          <t>Kibel signs $18.5M refi with PNC Bank for 119-unit rental in Turtle Bay</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>https://www.pincusco.com/apex-investments-files-plans-for-224-units-in-east-flatbush/</t>
+          <t>https://www.pincusco.com/kibel-signs-18-5m-refi-with-pnc-bank-for-119-unit-rental-in-turtle-bay/</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Apex Investments submitted a new building construction project for a 224-unit, 198,437-square-foot residential (R-2) building</t>
+          <t>Kibel Companies through the entity Kbl 51st Strret Limited Partnership as borrower signed a refi</t>
         </is>
       </c>
       <c r="D4" t="inlineStr"/>
@@ -568,7 +568,177 @@
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>Development 530 Utica Avenue axonometric diagram, two views (Credit - Shay Alster architect via DOB) Apex Investments submitted a new building construction project for a 224-unit, 198,437-square-foot residential (R-2) building at 530 Utica Avenue in East Flatbush, Brooklyn. The plan was filed on June 4, 2026. It calls for the construction of a 177-foot-tall, fifteen-story building and was filed with the New York City Department of Buildings under job number B01400199. The project is described in the filing as: filing herewith to erect a 15 story mix use building as per plans. The applicant is the Registered Architect Shay Alster of Gf55 Architects Llp. Mimi Ho submitted the plans. ZD1 DOB Zoning Diagram 530 Utica Avenue The 16-story mixed-use building comprises 224 apartments spread across floors 2 through 15, with ground-floor retail and business offices. The cellar houses residential amenities including a laundry, playroom, lounge, and computer room, alongside mercantile storage and bike facilities.</t>
+          <t>Transfers 300 East 51st Street aka 956 Second Avenue (Credit - Cyclomedia) Kibel Companies through the entity Kbl 51st Strret Limited Partnership as borrower signed a refi loan with lender PNC Bank valued at $18.5 million for the 119-unit residential elevator building (D6) at 956 Second Avenue in Turtle Bay, Manhattan. The deal closed on June 1, 2026 and was recorded on June 5, 2026. The prior lender was Series 2016-K57 serviced by Trimont which held debt that had an original loan amount of $18 million. The property has 115,860 square feet of built space according to a PincusCo analysis of city data. The loan price per built square foot is $159 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) The signatory for Kibel Companies, which is also known as Kibel Company, was Lee Ryback. The signatory for PNC Bank was Tara Suaye. Prior sales, articles and revenue The owners according to the Department of Housing Preservation and Development includes Peter Levenson, head officer and Serso Cordero, site manager. The business entities are Kibel Companies Llc a</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Rotem Cohen files plans for 12 units in Greenpoint</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>https://www.pincusco.com/rotem-cohen-files-plans-for-12-units-in-greenpoint/</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Rotem Cohen submitted a new building construction project for a 12-unit, 22,272-square-foot residential (R-2) building</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr"/>
+      <c r="E5" t="inlineStr"/>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>PincusCo</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>PincusCo - Home</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>Development 508 Graham Avenue axonometric diagram (Credit - Stephen Conte architect via DOB) Rotem Cohen submitted a new building construction project for a 12-unit, 22,272-square-foot residential (R-2) building at 508 Graham Avenue in Greenpoint, Brooklyn. The plan was filed on June 3, 2026. It calls for the construction of a 55-foot-tall, five-story building and was filed with the New York City Department of Buildings under job number B01404767. The project is described in the filing as: propose new 5-story residential building as per plan. obtain new c of o.. The applicant is the Registered Architect Stephen Conte of StudiosC Architecture PLLC. The first floor has a gym for the residents and one apartment. Floors two to four have three apartments each. The fifth and penthouse floors each have half of a single duplex apartment. There is no retail or commercial space in the building. The most recent ownership change was in 2012 when Kwong C. Chiu as signatory for both buyer and seller, transferred ownership from one entity to another in a zero dollar exchange. 508 Graham Avenue</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>HUBB NYC pays $6.8M to GAIA Real Estate for 16-unit UWS walkup</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>https://www.pincusco.com/hubb-nyc-pays-6-8m-to-gaia-real-estate-for-16-unit-uws-walkup/</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>HUBB NYC through the entity 12 W. 104th St LLC paid $6.8 million to GAIA</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr"/>
+      <c r="E6" t="inlineStr"/>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>PincusCo</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>PincusCo - Home</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>Transfers 12 West 104th Street (Credit - Cyclomedia) HUBB NYC through the entity 12 W. 104th St LLC paid $6.8 million to GAIA Real Estate through the entity 12 West 104 Street Owner LLC for the 16-unit residential walkup building (C4) at 12 West 104th Street in Upper West Side, Manhattan. The expected use is cash flowing. The deal closed on May 21, 2026 and was recorded on June 8, 2026. The property has 11,265 square feet of built space according to a PincusCo analysis of city data. The sale price per built square foot is $608 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) The seller bought the property on June 11, 2019, for $8.1 million. The signatory for GAIA Real Estate was Linyun Sun. The signatory for HUBB NYC was John P. McCarthy and Steve Dluzyn . The contract date was April 29, 2026. Prior sales, articles and revenue Prior to this transaction, PincusCo has records that the buyer HUBB NYC purchased eight properties in seven transactions for a total of $239.8 million and sold eight properties in seven transactions for a total of $34.2 millio</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Breaking Ground pays $12M for LIC dev site, owned for 76 years</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>https://www.pincusco.com/breaking-ground-pays-12m-for-lic-dev-site-owned-for-76-years/</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Breaking Ground through the entity Breaking Ground II Housing Development Fund Corp paid $12 million</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr"/>
+      <c r="E7" t="inlineStr"/>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>PincusCo</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>PincusCo - Home</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>Transfers 37-25 21st Street (Credit - Cyclomedia) Breaking Ground through the entity Breaking Ground II Housing Development Fund Corp paid $12 million to Lupoli Holdings Partnership through the entity Yardley Associates, LLC for the industrial building (G2) at 37-25 21st Street, the industrial building (G2) at 37-07 21st Street, and development parcel (V1) at 37-12 Rear 22nd Street in Long Island City, Queens. The expected use is ground up development. The deal closed on May 19, 2026 and was recorded on June 8, 2026. The three properties have 9,032 square feet of built space and 106,902 square feet of additional air rights for a total buildable of 115,930 square feet according to a PincusCo analysis of city data. The sale price per built square foot is $1,328 and the price per buildable square foot is $103 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) The signatory for Lupoli Holdings Partnership was Joseph Onorato . The signatory for Breaking Ground was David Walsh . The contract date was November 25, 2025. The Lupoli family’s Charles Lupoli acq</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>David Brecher pays $13.5M for the 49-unit rental in Clinton Hill</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>https://www.pincusco.com/david-brecher-pays-13-5m-for-the-49-unit-rental-in-clinton-hill/</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>David Brecher through the entity Brelan 420 Clinton LLC paid $13.5 million to Leslie Westreich</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr"/>
+      <c r="E8" t="inlineStr"/>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>PincusCo</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>PincusCo - Home</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>Transfers 419 Vanderbilt Avenue (Credit - Cyclomedia) David Brecher through the entity Brelan 420 Clinton LLC paid $13.5 million to Leslie Westreich through the entity 420 Clinton LLC for the 49-unit residential elevator building (D3) at 419 Vanderbilt Avenue in Clinton Hill, Brooklyn. The expected use is cash flowing. The deal closed on May 29, 2026 and was recorded on June 8, 2026. The property has 60,720 square feet of built space according to a PincusCo analysis of city data. The sale price per built square foot is $222 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) The seller bought the property on March 26, 2008, for $7.5 million. The signatory for Leslie Westreich was Leslie Westreich. The signatory for David Brecher was David Brecher. The contract date was May 29, 2026. To finance the purchase, David Brecher borrowed $7.9 million from CBRE Capital Markets . The signatory for the lender was Adam Holmes . Prior sales, articles and revenue Prior to this transaction, PincusCo has records that the buyer David Brecher purchased two properties in</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Sanders Investments sells 10-unit walkup in Chelsea</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>https://www.pincusco.com/sanders-investments-sells-10-unit-walkup-in-chelsea/</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>The entity Leoni Realty LLC paid $2.9 million to Sanders Investments through the entity London</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr"/>
+      <c r="E9" t="inlineStr"/>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>PincusCo</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>PincusCo - Home</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>Transfers 406 W 22St (Credit - Cyclomedia) The entity Leoni Realty LLC paid $2.9 million to Sanders Investments through the entity London Apartments II LLC for the 10-unit residential walkup building (C5) at 406 W 22St in Chelsea, Manhattan. The expected use is cash flowing. The deal closed on May 27, 2026 and was recorded on June 8, 2026. The property has 3,990 square feet of built space according to a PincusCo analysis of city data. The sale price per built square foot is $726 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) The seller bought the property on March 23, 2007, for $2.6 million. The signatory for Sanders Investments was Susan Sanders . The signatory for the buyer was Francis Patrick Bowers. The contract date was April 21, 2026. Prior sales, articles and revenue Prior to this transaction, PincusCo has no record that the buyer Francis Patrick Bowers had purchased any other properties and has no record it sold any properties over the past 24 months. The seller Sanders Investments had not purchased any other properties and had not sold an</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto update queens news 2026-06-10T16:05:05Z
</commit_message>
<xml_diff>
--- a/data/output/queens_dev_news.xlsx
+++ b/data/output/queens_dev_news.xlsx
@@ -473,17 +473,17 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Liberty One Group signs $9.7M refi with M&amp;T in Cypress Hills</t>
+          <t>David Tabak, Borough Developers sign $23.5M loan for 99-unit Williamsburg project</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>https://www.pincusco.com/liberty-one-group-signs-9-7m-refi-with-mt-for-two-properties-in-cypress-hills/</t>
+          <t>https://www.pincusco.com/david-tabak-borough-developers-sign-23-5m-loan-for-99-unit-williamsburg-project/</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Liberty One Group through the entity 74 Eldert Realty LLC as borrower signed a refi</t>
+          <t>David Tabak and Borough Developers through the entity One Fifty Nine B LLC as borrower</t>
         </is>
       </c>
       <c r="D2" t="inlineStr"/>
@@ -500,24 +500,24 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>Transfers 74 Eldert Lane (Credit - Cyclomedia) Liberty One Group through the entity 74 Eldert Realty LLC as borrower signed a refi loan with lender M&amp;T Bank through the entity Manufacturers And Traders Trust Company valued at $9.7 million for two properties including the specialty building (M9) at 74 Eldert Lane in Cypress Hills, Brooklyn and industrial building (G7) at 82 Eldert Lane in Cypress Hills, Brooklyn. The deal closed on May 19, 2026 and was recorded on June 5, 2026. The prior lender was M&amp;T Bank which held debt that had an original loan amount of $7.8 million.The two properties have 15,624 square feet of built space and 3,123 square feet of additional air rights according to a PincusCo analysis of city data. The loan price per built square foot is $620 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) The signatory for Liberty One Group was Joel Shafran . The signatory for M&amp;T Bank was Adam Bavifard . Because multiple properties have been transacted, some of the following sections will follow the property with the largest assessed value, w</t>
+          <t>Transfers 159 Broadway axonometric diagram (Credit - Diagram by Paul D. Taylor architect via DOB, street view by Cyclomedia) David Tabak and Borough Developers through the entity One Fifty Nine B LLC as borrower signed a new construction loan with lender Valley National Bank valued at $23.5 million for a 99-unit development site at 159 Broadway in Williamsburg, Brooklyn. On this site, there is a new building project, B01327363, for a 99-unit, 97,166 square-foot residential (R-2) building submitted by Borough Developers and filed by Mendel Berkowitz with plans filed December 11, 2025 and it has not been permitted yet. David Tabak as ground tenant signed a lease valued at $3.1 million with fee owner Joyland Management in January 2026. The loan closed on May 5, 2026 and was recorded on June 8, 2026. The loan price per planned development square foot is $242 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) This loan price does not take into consideration the $30 million in debt Joyland Management borrowed. The signatory for David Tabak and Borough Devel</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Vijayalayan Krishnan pays $2.5M to HAP Investments in East Harlem</t>
+          <t>Pan Am Equities to add 15 apartments to Greenwich Village rental</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>https://www.pincusco.com/vijayalayan-krishnan-pays-2-5m-to-hap-investments-in-east-harlem/</t>
+          <t>https://www.pincusco.com/pan-am-equities-to-add-15-apartments-to-greenwich-village-rental/</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Vijayalayan Krishnan through the entity 419 Tavo LLC paid $2.5 million to HAP Investments through</t>
+          <t>The Manocherian family’s Pan Am Equities submitted a major alteration application to add 15 units</t>
         </is>
       </c>
       <c r="D3" t="inlineStr"/>
@@ -534,24 +534,24 @@
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>Transfers 419 East 117th Street (Credit - Cyclomedia) Vijayalayan Krishnan through the entity 419 Tavo LLC paid $2.5 million to HAP Investments through the entity E117 Mazal Holdings LLC for the eight-unit residential walkup building (C1) at 419 East 117th Street in East Harlem, Manhattan. The expected use is cash flowing. The deal closed on May 29, 2026 and was recorded on June 5, 2026. The property has 5,655 square feet of built space and 18 square feet of additional air rights for a total buildable of 5,676 square feet according to a PincusCo analysis of city data. The sale price per built square foot is $437 and the price per buildable square foot is $436 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) The seller bought the property on December 20, 2010, for $610,000. The signatory for HAP Investments was Eran Polack . The signatory for Vijayalayan Krishnan was Vijayalayan Krishnan. The contract date was February 18, 2026. Prior sales, articles and revenue Prior to this transaction, PincusCo has no record that the buyer Vijayalayan Krishnan had</t>
+          <t xml:space="preserve">Development 24-26 East 13th Street (Credit - Cyclomedia) The Manocherian family’s Pan Am Equities submitted a major alteration application to add 15 units to the existing 24-unit rental building at 24-26 East 13th Street in Greenwich Village, Manhattan, to result in a total of 39 residential units. The plan was filed on June 8, 2026. It calls for the alteration of uses in the 59-foot-tall, six-story building and was filed with the New York City Department of Buildings under job number M01302381. The project is described in the filing as: residential conversion on mezzanine, 2nd and 3rd floors as per plans submitted herewith, work includes removal and construction of non-bearing partitions, flooring lighting and ceiling, and replace windows at mezzanine. The applicant is the Registered Architect Frank Denner of Frank Denner Architect. Geoff Ringler of Pan Am Equities submitted the plans. The apartments will replace space previously occupied by the New York Health &amp; Racquet Club, which closed in 2020, amid the Covid closures. Space on the first floor and lower level will remain a gym or health club use. The plans call for the lower portion of two duplexes on the mezzanine level, the </t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Kibel signs $18.5M refi with PNC Bank for 119-unit rental in Turtle Bay</t>
+          <t>Raimondo Zaytoune pays $3.6M to Jemal family for retail in Sheepshead Bay</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>https://www.pincusco.com/kibel-signs-18-5m-refi-with-pnc-bank-for-119-unit-rental-in-turtle-bay/</t>
+          <t>https://www.pincusco.com/raimondo-zaytoune-pays-3-6m-to-jemal-family-for-retail-in-sheepshead-bay/</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Kibel Companies through the entity Kbl 51st Strret Limited Partnership as borrower signed a refi</t>
+          <t>Raimondo Zaytoune through the entity Niceland Realty LLC paid $3.6 million to Jemal family members</t>
         </is>
       </c>
       <c r="D4" t="inlineStr"/>
@@ -568,24 +568,24 @@
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>Transfers 300 East 51st Street aka 956 Second Avenue (Credit - Cyclomedia) Kibel Companies through the entity Kbl 51st Strret Limited Partnership as borrower signed a refi loan with lender PNC Bank valued at $18.5 million for the 119-unit residential elevator building (D6) at 956 Second Avenue in Turtle Bay, Manhattan. The deal closed on June 1, 2026 and was recorded on June 5, 2026. The prior lender was Series 2016-K57 serviced by Trimont which held debt that had an original loan amount of $18 million. The property has 115,860 square feet of built space according to a PincusCo analysis of city data. The loan price per built square foot is $159 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) The signatory for Kibel Companies, which is also known as Kibel Company, was Lee Ryback. The signatory for PNC Bank was Tara Suaye. Prior sales, articles and revenue The owners according to the Department of Housing Preservation and Development includes Peter Levenson, head officer and Serso Cordero, site manager. The business entities are Kibel Companies Llc a</t>
+          <t>Transfers 3696 Nostrand Avenue (Credit - Cyclomedia) Raimondo Zaytoune through the entity Niceland Realty LLC paid $3.6 million to Jemal family members who lead ISJ Management and JJ Operating through the entity Jelco Nostrand LLC (and others) for the retail (K1) at 3696 Nostrand Avenue in Sheepshead Bay, Brooklyn. The expected use is cash flowing. The deal closed on April 27, 2026 and was recorded on June 9, 2026. The property has 9,626 square feet of built space and 2,111 square feet of additional air rights for a total buildable of 11,731 square feet according to a PincusCo analysis of city data. The sale price per built square foot is $373 and the price per buildable square foot is $306 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) The signatory for ISJ Management and JJ Operating was Isaac S. Jemal , Samuel J. Jemal , and Robert Spiegelman . The signatory for Raimondo Zaytoune was Raimondo Zaytoune. The contract date was February 5, 2026. Prior sales, articles and revenue Prior to this transaction, PincusCo has records that the buyer Raimond</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Rotem Cohen files plans for 12 units in Greenpoint</t>
+          <t>Namdar’s $275M purchase of office in Midtown West from ESRT is recorded</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>https://www.pincusco.com/rotem-cohen-files-plans-for-12-units-in-greenpoint/</t>
+          <t>https://www.pincusco.com/namdar-realty-group-pays-275m-to-esrt-for-office-in-midtown-west/</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Rotem Cohen submitted a new building construction project for a 12-unit, 22,272-square-foot residential (R-2) building</t>
+          <t>Namdar Realty Group through the entity Fifty Seventh 8th Realty LLC paid $275 million to</t>
         </is>
       </c>
       <c r="D5" t="inlineStr"/>
@@ -602,24 +602,24 @@
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>Development 508 Graham Avenue axonometric diagram (Credit - Stephen Conte architect via DOB) Rotem Cohen submitted a new building construction project for a 12-unit, 22,272-square-foot residential (R-2) building at 508 Graham Avenue in Greenpoint, Brooklyn. The plan was filed on June 3, 2026. It calls for the construction of a 55-foot-tall, five-story building and was filed with the New York City Department of Buildings under job number B01404767. The project is described in the filing as: propose new 5-story residential building as per plan. obtain new c of o.. The applicant is the Registered Architect Stephen Conte of StudiosC Architecture PLLC. The first floor has a gym for the residents and one apartment. Floors two to four have three apartments each. The fifth and penthouse floors each have half of a single duplex apartment. There is no retail or commercial space in the building. The most recent ownership change was in 2012 when Kwong C. Chiu as signatory for both buyer and seller, transferred ownership from one entity to another in a zero dollar exchange. 508 Graham Avenue</t>
+          <t>Transfers 250 West 57th Street (Credit - Cyclomedia) Namdar Realty Group through the entity Fifty Seventh 8th Realty LLC paid $275 million to Empire State Realty Trust through the entity ESRT 250 West 57th St., L.L.C. for the office building (O4) at 250 West 57th Street in Midtown West, Manhattan. The expected use is cash flowing. The deal closed on June 1, 2026 and was recorded on June 9, 2026. The property has 435,677 square feet of built space according to a PincusCo analysis of city data. The sale price per built square foot is $631 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) The Real Deal reported on this in April after it went into contract. The signatory for Empire State Realty Trust was Stephen V. Horn . The signatory for Namdar Realty Group was Igal Namdar . The contract date was April 1, 2026. Namdar Realty Group also assumed a $180 million securitized mortgage, Series 2020-BNK-29. Prior sales, articles and revenue</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>HUBB NYC pays $6.8M to GAIA Real Estate for 16-unit UWS walkup</t>
+          <t>Restaurateurs pay $5.9M to Stephen L. Green for retail in Greenwich Village, 4th buy</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>https://www.pincusco.com/hubb-nyc-pays-6-8m-to-gaia-real-estate-for-16-unit-uws-walkup/</t>
+          <t>https://www.pincusco.com/restaurateurs-pay-5-9m-to-stephen-l-green-for-retail-in-greenwich-village-2nd-buy/</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>HUBB NYC through the entity 12 W. 104th St LLC paid $6.8 million to GAIA</t>
+          <t>The restaurateur-owned Hammock Development through the entity 12 East 12th LLC paid $5.9 million to</t>
         </is>
       </c>
       <c r="D6" t="inlineStr"/>
@@ -636,24 +636,24 @@
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>Transfers 12 West 104th Street (Credit - Cyclomedia) HUBB NYC through the entity 12 W. 104th St LLC paid $6.8 million to GAIA Real Estate through the entity 12 West 104 Street Owner LLC for the 16-unit residential walkup building (C4) at 12 West 104th Street in Upper West Side, Manhattan. The expected use is cash flowing. The deal closed on May 21, 2026 and was recorded on June 8, 2026. The property has 11,265 square feet of built space according to a PincusCo analysis of city data. The sale price per built square foot is $608 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) The seller bought the property on June 11, 2019, for $8.1 million. The signatory for GAIA Real Estate was Linyun Sun. The signatory for HUBB NYC was John P. McCarthy and Steve Dluzyn . The contract date was April 29, 2026. Prior sales, articles and revenue Prior to this transaction, PincusCo has records that the buyer HUBB NYC purchased eight properties in seven transactions for a total of $239.8 million and sold eight properties in seven transactions for a total of $34.2 millio</t>
+          <t>Transfers 12 East 12th Street (Credit - Cyclomedia) The restaurateur-owned Hammock Development through the entity 12 East 12th LLC paid $5.9 million to SL Green Realty founder Stephen L. Green through the entity 12/12 Realty Associates LLC for the retail condo at 12 East 12th Street in Greenwich Village, Manhattan. The expected use is owner-occupied. This is their fourth purchase since 2022. Crain’s New York reported on the transaction yesterday. The buyers Stefano Secchi and David Switzer of Hammock Development, own the Michelin-starred restaurant Rezdora at 27 East 20th Street. They own that building and bought the adjacent building at 25 East 20th Street, last year for $6 million. They also bought 86 University Place for $8 million last year, and 913 Broadway in 2022 for $7.5 million. The deal closed on June 5, 2026 and was recorded on June 9, 2026. The property has 4,500 square feet of built space according to a PincusCo analysis of city data. The sale price per built square foot is $1,311 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) The sig</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Breaking Ground pays $12M for LIC dev site, owned for 76 years</t>
+          <t>Imperial Sterling pays $15.1M to Bluejay Management for office in Flatiron District</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>https://www.pincusco.com/breaking-ground-pays-12m-for-lic-dev-site-owned-for-76-years/</t>
+          <t>https://www.pincusco.com/imperial-sterling-pays-15-1m-to-bluejay-management-for-office-in-flatiron-district/</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Breaking Ground through the entity Breaking Ground II Housing Development Fund Corp paid $12 million</t>
+          <t>Imperial Sterling through the entity 22w23, LLC paid $15.1 million to Bluejay Management, Noah Spiegel,</t>
         </is>
       </c>
       <c r="D7" t="inlineStr"/>
@@ -670,24 +670,24 @@
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>Transfers 37-25 21st Street (Credit - Cyclomedia) Breaking Ground through the entity Breaking Ground II Housing Development Fund Corp paid $12 million to Lupoli Holdings Partnership through the entity Yardley Associates, LLC for the industrial building (G2) at 37-25 21st Street, the industrial building (G2) at 37-07 21st Street, and development parcel (V1) at 37-12 Rear 22nd Street in Long Island City, Queens. The expected use is ground up development. The deal closed on May 19, 2026 and was recorded on June 8, 2026. The three properties have 9,032 square feet of built space and 106,902 square feet of additional air rights for a total buildable of 115,930 square feet according to a PincusCo analysis of city data. The sale price per built square foot is $1,328 and the price per buildable square foot is $103 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) The signatory for Lupoli Holdings Partnership was Joseph Onorato . The signatory for Breaking Ground was David Walsh . The contract date was November 25, 2025. The Lupoli family’s Charles Lupoli acq</t>
+          <t>Transfers 22 West 23rd Street (Credit - Cyclomedia) Imperial Sterling through the entity 22w23, LLC paid $15.1 million to Bluejay Management, Noah Spiegel, and David Spiegel through the entity Bj23 Partners LLC for the office building (O5) at 22 West 23rd Street in Flatiron District, Manhattan. The expected use is cash flowing. The deal closed on June 2, 2026 and was recorded on June 9, 2026. The property has 13,125 square feet of built space and 14,516 square feet of additional air rights for a total buildable of 27,650 square feet according to a PincusCo analysis of city data. The sale price per built square foot is $1,146 and the price per buildable square foot is $544 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) The seller bought the property on September 14, 2023, for $9.7 million. The signatory for Bluejay Management was Marc Jacobwitz, Noah Spiegel, and David Spiegel. The signatory for Imperial Sterling was Jerrold Levy . The contract date was February 24, 2026. Prior sales, articles and revenue Prior to this transaction, PincusCo has rec</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>David Brecher pays $13.5M for the 49-unit rental in Clinton Hill</t>
+          <t>Moinian Group signs $240M loan at new 250-unit rental in FiDi</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>https://www.pincusco.com/david-brecher-pays-13-5m-for-the-49-unit-rental-in-clinton-hill/</t>
+          <t>https://www.pincusco.com/moinian-group-signs-240m-loan-at-new-250-unit-rental-in-fidi/</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>David Brecher through the entity Brelan 420 Clinton LLC paid $13.5 million to Leslie Westreich</t>
+          <t>Moinian Group through the entity 102-110 John Mazal LLC as borrower signed a refi loan</t>
         </is>
       </c>
       <c r="D8" t="inlineStr"/>
@@ -704,24 +704,24 @@
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>Transfers 419 Vanderbilt Avenue (Credit - Cyclomedia) David Brecher through the entity Brelan 420 Clinton LLC paid $13.5 million to Leslie Westreich through the entity 420 Clinton LLC for the 49-unit residential elevator building (D3) at 419 Vanderbilt Avenue in Clinton Hill, Brooklyn. The expected use is cash flowing. The deal closed on May 29, 2026 and was recorded on June 8, 2026. The property has 60,720 square feet of built space according to a PincusCo analysis of city data. The sale price per built square foot is $222 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) The seller bought the property on March 26, 2008, for $7.5 million. The signatory for Leslie Westreich was Leslie Westreich. The signatory for David Brecher was David Brecher. The contract date was May 29, 2026. To finance the purchase, David Brecher borrowed $7.9 million from CBRE Capital Markets . The signatory for the lender was Adam Holmes . Prior sales, articles and revenue Prior to this transaction, PincusCo has records that the buyer David Brecher purchased two properties in</t>
+          <t>Transfers 110 John Street (Credit - Cyclomedia) Moinian Group through the entity 102-110 John Mazal LLC as borrower signed a refi loan with lender Acore Capital through the entity ACP III REIT JPM, LLC valued at $240 million for the 250-unit residential elevator building (D8) at 110 John Street in Financial District, Manhattan. On the lot, there was a new building construction project, 121188053, for a 250-unit, 213,017 square-foot residential (R-2) building. The project was submitted by Moinian Group and filed by Aron Kirsch with plans filed March 27, 2018 and permitted August 25, 2023. The city issued an initial certificate of occupancy in January 2026. The deal closed on June 1, 2026 and was recorded on June 8, 2026. The prior lender was BDT &amp; MSD Partners which held debt that had an original loan amount of $169 million. The property has 235,688 square feet of built space according to a PincusCo analysis of city data. The loan price per built square foot is $1,018 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) The signatory for Moinian Group wa</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Sanders Investments sells 10-unit walkup in Chelsea</t>
+          <t>Red Apple Group signs $83.5M refi for 205-unit rental in Downtown Brooklyn</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>https://www.pincusco.com/sanders-investments-sells-10-unit-walkup-in-chelsea/</t>
+          <t>https://www.pincusco.com/red-apple-group-signs-83-5m-refi-for-205-unit-rental-in-downtown-brooklyn/</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>The entity Leoni Realty LLC paid $2.9 million to Sanders Investments through the entity London</t>
+          <t>Red Apple Group through the entity Red Apple 81 Fleet Place Development, LLC as borrower</t>
         </is>
       </c>
       <c r="D9" t="inlineStr"/>
@@ -738,7 +738,7 @@
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>Transfers 406 W 22St (Credit - Cyclomedia) The entity Leoni Realty LLC paid $2.9 million to Sanders Investments through the entity London Apartments II LLC for the 10-unit residential walkup building (C5) at 406 W 22St in Chelsea, Manhattan. The expected use is cash flowing. The deal closed on May 27, 2026 and was recorded on June 8, 2026. The property has 3,990 square feet of built space according to a PincusCo analysis of city data. The sale price per built square foot is $726 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) The seller bought the property on March 23, 2007, for $2.6 million. The signatory for Sanders Investments was Susan Sanders . The signatory for the buyer was Francis Patrick Bowers. The contract date was April 21, 2026. Prior sales, articles and revenue Prior to this transaction, PincusCo has no record that the buyer Francis Patrick Bowers had purchased any other properties and has no record it sold any properties over the past 24 months. The seller Sanders Investments had not purchased any other properties and had not sold an</t>
+          <t>Transfers 81 Fleet Place (Credit - Cyclomedia) Red Apple Group through the entity Red Apple 81 Fleet Place Development, LLC as borrower signed a refi loan with lender U.S. Bank valued at $83.5 million for the 205-unit residential elevator building (D6) at 81 Fleet Place in Downtown Brooklyn, Brooklyn. The deal closed on May 28, 2026 and was recorded on June 8, 2026. The prior lender was U.S. Bank which held debt that had provided an original loan amount of $86 million in May 2019. The property has 265,417 square feet of built space according to a PincusCo analysis of city data. The loan price per built square foot is $314 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) The signatory for Red Apple Group was John Catsimatidis . The signatory for U.S. Bank was Matthew Gumnic . Prior sales, articles and revenue The owners according to the Department of Housing Preservation and Development includes John Catsimatidis, head officer and Charles D’Amico , officer. The business entities are Red Apple Property Management LLC and Red Apple 81 Fleet Place Devel</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto update queens news 2026-06-11T16:18:58Z
</commit_message>
<xml_diff>
--- a/data/output/queens_dev_news.xlsx
+++ b/data/output/queens_dev_news.xlsx
@@ -473,17 +473,17 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>David Tabak, Borough Developers sign $23.5M loan for 99-unit Williamsburg project</t>
+          <t>Yellow Jacket Ventures pays $2.5M for 49-unit rental in Soundview</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>https://www.pincusco.com/david-tabak-borough-developers-sign-23-5m-loan-for-99-unit-williamsburg-project/</t>
+          <t>https://www.pincusco.com/yellow-jacket-ventures-pays-2-5m-for-49-unit-rental-in-soundview/</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>David Tabak and Borough Developers through the entity One Fifty Nine B LLC as borrower</t>
+          <t>Yellow Jacket Ventures through the entity Commonwealth Bronx LLC paid $2.5 million to Marco Cepeda</t>
         </is>
       </c>
       <c r="D2" t="inlineStr"/>
@@ -500,24 +500,24 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>Transfers 159 Broadway axonometric diagram (Credit - Diagram by Paul D. Taylor architect via DOB, street view by Cyclomedia) David Tabak and Borough Developers through the entity One Fifty Nine B LLC as borrower signed a new construction loan with lender Valley National Bank valued at $23.5 million for a 99-unit development site at 159 Broadway in Williamsburg, Brooklyn. On this site, there is a new building project, B01327363, for a 99-unit, 97,166 square-foot residential (R-2) building submitted by Borough Developers and filed by Mendel Berkowitz with plans filed December 11, 2025 and it has not been permitted yet. David Tabak as ground tenant signed a lease valued at $3.1 million with fee owner Joyland Management in January 2026. The loan closed on May 5, 2026 and was recorded on June 8, 2026. The loan price per planned development square foot is $242 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) This loan price does not take into consideration the $30 million in debt Joyland Management borrowed. The signatory for David Tabak and Borough Devel</t>
+          <t>Transfers 1326 Commonwealth Avenue (Credit - Cyclomedia) Yellow Jacket Ventures through the entity Commonwealth Bronx LLC paid $2.5 million to Marco Cepeda through the entity 2332 Walton Realty Inc. for the 49-unit residential elevator building (D1) at 1326 Commonwealth in Soundview, Bronx. The expected use is cash flowing. The deal closed on May 28, 2026 and was recorded on June 9, 2026. The property has 35,624 square feet of built space according to a PincusCo analysis of city data. The sale price per built square foot is $68 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) The seller bought the property on May 31, 2007, for $3.9 million. The signatory for Marco Cepeda was Marco Cepeda. The signatory for Yellow Jacket Ventures was Akiva J. Kurland . The contract date was April 27, 2026. Prior sales, articles and revenue Prior to this transaction, PincusCo has records that the buyer Yellow Jacket Ventures purchased two properties in two transactions for a total of $12.4 million and has no record it sold any properties over the past 24 months. The s</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Pan Am Equities to add 15 apartments to Greenwich Village rental</t>
+          <t>Vega sells single-family conversion for $16M in Cobble Hill, was $3.85M in 2020</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>https://www.pincusco.com/pan-am-equities-to-add-15-apartments-to-greenwich-village-rental/</t>
+          <t>https://www.pincusco.com/vega-sells-single-family-conversion-for-16m-in-cobble-hill-was-3-85m-in-2020/</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>The Manocherian family’s Pan Am Equities submitted a major alteration application to add 15 units</t>
+          <t>The entity Cobble Chill LLC in care of Sullivan &amp; Cromwell paid $16 million to</t>
         </is>
       </c>
       <c r="D3" t="inlineStr"/>
@@ -534,24 +534,24 @@
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Development 24-26 East 13th Street (Credit - Cyclomedia) The Manocherian family’s Pan Am Equities submitted a major alteration application to add 15 units to the existing 24-unit rental building at 24-26 East 13th Street in Greenwich Village, Manhattan, to result in a total of 39 residential units. The plan was filed on June 8, 2026. It calls for the alteration of uses in the 59-foot-tall, six-story building and was filed with the New York City Department of Buildings under job number M01302381. The project is described in the filing as: residential conversion on mezzanine, 2nd and 3rd floors as per plans submitted herewith, work includes removal and construction of non-bearing partitions, flooring lighting and ceiling, and replace windows at mezzanine. The applicant is the Registered Architect Frank Denner of Frank Denner Architect. Geoff Ringler of Pan Am Equities submitted the plans. The apartments will replace space previously occupied by the New York Health &amp; Racquet Club, which closed in 2020, amid the Covid closures. Space on the first floor and lower level will remain a gym or health club use. The plans call for the lower portion of two duplexes on the mezzanine level, the </t>
+          <t>Transfers 205 Clinton Street (Credit - Cyclomedia) The entity Cobble Chill LLC in care of Sullivan &amp; Cromwell paid $16 million to Vega Management through the entity 205 Clinton Street, LLC for the single-family building (A4) at 205 Clinton Street in Cobble Hill, Brooklyn, converted from a four-family. The expected use is cash flowing. The deal closed on May 26, 2026 and was recorded on June 9, 2026. The property has 4,935 square feet of built space and 540 square feet of additional air rights for a total buildable of 5,467 square feet according to a PincusCo analysis of city data. The sale price per built square foot is $3,242 and the price per buildable square foot is $2,926 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) The sellers bought the property on June 30, 2020, for $3.85 million. The signatory for Vega Management was Allen Schifino . The signatory for Sullivan &amp; Cromwell registered buyer was Alison Hirsch. The contract date was May 5, 2026. Brandon Hornbeck of 205 Clinton Street, LLC submitted a major alteration application for the conve</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Raimondo Zaytoune pays $3.6M to Jemal family for retail in Sheepshead Bay</t>
+          <t>Isaac Friedman files plans for 20 units in East Flatbush</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>https://www.pincusco.com/raimondo-zaytoune-pays-3-6m-to-jemal-family-for-retail-in-sheepshead-bay/</t>
+          <t>https://www.pincusco.com/isaac-friedman-files-plans-for-20-units-in-east-flatbush/</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Raimondo Zaytoune through the entity Niceland Realty LLC paid $3.6 million to Jemal family members</t>
+          <t>Isaac Friedman submitted a new building construction project for a 20-unit, 13,627-square-foot residential (R-2) building</t>
         </is>
       </c>
       <c r="D4" t="inlineStr"/>
@@ -568,24 +568,24 @@
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>Transfers 3696 Nostrand Avenue (Credit - Cyclomedia) Raimondo Zaytoune through the entity Niceland Realty LLC paid $3.6 million to Jemal family members who lead ISJ Management and JJ Operating through the entity Jelco Nostrand LLC (and others) for the retail (K1) at 3696 Nostrand Avenue in Sheepshead Bay, Brooklyn. The expected use is cash flowing. The deal closed on April 27, 2026 and was recorded on June 9, 2026. The property has 9,626 square feet of built space and 2,111 square feet of additional air rights for a total buildable of 11,731 square feet according to a PincusCo analysis of city data. The sale price per built square foot is $373 and the price per buildable square foot is $306 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) The signatory for ISJ Management and JJ Operating was Isaac S. Jemal , Samuel J. Jemal , and Robert Spiegelman . The signatory for Raimondo Zaytoune was Raimondo Zaytoune. The contract date was February 5, 2026. Prior sales, articles and revenue Prior to this transaction, PincusCo has records that the buyer Raimond</t>
+          <t>Development 258 East 53rd Street isometric diagram (Credit - Navkiran Cheema professional engineer via DOB) Isaac Friedman submitted a new building construction project for a 20-unit, 13,627-square-foot residential (R-2) building at 258 East 53rd Street in East Flatbush, Brooklyn. The plan was filed on June 9, 2026. It calls for the construction of a 40-foot-tall, four-story building and was filed with the New York City Department of Buildings under job number B01410734. The project is described in the filing as: application filed herewith to erect a new 4-story and penthouse, 20-family residential building. The applicant is the Professional Engineer Navkiran Cheema of KMA Designs LLC. 258 East 53rd Street The neighborhood In East Flatbush, The bulk, or 32 percent of the 42.6 million square feet of commercial built space are elevator buildings, with walkup buildings next occupying 24 percent of the space. In sales, East Flatbush has near average sales volume among other neighborhoods with $489.6 million in sales volume in the last two years and is the 16th highest in Brooklyn. For development, East Flatbush has near average amount of major developments among other neighborhoods and</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Namdar’s $275M purchase of office in Midtown West from ESRT is recorded</t>
+          <t>Celaj Management pays $6.3M for 29-unit walkup in Harlem</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>https://www.pincusco.com/namdar-realty-group-pays-275m-to-esrt-for-office-in-midtown-west/</t>
+          <t>https://www.pincusco.com/celaj-management-pays-6-3m-for-29-unit-walkup-in-harlem/</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Namdar Realty Group through the entity Fifty Seventh 8th Realty LLC paid $275 million to</t>
+          <t>Celaj Management through the entity Central Park North Realty Associates LLC paid $6.3 million to</t>
         </is>
       </c>
       <c r="D5" t="inlineStr"/>
@@ -602,24 +602,24 @@
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>Transfers 250 West 57th Street (Credit - Cyclomedia) Namdar Realty Group through the entity Fifty Seventh 8th Realty LLC paid $275 million to Empire State Realty Trust through the entity ESRT 250 West 57th St., L.L.C. for the office building (O4) at 250 West 57th Street in Midtown West, Manhattan. The expected use is cash flowing. The deal closed on June 1, 2026 and was recorded on June 9, 2026. The property has 435,677 square feet of built space according to a PincusCo analysis of city data. The sale price per built square foot is $631 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) The Real Deal reported on this in April after it went into contract. The signatory for Empire State Realty Trust was Stephen V. Horn . The signatory for Namdar Realty Group was Igal Namdar . The contract date was April 1, 2026. Namdar Realty Group also assumed a $180 million securitized mortgage, Series 2020-BNK-29. Prior sales, articles and revenue</t>
+          <t xml:space="preserve">Transfers 9 Central Park North (Credit - Cyclomedia) Celaj Management through the entity Central Park North Realty Associates LLC paid $6.3 million to the Rickman family through the entity 9-11 Realty Associates, LLC for the 29-unit residential walkup building (C7) at 9 Central Park North in Harlem, Manhattan. The expected use is cash flowing. The deal closed on May 28, 2026 and was recorded on June 10, 2026. The property has 23,640 square feet of built space and 16,467 square feet of additional air rights for a total buildable of 40,135 square feet according to a PincusCo analysis of city data. The sale price per built square foot is $268 and the price per buildable square foot is $158 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) The seller bought the property on April 27, 2017, for $13.7 million. The signatory for Hale Rickman was Stephen S. Siminou . The signatory for Celaj Management was Bashkim Celaj . The contract date was June 16, 2025. Prior sales, articles and revenue Prior to this transaction, PincusCo has records that the buyer Celaj </t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Restaurateurs pay $5.9M to Stephen L. Green for retail in Greenwich Village, 4th buy</t>
+          <t>Yehudis Klein pays $9.2M for 20-unit rental in East Harlem</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>https://www.pincusco.com/restaurateurs-pay-5-9m-to-stephen-l-green-for-retail-in-greenwich-village-2nd-buy/</t>
+          <t>https://www.pincusco.com/yehudis-klein-pays-9-2m-for-residential-elevator-in-east-harlem/</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>The restaurateur-owned Hammock Development through the entity 12 East 12th LLC paid $5.9 million to</t>
+          <t>Yehudis Klein through the entity 308 Property Ny LLC paid $9.2 million to Boleslav Ryzinski</t>
         </is>
       </c>
       <c r="D6" t="inlineStr"/>
@@ -636,24 +636,24 @@
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>Transfers 12 East 12th Street (Credit - Cyclomedia) The restaurateur-owned Hammock Development through the entity 12 East 12th LLC paid $5.9 million to SL Green Realty founder Stephen L. Green through the entity 12/12 Realty Associates LLC for the retail condo at 12 East 12th Street in Greenwich Village, Manhattan. The expected use is owner-occupied. This is their fourth purchase since 2022. Crain’s New York reported on the transaction yesterday. The buyers Stefano Secchi and David Switzer of Hammock Development, own the Michelin-starred restaurant Rezdora at 27 East 20th Street. They own that building and bought the adjacent building at 25 East 20th Street, last year for $6 million. They also bought 86 University Place for $8 million last year, and 913 Broadway in 2022 for $7.5 million. The deal closed on June 5, 2026 and was recorded on June 9, 2026. The property has 4,500 square feet of built space according to a PincusCo analysis of city data. The sale price per built square foot is $1,311 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) The sig</t>
+          <t>Transfers 308 East 109th Street (Credit - Cyclomedia) Yehudis Klein through the entity 308 Property Ny LLC paid $9.2 million to Boleslav Ryzinski and Douglas Fierro through the entity 308 E 109th Street LLC for the 20-unit residential elevator building (D7) at 308 East 109th Street in East Harlem, Manhattan. The expected use is cash flowing. The deal closed on May 13, 2026 and was recorded on June 10, 2026. The property has 24,655 square feet of built space and 11,700 square feet of additional air rights for a total buildable of 36,359 square feet according to a PincusCo analysis of city data. The sale price per built square foot is $373 and the price per buildable square foot is $253 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) The seller bought the property on December 19, 2012, for $3.2 million. The signatory for Boleslav Ryzinski and Douglas Fierro was Douglas Fierro. The signatory for Yehudis Klein was Yehudis Klein. The contract date was January 16, 2026. The sellers in 2014 planned to divide the building into 20 residential condominium un</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Imperial Sterling pays $15.1M to Bluejay Management for office in Flatiron District</t>
+          <t>India-rooted spiritual group pays $11.8M for commercial condo in LIC</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>https://www.pincusco.com/imperial-sterling-pays-15-1m-to-bluejay-management-for-office-in-flatiron-district/</t>
+          <t>https://www.pincusco.com/india-rooted-spiritual-group-pays-11-8m-for-commercial-condo-in-lic/</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Imperial Sterling through the entity 22w23, LLC paid $15.1 million to Bluejay Management, Noah Spiegel,</t>
+          <t>The religious group with its origins in India, Radha Soami Satsang Beas, through the entity</t>
         </is>
       </c>
       <c r="D7" t="inlineStr"/>
@@ -670,24 +670,24 @@
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>Transfers 22 West 23rd Street (Credit - Cyclomedia) Imperial Sterling through the entity 22w23, LLC paid $15.1 million to Bluejay Management, Noah Spiegel, and David Spiegel through the entity Bj23 Partners LLC for the office building (O5) at 22 West 23rd Street in Flatiron District, Manhattan. The expected use is cash flowing. The deal closed on June 2, 2026 and was recorded on June 9, 2026. The property has 13,125 square feet of built space and 14,516 square feet of additional air rights for a total buildable of 27,650 square feet according to a PincusCo analysis of city data. The sale price per built square foot is $1,146 and the price per buildable square foot is $544 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) The seller bought the property on September 14, 2023, for $9.7 million. The signatory for Bluejay Management was Marc Jacobwitz, Noah Spiegel, and David Spiegel. The signatory for Imperial Sterling was Jerrold Levy . The contract date was February 24, 2026. Prior sales, articles and revenue Prior to this transaction, PincusCo has rec</t>
+          <t>Transfers 11-36 45th Road (Credit - Cyclomedia) The religious group with its origins in India, Radha Soami Satsang Beas, through the entity Radha Soami Society Beas-America, paid $11.8 million to Century Development Group through the entity MPS Two, LLC for a 30,548-square-foot commercial condominium unit as well as additional parking spaces, at 11-36 45th Road in Long Island City, Queens. The expected use is owner-occupied. The deal closed on May 21, 2026 and was recorded on June 10, 2026. The 13 properties have zero square feet of built space according to a PincusCo analysis of city data. The sale price per built square foot is $386 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet of the unit, 30,548, as reported in public records.) The signatory for Century Development Group was Stavroula Tsolis . The signatory for Radha Soami Satsang Beas was Rajan Shamdasani . The contract date was May 31, 2019. Prior sales, articles and revenue Prior to this transaction, PincusCo has no record that the buyer Radha Soami Satsang Beas had purchased any other properties and has no record it sold any properties over the past 24 months.</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Moinian Group signs $240M loan at new 250-unit rental in FiDi</t>
+          <t>Susan Ting, Austin Ting, pay $16.2M to ARCTRUST for retail in Unionport</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>https://www.pincusco.com/moinian-group-signs-240m-loan-at-new-250-unit-rental-in-fidi/</t>
+          <t>https://www.pincusco.com/susan-ting-austin-ting-pays-16-2m-to-arctrust-for-three-properties-in-unionport/</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Moinian Group through the entity 102-110 John Mazal LLC as borrower signed a refi loan</t>
+          <t>Susan Ting and Austin Ting through the entity Jackson Ht. Roosevelt Development Corp. paid $16.2</t>
         </is>
       </c>
       <c r="D8" t="inlineStr"/>
@@ -704,24 +704,24 @@
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>Transfers 110 John Street (Credit - Cyclomedia) Moinian Group through the entity 102-110 John Mazal LLC as borrower signed a refi loan with lender Acore Capital through the entity ACP III REIT JPM, LLC valued at $240 million for the 250-unit residential elevator building (D8) at 110 John Street in Financial District, Manhattan. On the lot, there was a new building construction project, 121188053, for a 250-unit, 213,017 square-foot residential (R-2) building. The project was submitted by Moinian Group and filed by Aron Kirsch with plans filed March 27, 2018 and permitted August 25, 2023. The city issued an initial certificate of occupancy in January 2026. The deal closed on June 1, 2026 and was recorded on June 8, 2026. The prior lender was BDT &amp; MSD Partners which held debt that had an original loan amount of $169 million. The property has 235,688 square feet of built space according to a PincusCo analysis of city data. The loan price per built square foot is $1,018 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) The signatory for Moinian Group wa</t>
+          <t>Top Story Transfers 2244 Westchester Avenue (Credit - Cyclomedia) Susan Ting and Austin Ting through the entity Jackson Ht. Roosevelt Development Corp. paid $16.2 million to ARCTRUST through the entity Bronx Westchester A2 LLC for the retail building (K7) at 2244 Westchester Avenue in Unionport, the Bronx, and adjacent and parking (G7) at 2246 Westchester Avenue and at 2248 Westchester Avenue. This is the headquarters location for lender Ponce Bank . ARCTRUST bought these three properties in November 2021 for $16.1 million. The deal closed on June 3, 2026 and was recorded on June 10, 2026. The three properties have 29,819 square feet of built space and 30,937 square feet of additional air rights for a total buildable of 60,705 square feet according to a PincusCo analysis of city data. The sale price per built square foot is $544 and the price per buildable square foot is $267 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) The signatory for ARCTRUST was Gary S. Baumann . The signatories for Susan Ting and Austin Ting were Susan Ting and Austin Ting</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Red Apple Group signs $83.5M refi for 205-unit rental in Downtown Brooklyn</t>
+          <t>GRE, Mark J. Schwartz, pay $5.7M to Sharp Management for walkups in Longwood</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>https://www.pincusco.com/red-apple-group-signs-83-5m-refi-for-205-unit-rental-in-downtown-brooklyn/</t>
+          <t>https://www.pincusco.com/gre-mark-j-schwartz-pay-5-7m-to-sharp-management-for-walkups-in-longwood/</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Red Apple Group through the entity Red Apple 81 Fleet Place Development, LLC as borrower</t>
+          <t>GRE Holdings and Mark J. Schwartz through the entity Cauldwell Avenue Housing Associates LLC paid</t>
         </is>
       </c>
       <c r="D9" t="inlineStr"/>
@@ -738,7 +738,7 @@
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>Transfers 81 Fleet Place (Credit - Cyclomedia) Red Apple Group through the entity Red Apple 81 Fleet Place Development, LLC as borrower signed a refi loan with lender U.S. Bank valued at $83.5 million for the 205-unit residential elevator building (D6) at 81 Fleet Place in Downtown Brooklyn, Brooklyn. The deal closed on May 28, 2026 and was recorded on June 8, 2026. The prior lender was U.S. Bank which held debt that had provided an original loan amount of $86 million in May 2019. The property has 265,417 square feet of built space according to a PincusCo analysis of city data. The loan price per built square foot is $314 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) The signatory for Red Apple Group was John Catsimatidis . The signatory for U.S. Bank was Matthew Gumnic . Prior sales, articles and revenue The owners according to the Department of Housing Preservation and Development includes John Catsimatidis, head officer and Charles D’Amico , officer. The business entities are Red Apple Property Management LLC and Red Apple 81 Fleet Place Devel</t>
+          <t xml:space="preserve">Transfers 643 Cauldwell Avenue (Credit - Cyclomedia) GRE Holdings and Mark J. Schwartz through the entity Cauldwell Avenue Housing Associates LLC paid $5.7 million to Sharp Management through the entity Bronx Sharp Realty LLC for the 41-unit residential walkup building (C1) at 643 Cauldwell Avenue in Longwood, Bronx and 43-unit residential walkup building (C1) at 647 Cauldwell Avenue in Longwood, Bronx. The expected use is cash flowing. The deal closed on May 27, 2026 and was recorded on June 10, 2026. The two properties have 57,408 square feet of built space according to a PincusCo analysis of city data. The sale price per built square foot is $98 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) The signatory for Sharp Management was Martin Kirzner . The signatory for Mark J. Schwartz and GRE Holdings was David Koshers . The contract date was April 17, 2026. Gilman Management rebranded as GRE Holdings. Because multiple properties have been transacted, some of the following sections will follow the property with the largest assessed value, which in </t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto update queens news 2026-06-12T15:36:12Z
</commit_message>
<xml_diff>
--- a/data/output/queens_dev_news.xlsx
+++ b/data/output/queens_dev_news.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H9"/>
+  <dimension ref="A1:H6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -473,17 +473,17 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Yellow Jacket Ventures pays $2.5M for 49-unit rental in Soundview</t>
+          <t>Century Development Group signs $43.4M construction loan for 116-unit project in Flushing</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>https://www.pincusco.com/yellow-jacket-ventures-pays-2-5m-for-49-unit-rental-in-soundview/</t>
+          <t>https://www.pincusco.com/century-development-group-signs-43-4m-construction-loan-for-116-unit-project-in-flushing/</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Yellow Jacket Ventures through the entity Commonwealth Bronx LLC paid $2.5 million to Marco Cepeda</t>
+          <t>Century Development Group through the entity 35 Ave Xu Holdings, LLC as borrower signed a</t>
         </is>
       </c>
       <c r="D2" t="inlineStr"/>
@@ -500,24 +500,24 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>Transfers 1326 Commonwealth Avenue (Credit - Cyclomedia) Yellow Jacket Ventures through the entity Commonwealth Bronx LLC paid $2.5 million to Marco Cepeda through the entity 2332 Walton Realty Inc. for the 49-unit residential elevator building (D1) at 1326 Commonwealth in Soundview, Bronx. The expected use is cash flowing. The deal closed on May 28, 2026 and was recorded on June 9, 2026. The property has 35,624 square feet of built space according to a PincusCo analysis of city data. The sale price per built square foot is $68 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) The seller bought the property on May 31, 2007, for $3.9 million. The signatory for Marco Cepeda was Marco Cepeda. The signatory for Yellow Jacket Ventures was Akiva J. Kurland . The contract date was April 27, 2026. Prior sales, articles and revenue Prior to this transaction, PincusCo has records that the buyer Yellow Jacket Ventures purchased two properties in two transactions for a total of $12.4 million and has no record it sold any properties over the past 24 months. The s</t>
+          <t>Transfers 33-75 Farrington Street isometric diagram (Credit - Raymond Chan architect via DOB) Century Development Group through the entity 35 Ave Xu Holdings, LLC as borrower signed a new construction loan with lender Bank Hapoalim valued at $43.4 million for the development site (V1) at 33-75 Farrington Street in Flushing, Queens, with plans for a 116-unit building. On the lot, there is one active new building construction project, Q08048244, for a 116-unit, 78,653-square-foot residential (R-2) building. The project was submitted by Century Development Group and filed by George Xu with plans filed January 4, 2023 and it has not been permitted yet. When the project was originally filed in 2023, it called for 98 units. The loan closed on May 29, 2026 and was recorded on June 11, 2026. The prior lender was Golden Bank which held debt that had an original loan amount of $8.8 million. The loan price per planned development square foot is $552 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) The owner bought the property on March 14, 2019, for $16 millio</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Vega sells single-family conversion for $16M in Cobble Hill, was $3.85M in 2020</t>
+          <t>GO Residential pays $222.6M to SL Green Realty for rental in Financial District</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>https://www.pincusco.com/vega-sells-single-family-conversion-for-16m-in-cobble-hill-was-3-85m-in-2020/</t>
+          <t>https://www.pincusco.com/go-residential-pays-220-5m-to-sl-green-realty-for-rental-in-financial-district/</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>The entity Cobble Chill LLC in care of Sullivan &amp; Cromwell paid $16 million to</t>
+          <t>GO Residential paid $222.6 million to SL Green Realty for a 209-unit rental condominium and</t>
         </is>
       </c>
       <c r="D3" t="inlineStr"/>
@@ -534,24 +534,24 @@
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>Transfers 205 Clinton Street (Credit - Cyclomedia) The entity Cobble Chill LLC in care of Sullivan &amp; Cromwell paid $16 million to Vega Management through the entity 205 Clinton Street, LLC for the single-family building (A4) at 205 Clinton Street in Cobble Hill, Brooklyn, converted from a four-family. The expected use is cash flowing. The deal closed on May 26, 2026 and was recorded on June 9, 2026. The property has 4,935 square feet of built space and 540 square feet of additional air rights for a total buildable of 5,467 square feet according to a PincusCo analysis of city data. The sale price per built square foot is $3,242 and the price per buildable square foot is $2,926 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) The sellers bought the property on June 30, 2020, for $3.85 million. The signatory for Vega Management was Allen Schifino . The signatory for Sullivan &amp; Cromwell registered buyer was Alison Hirsch. The contract date was May 5, 2026. Brandon Hornbeck of 205 Clinton Street, LLC submitted a major alteration application for the conve</t>
+          <t>Transfers 185 Broadway (Credit - Cyclomedia) GO Residential paid $222.6 million to SL Green Realty for a 209-unit rental condominium and a retail condominium at 183-185 Broadway and 7 Dey Street and in Financial District. SL Green Realty disclosed the transaction on March 16, 2026, with the price of $222.6 million. The transfer prices in city property records, used in the descriptions below, total $220.5 million. GO Residential through the entity GO Dey LLC paid $190 million to SL Green Realty through the entity 183 Broadway Owner LLC for the 209-unit rental condo at 7 Dey Street in Financial District, Manhattan. The expected use is cash flowing. The deal closed on May 27, 2026 and was recorded on June 11, 2026. The property has 183,214 square feet of built space according to a PincusCo analysis of city data. The sale price per built square foot is $1,037 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) GO Residential through the entity GO Dey LLC paid $30.5 million to SL Green Realty through the entity 183 Broadway Owner LLC for the retail condo at</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Isaac Friedman files plans for 20 units in East Flatbush</t>
+          <t>George Sakellaris pays $4.8M for 70-unit rental in North Corona</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>https://www.pincusco.com/isaac-friedman-files-plans-for-20-units-in-east-flatbush/</t>
+          <t>https://www.pincusco.com/george-sakellaris-pays-4-8m-for-residential-elevator-in-north-corona/</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Isaac Friedman submitted a new building construction project for a 20-unit, 13,627-square-foot residential (R-2) building</t>
+          <t>George Sakellaris through the entity 39-06 114 St Realty LLC paid $4.8 million to the</t>
         </is>
       </c>
       <c r="D4" t="inlineStr"/>
@@ -568,24 +568,24 @@
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>Development 258 East 53rd Street isometric diagram (Credit - Navkiran Cheema professional engineer via DOB) Isaac Friedman submitted a new building construction project for a 20-unit, 13,627-square-foot residential (R-2) building at 258 East 53rd Street in East Flatbush, Brooklyn. The plan was filed on June 9, 2026. It calls for the construction of a 40-foot-tall, four-story building and was filed with the New York City Department of Buildings under job number B01410734. The project is described in the filing as: application filed herewith to erect a new 4-story and penthouse, 20-family residential building. The applicant is the Professional Engineer Navkiran Cheema of KMA Designs LLC. 258 East 53rd Street The neighborhood In East Flatbush, The bulk, or 32 percent of the 42.6 million square feet of commercial built space are elevator buildings, with walkup buildings next occupying 24 percent of the space. In sales, East Flatbush has near average sales volume among other neighborhoods with $489.6 million in sales volume in the last two years and is the 16th highest in Brooklyn. For development, East Flatbush has near average amount of major developments among other neighborhoods and</t>
+          <t>Transfers 39-06 114th Street (Credit - Cyclomedia) George Sakellaris through the entity 39-06 114 St Realty LLC paid $4.8 million to the entity Wilco Holding, Inc. for the 70-unit residential elevator building (D3) at 39-06 114th Street in North Corona, Queens. The expected use is cash flowing. The deal closed on June 3, 2026 and was recorded on June 11, 2026. The property has 40,936 square feet of built space and 12,250 square feet of additional air rights for a total buildable of 53,156 square feet according to a PincusCo analysis of city data. The sale price per built square foot is $116 and the price per buildable square foot is $89 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) The signatory for the sellers, the Niarakis family, was Lisa A. Lolis . The signatory for George Sakellaris was George Sakellaris. The contract date was January 25, 2026. The buyer entity was in care of Alma Realty. Prior sales, articles and revenue Prior to this transaction, PincusCo has no record that the buyer George Sakellaris had purchased any other properties and</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Celaj Management pays $6.3M for 29-unit walkup in Harlem</t>
+          <t>Klisman Vrucaj files plans for 10 units in East Morrisania</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>https://www.pincusco.com/celaj-management-pays-6-3m-for-29-unit-walkup-in-harlem/</t>
+          <t>https://www.pincusco.com/klisman-vrucaj-files-plans-for-10-units-in-east-morrisania/</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Celaj Management through the entity Central Park North Realty Associates LLC paid $6.3 million to</t>
+          <t>Klisman Vrucaj submitted a new building construction project for a 10-unit, 6,001-square-foot residential (R-2) building</t>
         </is>
       </c>
       <c r="D5" t="inlineStr"/>
@@ -602,24 +602,24 @@
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Transfers 9 Central Park North (Credit - Cyclomedia) Celaj Management through the entity Central Park North Realty Associates LLC paid $6.3 million to the Rickman family through the entity 9-11 Realty Associates, LLC for the 29-unit residential walkup building (C7) at 9 Central Park North in Harlem, Manhattan. The expected use is cash flowing. The deal closed on May 28, 2026 and was recorded on June 10, 2026. The property has 23,640 square feet of built space and 16,467 square feet of additional air rights for a total buildable of 40,135 square feet according to a PincusCo analysis of city data. The sale price per built square foot is $268 and the price per buildable square foot is $158 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) The seller bought the property on April 27, 2017, for $13.7 million. The signatory for Hale Rickman was Stephen S. Siminou . The signatory for Celaj Management was Bashkim Celaj . The contract date was June 16, 2025. Prior sales, articles and revenue Prior to this transaction, PincusCo has records that the buyer Celaj </t>
+          <t>Development 1410 Longfellow Avenue axonometric diagram (Credit - John Backos architect via DOB) Klisman Vrucaj submitted a new building construction project for a 10-unit, 6,001-square-foot residential (R-2) building at 1410 Longfellow Avenue in East Morrisania, Bronx. The plan was filed on June 10, 2026. It calls for the construction of a 50-foot-tall, four-story building and was filed with the New York City Department of Buildings under job number X01413550. The project is described in the filing as: new 4 -story residential building. The applicant is the Registered Architect John Backos of Grid Drafting And Consulting Llc. 1410 Longfellow Avenue The neighborhood In East Morrisania, The bulk, or 43 percent of the 12 million square feet of commercial built space are elevator buildings, with walkup buildings next occupying 30 percent of the space. In sales, East Morrisania has near average sales volume among other neighborhoods with $133.9 million in sales volume in the last two years and is the 9th highest in Bronx. For development, East Morrisania has near average amount of major developments among other neighborhoods and is the 6th highest in Bronx. It had 1.4 million square fee</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Yehudis Klein pays $9.2M for 20-unit rental in East Harlem</t>
+          <t>JMH Development, AG Paratus pay $23.5M to Arbor for two properties in East Village</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>https://www.pincusco.com/yehudis-klein-pays-9-2m-for-residential-elevator-in-east-harlem/</t>
+          <t>https://www.pincusco.com/jmh-development-ag-paratus-pay-23-5m-to-arbor-for-two-properties-in-east-village/</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Yehudis Klein through the entity 308 Property Ny LLC paid $9.2 million to Boleslav Ryzinski</t>
+          <t>JMH Development and AG Paratus through the entity 111-113 E12 LLC paid $23.5 million to</t>
         </is>
       </c>
       <c r="D6" t="inlineStr"/>
@@ -636,109 +636,7 @@
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>Transfers 308 East 109th Street (Credit - Cyclomedia) Yehudis Klein through the entity 308 Property Ny LLC paid $9.2 million to Boleslav Ryzinski and Douglas Fierro through the entity 308 E 109th Street LLC for the 20-unit residential elevator building (D7) at 308 East 109th Street in East Harlem, Manhattan. The expected use is cash flowing. The deal closed on May 13, 2026 and was recorded on June 10, 2026. The property has 24,655 square feet of built space and 11,700 square feet of additional air rights for a total buildable of 36,359 square feet according to a PincusCo analysis of city data. The sale price per built square foot is $373 and the price per buildable square foot is $253 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) The seller bought the property on December 19, 2012, for $3.2 million. The signatory for Boleslav Ryzinski and Douglas Fierro was Douglas Fierro. The signatory for Yehudis Klein was Yehudis Klein. The contract date was January 16, 2026. The sellers in 2014 planned to divide the building into 20 residential condominium un</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>India-rooted spiritual group pays $11.8M for commercial condo in LIC</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>https://www.pincusco.com/india-rooted-spiritual-group-pays-11-8m-for-commercial-condo-in-lic/</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>The religious group with its origins in India, Radha Soami Satsang Beas, through the entity</t>
-        </is>
-      </c>
-      <c r="D7" t="inlineStr"/>
-      <c r="E7" t="inlineStr"/>
-      <c r="F7" t="inlineStr">
-        <is>
-          <t>PincusCo</t>
-        </is>
-      </c>
-      <c r="G7" t="inlineStr">
-        <is>
-          <t>PincusCo - Home</t>
-        </is>
-      </c>
-      <c r="H7" t="inlineStr">
-        <is>
-          <t>Transfers 11-36 45th Road (Credit - Cyclomedia) The religious group with its origins in India, Radha Soami Satsang Beas, through the entity Radha Soami Society Beas-America, paid $11.8 million to Century Development Group through the entity MPS Two, LLC for a 30,548-square-foot commercial condominium unit as well as additional parking spaces, at 11-36 45th Road in Long Island City, Queens. The expected use is owner-occupied. The deal closed on May 21, 2026 and was recorded on June 10, 2026. The 13 properties have zero square feet of built space according to a PincusCo analysis of city data. The sale price per built square foot is $386 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet of the unit, 30,548, as reported in public records.) The signatory for Century Development Group was Stavroula Tsolis . The signatory for Radha Soami Satsang Beas was Rajan Shamdasani . The contract date was May 31, 2019. Prior sales, articles and revenue Prior to this transaction, PincusCo has no record that the buyer Radha Soami Satsang Beas had purchased any other properties and has no record it sold any properties over the past 24 months.</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>Susan Ting, Austin Ting, pay $16.2M to ARCTRUST for retail in Unionport</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>https://www.pincusco.com/susan-ting-austin-ting-pays-16-2m-to-arctrust-for-three-properties-in-unionport/</t>
-        </is>
-      </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>Susan Ting and Austin Ting through the entity Jackson Ht. Roosevelt Development Corp. paid $16.2</t>
-        </is>
-      </c>
-      <c r="D8" t="inlineStr"/>
-      <c r="E8" t="inlineStr"/>
-      <c r="F8" t="inlineStr">
-        <is>
-          <t>PincusCo</t>
-        </is>
-      </c>
-      <c r="G8" t="inlineStr">
-        <is>
-          <t>PincusCo - Home</t>
-        </is>
-      </c>
-      <c r="H8" t="inlineStr">
-        <is>
-          <t>Top Story Transfers 2244 Westchester Avenue (Credit - Cyclomedia) Susan Ting and Austin Ting through the entity Jackson Ht. Roosevelt Development Corp. paid $16.2 million to ARCTRUST through the entity Bronx Westchester A2 LLC for the retail building (K7) at 2244 Westchester Avenue in Unionport, the Bronx, and adjacent and parking (G7) at 2246 Westchester Avenue and at 2248 Westchester Avenue. This is the headquarters location for lender Ponce Bank . ARCTRUST bought these three properties in November 2021 for $16.1 million. The deal closed on June 3, 2026 and was recorded on June 10, 2026. The three properties have 29,819 square feet of built space and 30,937 square feet of additional air rights for a total buildable of 60,705 square feet according to a PincusCo analysis of city data. The sale price per built square foot is $544 and the price per buildable square foot is $267 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) The signatory for ARCTRUST was Gary S. Baumann . The signatories for Susan Ting and Austin Ting were Susan Ting and Austin Ting</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>GRE, Mark J. Schwartz, pay $5.7M to Sharp Management for walkups in Longwood</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>https://www.pincusco.com/gre-mark-j-schwartz-pay-5-7m-to-sharp-management-for-walkups-in-longwood/</t>
-        </is>
-      </c>
-      <c r="C9" t="inlineStr">
-        <is>
-          <t>GRE Holdings and Mark J. Schwartz through the entity Cauldwell Avenue Housing Associates LLC paid</t>
-        </is>
-      </c>
-      <c r="D9" t="inlineStr"/>
-      <c r="E9" t="inlineStr"/>
-      <c r="F9" t="inlineStr">
-        <is>
-          <t>PincusCo</t>
-        </is>
-      </c>
-      <c r="G9" t="inlineStr">
-        <is>
-          <t>PincusCo - Home</t>
-        </is>
-      </c>
-      <c r="H9" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Transfers 643 Cauldwell Avenue (Credit - Cyclomedia) GRE Holdings and Mark J. Schwartz through the entity Cauldwell Avenue Housing Associates LLC paid $5.7 million to Sharp Management through the entity Bronx Sharp Realty LLC for the 41-unit residential walkup building (C1) at 643 Cauldwell Avenue in Longwood, Bronx and 43-unit residential walkup building (C1) at 647 Cauldwell Avenue in Longwood, Bronx. The expected use is cash flowing. The deal closed on May 27, 2026 and was recorded on June 10, 2026. The two properties have 57,408 square feet of built space according to a PincusCo analysis of city data. The sale price per built square foot is $98 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) The signatory for Sharp Management was Martin Kirzner . The signatory for Mark J. Schwartz and GRE Holdings was David Koshers . The contract date was April 17, 2026. Gilman Management rebranded as GRE Holdings. Because multiple properties have been transacted, some of the following sections will follow the property with the largest assessed value, which in </t>
+          <t>Chart_Frontpage Top Story Transfers 113 East 12th Street (Credit - Cyclomedia) JMH Development and AG Paratus through the entity 111-113 E12 LLC paid $23.5 million to Arbor Realty Trust through the entity 111-113 E 12th Property LLC for the nine-unit residential walkup building (C7) at 111 East 12th Street in East Village, Manhattan and four-unit mixed-use building (S4) at 113 East 12th Street in East Village, Manhattan. The expected use is cash flowing. The deal closed on May 29, 2026 and was recorded on June 11, 2026. The two properties have 16,639 square feet of built space and 15,258 square feet of additional air rights for a total buildable of 31,893 square feet according to a PincusCo analysis of city data. The sale price per built square foot is $1,412 and the price per buildable square foot is $736 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) The signatory for Arbor Realty Trust was Maurice Kaufman . The signatory for JMH Development and AG Paratus was Jason Halpern . The contract date was January 9, 2026. Because multiple properties hav</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto update queens news 2026-06-13T14:22:50Z
</commit_message>
<xml_diff>
--- a/data/output/queens_dev_news.xlsx
+++ b/data/output/queens_dev_news.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H6"/>
+  <dimension ref="A1:H4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -473,17 +473,17 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Century Development Group signs $43.4M construction loan for 116-unit project in Flushing</t>
+          <t>CRE8 Equities signs $5.5M refi with Citibank for retail in SoHo</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>https://www.pincusco.com/century-development-group-signs-43-4m-construction-loan-for-116-unit-project-in-flushing/</t>
+          <t>https://www.pincusco.com/cre8-equities-signs-5-5m-refi-with-citibank-for-retail-in-soho/</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Century Development Group through the entity 35 Ave Xu Holdings, LLC as borrower signed a</t>
+          <t>CRE8 Equities through the entity New Way Holdings IV LLC as borrower signed a refi</t>
         </is>
       </c>
       <c r="D2" t="inlineStr"/>
@@ -500,24 +500,24 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>Transfers 33-75 Farrington Street isometric diagram (Credit - Raymond Chan architect via DOB) Century Development Group through the entity 35 Ave Xu Holdings, LLC as borrower signed a new construction loan with lender Bank Hapoalim valued at $43.4 million for the development site (V1) at 33-75 Farrington Street in Flushing, Queens, with plans for a 116-unit building. On the lot, there is one active new building construction project, Q08048244, for a 116-unit, 78,653-square-foot residential (R-2) building. The project was submitted by Century Development Group and filed by George Xu with plans filed January 4, 2023 and it has not been permitted yet. When the project was originally filed in 2023, it called for 98 units. The loan closed on May 29, 2026 and was recorded on June 11, 2026. The prior lender was Golden Bank which held debt that had an original loan amount of $8.8 million. The loan price per planned development square foot is $552 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) The owner bought the property on March 14, 2019, for $16 millio</t>
+          <t>Transfers 180 Sixth Avenue retail (Credit - Cyclomedia) CRE8 Equities through the entity New Way Holdings IV LLC as borrower signed a refi loan with lender Hanmi Bank valued at $5.5 million for the retail condo at 180 Sixth Avenue in SoHo, Manhattan. The deal closed on May 26, 2026 and was recorded on June 10, 2026. The prior lender was Emerald Creek Capital which held debt that had an original loan amount of $4 million. The property has 14,717 square feet of built space according to a PincusCo analysis of city data. The loan price per built square foot is $373 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) The owner bought the property on November 8, 2024, for $7.3 million. The signatory for CRE8 Equities was Sheng Zeng . The signatory for Hanmi Bank was Eunice Eunyoung Nam . The property The retail condo in SoHo has 14,717 square feet of built space according to a PincusCo analysis of city data. The parcel has a total lot size of 14,717 square feet. The city-designated market value for the property in 2022 is $10.1 million. Hanmi Bank May 26, 20</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>GO Residential pays $222.6M to SL Green Realty for rental in Financial District</t>
+          <t>Global One Investments signs $22.4M refi with Citibank for residential elevator in Riverdale</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>https://www.pincusco.com/go-residential-pays-220-5m-to-sl-green-realty-for-rental-in-financial-district/</t>
+          <t>https://www.pincusco.com/global-one-investments-signs-22-4m-refi-with-citibank-for-residential-elevator-in-riverdale/</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>GO Residential paid $222.6 million to SL Green Realty for a 209-unit rental condominium and</t>
+          <t>Global One Investments through the entity Henry Hudson Nelson Apartments LLC as borrower signed a</t>
         </is>
       </c>
       <c r="D3" t="inlineStr"/>
@@ -534,24 +534,24 @@
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>Transfers 185 Broadway (Credit - Cyclomedia) GO Residential paid $222.6 million to SL Green Realty for a 209-unit rental condominium and a retail condominium at 183-185 Broadway and 7 Dey Street and in Financial District. SL Green Realty disclosed the transaction on March 16, 2026, with the price of $222.6 million. The transfer prices in city property records, used in the descriptions below, total $220.5 million. GO Residential through the entity GO Dey LLC paid $190 million to SL Green Realty through the entity 183 Broadway Owner LLC for the 209-unit rental condo at 7 Dey Street in Financial District, Manhattan. The expected use is cash flowing. The deal closed on May 27, 2026 and was recorded on June 11, 2026. The property has 183,214 square feet of built space according to a PincusCo analysis of city data. The sale price per built square foot is $1,037 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) GO Residential through the entity GO Dey LLC paid $30.5 million to SL Green Realty through the entity 183 Broadway Owner LLC for the retail condo at</t>
+          <t>Transfers 3240 Henry Hudson Parkway East (Credit - Cyclomedia) Global One Investments through the entity Henry Hudson Nelson Apartments LLC as borrower signed a refi loan with lender Citibank valued at $22.4 million for the 108-unit residential elevator building (D1) at 3240 Henry Hudson Pkwy East in Riverdale, the Bronx. Global One Investments, led by managing partners Michael Gerstein and Robert Nelson, owns real estate, while its affiliated company Nelson Management Group manages property. The loan closed on May 1, 2026 and was recorded on June 10, 2026. The prior lender was Flagstar Bank which held debt that had an original loan amount of $22.5 million. The property has 163,197 square feet of built space and 57,304 square feet of additional air rights for a total buildable of 220,400 square feet according to a PincusCo analysis of city data. The loan price per built square foot is $137 and the price per buildable square foot is $101 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) The owner bought the property on March 27, 2019, for $35.6 millio</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>George Sakellaris pays $4.8M for 70-unit rental in North Corona</t>
+          <t>Likely dev site in Long Island City sells for $4.8M</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>https://www.pincusco.com/george-sakellaris-pays-4-8m-for-residential-elevator-in-north-corona/</t>
+          <t>https://www.pincusco.com/likely-dev-site-in-long-island-city-sells-for-4-8m/</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>George Sakellaris through the entity 39-06 114 St Realty LLC paid $4.8 million to the</t>
+          <t>The entity 1148 44dr NY LLC, in care of the law firm Yang &amp; Yang,</t>
         </is>
       </c>
       <c r="D4" t="inlineStr"/>
@@ -568,75 +568,7 @@
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>Transfers 39-06 114th Street (Credit - Cyclomedia) George Sakellaris through the entity 39-06 114 St Realty LLC paid $4.8 million to the entity Wilco Holding, Inc. for the 70-unit residential elevator building (D3) at 39-06 114th Street in North Corona, Queens. The expected use is cash flowing. The deal closed on June 3, 2026 and was recorded on June 11, 2026. The property has 40,936 square feet of built space and 12,250 square feet of additional air rights for a total buildable of 53,156 square feet according to a PincusCo analysis of city data. The sale price per built square foot is $116 and the price per buildable square foot is $89 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) The signatory for the sellers, the Niarakis family, was Lisa A. Lolis . The signatory for George Sakellaris was George Sakellaris. The contract date was January 25, 2026. The buyer entity was in care of Alma Realty. Prior sales, articles and revenue Prior to this transaction, PincusCo has no record that the buyer George Sakellaris had purchased any other properties and</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>Klisman Vrucaj files plans for 10 units in East Morrisania</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>https://www.pincusco.com/klisman-vrucaj-files-plans-for-10-units-in-east-morrisania/</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>Klisman Vrucaj submitted a new building construction project for a 10-unit, 6,001-square-foot residential (R-2) building</t>
-        </is>
-      </c>
-      <c r="D5" t="inlineStr"/>
-      <c r="E5" t="inlineStr"/>
-      <c r="F5" t="inlineStr">
-        <is>
-          <t>PincusCo</t>
-        </is>
-      </c>
-      <c r="G5" t="inlineStr">
-        <is>
-          <t>PincusCo - Home</t>
-        </is>
-      </c>
-      <c r="H5" t="inlineStr">
-        <is>
-          <t>Development 1410 Longfellow Avenue axonometric diagram (Credit - John Backos architect via DOB) Klisman Vrucaj submitted a new building construction project for a 10-unit, 6,001-square-foot residential (R-2) building at 1410 Longfellow Avenue in East Morrisania, Bronx. The plan was filed on June 10, 2026. It calls for the construction of a 50-foot-tall, four-story building and was filed with the New York City Department of Buildings under job number X01413550. The project is described in the filing as: new 4 -story residential building. The applicant is the Registered Architect John Backos of Grid Drafting And Consulting Llc. 1410 Longfellow Avenue The neighborhood In East Morrisania, The bulk, or 43 percent of the 12 million square feet of commercial built space are elevator buildings, with walkup buildings next occupying 30 percent of the space. In sales, East Morrisania has near average sales volume among other neighborhoods with $133.9 million in sales volume in the last two years and is the 9th highest in Bronx. For development, East Morrisania has near average amount of major developments among other neighborhoods and is the 6th highest in Bronx. It had 1.4 million square fee</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>JMH Development, AG Paratus pay $23.5M to Arbor for two properties in East Village</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>https://www.pincusco.com/jmh-development-ag-paratus-pay-23-5m-to-arbor-for-two-properties-in-east-village/</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>JMH Development and AG Paratus through the entity 111-113 E12 LLC paid $23.5 million to</t>
-        </is>
-      </c>
-      <c r="D6" t="inlineStr"/>
-      <c r="E6" t="inlineStr"/>
-      <c r="F6" t="inlineStr">
-        <is>
-          <t>PincusCo</t>
-        </is>
-      </c>
-      <c r="G6" t="inlineStr">
-        <is>
-          <t>PincusCo - Home</t>
-        </is>
-      </c>
-      <c r="H6" t="inlineStr">
-        <is>
-          <t>Chart_Frontpage Top Story Transfers 113 East 12th Street (Credit - Cyclomedia) JMH Development and AG Paratus through the entity 111-113 E12 LLC paid $23.5 million to Arbor Realty Trust through the entity 111-113 E 12th Property LLC for the nine-unit residential walkup building (C7) at 111 East 12th Street in East Village, Manhattan and four-unit mixed-use building (S4) at 113 East 12th Street in East Village, Manhattan. The expected use is cash flowing. The deal closed on May 29, 2026 and was recorded on June 11, 2026. The two properties have 16,639 square feet of built space and 15,258 square feet of additional air rights for a total buildable of 31,893 square feet according to a PincusCo analysis of city data. The sale price per built square foot is $1,412 and the price per buildable square foot is $736 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) The signatory for Arbor Realty Trust was Maurice Kaufman . The signatory for JMH Development and AG Paratus was Jason Halpern . The contract date was January 9, 2026. Because multiple properties hav</t>
+          <t>Transfers 11-48 44th Drive (Credit - Cyclomedia) The entity 1148 44dr NY LLC, in care of the law firm Yang &amp; Yang, paid $4.8 million to the entity 1148 44 Dr LLC for the industrial building (G2) at 11-48 44th Drive in Long Island City, Queens. The expected use is ground up development. The deal closed on May 29, 2026 and was recorded on June 11, 2026. The property has 3,700 square feet of built space and 18,862 square feet of additional air rights for a total buildable of 22,575 square feet according to a PincusCo analysis of city data. The sale price per built square foot is $1,283 and the price per buildable square foot is $210 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) The signatory for the seller was Giovanni Gugliotta. The contract date was March 25, 2025. Prior sales, articles and revenue Prior to this transaction, PincusCo has no record that the buyer Yung &amp; Yung registered had purchased any other properties and has no record it sold any properties over the past 24 months. The seller Giovanni Gugliotta had not purchased any other proper</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto update queens news 2026-06-14T14:26:02Z
</commit_message>
<xml_diff>
--- a/data/output/queens_dev_news.xlsx
+++ b/data/output/queens_dev_news.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H4"/>
+  <dimension ref="A1:H1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -467,108 +467,6 @@
       <c r="H1" s="1" t="inlineStr">
         <is>
           <t>content_preview</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>CRE8 Equities signs $5.5M refi with Citibank for retail in SoHo</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>https://www.pincusco.com/cre8-equities-signs-5-5m-refi-with-citibank-for-retail-in-soho/</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>CRE8 Equities through the entity New Way Holdings IV LLC as borrower signed a refi</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr"/>
-      <c r="E2" t="inlineStr"/>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t>PincusCo</t>
-        </is>
-      </c>
-      <c r="G2" t="inlineStr">
-        <is>
-          <t>PincusCo - Home</t>
-        </is>
-      </c>
-      <c r="H2" t="inlineStr">
-        <is>
-          <t>Transfers 180 Sixth Avenue retail (Credit - Cyclomedia) CRE8 Equities through the entity New Way Holdings IV LLC as borrower signed a refi loan with lender Hanmi Bank valued at $5.5 million for the retail condo at 180 Sixth Avenue in SoHo, Manhattan. The deal closed on May 26, 2026 and was recorded on June 10, 2026. The prior lender was Emerald Creek Capital which held debt that had an original loan amount of $4 million. The property has 14,717 square feet of built space according to a PincusCo analysis of city data. The loan price per built square foot is $373 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) The owner bought the property on November 8, 2024, for $7.3 million. The signatory for CRE8 Equities was Sheng Zeng . The signatory for Hanmi Bank was Eunice Eunyoung Nam . The property The retail condo in SoHo has 14,717 square feet of built space according to a PincusCo analysis of city data. The parcel has a total lot size of 14,717 square feet. The city-designated market value for the property in 2022 is $10.1 million. Hanmi Bank May 26, 20</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>Global One Investments signs $22.4M refi with Citibank for residential elevator in Riverdale</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>https://www.pincusco.com/global-one-investments-signs-22-4m-refi-with-citibank-for-residential-elevator-in-riverdale/</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>Global One Investments through the entity Henry Hudson Nelson Apartments LLC as borrower signed a</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr"/>
-      <c r="E3" t="inlineStr"/>
-      <c r="F3" t="inlineStr">
-        <is>
-          <t>PincusCo</t>
-        </is>
-      </c>
-      <c r="G3" t="inlineStr">
-        <is>
-          <t>PincusCo - Home</t>
-        </is>
-      </c>
-      <c r="H3" t="inlineStr">
-        <is>
-          <t>Transfers 3240 Henry Hudson Parkway East (Credit - Cyclomedia) Global One Investments through the entity Henry Hudson Nelson Apartments LLC as borrower signed a refi loan with lender Citibank valued at $22.4 million for the 108-unit residential elevator building (D1) at 3240 Henry Hudson Pkwy East in Riverdale, the Bronx. Global One Investments, led by managing partners Michael Gerstein and Robert Nelson, owns real estate, while its affiliated company Nelson Management Group manages property. The loan closed on May 1, 2026 and was recorded on June 10, 2026. The prior lender was Flagstar Bank which held debt that had an original loan amount of $22.5 million. The property has 163,197 square feet of built space and 57,304 square feet of additional air rights for a total buildable of 220,400 square feet according to a PincusCo analysis of city data. The loan price per built square foot is $137 and the price per buildable square foot is $101 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) The owner bought the property on March 27, 2019, for $35.6 millio</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>Likely dev site in Long Island City sells for $4.8M</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>https://www.pincusco.com/likely-dev-site-in-long-island-city-sells-for-4-8m/</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>The entity 1148 44dr NY LLC, in care of the law firm Yang &amp; Yang,</t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr"/>
-      <c r="E4" t="inlineStr"/>
-      <c r="F4" t="inlineStr">
-        <is>
-          <t>PincusCo</t>
-        </is>
-      </c>
-      <c r="G4" t="inlineStr">
-        <is>
-          <t>PincusCo - Home</t>
-        </is>
-      </c>
-      <c r="H4" t="inlineStr">
-        <is>
-          <t>Transfers 11-48 44th Drive (Credit - Cyclomedia) The entity 1148 44dr NY LLC, in care of the law firm Yang &amp; Yang, paid $4.8 million to the entity 1148 44 Dr LLC for the industrial building (G2) at 11-48 44th Drive in Long Island City, Queens. The expected use is ground up development. The deal closed on May 29, 2026 and was recorded on June 11, 2026. The property has 3,700 square feet of built space and 18,862 square feet of additional air rights for a total buildable of 22,575 square feet according to a PincusCo analysis of city data. The sale price per built square foot is $1,283 and the price per buildable square foot is $210 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) The signatory for the seller was Giovanni Gugliotta. The contract date was March 25, 2025. Prior sales, articles and revenue Prior to this transaction, PincusCo has no record that the buyer Yung &amp; Yung registered had purchased any other properties and has no record it sold any properties over the past 24 months. The seller Giovanni Gugliotta had not purchased any other proper</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto update queens news 2026-06-15T17:26:28Z
</commit_message>
<xml_diff>
--- a/data/output/queens_dev_news.xlsx
+++ b/data/output/queens_dev_news.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H1"/>
+  <dimension ref="A1:H10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -470,6 +470,312 @@
         </is>
       </c>
     </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Michael Aryeh, RoeCo LLC, Yassky sign $8.8M refi with Flushing Bank for 52-unit rental in Washington Heights</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>https://www.pincusco.com/michael-aryeh-roeco-llc-yassky-sign-8-8m-refi-with-flushing-bank-for-52-unit-rental-in-washington-heights/</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Michael Aryeh, RoeCo LLC, and Yassky Properties through the entity 113 West LLC as borrower</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr"/>
+      <c r="E2" t="inlineStr"/>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>PincusCo</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>PincusCo - Home</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>Transfers Michael Aryeh, RoeCo LLC, and Yassky Properties through the entity 113 West LLC as borrower signed a refi loan with lender Flushing Bank through the entity Flushing Bank valued at $8.8 million for the 52-unit residential elevator building (D7) at 220 Wadsworth Avenue in Washington Heights, Manhattan. The deal closed on May 28, 2026 and was recorded on June 11, 2026. The prior lender was an affiliate of the Manocherian family which held debt that had an original loan amount of $5.2 million. The property has 56,652 square feet of built space according to a PincusCo analysis of city data. The loan price per built square foot is $155 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) The owner bought the property on August 15, 2016, for $15.6 million. The signatory for Michael Aryeh , RoeCo LLC , and Yassky Properties was Scott Solomon , Charles Yassky , and Michael Aryeh. The signatory for Flushing Bank was H. Michael Lynch . Prior sales, articles and revenue The owners according to the Department of Housing Preservation and Development include</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Loketch Group pays $11M for 17-unit dev site in Fort Greene</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>https://www.pincusco.com/loketch-group-pays-11m-for-17-unit-dev-site-in-fort-greene/</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Loketch Group through the entity 158 Oxford LLC paid $11 million to Marc E. Lambrechts</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr"/>
+      <c r="E3" t="inlineStr"/>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>PincusCo</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>PincusCo - Home</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>Transfers 158 South Oxford Street (Credit - Cyclomedia) Loketch Group through the entity 158 Oxford LLC paid $11 million to Marc E. Lambrechts through the entity 158 Ny LLC for the development site at 158 South Oxford Street in Fort Greene, Brooklyn. The expected use is ground up development. On the lot, there is one active new building construction project, B01329666, for a 17-unit, 22,947 square-foot residential (R-2) building. The project was submitted by Borough Developers and filed by Shimon Kleinman with plans filed December 18, 2025 and it has not been permitted yet. The development is now led by Loketch Group, according to filings with the Department of Building. The deal closed on June 4, 2026 and was recorded on June 12, 2026. The property has 5,400 square feet of built space and 17,595 square feet of additional air rights for a total buildable of 23,000 square feet according to a PincusCo analysis of city data. The sale price per built square foot is $2,037 and the price per buildable square foot is $478 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights ha</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Midwood Investment, Niarchos family pay $41M to Samco for retail in Greenwich Village</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>https://www.pincusco.com/midwood-investment-niarchos-family-pay-41m-to-samco-for-retail-in-greenwich-village/</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Midwood Investment &amp; Development and Stavros Niarchos family through the entity One Greenwich Retail Ecu</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr"/>
+      <c r="E4" t="inlineStr"/>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>PincusCo</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>PincusCo - Home</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>Chart_Frontpage Transfers 403 Avenue Of Americas (Credit - Cyclomedia) Midwood Investment &amp; Development and Stavros Niarchos family through the entity One Greenwich Retail Ecu Tic LLC paid $41 million to Samco Properties through the entity 405 Sixth LLC for the retail building (K1) at 403 Sixth Avenue in Greenwich Village, Manhattan. The expected use is cash flowing. The deal closed on June 8, 2026 and was recorded on June 12, 2026. The property has 18,564 square feet of built space and 26,103 square feet of additional air rights for a total buildable of 44,675 square feet according to a PincusCo analysis of city data. The sale price per built square foot is $2,208 and the price per buildable square foot is $917 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) The signatory for Samco Properties was Joshua Smith . The signatory for Midwood Investment &amp; Development and Niarchos family was John Usdan and Jonathan Spice and Claus Zellner . Spice and Zellner are both affiliated with the Niarchos family, which operates several companies including Poseidon</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Shahram John Gatan pays $6.5M for 31-unit walkup in Yorkville</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>https://www.pincusco.com/shahram-john-gatan-pays-6-5m-for-residential-walkup-in-yorkville/</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Shahram John Gatan through the entity BH 437 LLC paid $6.5 million to the Intner</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr"/>
+      <c r="E5" t="inlineStr"/>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>PincusCo</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>PincusCo - Home</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>Transfers 437 East 80th Street (Credit - Cyclomedia) Shahram John Gatan through the entity BH 437 LLC paid $6.5 million to the Intner family Robert J. Intner through the entity 80th Street I LLC for the 31-unit residential walkup building (C7) at 437 East 80th Street in Yorkville, Manhattan. The expected use is cash flowing. The deal closed on May 12, 2026 and was recorded on June 12, 2026. The property has 23,346 square feet of built space according to a PincusCo analysis of city data. The sale price per built square foot is $280 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) The signatory for the Intner family was Robert J. Intner . The signatory for Shahram John Gatan was John Gatan. The contract date was March 11, 2026. Melvin H. Intner bought the parcel in 1976. Prior sales, articles and revenue Prior to this transaction, PincusCo has no record that the buyer Shahram John Gatan had purchased any other properties and has no record it sold any properties over the past 24 months. The seller Robert J. Intner had not purchased any other properties</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Artan Prelaj pays $7.2M for 99-unit dev site in Tremont</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>https://www.pincusco.com/artan-prelaj-pays-7-2m-for-99-unit-dev-site-in-tremont/</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Artan Prelaj through the entity 2923-35 Third LLC paid $7.2 million to Aleksander Lakal through</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr"/>
+      <c r="E6" t="inlineStr"/>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>PincusCo</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>PincusCo - Home</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>Transfers 4121 3rd Avenue (Credit - Cyclomedia) Artan Prelaj through the entity 2923-35 Third LLC paid $7.2 million to Aleksander Lakal through the entity 4119 Third LLC for the industrial building (G7) at 4121 3rd Avenue in Tremont, Bronx. The expected use is ground up development. On the lot, there is one active new building construction project, X01223342, for a 99-unit, 69,577 square-foot residential (R-2) building. The project was submitted by Aleksander Lakaj and filed by Alex Lakaj with plans filed July 31, 2025 and it has not been permitted yet. The deal closed on May 28, 2026 and was recorded on June 12, 2026. The sale price price per planned construction square foot is $103 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) The seller bought the property on July 1, 2024, for $7.5 million. The signatory for Aleksander Lakal was Aleksander Lakal. The signatory for Artan Prelaj was Artan Prelaj. The contract date was March 31, 2025. Prior sales, articles and revenue Prior to this transaction, PincusCo has no record that the buyer Artan Prelaj h</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Juan Qing Lu pays $8M for Sirico’s banquet hall in Dyker Heights</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>https://www.pincusco.com/juan-qing-lu-pays-8m-to-hercules-sirico-and-james-t-sirico-for-five-properties-in-dyker-heights/</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Juan Qing Lu through the entity JMAL Group LLC paid $8 million to the Sirico</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr"/>
+      <c r="E7" t="inlineStr"/>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>PincusCo</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>PincusCo - Home</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Transfers 8017 13th Avenue, et al (Credit - Cyclomedia) Juan Qing Lu through the entity JMAL Group LLC paid $8 million to the Sirico family through the entity JHS Realty Associates for Sirico’s Caterers banquet hall covering five tax lots making up the retail at 8023 13th Avenue in Dyker Heights, Brooklyn. The deal closed on June 1, 2026 and was recorded on June 12, 2026. The five properties have 14,160 square feet of built space and 7,240 square feet of additional air rights for a total buildable of 21,000 square feet according to a PincusCo analysis of city data. The sale price per built square foot is $564 and the price per buildable square foot is $380 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) The signatory for Hercules Sirico and James T. Sirico was Hercules Sirico and James T. Sirico. The signatory for Juan Qing Lu was Juan Qing Lu. The contract date was June 30, 2025. The Sirico family members were owners of Sirico’s Caterers, which is permanently closed as of late May, according to local media. Prior sales, articles and revenue Prior </t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Hawkins Way pays $80M in sale-leaseback with college for dorm in Lincoln Square</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>https://www.pincusco.com/hawkins-way-pays-80m-in-sale-leaseback-with-college-for-dorm-in-lincoln-square/</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Hawkins Way Capital through the entity 117 W 70th Owner, LLC paid $80 million to</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr"/>
+      <c r="E8" t="inlineStr"/>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>PincusCo</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>PincusCo - Home</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>Top Story Transfers 117 West 70th Street (Credit - Cyclomedia) Hawkins Way Capital through the entity 117 W 70th Owner, LLC paid $80 million to American Musical and Dramatic Academy through the entity Manhattan Stratford Arms, Inc. for the dormitory, also known as a residence hall, building (H8) at 117 West 70th Street in Lincoln Square, Manhattan. The expected use is cash flowing as part of a sale-leaseback agreement. The American Musical Dramatic Academy, also known as AMDA, executed a $23 million sale-leaseback in 2023 in Los Angeles. The deal closed on May 7, 2026 and was recorded on June 12, 2026. The property has 75,313 square feet of built space according to a PincusCo analysis of city data. The sale price per built square foot is $1,062 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) The signatory for American Musical and Dramatic Academy was David Silverman . The signatory for Hawkins Way Capital was Joshua Bird . The contract date was May 7, 2026. Simultaneously with the purchase, the parties signed a 31-year lease commencing on May 7, 20</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Medical spa owner pays $5M to Collins Ogbolu for mixed-use in Harlem</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>https://www.pincusco.com/medical-spa-owner-pays-5m-to-collins-ogbolu-for-mixed-use-in-harlem/</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Richina Lukes, CEO of L’Elite MediSpa, through the entity Lenox 335, LLC paid $5 million</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr"/>
+      <c r="E9" t="inlineStr"/>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>PincusCo</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>PincusCo - Home</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Transfers 335 Lenox Avenue (Credit - Cyclomedia) Richina Lukes, CEO of L’Elite MediSpa, through the entity Lenox 335, LLC paid $5 million for the four-unit mixed-use building (S9) at 335 Lenox Avenue in Harlem, Manhattan. The expected use is owner-occupied. The location has been occupied by a different laser spa center, recent images of the building show. The deal closed on May 13, 2026 and was recorded on June 12, 2026. The property has 6,648 square feet of built space and 975 square feet of additional air rights for a total buildable of 7,623 square feet according to a PincusCo analysis of city data. The sale price per built square foot is $752 and the price per buildable square foot is $655 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) The signatory for Collins Ogbolu was Collins J. Ogbolu . The signatory for Richina Lukes was Richina J. Lukes. The contract date was January 29, 2026. Prior sales, articles and revenue Prior to this transaction, PincusCo has no record that the buyer Richina J. Lukes had purchased any other properties and has no </t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Vesper Holdings pays $2.8M to Cayuga Capital for mixed-use in Bushwick</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>https://www.pincusco.com/vesper-holdings-pays-2-8m-to-cayuga-capital-for-mixed-use-in-bushwick/</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Vesper Holdings through the entity 287 Wyckoff Assc. LLC paid $2.8 million to Cayuga Capital</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr"/>
+      <c r="E10" t="inlineStr"/>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>PincusCo</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>PincusCo - Home</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>Transfers 287 Wyckoff Avenue (Credit - Cyclomedia) Vesper Holdings through the entity 287 Wyckoff Assc. LLC paid $2.8 million to Cayuga Capital Management through the entity 287 Wyckoff LLC for the five-unit mixed-use building (S5) at 287 Wyckoff Avenue in Bushwick, Brooklyn. The expected use is cash flowing. The deal closed on May 20, 2026 and was recorded on June 12, 2026. The property has 4,050 square feet of built space and 1,101 square feet of additional air rights for a total buildable of 5,146 square feet according to a PincusCo analysis of city data. The sale price per built square foot is $691 and the price per buildable square foot is $544 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) The seller bought the property on April 29, 2015, for $1.2 million. The signatory for Cayuga Capital Management was Jacob Sacks . The signatory for Vesper Holdings was Elliot J. Tamir . The contract date was March 3, 2026. Prior sales, articles and revenue Prior to this transaction, PincusCo has no record that the buyer Vesper Holdings had purchased any ot</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
auto update queens news 2026-06-16T17:19:30Z
</commit_message>
<xml_diff>
--- a/data/output/queens_dev_news.xlsx
+++ b/data/output/queens_dev_news.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H10"/>
+  <dimension ref="A1:H5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -473,17 +473,17 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Michael Aryeh, RoeCo LLC, Yassky sign $8.8M refi with Flushing Bank for 52-unit rental in Washington Heights</t>
+          <t>Fei Guo pays $7.7M to Amos Financial for 19-unit rental in Clinton Hill</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>https://www.pincusco.com/michael-aryeh-roeco-llc-yassky-sign-8-8m-refi-with-flushing-bank-for-52-unit-rental-in-washington-heights/</t>
+          <t>https://www.pincusco.com/fei-guo-pays-7-7m-to-amos-financial-for-19-unit-rental-in-clinton-hill/</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Michael Aryeh, RoeCo LLC, and Yassky Properties through the entity 113 West LLC as borrower</t>
+          <t>Fei Guo through the entity Kg Atlantic Realty Holding Inc. paid $7.7 million through a</t>
         </is>
       </c>
       <c r="D2" t="inlineStr"/>
@@ -500,24 +500,24 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>Transfers Michael Aryeh, RoeCo LLC, and Yassky Properties through the entity 113 West LLC as borrower signed a refi loan with lender Flushing Bank through the entity Flushing Bank valued at $8.8 million for the 52-unit residential elevator building (D7) at 220 Wadsworth Avenue in Washington Heights, Manhattan. The deal closed on May 28, 2026 and was recorded on June 11, 2026. The prior lender was an affiliate of the Manocherian family which held debt that had an original loan amount of $5.2 million. The property has 56,652 square feet of built space according to a PincusCo analysis of city data. The loan price per built square foot is $155 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) The owner bought the property on August 15, 2016, for $15.6 million. The signatory for Michael Aryeh , RoeCo LLC , and Yassky Properties was Scott Solomon , Charles Yassky , and Michael Aryeh. The signatory for Flushing Bank was H. Michael Lynch . Prior sales, articles and revenue The owners according to the Department of Housing Preservation and Development include</t>
+          <t>Transfers 929 Atlantic Avenue (Credit - Cyclomedia) Fei Guo through the entity Kg Atlantic Realty Holding Inc. paid $7.7 million through a real estate owned sale to former lender Amos Financial for the 19-unit residential elevator building (D3) at 929 Atlantic Avenue in Clinton Hill, Brooklyn. The expected use is cash flowing. The deal closed on May 27, 2026 and was recorded on June 15, 2026. The property has 17,469 square feet of built space and 775 square feet of additional air rights for a total buildable of 18,240 square feet according to a PincusCo analysis of city data. The sale price per built square foot is $440 and the price per buildable square foot is $422 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) Amos Financial took title to the property on August 5, 2022. The signatory for Amos Financial was Ohannes Korogluyan . The signatory for Fei Guo was Fei Guo. The contract date was April 8, 2026. Prior sales, articles and revenue Prior to this transaction, PincusCo has no record that the buyer Fei Guo had purchased any other properties and</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Loketch Group pays $11M for 17-unit dev site in Fort Greene</t>
+          <t>99 units planned for Yossel Lichtman dev site in Greenpoint</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>https://www.pincusco.com/loketch-group-pays-11m-for-17-unit-dev-site-in-fort-greene/</t>
+          <t>https://www.pincusco.com/99-units-planned-for-yossel-lichtman-dev-site-in-greenpoint/</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Loketch Group through the entity 158 Oxford LLC paid $11 million to Marc E. Lambrechts</t>
+          <t>A new building construction project for a 99-unit, 105,210-square-foot residential (R-2) development at 70 West</t>
         </is>
       </c>
       <c r="D3" t="inlineStr"/>
@@ -534,24 +534,24 @@
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>Transfers 158 South Oxford Street (Credit - Cyclomedia) Loketch Group through the entity 158 Oxford LLC paid $11 million to Marc E. Lambrechts through the entity 158 Ny LLC for the development site at 158 South Oxford Street in Fort Greene, Brooklyn. The expected use is ground up development. On the lot, there is one active new building construction project, B01329666, for a 17-unit, 22,947 square-foot residential (R-2) building. The project was submitted by Borough Developers and filed by Shimon Kleinman with plans filed December 18, 2025 and it has not been permitted yet. The development is now led by Loketch Group, according to filings with the Department of Building. The deal closed on June 4, 2026 and was recorded on June 12, 2026. The property has 5,400 square feet of built space and 17,595 square feet of additional air rights for a total buildable of 23,000 square feet according to a PincusCo analysis of city data. The sale price per built square foot is $2,037 and the price per buildable square foot is $478 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights ha</t>
+          <t>Development 70 West Street axonometric diagram (Credit - Shmuel Wieder architect via DOB) A new building construction project for a 99-unit, 105,210-square-foot residential (R-2) development at 70 West Street in Greenpoint, Brooklyn, was filed on behalf of property owner and developer Yossel Lichtman. The plan was filed on June 11, 2026. It calls for the construction of a 95-foot-tall, nine-story building and was filed with the New York City Department of Buildings under job number B01411828. The project is described in the filing as: new 9 story and cellar mixed use building with 99 residential dwelling units. The applicant is the Registered Architect Shmuel Wieder of S. Wieder Architect P.C. Mendy Schwimmer submitted the plans. The ground floor includes five residential units along with a lobby, mail and package room, and 1,303 square feet of retail space. Floor two houses nine units plus recreation rooms. Floors three through six each contain 13 units. Floors seven, eight, and nine each hold 11 units. The cellar level accommodates mechanical systems, an electric meter room, water-sprinkler room, laundry facilities, a pet spa, trash compactor room, bicycle parking for 50 bicycles</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Midwood Investment, Niarchos family pay $41M to Samco for retail in Greenwich Village</t>
+          <t>Gotham Organization files 2 plans totaling 375 units in East New York</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>https://www.pincusco.com/midwood-investment-niarchos-family-pay-41m-to-samco-for-retail-in-greenwich-village/</t>
+          <t>https://www.pincusco.com/gotham-organization-files-2-plans-totaling-375-units-in-east-new-york/</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Midwood Investment &amp; Development and Stavros Niarchos family through the entity One Greenwich Retail Ecu</t>
+          <t>Gotham Organization filed two plans totaling 375 units in East New York, Brooklyn. In the</t>
         </is>
       </c>
       <c r="D4" t="inlineStr"/>
@@ -568,24 +568,24 @@
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>Chart_Frontpage Transfers 403 Avenue Of Americas (Credit - Cyclomedia) Midwood Investment &amp; Development and Stavros Niarchos family through the entity One Greenwich Retail Ecu Tic LLC paid $41 million to Samco Properties through the entity 405 Sixth LLC for the retail building (K1) at 403 Sixth Avenue in Greenwich Village, Manhattan. The expected use is cash flowing. The deal closed on June 8, 2026 and was recorded on June 12, 2026. The property has 18,564 square feet of built space and 26,103 square feet of additional air rights for a total buildable of 44,675 square feet according to a PincusCo analysis of city data. The sale price per built square foot is $2,208 and the price per buildable square foot is $917 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) The signatory for Samco Properties was Joshua Smith . The signatory for Midwood Investment &amp; Development and Niarchos family was John Usdan and Jonathan Spice and Claus Zellner . Spice and Zellner are both affiliated with the Niarchos family, which operates several companies including Poseidon</t>
+          <t>Development 12030 Flatlands Avenue axonometric diagram (Credit - Gloria Glas architect via DOB) Gotham Organization filed two plans totaling 375 units in East New York, Brooklyn. In the large, Gotham Organization submitted a new building construction project for a 206-unit, 144,132-square-foot residential (R-2) building at 12030 Flatlands Avenue in East New York, Brooklyn. The plan was filed on June 10, 2026. It calls for the construction of a 126-foot-tall, thirteen-story building and was filed with the New York City Department of Buildings under job number B01412655. The project is described in the filing as: construct new 13 story mixed use building as per plans filed. The applicant is the Registered Architect Gloria Glas of Slce Architects. David Picket of Gotham Organization submitted the plans. In the smaller, Gotham Organization submitted a new building construction project for a 169-unit, 173,805-square-foot residential (R-2) building at 395 Louisiana Avenue in East New York, Brooklyn. The plan was filed on June 10, 2026. It calls for the construction of a 114-foot-tall, twelve-story building and was filed with the New York City Department of Buildings under job number B014</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Shahram John Gatan pays $6.5M for 31-unit walkup in Yorkville</t>
+          <t>Gorjian Real Estate signs $14.7M refi with Chase for 50-unit rental in Hell’s Kitchen</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>https://www.pincusco.com/shahram-john-gatan-pays-6-5m-for-residential-walkup-in-yorkville/</t>
+          <t>https://www.pincusco.com/gorjian-real-estate-signs-14-7m-refi-with-chase-for-50-unit-rental-in-hells-kitchen/</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Shahram John Gatan through the entity BH 437 LLC paid $6.5 million to the Intner</t>
+          <t>Gorjian Real Estate Group through the entity GG West 57 Owner LLC as borrower signed</t>
         </is>
       </c>
       <c r="D5" t="inlineStr"/>
@@ -602,177 +602,7 @@
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>Transfers 437 East 80th Street (Credit - Cyclomedia) Shahram John Gatan through the entity BH 437 LLC paid $6.5 million to the Intner family Robert J. Intner through the entity 80th Street I LLC for the 31-unit residential walkup building (C7) at 437 East 80th Street in Yorkville, Manhattan. The expected use is cash flowing. The deal closed on May 12, 2026 and was recorded on June 12, 2026. The property has 23,346 square feet of built space according to a PincusCo analysis of city data. The sale price per built square foot is $280 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) The signatory for the Intner family was Robert J. Intner . The signatory for Shahram John Gatan was John Gatan. The contract date was March 11, 2026. Melvin H. Intner bought the parcel in 1976. Prior sales, articles and revenue Prior to this transaction, PincusCo has no record that the buyer Shahram John Gatan had purchased any other properties and has no record it sold any properties over the past 24 months. The seller Robert J. Intner had not purchased any other properties</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>Artan Prelaj pays $7.2M for 99-unit dev site in Tremont</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>https://www.pincusco.com/artan-prelaj-pays-7-2m-for-99-unit-dev-site-in-tremont/</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>Artan Prelaj through the entity 2923-35 Third LLC paid $7.2 million to Aleksander Lakal through</t>
-        </is>
-      </c>
-      <c r="D6" t="inlineStr"/>
-      <c r="E6" t="inlineStr"/>
-      <c r="F6" t="inlineStr">
-        <is>
-          <t>PincusCo</t>
-        </is>
-      </c>
-      <c r="G6" t="inlineStr">
-        <is>
-          <t>PincusCo - Home</t>
-        </is>
-      </c>
-      <c r="H6" t="inlineStr">
-        <is>
-          <t>Transfers 4121 3rd Avenue (Credit - Cyclomedia) Artan Prelaj through the entity 2923-35 Third LLC paid $7.2 million to Aleksander Lakal through the entity 4119 Third LLC for the industrial building (G7) at 4121 3rd Avenue in Tremont, Bronx. The expected use is ground up development. On the lot, there is one active new building construction project, X01223342, for a 99-unit, 69,577 square-foot residential (R-2) building. The project was submitted by Aleksander Lakaj and filed by Alex Lakaj with plans filed July 31, 2025 and it has not been permitted yet. The deal closed on May 28, 2026 and was recorded on June 12, 2026. The sale price price per planned construction square foot is $103 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) The seller bought the property on July 1, 2024, for $7.5 million. The signatory for Aleksander Lakal was Aleksander Lakal. The signatory for Artan Prelaj was Artan Prelaj. The contract date was March 31, 2025. Prior sales, articles and revenue Prior to this transaction, PincusCo has no record that the buyer Artan Prelaj h</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>Juan Qing Lu pays $8M for Sirico’s banquet hall in Dyker Heights</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>https://www.pincusco.com/juan-qing-lu-pays-8m-to-hercules-sirico-and-james-t-sirico-for-five-properties-in-dyker-heights/</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>Juan Qing Lu through the entity JMAL Group LLC paid $8 million to the Sirico</t>
-        </is>
-      </c>
-      <c r="D7" t="inlineStr"/>
-      <c r="E7" t="inlineStr"/>
-      <c r="F7" t="inlineStr">
-        <is>
-          <t>PincusCo</t>
-        </is>
-      </c>
-      <c r="G7" t="inlineStr">
-        <is>
-          <t>PincusCo - Home</t>
-        </is>
-      </c>
-      <c r="H7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Transfers 8017 13th Avenue, et al (Credit - Cyclomedia) Juan Qing Lu through the entity JMAL Group LLC paid $8 million to the Sirico family through the entity JHS Realty Associates for Sirico’s Caterers banquet hall covering five tax lots making up the retail at 8023 13th Avenue in Dyker Heights, Brooklyn. The deal closed on June 1, 2026 and was recorded on June 12, 2026. The five properties have 14,160 square feet of built space and 7,240 square feet of additional air rights for a total buildable of 21,000 square feet according to a PincusCo analysis of city data. The sale price per built square foot is $564 and the price per buildable square foot is $380 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) The signatory for Hercules Sirico and James T. Sirico was Hercules Sirico and James T. Sirico. The signatory for Juan Qing Lu was Juan Qing Lu. The contract date was June 30, 2025. The Sirico family members were owners of Sirico’s Caterers, which is permanently closed as of late May, according to local media. Prior sales, articles and revenue Prior </t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>Hawkins Way pays $80M in sale-leaseback with college for dorm in Lincoln Square</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>https://www.pincusco.com/hawkins-way-pays-80m-in-sale-leaseback-with-college-for-dorm-in-lincoln-square/</t>
-        </is>
-      </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>Hawkins Way Capital through the entity 117 W 70th Owner, LLC paid $80 million to</t>
-        </is>
-      </c>
-      <c r="D8" t="inlineStr"/>
-      <c r="E8" t="inlineStr"/>
-      <c r="F8" t="inlineStr">
-        <is>
-          <t>PincusCo</t>
-        </is>
-      </c>
-      <c r="G8" t="inlineStr">
-        <is>
-          <t>PincusCo - Home</t>
-        </is>
-      </c>
-      <c r="H8" t="inlineStr">
-        <is>
-          <t>Top Story Transfers 117 West 70th Street (Credit - Cyclomedia) Hawkins Way Capital through the entity 117 W 70th Owner, LLC paid $80 million to American Musical and Dramatic Academy through the entity Manhattan Stratford Arms, Inc. for the dormitory, also known as a residence hall, building (H8) at 117 West 70th Street in Lincoln Square, Manhattan. The expected use is cash flowing as part of a sale-leaseback agreement. The American Musical Dramatic Academy, also known as AMDA, executed a $23 million sale-leaseback in 2023 in Los Angeles. The deal closed on May 7, 2026 and was recorded on June 12, 2026. The property has 75,313 square feet of built space according to a PincusCo analysis of city data. The sale price per built square foot is $1,062 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) The signatory for American Musical and Dramatic Academy was David Silverman . The signatory for Hawkins Way Capital was Joshua Bird . The contract date was May 7, 2026. Simultaneously with the purchase, the parties signed a 31-year lease commencing on May 7, 20</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>Medical spa owner pays $5M to Collins Ogbolu for mixed-use in Harlem</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>https://www.pincusco.com/medical-spa-owner-pays-5m-to-collins-ogbolu-for-mixed-use-in-harlem/</t>
-        </is>
-      </c>
-      <c r="C9" t="inlineStr">
-        <is>
-          <t>Richina Lukes, CEO of L’Elite MediSpa, through the entity Lenox 335, LLC paid $5 million</t>
-        </is>
-      </c>
-      <c r="D9" t="inlineStr"/>
-      <c r="E9" t="inlineStr"/>
-      <c r="F9" t="inlineStr">
-        <is>
-          <t>PincusCo</t>
-        </is>
-      </c>
-      <c r="G9" t="inlineStr">
-        <is>
-          <t>PincusCo - Home</t>
-        </is>
-      </c>
-      <c r="H9" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Transfers 335 Lenox Avenue (Credit - Cyclomedia) Richina Lukes, CEO of L’Elite MediSpa, through the entity Lenox 335, LLC paid $5 million for the four-unit mixed-use building (S9) at 335 Lenox Avenue in Harlem, Manhattan. The expected use is owner-occupied. The location has been occupied by a different laser spa center, recent images of the building show. The deal closed on May 13, 2026 and was recorded on June 12, 2026. The property has 6,648 square feet of built space and 975 square feet of additional air rights for a total buildable of 7,623 square feet according to a PincusCo analysis of city data. The sale price per built square foot is $752 and the price per buildable square foot is $655 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) The signatory for Collins Ogbolu was Collins J. Ogbolu . The signatory for Richina Lukes was Richina J. Lukes. The contract date was January 29, 2026. Prior sales, articles and revenue Prior to this transaction, PincusCo has no record that the buyer Richina J. Lukes had purchased any other properties and has no </t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>Vesper Holdings pays $2.8M to Cayuga Capital for mixed-use in Bushwick</t>
-        </is>
-      </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>https://www.pincusco.com/vesper-holdings-pays-2-8m-to-cayuga-capital-for-mixed-use-in-bushwick/</t>
-        </is>
-      </c>
-      <c r="C10" t="inlineStr">
-        <is>
-          <t>Vesper Holdings through the entity 287 Wyckoff Assc. LLC paid $2.8 million to Cayuga Capital</t>
-        </is>
-      </c>
-      <c r="D10" t="inlineStr"/>
-      <c r="E10" t="inlineStr"/>
-      <c r="F10" t="inlineStr">
-        <is>
-          <t>PincusCo</t>
-        </is>
-      </c>
-      <c r="G10" t="inlineStr">
-        <is>
-          <t>PincusCo - Home</t>
-        </is>
-      </c>
-      <c r="H10" t="inlineStr">
-        <is>
-          <t>Transfers 287 Wyckoff Avenue (Credit - Cyclomedia) Vesper Holdings through the entity 287 Wyckoff Assc. LLC paid $2.8 million to Cayuga Capital Management through the entity 287 Wyckoff LLC for the five-unit mixed-use building (S5) at 287 Wyckoff Avenue in Bushwick, Brooklyn. The expected use is cash flowing. The deal closed on May 20, 2026 and was recorded on June 12, 2026. The property has 4,050 square feet of built space and 1,101 square feet of additional air rights for a total buildable of 5,146 square feet according to a PincusCo analysis of city data. The sale price per built square foot is $691 and the price per buildable square foot is $544 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) The seller bought the property on April 29, 2015, for $1.2 million. The signatory for Cayuga Capital Management was Jacob Sacks . The signatory for Vesper Holdings was Elliot J. Tamir . The contract date was March 3, 2026. Prior sales, articles and revenue Prior to this transaction, PincusCo has no record that the buyer Vesper Holdings had purchased any ot</t>
+          <t>Transfers 425 West 57th Street (Credit - Cyclomedia) Gorjian Real Estate Group through the entity GG West 57 Owner LLC as borrower signed a refi loan with lender JPMorgan Chase valued at $14.7 million for the 50-unit residential elevator building (D1) at 425 West 57th Street in Hell’s Kitchen, Manhattan. The deal closed on June 5, 2026 and was recorded on June 12, 2026. The prior lender was Prime Finance which held debt that had an original loan amount of $13.5 million.The property has 39,210 square feet of built space and 21,289 square feet of additional air rights for a total buildable of 60,452 square feet according to a PincusCo analysis of city data. The loan price per built square foot is $373 and the price per buildable square foot is $242 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) The owner bought the property on September 9, 2024, for $16.5 million. The signatory for Gorjian Real Estate Group was Cobby Gorjian . The signatory for JPMorgan Chase was Ursula Flores . Prior sales, articles and revenue The owners according to the Departmen</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto update queens news 2026-06-17T16:00:54Z
</commit_message>
<xml_diff>
--- a/data/output/queens_dev_news.xlsx
+++ b/data/output/queens_dev_news.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H5"/>
+  <dimension ref="A1:H10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -473,17 +473,17 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Fei Guo pays $7.7M to Amos Financial for 19-unit rental in Clinton Hill</t>
+          <t>Related signs $1.37B refi with Wells, Deutsche, Goldman, Morgan Stanley for 10 Hudson Yards</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>https://www.pincusco.com/fei-guo-pays-7-7m-to-amos-financial-for-19-unit-rental-in-clinton-hill/</t>
+          <t>https://www.pincusco.com/related-signs-1-37b-refi-with-wells-deutsche-goldman-morgan-stanley-for-10-hudson-yards/</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Fei Guo through the entity Kg Atlantic Realty Holding Inc. paid $7.7 million through a</t>
+          <t>Related Companies and partner Oxford Properties Group through the entity Legacy Yards Tenant LP as</t>
         </is>
       </c>
       <c r="D2" t="inlineStr"/>
@@ -500,24 +500,24 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>Transfers 929 Atlantic Avenue (Credit - Cyclomedia) Fei Guo through the entity Kg Atlantic Realty Holding Inc. paid $7.7 million through a real estate owned sale to former lender Amos Financial for the 19-unit residential elevator building (D3) at 929 Atlantic Avenue in Clinton Hill, Brooklyn. The expected use is cash flowing. The deal closed on May 27, 2026 and was recorded on June 15, 2026. The property has 17,469 square feet of built space and 775 square feet of additional air rights for a total buildable of 18,240 square feet according to a PincusCo analysis of city data. The sale price per built square foot is $440 and the price per buildable square foot is $422 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) Amos Financial took title to the property on August 5, 2022. The signatory for Amos Financial was Ohannes Korogluyan . The signatory for Fei Guo was Fei Guo. The contract date was April 8, 2026. Prior sales, articles and revenue Prior to this transaction, PincusCo has no record that the buyer Fei Guo had purchased any other properties and</t>
+          <t>Transfers 501 West 30th Street (Credit - Cyclomedia) Related Companies and partner Oxford Properties Group through the entity Legacy Yards Tenant LP as borrower signed a refi loan with lender Wells Fargo, Deutsche Bank, Goldman Sachs, and Morgan Stanley valued at $1.37 billion for the office building (O4) at 10 Hudson Yards, also known as 501 West 30th Street in Hudson Yards, Manhattan. The deal closed on June 5, 2026 and was recorded on June 16, 2026. The prior lender was a trust Hudson Yards 2016-10HY as serviced by Trimont which held debt that had an original loan amount of $900 million. The property has 1,835,464 square feet of built space according to a PincusCo analysis of city data. The loan price per built square foot is $746 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) The owner bought the property on May 31, 2022, for $870 million. The signatory for Related Companies and Oxford Properties Group was Andrew Rosen . The signatory for Wells Fargo , Deutsche Bank , Goldman Sachs , and Morgan Stanley was John G. Nicol , David Goodman , Brand</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>99 units planned for Yossel Lichtman dev site in Greenpoint</t>
+          <t>Signs + Decal Corp. seeks zoning change to build 128K industrial building in East Williamsburg</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>https://www.pincusco.com/99-units-planned-for-yossel-lichtman-dev-site-in-greenpoint/</t>
+          <t>https://www.pincusco.com/signs-decal-corp-seeks-zoning-change-to-build-128k-industrial-building-in-east-williamsburg/</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>A new building construction project for a 99-unit, 105,210-square-foot residential (R-2) development at 70 West</t>
+          <t>Signs + Decal Corp., led by the Khalfan family, seeks a zoning change in order</t>
         </is>
       </c>
       <c r="D3" t="inlineStr"/>
@@ -534,24 +534,24 @@
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>Development 70 West Street axonometric diagram (Credit - Shmuel Wieder architect via DOB) A new building construction project for a 99-unit, 105,210-square-foot residential (R-2) development at 70 West Street in Greenpoint, Brooklyn, was filed on behalf of property owner and developer Yossel Lichtman. The plan was filed on June 11, 2026. It calls for the construction of a 95-foot-tall, nine-story building and was filed with the New York City Department of Buildings under job number B01411828. The project is described in the filing as: new 9 story and cellar mixed use building with 99 residential dwelling units. The applicant is the Registered Architect Shmuel Wieder of S. Wieder Architect P.C. Mendy Schwimmer submitted the plans. The ground floor includes five residential units along with a lobby, mail and package room, and 1,303 square feet of retail space. Floor two houses nine units plus recreation rooms. Floors three through six each contain 13 units. Floors seven, eight, and nine each hold 11 units. The cellar level accommodates mechanical systems, an electric meter room, water-sprinkler room, laundry facilities, a pet spa, trash compactor room, bicycle parking for 50 bicycles</t>
+          <t>Development 410 Morgan Avenue (Credit - Google Earth) Signs + Decal Corp., led by the Khalfan family, seeks a zoning change in order to build a 128,750-square-foot, 14-story building at 410 Morgan Avenue in East Williamsburg, Brooklyn, on top of its current single-story manufacturing and distribution center. The proposed action would change the current M1-1 light manufacturing designation to a mix of M2-4A and M2-1A zoning districts, in a city block bounded by Withers Street, Vandervoort Avenue, Jackson Street, and Morgan Avenue. A representative for Signs + Decal Corp. filed the application June 16, 2026, with the Department of City Planning as part of the Uniform Land Use Review Process (ULURP). Application 2022K0252 LINK</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Gotham Organization files 2 plans totaling 375 units in East New York</t>
+          <t>Esat Gashi pays $2.4M for 35-unit rental in Bedford Park</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>https://www.pincusco.com/gotham-organization-files-2-plans-totaling-375-units-in-east-new-york/</t>
+          <t>https://www.pincusco.com/esat-gashi-pays-2-4m-for-35-unit-rental-in-bedford-park/</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Gotham Organization filed two plans totaling 375 units in East New York, Brooklyn. In the</t>
+          <t>Esat Gashi through the entity 2810 Morris Owners LLC paid $2.4 million to Stuart Oppenheimer</t>
         </is>
       </c>
       <c r="D4" t="inlineStr"/>
@@ -568,24 +568,24 @@
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>Development 12030 Flatlands Avenue axonometric diagram (Credit - Gloria Glas architect via DOB) Gotham Organization filed two plans totaling 375 units in East New York, Brooklyn. In the large, Gotham Organization submitted a new building construction project for a 206-unit, 144,132-square-foot residential (R-2) building at 12030 Flatlands Avenue in East New York, Brooklyn. The plan was filed on June 10, 2026. It calls for the construction of a 126-foot-tall, thirteen-story building and was filed with the New York City Department of Buildings under job number B01412655. The project is described in the filing as: construct new 13 story mixed use building as per plans filed. The applicant is the Registered Architect Gloria Glas of Slce Architects. David Picket of Gotham Organization submitted the plans. In the smaller, Gotham Organization submitted a new building construction project for a 169-unit, 173,805-square-foot residential (R-2) building at 395 Louisiana Avenue in East New York, Brooklyn. The plan was filed on June 10, 2026. It calls for the construction of a 114-foot-tall, twelve-story building and was filed with the New York City Department of Buildings under job number B014</t>
+          <t>Transfers 2810 Morris Avenue (Credit - Cyclomedia) Esat Gashi through the entity 2810 Morris Owners LLC paid $2.4 million to Stuart Oppenheimer through the entity 2810 Morris Ave. Corp. for the 35-unit residential elevator building (D1) at 2810 Morris Avenue in Bedford Park, Bronx. The expected use is cash flowing. The deal closed on June 2, 2026 and was recorded on June 15, 2026. The property has 36,900 square feet of built space and 5,985 square feet of additional air rights for a total buildable of 42,892 square feet according to a PincusCo analysis of city data. The sale price per built square foot is $65 and the price per buildable square foot is $55 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) The signatory for Stuart Oppenheimer was Stuart Oppenheimer. The signatory for Esat Gashi was Esat Gashi. The contract date was December 19, 2025. Prior sales, articles and revenue Prior to this transaction, PincusCo has records that the buyer Esat Gashi purchased three properties in three transactions for a total of $6.8 million and has no record it</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Gorjian Real Estate signs $14.7M refi with Chase for 50-unit rental in Hell’s Kitchen</t>
+          <t>Sackman Enterprises signs $36.5M refi with Berkadia for four walkups in East Village</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>https://www.pincusco.com/gorjian-real-estate-signs-14-7m-refi-with-chase-for-50-unit-rental-in-hells-kitchen/</t>
+          <t>https://www.pincusco.com/sackman-enterprises-signs-36-5m-refi-with-berkadia-for-four-walkups-in-east-village/</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Gorjian Real Estate Group through the entity GG West 57 Owner LLC as borrower signed</t>
+          <t>Sackman Enterprises through the entity E &amp; S Realty De LLC as borrower signed a</t>
         </is>
       </c>
       <c r="D5" t="inlineStr"/>
@@ -602,7 +602,177 @@
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>Transfers 425 West 57th Street (Credit - Cyclomedia) Gorjian Real Estate Group through the entity GG West 57 Owner LLC as borrower signed a refi loan with lender JPMorgan Chase valued at $14.7 million for the 50-unit residential elevator building (D1) at 425 West 57th Street in Hell’s Kitchen, Manhattan. The deal closed on June 5, 2026 and was recorded on June 12, 2026. The prior lender was Prime Finance which held debt that had an original loan amount of $13.5 million.The property has 39,210 square feet of built space and 21,289 square feet of additional air rights for a total buildable of 60,452 square feet according to a PincusCo analysis of city data. The loan price per built square foot is $373 and the price per buildable square foot is $242 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) The owner bought the property on September 9, 2024, for $16.5 million. The signatory for Gorjian Real Estate Group was Cobby Gorjian . The signatory for JPMorgan Chase was Ursula Flores . Prior sales, articles and revenue The owners according to the Departmen</t>
+          <t>Transfers Sackman Enterprises through the entity E &amp; S Realty De LLC as borrower signed a refi loan with lender Berkadia Commercial Mortgage valued at $36.5 million for four walkup properties with 96 residential units in the East Village of Manhattan, including the 26-unit walkup (C4) at 231 East 13th Street, the 24-unit walkup (C4) at 239 East 13th Street, and the 23-unit walkup (C4) at 235 East 13th Street. The deal closed on May 22, 2026 and was recorded on June 15, 2026. The prior lender was JPMorgan Chase which held debt that had an original loan amount of $25 million. The four properties have 59,646 square feet of built space according to a PincusCo analysis of city data. The loan price per built square foot is $611 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) The signatory for Sackman Enterprises was Alan Sackman . The signatory for Berkadia Commercial Mortgage was Megan Mather . Because multiple properties have been transacted, some of the following sections will follow the property with the largest assessed value, which in this case, is</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Yitzchok Lebowitz pays $2.4M for 3-family in Bedford Stuyvesant</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>https://www.pincusco.com/yitzchok-lebowitz-pays-2-4m-for-3-family-in-bedford-stuyvesant/</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Yitzchok Lebowitz through the entity 209 Skillman Place LLC paid $2.4 million to Pablo Cedeno</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr"/>
+      <c r="E6" t="inlineStr"/>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>PincusCo</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>PincusCo - Home</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Transfers 209 Skillman Street (Credit - Cyclomedia) Yitzchok Lebowitz through the entity 209 Skillman Place LLC paid $2.4 million to Pablo Cedeno for the three-unit building (C0) at 209 Skillman Street in Bedford Stuyvesant, Brooklyn. The expected use is cash flowing. The deal closed on May 14, 2026 and was recorded on June 15, 2026. The property has 2,520 square feet of built space and 1,237 square feet of additional air rights for a total buildable of 3,750 square feet according to a PincusCo analysis of city data. The sale price per built square foot is $932 and the price per buildable square foot is $626 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) The signatory for Pablo Cedeno was Pablo Cedeno. The signatory for Yitzchok Lebowitz was Yitzchok Lebowitz. The contract date was December 12, 2025. Prior sales, articles and revenue Prior to this transaction, PincusCo has records that the buyer Yitzchok Lebowitz purchased one property in one transaction for a total of $5.1 million and has no record it sold any properties over the past 24 months. </t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Rabsky Group signs $32M refi loan with Cross River Bank for office in Williamsburg</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>https://www.pincusco.com/rabsky-group-signs-32m-refi-loan-with-cross-river-bank-for-office-in-williamsburg/</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Rabsky Group through the entity 103 North 13th Street LLC as borrower signed a refi</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr"/>
+      <c r="E7" t="inlineStr"/>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>PincusCo</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>PincusCo - Home</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>Transfers 103 North 13th Street (Credit - Cyclomedia) Rabsky Group through the entity 103 North 13th Street LLC as borrower signed a refi loan with lender Cross River Bank valued at $32 million for the office building (O6) at 103 North 13th Street in Williamsburg, Brooklyn. The deal closed on June 5, 2026 and was recorded on June 15, 2026. The prior lender was Deutsche Bank which held debt that had an original loan amount of $41.5 million.The property has 62,779 square feet of built space according to a PincusCo analysis of city data. The loan price per built square foot is $509 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) The owner bought the property on June 2, 2014, for $8.2 million. The signatory for Rabsky Group was Shimon Dushinsky . The signatory for Cross River Bank was Shimon Eisikowicz . Prior sales, articles and revenue The 62,779-square-foot property generated revenue of $2.5 million or $41 per square foot, according to the most recent income and expense figures. The property</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Furen Dai pays $2.4M to Ambrosino Equities for industrial in East Williamsburg</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>https://www.pincusco.com/furen-dai-pays-2-4m-to-ambrosino-equities-for-industrial-in-east-williamsburg/</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Furen Dai through the entity 972 Metropolitan Management LLC paid $2.4 million to Ambrosino Equities</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr"/>
+      <c r="E8" t="inlineStr"/>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>PincusCo</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>PincusCo - Home</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Transfers 972 Metropolitan Avenue (Credit - Cyclomedia) Furen Dai through the entity 972 Metropolitan Management LLC paid $2.4 million to Ambrosino Equities through the entity 972 Metro LLC for the industrial building (F5) at 972 Metropolitan Avenue in East Williamsburg, Brooklyn. The deal closed on May 28, 2026 and was recorded on June 15, 2026. The property has 3,179 square feet of built space for a total buildable of 3,190 square feet according to a PincusCo analysis of city data. The sale price per built square foot is $754 and the price per buildable square foot is $752 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) The signatory for Ambrosino Equities was Antonio Ambrosino . The signatory for Furen Dai was Furen Dai. The contract date was January 30, 2026. Prior sales, articles and revenue Prior to this transaction, PincusCo has no record that the buyer had purchased any other properties and has no record it sold any properties over the past 24 months. The seller Ambrosino Equities had not purchased any other properties and had not sold any </t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Glenwood Management signs $38M refi with Wells Fargo for 272-unit rental in Yorkville</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>https://www.pincusco.com/glenwood-management-signs-38m-refi-with-wells-fargo-for-272-unit-rental-in-yorkville/</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Glenwood Management through the entity 92nd Realty LLC as borrower signed a refi loan with</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr"/>
+      <c r="E9" t="inlineStr"/>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>PincusCo</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>PincusCo - Home</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>Transfers 1775 York Avenue (Credit - Cyclomedia) Glenwood Management through the entity 92nd Realty LLC as borrower signed a refi loan with lender Wells Fargo valued at $38 million for the 272-unit residential elevator building (D6) at 1775 York Avenue in Yorkville, Manhattan. The deal closed on June 4, 2026 and was recorded on June 15, 2026. The prior lender was Fannie Mae which held debt that had an original loan amount of $57 million. The property has 347,118 square feet of built space according to a PincusCo analysis of city data. The loan price per built square foot is $109 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) The signatory for Glenwood Management was Howard Swarzman . The signatory for Wells Fargo was Tom Merkle . Prior sales, articles and revenue The owners according to the Department of Housing Preservation and Development includes Carole Pittelman , head officer and New Hyde Park Realty L.P, shareholder. The business entities are Glenwood Management Corp. and 92nd Realty LLC. The 347,118-square-foot property generated revenue of</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Iglesia Pentecostal La Santa Ciudad pays $3.1M to Meir Zarchi for mixed-use in East Harlem</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>https://www.pincusco.com/iglesia-pentecostal-la-santa-ciudad-pays-3-1m-to-meir-zarchi-for-mixed-use-in-east-harlem/</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Iglesia Pentecostal La Santa Ciudad through the entity Iglesia Pentecostal La Santa Ciudad, Inc. paid</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr"/>
+      <c r="E10" t="inlineStr"/>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>PincusCo</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>PincusCo - Home</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>Transfers 2323 1st Avenue (Credit - Cyclomedia) Iglesia Pentecostal La Santa Ciudad through the entity Iglesia Pentecostal La Santa Ciudad, Inc. paid $3.1 million to Meir Zarchi through the entity 2323 1st Ave LLC for the mixed-use building (K4) at 2323 1st Avenue in East Harlem, Manhattan. The expected use is owner-occupied. The deal closed on May 21, 2026 and was recorded on June 15, 2026. The property has 4,500 square feet of built space and 6,932 square feet of additional air rights for a total buildable of 11,440 square feet according to a PincusCo analysis of city data. The sale price per built square foot is $688 and the price per buildable square foot is $270 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) The seller bought the property on September 29, 2016, for $2.5 million. The signatory for Meir Zarchi was Avinoan Rosenfeid . The signatory for Iglesia Pentecostal La Santa Ciudad was Victor Pimentel. The contract date was April 1, 2026. Prior sales, articles and revenue Prior to this transaction, PincusCo has no record that the buyer Igl</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto update queens news 2026-06-18T15:50:51Z
</commit_message>
<xml_diff>
--- a/data/output/queens_dev_news.xlsx
+++ b/data/output/queens_dev_news.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H10"/>
+  <dimension ref="A1:H8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -473,17 +473,17 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Related signs $1.37B refi with Wells, Deutsche, Goldman, Morgan Stanley for 10 Hudson Yards</t>
+          <t>Arkview Capital acquires Midtown West parking from Tribeach Holdings in $6M deed-in-lieu</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>https://www.pincusco.com/related-signs-1-37b-refi-with-wells-deutsche-goldman-morgan-stanley-for-10-hudson-yards/</t>
+          <t>https://www.pincusco.com/arkview-capital-pays-6m-to-tribeach-holdings-for-parking-space-in-midtown-west/</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Related Companies and partner Oxford Properties Group through the entity Legacy Yards Tenant LP as</t>
+          <t>Arkview Capital through the entity Ark FP Holdings Llc acquired from Tribeach Holdings through the</t>
         </is>
       </c>
       <c r="D2" t="inlineStr"/>
@@ -500,24 +500,24 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>Transfers 501 West 30th Street (Credit - Cyclomedia) Related Companies and partner Oxford Properties Group through the entity Legacy Yards Tenant LP as borrower signed a refi loan with lender Wells Fargo, Deutsche Bank, Goldman Sachs, and Morgan Stanley valued at $1.37 billion for the office building (O4) at 10 Hudson Yards, also known as 501 West 30th Street in Hudson Yards, Manhattan. The deal closed on June 5, 2026 and was recorded on June 16, 2026. The prior lender was a trust Hudson Yards 2016-10HY as serviced by Trimont which held debt that had an original loan amount of $900 million. The property has 1,835,464 square feet of built space according to a PincusCo analysis of city data. The loan price per built square foot is $746 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) The owner bought the property on May 31, 2022, for $870 million. The signatory for Related Companies and Oxford Properties Group was Andrew Rosen . The signatory for Wells Fargo , Deutsche Bank , Goldman Sachs , and Morgan Stanley was John G. Nicol , David Goodman , Brand</t>
+          <t>Transfers 145 West 47th Street (Credit - Cyclomedia) Arkview Capital through the entity Ark FP Holdings Llc acquired from Tribeach Holdings through the entity Fastnet Parking LLC, the parking commercial condominium unit at 145 West 47th Street in Midtown West, Manhattan, through a $6 million deed-in-lieu of foreclosure. The expected use is hold for sale. The deal closed on June 1, 2026 and was recorded on June 17, 2026. The property has 30,233 square feet of built space according to a PincusCo analysis of city data. The sale price per built square foot is $198 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) The seller bought the property on May 31, 2022, for $3.8 million. The signatory for Tribeach Holdings was Adrian Stroie . The signatory for Arkview Capital was Vijay Mehta . The contract date was June 1, 2026. The document is titled a deed in lieu of foreclosure. Tribeach Holdings borrowed $5.6 million from Arkview Capital for the parking unit in 145 West 47th Street, Midtown West, Manhattan on April 26, 2024. The rest of the building is a hotel</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Signs + Decal Corp. seeks zoning change to build 128K industrial building in East Williamsburg</t>
+          <t>Vilson Lumaj pays $10M for dev site in Tremont</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>https://www.pincusco.com/signs-decal-corp-seeks-zoning-change-to-build-128k-industrial-building-in-east-williamsburg/</t>
+          <t>https://www.pincusco.com/vilson-lumaj-pays-10m-for-dev-site-in-tremont/</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Signs + Decal Corp., led by the Khalfan family, seeks a zoning change in order</t>
+          <t>Vilson Lumaj through the entity 761 East Tremont Avenue LLC paid $10 million to Shmouel</t>
         </is>
       </c>
       <c r="D3" t="inlineStr"/>
@@ -534,24 +534,24 @@
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>Development 410 Morgan Avenue (Credit - Google Earth) Signs + Decal Corp., led by the Khalfan family, seeks a zoning change in order to build a 128,750-square-foot, 14-story building at 410 Morgan Avenue in East Williamsburg, Brooklyn, on top of its current single-story manufacturing and distribution center. The proposed action would change the current M1-1 light manufacturing designation to a mix of M2-4A and M2-1A zoning districts, in a city block bounded by Withers Street, Vandervoort Avenue, Jackson Street, and Morgan Avenue. A representative for Signs + Decal Corp. filed the application June 16, 2026, with the Department of City Planning as part of the Uniform Land Use Review Process (ULURP). Application 2022K0252 LINK</t>
+          <t>Transfers 761 East Tremont Avenue (Credit - Cyclomedia) Vilson Lumaj through the entity 761 East Tremont Avenue LLC paid $10 million to Shmouel Toledano through the entity Strong Equities, Inc. for the retail building (K1) at 761 East Tremont Avenue in Tremont, Bronx. The expected use is ground up development. The deal closed on June 12, 2026 and was recorded on June 17, 2026. The property has 15,555 square feet of built space and 54,425 square feet of additional air rights for a total buildable of 70,000 square feet according to a PincusCo analysis of city data. The sale price per built square foot is $642 and the price per buildable square foot is $142 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) The signatory for Shmouel Toledano was Shmouel Toledano. The signatory for Vilson Lumaj was Vilson Lumaj . The contract date was March 23, 2026. A Rosewood Realty Group team of Jonah Corney, Mike Kerwin and Mark Steinmetz brokered the sale. The property was being marketing as a development site, 761-769 East Tremont Avenue listing. Prior sales, articl</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Esat Gashi pays $2.4M for 35-unit rental in Bedford Park</t>
+          <t>Educational Institute Oholei Torah of Brooklyn pays $16.1M for school in Crown Heights</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>https://www.pincusco.com/esat-gashi-pays-2-4m-for-35-unit-rental-in-bedford-park/</t>
+          <t>https://www.pincusco.com/educational-institute-oholei-torah-of-brooklyn-pays-16-1m-to-taormina-holding-for-specialty-in-crown-heights/</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Esat Gashi through the entity 2810 Morris Owners LLC paid $2.4 million to Stuart Oppenheimer</t>
+          <t>Educational Institute Oholei Torah of Brooklyn through the entity Ot 402 Eastern LLC paid $16.1</t>
         </is>
       </c>
       <c r="D4" t="inlineStr"/>
@@ -568,24 +568,24 @@
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>Transfers 2810 Morris Avenue (Credit - Cyclomedia) Esat Gashi through the entity 2810 Morris Owners LLC paid $2.4 million to Stuart Oppenheimer through the entity 2810 Morris Ave. Corp. for the 35-unit residential elevator building (D1) at 2810 Morris Avenue in Bedford Park, Bronx. The expected use is cash flowing. The deal closed on June 2, 2026 and was recorded on June 15, 2026. The property has 36,900 square feet of built space and 5,985 square feet of additional air rights for a total buildable of 42,892 square feet according to a PincusCo analysis of city data. The sale price per built square foot is $65 and the price per buildable square foot is $55 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) The signatory for Stuart Oppenheimer was Stuart Oppenheimer. The signatory for Esat Gashi was Esat Gashi. The contract date was December 19, 2025. Prior sales, articles and revenue Prior to this transaction, PincusCo has records that the buyer Esat Gashi purchased three properties in three transactions for a total of $6.8 million and has no record it</t>
+          <t>Transfers 402 Eastern Parkway (Credit - Cyclomedia) Educational Institute Oholei Torah of Brooklyn through the entity Ot 402 Eastern LLC paid $16.1 million to Taormina Holding through the entity Eastern Union Properties, Inc. for the school building (W1) at 402 Eastern Parkway in Crown Heights, Brooklyn. The expected use is owner-occupied. The deal closed on June 3, 2026 and was recorded on June 17, 2026. The property has 57,840 square feet of built space according to a PincusCo analysis of city data. The sale price per built square foot is $277 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) The signatory for Taormina Holding was Joseph Taormina . The signatory for Educational Institute Oholei Torah of Brooklyn was Shmuel Brook. The contract date was February 10, 2026. New York Business Journal reported on this purchase yesterday. Prior sales, articles and revenue Prior to this transaction, PincusCo has records that the buyer Educational Institute Oholei Torah of Brooklyn purchased one property in one transaction for a total of $8.5 million and ha</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Sackman Enterprises signs $36.5M refi with Berkadia for four walkups in East Village</t>
+          <t>Hartz Mountain Industries pays $4.8M for dev site in SoHo</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>https://www.pincusco.com/sackman-enterprises-signs-36-5m-refi-with-berkadia-for-four-walkups-in-east-village/</t>
+          <t>https://www.pincusco.com/hartz-mountain-industries-pays-4-8m-for-dev-site-in-soho/</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Sackman Enterprises through the entity E &amp; S Realty De LLC as borrower signed a</t>
+          <t>Hartz Mountain Industries through the entity 391 Canal Street Soho LLC paid $4.8 million to</t>
         </is>
       </c>
       <c r="D5" t="inlineStr"/>
@@ -602,24 +602,24 @@
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>Transfers Sackman Enterprises through the entity E &amp; S Realty De LLC as borrower signed a refi loan with lender Berkadia Commercial Mortgage valued at $36.5 million for four walkup properties with 96 residential units in the East Village of Manhattan, including the 26-unit walkup (C4) at 231 East 13th Street, the 24-unit walkup (C4) at 239 East 13th Street, and the 23-unit walkup (C4) at 235 East 13th Street. The deal closed on May 22, 2026 and was recorded on June 15, 2026. The prior lender was JPMorgan Chase which held debt that had an original loan amount of $25 million. The four properties have 59,646 square feet of built space according to a PincusCo analysis of city data. The loan price per built square foot is $611 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) The signatory for Sackman Enterprises was Alan Sackman . The signatory for Berkadia Commercial Mortgage was Megan Mather . Because multiple properties have been transacted, some of the following sections will follow the property with the largest assessed value, which in this case, is</t>
+          <t>Transfers 391 Canal Street (Credit - Cyclomedia) Hartz Mountain Industries through the entity 391 Canal Street Soho LLC paid $4.8 million to Tomer Hillel through the entity H Mazal LLC for the retail building (K1) at 391 Canal Street in SoHo, Manhattan. The expected use is ground up development. The deal closed on June 12, 2026 and was recorded on June 17, 2026. The property has 2,208 square feet of built space and 13,979 square feet of additional air rights for a total buildable of 16,180 square feet according to a PincusCo analysis of city data. The sale price per built square foot is $2,196 and the price per buildable square foot is $299 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) The seller bought the property on September 10, 2024, for $3 million. The signatory for Tomer Hillel was Tomer Hillel. The signatory for Hartz Mountain Industries was Phillip R. Patton . The contract date was May 14, 2026. Prior sales, articles and revenue Prior to this transaction, PincusCo has no record that the buyer Hartz Mountain Industries had purchased any o</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Yitzchok Lebowitz pays $2.4M for 3-family in Bedford Stuyvesant</t>
+          <t>Nalcorp pays $21.7M to Altmark Group for 297-unit dev site in Mott Haven</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>https://www.pincusco.com/yitzchok-lebowitz-pays-2-4m-for-3-family-in-bedford-stuyvesant/</t>
+          <t>https://www.pincusco.com/nalcorp-pays-21-7m-to-altmark-group-for-297-unit-dev-site-in-mott-haven/</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Yitzchok Lebowitz through the entity 209 Skillman Place LLC paid $2.4 million to Pablo Cedeno</t>
+          <t>Nalcorp through the entity 122 Blvd 134 St LLC paid $21.7 million to Altmark Group</t>
         </is>
       </c>
       <c r="D6" t="inlineStr"/>
@@ -636,24 +636,24 @@
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t xml:space="preserve">Transfers 209 Skillman Street (Credit - Cyclomedia) Yitzchok Lebowitz through the entity 209 Skillman Place LLC paid $2.4 million to Pablo Cedeno for the three-unit building (C0) at 209 Skillman Street in Bedford Stuyvesant, Brooklyn. The expected use is cash flowing. The deal closed on May 14, 2026 and was recorded on June 15, 2026. The property has 2,520 square feet of built space and 1,237 square feet of additional air rights for a total buildable of 3,750 square feet according to a PincusCo analysis of city data. The sale price per built square foot is $932 and the price per buildable square foot is $626 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) The signatory for Pablo Cedeno was Pablo Cedeno. The signatory for Yitzchok Lebowitz was Yitzchok Lebowitz. The contract date was December 12, 2025. Prior sales, articles and revenue Prior to this transaction, PincusCo has records that the buyer Yitzchok Lebowitz purchased one property in one transaction for a total of $5.1 million and has no record it sold any properties over the past 24 months. </t>
+          <t>Top Story Transfers 122 Bruckner Boulevard, 20 Brook Avenue, 521 East 132nd Street (Credit - Google Earth) Nalcorp through the entity 122 Blvd 134 St LLC paid $21.7 million to Altmark Group through the entity 122 Bruckner Development LLC for three adjacent tax lots in Mott Haven, the Bronx, where the buyer has filed plans for a total of 297 units in three projects. The parcels are the industrial building (G9) at 517 East 132nd Street, the industrial building (F5) at 519 East 132nd Street, and the specialty building (Z9) at 122 Bruckner Boulevard. The expected use is ground up development. The deal closed on June 12, 2026 and was recorded on June 17, 2026. The three properties have 19,866 square feet of built space and 152,917 square feet of additional air rights for a total buildable of 172,774 square feet according to a PincusCo analysis of city data. The sale price per built square foot is $1,092 and the price per buildable square foot is $125 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) The signatory for Altmark Group was Adi Altmark . The si</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Rabsky Group signs $32M refi loan with Cross River Bank for office in Williamsburg</t>
+          <t>Palwinder Singh signs $10M construction loan for 32-unit project in LIC</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>https://www.pincusco.com/rabsky-group-signs-32m-refi-loan-with-cross-river-bank-for-office-in-williamsburg/</t>
+          <t>https://www.pincusco.com/palwinder-singh-signs-10m-construction-loan-for-32-unit-project-in-lic/</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Rabsky Group through the entity 103 North 13th Street LLC as borrower signed a refi</t>
+          <t>Palwinder Singh through the entity 31st Street LIC Property LLC as borrower signed a new</t>
         </is>
       </c>
       <c r="D7" t="inlineStr"/>
@@ -670,24 +670,24 @@
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>Transfers 103 North 13th Street (Credit - Cyclomedia) Rabsky Group through the entity 103 North 13th Street LLC as borrower signed a refi loan with lender Cross River Bank valued at $32 million for the office building (O6) at 103 North 13th Street in Williamsburg, Brooklyn. The deal closed on June 5, 2026 and was recorded on June 15, 2026. The prior lender was Deutsche Bank which held debt that had an original loan amount of $41.5 million.The property has 62,779 square feet of built space according to a PincusCo analysis of city data. The loan price per built square foot is $509 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) The owner bought the property on June 2, 2014, for $8.2 million. The signatory for Rabsky Group was Shimon Dushinsky . The signatory for Cross River Bank was Shimon Eisikowicz . Prior sales, articles and revenue The 62,779-square-foot property generated revenue of $2.5 million or $41 per square foot, according to the most recent income and expense figures. The property</t>
+          <t xml:space="preserve">Transfers 36-32 31st Street axonometric diagram (Credit - Gerald Caliendo architect via DOB) Palwinder Singh through the entity 31st Street LIC Property LLC as borrower signed a new construction loan with lender Ponce Bank valued at $10 million for the 32-unit development project at 36-31 31st Street in Long Island City, Queens. On the lot, there is one active new building construction project, Q01136795, for a 32-unit, 22,381 square-foot residential (R-2) building. The project was submitted by Palwinder Singh and filed by Palwinder Singh with plans filed November 5, 2024 and it has not been permitted yet. The deal closed on June 8, 2026 and was recorded on June 15, 2026. The property has zero square feet of built space and 17,214 square feet of additional air rights for a total buildable of 17,214 square feet according to a PincusCo analysis of city data. The loan price per planned development zoning square foot is $447 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) The owner bought the property on August 8, 2024, for $3.4 million. The signatory </t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Furen Dai pays $2.4M to Ambrosino Equities for industrial in East Williamsburg</t>
+          <t>Joel Schwartz signs $28.5M construction loan with S3 for 60-unit dev site in Bushwick</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>https://www.pincusco.com/furen-dai-pays-2-4m-to-ambrosino-equities-for-industrial-in-east-williamsburg/</t>
+          <t>https://www.pincusco.com/joel-schwartz-signs-28-5m-construction-loan-with-s3-for-60-unit-dev-site-in-bushwick/</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Furen Dai through the entity 972 Metropolitan Management LLC paid $2.4 million to Ambrosino Equities</t>
+          <t>Joel Schwartz through the entity Grove Menahan BK LLC as borrower signed a new construction</t>
         </is>
       </c>
       <c r="D8" t="inlineStr"/>
@@ -704,75 +704,7 @@
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t xml:space="preserve">Transfers 972 Metropolitan Avenue (Credit - Cyclomedia) Furen Dai through the entity 972 Metropolitan Management LLC paid $2.4 million to Ambrosino Equities through the entity 972 Metro LLC for the industrial building (F5) at 972 Metropolitan Avenue in East Williamsburg, Brooklyn. The deal closed on May 28, 2026 and was recorded on June 15, 2026. The property has 3,179 square feet of built space for a total buildable of 3,190 square feet according to a PincusCo analysis of city data. The sale price per built square foot is $754 and the price per buildable square foot is $752 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) The signatory for Ambrosino Equities was Antonio Ambrosino . The signatory for Furen Dai was Furen Dai. The contract date was January 30, 2026. Prior sales, articles and revenue Prior to this transaction, PincusCo has no record that the buyer had purchased any other properties and has no record it sold any properties over the past 24 months. The seller Ambrosino Equities had not purchased any other properties and had not sold any </t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>Glenwood Management signs $38M refi with Wells Fargo for 272-unit rental in Yorkville</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>https://www.pincusco.com/glenwood-management-signs-38m-refi-with-wells-fargo-for-272-unit-rental-in-yorkville/</t>
-        </is>
-      </c>
-      <c r="C9" t="inlineStr">
-        <is>
-          <t>Glenwood Management through the entity 92nd Realty LLC as borrower signed a refi loan with</t>
-        </is>
-      </c>
-      <c r="D9" t="inlineStr"/>
-      <c r="E9" t="inlineStr"/>
-      <c r="F9" t="inlineStr">
-        <is>
-          <t>PincusCo</t>
-        </is>
-      </c>
-      <c r="G9" t="inlineStr">
-        <is>
-          <t>PincusCo - Home</t>
-        </is>
-      </c>
-      <c r="H9" t="inlineStr">
-        <is>
-          <t>Transfers 1775 York Avenue (Credit - Cyclomedia) Glenwood Management through the entity 92nd Realty LLC as borrower signed a refi loan with lender Wells Fargo valued at $38 million for the 272-unit residential elevator building (D6) at 1775 York Avenue in Yorkville, Manhattan. The deal closed on June 4, 2026 and was recorded on June 15, 2026. The prior lender was Fannie Mae which held debt that had an original loan amount of $57 million. The property has 347,118 square feet of built space according to a PincusCo analysis of city data. The loan price per built square foot is $109 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) The signatory for Glenwood Management was Howard Swarzman . The signatory for Wells Fargo was Tom Merkle . Prior sales, articles and revenue The owners according to the Department of Housing Preservation and Development includes Carole Pittelman , head officer and New Hyde Park Realty L.P, shareholder. The business entities are Glenwood Management Corp. and 92nd Realty LLC. The 347,118-square-foot property generated revenue of</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>Iglesia Pentecostal La Santa Ciudad pays $3.1M to Meir Zarchi for mixed-use in East Harlem</t>
-        </is>
-      </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>https://www.pincusco.com/iglesia-pentecostal-la-santa-ciudad-pays-3-1m-to-meir-zarchi-for-mixed-use-in-east-harlem/</t>
-        </is>
-      </c>
-      <c r="C10" t="inlineStr">
-        <is>
-          <t>Iglesia Pentecostal La Santa Ciudad through the entity Iglesia Pentecostal La Santa Ciudad, Inc. paid</t>
-        </is>
-      </c>
-      <c r="D10" t="inlineStr"/>
-      <c r="E10" t="inlineStr"/>
-      <c r="F10" t="inlineStr">
-        <is>
-          <t>PincusCo</t>
-        </is>
-      </c>
-      <c r="G10" t="inlineStr">
-        <is>
-          <t>PincusCo - Home</t>
-        </is>
-      </c>
-      <c r="H10" t="inlineStr">
-        <is>
-          <t>Transfers 2323 1st Avenue (Credit - Cyclomedia) Iglesia Pentecostal La Santa Ciudad through the entity Iglesia Pentecostal La Santa Ciudad, Inc. paid $3.1 million to Meir Zarchi through the entity 2323 1st Ave LLC for the mixed-use building (K4) at 2323 1st Avenue in East Harlem, Manhattan. The expected use is owner-occupied. The deal closed on May 21, 2026 and was recorded on June 15, 2026. The property has 4,500 square feet of built space and 6,932 square feet of additional air rights for a total buildable of 11,440 square feet according to a PincusCo analysis of city data. The sale price per built square foot is $688 and the price per buildable square foot is $270 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) The seller bought the property on September 29, 2016, for $2.5 million. The signatory for Meir Zarchi was Avinoan Rosenfeid . The signatory for Iglesia Pentecostal La Santa Ciudad was Victor Pimentel. The contract date was April 1, 2026. Prior sales, articles and revenue Prior to this transaction, PincusCo has no record that the buyer Igl</t>
+          <t xml:space="preserve">Transfers 111 Grove Street rendering (Credit - Diego Aguilera Architects via DOB) Joel Schwartz through the entity Grove Menahan BK LLC as borrower signed a new construction loan with lender S3 Capital through the entity S3 Re Menahan Grove Funding LLC valued at $28.5 million for the two-parcel development site at 111 Grove Street in Bushwick, Brooklyn. The loan closed on June 1, 2026 and was recorded on June 16, 2026. The loan price per planned zoning square foot is $659 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) The signatory for Joel Schwartz was Joel Schwartz. Joel Schwartz through the entity Grove Menahan BK LLC bought the site for $6 million from Moshe Granit through the entity 115-117 Grove St LLC on June 1, 2026. There is a new building project, B01391270, for a 60-unit, 43,227 square-foot residential (R-2) building submitted by Jerome Zwick and filed by Jerome Zwick with plans filed May 6, 2026 and it has not been permitted yet. The six-story building project has 10 residential units on each floor from one to six. There are no retail </t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto update queens news 2026-06-19T15:38:55Z
</commit_message>
<xml_diff>
--- a/data/output/queens_dev_news.xlsx
+++ b/data/output/queens_dev_news.xlsx
@@ -473,17 +473,17 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Arkview Capital acquires Midtown West parking from Tribeach Holdings in $6M deed-in-lieu</t>
+          <t>Rudin ups debt from $76M to $140M with PGIM for office in Flatiron District</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>https://www.pincusco.com/arkview-capital-pays-6m-to-tribeach-holdings-for-parking-space-in-midtown-west/</t>
+          <t>https://www.pincusco.com/rudin-ups-debt-from-76m-to-140m-with-pgim-for-office-in-flatiron-district/</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Arkview Capital through the entity Ark FP Holdings Llc acquired from Tribeach Holdings through the</t>
+          <t>Rudin Management through the entity 41 Madiosn L.P. as borrower signed a refi loan with</t>
         </is>
       </c>
       <c r="D2" t="inlineStr"/>
@@ -500,24 +500,24 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>Transfers 145 West 47th Street (Credit - Cyclomedia) Arkview Capital through the entity Ark FP Holdings Llc acquired from Tribeach Holdings through the entity Fastnet Parking LLC, the parking commercial condominium unit at 145 West 47th Street in Midtown West, Manhattan, through a $6 million deed-in-lieu of foreclosure. The expected use is hold for sale. The deal closed on June 1, 2026 and was recorded on June 17, 2026. The property has 30,233 square feet of built space according to a PincusCo analysis of city data. The sale price per built square foot is $198 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) The seller bought the property on May 31, 2022, for $3.8 million. The signatory for Tribeach Holdings was Adrian Stroie . The signatory for Arkview Capital was Vijay Mehta . The contract date was June 1, 2026. The document is titled a deed in lieu of foreclosure. Tribeach Holdings borrowed $5.6 million from Arkview Capital for the parking unit in 145 West 47th Street, Midtown West, Manhattan on April 26, 2024. The rest of the building is a hotel</t>
+          <t>Transfers 41 Madison Avenue (Credit - Cyclomedia) Rudin Management through the entity 41 Madiosn L.P. as borrower signed a refi loan with lender PGIM Real Estate through the entity The Prudential Insurance Company Of America valued at $140 million for the office building (O4) at 41 Madison Avenue in Flatiron District, Manhattan. The deal closed on June 11, 2026 and was recorded on June 17, 2026. The prior lender was PGIM Real Estate which provide debt that had an original loan amount of $76 million in June 2016. The property has 524,937 square feet of built space according to a PincusCo analysis of city data. The loan price per built square foot is $266 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) The signatory for Rudin Management was Andrew Migdon . The signatory for PGIM Real Estate was Mark Kramer . Prior sales, articles and revenue The 524,937-square-foot property generated revenue of $29.4 million or $56 per square foot, according to the most recent income and expense figures.</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Vilson Lumaj pays $10M for dev site in Tremont</t>
+          <t>Related Companies signs $76.5M refi Walker &amp; Dunlop, Pretium for residential elevator in Chelsea</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>https://www.pincusco.com/vilson-lumaj-pays-10m-for-dev-site-in-tremont/</t>
+          <t>https://www.pincusco.com/related-companies-signs-76-5m-refi-with-walker-dunlop-pretium-for-residential-elevator-in-chelsea/</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Vilson Lumaj through the entity 761 East Tremont Avenue LLC paid $10 million to Shmouel</t>
+          <t>Related Companies with nonprofit partner Settlement Housing Fund through the entity French Apartments Housing Company</t>
         </is>
       </c>
       <c r="D3" t="inlineStr"/>
@@ -534,24 +534,24 @@
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>Transfers 761 East Tremont Avenue (Credit - Cyclomedia) Vilson Lumaj through the entity 761 East Tremont Avenue LLC paid $10 million to Shmouel Toledano through the entity Strong Equities, Inc. for the retail building (K1) at 761 East Tremont Avenue in Tremont, Bronx. The expected use is ground up development. The deal closed on June 12, 2026 and was recorded on June 17, 2026. The property has 15,555 square feet of built space and 54,425 square feet of additional air rights for a total buildable of 70,000 square feet according to a PincusCo analysis of city data. The sale price per built square foot is $642 and the price per buildable square foot is $142 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) The signatory for Shmouel Toledano was Shmouel Toledano. The signatory for Vilson Lumaj was Vilson Lumaj . The contract date was March 23, 2026. A Rosewood Realty Group team of Jonah Corney, Mike Kerwin and Mark Steinmetz brokered the sale. The property was being marketing as a development site, 761-769 East Tremont Avenue listing. Prior sales, articl</t>
+          <t>Transfers 324 West 30th Street (Credit - Cyclomedia) Related Companies with nonprofit partner Settlement Housing Fund through the entity French Apartments Housing Company as borrower signed a refi loan with lender Walker &amp; Dunlop and Pretium through the entity WD Impact Originator I, LLC valued at $76.5 million for the 223-unit residential elevator building (D5) at 324 West 30th Street in Chelsea, Manhattan. The deal closed on June 1, 2026, and was recorded on June 17, 2026. The prior lender was Fannie Mae which held debt that had an original loan amount of $75 million.The property has 147,888 square feet of built space according to a PincusCo analysis of city data. The loan price per built square foot is $517 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) The signatory for Related Companies and Settlement Housing Fund was Matthew Finkle and Jacqueline Tom . The signatory for Walker &amp; Dunlop and Pretium was Christopher Weidler . Prior sales, articles and revenue The owners according to the Department of Housing Preservation and Development include</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Educational Institute Oholei Torah of Brooklyn pays $16.1M for school in Crown Heights</t>
+          <t>Payam Moradof, Frank Tehrani sign $9.2M refi with Chase for 29-unit rental in Astoria</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>https://www.pincusco.com/educational-institute-oholei-torah-of-brooklyn-pays-16-1m-to-taormina-holding-for-specialty-in-crown-heights/</t>
+          <t>https://www.pincusco.com/payam-moradof-frank-tehrani-sign-9-2m-refi-with-chase-for-29-unit-rental-in-astoria/</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Educational Institute Oholei Torah of Brooklyn through the entity Ot 402 Eastern LLC paid $16.1</t>
+          <t>Payam Moradof and Frank Tehrani through the entity Asto Crest Holding LLC as borrower signed</t>
         </is>
       </c>
       <c r="D4" t="inlineStr"/>
@@ -568,24 +568,24 @@
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>Transfers 402 Eastern Parkway (Credit - Cyclomedia) Educational Institute Oholei Torah of Brooklyn through the entity Ot 402 Eastern LLC paid $16.1 million to Taormina Holding through the entity Eastern Union Properties, Inc. for the school building (W1) at 402 Eastern Parkway in Crown Heights, Brooklyn. The expected use is owner-occupied. The deal closed on June 3, 2026 and was recorded on June 17, 2026. The property has 57,840 square feet of built space according to a PincusCo analysis of city data. The sale price per built square foot is $277 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) The signatory for Taormina Holding was Joseph Taormina . The signatory for Educational Institute Oholei Torah of Brooklyn was Shmuel Brook. The contract date was February 10, 2026. New York Business Journal reported on this purchase yesterday. Prior sales, articles and revenue Prior to this transaction, PincusCo has records that the buyer Educational Institute Oholei Torah of Brooklyn purchased one property in one transaction for a total of $8.5 million and ha</t>
+          <t>Transfers 23-33 Astoria Boulevard i (Credit - Cyclomedia) Payam Moradof and Frank Tehrani through the entity Asto Crest Holding LLC as borrower signed a refi loan with lender JPMorgan Chase valued at $9.2 million for the 29-unit residential elevator building (D6) at 23-33 Astoria Boulevard in Astoria, Queens. The deal closed on May 18, 2026 and was recorded on June 17, 2026. The prior lender was Valley National Bank which held debt that had an original loan amount of $9 million.The property has 21,946 square feet of built space and 1,735 square feet of additional air rights for a total buildable of 23,670 square feet according to a PincusCo analysis of city data. The loan price per built square foot is $420 and the price per buildable square foot is $389 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) The owner bought the property on December 27, 2019, for $2.4 million. The signatory for Payam Moradof and Frank Tehrani was Payam Moradof and Frank Tehrani. The signatory for JPMorgan Chase was Ursula Flores . Prior sales, articles and revenue The 21,</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Hartz Mountain Industries pays $4.8M for dev site in SoHo</t>
+          <t>Vesper Holdings pays $3M to Cayuga Capital for 5-unit walkup in Bushwick</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>https://www.pincusco.com/hartz-mountain-industries-pays-4-8m-for-dev-site-in-soho/</t>
+          <t>https://www.pincusco.com/vesper-holdings-pays-3m-to-cayuga-capital-for-5-unit-walkup-in-bushwick/</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Hartz Mountain Industries through the entity 391 Canal Street Soho LLC paid $4.8 million to</t>
+          <t>Vesper Holdings through the entity 285 Troutman Assc. LLC paid $3 million to Cayuga Capital</t>
         </is>
       </c>
       <c r="D5" t="inlineStr"/>
@@ -602,24 +602,24 @@
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>Transfers 391 Canal Street (Credit - Cyclomedia) Hartz Mountain Industries through the entity 391 Canal Street Soho LLC paid $4.8 million to Tomer Hillel through the entity H Mazal LLC for the retail building (K1) at 391 Canal Street in SoHo, Manhattan. The expected use is ground up development. The deal closed on June 12, 2026 and was recorded on June 17, 2026. The property has 2,208 square feet of built space and 13,979 square feet of additional air rights for a total buildable of 16,180 square feet according to a PincusCo analysis of city data. The sale price per built square foot is $2,196 and the price per buildable square foot is $299 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) The seller bought the property on September 10, 2024, for $3 million. The signatory for Tomer Hillel was Tomer Hillel. The signatory for Hartz Mountain Industries was Phillip R. Patton . The contract date was May 14, 2026. Prior sales, articles and revenue Prior to this transaction, PincusCo has no record that the buyer Hartz Mountain Industries had purchased any o</t>
+          <t>Transfers 285 Troutman Street (Credit - Cyclomedia) Vesper Holdings through the entity 285 Troutman Assc. LLC paid $3 million to Cayuga Capital Management through the entity Castor Development LLC for the five-unit residential walkup building (C2) at 285 Troutman Street in Bushwick, Brooklyn. The expected use is cash flowing. The deal closed on May 20, 2026 and was recorded on June 17, 2026. The property has 3,750 square feet of built space and 2,325 square feet of additional air rights for a total buildable of 6,075 square feet according to a PincusCo analysis of city data. The sale price per built square foot is $813 and the price per buildable square foot is $502 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) The seller bought the property on March 27, 2017, for $2.3 million. The signatory for Cayuga Capital Management was Jacob Sacks . The signatory for Vesper Holdings was Elliot J. Tamir . The contract date was March 3, 2026. Prior sales, articles and revenue Prior to this transaction, PincusCo has records that the buyer Vesper Holdings purch</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Nalcorp pays $21.7M to Altmark Group for 297-unit dev site in Mott Haven</t>
+          <t>Cohen family pays $3.3M to 7-Eleven for dev site in Jamaica</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>https://www.pincusco.com/nalcorp-pays-21-7m-to-altmark-group-for-297-unit-dev-site-in-mott-haven/</t>
+          <t>https://www.pincusco.com/cohen-family-pays-3-3m-to-7-eleven-for-dev-site-in-jamaica/</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Nalcorp through the entity 122 Blvd 134 St LLC paid $21.7 million to Altmark Group</t>
+          <t>The Cohen family behind Daniel Group and Leviathan Capital through the entity 148 Lib LLC</t>
         </is>
       </c>
       <c r="D6" t="inlineStr"/>
@@ -636,24 +636,24 @@
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>Top Story Transfers 122 Bruckner Boulevard, 20 Brook Avenue, 521 East 132nd Street (Credit - Google Earth) Nalcorp through the entity 122 Blvd 134 St LLC paid $21.7 million to Altmark Group through the entity 122 Bruckner Development LLC for three adjacent tax lots in Mott Haven, the Bronx, where the buyer has filed plans for a total of 297 units in three projects. The parcels are the industrial building (G9) at 517 East 132nd Street, the industrial building (F5) at 519 East 132nd Street, and the specialty building (Z9) at 122 Bruckner Boulevard. The expected use is ground up development. The deal closed on June 12, 2026 and was recorded on June 17, 2026. The three properties have 19,866 square feet of built space and 152,917 square feet of additional air rights for a total buildable of 172,774 square feet according to a PincusCo analysis of city data. The sale price per built square foot is $1,092 and the price per buildable square foot is $125 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) The signatory for Altmark Group was Adi Altmark . The si</t>
+          <t>Transfers 148-27 Liberty Avenue (Credit - Cyclomedia) The Cohen family behind Daniel Group and Leviathan Capital through the entity 148 Lib LLC paid $3.3 million to 7-Eleven through the entity Speedway LLC for the vacant development site at 148-27 Liberty Avenue in Jamaica, Queens. The expected use if ground up development. The deal closed on May 29, 2026 and was recorded on June 17, 2026. The property has 289 square feet of built space and 84,000 square feet of additional air rights for a total buildable of 84,280 square feet according to a PincusCo analysis of city data. The sale price per built square foot is $11,418 and the price per buildable square foot is $39 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) The signatory for 7-Eleven was David J. Colletti Jr. . The signatory for Daniel Group was Edward J. Bullard Jr. . The contract date was October 20, 2025. Prior sales, articles and revenue Prior to this transaction, PincusCo has records that the buyer Daniel Group purchased four properties in four transactions for a total of $14.8 million a</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Palwinder Singh signs $10M construction loan for 32-unit project in LIC</t>
+          <t>David Werner, 601W Companies’ $265.2M purchase of Rockpoint office in Midtown East gets recorded</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>https://www.pincusco.com/palwinder-singh-signs-10m-construction-loan-for-32-unit-project-in-lic/</t>
+          <t>https://www.pincusco.com/david-werner-601w-companiess-265-2m-purchase-of-rockpoint-office-in-midtown-east-gets-recorded/</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Palwinder Singh through the entity 31st Street LIC Property LLC as borrower signed a new</t>
+          <t>David Werner Real Estate Investments and 601W Companies through the entity One Dag Owner Lp</t>
         </is>
       </c>
       <c r="D7" t="inlineStr"/>
@@ -670,24 +670,24 @@
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t xml:space="preserve">Transfers 36-32 31st Street axonometric diagram (Credit - Gerald Caliendo architect via DOB) Palwinder Singh through the entity 31st Street LIC Property LLC as borrower signed a new construction loan with lender Ponce Bank valued at $10 million for the 32-unit development project at 36-31 31st Street in Long Island City, Queens. On the lot, there is one active new building construction project, Q01136795, for a 32-unit, 22,381 square-foot residential (R-2) building. The project was submitted by Palwinder Singh and filed by Palwinder Singh with plans filed November 5, 2024 and it has not been permitted yet. The deal closed on June 8, 2026 and was recorded on June 15, 2026. The property has zero square feet of built space and 17,214 square feet of additional air rights for a total buildable of 17,214 square feet according to a PincusCo analysis of city data. The loan price per planned development zoning square foot is $447 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) The owner bought the property on August 8, 2024, for $3.4 million. The signatory </t>
+          <t>Transfers 885 2nd Avenue (Credit - Cyclomedia) David Werner Real Estate Investments and 601W Companies through the entity One Dag Owner Lp paid $265.2 million to Rockpoint Group through the entity 885 Second Avenue Owner LLC for the office building (O4) at 885 2nd Avenue in Midtown East, Manhattan. The expected use is cash flowing. The deal closed on June 5, 2026 and was recorded on June 18, 2026. The property has 805,467 square feet of built space according to a PincusCo analysis of city data. The sale price per built square foot is $329 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) The seller bought the property in January 2019, for $565.75 million. The signatory for Rockpoint Group was Joseph A. Goldman . The signatory for David Werner Real Estate Investments and 601W Companies was David Werner . The contract date was November 26, 2025. Simultaneously with the purchase, David Werner terminated the 49-year ground lease Rockpoint had created just after buying the property in 2019. At that time, the Rockpoint buyer entity executed the 49-year gro</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Joel Schwartz signs $28.5M construction loan with S3 for 60-unit dev site in Bushwick</t>
+          <t>Realterm pays $10.3M for industrial in Hunts Point</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>https://www.pincusco.com/joel-schwartz-signs-28-5m-construction-loan-with-s3-for-60-unit-dev-site-in-bushwick/</t>
+          <t>https://www.pincusco.com/realterm-pays-10-3m-for-industrial-in-hunts-point/</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Joel Schwartz through the entity Grove Menahan BK LLC as borrower signed a new construction</t>
+          <t>Logistics firm Realterm through the entity RLF V East, LLC paid $10.3 million through the</t>
         </is>
       </c>
       <c r="D8" t="inlineStr"/>
@@ -704,7 +704,7 @@
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t xml:space="preserve">Transfers 111 Grove Street rendering (Credit - Diego Aguilera Architects via DOB) Joel Schwartz through the entity Grove Menahan BK LLC as borrower signed a new construction loan with lender S3 Capital through the entity S3 Re Menahan Grove Funding LLC valued at $28.5 million for the two-parcel development site at 111 Grove Street in Bushwick, Brooklyn. The loan closed on June 1, 2026 and was recorded on June 16, 2026. The loan price per planned zoning square foot is $659 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) The signatory for Joel Schwartz was Joel Schwartz. Joel Schwartz through the entity Grove Menahan BK LLC bought the site for $6 million from Moshe Granit through the entity 115-117 Grove St LLC on June 1, 2026. There is a new building project, B01391270, for a 60-unit, 43,227 square-foot residential (R-2) building submitted by Jerome Zwick and filed by Jerome Zwick with plans filed May 6, 2026 and it has not been permitted yet. The six-story building project has 10 residential units on each floor from one to six. There are no retail </t>
+          <t>Transfers 891 Garrison Avenue (Credit - Cyclomedia) Logistics firm Realterm through the entity RLF V East, LLC paid $10.3 million through the entity CJC Garrison 935 LLC for the industrial building (G1) at 891 Garrison Avenue in Hunts Point, Bronx. The deal closed on May 8, 2026 and was recorded on June 18, 2026. The property has 9,200 square feet of built space and 70,938 square feet of additional air rights for a total buildable of 80,156 square feet according to a PincusCo analysis of city data. The sale price per built square foot is $1,116 and the price per buildable square foot is $128 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) The seller bought the property on May 4, 2015, for $226,456. The signatory for Barry Haskell , Shelley Won, and Kimberli Silverstein was Barry Haskell . The signatory for Realterm was Edward Brickley . The contract date was December 23, 2025. Prior sales, articles and revenue Prior to this transaction, PincusCo has no record that the buyer Realterm had purchased any other properties and has no record it sold any p</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto update queens news 2026-06-20T14:27:54Z
</commit_message>
<xml_diff>
--- a/data/output/queens_dev_news.xlsx
+++ b/data/output/queens_dev_news.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H8"/>
+  <dimension ref="A1:H2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -473,238 +473,42 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Rudin ups debt from $76M to $140M with PGIM for office in Flatiron District</t>
+          <t>Luma’s Façade Progresses at 10-39 49th Avenue in Long Island City, Queens</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>https://www.pincusco.com/rudin-ups-debt-from-76m-to-140m-with-pgim-for-office-in-flatiron-district/</t>
+          <t>https://newyorkyimby.com/2026/06/lumas-facade-progresses-at-10-39-49th-avenue-in-long-island-city-queens.html</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Rudin Management through the entity 41 Madiosn L.P. as borrower signed a refi loan with</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr"/>
-      <c r="E2" t="inlineStr"/>
+          <t>Exterior work is progressing on Luma, a six-story residential building at 10-39 49th Avenue in &lt;a href="https://newyorkyimby.com/neighborhoods/long-island-city"&gt;Long Island City&lt;/a&gt;, Queens. Designed by Angelo Ng &amp;#38; Anthony Ng Architects Studio and developed by Yong Chen, the 65-foot-tall structure will yield 35 condominium units with an average scope of 685 square feet. The project will also include 13 open parking spaces and six enclosed parking spaces, according to permits filed last December. The property is located between Jackson Avenue and Vernon Boulevard.</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>2026-06-20T12:00:21+00:00</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>Sat, 20 Jun 2026 12:00:21 +0000</t>
+        </is>
+      </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>PincusCo</t>
+          <t>YIMBY</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>PincusCo - Home</t>
+          <t>YIMBY - Long Island City</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>Transfers 41 Madison Avenue (Credit - Cyclomedia) Rudin Management through the entity 41 Madiosn L.P. as borrower signed a refi loan with lender PGIM Real Estate through the entity The Prudential Insurance Company Of America valued at $140 million for the office building (O4) at 41 Madison Avenue in Flatiron District, Manhattan. The deal closed on June 11, 2026 and was recorded on June 17, 2026. The prior lender was PGIM Real Estate which provide debt that had an original loan amount of $76 million in June 2016. The property has 524,937 square feet of built space according to a PincusCo analysis of city data. The loan price per built square foot is $266 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) The signatory for Rudin Management was Andrew Migdon . The signatory for PGIM Real Estate was Mark Kramer . Prior sales, articles and revenue The 524,937-square-foot property generated revenue of $29.4 million or $56 per square foot, according to the most recent income and expense figures.</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>Related Companies signs $76.5M refi Walker &amp; Dunlop, Pretium for residential elevator in Chelsea</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>https://www.pincusco.com/related-companies-signs-76-5m-refi-with-walker-dunlop-pretium-for-residential-elevator-in-chelsea/</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>Related Companies with nonprofit partner Settlement Housing Fund through the entity French Apartments Housing Company</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr"/>
-      <c r="E3" t="inlineStr"/>
-      <c r="F3" t="inlineStr">
-        <is>
-          <t>PincusCo</t>
-        </is>
-      </c>
-      <c r="G3" t="inlineStr">
-        <is>
-          <t>PincusCo - Home</t>
-        </is>
-      </c>
-      <c r="H3" t="inlineStr">
-        <is>
-          <t>Transfers 324 West 30th Street (Credit - Cyclomedia) Related Companies with nonprofit partner Settlement Housing Fund through the entity French Apartments Housing Company as borrower signed a refi loan with lender Walker &amp; Dunlop and Pretium through the entity WD Impact Originator I, LLC valued at $76.5 million for the 223-unit residential elevator building (D5) at 324 West 30th Street in Chelsea, Manhattan. The deal closed on June 1, 2026, and was recorded on June 17, 2026. The prior lender was Fannie Mae which held debt that had an original loan amount of $75 million.The property has 147,888 square feet of built space according to a PincusCo analysis of city data. The loan price per built square foot is $517 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) The signatory for Related Companies and Settlement Housing Fund was Matthew Finkle and Jacqueline Tom . The signatory for Walker &amp; Dunlop and Pretium was Christopher Weidler . Prior sales, articles and revenue The owners according to the Department of Housing Preservation and Development include</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>Payam Moradof, Frank Tehrani sign $9.2M refi with Chase for 29-unit rental in Astoria</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>https://www.pincusco.com/payam-moradof-frank-tehrani-sign-9-2m-refi-with-chase-for-29-unit-rental-in-astoria/</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>Payam Moradof and Frank Tehrani through the entity Asto Crest Holding LLC as borrower signed</t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr"/>
-      <c r="E4" t="inlineStr"/>
-      <c r="F4" t="inlineStr">
-        <is>
-          <t>PincusCo</t>
-        </is>
-      </c>
-      <c r="G4" t="inlineStr">
-        <is>
-          <t>PincusCo - Home</t>
-        </is>
-      </c>
-      <c r="H4" t="inlineStr">
-        <is>
-          <t>Transfers 23-33 Astoria Boulevard i (Credit - Cyclomedia) Payam Moradof and Frank Tehrani through the entity Asto Crest Holding LLC as borrower signed a refi loan with lender JPMorgan Chase valued at $9.2 million for the 29-unit residential elevator building (D6) at 23-33 Astoria Boulevard in Astoria, Queens. The deal closed on May 18, 2026 and was recorded on June 17, 2026. The prior lender was Valley National Bank which held debt that had an original loan amount of $9 million.The property has 21,946 square feet of built space and 1,735 square feet of additional air rights for a total buildable of 23,670 square feet according to a PincusCo analysis of city data. The loan price per built square foot is $420 and the price per buildable square foot is $389 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) The owner bought the property on December 27, 2019, for $2.4 million. The signatory for Payam Moradof and Frank Tehrani was Payam Moradof and Frank Tehrani. The signatory for JPMorgan Chase was Ursula Flores . Prior sales, articles and revenue The 21,</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>Vesper Holdings pays $3M to Cayuga Capital for 5-unit walkup in Bushwick</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>https://www.pincusco.com/vesper-holdings-pays-3m-to-cayuga-capital-for-5-unit-walkup-in-bushwick/</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>Vesper Holdings through the entity 285 Troutman Assc. LLC paid $3 million to Cayuga Capital</t>
-        </is>
-      </c>
-      <c r="D5" t="inlineStr"/>
-      <c r="E5" t="inlineStr"/>
-      <c r="F5" t="inlineStr">
-        <is>
-          <t>PincusCo</t>
-        </is>
-      </c>
-      <c r="G5" t="inlineStr">
-        <is>
-          <t>PincusCo - Home</t>
-        </is>
-      </c>
-      <c r="H5" t="inlineStr">
-        <is>
-          <t>Transfers 285 Troutman Street (Credit - Cyclomedia) Vesper Holdings through the entity 285 Troutman Assc. LLC paid $3 million to Cayuga Capital Management through the entity Castor Development LLC for the five-unit residential walkup building (C2) at 285 Troutman Street in Bushwick, Brooklyn. The expected use is cash flowing. The deal closed on May 20, 2026 and was recorded on June 17, 2026. The property has 3,750 square feet of built space and 2,325 square feet of additional air rights for a total buildable of 6,075 square feet according to a PincusCo analysis of city data. The sale price per built square foot is $813 and the price per buildable square foot is $502 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) The seller bought the property on March 27, 2017, for $2.3 million. The signatory for Cayuga Capital Management was Jacob Sacks . The signatory for Vesper Holdings was Elliot J. Tamir . The contract date was March 3, 2026. Prior sales, articles and revenue Prior to this transaction, PincusCo has records that the buyer Vesper Holdings purch</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>Cohen family pays $3.3M to 7-Eleven for dev site in Jamaica</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>https://www.pincusco.com/cohen-family-pays-3-3m-to-7-eleven-for-dev-site-in-jamaica/</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>The Cohen family behind Daniel Group and Leviathan Capital through the entity 148 Lib LLC</t>
-        </is>
-      </c>
-      <c r="D6" t="inlineStr"/>
-      <c r="E6" t="inlineStr"/>
-      <c r="F6" t="inlineStr">
-        <is>
-          <t>PincusCo</t>
-        </is>
-      </c>
-      <c r="G6" t="inlineStr">
-        <is>
-          <t>PincusCo - Home</t>
-        </is>
-      </c>
-      <c r="H6" t="inlineStr">
-        <is>
-          <t>Transfers 148-27 Liberty Avenue (Credit - Cyclomedia) The Cohen family behind Daniel Group and Leviathan Capital through the entity 148 Lib LLC paid $3.3 million to 7-Eleven through the entity Speedway LLC for the vacant development site at 148-27 Liberty Avenue in Jamaica, Queens. The expected use if ground up development. The deal closed on May 29, 2026 and was recorded on June 17, 2026. The property has 289 square feet of built space and 84,000 square feet of additional air rights for a total buildable of 84,280 square feet according to a PincusCo analysis of city data. The sale price per built square foot is $11,418 and the price per buildable square foot is $39 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) The signatory for 7-Eleven was David J. Colletti Jr. . The signatory for Daniel Group was Edward J. Bullard Jr. . The contract date was October 20, 2025. Prior sales, articles and revenue Prior to this transaction, PincusCo has records that the buyer Daniel Group purchased four properties in four transactions for a total of $14.8 million a</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>David Werner, 601W Companies’ $265.2M purchase of Rockpoint office in Midtown East gets recorded</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>https://www.pincusco.com/david-werner-601w-companiess-265-2m-purchase-of-rockpoint-office-in-midtown-east-gets-recorded/</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>David Werner Real Estate Investments and 601W Companies through the entity One Dag Owner Lp</t>
-        </is>
-      </c>
-      <c r="D7" t="inlineStr"/>
-      <c r="E7" t="inlineStr"/>
-      <c r="F7" t="inlineStr">
-        <is>
-          <t>PincusCo</t>
-        </is>
-      </c>
-      <c r="G7" t="inlineStr">
-        <is>
-          <t>PincusCo - Home</t>
-        </is>
-      </c>
-      <c r="H7" t="inlineStr">
-        <is>
-          <t>Transfers 885 2nd Avenue (Credit - Cyclomedia) David Werner Real Estate Investments and 601W Companies through the entity One Dag Owner Lp paid $265.2 million to Rockpoint Group through the entity 885 Second Avenue Owner LLC for the office building (O4) at 885 2nd Avenue in Midtown East, Manhattan. The expected use is cash flowing. The deal closed on June 5, 2026 and was recorded on June 18, 2026. The property has 805,467 square feet of built space according to a PincusCo analysis of city data. The sale price per built square foot is $329 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) The seller bought the property in January 2019, for $565.75 million. The signatory for Rockpoint Group was Joseph A. Goldman . The signatory for David Werner Real Estate Investments and 601W Companies was David Werner . The contract date was November 26, 2025. Simultaneously with the purchase, David Werner terminated the 49-year ground lease Rockpoint had created just after buying the property in 2019. At that time, the Rockpoint buyer entity executed the 49-year gro</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>Realterm pays $10.3M for industrial in Hunts Point</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>https://www.pincusco.com/realterm-pays-10-3m-for-industrial-in-hunts-point/</t>
-        </is>
-      </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>Logistics firm Realterm through the entity RLF V East, LLC paid $10.3 million through the</t>
-        </is>
-      </c>
-      <c r="D8" t="inlineStr"/>
-      <c r="E8" t="inlineStr"/>
-      <c r="F8" t="inlineStr">
-        <is>
-          <t>PincusCo</t>
-        </is>
-      </c>
-      <c r="G8" t="inlineStr">
-        <is>
-          <t>PincusCo - Home</t>
-        </is>
-      </c>
-      <c r="H8" t="inlineStr">
-        <is>
-          <t>Transfers 891 Garrison Avenue (Credit - Cyclomedia) Logistics firm Realterm through the entity RLF V East, LLC paid $10.3 million through the entity CJC Garrison 935 LLC for the industrial building (G1) at 891 Garrison Avenue in Hunts Point, Bronx. The deal closed on May 8, 2026 and was recorded on June 18, 2026. The property has 9,200 square feet of built space and 70,938 square feet of additional air rights for a total buildable of 80,156 square feet according to a PincusCo analysis of city data. The sale price per built square foot is $1,116 and the price per buildable square foot is $128 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) The seller bought the property on May 4, 2015, for $226,456. The signatory for Barry Haskell , Shelley Won, and Kimberli Silverstein was Barry Haskell . The signatory for Realterm was Edward Brickley . The contract date was December 23, 2025. Prior sales, articles and revenue Prior to this transaction, PincusCo has no record that the buyer Realterm had purchased any other properties and has no record it sold any p</t>
+          <t>By: Michael Young and Matt Pruznick 8:00 am on June 20, 2026 Exterior work is progressing on Luma, a six-story residential building at 10-39 49th Avenue in Long Island City, Queens. Designed by Angelo Ng &amp; Anthony Ng Architects Studio and developed by Yong Chen, the 65-foot-tall structure will yield 35 condominium units with an average scope of 685 square feet. The project will also include 13 open parking spaces and six enclosed parking spaces, according to permits filed last December. The property is located between Jackson Avenue and Vernon Boulevard. The reinforced concrete superstructure stands topped out with its main southern elevation largely enclosed in a glass curtain wall. The massing incorporates several setbacks on the fifth and sixth floors, and the building features multiple balconies and a loggia terrace at the southwest corner of the fifth story. Scaffolding and netting cover the windowless western lot line wall as crews work to finish the side profiles. 10-39 49th Avenue. Photo by Michael Young. 10-39 49th Avenue. Photo by Michael Young. 10-39 49th Avenue. Photo by Michael Young.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto update queens news 2026-06-21T14:30:52Z
</commit_message>
<xml_diff>
--- a/data/output/queens_dev_news.xlsx
+++ b/data/output/queens_dev_news.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H2"/>
+  <dimension ref="A1:H1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -467,48 +467,6 @@
       <c r="H1" s="1" t="inlineStr">
         <is>
           <t>content_preview</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>Luma’s Façade Progresses at 10-39 49th Avenue in Long Island City, Queens</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>https://newyorkyimby.com/2026/06/lumas-facade-progresses-at-10-39-49th-avenue-in-long-island-city-queens.html</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>Exterior work is progressing on Luma, a six-story residential building at 10-39 49th Avenue in &lt;a href="https://newyorkyimby.com/neighborhoods/long-island-city"&gt;Long Island City&lt;/a&gt;, Queens. Designed by Angelo Ng &amp;#38; Anthony Ng Architects Studio and developed by Yong Chen, the 65-foot-tall structure will yield 35 condominium units with an average scope of 685 square feet. The project will also include 13 open parking spaces and six enclosed parking spaces, according to permits filed last December. The property is located between Jackson Avenue and Vernon Boulevard.</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>2026-06-20T12:00:21+00:00</t>
-        </is>
-      </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>Sat, 20 Jun 2026 12:00:21 +0000</t>
-        </is>
-      </c>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t>YIMBY</t>
-        </is>
-      </c>
-      <c r="G2" t="inlineStr">
-        <is>
-          <t>YIMBY - Long Island City</t>
-        </is>
-      </c>
-      <c r="H2" t="inlineStr">
-        <is>
-          <t>By: Michael Young and Matt Pruznick 8:00 am on June 20, 2026 Exterior work is progressing on Luma, a six-story residential building at 10-39 49th Avenue in Long Island City, Queens. Designed by Angelo Ng &amp; Anthony Ng Architects Studio and developed by Yong Chen, the 65-foot-tall structure will yield 35 condominium units with an average scope of 685 square feet. The project will also include 13 open parking spaces and six enclosed parking spaces, according to permits filed last December. The property is located between Jackson Avenue and Vernon Boulevard. The reinforced concrete superstructure stands topped out with its main southern elevation largely enclosed in a glass curtain wall. The massing incorporates several setbacks on the fifth and sixth floors, and the building features multiple balconies and a loggia terrace at the southwest corner of the fifth story. Scaffolding and netting cover the windowless western lot line wall as crews work to finish the side profiles. 10-39 49th Avenue. Photo by Michael Young. 10-39 49th Avenue. Photo by Michael Young. 10-39 49th Avenue. Photo by Michael Young.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto update queens news 2026-06-22T17:12:04Z
</commit_message>
<xml_diff>
--- a/data/output/queens_dev_news.xlsx
+++ b/data/output/queens_dev_news.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H1"/>
+  <dimension ref="A1:H9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -470,6 +470,278 @@
         </is>
       </c>
     </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Grun Group files two plans totaling 108 units in Kew Gardens</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>https://www.pincusco.com/grun-group-files-two-plans-totaling-108-units-in-kew-gardens/</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>The Grun Group filed two new development plans with the city’s Department of Buildings last</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr"/>
+      <c r="E2" t="inlineStr"/>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>PincusCo</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>PincusCo - Home</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>Development Grosvenor Lane (Credit - Naresh K. Mahangu professional engineer via DOB) The Grun Group filed two new development plans with the city’s Department of Buildings last week totaling 108 units in Kew Gardens, Queens. In the larger, Grun Group submitted a new building construction project for a 58-unit, 34,684-square-foot residential (R-2) building at 116-18 Grosvenor Lane in Kew Gardens, Queens. The plan was filed on June 16, 2026. It calls for the construction of a 85-foot-tall, nine-story building and was filed with the New York City Department of Buildings under job number Q01415856. The project is described in the filing as: 9 story residential building. The applicant is the Professional Engineer Naresh Mahangu of NKM Engineering Pllc. Yonah Grunhut of Grun Group submitted the plans. 116-18 Grosvenor Lane In the smaller, Grun Group submitted a new building construction project for a 50-unit, 32,258-square-foot residential (R-2) building at 116-14 Grosvenor Lane in Kew Gardens, Queens. The plan was filed on June 16, 2026. It calls for the construction of a 85-foot-tall, nine-story building and was filed with the New York City Department of Buildings under job number Q01</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>MRR Development signs $200M refi with Bank Hapoalim for two properties in Midtown East</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>https://www.pincusco.com/mrr-development-signs-200m-refi-with-bank-hapoalim-for-two-properties-in-midtown-east/</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>MRR Development through the entity Mrr 1326 LLC as borrower signed a refi loan with</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr"/>
+      <c r="E3" t="inlineStr"/>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>PincusCo</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>PincusCo - Home</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>Transfers 126 east 57th Street (Credit - Cyclomedia) MRR Development through the entity Mrr 1326 LLC as borrower signed a refi loan with lender Bank Hapoalim through the entity Bank Hapoalim B.M. valued at $200 million for the 145-unit residential elevator building (D6) at 126 East 57th Street in Midtown East, Manhattan, and a small office building that is adjacent, at 127 East 56th Street. The deal closed on June 2, 2026 and was recorded on June 18, 2026. The prior lender was Bank OZK which held debt that had an original loan amount of $170 million. The two properties have 205,102 square feet of built space and 9,517 square feet of additional air rights according to a PincusCo analysis of city data. The loan price per built square foot is $975 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) The signatory for MRR Development was Rotem Rosen . This is a $200 million loan composed of $30 million in additional construction debt, mostly a project mortgage, on top of existing $170 million construction loan originated by Bank OZK. Prior sales, articles a</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Or Trabelsi signs $6M acquisition loan with S3 Capital for 22-unit walkup in Garment District</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>https://www.pincusco.com/or-trabelsi-signs-6m-acquisition-loan-with-s3-capital-for-22-unit-walkup-in-garment-district/</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Or Trabelsi through the entity 510 AIC LLC as borrower signed an acquisition loan with</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr"/>
+      <c r="E4" t="inlineStr"/>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>PincusCo</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>PincusCo - Home</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>Transfers 510 Ninth Avenue (Credit - Cyclomedia) Or Trabelsi through the entity 510 AIC LLC as borrower signed an acquisition loan with lender S3 Capital through the entity S3 RE Perpetual Yield Funding LLC valued at $6 million for the 22-unit residential walkup building (C7) at 510 Ninth Avenue in the Garment District, Manhattan. The deal closed on February 23, 2026 and was recorded on June 18, 2026. The property has 11,341 square feet of built space and 3,503 square feet of additional air rights for a total buildable of 14,851 square feet according to a PincusCo analysis of city data. The loan price per built square foot is $529 and the price per buildable square foot is $404 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) The owner bought the property on February 23, 2026, for $5.5 million. The signatory for Or Trabelsi was Michael Raymond Mintz and Or Trabelsi. Prior sales, articles and revenue The owners according to the Department of Housing Preservation and Development includes Yuval Plattner, head officer and Michael Mintz , officer. The bu</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Green Street Group pays $2.9M for office in Tribeca</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>https://www.pincusco.com/green-street-group-pays-2-9m-for-office-in-tribeca/</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Green Street Group through the entity 141 West Broadway LLC paid $2.9 million through an</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr"/>
+      <c r="E5" t="inlineStr"/>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>PincusCo</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>PincusCo - Home</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>Transfers 141 West Broadway (Credit - Cyclomedia) Green Street Group through the entity 141 West Broadway LLC paid $2.9 million through an estate sale to the Pantzer family through the entity Three Reddy LLC for the office building (O2) at 141 West Broadway in Tribeca, Manhattan. The expected use is cash flowing. The deal closed on June 15, 2026 and was recorded on June 18, 2026. The property has 2,500 square feet of built space and 2,515 square feet of additional air rights for a total buildable of 5,014 square feet according to a PincusCo analysis of city data. The sale price per built square foot is $1,160 and the price per buildable square foot is $578 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) The signatory for the family of the late restaurateur Joan Pantzer was Dennis W. Pantzer . The signatory for Green Street Group was Joshua Greenberg . The contract date was March 12, 2025. Joan Pantzer died in 2024. She started the restaurant that became the Odeon, located next door at 145 West Broadway. Prior sales, articles and revenue Prior to th</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Bastone family signs $5.8M loan with Galinn Fund for The Pine restaurant in Bronx</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>https://www.pincusco.com/bastone-family-signs-5-8m-loan-with-galinn-fund-for-the-pine-restaurant-in-bronx/</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>The Bastone family through the entity 1911-1913 Bronxdale Avenue Realty LLC as borrower signed a</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr"/>
+      <c r="E6" t="inlineStr"/>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>PincusCo</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>PincusCo - Home</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>Transfers 1913 Bronxdale Avenue (Credit - Cyclomedia) The Bastone family through the entity 1911-1913 Bronxdale Avenue Realty LLC as borrower signed a loan with lender Galinn Fund through the entity The Galinn Fund LLC valued at $5.8 million for five tax lots that form the location of the The Pine restaurant and banquet hall, including the retail building (K1) at 1907 Bronxdale Avenue in Van Nest, Bronx, mixed-use building (K4) at 1913 Bronxdale Avenue in Van Nest, Bronx, and parking (G7) at 1903 Bronxdale Avenue in Van Nest, Bronx. The main address for the restaurant is 1913 Bronxdale Avenue. The deal closed on June 10, 2026 and was recorded on June 18, 2026. A prior lender, Noble Capital Management, provided debt that had an original loan amount of $3 million. The five properties have 15,996 square feet of built space and 16,525 square feet of additional air rights for a total buildable of 32,487 square feet according to a PincusCo analysis of city data. The loan price per built square foot is $362 and the price per buildable square foot is $178 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public rec</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Jun Kil, Suk Chang pay $3M for retail in Queens Village</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>https://www.pincusco.com/jun-kil-suk-chang-pay-3m-for-retail-in-queens-village/</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Jun Bum Kil and Suk Nyo Chang through the entity 216 Hillside LLC paid $3</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr"/>
+      <c r="E7" t="inlineStr"/>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>PincusCo</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>PincusCo - Home</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>Transfers 216-20 Hillside Avenue (Credit - Cyclomedia) Jun Bum Kil and Suk Nyo Chang through the entity 216 Hillside LLC paid $3 million to the Zirinsky family through the entity Hillside Metro Associates LLC for the retail building (K1) at 216-20 Hillside Avenue in Queens Village, Queens. The expected use is owner-occupied, for the grocery store John’s Farm Market. The deal closed on June 5, 2026 and was recorded on June 18, 2026. The property has 4,500 square feet of built space and 4,440 square feet of additional air rights for a total buildable of 9,000 square feet according to a PincusCo analysis of city data. The sale price per built square foot is $666 and the price per buildable square foot is $333 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) The signatory for Cynthia Zirinsky was Jerome L. Levine, Cynthia Eckes , Susan Zirinsky, John Zirinsky , and William Zirinsky. The signatory for Jun Bum Kil and Suk Nyo Chang was Jun B. Kil . The contract date was May 14, 2026. The sellers are the descendants of the married couple Richard William Zi</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Heskel’s Asset Management signs $8.6M refi with FourLeaf for 62-unit rental in Washington Heights</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>https://www.pincusco.com/heskels-asset-management-signs-8-6m-refi-with-fourleaf-for-62-unit-rental-in-washington-heights/</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Heskel’s Asset Management through the entity Heskel’s FW Realty LLC as borrower signed a refi</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr"/>
+      <c r="E8" t="inlineStr"/>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>PincusCo</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>PincusCo - Home</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>Transfers 567 Ft. Washington Avenue (Credit - Cyclomedia) Heskel’s Asset Management through the entity Heskel’s FW Realty LLC as borrower signed a refi loan with lender FourLeaf Federal Credit Union through the entity Fourleaf Federal Credit Union valued at $8.6 million for the 62-unit residential elevator building (D1) at 567 Ft Washington Avenue in Washington Heights, Manhattan. The deal closed on June 12, 2026 and was recorded on June 18, 2026. The prior lender was Webster Bank which held debt that had an original loan amount of $9.9 million.The property has 59,976 square feet of built space according to a PincusCo analysis of city data. The loan price per built square foot is $143 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) The signatory for Heskel’s Asset Management was Ramin Sarraf . The signatory for FourLeaf Federal Credit Union was Julian Cokro . Prior sales, articles and revenue The owners according to the Department of Housing Preservation and Development includes Ramin Sarraf, head officer and Elvis Debernardo, site manager. The bus</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>P. Zaccaro signs $32.8M refi with Derby Copeland for properties in Nolita, Chinatown, SoHo</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>https://www.pincusco.com/p-zaccaro-signs-32-8m-refi-with-derby-copeland-for-properties-in-nolita-chinatown-soho/</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>P. Zaccaro through the entity 1-3 Mott And 218 Lafayette Street Partners, LLC as borrower</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr"/>
+      <c r="E9" t="inlineStr"/>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>PincusCo</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>PincusCo - Home</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>Transfers 218 Lafayette Street (Credit - Cyclomedia) P. Zaccaro through the entity 1-3 Mott And 218 Lafayette Street Partners, LLC as borrower signed a refi loan with lender Derby Copeland Capital through the entity DCC Remmcf Seller Atlas, LLC valued at $32.8 million for three properties in Manhattan with 27 residential units including the 24-unit residential walkup building (C7) at 241 Mulberry Street in Nolita, the three-unit mixed-use building (K4) at 1-3 Mott Street in Chinatown, and mixed-use building (K2) at 218 Lafayette Street in SoHo. The deal closed on May 11, 2026 and was recorded on June 18, 2026. The prior lender was Oceanview Life and Annuity Company. The three properties have 26,026 square feet of built space and 10,145 square feet of additional air rights for a total buildable of 35,266 square feet according to a PincusCo analysis of city data. The loan price per built square foot is $1,258 and the price per buildable square foot is $928 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) The signatory for P. Zaccaro was John A. Zaccar</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
auto update queens news 2026-06-23T15:22:50Z
</commit_message>
<xml_diff>
--- a/data/output/queens_dev_news.xlsx
+++ b/data/output/queens_dev_news.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H9"/>
+  <dimension ref="A1:H10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -473,17 +473,17 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Grun Group files two plans totaling 108 units in Kew Gardens</t>
+          <t>Derek Fraser files plans for 26 units in Ditmars Steinway</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>https://www.pincusco.com/grun-group-files-two-plans-totaling-108-units-in-kew-gardens/</t>
+          <t>https://www.pincusco.com/derek-fraser-files-plans-for-26-units-in-ditmars-steinway/</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>The Grun Group filed two new development plans with the city’s Department of Buildings last</t>
+          <t>Derek Fraser submitted a new building construction project for a 26-unit, 17,416-square-foot residential (R-2) building</t>
         </is>
       </c>
       <c r="D2" t="inlineStr"/>
@@ -500,24 +500,24 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>Development Grosvenor Lane (Credit - Naresh K. Mahangu professional engineer via DOB) The Grun Group filed two new development plans with the city’s Department of Buildings last week totaling 108 units in Kew Gardens, Queens. In the larger, Grun Group submitted a new building construction project for a 58-unit, 34,684-square-foot residential (R-2) building at 116-18 Grosvenor Lane in Kew Gardens, Queens. The plan was filed on June 16, 2026. It calls for the construction of a 85-foot-tall, nine-story building and was filed with the New York City Department of Buildings under job number Q01415856. The project is described in the filing as: 9 story residential building. The applicant is the Professional Engineer Naresh Mahangu of NKM Engineering Pllc. Yonah Grunhut of Grun Group submitted the plans. 116-18 Grosvenor Lane In the smaller, Grun Group submitted a new building construction project for a 50-unit, 32,258-square-foot residential (R-2) building at 116-14 Grosvenor Lane in Kew Gardens, Queens. The plan was filed on June 16, 2026. It calls for the construction of a 85-foot-tall, nine-story building and was filed with the New York City Department of Buildings under job number Q01</t>
+          <t>Development 23-01 31st Street axonometric diagram (Credit - Harriet Nikakis architect via DOB) Derek Fraser submitted a new building construction project for a 26-unit, 17,416-square-foot residential (R-2) building at 23-01 31st Street in Ditmars Steinway, Queens. The plan was filed on June 18, 2026. It calls for the construction of a 84-foot-tall, eight-story building and was filed with the New York City Department of Buildings under job number Q01257109. The project is described in the filing as: new 8-story building 26 units, with commercial and community facility.. The applicant is the Registered Architect Harriet Nikakis of Hcn Design. Derek Fraser of Derek Fraser submitted the plans. The most recent property records show Pericles Notias purchased this parcel for $4.2 million in February 2024. 23-01 31st Street The neighborhood</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>MRR Development signs $200M refi with Bank Hapoalim for two properties in Midtown East</t>
+          <t>Slate Property Group signs $86.2M refi with Ares for 186-unit rental in LIC</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>https://www.pincusco.com/mrr-development-signs-200m-refi-with-bank-hapoalim-for-two-properties-in-midtown-east/</t>
+          <t>https://www.pincusco.com/slate-property-group-signs-86-2m-refi-with-ares-for-186-unit-rental-in-lic/</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>MRR Development through the entity Mrr 1326 LLC as borrower signed a refi loan with</t>
+          <t>Slate Property Group through the entity 37-11 30th Street Holdings LLC as borrower signed a</t>
         </is>
       </c>
       <c r="D3" t="inlineStr"/>
@@ -534,24 +534,24 @@
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>Transfers 126 east 57th Street (Credit - Cyclomedia) MRR Development through the entity Mrr 1326 LLC as borrower signed a refi loan with lender Bank Hapoalim through the entity Bank Hapoalim B.M. valued at $200 million for the 145-unit residential elevator building (D6) at 126 East 57th Street in Midtown East, Manhattan, and a small office building that is adjacent, at 127 East 56th Street. The deal closed on June 2, 2026 and was recorded on June 18, 2026. The prior lender was Bank OZK which held debt that had an original loan amount of $170 million. The two properties have 205,102 square feet of built space and 9,517 square feet of additional air rights according to a PincusCo analysis of city data. The loan price per built square foot is $975 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) The signatory for MRR Development was Rotem Rosen . This is a $200 million loan composed of $30 million in additional construction debt, mostly a project mortgage, on top of existing $170 million construction loan originated by Bank OZK. Prior sales, articles a</t>
+          <t xml:space="preserve">Transfers 37-05 30th Street (Credit - Cyclomedia) Slate Property Group through the entity 37-11 30th Street Holdings LLC as borrower signed a refi loan with lender Ares Management through the entity Ares Commercial Real Estate Servicer LLC valued at $86.2 million for the mixed-use, 186-residential unit building at 37-05 30th Street in Long Island City, Queens. The buildings is divided into five commercial condominiums, all covered by this loan. The deal closed on June 1, 2026 and was recorded on June 22, 2026. The prior lender was PCCP which held debt that had an original loan amount of $85 million. The five condo units have 188,419 square feet of built space according to a PincusCo analysis of city data. The loan price per built square foot is $457 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) The signatory for Slate Property Group was Martin Nussbaum . The property The rental condo with 186 residential units in Long Island City has 188,419 square feet of built space according to a PincusCo analysis of city data. The parcel has a total lot size </t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Or Trabelsi signs $6M acquisition loan with S3 Capital for 22-unit walkup in Garment District</t>
+          <t>Madison Realty Capital signs $104.8M refi for 419-unit rental in Rego Park</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>https://www.pincusco.com/or-trabelsi-signs-6m-acquisition-loan-with-s3-capital-for-22-unit-walkup-in-garment-district/</t>
+          <t>https://www.pincusco.com/madison-realty-capital-signs-104-8m-refi-for-419-unit-rental-in-rego-park/</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Or Trabelsi through the entity 510 AIC LLC as borrower signed an acquisition loan with</t>
+          <t>Madison Realty Capital through the entity 62-60 99th Street Owner II LLC as borrower signed</t>
         </is>
       </c>
       <c r="D4" t="inlineStr"/>
@@ -568,24 +568,24 @@
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>Transfers 510 Ninth Avenue (Credit - Cyclomedia) Or Trabelsi through the entity 510 AIC LLC as borrower signed an acquisition loan with lender S3 Capital through the entity S3 RE Perpetual Yield Funding LLC valued at $6 million for the 22-unit residential walkup building (C7) at 510 Ninth Avenue in the Garment District, Manhattan. The deal closed on February 23, 2026 and was recorded on June 18, 2026. The property has 11,341 square feet of built space and 3,503 square feet of additional air rights for a total buildable of 14,851 square feet according to a PincusCo analysis of city data. The loan price per built square foot is $529 and the price per buildable square foot is $404 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) The owner bought the property on February 23, 2026, for $5.5 million. The signatory for Or Trabelsi was Michael Raymond Mintz and Or Trabelsi. Prior sales, articles and revenue The owners according to the Department of Housing Preservation and Development includes Yuval Plattner, head officer and Michael Mintz , officer. The bu</t>
+          <t>Transfers 62-60 99th Street (Credit - Cyclomedia) Madison Realty Capital through the entity 62-60 99th Street Owner II LLC as borrower signed a refi loan with lenders Community Preservation Corporation and Related Companies through the entity Sig RCRS D Mf 2023 Venture LLC valued at $104.8 million for the 419-unit residential elevator building (D7) at 62-60 99th Street in Rego Park, Queens. The deal closed on June 11, 2026 and was recorded on June 22, 2026. The prior lenders were Community Preservation Corporation and Related Companies which held debt that had an original loan amount of $105 million. The property has 503,000 square feet of built space according to a PincusCo analysis of city data. The loan price per built square foot is $208 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) Madison Realty Capital bought the property on June 30, 2016, for $$135.5 million. The signatory for Madison Realty Capital was David Speiser . The signatory for Community Preservation Corporation and Related Companies was Robert Riggs . Prior sales, articles and r</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Green Street Group pays $2.9M for office in Tribeca</t>
+          <t>Christian Michel pays $3.9M to Witnick Real Estate for 8-unit walkup in Park Slope</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>https://www.pincusco.com/green-street-group-pays-2-9m-for-office-in-tribeca/</t>
+          <t>https://www.pincusco.com/christian-michel-pays-3-9m-to-witnick-real-estate-for-8-unit-walkup-in-park-slope/</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Green Street Group through the entity 141 West Broadway LLC paid $2.9 million through an</t>
+          <t>Christian Michel through the entity 817 8th Avenue LLC paid $3.9 million to Witnick Real</t>
         </is>
       </c>
       <c r="D5" t="inlineStr"/>
@@ -602,24 +602,24 @@
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>Transfers 141 West Broadway (Credit - Cyclomedia) Green Street Group through the entity 141 West Broadway LLC paid $2.9 million through an estate sale to the Pantzer family through the entity Three Reddy LLC for the office building (O2) at 141 West Broadway in Tribeca, Manhattan. The expected use is cash flowing. The deal closed on June 15, 2026 and was recorded on June 18, 2026. The property has 2,500 square feet of built space and 2,515 square feet of additional air rights for a total buildable of 5,014 square feet according to a PincusCo analysis of city data. The sale price per built square foot is $1,160 and the price per buildable square foot is $578 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) The signatory for the family of the late restaurateur Joan Pantzer was Dennis W. Pantzer . The signatory for Green Street Group was Joshua Greenberg . The contract date was March 12, 2025. Joan Pantzer died in 2024. She started the restaurant that became the Odeon, located next door at 145 West Broadway. Prior sales, articles and revenue Prior to th</t>
+          <t>Transfers 817 8th Avenue (Credit - Cyclomedia) Christian Michel through the entity 817 8th Avenue LLC paid $3.9 million to Witnick Real Estate Partners through the entity 817 8th Partners LLC for the eight-unit residential walkup building (C1) at 817 8th Avenue in Park Slope, Brooklyn. The expected use is cash flowing. The deal closed on June 10, 2026 and was recorded on June 22, 2026. The property has 5,576 square feet of built space and 641 square feet of additional air rights for a total buildable of 6,210 square feet according to a PincusCo analysis of city data. The sale price per built square foot is $703 and the price per buildable square foot is $631 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) The seller bought the property on January 16, 2019, for $3.6 million. The signatory for Witnick Real Estate Partners was Ramiel Ben Yehuda . The signatory for Christian Michel was Christian Michel. The contract date was February 18, 2026. Prior sales, articles and revenue Prior to this transaction, PincusCo has no record that the buyer Christian M</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Bastone family signs $5.8M loan with Galinn Fund for The Pine restaurant in Bronx</t>
+          <t>Chen Xi Li pays $4.5M for mixed-use in Flushing</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>https://www.pincusco.com/bastone-family-signs-5-8m-loan-with-galinn-fund-for-the-pine-restaurant-in-bronx/</t>
+          <t>https://www.pincusco.com/chen-xi-li-pays-4-5m-for-mixed-use-in-flushing/</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>The Bastone family through the entity 1911-1913 Bronxdale Avenue Realty LLC as borrower signed a</t>
+          <t>Chen Xi Li through the entity Teng Di NY 99 LLC paid $4.5 million to</t>
         </is>
       </c>
       <c r="D6" t="inlineStr"/>
@@ -636,24 +636,24 @@
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>Transfers 1913 Bronxdale Avenue (Credit - Cyclomedia) The Bastone family through the entity 1911-1913 Bronxdale Avenue Realty LLC as borrower signed a loan with lender Galinn Fund through the entity The Galinn Fund LLC valued at $5.8 million for five tax lots that form the location of the The Pine restaurant and banquet hall, including the retail building (K1) at 1907 Bronxdale Avenue in Van Nest, Bronx, mixed-use building (K4) at 1913 Bronxdale Avenue in Van Nest, Bronx, and parking (G7) at 1903 Bronxdale Avenue in Van Nest, Bronx. The main address for the restaurant is 1913 Bronxdale Avenue. The deal closed on June 10, 2026 and was recorded on June 18, 2026. A prior lender, Noble Capital Management, provided debt that had an original loan amount of $3 million. The five properties have 15,996 square feet of built space and 16,525 square feet of additional air rights for a total buildable of 32,487 square feet according to a PincusCo analysis of city data. The loan price per built square foot is $362 and the price per buildable square foot is $178 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public rec</t>
+          <t xml:space="preserve">Transfers 37-02 Prince Street (Credit - Cyclomedia) Chen Xi Li through the entity Teng Di NY 99 LLC paid $4.5 million to Jong Yoon through the entity Yn World, LLC for the two-unit mixed-use building (K4) at 37-02 Prince Street in Flushing, Queens. The expected use is cash flowing. The deal closed on June 9, 2026 and was recorded on June 22, 2026. The property has 3,777 square feet of built space according to a PincusCo analysis of city data. The sale price per built square foot is $1,191 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) The seller bought the property on December 22, 2006, for $2.7 million. The signatory for Jong Yoon was Jong S. Yoon . The signatory for Chen Xi Li was Chen Xi Li. The contract date was April 1, 2026. Prior sales, articles and revenue Prior to this transaction, PincusCo has no record that the buyer Chen Xi Li had purchased any other properties and has no record it sold any properties over the past 24 months. The seller Jong Yoon had not purchased any other properties and had not sold any properties over the same time </t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Jun Kil, Suk Chang pay $3M for retail in Queens Village</t>
+          <t>Janet Huang, Judy Mock, Huei Hsiang Wang pay $12.6M Dan Ohebshalom retail in Elmhurst</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>https://www.pincusco.com/jun-kil-suk-chang-pay-3m-for-retail-in-queens-village/</t>
+          <t>https://www.pincusco.com/janet-huang-judy-mock-huei-hsiang-wang-pay-12-6m-dan-ohebshalom-retail-in-elmhurst/</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Jun Bum Kil and Suk Nyo Chang through the entity 216 Hillside LLC paid $3</t>
+          <t>Janet Huang, Judy Mock, and Huei Hsiang Wang through the entity Jktw Laguardia Holding LLC</t>
         </is>
       </c>
       <c r="D7" t="inlineStr"/>
@@ -670,24 +670,24 @@
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>Transfers 216-20 Hillside Avenue (Credit - Cyclomedia) Jun Bum Kil and Suk Nyo Chang through the entity 216 Hillside LLC paid $3 million to the Zirinsky family through the entity Hillside Metro Associates LLC for the retail building (K1) at 216-20 Hillside Avenue in Queens Village, Queens. The expected use is owner-occupied, for the grocery store John’s Farm Market. The deal closed on June 5, 2026 and was recorded on June 18, 2026. The property has 4,500 square feet of built space and 4,440 square feet of additional air rights for a total buildable of 9,000 square feet according to a PincusCo analysis of city data. The sale price per built square foot is $666 and the price per buildable square foot is $333 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) The signatory for Cynthia Zirinsky was Jerome L. Levine, Cynthia Eckes , Susan Zirinsky, John Zirinsky , and William Zirinsky. The signatory for Jun Bum Kil and Suk Nyo Chang was Jun B. Kil . The contract date was May 14, 2026. The sellers are the descendants of the married couple Richard William Zi</t>
+          <t>Transfers 81-11 Broadway (Credit - Cyclomedia) Janet Huang, Judy Mock, and Huei Hsiang Wang through the entity Jktw Laguardia Holding LLC paid $12.6 million to Daniel Ohebshalom ‘s Keystone Management through the entity Highpoint Associates IX, LLC for the retail building (K1) at 81-11 Broadway and the retail building (K1) at 81-01 Broadway in Elmhurst, Queens. The deal closed on June 15, 2026 and was recorded on June 22, 2026. The two properties have 20,000 square feet of built space and 62,781 square feet of additional air rights for a total buildable of 82,724 square feet according to a PincusCo analysis of city data. The sale price per built square foot is $630 and the price per buildable square foot is $152 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) The signatory for Keystone Management was Anthony J. Schlur. The signatory for Janet Huang, Judy Mock , and Huei Hsiang Wang was Janet Huang, Judy Mock, and Huei Hsiang Wang. The contract date was June 19, 2026. These buyers, five days earlier on June 10, 2026, sold a parking lot to Azimuth De</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Heskel’s Asset Management signs $8.6M refi with FourLeaf for 62-unit rental in Washington Heights</t>
+          <t>Azimuth, Vertical Realty pay $12.9M for parking lot in Jackson Heights</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>https://www.pincusco.com/heskels-asset-management-signs-8-6m-refi-with-fourleaf-for-62-unit-rental-in-washington-heights/</t>
+          <t>https://www.pincusco.com/azimuth-vertical-realty-pay-12-9m-for-industrial-in-jackson-heights/</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Heskel’s Asset Management through the entity Heskel’s FW Realty LLC as borrower signed a refi</t>
+          <t>Azimuth Development Group and Vertical Realty Capital through the entity AZ LGA Owner LLC paid</t>
         </is>
       </c>
       <c r="D8" t="inlineStr"/>
@@ -704,24 +704,24 @@
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>Transfers 567 Ft. Washington Avenue (Credit - Cyclomedia) Heskel’s Asset Management through the entity Heskel’s FW Realty LLC as borrower signed a refi loan with lender FourLeaf Federal Credit Union through the entity Fourleaf Federal Credit Union valued at $8.6 million for the 62-unit residential elevator building (D1) at 567 Ft Washington Avenue in Washington Heights, Manhattan. The deal closed on June 12, 2026 and was recorded on June 18, 2026. The prior lender was Webster Bank which held debt that had an original loan amount of $9.9 million.The property has 59,976 square feet of built space according to a PincusCo analysis of city data. The loan price per built square foot is $143 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) The signatory for Heskel’s Asset Management was Ramin Sarraf . The signatory for FourLeaf Federal Credit Union was Julian Cokro . Prior sales, articles and revenue The owners according to the Department of Housing Preservation and Development includes Ramin Sarraf, head officer and Elvis Debernardo, site manager. The bus</t>
+          <t>Transfers 90-26 Grand Central Parkway (Credit - Cyclomedia) Azimuth Development Group and Vertical Realty Capital through the entity AZ LGA Owner LLC paid $12.9 million to Janet Huang, Judy Mock, and Huei Hsiang Wang through the entity Jktw LaGuardia Holding LLC for the parking lot (G7) at 90-26 Grand Central Parkway in Jackson Heights, Queens. The deal closed on June 10, 2026 and was recorded on June 22, 2026. The property has zero square feet of built space and 29,135 square feet of additional air rights for a total buildable of 29,135 square feet according to a PincusCo analysis of city data. The sale price per buildable square foot is $444 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) The signatory for Janet Huang, Judy Mock , and Huei Hsiang Wang was Janet Huang, Judy Mock, and Huei Hsiang Wang. The signatory for Azimuth Development Group and Vertical Realty Capital was Guido Subotovsky and Jake Feldman . The contract date was May 15, 2026. The sellers, five days later on June 15, 2026, paid $12.6 million for retail in Elmhurst, Queens. Prio</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>P. Zaccaro signs $32.8M refi with Derby Copeland for properties in Nolita, Chinatown, SoHo</t>
+          <t>Sendowskis pay $17M for walkups in Lincoln Square, paid $45.5M for adjacent building</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>https://www.pincusco.com/p-zaccaro-signs-32-8m-refi-with-derby-copeland-for-properties-in-nolita-chinatown-soho/</t>
+          <t>https://www.pincusco.com/sendowskis-pay-17m-for-walkups-in-lincoln-square-paid-45-5m-for-adjacent-building/</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>P. Zaccaro through the entity 1-3 Mott And 218 Lafayette Street Partners, LLC as borrower</t>
+          <t>Janusz Sendowski and Oren Sendowski through the entity 15 W64, LLC paid $17 million to</t>
         </is>
       </c>
       <c r="D9" t="inlineStr"/>
@@ -738,7 +738,41 @@
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>Transfers 218 Lafayette Street (Credit - Cyclomedia) P. Zaccaro through the entity 1-3 Mott And 218 Lafayette Street Partners, LLC as borrower signed a refi loan with lender Derby Copeland Capital through the entity DCC Remmcf Seller Atlas, LLC valued at $32.8 million for three properties in Manhattan with 27 residential units including the 24-unit residential walkup building (C7) at 241 Mulberry Street in Nolita, the three-unit mixed-use building (K4) at 1-3 Mott Street in Chinatown, and mixed-use building (K2) at 218 Lafayette Street in SoHo. The deal closed on May 11, 2026 and was recorded on June 18, 2026. The prior lender was Oceanview Life and Annuity Company. The three properties have 26,026 square feet of built space and 10,145 square feet of additional air rights for a total buildable of 35,266 square feet according to a PincusCo analysis of city data. The loan price per built square foot is $1,258 and the price per buildable square foot is $928 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) The signatory for P. Zaccaro was John A. Zaccar</t>
+          <t xml:space="preserve">Transfers 15 West 64th Street (Credit - Cyclomedia) Janusz Sendowski and Oren Sendowski through the entity 15 W64, LLC paid $17 million to Elliot Sohayegh through the entity NYC 6400 Holdings LLC for the 20-unit residential walkup building (C4) at 15 West 64th Street and the 20-unit residential walkup building (C4) at 15A West 64th Street in Lincoln Square, Manhattan. The expected use is cash flowing. The buildings are on adjacent lots to the 86-unit residential elevator building (D1) at 10 West 65th Street which the Sendowski family bought last year for $45.5 million. The new deal closed on April 28, 2026 and was recorded on June 22, 2026. The two properties have 18,830 square feet of built space and 11,395 square feet of additional air rights for a total buildable of 30,220 square feet according to a PincusCo analysis of city data. The sale price per built square foot is $902 and the price per buildable square foot is $562 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) The signatory for Elliot Sohayegh was Stephen S. Siminou . The signatory for </t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>TA Realty pays $79.2M to Bregman Organization for Staten Island shopping center</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>https://www.pincusco.com/ta-realty-pays-79-2m-to-bregman-organization-for-shopping-center-in-new-dorp-beach/</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>TA Realty through the entity Scrs Tysen Park LLC paid $79.2 million to Bregman Organization</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr"/>
+      <c r="E10" t="inlineStr"/>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>PincusCo</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>PincusCo - Home</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>Chart_Frontpage Top Story Transfers 2754 Hylan Boulevard (Credit - Cyclomedia) TA Realty through the entity Scrs Tysen Park LLC paid $79.2 million to Bregman Organization through the entity Park Tysen Associates, LLC for Tysens Park Shopping Center (K6) at the addresses 2712 Hylan Boulevard at 2754 Hylan Boulevard in New Dorp Beach, Staten Island. The expected use is cash flowing. The deal closed on May 19, 2026 and was recorded on June 22, 2026. The two properties have 184,204 square feet of built space and 632,284 square feet of additional air rights for a total buildable of 818,733 square feet according to a PincusCo analysis of city data. The sale price per built square foot is $429 and the price per buildable square foot is $96 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) The signatory for Bregman Organization was Paul A. Bregman . The signatory for TA Realty was James P. Raisides . The contract date was February 19, 2026. The seller is an LLC, that was formerly a partnership, of a group of families that has owned the property for several d</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto update queens news 2026-06-24T14:52:08Z
</commit_message>
<xml_diff>
--- a/data/output/queens_dev_news.xlsx
+++ b/data/output/queens_dev_news.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H10"/>
+  <dimension ref="A1:H9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -473,17 +473,17 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Derek Fraser files plans for 26 units in Ditmars Steinway</t>
+          <t>Oleksandr Nad signs $13M construction loan with Colorado Federal for 18-unit project in Two Bridges</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>https://www.pincusco.com/derek-fraser-files-plans-for-26-units-in-ditmars-steinway/</t>
+          <t>https://www.pincusco.com/oleksandr-nad-signs-13m-construction-loan-with-colorado-federal-for-18-unit-project-in-two-bridges/</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Derek Fraser submitted a new building construction project for a 26-unit, 17,416-square-foot residential (R-2) building</t>
+          <t>Oleksandr Nad through the entity 83 Madison Holdings LLC as borrower signed a new construction</t>
         </is>
       </c>
       <c r="D2" t="inlineStr"/>
@@ -500,24 +500,24 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>Development 23-01 31st Street axonometric diagram (Credit - Harriet Nikakis architect via DOB) Derek Fraser submitted a new building construction project for a 26-unit, 17,416-square-foot residential (R-2) building at 23-01 31st Street in Ditmars Steinway, Queens. The plan was filed on June 18, 2026. It calls for the construction of a 84-foot-tall, eight-story building and was filed with the New York City Department of Buildings under job number Q01257109. The project is described in the filing as: new 8-story building 26 units, with commercial and community facility.. The applicant is the Registered Architect Harriet Nikakis of Hcn Design. Derek Fraser of Derek Fraser submitted the plans. The most recent property records show Pericles Notias purchased this parcel for $4.2 million in February 2024. 23-01 31st Street The neighborhood</t>
+          <t>Transfers 83 Madison Street axonometric diagram (Credit - Zarina Kindo architect via DOB) Oleksandr Nad through the entity 83 Madison Holdings LLC as borrower signed a new construction loan with lender Colorado Federal Savings Bank valued at $13 million for the 18-unit development project at 83 Madison Street in Two Bridges, Manhattan. On the lot, there is one active new building construction project, M00979759, for an 18-unit, 24,041 square-foot residential (R-2) building. The project was submitted by Oleksandr Nad on December 21, 2023 and permitted March 10, 2026. The loan closed on May 29, 2026 and was recorded on June 22, 2026. The prior lender was Colorado Federal Savings Bank which held debt that had an original loan amount of $2.4 million. The loan price per planned development square foot is $541 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) The owner bought the property on November 21, 2023, for $5.2 million. The signatory for Oleksandr Nad was Oleksandr Nad. The property The specialty building in Two Bridges has 7,556 square feet of bui</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Slate Property Group signs $86.2M refi with Ares for 186-unit rental in LIC</t>
+          <t>CW Realty Group signs 99-year lease valued at $9.7M with Kimco for LIC dev site</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>https://www.pincusco.com/slate-property-group-signs-86-2m-refi-with-ares-for-186-unit-rental-in-lic/</t>
+          <t>https://www.pincusco.com/cw-realty-group-signs-99-year-lease-valued-at-9-7m-with-kimco-for-lic-dev-site/</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Slate Property Group through the entity 37-11 30th Street Holdings LLC as borrower signed a</t>
+          <t>CW Realty Group through the entity 44 Drive GL LLC as tenant signed a ground</t>
         </is>
       </c>
       <c r="D3" t="inlineStr"/>
@@ -534,24 +534,24 @@
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Transfers 37-05 30th Street (Credit - Cyclomedia) Slate Property Group through the entity 37-11 30th Street Holdings LLC as borrower signed a refi loan with lender Ares Management through the entity Ares Commercial Real Estate Servicer LLC valued at $86.2 million for the mixed-use, 186-residential unit building at 37-05 30th Street in Long Island City, Queens. The buildings is divided into five commercial condominiums, all covered by this loan. The deal closed on June 1, 2026 and was recorded on June 22, 2026. The prior lender was PCCP which held debt that had an original loan amount of $85 million. The five condo units have 188,419 square feet of built space according to a PincusCo analysis of city data. The loan price per built square foot is $457 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) The signatory for Slate Property Group was Martin Nussbaum . The property The rental condo with 186 residential units in Long Island City has 188,419 square feet of built space according to a PincusCo analysis of city data. The parcel has a total lot size </t>
+          <t>Chart_Frontpage Transfers 21-02 44th Drive (Credit - Cyclomedia) CW Realty Group through the entity 44 Drive GL LLC as tenant signed a ground lease valued at $9.7 million with landlord Kimco Realty through the entity Market Shop 1696, LLC covering the retail building (K1) at 21-02 44th Drive in Long Island City, Queens. The expected use is ground up development. The deal closed on June 11, 2026 and was recorded on June 23, 2026. The property has 6,000 square feet of built space and 34,304 square feet of additional air rights for a total buildable of 40,334 square feet according to a PincusCo analysis of city data. The sale price per built square foot is $1,610 and the price per buildable square foot is $239 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) Kimco Realty bought the property on December 27, 2012, for $3.6 million. The signatory for Kimco Realty was Alexis Y. Adams . The signatory for CW Realty Group was Cheskie Weisz . This is a 99-year ground lease lease. Kimco and CW Realty Group each have a right of first refusal to acquire the other</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Madison Realty Capital signs $104.8M refi for 419-unit rental in Rego Park</t>
+          <t>Ridwan Kabir pays $4.3M for office in Hollis</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>https://www.pincusco.com/madison-realty-capital-signs-104-8m-refi-for-419-unit-rental-in-rego-park/</t>
+          <t>https://www.pincusco.com/ridwan-kabir-pays-4-3m-for-office-in-hollis/</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Madison Realty Capital through the entity 62-60 99th Street Owner II LLC as borrower signed</t>
+          <t>Ridwan Kabir through the entity 189 Hillside Plaza LLC paid $4.3 million to Shahid Ali</t>
         </is>
       </c>
       <c r="D4" t="inlineStr"/>
@@ -568,24 +568,24 @@
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>Transfers 62-60 99th Street (Credit - Cyclomedia) Madison Realty Capital through the entity 62-60 99th Street Owner II LLC as borrower signed a refi loan with lenders Community Preservation Corporation and Related Companies through the entity Sig RCRS D Mf 2023 Venture LLC valued at $104.8 million for the 419-unit residential elevator building (D7) at 62-60 99th Street in Rego Park, Queens. The deal closed on June 11, 2026 and was recorded on June 22, 2026. The prior lenders were Community Preservation Corporation and Related Companies which held debt that had an original loan amount of $105 million. The property has 503,000 square feet of built space according to a PincusCo analysis of city data. The loan price per built square foot is $208 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) Madison Realty Capital bought the property on June 30, 2016, for $$135.5 million. The signatory for Madison Realty Capital was David Speiser . The signatory for Community Preservation Corporation and Related Companies was Robert Riggs . Prior sales, articles and r</t>
+          <t>Transfers 189-10 Hillside Avenue (Credit - Cyclomedia) Ridwan Kabir through the entity 189 Hillside Plaza LLC paid $4.3 million to Shahid Ali through the entity Abpc LLC for the office building (O2) at 189-10 Hillside Avenue in Hollis, Queens. The deal closed on May 29, 2026 and was recorded on June 23, 2026. The property has 17,600 square feet of built space and 14,598 square feet of additional air rights for a total buildable of 32,202 square feet according to a PincusCo analysis of city data. The sale price per built square foot is $244 and the price per buildable square foot is $133 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) The seller bought the property on September 23, 2020, for $4.5 million. The signatory for Shahid Ali was Shahid Ali. The signatory for Ridwan Kabir was Ridwan Kabir. The contract date was January 6, 2026. Prior sales, articles and revenue Prior to this transaction, PincusCo has no record that the buyer Ridwan Kabir had purchased any other properties and sold one property in one transaction for a total of $3.6 million o</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Christian Michel pays $3.9M to Witnick Real Estate for 8-unit walkup in Park Slope</t>
+          <t>Gora Group pays $16.8M to Treeline Companies for office in Brooklyn Heights</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>https://www.pincusco.com/christian-michel-pays-3-9m-to-witnick-real-estate-for-8-unit-walkup-in-park-slope/</t>
+          <t>https://www.pincusco.com/gora-group-pays-16-8m-to-treeline-companies-for-office-in-brooklyn-heights/</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Christian Michel through the entity 817 8th Avenue LLC paid $3.9 million to Witnick Real</t>
+          <t>Gora Group through the entity 188 Montague LLC paid $16.8 million to Treeline Companies through</t>
         </is>
       </c>
       <c r="D5" t="inlineStr"/>
@@ -602,24 +602,24 @@
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>Transfers 817 8th Avenue (Credit - Cyclomedia) Christian Michel through the entity 817 8th Avenue LLC paid $3.9 million to Witnick Real Estate Partners through the entity 817 8th Partners LLC for the eight-unit residential walkup building (C1) at 817 8th Avenue in Park Slope, Brooklyn. The expected use is cash flowing. The deal closed on June 10, 2026 and was recorded on June 22, 2026. The property has 5,576 square feet of built space and 641 square feet of additional air rights for a total buildable of 6,210 square feet according to a PincusCo analysis of city data. The sale price per built square foot is $703 and the price per buildable square foot is $631 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) The seller bought the property on January 16, 2019, for $3.6 million. The signatory for Witnick Real Estate Partners was Ramiel Ben Yehuda . The signatory for Christian Michel was Christian Michel. The contract date was February 18, 2026. Prior sales, articles and revenue Prior to this transaction, PincusCo has no record that the buyer Christian M</t>
+          <t>Transfers 188 Montague Street (Credit - Cyclomedia) Gora Group through the entity 188 Montague LLC paid $16.8 million to Treeline Companies through the entity Treeline 188 Montague LLC for the office building (O6) at 188 Montague Street in Brooklyn Heights, Brooklyn. The expected use is cash flowing. The deal closed on June 10, 2026 and was recorded on June 23, 2026. The property has 48,050 square feet of built space and 23,976 square feet of additional air rights for a total buildable of 72,000 square feet according to a PincusCo analysis of city data. The sale price per built square foot is $349 and the price per buildable square foot is $233 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) The signatory for Treeline Companies was Michael Schor . The signatory for Gora Group was Samuel Friedman . The contract date was February 2, 2026. Crain’s reported on the sale previously, noting that Treeline acquired the property in 1993 for $5.2 million. The 1993 purchase was through a foreclosure auction, a review of city records found. Prior sales, article</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Chen Xi Li pays $4.5M for mixed-use in Flushing</t>
+          <t>Imperial Sterling pays $13M for retail in Carnegie Hill</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>https://www.pincusco.com/chen-xi-li-pays-4-5m-for-mixed-use-in-flushing/</t>
+          <t>https://www.pincusco.com/imperial-sterling-pays-13m-for-retail-in-carnegie-hill/</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Chen Xi Li through the entity Teng Di NY 99 LLC paid $4.5 million to</t>
+          <t>Imperial Sterling through the entity Imperial Madison, LLC paid $13 million to Keith Kantrowitz and</t>
         </is>
       </c>
       <c r="D6" t="inlineStr"/>
@@ -636,24 +636,24 @@
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t xml:space="preserve">Transfers 37-02 Prince Street (Credit - Cyclomedia) Chen Xi Li through the entity Teng Di NY 99 LLC paid $4.5 million to Jong Yoon through the entity Yn World, LLC for the two-unit mixed-use building (K4) at 37-02 Prince Street in Flushing, Queens. The expected use is cash flowing. The deal closed on June 9, 2026 and was recorded on June 22, 2026. The property has 3,777 square feet of built space according to a PincusCo analysis of city data. The sale price per built square foot is $1,191 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) The seller bought the property on December 22, 2006, for $2.7 million. The signatory for Jong Yoon was Jong S. Yoon . The signatory for Chen Xi Li was Chen Xi Li. The contract date was April 1, 2026. Prior sales, articles and revenue Prior to this transaction, PincusCo has no record that the buyer Chen Xi Li had purchased any other properties and has no record it sold any properties over the past 24 months. The seller Jong Yoon had not purchased any other properties and had not sold any properties over the same time </t>
+          <t>Top Story Transfers 1295 Madison Avenue (Credit - Cyclomedia) Imperial Sterling through the entity Imperial Madison, LLC paid $13 million to Keith Kantrowitz and musician Ryan Tedder‘s Patriot Real Estate Holdings through the entity MRK Jacksonville, LLC for the retail condo at 1295 Madison Avenue in Carnegie Hill, Manhattan. The expected use is cash flowing. The deal closed on June 11, 2026 and was recorded on June 23, 2026. The property has 3,024 square feet of built space according to a PincusCo analysis of city data. The sale price per built square foot is $4,298 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) The seller bought the property on November 9, 2023, for $11 million. The signatory for Keith Kantrowitz and Patriot Real Estate Holdings was Nelson Braff and Keith Kantrowitz. The signatory for Imperial Sterling was Jerrold G. Levy . The contract date was March 24, 2026. Prior sales, articles and revenue Prior to this transaction, PincusCo has records that the buyer Imperial Sterling purchased two properties in two transactions for a tota</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Janet Huang, Judy Mock, Huei Hsiang Wang pay $12.6M Dan Ohebshalom retail in Elmhurst</t>
+          <t>Jacob Kohn pays $5M to Cycamore Capital for mixed-use in Bedford Stuyvesant</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>https://www.pincusco.com/janet-huang-judy-mock-huei-hsiang-wang-pay-12-6m-dan-ohebshalom-retail-in-elmhurst/</t>
+          <t>https://www.pincusco.com/jacob-kohn-pays-5m-to-cycamore-capital-for-mixed-use-in-bedford-stuyvesant/</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Janet Huang, Judy Mock, and Huei Hsiang Wang through the entity Jktw Laguardia Holding LLC</t>
+          <t>Jacob Kohn through the entity Myrtle Kent Development LLC paid $5 million to Cycamore Capital</t>
         </is>
       </c>
       <c r="D7" t="inlineStr"/>
@@ -670,24 +670,24 @@
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>Transfers 81-11 Broadway (Credit - Cyclomedia) Janet Huang, Judy Mock, and Huei Hsiang Wang through the entity Jktw Laguardia Holding LLC paid $12.6 million to Daniel Ohebshalom ‘s Keystone Management through the entity Highpoint Associates IX, LLC for the retail building (K1) at 81-11 Broadway and the retail building (K1) at 81-01 Broadway in Elmhurst, Queens. The deal closed on June 15, 2026 and was recorded on June 22, 2026. The two properties have 20,000 square feet of built space and 62,781 square feet of additional air rights for a total buildable of 82,724 square feet according to a PincusCo analysis of city data. The sale price per built square foot is $630 and the price per buildable square foot is $152 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) The signatory for Keystone Management was Anthony J. Schlur. The signatory for Janet Huang, Judy Mock , and Huei Hsiang Wang was Janet Huang, Judy Mock, and Huei Hsiang Wang. The contract date was June 19, 2026. These buyers, five days earlier on June 10, 2026, sold a parking lot to Azimuth De</t>
+          <t xml:space="preserve">Transfers 620 Myrtle Avenue (Credit - Cyclomedia) Jacob Kohn through the entity Myrtle Kent Development LLC paid $5 million to Cycamore Capital through the entity 620 Myrtle Avenue, LLC for the four-unit mixed-use building (S4) at 620 Myrtle Avenue in Bedford Stuyvesant, Brooklyn. The deal closed on June 3, 2026 and was recorded on June 23, 2026. The property has 5,625 square feet of built space and 5,560 square feet of additional air rights for a total buildable of 11,176 square feet according to a PincusCo analysis of city data. The sale price per built square foot is $888 and the price per buildable square foot is $447 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) The seller bought the property on November 14, 2019, for $3.1 million. The signatory for Cycamore Capital was Kenneth P. Horowitz . The signatory for Jacob Kohn was Jacob Kohn. The contract date was May 1, 2025. PincusCo analysis indicates this Jacob Kohn is not the same individual with the same name at Jay Group. Prior sales, articles and revenue Prior to this transaction, PincusCo </t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Azimuth, Vertical Realty pay $12.9M for parking lot in Jackson Heights</t>
+          <t>Andras Fenyves pays $2.9M for mixed-use in Bedford Stuyvesant</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>https://www.pincusco.com/azimuth-vertical-realty-pay-12-9m-for-industrial-in-jackson-heights/</t>
+          <t>https://www.pincusco.com/andras-fenyves-pays-2-9m-for-mixed-use-in-bedford-stuyvesant/</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Azimuth Development Group and Vertical Realty Capital through the entity AZ LGA Owner LLC paid</t>
+          <t>Andras Fenyves through the entity 1276 Broadway LLC paid $2.9 million to Joseph Felix through</t>
         </is>
       </c>
       <c r="D8" t="inlineStr"/>
@@ -704,24 +704,24 @@
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>Transfers 90-26 Grand Central Parkway (Credit - Cyclomedia) Azimuth Development Group and Vertical Realty Capital through the entity AZ LGA Owner LLC paid $12.9 million to Janet Huang, Judy Mock, and Huei Hsiang Wang through the entity Jktw LaGuardia Holding LLC for the parking lot (G7) at 90-26 Grand Central Parkway in Jackson Heights, Queens. The deal closed on June 10, 2026 and was recorded on June 22, 2026. The property has zero square feet of built space and 29,135 square feet of additional air rights for a total buildable of 29,135 square feet according to a PincusCo analysis of city data. The sale price per buildable square foot is $444 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) The signatory for Janet Huang, Judy Mock , and Huei Hsiang Wang was Janet Huang, Judy Mock, and Huei Hsiang Wang. The signatory for Azimuth Development Group and Vertical Realty Capital was Guido Subotovsky and Jake Feldman . The contract date was May 15, 2026. The sellers, five days later on June 15, 2026, paid $12.6 million for retail in Elmhurst, Queens. Prio</t>
+          <t>Transfers 1276 Broadway (Credit - Cyclomedia) Andras Fenyves through the entity 1276 Broadway LLC paid $2.9 million to Joseph Felix through the entity Triangle Square Corp. for the two-unit mixed-use building (S9) at 1276 Broadway in Bedford Stuyvesant, Brooklyn. The expected use is cash flowing. The deal closed on June 10, 2026 and was recorded on June 22, 2026. The property has 4,626 square feet of built space and 7,301 square feet of additional air rights for a total buildable of 11,920 square feet according to a PincusCo analysis of city data. The sale price per built square foot is $626 and the price per buildable square foot is $243 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) The signatory for Joseph Felix was Joseph Felix. The signatory for Andras Fenyves was Andras Fenyves. The contract date was January 12, 2026. Prior sales, articles and revenue Prior to this transaction, PincusCo has no record that the buyer Andras Fenyves had purchased any other properties and has no record it sold any properties over the past 24 months. The seller J</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Sendowskis pay $17M for walkups in Lincoln Square, paid $45.5M for adjacent building</t>
+          <t>Westbridge Realty Group files plans for 72 units in Washington Heights</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>https://www.pincusco.com/sendowskis-pay-17m-for-walkups-in-lincoln-square-paid-45-5m-for-adjacent-building/</t>
+          <t>https://www.pincusco.com/westbridge-realty-group-files-plans-for-72-units-in-washington-heights/</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Janusz Sendowski and Oren Sendowski through the entity 15 W64, LLC paid $17 million to</t>
+          <t>Westbridge Realty Group submitted a new building construction project for a 72-unit, 56,615-square-foot residential (R-2)</t>
         </is>
       </c>
       <c r="D9" t="inlineStr"/>
@@ -738,41 +738,7 @@
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t xml:space="preserve">Transfers 15 West 64th Street (Credit - Cyclomedia) Janusz Sendowski and Oren Sendowski through the entity 15 W64, LLC paid $17 million to Elliot Sohayegh through the entity NYC 6400 Holdings LLC for the 20-unit residential walkup building (C4) at 15 West 64th Street and the 20-unit residential walkup building (C4) at 15A West 64th Street in Lincoln Square, Manhattan. The expected use is cash flowing. The buildings are on adjacent lots to the 86-unit residential elevator building (D1) at 10 West 65th Street which the Sendowski family bought last year for $45.5 million. The new deal closed on April 28, 2026 and was recorded on June 22, 2026. The two properties have 18,830 square feet of built space and 11,395 square feet of additional air rights for a total buildable of 30,220 square feet according to a PincusCo analysis of city data. The sale price per built square foot is $902 and the price per buildable square foot is $562 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) The signatory for Elliot Sohayegh was Stephen S. Siminou . The signatory for </t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>TA Realty pays $79.2M to Bregman Organization for Staten Island shopping center</t>
-        </is>
-      </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>https://www.pincusco.com/ta-realty-pays-79-2m-to-bregman-organization-for-shopping-center-in-new-dorp-beach/</t>
-        </is>
-      </c>
-      <c r="C10" t="inlineStr">
-        <is>
-          <t>TA Realty through the entity Scrs Tysen Park LLC paid $79.2 million to Bregman Organization</t>
-        </is>
-      </c>
-      <c r="D10" t="inlineStr"/>
-      <c r="E10" t="inlineStr"/>
-      <c r="F10" t="inlineStr">
-        <is>
-          <t>PincusCo</t>
-        </is>
-      </c>
-      <c r="G10" t="inlineStr">
-        <is>
-          <t>PincusCo - Home</t>
-        </is>
-      </c>
-      <c r="H10" t="inlineStr">
-        <is>
-          <t>Chart_Frontpage Top Story Transfers 2754 Hylan Boulevard (Credit - Cyclomedia) TA Realty through the entity Scrs Tysen Park LLC paid $79.2 million to Bregman Organization through the entity Park Tysen Associates, LLC for Tysens Park Shopping Center (K6) at the addresses 2712 Hylan Boulevard at 2754 Hylan Boulevard in New Dorp Beach, Staten Island. The expected use is cash flowing. The deal closed on May 19, 2026 and was recorded on June 22, 2026. The two properties have 184,204 square feet of built space and 632,284 square feet of additional air rights for a total buildable of 818,733 square feet according to a PincusCo analysis of city data. The sale price per built square foot is $429 and the price per buildable square foot is $96 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) The signatory for Bregman Organization was Paul A. Bregman . The signatory for TA Realty was James P. Raisides . The contract date was February 19, 2026. The seller is an LLC, that was formerly a partnership, of a group of families that has owned the property for several d</t>
+          <t>Development Rendering of 671 West 187th Street, with an alternate address of 673 West 187th Street (Credit - Leandro Nils Dickson architect via DOB) Westbridge Realty Group submitted a new building construction project for a 72-unit, 56,615-square-foot residential (R-2) building at 671 West 187th Street, with an alternate address of 673 West 187th Street, in Washington Heights, Manhattan. The plan was filed on June 19, 2026. It calls for the construction of a 155-foot-tall, sixteen-story building and was filed with the New York City Department of Buildings under job number M01417673. The project is described in the filing as: development hub job by default; as project is greater than seven (7) stories, per service notice posted april 16, 2021 such jobs shall be assigned to the development hub unit – subject building is a sixteen story building.. The applicant is the Registered Architect Leandro Dickson of Leandro Nils Dickson Architect. Steven Westreich of Westbridge Realty Group submitted the plans. The building does not have any retail or commercial space. 673 West 187th Street The neighborhood</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto update queens news 2026-06-25T15:09:15Z
</commit_message>
<xml_diff>
--- a/data/output/queens_dev_news.xlsx
+++ b/data/output/queens_dev_news.xlsx
@@ -473,17 +473,17 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Oleksandr Nad signs $13M construction loan with Colorado Federal for 18-unit project in Two Bridges</t>
+          <t>Sackman Enterprises, John Pearson pay $2.1M for 5-unit walkup in Harlem</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>https://www.pincusco.com/oleksandr-nad-signs-13m-construction-loan-with-colorado-federal-for-18-unit-project-in-two-bridges/</t>
+          <t>https://www.pincusco.com/sackman-enterprises-john-pearson-pays-2-1m-for-5-unit-walkup-in-harlem/</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Oleksandr Nad through the entity 83 Madison Holdings LLC as borrower signed a new construction</t>
+          <t>Sackman Enterprises and John Pearson through the entity Grace Church Community Redevelopment LLC paid $2.1</t>
         </is>
       </c>
       <c r="D2" t="inlineStr"/>
@@ -500,24 +500,24 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>Transfers 83 Madison Street axonometric diagram (Credit - Zarina Kindo architect via DOB) Oleksandr Nad through the entity 83 Madison Holdings LLC as borrower signed a new construction loan with lender Colorado Federal Savings Bank valued at $13 million for the 18-unit development project at 83 Madison Street in Two Bridges, Manhattan. On the lot, there is one active new building construction project, M00979759, for an 18-unit, 24,041 square-foot residential (R-2) building. The project was submitted by Oleksandr Nad on December 21, 2023 and permitted March 10, 2026. The loan closed on May 29, 2026 and was recorded on June 22, 2026. The prior lender was Colorado Federal Savings Bank which held debt that had an original loan amount of $2.4 million. The loan price per planned development square foot is $541 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) The owner bought the property on November 21, 2023, for $5.2 million. The signatory for Oleksandr Nad was Oleksandr Nad. The property The specialty building in Two Bridges has 7,556 square feet of bui</t>
+          <t>Transfers 314 West 139th Street (Credit - Cyclomedia) Sackman Enterprises and John Pearson through the entity Grace Church Community Redevelopment LLC paid $2.1 million to Grace Congregational Church of Harlem through the entity Grace Congregational Church Of Harlem, Inc. for the five-unit residential walkup building (C2) at 314 West 139th Street in Harlem, Manhattan. The expected use is cash flowing. The deal closed on June 12, 2026 and was recorded on June 23, 2026. The property has 4,280 square feet of built space and 1,906 square feet of additional air rights for a total buildable of 6,188 square feet according to a PincusCo analysis of city data. The sale price per built square foot is $490 and the price per buildable square foot is $339 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) The signatory for Grace Congregational Church of Harlem was Nigel Pearce. The signatory for Sackman Enterprises and John Pearson was Alan Sackman . The contract date was January 17, 2020. John Pearson owns have and Sackman owns half. Crain’s reported previously o</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>CW Realty Group signs 99-year lease valued at $9.7M with Kimco for LIC dev site</t>
+          <t>Poise Property Group signs $16.2M construction loan for 20-unit dev site in Greenpoint</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>https://www.pincusco.com/cw-realty-group-signs-99-year-lease-valued-at-9-7m-with-kimco-for-lic-dev-site/</t>
+          <t>https://www.pincusco.com/poise-property-group-signs-16-2m-construction-loan-for-20-unit-dev-site-in-greenpoint/</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>CW Realty Group through the entity 44 Drive GL LLC as tenant signed a ground</t>
+          <t>Poise Property Group through the entity 55 Eckford St LLC as borrower signed a initial</t>
         </is>
       </c>
       <c r="D3" t="inlineStr"/>
@@ -534,24 +534,24 @@
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>Chart_Frontpage Transfers 21-02 44th Drive (Credit - Cyclomedia) CW Realty Group through the entity 44 Drive GL LLC as tenant signed a ground lease valued at $9.7 million with landlord Kimco Realty through the entity Market Shop 1696, LLC covering the retail building (K1) at 21-02 44th Drive in Long Island City, Queens. The expected use is ground up development. The deal closed on June 11, 2026 and was recorded on June 23, 2026. The property has 6,000 square feet of built space and 34,304 square feet of additional air rights for a total buildable of 40,334 square feet according to a PincusCo analysis of city data. The sale price per built square foot is $1,610 and the price per buildable square foot is $239 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) Kimco Realty bought the property on December 27, 2012, for $3.6 million. The signatory for Kimco Realty was Alexis Y. Adams . The signatory for CW Realty Group was Cheskie Weisz . This is a 99-year ground lease lease. Kimco and CW Realty Group each have a right of first refusal to acquire the other</t>
+          <t xml:space="preserve">Transfers 55 Eckford Street axonometric diagram (Credit - Murat Mutlu architect via DOB) Poise Property Group through the entity 55 Eckford St LLC as borrower signed a initial loan with lender Colorado Federal Savings Bank through the entity Colorado Federalsavings Bank valued at $16.2 million for the 26-unit development building (V1) at 55 Eckford Street in Greenpoint, Brooklyn. On the lot, there is one active new building construction project, B01167721, for a 20-unit, 22,406 square-foot residential (R-2) building. The project was submitted by Poise Property Group and filed by Daniel Kaykov with plans filed January 27, 2025 and permitted November 21, 2025. The deal closed on May 21, 2026 and was recorded on June 23, 2026. The property has 42,449 square feet of built space and 20,752 square feet of additional air rights according to a PincusCo analysis of city data. The loan price per built square foot is $381 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) The owner bought the property on April 24, 2024, for $7.2 million. The signatory for Poise </t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Ridwan Kabir pays $4.3M for office in Hollis</t>
+          <t>Lonicera Partners signs $150M loan with PNC for 314-unit rental in Downtown Brooklyn</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>https://www.pincusco.com/ridwan-kabir-pays-4-3m-for-office-in-hollis/</t>
+          <t>https://www.pincusco.com/lonicera-partners-signs-150m-loan-with-pnc-for-314-unit-rental-in-downtown-brooklyn/</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Ridwan Kabir through the entity 189 Hillside Plaza LLC paid $4.3 million to Shahid Ali</t>
+          <t>Lonicera Partners through the entity Hanover Tower Owner LLC as borrower signed a loan with</t>
         </is>
       </c>
       <c r="D4" t="inlineStr"/>
@@ -568,24 +568,24 @@
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>Transfers 189-10 Hillside Avenue (Credit - Cyclomedia) Ridwan Kabir through the entity 189 Hillside Plaza LLC paid $4.3 million to Shahid Ali through the entity Abpc LLC for the office building (O2) at 189-10 Hillside Avenue in Hollis, Queens. The deal closed on May 29, 2026 and was recorded on June 23, 2026. The property has 17,600 square feet of built space and 14,598 square feet of additional air rights for a total buildable of 32,202 square feet according to a PincusCo analysis of city data. The sale price per built square foot is $244 and the price per buildable square foot is $133 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) The seller bought the property on September 23, 2020, for $4.5 million. The signatory for Shahid Ali was Shahid Ali. The signatory for Ridwan Kabir was Ridwan Kabir. The contract date was January 6, 2026. Prior sales, articles and revenue Prior to this transaction, PincusCo has no record that the buyer Ridwan Kabir had purchased any other properties and sold one property in one transaction for a total of $3.6 million o</t>
+          <t>Transfers 15 Hanover Place (Credit - Cyclomedia) Lonicera Partners through the entity Hanover Tower Owner LLC as borrower signed a loan with lender PNC Bank through the entity Pnc Bank, National Association valued at $150 million for the 314-unit residential elevator building (D6) at 15 Hanover Place in Downtown Brooklyn, Brooklyn. The deal closed on June 16, 2026 and was recorded on June 23, 2026. The prior lender was Santander Bank which held debt that had an original loan amount of $134 million. The property has 281,511 square feet of built space according to a PincusCo analysis of city data. The loan price per built square foot is $532 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) The signatory for Lonicera Partners was Jamie Anthony . The signatory for PNC Bank was Heather Finnegan . Prior sales, articles and revenue The owners according to the Department of Housing Preservation and Development includes Lucian Cohen, head officer and Wilson Acosta, agent. The business entities are Rose Property Mgmt Grp Llc and Hanover Tower Owner Llc. The 2</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Gora Group pays $16.8M to Treeline Companies for office in Brooklyn Heights</t>
+          <t>LBA Realty signs $22.8M refi loan with City National Bank for three properties in Red Hook</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>https://www.pincusco.com/gora-group-pays-16-8m-to-treeline-companies-for-office-in-brooklyn-heights/</t>
+          <t>https://www.pincusco.com/lba-realty-signs-22-8m-refi-loan-with-city-national-bank-for-three-properties-in-red-hook/</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Gora Group through the entity 188 Montague LLC paid $16.8 million to Treeline Companies through</t>
+          <t>LBA Realty through the entity 110 Beard Street, LLC as borrower signed a refi loan</t>
         </is>
       </c>
       <c r="D5" t="inlineStr"/>
@@ -602,24 +602,24 @@
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>Transfers 188 Montague Street (Credit - Cyclomedia) Gora Group through the entity 188 Montague LLC paid $16.8 million to Treeline Companies through the entity Treeline 188 Montague LLC for the office building (O6) at 188 Montague Street in Brooklyn Heights, Brooklyn. The expected use is cash flowing. The deal closed on June 10, 2026 and was recorded on June 23, 2026. The property has 48,050 square feet of built space and 23,976 square feet of additional air rights for a total buildable of 72,000 square feet according to a PincusCo analysis of city data. The sale price per built square foot is $349 and the price per buildable square foot is $233 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) The signatory for Treeline Companies was Michael Schor . The signatory for Gora Group was Samuel Friedman . The contract date was February 2, 2026. Crain’s reported on the sale previously, noting that Treeline acquired the property in 1993 for $5.2 million. The 1993 purchase was through a foreclosure auction, a review of city records found. Prior sales, article</t>
+          <t>Transfers 236 Richards Street, 110 Beard Street (Credit - Cyclomedia) LBA Realty through the entity 110 Beard Street, LLC as borrower signed a refi loan with lender City National Bank through the entity City National Bank valued at $22.8 million for three properties including the industrial building (E1) at 236 Richards Street in Red Hook, Brooklyn, industrial building (E1) at 118 Beard Street in Red Hook, Brooklyn, and hotel building (H8) at 116 Beard Street in Red Hook, Brooklyn. The deal closed on May 29, 2026 and was recorded on June 23, 2026. The prior lender was City National Bank which held debt that had an original loan amount of $22.8 million.The three properties have 97,130 square feet of built space and 96,636 square feet of additional air rights for a total buildable of 193,800 square feet according to a PincusCo analysis of city data. The loan price per built square foot is $234 and the price per buildable square foot is $117 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) The signatory for LBA Realty was Michael Memoly . The signatory</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Imperial Sterling pays $13M for retail in Carnegie Hill</t>
+          <t>Moving company pays $18M to First Pioneer for office in LIC</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>https://www.pincusco.com/imperial-sterling-pays-13m-for-retail-in-carnegie-hill/</t>
+          <t>https://www.pincusco.com/moving-company-pays-18m-to-first-pioneer-for-office-in-lic/</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Imperial Sterling through the entity Imperial Madison, LLC paid $13 million to Keith Kantrowitz and</t>
+          <t>Piece of Cake Moving &amp; Storage through the entity Skillman 3302 LLC paid $18 million</t>
         </is>
       </c>
       <c r="D6" t="inlineStr"/>
@@ -636,24 +636,24 @@
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>Top Story Transfers 1295 Madison Avenue (Credit - Cyclomedia) Imperial Sterling through the entity Imperial Madison, LLC paid $13 million to Keith Kantrowitz and musician Ryan Tedder‘s Patriot Real Estate Holdings through the entity MRK Jacksonville, LLC for the retail condo at 1295 Madison Avenue in Carnegie Hill, Manhattan. The expected use is cash flowing. The deal closed on June 11, 2026 and was recorded on June 23, 2026. The property has 3,024 square feet of built space according to a PincusCo analysis of city data. The sale price per built square foot is $4,298 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) The seller bought the property on November 9, 2023, for $11 million. The signatory for Keith Kantrowitz and Patriot Real Estate Holdings was Nelson Braff and Keith Kantrowitz. The signatory for Imperial Sterling was Jerrold G. Levy . The contract date was March 24, 2026. Prior sales, articles and revenue Prior to this transaction, PincusCo has records that the buyer Imperial Sterling purchased two properties in two transactions for a tota</t>
+          <t>Transfers 33-02 Skillman Avenue (Credit - Cyclomedia) Piece of Cake Moving &amp; Storage through the entity Skillman 3302 LLC paid $18 million to First Pioneer Properties through the entity Skillman Avenue Corp. for the office building (O5) at 33-02 Skillman Avenue in Long Island City, Queens. The expected use is owner-occupied. The deal closed on June 5, 2026 and was recorded on June 24, 2026. The property has 89,315 square feet of built space according to a PincusCo analysis of city data. The sale price per built square foot is $201 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) The signatory for First Pioneer Properties was Suresh Sani . The contract date was February 27, 2026. Prior sales, articles and revenue Prior to this transaction, PincusCo has records that the buyer Piece Of Cake Moving &amp; Storage purchased one property in one transaction for a total of $12 million and has no record it sold any properties over the past 24 months. The seller First Pioneer Properties had not purchased any other properties and had not sold any properties over th</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Jacob Kohn pays $5M to Cycamore Capital for mixed-use in Bedford Stuyvesant</t>
+          <t>Mendel Fleischman pays $9.2M for 24-unit dev site in East Williamsburg</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>https://www.pincusco.com/jacob-kohn-pays-5m-to-cycamore-capital-for-mixed-use-in-bedford-stuyvesant/</t>
+          <t>https://www.pincusco.com/mendel-fleischman-pays-9-2m-for-24-unit-dev-site-in-east-williamsburg/</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Jacob Kohn through the entity Myrtle Kent Development LLC paid $5 million to Cycamore Capital</t>
+          <t>Mendel Fleischman paid $9.2 million to Salvatore Gargano for a development site in East Williamsburg,</t>
         </is>
       </c>
       <c r="D7" t="inlineStr"/>
@@ -670,24 +670,24 @@
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t xml:space="preserve">Transfers 620 Myrtle Avenue (Credit - Cyclomedia) Jacob Kohn through the entity Myrtle Kent Development LLC paid $5 million to Cycamore Capital through the entity 620 Myrtle Avenue, LLC for the four-unit mixed-use building (S4) at 620 Myrtle Avenue in Bedford Stuyvesant, Brooklyn. The deal closed on June 3, 2026 and was recorded on June 23, 2026. The property has 5,625 square feet of built space and 5,560 square feet of additional air rights for a total buildable of 11,176 square feet according to a PincusCo analysis of city data. The sale price per built square foot is $888 and the price per buildable square foot is $447 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) The seller bought the property on November 14, 2019, for $3.1 million. The signatory for Cycamore Capital was Kenneth P. Horowitz . The signatory for Jacob Kohn was Jacob Kohn. The contract date was May 1, 2025. PincusCo analysis indicates this Jacob Kohn is not the same individual with the same name at Jay Group. Prior sales, articles and revenue Prior to this transaction, PincusCo </t>
+          <t>Transfers 241 Conselyea Street axonometric diagram (Credit Nickolas Kazalas architect via DOB) Mendel Fleischman paid $9.2 million to Salvatore Gargano for a development site in East Williamsburg, Brooklyn, in two transactions with the same seller. On the lot, there is one active new building construction project, B00497676, for a 24-unit, 18,255 square-foot R-2 building. The project was submitted by Salvatore Gargano with plans filed June 3, 2021 and permitted January 26, 2024. In the first, Mendel Fleischman through the entity 239 Garden LLC paid $4.6 million to Salvatore Gargano through the entity 239 Conselyea LLC for the development parcel (V0) at 239 Conselyea Street in East Williamsburg, Brooklyn. The expected use is ground up development. The deal closed on June 11, 2026 and was recorded on June 24, 2026. The property has zero square feet of built space and 7,458 square feet of additional air rights for a total buildable of 7,458 square feet according to a PincusCo analysis of city data. The sale price per buildable square foot is $616 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Andras Fenyves pays $2.9M for mixed-use in Bedford Stuyvesant</t>
+          <t>Makkos Equities pays $7M to Birchwood Properties for 11-unit walkup in Yorkville</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>https://www.pincusco.com/andras-fenyves-pays-2-9m-for-mixed-use-in-bedford-stuyvesant/</t>
+          <t>https://www.pincusco.com/makkos-equities-pays-7m-to-birchwood-properties-for-11-unit-walkup-in-yorkville/</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Andras Fenyves through the entity 1276 Broadway LLC paid $2.9 million to Joseph Felix through</t>
+          <t>Makkos Equities through the entity 67-65 Greene Street, LLC paid $7 million to Birchwood Properties</t>
         </is>
       </c>
       <c r="D8" t="inlineStr"/>
@@ -704,24 +704,24 @@
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>Transfers 1276 Broadway (Credit - Cyclomedia) Andras Fenyves through the entity 1276 Broadway LLC paid $2.9 million to Joseph Felix through the entity Triangle Square Corp. for the two-unit mixed-use building (S9) at 1276 Broadway in Bedford Stuyvesant, Brooklyn. The expected use is cash flowing. The deal closed on June 10, 2026 and was recorded on June 22, 2026. The property has 4,626 square feet of built space and 7,301 square feet of additional air rights for a total buildable of 11,920 square feet according to a PincusCo analysis of city data. The sale price per built square foot is $626 and the price per buildable square foot is $243 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) The signatory for Joseph Felix was Joseph Felix. The signatory for Andras Fenyves was Andras Fenyves. The contract date was January 12, 2026. Prior sales, articles and revenue Prior to this transaction, PincusCo has no record that the buyer Andras Fenyves had purchased any other properties and has no record it sold any properties over the past 24 months. The seller J</t>
+          <t>Transfers 1594 York Avenue (Credit - Cyclomedia) Makkos Equities through the entity 67-65 Greene Street, LLC paid $7 million to Birchwood Properties through the entity York 84 LLC for the 11-unit residential walkup building (C7) at 1594 York Avenue in Yorkville, Manhattan. The expected use is cash flowing. The deal closed on June 16, 2026 and was recorded on June 24, 2026. The property has 11,650 square feet of built space and 12,838 square feet of additional air rights for a total buildable of 24,500 square feet according to a PincusCo analysis of city data. The sale price per built square foot is $605 and the price per buildable square foot is $287 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) The signatory for Birchwood Properties was Robert Spitalnick . The signatory for Makkos Equities was George Makkos . The contract date was April 16, 2026. Prior sales, articles and revenue Prior to this transaction, PincusCo has no record that the buyer Makkos Equities had purchased any other properties and sold two properties in one transaction for a tot</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Westbridge Realty Group files plans for 72 units in Washington Heights</t>
+          <t>CareRite Centers pays $58.2M to Grand Healthcare for nursing facility in Whitestone</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>https://www.pincusco.com/westbridge-realty-group-files-plans-for-72-units-in-washington-heights/</t>
+          <t>https://www.pincusco.com/carerite-centers-pays-58-2m-to-grand-healthcare-for-two-properties-in-whitestone/</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Westbridge Realty Group submitted a new building construction project for a 72-unit, 56,615-square-foot residential (R-2)</t>
+          <t>CareRite Centers through the entity Forbes Ventures LLC paid $58.2 million to Grand Healthcare through</t>
         </is>
       </c>
       <c r="D9" t="inlineStr"/>
@@ -738,7 +738,7 @@
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>Development Rendering of 671 West 187th Street, with an alternate address of 673 West 187th Street (Credit - Leandro Nils Dickson architect via DOB) Westbridge Realty Group submitted a new building construction project for a 72-unit, 56,615-square-foot residential (R-2) building at 671 West 187th Street, with an alternate address of 673 West 187th Street, in Washington Heights, Manhattan. The plan was filed on June 19, 2026. It calls for the construction of a 155-foot-tall, sixteen-story building and was filed with the New York City Department of Buildings under job number M01417673. The project is described in the filing as: development hub job by default; as project is greater than seven (7) stories, per service notice posted april 16, 2021 such jobs shall be assigned to the development hub unit – subject building is a sixteen story building.. The applicant is the Registered Architect Leandro Dickson of Leandro Nils Dickson Architect. Steven Westreich of Westbridge Realty Group submitted the plans. The building does not have any retail or commercial space. 673 West 187th Street The neighborhood</t>
+          <t>Transfers 157-15 19th Avenue (Credit - Cyclomedia) CareRite Centers through the entity Forbes Ventures LLC paid $58.2 million to Grand Healthcare through the entity Clearview Land LLC for the Grand Rehabilitation and Nursing at Queens specialty building (I6) at 157-15 19th Avenue in Whitestone, Queens and a parking lot (G7) across the street on 19th Avenue. The expected use is cash flowing. The deal closed on April 28, 2026 and was recorded on June 24, 2026. The two properties have 47,000 square feet of built space and 10,169 square feet of additional air rights according to a PincusCo analysis of city data. The sale price per built square foot is $1,237 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) The signatory for Grand Healthcare was Jeremy B. Strauss . The signatory for CareRite Centers was Mark Friedman . The contract date was February 1, 2026. Because multiple properties have been transacted, some of the following sections will follow the property with the largest assessed value, which in this case, is the property on 157-15 19th Avenue. P</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto update queens news 2026-06-26T14:45:27Z
</commit_message>
<xml_diff>
--- a/data/output/queens_dev_news.xlsx
+++ b/data/output/queens_dev_news.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H9"/>
+  <dimension ref="A1:H7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -473,17 +473,17 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Sackman Enterprises, John Pearson pay $2.1M for 5-unit walkup in Harlem</t>
+          <t>Loketch Group signs $22.6M construction loan with iCross for 17-unit project in Fort Greene</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>https://www.pincusco.com/sackman-enterprises-john-pearson-pays-2-1m-for-5-unit-walkup-in-harlem/</t>
+          <t>https://www.pincusco.com/loketch-group-signs-22-6m-construction-loan-with-icross-for-17-unit-project-in-fort-greene/</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Sackman Enterprises and John Pearson through the entity Grace Church Community Redevelopment LLC paid $2.1</t>
+          <t>Loketch Group through the entity 158 Oxford LLC as borrower signed a new construction loan</t>
         </is>
       </c>
       <c r="D2" t="inlineStr"/>
@@ -500,24 +500,24 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>Transfers 314 West 139th Street (Credit - Cyclomedia) Sackman Enterprises and John Pearson through the entity Grace Church Community Redevelopment LLC paid $2.1 million to Grace Congregational Church of Harlem through the entity Grace Congregational Church Of Harlem, Inc. for the five-unit residential walkup building (C2) at 314 West 139th Street in Harlem, Manhattan. The expected use is cash flowing. The deal closed on June 12, 2026 and was recorded on June 23, 2026. The property has 4,280 square feet of built space and 1,906 square feet of additional air rights for a total buildable of 6,188 square feet according to a PincusCo analysis of city data. The sale price per built square foot is $490 and the price per buildable square foot is $339 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) The signatory for Grace Congregational Church of Harlem was Nigel Pearce. The signatory for Sackman Enterprises and John Pearson was Alan Sackman . The contract date was January 17, 2020. John Pearson owns have and Sackman owns half. Crain’s reported previously o</t>
+          <t>Transfers 158 South Oxford Street (Credit - Cyclomedia) Loketch Group through the entity 158 Oxford LLC as borrower signed a new construction loan with lender iCross Capital through the entity Elite 105 LLC valued at $22.6 million for the two-unit 1-4 family building (B3) at 158 South Oxford Street in Fort Greene, Brooklyn. On the lot, there is one active new building construction project, B01329666, for a 17-unit, 22,947 square-foot residential (R-2) building. The project was submitted by Borough Developers and filed by Shimon Kleinman with plans filed December 18, 2025 and it has not been permitted yet. The deal closed on June 4, 2026 and was recorded on June 24, 2026. The property has 5,400 square feet of built space and 17,595 square feet of additional air rights for a total buildable of 23,000 square feet according to a PincusCo analysis of city data. The loan price per built square foot is $4,185 and the price per buildable square foot is $982 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) The owner bought the property on June 4, 2026, for $</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Poise Property Group signs $16.2M construction loan for 20-unit dev site in Greenpoint</t>
+          <t>Menacham Harfenes files plans for 80 units in Longwood</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>https://www.pincusco.com/poise-property-group-signs-16-2m-construction-loan-for-20-unit-dev-site-in-greenpoint/</t>
+          <t>https://www.pincusco.com/menacham-harfenes-files-plans-for-80-units-in-longwood/</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Poise Property Group through the entity 55 Eckford St LLC as borrower signed a initial</t>
+          <t>Menacham Harfenes submitted a new building construction project for an 80-unit, 69,543-square-foot residential (R-2) building</t>
         </is>
       </c>
       <c r="D3" t="inlineStr"/>
@@ -534,24 +534,24 @@
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Transfers 55 Eckford Street axonometric diagram (Credit - Murat Mutlu architect via DOB) Poise Property Group through the entity 55 Eckford St LLC as borrower signed a initial loan with lender Colorado Federal Savings Bank through the entity Colorado Federalsavings Bank valued at $16.2 million for the 26-unit development building (V1) at 55 Eckford Street in Greenpoint, Brooklyn. On the lot, there is one active new building construction project, B01167721, for a 20-unit, 22,406 square-foot residential (R-2) building. The project was submitted by Poise Property Group and filed by Daniel Kaykov with plans filed January 27, 2025 and permitted November 21, 2025. The deal closed on May 21, 2026 and was recorded on June 23, 2026. The property has 42,449 square feet of built space and 20,752 square feet of additional air rights according to a PincusCo analysis of city data. The loan price per built square foot is $381 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) The owner bought the property on April 24, 2024, for $7.2 million. The signatory for Poise </t>
+          <t>Development 895 Reverend James A Polite Avenue rendering (Credit - Nikolai Katz architect via DOB) Menacham Harfenes submitted a new building construction project for an 80-unit, 69,543-square-foot residential (R-2) building at 895 Reverend James A Polite Avenue in Longwood, Bronx. The plan was filed on June 24, 2026. It calls for the construction of a 74-foot-tall, seven-story building and was filed with the New York City Department of Buildings under job number X01410192. The project is described in the filing as: proposed new 7 story residential building. The applicant is the Registered Architect Nikolai Katz of Nikolai Katz Architect . 895 Reverend James A Polite Avenue The neighborhood In Longwood, The bulk, or 44 percent of the 22.3 million square feet of commercial built space are elevator buildings, with walkup buildings next occupying 27 percent of the space. In sales, Longwood has near average sales volume among other neighborhoods with $110.1 million in sales volume in the last two years and is the 12th highest in Bronx. For development, Longwood has near average amount of major developments among other neighborhoods and is the 2nd highest in Bronx. It had 3.7 million sq</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Lonicera Partners signs $150M loan with PNC for 314-unit rental in Downtown Brooklyn</t>
+          <t>JPMorgan Chase takes title to retail in Chelsea, $38.2M transfer value</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>https://www.pincusco.com/lonicera-partners-signs-150m-loan-with-pnc-for-314-unit-rental-in-downtown-brooklyn/</t>
+          <t>https://www.pincusco.com/jpmorgan-chase-takes-title-to-retail-in-chelsea-38-2m-transfer-value/</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Lonicera Partners through the entity Hanover Tower Owner LLC as borrower signed a loan with</t>
+          <t>JPMorgan Chase through the entity MW Tolero Holding Corp. acquired through bankruptcy with a credit</t>
         </is>
       </c>
       <c r="D4" t="inlineStr"/>
@@ -568,24 +568,24 @@
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>Transfers 15 Hanover Place (Credit - Cyclomedia) Lonicera Partners through the entity Hanover Tower Owner LLC as borrower signed a loan with lender PNC Bank through the entity Pnc Bank, National Association valued at $150 million for the 314-unit residential elevator building (D6) at 15 Hanover Place in Downtown Brooklyn, Brooklyn. The deal closed on June 16, 2026 and was recorded on June 23, 2026. The prior lender was Santander Bank which held debt that had an original loan amount of $134 million. The property has 281,511 square feet of built space according to a PincusCo analysis of city data. The loan price per built square foot is $532 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) The signatory for Lonicera Partners was Jamie Anthony . The signatory for PNC Bank was Heather Finnegan . Prior sales, articles and revenue The owners according to the Department of Housing Preservation and Development includes Lucian Cohen, head officer and Wilson Acosta, agent. The business entities are Rose Property Mgmt Grp Llc and Hanover Tower Owner Llc. The 2</t>
+          <t>Transfers 547 West 27th Street (Credit - Cyclomedia) JPMorgan Chase through the entity MW Tolero Holding Corp. acquired through bankruptcy with a credit bid as the former lender the retail building (K2) at 547 West 27th Street in Chelsea, Manhattan. The expected use is hold for sale. The transfer price in city records was $38.2 million. The former owner, the debtor, was James Pastreich’s Pinetree Group through the entity Mariners Gate, LLC. The transfer closed on June 18, 2026 and was recorded on June 25, 2026. The property has 97,200 square feet of built space and 32,649 square feet of additional air rights for a total buildable of 129,908 square feet according to a PincusCo analysis of city data. The sale price per built square foot is $393 and the price per buildable square foot is $294 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) The signatory for Pinetree Group was James Y.A. Pastreich. The signatory for JPMorgan Chase was Andrew Bergman . The contract date was June 18, 2026. PincusCo reported on a scheduled foreclosure auction. Pastreich p</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>LBA Realty signs $22.8M refi loan with City National Bank for three properties in Red Hook</t>
+          <t>Blue Light Capital pays $61.2M for three Greenwich Village retail condos in foreclosure</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>https://www.pincusco.com/lba-realty-signs-22-8m-refi-loan-with-city-national-bank-for-three-properties-in-red-hook/</t>
+          <t>https://www.pincusco.com/blue-light-capital-pays-61-2m-for-three-retail-properties-in-greenwich-village-in-foreclosure/</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>LBA Realty through the entity 110 Beard Street, LLC as borrower signed a refi loan</t>
+          <t>Blue Light Capital through the entity BL East 8th Street LLC paid $61.2 million through</t>
         </is>
       </c>
       <c r="D5" t="inlineStr"/>
@@ -602,24 +602,24 @@
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>Transfers 236 Richards Street, 110 Beard Street (Credit - Cyclomedia) LBA Realty through the entity 110 Beard Street, LLC as borrower signed a refi loan with lender City National Bank through the entity City National Bank valued at $22.8 million for three properties including the industrial building (E1) at 236 Richards Street in Red Hook, Brooklyn, industrial building (E1) at 118 Beard Street in Red Hook, Brooklyn, and hotel building (H8) at 116 Beard Street in Red Hook, Brooklyn. The deal closed on May 29, 2026 and was recorded on June 23, 2026. The prior lender was City National Bank which held debt that had an original loan amount of $22.8 million.The three properties have 97,130 square feet of built space and 96,636 square feet of additional air rights for a total buildable of 193,800 square feet according to a PincusCo analysis of city data. The loan price per built square foot is $234 and the price per buildable square foot is $117 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) The signatory for LBA Realty was Michael Memoly . The signatory</t>
+          <t>Top Story Transfers 21 University Place (Credit - Cyclomedia) Blue Light Capital through the entity BL East 8th Street LLC paid $61.2 million through a judicial foreclosure for three retail condominium units at 60 East 9th Street, 21 University Place and 40 East 9th Street in Greenwich Village, Manhattan. The expected use is cash flowing. The former owner was an entity in care of Rose Associates, which lost the properties in the foreclosure action, 850412/2025, that Voya Financial brought in 2025 alleging a $60 million loan was in default. At the time, a spokesperson for Rose Associates said in an email, “Rose Associates doesn’t own that property and is not a party to the loan foreclosure.” The deal closed on June 17, 2026 and was recorded on June 25, 2026. The three properties have 115,476 square feet of built space according to a PincusCo analysis of city data. The sale price per built square foot is $529 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) The signatory for Blue Light Capital , which includes Greg Manocherian as an investor, was Scot</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Moving company pays $18M to First Pioneer for office in LIC</t>
+          <t>Neel Dvivedi pays $9.85M to AMCC Corp. for dev site in Long Island City</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>https://www.pincusco.com/moving-company-pays-18m-to-first-pioneer-for-office-in-lic/</t>
+          <t>https://www.pincusco.com/neel-dvivedi-pays-9-85m-to-amcc-corp-for-industrial-in-long-island-city/</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Piece of Cake Moving &amp; Storage through the entity Skillman 3302 LLC paid $18 million</t>
+          <t>Neel Dvivedi paid $9.85 million to AMCC Corp. for a two-parcel development site in Long</t>
         </is>
       </c>
       <c r="D6" t="inlineStr"/>
@@ -636,24 +636,24 @@
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>Transfers 33-02 Skillman Avenue (Credit - Cyclomedia) Piece of Cake Moving &amp; Storage through the entity Skillman 3302 LLC paid $18 million to First Pioneer Properties through the entity Skillman Avenue Corp. for the office building (O5) at 33-02 Skillman Avenue in Long Island City, Queens. The expected use is owner-occupied. The deal closed on June 5, 2026 and was recorded on June 24, 2026. The property has 89,315 square feet of built space according to a PincusCo analysis of city data. The sale price per built square foot is $201 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) The signatory for First Pioneer Properties was Suresh Sani . The contract date was February 27, 2026. Prior sales, articles and revenue Prior to this transaction, PincusCo has records that the buyer Piece Of Cake Moving &amp; Storage purchased one property in one transaction for a total of $12 million and has no record it sold any properties over the past 24 months. The seller First Pioneer Properties had not purchased any other properties and had not sold any properties over th</t>
+          <t>Chart_Frontpage Transfers 50-16 Vernon Boulevard (Credit - Cyclomedia) Neel Dvivedi paid $9.85 million to AMCC Corp. for a two-parcel development site in Long Island City, Queens, in two transactions. New York City Department of Buildings applications have been filed to demolish both buildings. In the first, Neel Dvivedi through the entity Op Vernon LLC paid $5.95 million to AMCC Corp. through the entity 50-18 Realty Corp. for the industrial building (E2) at 50-16 Vernon Boulevard in Long Island City, Queens. The deal closed on June 17, 2026 and was recorded on June 25, 2026. The property has 10,000 square feet of built space and 5,000 square feet of additional air rights for a total buildable of 15,000 square feet according to a PincusCo analysis of city data. The sale price per built square foot is $590 and the price per buildable square foot is $393 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) In the second, Neel Dvivedi through the entity Op Vernon LLC paid $3.9 million to AMCC Corp. through the entity 5014 Vernon Realty LLC for the two-unit</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Mendel Fleischman pays $9.2M for 24-unit dev site in East Williamsburg</t>
+          <t>Jane Capital pays $4.1M for 7-unit walkup in Bushwick</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>https://www.pincusco.com/mendel-fleischman-pays-9-2m-for-24-unit-dev-site-in-east-williamsburg/</t>
+          <t>https://www.pincusco.com/jane-capital-pays-4-1m-for-7-unit-walkup-in-bushwick/</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Mendel Fleischman paid $9.2 million to Salvatore Gargano for a development site in East Williamsburg,</t>
+          <t>Jane Capital through the entity 247 Starr LLC paid $4.1 million to Todor Sfera through</t>
         </is>
       </c>
       <c r="D7" t="inlineStr"/>
@@ -670,75 +670,7 @@
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>Transfers 241 Conselyea Street axonometric diagram (Credit Nickolas Kazalas architect via DOB) Mendel Fleischman paid $9.2 million to Salvatore Gargano for a development site in East Williamsburg, Brooklyn, in two transactions with the same seller. On the lot, there is one active new building construction project, B00497676, for a 24-unit, 18,255 square-foot R-2 building. The project was submitted by Salvatore Gargano with plans filed June 3, 2021 and permitted January 26, 2024. In the first, Mendel Fleischman through the entity 239 Garden LLC paid $4.6 million to Salvatore Gargano through the entity 239 Conselyea LLC for the development parcel (V0) at 239 Conselyea Street in East Williamsburg, Brooklyn. The expected use is ground up development. The deal closed on June 11, 2026 and was recorded on June 24, 2026. The property has zero square feet of built space and 7,458 square feet of additional air rights for a total buildable of 7,458 square feet according to a PincusCo analysis of city data. The sale price per buildable square foot is $616 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>Makkos Equities pays $7M to Birchwood Properties for 11-unit walkup in Yorkville</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>https://www.pincusco.com/makkos-equities-pays-7m-to-birchwood-properties-for-11-unit-walkup-in-yorkville/</t>
-        </is>
-      </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>Makkos Equities through the entity 67-65 Greene Street, LLC paid $7 million to Birchwood Properties</t>
-        </is>
-      </c>
-      <c r="D8" t="inlineStr"/>
-      <c r="E8" t="inlineStr"/>
-      <c r="F8" t="inlineStr">
-        <is>
-          <t>PincusCo</t>
-        </is>
-      </c>
-      <c r="G8" t="inlineStr">
-        <is>
-          <t>PincusCo - Home</t>
-        </is>
-      </c>
-      <c r="H8" t="inlineStr">
-        <is>
-          <t>Transfers 1594 York Avenue (Credit - Cyclomedia) Makkos Equities through the entity 67-65 Greene Street, LLC paid $7 million to Birchwood Properties through the entity York 84 LLC for the 11-unit residential walkup building (C7) at 1594 York Avenue in Yorkville, Manhattan. The expected use is cash flowing. The deal closed on June 16, 2026 and was recorded on June 24, 2026. The property has 11,650 square feet of built space and 12,838 square feet of additional air rights for a total buildable of 24,500 square feet according to a PincusCo analysis of city data. The sale price per built square foot is $605 and the price per buildable square foot is $287 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) The signatory for Birchwood Properties was Robert Spitalnick . The signatory for Makkos Equities was George Makkos . The contract date was April 16, 2026. Prior sales, articles and revenue Prior to this transaction, PincusCo has no record that the buyer Makkos Equities had purchased any other properties and sold two properties in one transaction for a tot</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>CareRite Centers pays $58.2M to Grand Healthcare for nursing facility in Whitestone</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>https://www.pincusco.com/carerite-centers-pays-58-2m-to-grand-healthcare-for-two-properties-in-whitestone/</t>
-        </is>
-      </c>
-      <c r="C9" t="inlineStr">
-        <is>
-          <t>CareRite Centers through the entity Forbes Ventures LLC paid $58.2 million to Grand Healthcare through</t>
-        </is>
-      </c>
-      <c r="D9" t="inlineStr"/>
-      <c r="E9" t="inlineStr"/>
-      <c r="F9" t="inlineStr">
-        <is>
-          <t>PincusCo</t>
-        </is>
-      </c>
-      <c r="G9" t="inlineStr">
-        <is>
-          <t>PincusCo - Home</t>
-        </is>
-      </c>
-      <c r="H9" t="inlineStr">
-        <is>
-          <t>Transfers 157-15 19th Avenue (Credit - Cyclomedia) CareRite Centers through the entity Forbes Ventures LLC paid $58.2 million to Grand Healthcare through the entity Clearview Land LLC for the Grand Rehabilitation and Nursing at Queens specialty building (I6) at 157-15 19th Avenue in Whitestone, Queens and a parking lot (G7) across the street on 19th Avenue. The expected use is cash flowing. The deal closed on April 28, 2026 and was recorded on June 24, 2026. The two properties have 47,000 square feet of built space and 10,169 square feet of additional air rights according to a PincusCo analysis of city data. The sale price per built square foot is $1,237 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) The signatory for Grand Healthcare was Jeremy B. Strauss . The signatory for CareRite Centers was Mark Friedman . The contract date was February 1, 2026. Because multiple properties have been transacted, some of the following sections will follow the property with the largest assessed value, which in this case, is the property on 157-15 19th Avenue. P</t>
+          <t>Transfers 247 Starr Street (Credit - Cyclomedia) Jane Capital through the entity 247 Starr LLC paid $4.1 million to Todor Sfera through the entity 247 Starr Street, Inc for the seven-unit residential walkup building (C7) at 247 Starr Street in Bushwick, Brooklyn. The expected use is cash flowing. The deal closed on June 2, 2026 and was recorded on June 25, 2026. The property has 7,500 square feet of built space according to a PincusCo analysis of city data. The sale price per built square foot is $546 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) The seller bought the property on August 9, 2005, for $700,000. The signatory for Todor Sfera was Todor Sfera. The signatory for Jane Capital was Laurent Wendum . The contract date was April 6, 2026. Prior sales, articles and revenue Prior to this transaction, PincusCo has records that the buyer Jane Capital purchased one property in one transaction for a total of $2.8 million and has no record it sold any properties over the past 24 months. The seller Todor Sfera had not purchased any other properties a</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto update queens news 2026-06-27T14:04:42Z
</commit_message>
<xml_diff>
--- a/data/output/queens_dev_news.xlsx
+++ b/data/output/queens_dev_news.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H7"/>
+  <dimension ref="A1:H1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -467,210 +467,6 @@
       <c r="H1" s="1" t="inlineStr">
         <is>
           <t>content_preview</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>Loketch Group signs $22.6M construction loan with iCross for 17-unit project in Fort Greene</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>https://www.pincusco.com/loketch-group-signs-22-6m-construction-loan-with-icross-for-17-unit-project-in-fort-greene/</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>Loketch Group through the entity 158 Oxford LLC as borrower signed a new construction loan</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr"/>
-      <c r="E2" t="inlineStr"/>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t>PincusCo</t>
-        </is>
-      </c>
-      <c r="G2" t="inlineStr">
-        <is>
-          <t>PincusCo - Home</t>
-        </is>
-      </c>
-      <c r="H2" t="inlineStr">
-        <is>
-          <t>Transfers 158 South Oxford Street (Credit - Cyclomedia) Loketch Group through the entity 158 Oxford LLC as borrower signed a new construction loan with lender iCross Capital through the entity Elite 105 LLC valued at $22.6 million for the two-unit 1-4 family building (B3) at 158 South Oxford Street in Fort Greene, Brooklyn. On the lot, there is one active new building construction project, B01329666, for a 17-unit, 22,947 square-foot residential (R-2) building. The project was submitted by Borough Developers and filed by Shimon Kleinman with plans filed December 18, 2025 and it has not been permitted yet. The deal closed on June 4, 2026 and was recorded on June 24, 2026. The property has 5,400 square feet of built space and 17,595 square feet of additional air rights for a total buildable of 23,000 square feet according to a PincusCo analysis of city data. The loan price per built square foot is $4,185 and the price per buildable square foot is $982 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) The owner bought the property on June 4, 2026, for $</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>Menacham Harfenes files plans for 80 units in Longwood</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>https://www.pincusco.com/menacham-harfenes-files-plans-for-80-units-in-longwood/</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>Menacham Harfenes submitted a new building construction project for an 80-unit, 69,543-square-foot residential (R-2) building</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr"/>
-      <c r="E3" t="inlineStr"/>
-      <c r="F3" t="inlineStr">
-        <is>
-          <t>PincusCo</t>
-        </is>
-      </c>
-      <c r="G3" t="inlineStr">
-        <is>
-          <t>PincusCo - Home</t>
-        </is>
-      </c>
-      <c r="H3" t="inlineStr">
-        <is>
-          <t>Development 895 Reverend James A Polite Avenue rendering (Credit - Nikolai Katz architect via DOB) Menacham Harfenes submitted a new building construction project for an 80-unit, 69,543-square-foot residential (R-2) building at 895 Reverend James A Polite Avenue in Longwood, Bronx. The plan was filed on June 24, 2026. It calls for the construction of a 74-foot-tall, seven-story building and was filed with the New York City Department of Buildings under job number X01410192. The project is described in the filing as: proposed new 7 story residential building. The applicant is the Registered Architect Nikolai Katz of Nikolai Katz Architect . 895 Reverend James A Polite Avenue The neighborhood In Longwood, The bulk, or 44 percent of the 22.3 million square feet of commercial built space are elevator buildings, with walkup buildings next occupying 27 percent of the space. In sales, Longwood has near average sales volume among other neighborhoods with $110.1 million in sales volume in the last two years and is the 12th highest in Bronx. For development, Longwood has near average amount of major developments among other neighborhoods and is the 2nd highest in Bronx. It had 3.7 million sq</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>JPMorgan Chase takes title to retail in Chelsea, $38.2M transfer value</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>https://www.pincusco.com/jpmorgan-chase-takes-title-to-retail-in-chelsea-38-2m-transfer-value/</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>JPMorgan Chase through the entity MW Tolero Holding Corp. acquired through bankruptcy with a credit</t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr"/>
-      <c r="E4" t="inlineStr"/>
-      <c r="F4" t="inlineStr">
-        <is>
-          <t>PincusCo</t>
-        </is>
-      </c>
-      <c r="G4" t="inlineStr">
-        <is>
-          <t>PincusCo - Home</t>
-        </is>
-      </c>
-      <c r="H4" t="inlineStr">
-        <is>
-          <t>Transfers 547 West 27th Street (Credit - Cyclomedia) JPMorgan Chase through the entity MW Tolero Holding Corp. acquired through bankruptcy with a credit bid as the former lender the retail building (K2) at 547 West 27th Street in Chelsea, Manhattan. The expected use is hold for sale. The transfer price in city records was $38.2 million. The former owner, the debtor, was James Pastreich’s Pinetree Group through the entity Mariners Gate, LLC. The transfer closed on June 18, 2026 and was recorded on June 25, 2026. The property has 97,200 square feet of built space and 32,649 square feet of additional air rights for a total buildable of 129,908 square feet according to a PincusCo analysis of city data. The sale price per built square foot is $393 and the price per buildable square foot is $294 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) The signatory for Pinetree Group was James Y.A. Pastreich. The signatory for JPMorgan Chase was Andrew Bergman . The contract date was June 18, 2026. PincusCo reported on a scheduled foreclosure auction. Pastreich p</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>Blue Light Capital pays $61.2M for three Greenwich Village retail condos in foreclosure</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>https://www.pincusco.com/blue-light-capital-pays-61-2m-for-three-retail-properties-in-greenwich-village-in-foreclosure/</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>Blue Light Capital through the entity BL East 8th Street LLC paid $61.2 million through</t>
-        </is>
-      </c>
-      <c r="D5" t="inlineStr"/>
-      <c r="E5" t="inlineStr"/>
-      <c r="F5" t="inlineStr">
-        <is>
-          <t>PincusCo</t>
-        </is>
-      </c>
-      <c r="G5" t="inlineStr">
-        <is>
-          <t>PincusCo - Home</t>
-        </is>
-      </c>
-      <c r="H5" t="inlineStr">
-        <is>
-          <t>Top Story Transfers 21 University Place (Credit - Cyclomedia) Blue Light Capital through the entity BL East 8th Street LLC paid $61.2 million through a judicial foreclosure for three retail condominium units at 60 East 9th Street, 21 University Place and 40 East 9th Street in Greenwich Village, Manhattan. The expected use is cash flowing. The former owner was an entity in care of Rose Associates, which lost the properties in the foreclosure action, 850412/2025, that Voya Financial brought in 2025 alleging a $60 million loan was in default. At the time, a spokesperson for Rose Associates said in an email, “Rose Associates doesn’t own that property and is not a party to the loan foreclosure.” The deal closed on June 17, 2026 and was recorded on June 25, 2026. The three properties have 115,476 square feet of built space according to a PincusCo analysis of city data. The sale price per built square foot is $529 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) The signatory for Blue Light Capital , which includes Greg Manocherian as an investor, was Scot</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>Neel Dvivedi pays $9.85M to AMCC Corp. for dev site in Long Island City</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>https://www.pincusco.com/neel-dvivedi-pays-9-85m-to-amcc-corp-for-industrial-in-long-island-city/</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>Neel Dvivedi paid $9.85 million to AMCC Corp. for a two-parcel development site in Long</t>
-        </is>
-      </c>
-      <c r="D6" t="inlineStr"/>
-      <c r="E6" t="inlineStr"/>
-      <c r="F6" t="inlineStr">
-        <is>
-          <t>PincusCo</t>
-        </is>
-      </c>
-      <c r="G6" t="inlineStr">
-        <is>
-          <t>PincusCo - Home</t>
-        </is>
-      </c>
-      <c r="H6" t="inlineStr">
-        <is>
-          <t>Chart_Frontpage Transfers 50-16 Vernon Boulevard (Credit - Cyclomedia) Neel Dvivedi paid $9.85 million to AMCC Corp. for a two-parcel development site in Long Island City, Queens, in two transactions. New York City Department of Buildings applications have been filed to demolish both buildings. In the first, Neel Dvivedi through the entity Op Vernon LLC paid $5.95 million to AMCC Corp. through the entity 50-18 Realty Corp. for the industrial building (E2) at 50-16 Vernon Boulevard in Long Island City, Queens. The deal closed on June 17, 2026 and was recorded on June 25, 2026. The property has 10,000 square feet of built space and 5,000 square feet of additional air rights for a total buildable of 15,000 square feet according to a PincusCo analysis of city data. The sale price per built square foot is $590 and the price per buildable square foot is $393 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) In the second, Neel Dvivedi through the entity Op Vernon LLC paid $3.9 million to AMCC Corp. through the entity 5014 Vernon Realty LLC for the two-unit</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>Jane Capital pays $4.1M for 7-unit walkup in Bushwick</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>https://www.pincusco.com/jane-capital-pays-4-1m-for-7-unit-walkup-in-bushwick/</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>Jane Capital through the entity 247 Starr LLC paid $4.1 million to Todor Sfera through</t>
-        </is>
-      </c>
-      <c r="D7" t="inlineStr"/>
-      <c r="E7" t="inlineStr"/>
-      <c r="F7" t="inlineStr">
-        <is>
-          <t>PincusCo</t>
-        </is>
-      </c>
-      <c r="G7" t="inlineStr">
-        <is>
-          <t>PincusCo - Home</t>
-        </is>
-      </c>
-      <c r="H7" t="inlineStr">
-        <is>
-          <t>Transfers 247 Starr Street (Credit - Cyclomedia) Jane Capital through the entity 247 Starr LLC paid $4.1 million to Todor Sfera through the entity 247 Starr Street, Inc for the seven-unit residential walkup building (C7) at 247 Starr Street in Bushwick, Brooklyn. The expected use is cash flowing. The deal closed on June 2, 2026 and was recorded on June 25, 2026. The property has 7,500 square feet of built space according to a PincusCo analysis of city data. The sale price per built square foot is $546 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) The seller bought the property on August 9, 2005, for $700,000. The signatory for Todor Sfera was Todor Sfera. The signatory for Jane Capital was Laurent Wendum . The contract date was April 6, 2026. Prior sales, articles and revenue Prior to this transaction, PincusCo has records that the buyer Jane Capital purchased one property in one transaction for a total of $2.8 million and has no record it sold any properties over the past 24 months. The seller Todor Sfera had not purchased any other properties a</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto update queens news 2026-07-01T15:10:09Z
</commit_message>
<xml_diff>
--- a/data/output/queens_dev_news.xlsx
+++ b/data/output/queens_dev_news.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H1"/>
+  <dimension ref="A1:H2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -467,6 +467,40 @@
       <c r="H1" s="1" t="inlineStr">
         <is>
           <t>content_preview</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Urban Realty Partners pays $45M for 415-unit dev site in Flushing</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>https://www.pincusco.com/urban-realty-partners-pays-45m-to-mar-mar-realty-for-415-unit-dev-site-in-flushing/</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Urban Realty Partners through the entity Whitestone Owner LLC paid $45 million to Mar Mar</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr"/>
+      <c r="E2" t="inlineStr"/>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>PincusCo</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>PincusCo - Home</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>Chart_Frontpage Transfers 30-05 Farrington Street illustrative rendering (Credit - Raymond Chan architect via DOB) Continue reading with a PincusCo subscription Sign up for a paid subscription to view this content. Already a subscriber? Log in here.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto update queens news 2026-07-02T14:26:54Z
</commit_message>
<xml_diff>
--- a/data/output/queens_dev_news.xlsx
+++ b/data/output/queens_dev_news.xlsx
@@ -473,34 +473,42 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Urban Realty Partners pays $45M for 415-unit dev site in Flushing</t>
+          <t>Permits Filed for 31-08 31st Avenue in Astoria, Queens</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>https://www.pincusco.com/urban-realty-partners-pays-45m-to-mar-mar-realty-for-415-unit-dev-site-in-flushing/</t>
+          <t>https://newyorkyimby.com/2026/07/permits-filed-for-31-08-31st-avenue-in-astoria-queens.html</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Urban Realty Partners through the entity Whitestone Owner LLC paid $45 million to Mar Mar</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr"/>
-      <c r="E2" t="inlineStr"/>
+          <t>Permits have been filed for a nine-story mixed-use building at 31-08 31st Avenue in &lt;a href="https://newyorkyimby.com/neighborhoods/astoria"&gt;Astoria&lt;/a&gt;, Queens. Located between 31st Street and 32nd Street, the lot is near the 30th Avenue subway station, served by the N and W trains. Zengwen Ye of Arch 31 LLC is listed as the owner behind the applications.</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>2026-07-02T10:30:12+00:00</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>Thu, 02 Jul 2026 10:30:12 +0000</t>
+        </is>
+      </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>PincusCo</t>
+          <t>YIMBY</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>PincusCo - Home</t>
+          <t>YIMBY - Astoria</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>Chart_Frontpage Transfers 30-05 Farrington Street illustrative rendering (Credit - Raymond Chan architect via DOB) Continue reading with a PincusCo subscription Sign up for a paid subscription to view this content. Already a subscriber? Log in here.</t>
+          <t>By: Vanessa Londono 6:30 am on July 2, 2026 Permits have been filed for a nine-story mixed-use building at 31-08 31st Avenue in Astoria, Queens. Located between 31st Street and 32nd Street, the lot is near the 30th Avenue subway station, served by the N and W trains. Zengwen Ye of Arch 31 LLC is listed as the owner behind the applications. The proposed 95-foot-tall development will yield 37,694 square feet, with 35,864 square feet designated for residential space, 1,441 square feet for commercial space, and 389 square feet for community facility space. The building will have 48 residences, most likely rentals based on the average unit scope of 747 square feet. The concrete-based structure will also have a cellar and a 31-foot-long rear yard. Chang Tan of Tan Architect P.C is listed as the architect of record. Demolition permits filed for the two-story structure on the site. An estimated completion date has not been announced. Subscribe to YIMBY’s daily e-mail Follow YIMBYgram for real-time photo updates Like YIMBY on Facebook Follow YIMBY’s Twitter for the latest in YIMBYnews</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto update queens news 2026-07-03T14:30:07Z
</commit_message>
<xml_diff>
--- a/data/output/queens_dev_news.xlsx
+++ b/data/output/queens_dev_news.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H2"/>
+  <dimension ref="A1:H1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -467,48 +467,6 @@
       <c r="H1" s="1" t="inlineStr">
         <is>
           <t>content_preview</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>Permits Filed for 31-08 31st Avenue in Astoria, Queens</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>https://newyorkyimby.com/2026/07/permits-filed-for-31-08-31st-avenue-in-astoria-queens.html</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>Permits have been filed for a nine-story mixed-use building at 31-08 31st Avenue in &lt;a href="https://newyorkyimby.com/neighborhoods/astoria"&gt;Astoria&lt;/a&gt;, Queens. Located between 31st Street and 32nd Street, the lot is near the 30th Avenue subway station, served by the N and W trains. Zengwen Ye of Arch 31 LLC is listed as the owner behind the applications.</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>2026-07-02T10:30:12+00:00</t>
-        </is>
-      </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>Thu, 02 Jul 2026 10:30:12 +0000</t>
-        </is>
-      </c>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t>YIMBY</t>
-        </is>
-      </c>
-      <c r="G2" t="inlineStr">
-        <is>
-          <t>YIMBY - Astoria</t>
-        </is>
-      </c>
-      <c r="H2" t="inlineStr">
-        <is>
-          <t>By: Vanessa Londono 6:30 am on July 2, 2026 Permits have been filed for a nine-story mixed-use building at 31-08 31st Avenue in Astoria, Queens. Located between 31st Street and 32nd Street, the lot is near the 30th Avenue subway station, served by the N and W trains. Zengwen Ye of Arch 31 LLC is listed as the owner behind the applications. The proposed 95-foot-tall development will yield 37,694 square feet, with 35,864 square feet designated for residential space, 1,441 square feet for commercial space, and 389 square feet for community facility space. The building will have 48 residences, most likely rentals based on the average unit scope of 747 square feet. The concrete-based structure will also have a cellar and a 31-foot-long rear yard. Chang Tan of Tan Architect P.C is listed as the architect of record. Demolition permits filed for the two-story structure on the site. An estimated completion date has not been announced. Subscribe to YIMBY’s daily e-mail Follow YIMBYgram for real-time photo updates Like YIMBY on Facebook Follow YIMBY’s Twitter for the latest in YIMBYnews</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto update queens news 2026-07-07T15:10:40Z
</commit_message>
<xml_diff>
--- a/data/output/queens_dev_news.xlsx
+++ b/data/output/queens_dev_news.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H1"/>
+  <dimension ref="A1:H3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -467,6 +467,86 @@
       <c r="H1" s="1" t="inlineStr">
         <is>
           <t>content_preview</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>99-Unit Project Remains on Hold at 43-42 43rd Street in Sunnyside, Queens</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>https://newyorkyimby.com/2026/07/99-unit-project-remains-on-hold-at-43-42-43rd-street-in-sunnyside-queens.html</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Construction is on hold at 43-42 43rd Street, the site of an eight-story mixed-use residential building in &lt;a href="https://newyorkyimby.com/category/sunnyside"&gt;Sunnyside&lt;/a&gt;, Queens. Designed by Gerald Caliendo Architects for John J. Ciafone of City View Construction Corp., the 79-foot-tall structure will span 73,762 square feet and yield 99 rental units with an average scope of 677 square feet. The project will also include 6,664 square feet of commercial space, two cellar levels, a 31-foot-long rear yard, and a 138-vehicle parking garage, according to permits filed in November 2021. The property is located at the northwest corner of 43rd Street and Roosevelt Avenue.</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>2026-07-07T11:00:58+00:00</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>Tue, 07 Jul 2026 11:00:58 +0000</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>YIMBY</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>YIMBY - Sunnyside</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>By: Michael Young and Matt Pruznick 7:00 am on July 7, 2026 Construction is on hold at 43-42 43rd Street, the site of an eight-story mixed-use residential building in Sunnyside, Queens. Designed by Gerald Caliendo Architects for John J. Ciafone of City View Construction Corp., the 79-foot-tall structure will span 73,762 square feet and yield 99 rental units with an average scope of 677 square feet. The project will also include 6,664 square feet of commercial space, two cellar levels, a 31-foot-long rear yard, and a 138-vehicle parking garage, according to permits filed in November 2021. The property is located at the northwest corner of 43rd Street and Roosevelt Avenue. The site sits partially unearthed behind the construction fencing. It’s unclear when work will resume on the project. 43-42 43rd Street. Photo by Michael Young. 43-42 43rd Street. Photo by Michael Young. 43-42 43rd Street. Photo by Michael Young.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Cheskel Salamon buys two buildings for $4M in Bedford Park, likely dev site</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>https://www.pincusco.com/cheskel-salamon-buys-two-buildings-for-4m-in-bedford-park-likely-dev-site/</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Cheskel Salamon paid $4.06 million for two adjacent buildings at 2814 and 2818 Morris Avenue</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>NaT</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr"/>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>PincusCo</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>PincusCo - Home</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>Transfers 2814 Morris Avenue (Credit - Cyclomedia) Cheskel Salamon paid $4.06 million for two adjacent buildings at 2814 and 2818 Morris Avenue in Bedford Park, the Bronx, that are likely to be demolished to make way for a new development. In the first, Cheskel Salamon through the entity 2814-2818 Morris Owner LLC paid $2.6 million to Martin Ortega for the three-unit building (C0) at 2814 Morris Avenue. The deal closed on June 17, 2026 and was recorded on July 2, 2026. The property has 5,253 square feet of built space and 23,433 square feet of additional air rights for a total buildable of 28,673 square feet according to a PincusCo analysis of city data. The sale price per built square foot is $494 and the price per buildable square foot is $90 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) The signatory for Martin Ortega was Martin Ortega. The signatory for Cheskel Salamon was Cheskel Salamon. The contract date was November 7, 2025. In the second, Cheskel Salamon through the entity 2814-2818 Morris Owner LLC paid $1.5 million to Bernardo Arias fo</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto update queens news 2026-07-08T14:37:40Z
</commit_message>
<xml_diff>
--- a/data/output/queens_dev_news.xlsx
+++ b/data/output/queens_dev_news.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H3"/>
+  <dimension ref="A1:H1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -467,86 +467,6 @@
       <c r="H1" s="1" t="inlineStr">
         <is>
           <t>content_preview</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>99-Unit Project Remains on Hold at 43-42 43rd Street in Sunnyside, Queens</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>https://newyorkyimby.com/2026/07/99-unit-project-remains-on-hold-at-43-42-43rd-street-in-sunnyside-queens.html</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>Construction is on hold at 43-42 43rd Street, the site of an eight-story mixed-use residential building in &lt;a href="https://newyorkyimby.com/category/sunnyside"&gt;Sunnyside&lt;/a&gt;, Queens. Designed by Gerald Caliendo Architects for John J. Ciafone of City View Construction Corp., the 79-foot-tall structure will span 73,762 square feet and yield 99 rental units with an average scope of 677 square feet. The project will also include 6,664 square feet of commercial space, two cellar levels, a 31-foot-long rear yard, and a 138-vehicle parking garage, according to permits filed in November 2021. The property is located at the northwest corner of 43rd Street and Roosevelt Avenue.</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>2026-07-07T11:00:58+00:00</t>
-        </is>
-      </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>Tue, 07 Jul 2026 11:00:58 +0000</t>
-        </is>
-      </c>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t>YIMBY</t>
-        </is>
-      </c>
-      <c r="G2" t="inlineStr">
-        <is>
-          <t>YIMBY - Sunnyside</t>
-        </is>
-      </c>
-      <c r="H2" t="inlineStr">
-        <is>
-          <t>By: Michael Young and Matt Pruznick 7:00 am on July 7, 2026 Construction is on hold at 43-42 43rd Street, the site of an eight-story mixed-use residential building in Sunnyside, Queens. Designed by Gerald Caliendo Architects for John J. Ciafone of City View Construction Corp., the 79-foot-tall structure will span 73,762 square feet and yield 99 rental units with an average scope of 677 square feet. The project will also include 6,664 square feet of commercial space, two cellar levels, a 31-foot-long rear yard, and a 138-vehicle parking garage, according to permits filed in November 2021. The property is located at the northwest corner of 43rd Street and Roosevelt Avenue. The site sits partially unearthed behind the construction fencing. It’s unclear when work will resume on the project. 43-42 43rd Street. Photo by Michael Young. 43-42 43rd Street. Photo by Michael Young. 43-42 43rd Street. Photo by Michael Young.</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>Cheskel Salamon buys two buildings for $4M in Bedford Park, likely dev site</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>https://www.pincusco.com/cheskel-salamon-buys-two-buildings-for-4m-in-bedford-park-likely-dev-site/</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>Cheskel Salamon paid $4.06 million for two adjacent buildings at 2814 and 2818 Morris Avenue</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>NaT</t>
-        </is>
-      </c>
-      <c r="E3" t="inlineStr"/>
-      <c r="F3" t="inlineStr">
-        <is>
-          <t>PincusCo</t>
-        </is>
-      </c>
-      <c r="G3" t="inlineStr">
-        <is>
-          <t>PincusCo - Home</t>
-        </is>
-      </c>
-      <c r="H3" t="inlineStr">
-        <is>
-          <t>Transfers 2814 Morris Avenue (Credit - Cyclomedia) Cheskel Salamon paid $4.06 million for two adjacent buildings at 2814 and 2818 Morris Avenue in Bedford Park, the Bronx, that are likely to be demolished to make way for a new development. In the first, Cheskel Salamon through the entity 2814-2818 Morris Owner LLC paid $2.6 million to Martin Ortega for the three-unit building (C0) at 2814 Morris Avenue. The deal closed on June 17, 2026 and was recorded on July 2, 2026. The property has 5,253 square feet of built space and 23,433 square feet of additional air rights for a total buildable of 28,673 square feet according to a PincusCo analysis of city data. The sale price per built square foot is $494 and the price per buildable square foot is $90 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) The signatory for Martin Ortega was Martin Ortega. The signatory for Cheskel Salamon was Cheskel Salamon. The contract date was November 7, 2025. In the second, Cheskel Salamon through the entity 2814-2818 Morris Owner LLC paid $1.5 million to Bernardo Arias fo</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto update queens news 2026-07-09T15:32:05Z
</commit_message>
<xml_diff>
--- a/data/output/queens_dev_news.xlsx
+++ b/data/output/queens_dev_news.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H1"/>
+  <dimension ref="A1:H4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -467,6 +467,108 @@
       <c r="H1" s="1" t="inlineStr">
         <is>
           <t>content_preview</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Anonymous buyer pays $6M to Plaxall for vacant lot in LIC</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>https://www.pincusco.com/anonymous-buyer-pays-6m-to-plaxall-for-vacant-lot-in-long-island-city/</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>The entity LIC Pacific LLC in care of the law firm Christodoulou &amp; Lau paid</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr"/>
+      <c r="E2" t="inlineStr"/>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>PincusCo</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>PincusCo - Home</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Transfers 49-09 5th Street (Credit - Cyclomedia) The entity LIC Pacific LLC in care of the law firm Christodoulou &amp; Lau paid $6 million to Plaxall through the entity PCI Green Realty, LLC for the industrial building (G7) at 49-09 5th Street in Long Island City, Queens. The deal closed on June 30, 2026 and was recorded on July 8, 2026. The property has zero square feet of built space and 15,000 square feet of additional air rights for a total buildable of 15,000 square feet according to a PincusCo analysis of city data. The sale price per buildable square foot is $400 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) The signatory for Plaxall was Leonard Matthew Quigley . The contract date was March 25, 2026. Prior sales, articles and revenue Prior to this transaction, PincusCo has records that the buyer registered with Christodoulou &amp; Lau purchased one property in one transaction for a total of $3.1 million and has no record it sold any properties over the past 24 months. The seller Plaxall had not purchased any other properties and had not sold any </t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Hung Pin Hung pays $6.5M for 30-unit dev site in Flushing</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>https://www.pincusco.com/hung-pin-hung-pays-6-5m-for-30-unit-rental-in-flushing/</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Hung Pin Hung through the entity 38th Avenue Flushing LLC paid $6.5 million to Terence</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr"/>
+      <c r="E3" t="inlineStr"/>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>PincusCo</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>PincusCo - Home</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>Transfers 144-14 38th Avenue (Credit - Cyclomedia) Hung Pin Hung through the entity 38th Avenue Flushing LLC paid $6.5 million to Terence Tai-Lin Cheng through the entity 144-14 38th, LLC for the 30-unit development site at 144-14 38th Avenue in Flushing, Queens. The expected use is ground up development On the lot, there was a new building construction project, 421571007, for a 30-unit, 27,850 square-foot residential (R-2) building. The project was submitted by Mike Cheng with plans filed October 30, 2017 and permitted March 24, 2022. The deal closed on June 30, 2026 and was recorded on July 8, 2026. The seller bought the property on September 15, 2017, for $4.7 million. The signatory for Terence Tai-Lin Cheng was Phyllis Cheng . The signatory for Hung Pin Hung was Hung Pin Hung. The contract date was May 15, 2026. Prior sales, articles and revenue Prior to this transaction, PincusCo has records that the buyer Hung Pin Hung purchased one property in one transaction for a total of $30 million and has no record it sold any properties over the past 24 months. The seller Terence Tai-Lin Cheng had not purchased any other properties and had not sold any properties over the same time per</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Raizel Feder signs $220M refi with BDT &amp; MSD Partners for large LIC dev site</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>https://www.pincusco.com/raizel-feder-signs-220m-refi-with-bdt-msd-partners-for-large-lic-dev-site/</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Raizel Feder through the entity 44-02 Ventures, LLC as borrower signed a refi loan with</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr"/>
+      <c r="E4" t="inlineStr"/>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>PincusCo</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>PincusCo - Home</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>Transfers 44-02 Vernon Boulevard (Credit - Cyclomedia) Raizel Feder through the entity 44-02 Ventures, LLC as borrower signed a refi loan with lender BDT &amp; MSD Partners through the entity Msd Rcof Partners XXVII, LLC valued at $220 million for three development properties including 44-02 Vernon Boulevard and 44-00 Vernon Boulevard in Long Island City, Queens. The deal closed on June 22, 2026 and was recorded on July 8, 2026. The prior lender was BDT &amp; MSD Partners which held debt that had an original loan amount of $165 million. The three properties have zero square feet of built space and 1,612,084 square feet of additional air rights for a total buildable of 1,612,084 square feet according to a PincusCo analysis of city data. The loan price per buildable square foot is $136 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) The signatory for Raizel Feder was Raizel Feder. The signatory for BDT &amp; MSD Partners was Kenneth Gerold . The prior borrowers for the $165 million loan from BDT were Harry Sussman and Bruce Teitelbaum. Court records indicated Ha</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto update queens news 2026-07-10T14:49:27Z
</commit_message>
<xml_diff>
--- a/data/output/queens_dev_news.xlsx
+++ b/data/output/queens_dev_news.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H4"/>
+  <dimension ref="A1:H1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -467,108 +467,6 @@
       <c r="H1" s="1" t="inlineStr">
         <is>
           <t>content_preview</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>Anonymous buyer pays $6M to Plaxall for vacant lot in LIC</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>https://www.pincusco.com/anonymous-buyer-pays-6m-to-plaxall-for-vacant-lot-in-long-island-city/</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>The entity LIC Pacific LLC in care of the law firm Christodoulou &amp; Lau paid</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr"/>
-      <c r="E2" t="inlineStr"/>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t>PincusCo</t>
-        </is>
-      </c>
-      <c r="G2" t="inlineStr">
-        <is>
-          <t>PincusCo - Home</t>
-        </is>
-      </c>
-      <c r="H2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Transfers 49-09 5th Street (Credit - Cyclomedia) The entity LIC Pacific LLC in care of the law firm Christodoulou &amp; Lau paid $6 million to Plaxall through the entity PCI Green Realty, LLC for the industrial building (G7) at 49-09 5th Street in Long Island City, Queens. The deal closed on June 30, 2026 and was recorded on July 8, 2026. The property has zero square feet of built space and 15,000 square feet of additional air rights for a total buildable of 15,000 square feet according to a PincusCo analysis of city data. The sale price per buildable square foot is $400 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) The signatory for Plaxall was Leonard Matthew Quigley . The contract date was March 25, 2026. Prior sales, articles and revenue Prior to this transaction, PincusCo has records that the buyer registered with Christodoulou &amp; Lau purchased one property in one transaction for a total of $3.1 million and has no record it sold any properties over the past 24 months. The seller Plaxall had not purchased any other properties and had not sold any </t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>Hung Pin Hung pays $6.5M for 30-unit dev site in Flushing</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>https://www.pincusco.com/hung-pin-hung-pays-6-5m-for-30-unit-rental-in-flushing/</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>Hung Pin Hung through the entity 38th Avenue Flushing LLC paid $6.5 million to Terence</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr"/>
-      <c r="E3" t="inlineStr"/>
-      <c r="F3" t="inlineStr">
-        <is>
-          <t>PincusCo</t>
-        </is>
-      </c>
-      <c r="G3" t="inlineStr">
-        <is>
-          <t>PincusCo - Home</t>
-        </is>
-      </c>
-      <c r="H3" t="inlineStr">
-        <is>
-          <t>Transfers 144-14 38th Avenue (Credit - Cyclomedia) Hung Pin Hung through the entity 38th Avenue Flushing LLC paid $6.5 million to Terence Tai-Lin Cheng through the entity 144-14 38th, LLC for the 30-unit development site at 144-14 38th Avenue in Flushing, Queens. The expected use is ground up development On the lot, there was a new building construction project, 421571007, for a 30-unit, 27,850 square-foot residential (R-2) building. The project was submitted by Mike Cheng with plans filed October 30, 2017 and permitted March 24, 2022. The deal closed on June 30, 2026 and was recorded on July 8, 2026. The seller bought the property on September 15, 2017, for $4.7 million. The signatory for Terence Tai-Lin Cheng was Phyllis Cheng . The signatory for Hung Pin Hung was Hung Pin Hung. The contract date was May 15, 2026. Prior sales, articles and revenue Prior to this transaction, PincusCo has records that the buyer Hung Pin Hung purchased one property in one transaction for a total of $30 million and has no record it sold any properties over the past 24 months. The seller Terence Tai-Lin Cheng had not purchased any other properties and had not sold any properties over the same time per</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>Raizel Feder signs $220M refi with BDT &amp; MSD Partners for large LIC dev site</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>https://www.pincusco.com/raizel-feder-signs-220m-refi-with-bdt-msd-partners-for-large-lic-dev-site/</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>Raizel Feder through the entity 44-02 Ventures, LLC as borrower signed a refi loan with</t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr"/>
-      <c r="E4" t="inlineStr"/>
-      <c r="F4" t="inlineStr">
-        <is>
-          <t>PincusCo</t>
-        </is>
-      </c>
-      <c r="G4" t="inlineStr">
-        <is>
-          <t>PincusCo - Home</t>
-        </is>
-      </c>
-      <c r="H4" t="inlineStr">
-        <is>
-          <t>Transfers 44-02 Vernon Boulevard (Credit - Cyclomedia) Raizel Feder through the entity 44-02 Ventures, LLC as borrower signed a refi loan with lender BDT &amp; MSD Partners through the entity Msd Rcof Partners XXVII, LLC valued at $220 million for three development properties including 44-02 Vernon Boulevard and 44-00 Vernon Boulevard in Long Island City, Queens. The deal closed on June 22, 2026 and was recorded on July 8, 2026. The prior lender was BDT &amp; MSD Partners which held debt that had an original loan amount of $165 million. The three properties have zero square feet of built space and 1,612,084 square feet of additional air rights for a total buildable of 1,612,084 square feet according to a PincusCo analysis of city data. The loan price per buildable square foot is $136 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) The signatory for Raizel Feder was Raizel Feder. The signatory for BDT &amp; MSD Partners was Kenneth Gerold . The prior borrowers for the $165 million loan from BDT were Harry Sussman and Bruce Teitelbaum. Court records indicated Ha</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto update queens news 2026-07-12T13:52:27Z
</commit_message>
<xml_diff>
--- a/data/output/queens_dev_news.xlsx
+++ b/data/output/queens_dev_news.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H1"/>
+  <dimension ref="A1:H2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -467,6 +467,48 @@
       <c r="H1" s="1" t="inlineStr">
         <is>
           <t>content_preview</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Rendering Revealed For Vernon Point at 44-68 Vernon Boulevard in Long Island City, Queens</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>https://newyorkyimby.com/2026/07/rendering-revealed-for-vernon-point-at-44-68-vernon-boulevard-in-long-island-city-queens.html</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>A new rendering has been revealed for Vernon Point, a planned 16-story residential building at 44-68 Vernon Boulevard in the Hunters Point section of &lt;a href="https://newyorkyimby.com/neighborhoods/long-island-city"&gt;Long Island City&lt;/a&gt;, Queens. Designed by Archimaera and developed by Elmrod Management, the 142,697-square-foot structure will yield 161 units and lower-level commercial space. The property is bounded by 44th Drive to the north, 45th Avenue to the south, and Vernon Boulevard to the east.</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>2026-07-12T12:00:01+00:00</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>Sun, 12 Jul 2026 12:00:01 +0000</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>YIMBY</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>YIMBY - Long Island City</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>By: Michael Young and Matt Pruznick 8:00 am on July 12, 2026 A new rendering has been revealed for Vernon Point, a planned 16-story residential building at 44-68 Vernon Boulevard in the Hunters Point section of Long Island City, Queens. Designed by Archimaera and developed by Elmrod Management, the 142,697-square-foot structure will yield 161 units and lower-level commercial space. The property is bounded by 44th Drive to the north, 45th Avenue to the south, and Vernon Boulevard to the east. The rendering looks southwest at the structure, previewing a monolithic massing with a chamfered eastern corner and a setback at its final level. The triple-height first story will be clad in a dark envelope with floor-to-ceiling glass, while the levels above will have a lighter gray façade surrounding columns of windows and glass doors leading to balconies. Landscaping and garden beds will flank the corner entrance to the building. The site is currently occupied by a low-rise industrial structure constructed in 1953. Elmrod Development acquired the property from an undisclosed seller for $28 million and recently secured $72.3 million in acquisition and construction financing from BridgeCity Ca</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto update queens news 2026-07-13T15:08:40Z
</commit_message>
<xml_diff>
--- a/data/output/queens_dev_news.xlsx
+++ b/data/output/queens_dev_news.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H2"/>
+  <dimension ref="A1:H1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -467,48 +467,6 @@
       <c r="H1" s="1" t="inlineStr">
         <is>
           <t>content_preview</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>Rendering Revealed For Vernon Point at 44-68 Vernon Boulevard in Long Island City, Queens</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>https://newyorkyimby.com/2026/07/rendering-revealed-for-vernon-point-at-44-68-vernon-boulevard-in-long-island-city-queens.html</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>A new rendering has been revealed for Vernon Point, a planned 16-story residential building at 44-68 Vernon Boulevard in the Hunters Point section of &lt;a href="https://newyorkyimby.com/neighborhoods/long-island-city"&gt;Long Island City&lt;/a&gt;, Queens. Designed by Archimaera and developed by Elmrod Management, the 142,697-square-foot structure will yield 161 units and lower-level commercial space. The property is bounded by 44th Drive to the north, 45th Avenue to the south, and Vernon Boulevard to the east.</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>2026-07-12T12:00:01+00:00</t>
-        </is>
-      </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>Sun, 12 Jul 2026 12:00:01 +0000</t>
-        </is>
-      </c>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t>YIMBY</t>
-        </is>
-      </c>
-      <c r="G2" t="inlineStr">
-        <is>
-          <t>YIMBY - Long Island City</t>
-        </is>
-      </c>
-      <c r="H2" t="inlineStr">
-        <is>
-          <t>By: Michael Young and Matt Pruznick 8:00 am on July 12, 2026 A new rendering has been revealed for Vernon Point, a planned 16-story residential building at 44-68 Vernon Boulevard in the Hunters Point section of Long Island City, Queens. Designed by Archimaera and developed by Elmrod Management, the 142,697-square-foot structure will yield 161 units and lower-level commercial space. The property is bounded by 44th Drive to the north, 45th Avenue to the south, and Vernon Boulevard to the east. The rendering looks southwest at the structure, previewing a monolithic massing with a chamfered eastern corner and a setback at its final level. The triple-height first story will be clad in a dark envelope with floor-to-ceiling glass, while the levels above will have a lighter gray façade surrounding columns of windows and glass doors leading to balconies. Landscaping and garden beds will flank the corner entrance to the building. The site is currently occupied by a low-rise industrial structure constructed in 1953. Elmrod Development acquired the property from an undisclosed seller for $28 million and recently secured $72.3 million in acquisition and construction financing from BridgeCity Ca</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto update queens news 2026-07-16T14:18:16Z
</commit_message>
<xml_diff>
--- a/data/output/queens_dev_news.xlsx
+++ b/data/output/queens_dev_news.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H1"/>
+  <dimension ref="A1:H2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -467,6 +467,40 @@
       <c r="H1" s="1" t="inlineStr">
         <is>
           <t>content_preview</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Catholic Homes signs $146.9M construction loan for 251-unit project in Tremont</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>https://www.pincusco.com/catholic-homes-signs-146-9m-construction-loan-for-251-unit-project-in-tremont/</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Catholic Homes through the entity Bathgate 178th Housing Development Fund Corporatio as borrower signed a</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr"/>
+      <c r="E2" t="inlineStr"/>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>PincusCo</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>PincusCo - Home</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>Transfers Two axonometric views of 484 East 178th Street (Credit - Fernando Villa architect via DOB) Continue reading with a PincusCo subscription Sign up for a paid subscription to view this content. Already a subscriber? Log in here. Continue Reading</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto update queens news 2026-07-17T13:59:51Z
</commit_message>
<xml_diff>
--- a/data/output/queens_dev_news.xlsx
+++ b/data/output/queens_dev_news.xlsx
@@ -473,17 +473,17 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Catholic Homes signs $146.9M construction loan for 251-unit project in Tremont</t>
+          <t>Lender Maverick acquires Hilson Management Garment District office for $49.95M</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>https://www.pincusco.com/catholic-homes-signs-146-9m-construction-loan-for-251-unit-project-in-tremont/</t>
+          <t>https://www.pincusco.com/lender-maverick-acquires-hilson-management-garment-district-office-for-49-95m/</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Catholic Homes through the entity Bathgate 178th Housing Development Fund Corporatio as borrower signed a</t>
+          <t>Maverick Real Estate Partners, a former lender on the property, through the entity Fifth Office</t>
         </is>
       </c>
       <c r="D2" t="inlineStr"/>
@@ -500,7 +500,7 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>Transfers Two axonometric views of 484 East 178th Street (Credit - Fernando Villa architect via DOB) Continue reading with a PincusCo subscription Sign up for a paid subscription to view this content. Already a subscriber? Log in here. Continue Reading</t>
+          <t xml:space="preserve">Chart_Frontpage Transfers 390 Fifth Avenue (Credit - Cyclomedia) Maverick Real Estate Partners, a former lender on the property, through the entity Fifth Office LLC took control from Hilson Management through the entity 390 Manager LLC, the office building (O6) at 390 Fifth Avenue in the Garment District, Manhattan, and related air rights, in an entity level transaction valued at $49.95 million. The deal closed on June 30, 2026 and was recorded on July 16, 2026. The building has 133,544 square feet of built space according to a PincusCo analysis of city data. The transfer price per built square foot is $374 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) With this entity level transaction that has the appearance of — but is not described as — a deed-in-lieu of foreclosure, Maverick Real Estate Partners took title to 390 Fifth Avenue and related air rights. Maverick bought the $50 million original principal debt on the asset in February 2024, then lent the Schwalbe family’s Hilson Management $47.4 million in March 2025, in a package with an initial </t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto update queens news 2026-07-18T13:45:07Z
</commit_message>
<xml_diff>
--- a/data/output/queens_dev_news.xlsx
+++ b/data/output/queens_dev_news.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H2"/>
+  <dimension ref="A1:H1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -467,40 +467,6 @@
       <c r="H1" s="1" t="inlineStr">
         <is>
           <t>content_preview</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>Lender Maverick acquires Hilson Management Garment District office for $49.95M</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>https://www.pincusco.com/lender-maverick-acquires-hilson-management-garment-district-office-for-49-95m/</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>Maverick Real Estate Partners, a former lender on the property, through the entity Fifth Office</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr"/>
-      <c r="E2" t="inlineStr"/>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t>PincusCo</t>
-        </is>
-      </c>
-      <c r="G2" t="inlineStr">
-        <is>
-          <t>PincusCo - Home</t>
-        </is>
-      </c>
-      <c r="H2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Chart_Frontpage Transfers 390 Fifth Avenue (Credit - Cyclomedia) Maverick Real Estate Partners, a former lender on the property, through the entity Fifth Office LLC took control from Hilson Management through the entity 390 Manager LLC, the office building (O6) at 390 Fifth Avenue in the Garment District, Manhattan, and related air rights, in an entity level transaction valued at $49.95 million. The deal closed on June 30, 2026 and was recorded on July 16, 2026. The building has 133,544 square feet of built space according to a PincusCo analysis of city data. The transfer price per built square foot is $374 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) With this entity level transaction that has the appearance of — but is not described as — a deed-in-lieu of foreclosure, Maverick Real Estate Partners took title to 390 Fifth Avenue and related air rights. Maverick bought the $50 million original principal debt on the asset in February 2024, then lent the Schwalbe family’s Hilson Management $47.4 million in March 2025, in a package with an initial </t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto update queens news 2026-07-20T14:31:19Z
</commit_message>
<xml_diff>
--- a/data/output/queens_dev_news.xlsx
+++ b/data/output/queens_dev_news.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H1"/>
+  <dimension ref="A1:H2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -467,6 +467,40 @@
       <c r="H1" s="1" t="inlineStr">
         <is>
           <t>content_preview</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Stylianos Aniftos signs $35M construction loan with Webster for 83-unit project in Astoria</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>https://www.pincusco.com/stylianos-aniftos-signs-35m-construction-loan-with-webster-bank-for-development-in-astoria/</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Stylianos Aniftos through the entity Aniska31 Realty, LLC as borrower signed a new construction loan</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr"/>
+      <c r="E2" t="inlineStr"/>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>PincusCo</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>PincusCo - Home</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>Transfers 25-60 31st Street axonometric diagram (Credit - Alexander Zhitnnik architect via DOB) Continue reading with a PincusCo subscription Sign up for a paid subscription to view this content. Already a subscriber? Log in here. Continue Reading</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto update queens news 2026-07-21T14:18:18Z
</commit_message>
<xml_diff>
--- a/data/output/queens_dev_news.xlsx
+++ b/data/output/queens_dev_news.xlsx
@@ -473,17 +473,17 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Stylianos Aniftos signs $35M construction loan with Webster for 83-unit project in Astoria</t>
+          <t>Jacob Fulop pays $4.1M for 8-unit walkup in Borough Park</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>https://www.pincusco.com/stylianos-aniftos-signs-35m-construction-loan-with-webster-bank-for-development-in-astoria/</t>
+          <t>https://www.pincusco.com/jacob-fulop-pays-4-1m-for-8-unit-walkup-in-borough-park/</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Stylianos Aniftos through the entity Aniska31 Realty, LLC as borrower signed a new construction loan</t>
+          <t>Jacob Fulop through the entity 1358 Lofts LLC paid $4.1 million to Michael C. Hecht</t>
         </is>
       </c>
       <c r="D2" t="inlineStr"/>
@@ -500,7 +500,7 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>Transfers 25-60 31st Street axonometric diagram (Credit - Alexander Zhitnnik architect via DOB) Continue reading with a PincusCo subscription Sign up for a paid subscription to view this content. Already a subscriber? Log in here. Continue Reading</t>
+          <t>Transfers 1358 57th Street (Credit - Cyclomedia) Jacob Fulop through the entity 1358 Lofts LLC paid $4.1 million to Michael C. Hecht through the entity Brevoort Realty LLC for the eight-unit residential walkup building (C1) at 1358 57th Street in Borough Park, Brooklyn. The expected use is cash flowing. The deal closed on July 13, 2026 and was recorded on July 20, 2026. The property has 8,140 square feet of built space according to a PincusCo analysis of city data. The sale price per built square foot is $503 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) The signatory for Michael C. Hecht was Michael C. Hecht. The signatory for Jacob Fulop was Jacob Fulop. The contract date was November 26, 2025. Prior sales, articles and revenue Prior to this transaction, PincusCo has records that the buyer Jacob Fulop purchased five properties in five transactions for a total of $40.7 million and sold one property in one transaction for a total of $10.5 million over the past 24 months. The seller Michael C. Hecht had not purchased any other properties and had n</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto update queens news 2026-07-22T14:19:29Z
</commit_message>
<xml_diff>
--- a/data/output/queens_dev_news.xlsx
+++ b/data/output/queens_dev_news.xlsx
@@ -473,34 +473,42 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Jacob Fulop pays $4.1M for 8-unit walkup in Borough Park</t>
+          <t>Permits Filed for 27-11 30th Avenue in Astoria, Queens</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>https://www.pincusco.com/jacob-fulop-pays-4-1m-for-8-unit-walkup-in-borough-park/</t>
+          <t>https://newyorkyimby.com/2026/07/permits-filed-for-27-11-30th-avenue-in-astoria-queens.html</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Jacob Fulop through the entity 1358 Lofts LLC paid $4.1 million to Michael C. Hecht</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr"/>
-      <c r="E2" t="inlineStr"/>
+          <t>Permits have been filed for a nine-story mixed-use building at 27-11 30th Avenue in &lt;a href="https://newyorkyimby.com/neighborhoods/astoria"&gt;Astoria&lt;/a&gt;, Queens. Located between 27th Street and 29th Street, the lot is near the 30th Avenue subway station, served by the N and W trains. Nicholas Notias of Neptune Mechanical, Inc. is listed as the owner behind the applications.</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>2026-07-22T10:30:23+00:00</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>Wed, 22 Jul 2026 10:30:23 +0000</t>
+        </is>
+      </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>PincusCo</t>
+          <t>YIMBY</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>PincusCo - Home</t>
+          <t>YIMBY - Astoria</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>Transfers 1358 57th Street (Credit - Cyclomedia) Jacob Fulop through the entity 1358 Lofts LLC paid $4.1 million to Michael C. Hecht through the entity Brevoort Realty LLC for the eight-unit residential walkup building (C1) at 1358 57th Street in Borough Park, Brooklyn. The expected use is cash flowing. The deal closed on July 13, 2026 and was recorded on July 20, 2026. The property has 8,140 square feet of built space according to a PincusCo analysis of city data. The sale price per built square foot is $503 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) The signatory for Michael C. Hecht was Michael C. Hecht. The signatory for Jacob Fulop was Jacob Fulop. The contract date was November 26, 2025. Prior sales, articles and revenue Prior to this transaction, PincusCo has records that the buyer Jacob Fulop purchased five properties in five transactions for a total of $40.7 million and sold one property in one transaction for a total of $10.5 million over the past 24 months. The seller Michael C. Hecht had not purchased any other properties and had n</t>
+          <t>By: Vanessa Londono 6:30 am on July 22, 2026 Permits have been filed for a nine-story mixed-use building at 27-11 30th Avenue in Astoria, Queens. Located between 27th Street and 29th Street, the lot is near the 30th Avenue subway station, served by the N and W trains. Nicholas Notias of Neptune Mechanical, Inc. is listed as the owner behind the applications. The proposed 95-foot-tall development will yield 20,266 square feet, with 18,105 square feet designated for residential space, 1,472 square feet of community facility space, and 689 square feet for commercial space. The building will have 26 residences, most likely rentals based on the average unit scope of 696 square feet. The concrete-based structure will also have a cellar, a 31-foot-long rear yard, and five open parking spaces. Harriet Nikakis of HCN Design is listed as the architect of record. Demolition permits have not been filed yet. An estimated completion date has not been announced. Subscribe to YIMBY’s daily e-mail Follow YIMBYgram for real-time photo updates Like YIMBY on Facebook Follow YIMBY’s Twitter for the latest in YIMBYnews</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto update queens news 2026-07-23T14:27:50Z
</commit_message>
<xml_diff>
--- a/data/output/queens_dev_news.xlsx
+++ b/data/output/queens_dev_news.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H2"/>
+  <dimension ref="A1:H3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -473,42 +473,68 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Permits Filed for 27-11 30th Avenue in Astoria, Queens</t>
+          <t>Prosper Property, HMG USA pay $24M to Forum Absolute for formerly stalled dev site in FiDi</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>https://newyorkyimby.com/2026/07/permits-filed-for-27-11-30th-avenue-in-astoria-queens.html</t>
+          <t>https://www.pincusco.com/prosper-property-hmg-usa-pay-24m-to-forum-absolute-for-formerly-stalled-dev-site-in-fidi/</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Permits have been filed for a nine-story mixed-use building at 27-11 30th Avenue in &lt;a href="https://newyorkyimby.com/neighborhoods/astoria"&gt;Astoria&lt;/a&gt;, Queens. Located between 27th Street and 29th Street, the lot is near the 30th Avenue subway station, served by the N and W trains. Nicholas Notias of Neptune Mechanical, Inc. is listed as the owner behind the applications.</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>2026-07-22T10:30:23+00:00</t>
-        </is>
-      </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>Wed, 22 Jul 2026 10:30:23 +0000</t>
-        </is>
-      </c>
+          <t>Prosper Property Group and the South Korea-based HMG USA Investment through the entity 65 West</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr"/>
+      <c r="E2" t="inlineStr"/>
       <c r="F2" t="inlineStr">
         <is>
-          <t>YIMBY</t>
+          <t>PincusCo</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>YIMBY - Astoria</t>
+          <t>PincusCo - Home</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>By: Vanessa Londono 6:30 am on July 22, 2026 Permits have been filed for a nine-story mixed-use building at 27-11 30th Avenue in Astoria, Queens. Located between 27th Street and 29th Street, the lot is near the 30th Avenue subway station, served by the N and W trains. Nicholas Notias of Neptune Mechanical, Inc. is listed as the owner behind the applications. The proposed 95-foot-tall development will yield 20,266 square feet, with 18,105 square feet designated for residential space, 1,472 square feet of community facility space, and 689 square feet for commercial space. The building will have 26 residences, most likely rentals based on the average unit scope of 696 square feet. The concrete-based structure will also have a cellar, a 31-foot-long rear yard, and five open parking spaces. Harriet Nikakis of HCN Design is listed as the architect of record. Demolition permits have not been filed yet. An estimated completion date has not been announced. Subscribe to YIMBY’s daily e-mail Follow YIMBYgram for real-time photo updates Like YIMBY on Facebook Follow YIMBY’s Twitter for the latest in YIMBYnews</t>
+          <t xml:space="preserve">Chart_Frontpage Transfers 65 West Broadway (Credit - Cyclomedia) Prosper Property Group and the South Korea-based HMG USA Investment through the entity 65 West Broadway Property Owner LLC paid $24 million to Forum Absolute Capital Partners through the entity Warren Murray Property Owner LLC for the development site at 65 West Broadway in Financial District, Manhattan. The expected use is cash flowing. The deal closed on July 9, 2026 and was recorded on July 22, 2026. The property has 66,668 square feet of built space according to a PincusCo analysis of city data. The sale price per built square foot is $359 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) On the lot, there is one active new building construction project, 121190497, for a 23-unit, 55,071 square-foot residential (R-2) building. The seller bought the property on May 5, 2015, for $50 million. The signatory for Forum Absolute Capital Partners was Eduard Naer . The signatory for Prosper Property Group and HMG USA Investment was Damien Smith . The contract date was April 14, 2026. The DOB </t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Bridges Development, A&amp;H buy foreclosed office in Sheepshead Bay for $31M</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>https://www.pincusco.com/bridges-development-ah-buy-foreclosed-office-in-sheepshead-bay-for-31m/</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Bridges Development Group and A&amp;H Acquisitions through the entity 1630 15th Street LLC paid $31</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr"/>
+      <c r="E3" t="inlineStr"/>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>PincusCo</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>PincusCo - Home</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>Transfers 1630 East 15th Street (Credit - Cyclomedia) Bridges Development Group and A&amp;H Acquisitions through the entity 1630 15th Street LLC paid $31 million to bondholders of a trust, Series 2018-Cor3 as serviced by Midland Loan Services, through the entity Comm 2018-Cor3 1630 East 15th Street LLC, for the office building (O5) at 1630 East 15th Street in Sheepshead Bay, Brooklyn. The expected use is cash flowing. The deal closed on July 13, 2026 and was recorded on July 22, 2026. The property has 229,926 square feet of built space according to a PincusCo analysis of city data. The sale price per built square foot is $134 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) The signatory for Series 2018-Cor3 and Midland Loan Services was Stephen Reynolds . The signatory for Bridges Development Group and A&amp;H Acquisitions was Marcus Adjmi . The contract date was April 14, 2026. Bridges and A&amp;H have partnered in the past, including in Crown Heights. Urban Edge Properties in 2020 bought the mixed-use building from Nightingale Properties and Steven Kassin an</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto update queens news 2026-07-24T14:08:28Z
</commit_message>
<xml_diff>
--- a/data/output/queens_dev_news.xlsx
+++ b/data/output/queens_dev_news.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H3"/>
+  <dimension ref="A1:H1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -467,74 +467,6 @@
       <c r="H1" s="1" t="inlineStr">
         <is>
           <t>content_preview</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>Prosper Property, HMG USA pay $24M to Forum Absolute for formerly stalled dev site in FiDi</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>https://www.pincusco.com/prosper-property-hmg-usa-pay-24m-to-forum-absolute-for-formerly-stalled-dev-site-in-fidi/</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>Prosper Property Group and the South Korea-based HMG USA Investment through the entity 65 West</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr"/>
-      <c r="E2" t="inlineStr"/>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t>PincusCo</t>
-        </is>
-      </c>
-      <c r="G2" t="inlineStr">
-        <is>
-          <t>PincusCo - Home</t>
-        </is>
-      </c>
-      <c r="H2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Chart_Frontpage Transfers 65 West Broadway (Credit - Cyclomedia) Prosper Property Group and the South Korea-based HMG USA Investment through the entity 65 West Broadway Property Owner LLC paid $24 million to Forum Absolute Capital Partners through the entity Warren Murray Property Owner LLC for the development site at 65 West Broadway in Financial District, Manhattan. The expected use is cash flowing. The deal closed on July 9, 2026 and was recorded on July 22, 2026. The property has 66,668 square feet of built space according to a PincusCo analysis of city data. The sale price per built square foot is $359 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) On the lot, there is one active new building construction project, 121190497, for a 23-unit, 55,071 square-foot residential (R-2) building. The seller bought the property on May 5, 2015, for $50 million. The signatory for Forum Absolute Capital Partners was Eduard Naer . The signatory for Prosper Property Group and HMG USA Investment was Damien Smith . The contract date was April 14, 2026. The DOB </t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>Bridges Development, A&amp;H buy foreclosed office in Sheepshead Bay for $31M</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>https://www.pincusco.com/bridges-development-ah-buy-foreclosed-office-in-sheepshead-bay-for-31m/</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>Bridges Development Group and A&amp;H Acquisitions through the entity 1630 15th Street LLC paid $31</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr"/>
-      <c r="E3" t="inlineStr"/>
-      <c r="F3" t="inlineStr">
-        <is>
-          <t>PincusCo</t>
-        </is>
-      </c>
-      <c r="G3" t="inlineStr">
-        <is>
-          <t>PincusCo - Home</t>
-        </is>
-      </c>
-      <c r="H3" t="inlineStr">
-        <is>
-          <t>Transfers 1630 East 15th Street (Credit - Cyclomedia) Bridges Development Group and A&amp;H Acquisitions through the entity 1630 15th Street LLC paid $31 million to bondholders of a trust, Series 2018-Cor3 as serviced by Midland Loan Services, through the entity Comm 2018-Cor3 1630 East 15th Street LLC, for the office building (O5) at 1630 East 15th Street in Sheepshead Bay, Brooklyn. The expected use is cash flowing. The deal closed on July 13, 2026 and was recorded on July 22, 2026. The property has 229,926 square feet of built space according to a PincusCo analysis of city data. The sale price per built square foot is $134 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) The signatory for Series 2018-Cor3 and Midland Loan Services was Stephen Reynolds . The signatory for Bridges Development Group and A&amp;H Acquisitions was Marcus Adjmi . The contract date was April 14, 2026. Bridges and A&amp;H have partnered in the past, including in Crown Heights. Urban Edge Properties in 2020 bought the mixed-use building from Nightingale Properties and Steven Kassin an</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto update queens news 2026-07-27T15:10:23Z
</commit_message>
<xml_diff>
--- a/data/output/queens_dev_news.xlsx
+++ b/data/output/queens_dev_news.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H1"/>
+  <dimension ref="A1:H2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -467,6 +467,40 @@
       <c r="H1" s="1" t="inlineStr">
         <is>
           <t>content_preview</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Lakhwinder Singh files plans for 99 units in Jamaica</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>https://www.pincusco.com/lakhwinder-singh-files-plans-for-99-units-in-jamaica/</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Lakhwinder Singh submitted a new building construction project for a 99-unit, 83,744-square-foot residential (R-2) building</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr"/>
+      <c r="E2" t="inlineStr"/>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>PincusCo</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>PincusCo - Home</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>Development 147-45 94th Avenue axonometric diagram and elevations (Credit - Ning Lu architect via DOB) Continue reading with a PincusCo subscription Sign up for a paid subscription to view this content. Already a subscriber? Log in here. Continue Reading</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto update queens news 2026-07-28T14:32:22Z
</commit_message>
<xml_diff>
--- a/data/output/queens_dev_news.xlsx
+++ b/data/output/queens_dev_news.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H2"/>
+  <dimension ref="A1:H3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -473,17 +473,17 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Lakhwinder Singh files plans for 99 units in Jamaica</t>
+          <t>Home Tile Center owner pays $5.5M for current location in LIC</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>https://www.pincusco.com/lakhwinder-singh-files-plans-for-99-units-in-jamaica/</t>
+          <t>https://www.pincusco.com/home-tile-center-owner-pays-5-5m-for-current-location-in-lic/</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Lakhwinder Singh submitted a new building construction project for a 99-unit, 83,744-square-foot residential (R-2) building</t>
+          <t>Theodore Doukakis of Home Tile Center of NY through the entity YRL Realty LLC paid</t>
         </is>
       </c>
       <c r="D2" t="inlineStr"/>
@@ -500,7 +500,41 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>Development 147-45 94th Avenue axonometric diagram and elevations (Credit - Ning Lu architect via DOB) Continue reading with a PincusCo subscription Sign up for a paid subscription to view this content. Already a subscriber? Log in here. Continue Reading</t>
+          <t>Transfers 33-09 37th Avenue (Credit - Cyclomedia) Theodore Doukakis of Home Tile Center of NY through the entity YRL Realty LLC paid $5.5 million to Woods &amp; Jaye Sales Company through the entity Woods &amp; Jaye Realty Company, LLC for the industrial building (E1) at 33-09 37th Avenue in Long Island City, Queens. The expected use is owner-occupied. Home Tile Center of NY is the current occupant of the building, according to the company website. The deal closed on July 8, 2026 and was recorded on July 27, 2026. The property has 9,566 square feet of built space according to a PincusCo analysis of city data. The sale price per built square foot is $574 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) The signatory for Woods &amp; Jaye Sales Company was Stephen C. Jaye . The signatory for Theodore Doukakis was Theodore Doukakis. The contract date was November 24, 2025. Theodore Doukakis is an executive with Home Tile Center of NY. Prior sales, articles and revenue Prior to this transaction, PincusCo has no record that the buyer Theodore Doukakis had purchased a</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Galinda Wang pays $4.6M to Ruxton Capital for 24-unit walkup in LIC</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>https://www.pincusco.com/galinda-wang-pays-4-6m-to-ruxton-capital-for-24-unit-walkup-in-lic/</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Galinda Wang through the entity Van Alst Court Apts LLC paid $4.6 million to Ruxton</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr"/>
+      <c r="E3" t="inlineStr"/>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>PincusCo</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>PincusCo - Home</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>Transfers 44-73 21st Street (Credit - Cyclomedia) Galinda Wang through the entity Van Alst Court Apts LLC paid $4.6 million to Ruxton Capital Group through the entity Drake Holding NY LLC for the 24-unit residential walkup building (C1) at 44-73 21st Street in Long Island City, Queens. The expected use is cash flowing. The deal closed on July 21, 2026 and was recorded on July 27, 2026. The property has 20,312 square feet of built space according to a PincusCo analysis of city data. The sale price per built square foot is $227 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) The seller bought the property on January 6, 2009, for $5.2 million. The signatory for Ruxton Capital Group was David Tannenhauser . The signatory for Galinda Wang was Galinda Wang. She often partners with Paul Tchao. The contract date was April 2, 2026. Prior sales, articles and revenue Prior to this transaction, PincusCo has records that the buyer Galinda Wang purchased one property in one transaction for a total of $7.3 million and has no record it sold any properties over the</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto update queens news 2026-07-29T14:29:15Z
</commit_message>
<xml_diff>
--- a/data/output/queens_dev_news.xlsx
+++ b/data/output/queens_dev_news.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H3"/>
+  <dimension ref="A1:H1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -467,74 +467,6 @@
       <c r="H1" s="1" t="inlineStr">
         <is>
           <t>content_preview</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>Home Tile Center owner pays $5.5M for current location in LIC</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>https://www.pincusco.com/home-tile-center-owner-pays-5-5m-for-current-location-in-lic/</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>Theodore Doukakis of Home Tile Center of NY through the entity YRL Realty LLC paid</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr"/>
-      <c r="E2" t="inlineStr"/>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t>PincusCo</t>
-        </is>
-      </c>
-      <c r="G2" t="inlineStr">
-        <is>
-          <t>PincusCo - Home</t>
-        </is>
-      </c>
-      <c r="H2" t="inlineStr">
-        <is>
-          <t>Transfers 33-09 37th Avenue (Credit - Cyclomedia) Theodore Doukakis of Home Tile Center of NY through the entity YRL Realty LLC paid $5.5 million to Woods &amp; Jaye Sales Company through the entity Woods &amp; Jaye Realty Company, LLC for the industrial building (E1) at 33-09 37th Avenue in Long Island City, Queens. The expected use is owner-occupied. Home Tile Center of NY is the current occupant of the building, according to the company website. The deal closed on July 8, 2026 and was recorded on July 27, 2026. The property has 9,566 square feet of built space according to a PincusCo analysis of city data. The sale price per built square foot is $574 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) The signatory for Woods &amp; Jaye Sales Company was Stephen C. Jaye . The signatory for Theodore Doukakis was Theodore Doukakis. The contract date was November 24, 2025. Theodore Doukakis is an executive with Home Tile Center of NY. Prior sales, articles and revenue Prior to this transaction, PincusCo has no record that the buyer Theodore Doukakis had purchased a</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>Galinda Wang pays $4.6M to Ruxton Capital for 24-unit walkup in LIC</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>https://www.pincusco.com/galinda-wang-pays-4-6m-to-ruxton-capital-for-24-unit-walkup-in-lic/</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>Galinda Wang through the entity Van Alst Court Apts LLC paid $4.6 million to Ruxton</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr"/>
-      <c r="E3" t="inlineStr"/>
-      <c r="F3" t="inlineStr">
-        <is>
-          <t>PincusCo</t>
-        </is>
-      </c>
-      <c r="G3" t="inlineStr">
-        <is>
-          <t>PincusCo - Home</t>
-        </is>
-      </c>
-      <c r="H3" t="inlineStr">
-        <is>
-          <t>Transfers 44-73 21st Street (Credit - Cyclomedia) Galinda Wang through the entity Van Alst Court Apts LLC paid $4.6 million to Ruxton Capital Group through the entity Drake Holding NY LLC for the 24-unit residential walkup building (C1) at 44-73 21st Street in Long Island City, Queens. The expected use is cash flowing. The deal closed on July 21, 2026 and was recorded on July 27, 2026. The property has 20,312 square feet of built space according to a PincusCo analysis of city data. The sale price per built square foot is $227 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) The seller bought the property on January 6, 2009, for $5.2 million. The signatory for Ruxton Capital Group was David Tannenhauser . The signatory for Galinda Wang was Galinda Wang. She often partners with Paul Tchao. The contract date was April 2, 2026. Prior sales, articles and revenue Prior to this transaction, PincusCo has records that the buyer Galinda Wang purchased one property in one transaction for a total of $7.3 million and has no record it sold any properties over the</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto update queens news 2026-07-30T14:28:56Z
</commit_message>
<xml_diff>
--- a/data/output/queens_dev_news.xlsx
+++ b/data/output/queens_dev_news.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H1"/>
+  <dimension ref="A1:H3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -467,6 +467,74 @@
       <c r="H1" s="1" t="inlineStr">
         <is>
           <t>content_preview</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Lightstone in contract to pay Pinnacle $88M for control of 172-unit UWS rental</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>https://www.pincusco.com/lightstone-in-contract-to-pay-pinnacle-88m-for-control-of-172-unit-uws-rental/</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>David Lichtenstein’s Lightstone Group through the entity LREP Acquisitions XIV LLC, as buyer signed a</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr"/>
+      <c r="E2" t="inlineStr"/>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>PincusCo</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>PincusCo - Home</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>Top Story Transfers 323 West 96th Street (Credit - Cyclomedia) Continue reading with a PincusCo subscription Sign up for a paid subscription to view this content. Already a subscriber? Log in here.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Qiang Chen files plans for 12 units in Astoria</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>https://www.pincusco.com/qiang-chen-files-plans-for-12-units-in-astoria/</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Qiang Chen submitted a new building construction project for a 12-unit, 11,812-square-foot residential (R-2) building</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr"/>
+      <c r="E3" t="inlineStr"/>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>PincusCo</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>PincusCo - Home</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>Development 11-23 31st Drive axonometric diagram (Credit - Hui Zeng architect via DOB) Continue reading with a PincusCo subscription Sign up for a paid subscription to view this content. Already a subscriber? Log in here. Continue Reading</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto update queens news 2026-07-31T14:31:27Z
</commit_message>
<xml_diff>
--- a/data/output/queens_dev_news.xlsx
+++ b/data/output/queens_dev_news.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H3"/>
+  <dimension ref="A1:H2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -473,17 +473,17 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Lightstone in contract to pay Pinnacle $88M for control of 172-unit UWS rental</t>
+          <t>Kostas Papadakis files plans for 54 units in Astoria</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>https://www.pincusco.com/lightstone-in-contract-to-pay-pinnacle-88m-for-control-of-172-unit-uws-rental/</t>
+          <t>https://www.pincusco.com/kostas-papadakis-files-plans-for-54-units-in-astoria/</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>David Lichtenstein’s Lightstone Group through the entity LREP Acquisitions XIV LLC, as buyer signed a</t>
+          <t>Kostas Papadakis submitted a new building construction project for a 54-unit, 64,650-square-foot residential (R-2) building</t>
         </is>
       </c>
       <c r="D2" t="inlineStr"/>
@@ -500,41 +500,7 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>Top Story Transfers 323 West 96th Street (Credit - Cyclomedia) Continue reading with a PincusCo subscription Sign up for a paid subscription to view this content. Already a subscriber? Log in here.</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>Qiang Chen files plans for 12 units in Astoria</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>https://www.pincusco.com/qiang-chen-files-plans-for-12-units-in-astoria/</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>Qiang Chen submitted a new building construction project for a 12-unit, 11,812-square-foot residential (R-2) building</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr"/>
-      <c r="E3" t="inlineStr"/>
-      <c r="F3" t="inlineStr">
-        <is>
-          <t>PincusCo</t>
-        </is>
-      </c>
-      <c r="G3" t="inlineStr">
-        <is>
-          <t>PincusCo - Home</t>
-        </is>
-      </c>
-      <c r="H3" t="inlineStr">
-        <is>
-          <t>Development 11-23 31st Drive axonometric diagram (Credit - Hui Zeng architect via DOB) Continue reading with a PincusCo subscription Sign up for a paid subscription to view this content. Already a subscriber? Log in here. Continue Reading</t>
+          <t>Development 42-18 31st Avenue axonometric diagram (Credit - Patrizia Cimino architect via DOB) Continue reading with a PincusCo subscription Sign up for a paid subscription to view this content. Already a subscriber? Log in here. Continue Reading</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto update queens news 2026-08-01T13:50:58Z
</commit_message>
<xml_diff>
--- a/data/output/queens_dev_news.xlsx
+++ b/data/output/queens_dev_news.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H2"/>
+  <dimension ref="A1:H1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -467,40 +467,6 @@
       <c r="H1" s="1" t="inlineStr">
         <is>
           <t>content_preview</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>Kostas Papadakis files plans for 54 units in Astoria</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>https://www.pincusco.com/kostas-papadakis-files-plans-for-54-units-in-astoria/</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>Kostas Papadakis submitted a new building construction project for a 54-unit, 64,650-square-foot residential (R-2) building</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr"/>
-      <c r="E2" t="inlineStr"/>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t>PincusCo</t>
-        </is>
-      </c>
-      <c r="G2" t="inlineStr">
-        <is>
-          <t>PincusCo - Home</t>
-        </is>
-      </c>
-      <c r="H2" t="inlineStr">
-        <is>
-          <t>Development 42-18 31st Avenue axonometric diagram (Credit - Patrizia Cimino architect via DOB) Continue reading with a PincusCo subscription Sign up for a paid subscription to view this content. Already a subscriber? Log in here. Continue Reading</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto update queens news 2026-08-04T14:37:07Z
</commit_message>
<xml_diff>
--- a/data/output/queens_dev_news.xlsx
+++ b/data/output/queens_dev_news.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H1"/>
+  <dimension ref="A1:H2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -467,6 +467,48 @@
       <c r="H1" s="1" t="inlineStr">
         <is>
           <t>content_preview</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Paragon LIC Nears Completion At 45-40 Vernon Boulevard In Long Island City, Queens</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>https://newyorkyimby.com/2026/08/paragon-lic-nears-completion-at-45-40-vernon-boulevard-in-long-island-city-queens.html</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Construction is nearing completion on Paragon LIC, a 23-story residential building at 45-40 Vernon Boulevard in &lt;a href="https://newyorkyimby.com/neighborhoods/long-island-city"&gt;Long Island City&lt;/a&gt;, Queens. Designed by Archimaera and developed and built by ZD Jasper, the 262-foot-tall structure spans 192,500 square feet and yields 182 condominium units, down from the 226 units listed in filings. The project will also include ground-floor retail space and a public waterfront park. The property is located between 45th Road and 46th Avenue.</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>2026-08-04T11:30:43+00:00</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>Tue, 04 Aug 2026 11:30:43 +0000</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>YIMBY</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>YIMBY - Long Island City</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>By: Max Gillespie 7:30 am on August 4, 2026 Construction is nearing completion on Paragon LIC, a 23-story residential building at 45-40 Vernon Boulevard in Long Island City, Queens. Designed by Archimaera and developed and built by ZD Jasper, the 262-foot-tall structure spans 192,500 square feet and yields 182 condominium units, down from the 226 units listed in filings. The project will also include ground-floor retail space and a public waterfront park. The property is located between 45th Road and 46th Avenue. Rendering of Paragon LIC. Credit: Redundant Pixel. Rendering of Paragon LIC. Credit: Redundant Pixel. Façade installation has drawn to a close since our last update in November 2025, when the reinforced concrete superstructure had just topped out. The tower is set back 80 feet from Vernon Boulevard behind the restored factory, its massing composed of staggered, double-height balcony boxes in copper-toned projecting frames that reference the site’s industrial past. The frames extend further at the northern end of the eastern profile and both ends of the northern face, forming terraces lined with glass railings, and the structure culminates in a glass-clad crown with vertica</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto update queens news 2026-08-05T14:29:22Z
</commit_message>
<xml_diff>
--- a/data/output/queens_dev_news.xlsx
+++ b/data/output/queens_dev_news.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H2"/>
+  <dimension ref="A1:H1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -467,48 +467,6 @@
       <c r="H1" s="1" t="inlineStr">
         <is>
           <t>content_preview</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>Paragon LIC Nears Completion At 45-40 Vernon Boulevard In Long Island City, Queens</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>https://newyorkyimby.com/2026/08/paragon-lic-nears-completion-at-45-40-vernon-boulevard-in-long-island-city-queens.html</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>Construction is nearing completion on Paragon LIC, a 23-story residential building at 45-40 Vernon Boulevard in &lt;a href="https://newyorkyimby.com/neighborhoods/long-island-city"&gt;Long Island City&lt;/a&gt;, Queens. Designed by Archimaera and developed and built by ZD Jasper, the 262-foot-tall structure spans 192,500 square feet and yields 182 condominium units, down from the 226 units listed in filings. The project will also include ground-floor retail space and a public waterfront park. The property is located between 45th Road and 46th Avenue.</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>2026-08-04T11:30:43+00:00</t>
-        </is>
-      </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>Tue, 04 Aug 2026 11:30:43 +0000</t>
-        </is>
-      </c>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t>YIMBY</t>
-        </is>
-      </c>
-      <c r="G2" t="inlineStr">
-        <is>
-          <t>YIMBY - Long Island City</t>
-        </is>
-      </c>
-      <c r="H2" t="inlineStr">
-        <is>
-          <t>By: Max Gillespie 7:30 am on August 4, 2026 Construction is nearing completion on Paragon LIC, a 23-story residential building at 45-40 Vernon Boulevard in Long Island City, Queens. Designed by Archimaera and developed and built by ZD Jasper, the 262-foot-tall structure spans 192,500 square feet and yields 182 condominium units, down from the 226 units listed in filings. The project will also include ground-floor retail space and a public waterfront park. The property is located between 45th Road and 46th Avenue. Rendering of Paragon LIC. Credit: Redundant Pixel. Rendering of Paragon LIC. Credit: Redundant Pixel. Façade installation has drawn to a close since our last update in November 2025, when the reinforced concrete superstructure had just topped out. The tower is set back 80 feet from Vernon Boulevard behind the restored factory, its massing composed of staggered, double-height balcony boxes in copper-toned projecting frames that reference the site’s industrial past. The frames extend further at the northern end of the eastern profile and both ends of the northern face, forming terraces lined with glass railings, and the structure culminates in a glass-clad crown with vertica</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto update queens news 2026-08-06T14:32:18Z
</commit_message>
<xml_diff>
--- a/data/output/queens_dev_news.xlsx
+++ b/data/output/queens_dev_news.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H1"/>
+  <dimension ref="A1:H2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -467,6 +467,40 @@
       <c r="H1" s="1" t="inlineStr">
         <is>
           <t>content_preview</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Daolin Hou files plans for 30 units in Astoria</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>https://www.pincusco.com/daolin-hou-files-plans-for-30-units-in-astoria/</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Daolin Hou submitted a new building construction project for a 30-unit, 37,832-square-foot residential (R-2) building</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr"/>
+      <c r="E2" t="inlineStr"/>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>PincusCo</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>PincusCo - Home</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>Development 30-88 Crescent Street axonometric diagram (Credit - Joon Ho Chai architect via DOB) Continue reading with a PincusCo subscription Sign up for a paid subscription to view this content. Already a subscriber? Log in here. Continue Reading</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto update queens news 2026-08-07T13:34:44Z
</commit_message>
<xml_diff>
--- a/data/output/queens_dev_news.xlsx
+++ b/data/output/queens_dev_news.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H2"/>
+  <dimension ref="A1:H3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -473,34 +473,80 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Daolin Hou files plans for 30 units in Astoria</t>
+          <t>Permits Filed for 30-88 Crescent Street in Astoria, Queens</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>https://www.pincusco.com/daolin-hou-files-plans-for-30-units-in-astoria/</t>
+          <t>https://newyorkyimby.com/2026/08/permits-filed-for-30-88-crescent-street-in-astoria-queens.html</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Daolin Hou submitted a new building construction project for a 30-unit, 37,832-square-foot residential (R-2) building</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr"/>
-      <c r="E2" t="inlineStr"/>
+          <t>Permits have been filed for a six-story residential building at 30-88 Crescent Street in &lt;a href="https://newyorkyimby.com/neighborhoods/astoria"&gt;Astoria&lt;/a&gt;, Queens. Located between 30th Drive and 31st Avenue, the lot is near the 30th Avenue subway station, served by the N and W trains. Daolin Hou of CCJ Capital LLC is listed as the owner behind the applications.</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>2026-08-07T10:30:17+00:00</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>Fri, 07 Aug 2026 10:30:17 +0000</t>
+        </is>
+      </c>
       <c r="F2" t="inlineStr">
         <is>
+          <t>YIMBY</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>YIMBY - Astoria</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>By: Vanessa Londono 6:30 am on August 7, 2026 Permits have been filed for a six-story residential building at 30-88 Crescent Street in Astoria, Queens. Located between 30th Drive and 31st Avenue, the lot is near the 30th Avenue subway station, served by the N and W trains. Daolin Hou of CCJ Capital LLC is listed as the owner behind the applications. The proposed 65-foot-tall development will yield 31,511 square feet designated for residential space. The building will have 30 residences, most likely condos based on the average unit scope of 1,050 square feet. The concrete-based structure will also have a penthouse, a 30-foot-long rear yard, 12 open parking spaces, and two enclosed parking spaces. Joon Ho Chai of James Chai Architect, P.C is listed as the architect of record. Demolition permits were filed in May for the residential building on the site. An estimated completion date has not been announced. Subscribe to YIMBY’s daily e-mail Follow YIMBYgram for real-time photo updates Like YIMBY on Facebook Follow YIMBY’s Twitter for the latest in YIMBYnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Art Partner affiliate pays $7M for commercial condos in Chelsea</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>https://www.pincusco.com/art-partner-affiliate-pays-7m-for-commercial-condos-in-chelsea/</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Art Partner through the entity Amberlight Holdings LLC paid $7 million to an affiliate of</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>NaT</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr"/>
+      <c r="F3" t="inlineStr">
+        <is>
           <t>PincusCo</t>
         </is>
       </c>
-      <c r="G2" t="inlineStr">
+      <c r="G3" t="inlineStr">
         <is>
           <t>PincusCo - Home</t>
         </is>
       </c>
-      <c r="H2" t="inlineStr">
-        <is>
-          <t>Development 30-88 Crescent Street axonometric diagram (Credit - Joon Ho Chai architect via DOB) Continue reading with a PincusCo subscription Sign up for a paid subscription to view this content. Already a subscriber? Log in here. Continue Reading</t>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>Transfers 545 West 25th Street (Credit - Cyclomedia) Art Partner through the entity Amberlight Holdings LLC paid $7 million to an affiliate of the public relations firm Karla Otto through the entity Okre, LLC for two commercial condominium units on the 11th and 12th floors of 545 West 25th Street in Chelsea, Manhattan. The expected use is owner-occupied. The deal closed on July 28, 2026 and was recorded on August 6, 2026. The two properties have 7,080 square feet of built space according to a PincusCo analysis of city data. The sale price per built square foot is $988 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) The signatory for Karla Otto was Lawrence Rader . The signatory for Art Partner was Steven Tanen . The contract date was March 3, 2026. Art Partner is a global creative agency that manages talent for the fashion and luxury industries, and lists its address on the 12th floor, according to its website. Amber Testino is an executive at the firm. Her husband Giovanni Testino founded Art Partner. On July 1, 2026, Gazelli Art House pays $7.5 m</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto update queens news 2026-08-08T13:10:18Z
</commit_message>
<xml_diff>
--- a/data/output/queens_dev_news.xlsx
+++ b/data/output/queens_dev_news.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H3"/>
+  <dimension ref="A1:H2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -473,27 +473,27 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Permits Filed for 30-88 Crescent Street in Astoria, Queens</t>
+          <t>Permits Filed for 43-27 56th Street in Woodside, Queens</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>https://newyorkyimby.com/2026/08/permits-filed-for-30-88-crescent-street-in-astoria-queens.html</t>
+          <t>https://newyorkyimby.com/2026/08/permits-filed-for-43-27-56th-street-in-woodside-queens.html</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Permits have been filed for a six-story residential building at 30-88 Crescent Street in &lt;a href="https://newyorkyimby.com/neighborhoods/astoria"&gt;Astoria&lt;/a&gt;, Queens. Located between 30th Drive and 31st Avenue, the lot is near the 30th Avenue subway station, served by the N and W trains. Daolin Hou of CCJ Capital LLC is listed as the owner behind the applications.</t>
+          <t>Permits have been filed for a nine-story mixed-use building at 43-27 56th Street in &lt;a href="https://newyorkyimby.com/neighborhoods/woodside"&gt;Woodside&lt;/a&gt;, Queens. Located between 43rd Avenue Street and Queens Boulevard, the lot is near the 52nd Street subway station, served by the 7 train. Markiel Chulpayev is listed as the owner behind the applications.</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>2026-08-07T10:30:17+00:00</t>
+          <t>2026-08-08T10:30:22+00:00</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>Fri, 07 Aug 2026 10:30:17 +0000</t>
+          <t>Sat, 08 Aug 2026 10:30:22 +0000</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
@@ -503,50 +503,12 @@
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>YIMBY - Astoria</t>
+          <t>YIMBY - Woodside</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>By: Vanessa Londono 6:30 am on August 7, 2026 Permits have been filed for a six-story residential building at 30-88 Crescent Street in Astoria, Queens. Located between 30th Drive and 31st Avenue, the lot is near the 30th Avenue subway station, served by the N and W trains. Daolin Hou of CCJ Capital LLC is listed as the owner behind the applications. The proposed 65-foot-tall development will yield 31,511 square feet designated for residential space. The building will have 30 residences, most likely condos based on the average unit scope of 1,050 square feet. The concrete-based structure will also have a penthouse, a 30-foot-long rear yard, 12 open parking spaces, and two enclosed parking spaces. Joon Ho Chai of James Chai Architect, P.C is listed as the architect of record. Demolition permits were filed in May for the residential building on the site. An estimated completion date has not been announced. Subscribe to YIMBY’s daily e-mail Follow YIMBYgram for real-time photo updates Like YIMBY on Facebook Follow YIMBY’s Twitter for the latest in YIMBYnews</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>Art Partner affiliate pays $7M for commercial condos in Chelsea</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>https://www.pincusco.com/art-partner-affiliate-pays-7m-for-commercial-condos-in-chelsea/</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>Art Partner through the entity Amberlight Holdings LLC paid $7 million to an affiliate of</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>NaT</t>
-        </is>
-      </c>
-      <c r="E3" t="inlineStr"/>
-      <c r="F3" t="inlineStr">
-        <is>
-          <t>PincusCo</t>
-        </is>
-      </c>
-      <c r="G3" t="inlineStr">
-        <is>
-          <t>PincusCo - Home</t>
-        </is>
-      </c>
-      <c r="H3" t="inlineStr">
-        <is>
-          <t>Transfers 545 West 25th Street (Credit - Cyclomedia) Art Partner through the entity Amberlight Holdings LLC paid $7 million to an affiliate of the public relations firm Karla Otto through the entity Okre, LLC for two commercial condominium units on the 11th and 12th floors of 545 West 25th Street in Chelsea, Manhattan. The expected use is owner-occupied. The deal closed on July 28, 2026 and was recorded on August 6, 2026. The two properties have 7,080 square feet of built space according to a PincusCo analysis of city data. The sale price per built square foot is $988 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) The signatory for Karla Otto was Lawrence Rader . The signatory for Art Partner was Steven Tanen . The contract date was March 3, 2026. Art Partner is a global creative agency that manages talent for the fashion and luxury industries, and lists its address on the 12th floor, according to its website. Amber Testino is an executive at the firm. Her husband Giovanni Testino founded Art Partner. On July 1, 2026, Gazelli Art House pays $7.5 m</t>
+          <t>By: Vanessa Londono 6:30 am on August 8, 2026 Permits have been filed for a nine-story mixed-use building at 43-27 56th Street in Woodside, Queens. Located between 43rd Avenue Street and Queens Boulevard, the lot is near the 52nd Street subway station, served by the 7 train. Markiel Chulpayev is listed as the owner behind the applications. The proposed 116-foot-tall development will yield 22,922 square feet, with 21,905 square feet designated for residential space and 1,016 square feet for commercial space. The building will have 32 residences, most likely rentals based on the average unit scope of 684 square feet. The concrete-based structure will also have a cellar. Alexander Zhitnik of Z Architecture is listed as the architect of record. Demolition permits have not been filed yet. An estimated completion date has not been announced. Subscribe to YIMBY’s daily e-mail Follow YIMBYgram for real-time photo updates Like YIMBY on Facebook Follow YIMBY’s Twitter for the latest in YIMBYnews</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto update queens news 2026-08-09T13:13:05Z
</commit_message>
<xml_diff>
--- a/data/output/queens_dev_news.xlsx
+++ b/data/output/queens_dev_news.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H2"/>
+  <dimension ref="A1:H1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -467,48 +467,6 @@
       <c r="H1" s="1" t="inlineStr">
         <is>
           <t>content_preview</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>Permits Filed for 43-27 56th Street in Woodside, Queens</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>https://newyorkyimby.com/2026/08/permits-filed-for-43-27-56th-street-in-woodside-queens.html</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>Permits have been filed for a nine-story mixed-use building at 43-27 56th Street in &lt;a href="https://newyorkyimby.com/neighborhoods/woodside"&gt;Woodside&lt;/a&gt;, Queens. Located between 43rd Avenue Street and Queens Boulevard, the lot is near the 52nd Street subway station, served by the 7 train. Markiel Chulpayev is listed as the owner behind the applications.</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>2026-08-08T10:30:22+00:00</t>
-        </is>
-      </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>Sat, 08 Aug 2026 10:30:22 +0000</t>
-        </is>
-      </c>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t>YIMBY</t>
-        </is>
-      </c>
-      <c r="G2" t="inlineStr">
-        <is>
-          <t>YIMBY - Woodside</t>
-        </is>
-      </c>
-      <c r="H2" t="inlineStr">
-        <is>
-          <t>By: Vanessa Londono 6:30 am on August 8, 2026 Permits have been filed for a nine-story mixed-use building at 43-27 56th Street in Woodside, Queens. Located between 43rd Avenue Street and Queens Boulevard, the lot is near the 52nd Street subway station, served by the 7 train. Markiel Chulpayev is listed as the owner behind the applications. The proposed 116-foot-tall development will yield 22,922 square feet, with 21,905 square feet designated for residential space and 1,016 square feet for commercial space. The building will have 32 residences, most likely rentals based on the average unit scope of 684 square feet. The concrete-based structure will also have a cellar. Alexander Zhitnik of Z Architecture is listed as the architect of record. Demolition permits have not been filed yet. An estimated completion date has not been announced. Subscribe to YIMBY’s daily e-mail Follow YIMBYgram for real-time photo updates Like YIMBY on Facebook Follow YIMBY’s Twitter for the latest in YIMBYnews</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto update queens news 2026-08-10T13:39:50Z
</commit_message>
<xml_diff>
--- a/data/output/queens_dev_news.xlsx
+++ b/data/output/queens_dev_news.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H1"/>
+  <dimension ref="A1:H4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -467,6 +467,108 @@
       <c r="H1" s="1" t="inlineStr">
         <is>
           <t>content_preview</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Pearl Realty Management acquires Sculptor, Longfellow office in LIC in $86.9M transfer</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>https://www.pincusco.com/pearl-realty-management-acquires-sculptor-capital-office-in-lic-in-86-9m-transfer/</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Pearl Realty Management through the entity 4310 23 St LLC acquired the office building (O6)</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr"/>
+      <c r="E2" t="inlineStr"/>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>PincusCo</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>PincusCo - Home</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>Transfers 43-10 23rd Street (Credit - Cyclomedia) Continue reading with a PincusCo subscription Sign up for a paid subscription to view this content. Already a subscriber? Log in here. Continue Reading</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Anthony Roussos files plans for 69 units in Astoria</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>https://www.pincusco.com/anthony-roussos-files-plans-for-69-units-in-astoria/</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Anthony Roussos submitted a new building construction project for a 69-unit, 77,748-square-foot residential (R-2) building</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr"/>
+      <c r="E3" t="inlineStr"/>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>PincusCo</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>PincusCo - Home</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>Development 25-05 35th Street elevation (Credit - Gerald Caliendo architect via DOB) Anthony Roussos submitted a new building construction project for a 69-unit, 77,748-square-foot residential (R-2) building at 25-05 35th Street in Astoria, Queens. The plan was filed on August 7, 2026. It calls for the construction of a 85-foot-tall, eight-story building and was filed with the New York City Department of Buildings under job number Q01426754. The project is described in the filing as: one new eight-story, mix-used building with 69 dwelling units and commercial space on the ground floor, a MIH site, and an ultra low energy building. The applicant is the Registered Architect Gerald Caliendo of Gerald Caliendo Architects . City property records show Anthony Roussos owns the property through Astoria Boulevard LLC. The neighborhood In Astoria, The bulk, or 36 percent of the 40.2 million square feet of commercial built space are walkup buildings, with elevator buildings next occupying 31 percent of the space. In sales, Astoria has near average sales volume among other neighborhoods with $794.6 million in sales volume in the last two years and is the 2nd highest in Queens. For development,</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>ZD Jasper seeks zoning change to facilitate approximately 214-unit project in Astoria</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>https://www.pincusco.com/zd-jasper-seeks-zoning-change-to-facilitate-approximately-214-unit-project-in-astoria/</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Great Neck–based developer ZD Jasper Realty, through entity ZDJ Steinway LLC, filed a land use</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr"/>
+      <c r="E4" t="inlineStr"/>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>PincusCo</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>PincusCo - Home</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>Development Top Story 34-39 to 34-49 Steinway Street (Credit - Cyclomedia) Continue reading with a PincusCo subscription Sign up for a paid subscription to view this content. Already a subscriber? Log in here.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto update queens news 2026-08-11T13:38:09Z
</commit_message>
<xml_diff>
--- a/data/output/queens_dev_news.xlsx
+++ b/data/output/queens_dev_news.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H4"/>
+  <dimension ref="A1:H1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -467,108 +467,6 @@
       <c r="H1" s="1" t="inlineStr">
         <is>
           <t>content_preview</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>Pearl Realty Management acquires Sculptor, Longfellow office in LIC in $86.9M transfer</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>https://www.pincusco.com/pearl-realty-management-acquires-sculptor-capital-office-in-lic-in-86-9m-transfer/</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>Pearl Realty Management through the entity 4310 23 St LLC acquired the office building (O6)</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr"/>
-      <c r="E2" t="inlineStr"/>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t>PincusCo</t>
-        </is>
-      </c>
-      <c r="G2" t="inlineStr">
-        <is>
-          <t>PincusCo - Home</t>
-        </is>
-      </c>
-      <c r="H2" t="inlineStr">
-        <is>
-          <t>Transfers 43-10 23rd Street (Credit - Cyclomedia) Continue reading with a PincusCo subscription Sign up for a paid subscription to view this content. Already a subscriber? Log in here. Continue Reading</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>Anthony Roussos files plans for 69 units in Astoria</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>https://www.pincusco.com/anthony-roussos-files-plans-for-69-units-in-astoria/</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>Anthony Roussos submitted a new building construction project for a 69-unit, 77,748-square-foot residential (R-2) building</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr"/>
-      <c r="E3" t="inlineStr"/>
-      <c r="F3" t="inlineStr">
-        <is>
-          <t>PincusCo</t>
-        </is>
-      </c>
-      <c r="G3" t="inlineStr">
-        <is>
-          <t>PincusCo - Home</t>
-        </is>
-      </c>
-      <c r="H3" t="inlineStr">
-        <is>
-          <t>Development 25-05 35th Street elevation (Credit - Gerald Caliendo architect via DOB) Anthony Roussos submitted a new building construction project for a 69-unit, 77,748-square-foot residential (R-2) building at 25-05 35th Street in Astoria, Queens. The plan was filed on August 7, 2026. It calls for the construction of a 85-foot-tall, eight-story building and was filed with the New York City Department of Buildings under job number Q01426754. The project is described in the filing as: one new eight-story, mix-used building with 69 dwelling units and commercial space on the ground floor, a MIH site, and an ultra low energy building. The applicant is the Registered Architect Gerald Caliendo of Gerald Caliendo Architects . City property records show Anthony Roussos owns the property through Astoria Boulevard LLC. The neighborhood In Astoria, The bulk, or 36 percent of the 40.2 million square feet of commercial built space are walkup buildings, with elevator buildings next occupying 31 percent of the space. In sales, Astoria has near average sales volume among other neighborhoods with $794.6 million in sales volume in the last two years and is the 2nd highest in Queens. For development,</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>ZD Jasper seeks zoning change to facilitate approximately 214-unit project in Astoria</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>https://www.pincusco.com/zd-jasper-seeks-zoning-change-to-facilitate-approximately-214-unit-project-in-astoria/</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>Great Neck–based developer ZD Jasper Realty, through entity ZDJ Steinway LLC, filed a land use</t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr"/>
-      <c r="E4" t="inlineStr"/>
-      <c r="F4" t="inlineStr">
-        <is>
-          <t>PincusCo</t>
-        </is>
-      </c>
-      <c r="G4" t="inlineStr">
-        <is>
-          <t>PincusCo - Home</t>
-        </is>
-      </c>
-      <c r="H4" t="inlineStr">
-        <is>
-          <t>Development Top Story 34-39 to 34-49 Steinway Street (Credit - Cyclomedia) Continue reading with a PincusCo subscription Sign up for a paid subscription to view this content. Already a subscriber? Log in here.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto update queens news 2026-08-13T13:41:56Z
</commit_message>
<xml_diff>
--- a/data/output/queens_dev_news.xlsx
+++ b/data/output/queens_dev_news.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H1"/>
+  <dimension ref="A1:H3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -467,6 +467,74 @@
       <c r="H1" s="1" t="inlineStr">
         <is>
           <t>content_preview</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Heights Advisors seeks zoning change to build 606 affordable units in Soundview</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>https://www.pincusco.com/heights-advisors-seeks-zoning-change-to-build-606-affordable-units-in-soundview/</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Brooklyn-based Heights Advisors submitted a land use application yesterday to facilitate the construction of a</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr"/>
+      <c r="E2" t="inlineStr"/>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>PincusCo</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>PincusCo - Home</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>Chart_Frontpage Development Top Story 945 White Plains Road is in red, additional areas subject to rezoning but not part of the project are in yellow Continue reading with a PincusCo subscription Sign up for a paid subscription to view this content.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>James Grech files plans for 75 units in Woodside</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>https://www.pincusco.com/james-grech-files-plans-for-75-units-in-woodside/</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>James Grech submitted a new building construction project for a 75-unit, 67,155-square-foot residential (R-2) building</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr"/>
+      <c r="E3" t="inlineStr"/>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>PincusCo</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>PincusCo - Home</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>Development 43-36 53rd Street axonometric diagram (Credit - Gerald Caliendo architect via DOB) Continue reading with a PincusCo subscription Sign up for a paid subscription to view this content. Already a subscriber? Log in here. Continue Reading</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto update queens news 2026-08-14T13:37:09Z
</commit_message>
<xml_diff>
--- a/data/output/queens_dev_news.xlsx
+++ b/data/output/queens_dev_news.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H3"/>
+  <dimension ref="A1:H2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -473,17 +473,17 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Heights Advisors seeks zoning change to build 606 affordable units in Soundview</t>
+          <t>Hung Pin Hung files plans for 30 units with community facility in Flushing</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>https://www.pincusco.com/heights-advisors-seeks-zoning-change-to-build-606-affordable-units-in-soundview/</t>
+          <t>https://www.pincusco.com/hung-pin-hung-files-plans-for-30-units-with-community-facility-in-flushing/</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Brooklyn-based Heights Advisors submitted a land use application yesterday to facilitate the construction of a</t>
+          <t>Hung Pin Hung submitted a new building construction project for a 30-unit, 41,463-square-foot residential (R-2)</t>
         </is>
       </c>
       <c r="D2" t="inlineStr"/>
@@ -500,41 +500,7 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>Chart_Frontpage Development Top Story 945 White Plains Road is in red, additional areas subject to rezoning but not part of the project are in yellow Continue reading with a PincusCo subscription Sign up for a paid subscription to view this content.</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>James Grech files plans for 75 units in Woodside</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>https://www.pincusco.com/james-grech-files-plans-for-75-units-in-woodside/</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>James Grech submitted a new building construction project for a 75-unit, 67,155-square-foot residential (R-2) building</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr"/>
-      <c r="E3" t="inlineStr"/>
-      <c r="F3" t="inlineStr">
-        <is>
-          <t>PincusCo</t>
-        </is>
-      </c>
-      <c r="G3" t="inlineStr">
-        <is>
-          <t>PincusCo - Home</t>
-        </is>
-      </c>
-      <c r="H3" t="inlineStr">
-        <is>
-          <t>Development 43-36 53rd Street axonometric diagram (Credit - Gerald Caliendo architect via DOB) Continue reading with a PincusCo subscription Sign up for a paid subscription to view this content. Already a subscriber? Log in here. Continue Reading</t>
+          <t>Development 144-14 38th Avenue axonometric diagram (Credit - Ralph Kowalczyk architect via DOB) Continue reading with a PincusCo subscription Sign up for a paid subscription to view this content. Already a subscriber? Log in here. Continue Reading</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto update queens news 2026-08-15T12:56:22Z
</commit_message>
<xml_diff>
--- a/data/output/queens_dev_news.xlsx
+++ b/data/output/queens_dev_news.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H2"/>
+  <dimension ref="A1:H1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -467,40 +467,6 @@
       <c r="H1" s="1" t="inlineStr">
         <is>
           <t>content_preview</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>Hung Pin Hung files plans for 30 units with community facility in Flushing</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>https://www.pincusco.com/hung-pin-hung-files-plans-for-30-units-with-community-facility-in-flushing/</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>Hung Pin Hung submitted a new building construction project for a 30-unit, 41,463-square-foot residential (R-2)</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr"/>
-      <c r="E2" t="inlineStr"/>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t>PincusCo</t>
-        </is>
-      </c>
-      <c r="G2" t="inlineStr">
-        <is>
-          <t>PincusCo - Home</t>
-        </is>
-      </c>
-      <c r="H2" t="inlineStr">
-        <is>
-          <t>Development 144-14 38th Avenue axonometric diagram (Credit - Ralph Kowalczyk architect via DOB) Continue reading with a PincusCo subscription Sign up for a paid subscription to view this content. Already a subscriber? Log in here. Continue Reading</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto update queens news 2026-08-18T13:05:16Z
</commit_message>
<xml_diff>
--- a/data/output/queens_dev_news.xlsx
+++ b/data/output/queens_dev_news.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H1"/>
+  <dimension ref="A1:H2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -467,6 +467,40 @@
       <c r="H1" s="1" t="inlineStr">
         <is>
           <t>content_preview</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Jian Yun Liu files plans for 30 units in Elmhurst</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>https://www.pincusco.com/jian-yun-liu-files-plans-for-30-units-in-elmhurst/</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Jian Yun Liu submitted a new building construction project for a 30-unit, 25,960-square-foot residential (R-2)</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr"/>
+      <c r="E2" t="inlineStr"/>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>PincusCo</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>PincusCo - Home</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>Development 44-07 69th Street axonometric diagram (Credit - Ning Lu architect via DOB) Continue reading with a PincusCo subscription Sign up for a paid subscription to view this content. Already a subscriber? Log in here. Continue Reading</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto update queens news 2026-08-19T13:06:10Z
</commit_message>
<xml_diff>
--- a/data/output/queens_dev_news.xlsx
+++ b/data/output/queens_dev_news.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H2"/>
+  <dimension ref="A1:H1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -467,40 +467,6 @@
       <c r="H1" s="1" t="inlineStr">
         <is>
           <t>content_preview</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>Jian Yun Liu files plans for 30 units in Elmhurst</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>https://www.pincusco.com/jian-yun-liu-files-plans-for-30-units-in-elmhurst/</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>Jian Yun Liu submitted a new building construction project for a 30-unit, 25,960-square-foot residential (R-2)</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr"/>
-      <c r="E2" t="inlineStr"/>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t>PincusCo</t>
-        </is>
-      </c>
-      <c r="G2" t="inlineStr">
-        <is>
-          <t>PincusCo - Home</t>
-        </is>
-      </c>
-      <c r="H2" t="inlineStr">
-        <is>
-          <t>Development 44-07 69th Street axonometric diagram (Credit - Ning Lu architect via DOB) Continue reading with a PincusCo subscription Sign up for a paid subscription to view this content. Already a subscriber? Log in here. Continue Reading</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto update queens news 2026-08-22T12:57:59Z
</commit_message>
<xml_diff>
--- a/data/output/queens_dev_news.xlsx
+++ b/data/output/queens_dev_news.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H1"/>
+  <dimension ref="A1:H3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -467,6 +467,74 @@
       <c r="H1" s="1" t="inlineStr">
         <is>
           <t>content_preview</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Palwinder Singh files plans for 75 units in Long Island City</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>https://www.pincusco.com/palwinder-singh-files-plans-for-75-units-in-long-island-city/</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Palwinder Singh submitted a new building construction project for a 75-unit, 66,499-square-foot residential (R-2) building</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr"/>
+      <c r="E2" t="inlineStr"/>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>PincusCo</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>PincusCo - Home</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>Development 5-33 47th Avenue axonometric diagram (Credit - Fariba Makooi architect via DOB) Continue reading with a PincusCo subscription Sign up for a paid subscription to view this content. Already a subscriber? Log in here. Continue Reading</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>William Xie of EliteX Enterprise files plans for 12 units in Astoria</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>https://www.pincusco.com/william-xie-of-elitex-enterprise-files-plans-for-12-units-in-astoria/</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>William Xie of EliteX Enterprise submitted a new building construction project for a 12-unit, 11,116-square-foot</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr"/>
+      <c r="E3" t="inlineStr"/>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>PincusCo</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>PincusCo - Home</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>Development 30-14 21st Street axonometric diagram (Credit - Chang H. Tan architect via DOB) Continue reading with a PincusCo subscription Sign up for a paid subscription to view this content. Already a subscriber? Log in here. Continue Reading</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto update queens news 2026-08-23T12:59:29Z
</commit_message>
<xml_diff>
--- a/data/output/queens_dev_news.xlsx
+++ b/data/output/queens_dev_news.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H3"/>
+  <dimension ref="A1:H1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -467,74 +467,6 @@
       <c r="H1" s="1" t="inlineStr">
         <is>
           <t>content_preview</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>Palwinder Singh files plans for 75 units in Long Island City</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>https://www.pincusco.com/palwinder-singh-files-plans-for-75-units-in-long-island-city/</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>Palwinder Singh submitted a new building construction project for a 75-unit, 66,499-square-foot residential (R-2) building</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr"/>
-      <c r="E2" t="inlineStr"/>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t>PincusCo</t>
-        </is>
-      </c>
-      <c r="G2" t="inlineStr">
-        <is>
-          <t>PincusCo - Home</t>
-        </is>
-      </c>
-      <c r="H2" t="inlineStr">
-        <is>
-          <t>Development 5-33 47th Avenue axonometric diagram (Credit - Fariba Makooi architect via DOB) Continue reading with a PincusCo subscription Sign up for a paid subscription to view this content. Already a subscriber? Log in here. Continue Reading</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>William Xie of EliteX Enterprise files plans for 12 units in Astoria</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>https://www.pincusco.com/william-xie-of-elitex-enterprise-files-plans-for-12-units-in-astoria/</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>William Xie of EliteX Enterprise submitted a new building construction project for a 12-unit, 11,116-square-foot</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr"/>
-      <c r="E3" t="inlineStr"/>
-      <c r="F3" t="inlineStr">
-        <is>
-          <t>PincusCo</t>
-        </is>
-      </c>
-      <c r="G3" t="inlineStr">
-        <is>
-          <t>PincusCo - Home</t>
-        </is>
-      </c>
-      <c r="H3" t="inlineStr">
-        <is>
-          <t>Development 30-14 21st Street axonometric diagram (Credit - Chang H. Tan architect via DOB) Continue reading with a PincusCo subscription Sign up for a paid subscription to view this content. Already a subscriber? Log in here. Continue Reading</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto update queens news 2026-08-24T13:10:28Z
</commit_message>
<xml_diff>
--- a/data/output/queens_dev_news.xlsx
+++ b/data/output/queens_dev_news.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H1"/>
+  <dimension ref="A1:H2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -467,6 +467,40 @@
       <c r="H1" s="1" t="inlineStr">
         <is>
           <t>content_preview</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Ken Huang buys $34.4M note from Maverick, secured by Xin Development site in Flushing</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>https://www.pincusco.com/ken-huang-buys-34-4m-note-from-maverick-secured-by-xin-development-site-in-flushing/</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Ken Huang through the entity Northern Blvd Lender LLC bought a note with an original</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr"/>
+      <c r="E2" t="inlineStr"/>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>PincusCo</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>PincusCo - Home</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>Chart_Frontpage Transfers 135-35 Northern Boulevard RKO Keith's Theater location (Credit - Google Earth) Continue reading with a PincusCo subscription Sign up for a paid subscription to view this content. Already a subscriber? Log in here.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto update queens news 2026-08-25T13:08:56Z
</commit_message>
<xml_diff>
--- a/data/output/queens_dev_news.xlsx
+++ b/data/output/queens_dev_news.xlsx
@@ -473,17 +473,17 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Ken Huang buys $34.4M note from Maverick, secured by Xin Development site in Flushing</t>
+          <t>CAVU signs $45.6M construction loan with Ponce for 87-unit project in LIC</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>https://www.pincusco.com/ken-huang-buys-34-4m-note-from-maverick-secured-by-xin-development-site-in-flushing/</t>
+          <t>https://www.pincusco.com/cavu-property-group-signs-45-6m-new-construction-loan-with-ponce-bank-for-industrial-in-long-island-city/</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Ken Huang through the entity Northern Blvd Lender LLC bought a note with an original</t>
+          <t>CAVU Property Group through the entity 32-20 38th Avenue LLC as borrower signed a new</t>
         </is>
       </c>
       <c r="D2" t="inlineStr"/>
@@ -500,7 +500,7 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>Chart_Frontpage Transfers 135-35 Northern Boulevard RKO Keith's Theater location (Credit - Google Earth) Continue reading with a PincusCo subscription Sign up for a paid subscription to view this content. Already a subscriber? Log in here.</t>
+          <t>Transfers CAVU Property Group 3-property development site (Credit - Google Earth) Continue reading with a PincusCo subscription Sign up for a paid subscription to view this content. Already a subscriber? Log in here. Continue Reading</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto update queens news 2026-08-26T13:13:18Z
</commit_message>
<xml_diff>
--- a/data/output/queens_dev_news.xlsx
+++ b/data/output/queens_dev_news.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H2"/>
+  <dimension ref="A1:H1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -467,40 +467,6 @@
       <c r="H1" s="1" t="inlineStr">
         <is>
           <t>content_preview</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>CAVU signs $45.6M construction loan with Ponce for 87-unit project in LIC</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>https://www.pincusco.com/cavu-property-group-signs-45-6m-new-construction-loan-with-ponce-bank-for-industrial-in-long-island-city/</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>CAVU Property Group through the entity 32-20 38th Avenue LLC as borrower signed a new</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr"/>
-      <c r="E2" t="inlineStr"/>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t>PincusCo</t>
-        </is>
-      </c>
-      <c r="G2" t="inlineStr">
-        <is>
-          <t>PincusCo - Home</t>
-        </is>
-      </c>
-      <c r="H2" t="inlineStr">
-        <is>
-          <t>Transfers CAVU Property Group 3-property development site (Credit - Google Earth) Continue reading with a PincusCo subscription Sign up for a paid subscription to view this content. Already a subscriber? Log in here. Continue Reading</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto update queens news 2026-08-27T22:13:55Z
</commit_message>
<xml_diff>
--- a/data/output/queens_dev_news.xlsx
+++ b/data/output/queens_dev_news.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H1"/>
+  <dimension ref="A1:H2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -467,6 +467,40 @@
       <c r="H1" s="1" t="inlineStr">
         <is>
           <t>content_preview</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>F&amp;T Group signs $123M construction loan with Maxim Capital for retail, office in Flushing</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>https://www.pincusco.com/ft-group-signs-123m-construction-loan-with-maxim-capital-for-retail-in-flushing/</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>F&amp;T Group through the entity Tdc Fc2 LLC as borrower signed a new construction loan</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr"/>
+      <c r="E2" t="inlineStr"/>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>PincusCo</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>PincusCo - Home</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>Transfers 37-01 138th Street aka Building E axonometric diagram (Credit - Frank A. Fusaro architect via DOB) Continue reading with a PincusCo subscription Sign up for a paid subscription to view this content. Already a subscriber? Log in here. Continue Reading</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto update queens news 2026-08-28T22:15:35Z
</commit_message>
<xml_diff>
--- a/data/output/queens_dev_news.xlsx
+++ b/data/output/queens_dev_news.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H2"/>
+  <dimension ref="A1:H1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -467,40 +467,6 @@
       <c r="H1" s="1" t="inlineStr">
         <is>
           <t>content_preview</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>F&amp;T Group signs $123M construction loan with Maxim Capital for retail, office in Flushing</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>https://www.pincusco.com/ft-group-signs-123m-construction-loan-with-maxim-capital-for-retail-in-flushing/</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>F&amp;T Group through the entity Tdc Fc2 LLC as borrower signed a new construction loan</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr"/>
-      <c r="E2" t="inlineStr"/>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t>PincusCo</t>
-        </is>
-      </c>
-      <c r="G2" t="inlineStr">
-        <is>
-          <t>PincusCo - Home</t>
-        </is>
-      </c>
-      <c r="H2" t="inlineStr">
-        <is>
-          <t>Transfers 37-01 138th Street aka Building E axonometric diagram (Credit - Frank A. Fusaro architect via DOB) Continue reading with a PincusCo subscription Sign up for a paid subscription to view this content. Already a subscriber? Log in here. Continue Reading</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto update queens news 2026-08-31T19:07:23Z
</commit_message>
<xml_diff>
--- a/data/output/queens_dev_news.xlsx
+++ b/data/output/queens_dev_news.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H1"/>
+  <dimension ref="A1:H2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -467,6 +467,40 @@
       <c r="H1" s="1" t="inlineStr">
         <is>
           <t>content_preview</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Domain, BLDG, Canyon sign $175.6M construction loan with Wells Fargo for 429 units in Astoria</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>https://www.pincusco.com/domain-bldg-canyon-sign-175-6m-construction-loan-with-wells-fargo-for-429-units-in-astoria/</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Domain Companies, BLDG Management, and Canyon Partners through the entities Domain 41st Street Site A</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr"/>
+      <c r="E2" t="inlineStr"/>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>PincusCo</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>PincusCo - Home</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>Transfers Axonometric diagrams of 35-53 41st Street (l.) and 35-38 41st Street (r.) (Credit - Paul Carr architect via DOB) Continue reading with a PincusCo subscription Sign up for a paid subscription to view this content. Already a subscriber? Log in here. Continue Reading</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto update queens news 2026-09-01T16:35:36Z
</commit_message>
<xml_diff>
--- a/data/output/queens_dev_news.xlsx
+++ b/data/output/queens_dev_news.xlsx
@@ -473,17 +473,17 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Domain, BLDG, Canyon sign $175.6M construction loan with Wells Fargo for 429 units in Astoria</t>
+          <t>Wharton Properties signs $5.2M refi with Peapack for retail in Longwood</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>https://www.pincusco.com/domain-bldg-canyon-sign-175-6m-construction-loan-with-wells-fargo-for-429-units-in-astoria/</t>
+          <t>https://www.pincusco.com/wharton-properties-signs-5-2m-refi-with-peapack-for-retail-in-longwood/</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Domain Companies, BLDG Management, and Canyon Partners through the entities Domain 41st Street Site A</t>
+          <t>Wharton Properties through the entity 2902 Third Avenue LLC as borrower signed a refi loan</t>
         </is>
       </c>
       <c r="D2" t="inlineStr"/>
@@ -500,7 +500,7 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>Transfers Axonometric diagrams of 35-53 41st Street (l.) and 35-38 41st Street (r.) (Credit - Paul Carr architect via DOB) Continue reading with a PincusCo subscription Sign up for a paid subscription to view this content. Already a subscriber? Log in here. Continue Reading</t>
+          <t>Transfers 2902 3rd Avenue (Credit - Cyclomedia) Wharton Properties through the entity 2902 Third Avenue LLC as borrower signed a refi loan with lender Peapack Private Bank &amp; Trust for the retail building (K1) at 2902 3rd Avenue in Longwood, Bronx. The deal closed on August 25, 2026 and was recorded on August 28, 2026. The prior lender was Flagstar Bank which held debt that had an original loan amount of $4.1 million. The property has 5,600 square feet of built space and 14,264 square feet of additional air rights for a total buildable of 19,866 square feet according to a PincusCo analysis of city data. The loan price per built square foot is $919 and the price per buildable square foot is $259 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) The owner bought the property on November 12, 2009, for $4 million. The signatory for Wharton Properties was Jeff Sutton . Prior sales, articles and revenue The 5,600-square-foot property generated revenue of $755,201 or $135 per square foot, according to the most recent income and expense figures. The property</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto update queens news 2026-09-02T16:31:58Z
</commit_message>
<xml_diff>
--- a/data/output/queens_dev_news.xlsx
+++ b/data/output/queens_dev_news.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H2"/>
+  <dimension ref="A1:H1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -467,40 +467,6 @@
       <c r="H1" s="1" t="inlineStr">
         <is>
           <t>content_preview</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>Wharton Properties signs $5.2M refi with Peapack for retail in Longwood</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>https://www.pincusco.com/wharton-properties-signs-5-2m-refi-with-peapack-for-retail-in-longwood/</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>Wharton Properties through the entity 2902 Third Avenue LLC as borrower signed a refi loan</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr"/>
-      <c r="E2" t="inlineStr"/>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t>PincusCo</t>
-        </is>
-      </c>
-      <c r="G2" t="inlineStr">
-        <is>
-          <t>PincusCo - Home</t>
-        </is>
-      </c>
-      <c r="H2" t="inlineStr">
-        <is>
-          <t>Transfers 2902 3rd Avenue (Credit - Cyclomedia) Wharton Properties through the entity 2902 Third Avenue LLC as borrower signed a refi loan with lender Peapack Private Bank &amp; Trust for the retail building (K1) at 2902 3rd Avenue in Longwood, Bronx. The deal closed on August 25, 2026 and was recorded on August 28, 2026. The prior lender was Flagstar Bank which held debt that had an original loan amount of $4.1 million. The property has 5,600 square feet of built space and 14,264 square feet of additional air rights for a total buildable of 19,866 square feet according to a PincusCo analysis of city data. The loan price per built square foot is $919 and the price per buildable square foot is $259 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) The owner bought the property on November 12, 2009, for $4 million. The signatory for Wharton Properties was Jeff Sutton . Prior sales, articles and revenue The 5,600-square-foot property generated revenue of $755,201 or $135 per square foot, according to the most recent income and expense figures. The property</t>
         </is>
       </c>
     </row>

</xml_diff>